<commit_message>
Scan results, 2026-09-16 13:46 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R13"/>
+  <dimension ref="A1:R52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1526,6 +1526,3190 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Unknown player</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Red Crystalline Refractor Stefanos Tsitsipas Relic Card 1/1!</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>700.00 USD</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/137740177241</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/VT4AAeSw2X5qqV-G/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15T15:17:09.000Z</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/EbMAAeSwfuZqqV-6/s-l1600.jpg | https://i.ebayimg.com/images/g/sI0AAeSwIWdqqV~S/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Unknown player</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>topps graphite tennis 3 Card Kayla Day Lot. Relic, Relic Auto and 15/15</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>last of 15 (15/15)</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>10.00 USD</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/820098688771</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/pTMAAeSwXfNqntLE/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07T15:06:04.000Z</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/WyMAAeSw4tlqntLF/s-l1600.jpg | https://i.ebayimg.com/images/g/usUAAeSwBSVqntLF/s-l1600.jpg | https://i.ebayimg.com/images/g/0bAAAeSwKpJqntLE/s-l1600.jpg | https://i.ebayimg.com/images/g/eBIAAeSwaExqntLF/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr"/>
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Borna Coric</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Tennis Borna Coric Active Metal Card Red #1/1 ACM-61</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>199.99 USD</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/227503451499?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2B6%2Bq2h%2BqfM9j4QSGqSeU%2BrSekrC1GwRRtu0X6AqQLd4vcGtJgUMnMh0YI07hUtKIFF9l6sV0Icn8J1ixfsQDc79G%2Fp4cXiJwvk%2Blf4hgfTaX9cdWHud899xMHd59EZxWAAoNta22zyj%2BTKbczlRHj0lm8nFoBTWadzprwqfwtjUmhjfyR3edJ7zFntroRcmb0%3D</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/BXwAAeSwZERqmQr6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03T05:53:05.000Z</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA)</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bTEAAeSwoxhqmQsD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>DANIIL MEDVEDEV</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>2026 TOPPS GRAPHITE TENNIS----DANIIL MEDVEDEV---RELIC CARD---15/15---BOOKEND</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>last of 15 (15/15)</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>74.99 USD</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287525164423?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2FYnwzJbREIIMDxeiy4fJYO61CqC4tUl1gGhxOMoXjLRgJTfMusgja9vXpHzSYprjj%2FhiIqo%2FS0yILNlpz19ce9e8WSVY4AQM97CSWIZ71Jk2zLuGorc%2B9Pud1YTxyRSEhL0oElMMV5CeJe7R5fuEI9FbsDU7Fb4D%2FnpOZUjiKfbQL7JeE1hQdtWWEeoD%2FbWDI%3D</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/PMUAAeSwtqtqf1hX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14T18:07:54.000Z</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/WQEAAeSwaRZqf1hj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr"/>
+      <c r="P17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Bublik</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Tennis Blue #46 Alexander Bublik 50/50 Tennis Card</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>8.49 USD</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287496465307?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2Fruz%2FI5o9aPfcff1bN4zE7OmJoEK48P13t8WPsxOeD9pUCwsuaeo6st7QUfKIBnkhk3LVjvUChzrM9a8rJ05LPyS0G3HGoy0iWdb8Dw1UqJGDpREjzzYWuHG3W3bQw%2BJhLJtsVJjbpIjKDCddskiKHLw4EGPjQ%2FyE5OOmv5t4K%2B%2BfAR0Aud%2F2BAT2viVtyZq4%3D</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/iIMAAeSwfRBqbb9G/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01T09:43:28.000Z</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/OxQAAeSwpwZqbb9M/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Camila Osorio</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Camila Osorio 2026 Topps Graphite Tennis Trading Card Relic Autograph #01/25</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>64.19 USD</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298456851095</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/AvEAAeSwFcFqPzx7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27T08:01:44.000Z</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/a0IAAeSwKxhqPzx0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr"/>
+      <c r="P19" s="2" t="inlineStr"/>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Carel Ngounoue</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Carel Ngounoue 1/1 Topps Graphite Black Shimmer One Of One SSP Tennis Card</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>850.00 USD</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/800226920152</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/WVsAAeSwS95qOZKb/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T19:53:38.000Z</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/yikAAeSwyadqOZKa/s-l1600.jpg | https://i.ebayimg.com/images/g/3zUAAeSwnudqOZKa/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Nick Kyrgios</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Nick Kyrgios Topps Graphite Pink Parallel 01/15 Tennis Card SSP Refractor</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>69.99 USD</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/800226799485</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/p~UAAeSw~4xqOYuj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T19:24:50.000Z</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bTwAAeSwdi1qOYuj/s-l1600.jpg | https://i.ebayimg.com/images/g/r4UAAeSw6B9qOYuj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Mirra Andreeva Patch Auto 1/1 Rookie Card</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>15000.00 USD</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257546756801?amdata=enc%3AAQALAAAAsCHNgUiiE%2FjQhlDTaMiAde8Om4p0XfqaLeUlS%2BsoDARvZySlirkqbUQtRpQxrY3HleyxbiqQnRfq3OINyC03FrW7bbYEa4161aBIk6OKjVdW0u5PomsHQXypBvteYXU9EHQXqWi4FRU07xNV0XPyHCHoF4PP4aeMYDmst%2FtYH482aI3aJNKinAl8qRREojb%2BEKWMokF76kKWU43G1jKiqXKrJHdQZ58BMq7DdONgfFqA</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nNQAAeSw3YRqJiwb/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04T17:52:00.000Z</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/xGoAAeSwfE5qIbo1/s-l1600.jpg | https://i.ebayimg.com/images/g/nAEAAeSwEBNqIbo1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr"/>
+      <c r="P22" s="2" t="inlineStr"/>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Luciano Darderi</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Tennis Luciano Darderi 75/75 Green Refractor Relic Card</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>75/75</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>last of 75 (75/75)</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>15.77 USD</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298373879293?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8eYvEiQBX1%2BBEHsTF1xj6m1SRW7pfzFQVoBdrm7tx7PKz9K%2FAJxblvXinRI41FDSvhYqBHo86ovgRJ7pCTw9gPvxNqHSWUeOuw6wVkX7dN11s2QRWVOY08EC1xKD9CLVyIHcgTbbR%2BXxSM1D%2BScqEzfCyFMIgUMKLnNGLBEwlofcTb93t7jzEdv0%2FtF%2B%2F8z9c%3D</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/i9YAAeSwIOxqHUto/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01T09:30:01.000Z</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XlcAAeSw6SZqHUto/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr"/>
+      <c r="Q23" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Elisabetta Cocciaretto</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Topps Graphite Elisabetta Cocciaretto Serial #76 10/10 Tennis Card 2026</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>18.99 USD</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/198365080155?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2BD6dWgJ71IG6a2PKzeeBgXKWvUHWTLS923MqbN4q3uxhTSl%2F3xccDdvFjLfSuJVbvA30W5gYO9GCJ8Z%2FDKwOiJUnEDqp2q7yxSlG7BRfhk7PxvMo4X8KRYSOClP3COFYfzTqwhSkkWT8roRwhuBTjdT0Fo2RX9yHlDaaqqYn%2BG8cQl0JpTdSToclGIEnHwr%2Bs%3D</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/EIAAAeSw9fpqC8F8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19T01:49:18.000Z</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/boUAAeSwnSNqC8Fy/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr"/>
+      <c r="P24" s="2" t="inlineStr"/>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Monica Seles</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Tennis Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Monica Seles On Card Auto PSA 10 1/10 SSP 2024 Topps Graphite #GS-MSS Signatures</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>300.00 USD</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/397747917046?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8kMFHfzkc6WzgrzFUZ3Xs%2FFlX6Uo0Z%2FyuLOpO949ZYOdHpFVhaXlfOb5U%2FI%2BZblFH0pItYHZB4fd2Od%2Fqcm%2BJPevGAlP4ziB6Ni7zlAXj3VCN9fP%2FwbUoqMAlweCF8uWfX8L3dAFcdzxF7DN3%2BQN%2BZ%2FrIFGPQf1jrXC61fyySAtGCoVsJrj4PatHgT4CrVj6k%3D</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TE0AAeSwiuFpwDCy/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22T18:12:46.000Z</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>PSA 10</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr"/>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Shintaro Mochizuki</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Graphite Signature Relics</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>SHINTARO MOCHIZUHI 2024 GSR-SMI Topps Graphite Auto/Relic card S#01/10 in holder</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>59.00 USD</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/127387966107</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/W5UAAeSw11No0aMm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>2025-09-22T19:29:02.000Z</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/T84AAeSwKfJo0aMn/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr"/>
+      <c r="P26" s="2" t="inlineStr"/>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Unknown player</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>VICTORIA J KASINTSEVA 2024 TRA-VJK Topps Graphite Tour Relic autograph card 1/15</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>54.00 USD</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/127259572128</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/X-IAAeSwzqlogTbW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>2025-07-23T19:32:29.000Z</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Um8AAeSw2GBogTbW/s-l1600.jpg | https://i.ebayimg.com/images/g/hj4AAeSwIN5ogTbW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr"/>
+      <c r="P27" s="2" t="inlineStr"/>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Belinda Bencic</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite Tennis</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Tennis #GS-BBE Belinda Bencic Pink On Card Auto 15/15</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>last of 15 (15/15)</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>149.99 USD</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/376300010067</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/A4cAAeSwbN5oPSZq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>2025-06-02T04:20:36.000Z</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gi8AAeSwY7VoPSZy/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr"/>
+      <c r="Q28" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Shintaro Mochizuki</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Graphite Signature Relics</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>SHINTARO MOCHIZUHI 2024 GSR-SMI Topps Graphite Auto/Relic card S#01/15 in holder</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>54.00 USD</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/127045654733</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HKUAAOSwx35n-DoJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>2025-04-10T21:41:55.000Z</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/GwYAAOSwPkFn-DoI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr"/>
+      <c r="P29" s="2" t="inlineStr"/>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Kilian Feldbausch</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Graphite Signature Relics</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>KILIAN FELDBAUSCH 2024 GSR-KFH Topps Graphite Auto/Relic card S#01/15 in holder</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>54.00 USD</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/127033222286</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8ogAAOSw9Sdn7~rX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>2025-04-04T15:46:51.000Z</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/UfsAAOSwKcNn7~rW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr"/>
+      <c r="P30" s="2" t="inlineStr"/>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Unknown player</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite Signature</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>MIOMIR KECMANOVIC 2024 GS-MKC Topps Graphite AUTOGRAPH card in new holder 1/15</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>57.00 USD</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/127017907908</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/EZ4AAOSwrNln5azk/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>2025-03-27T20:04:04.000Z</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RaAAAOSwcjNn5azk/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr"/>
+      <c r="P31" s="2" t="inlineStr"/>
+      <c r="Q31" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Andrey Rublev</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Tennis Active Metal Card Red #42 Andrey Rublev 1/1</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>999.99 USD</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/197113232571</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/f98AAeSwkMtn1ix~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>2025-03-16T01:42:51.000Z</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ZNgAAeSwk81n1iyA/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr"/>
+      <c r="Q32" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>PRISKA NUGROHO</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>PRISKA NUGROHO 2024 GSR-PNO Topps Graphite Signature Relics card 01/10 MINT RC</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>79.00 USD</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/126969903958</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/q6cAAeSw~fNolSCg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>2025-03-02T00:38:23.000Z</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/sv0AAeSwwa5olSCg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr"/>
+      <c r="P33" s="2" t="inlineStr"/>
+      <c r="Q33" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Unknown player</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Tennis Daniel Rincon Rookie Blue On Card Auto 50/50 RC SP</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>11.99 USD</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/286266311195</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/kpsAAOSwO~NniC2d/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>2025-01-15T21:50:49.000Z</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/S9wAAOSwqTRniC2d/s-l1600.jpg | https://i.ebayimg.com/images/g/OsMAAOSw3ZxniC2h/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr"/>
+      <c r="Q34" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Unknown player</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Tennis Abdullah Shelbayh Blue On Card Rookie Auto 01/50 RC</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>13.99 USD</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/286254571840</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/oHEAAOSw1SpnftKk/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>2025-01-08T19:32:14.000Z</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/o1MAAOSwCyRnftKk/s-l1600.jpg | https://i.ebayimg.com/images/g/GLwAAOSwzptnftKk/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="inlineStr"/>
+      <c r="Q35" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Emma Navarro</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Tennis Emma Navarro White Refractor On Card AUTO #d 10/10</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>339.99 USD</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/286226453301</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:45 UTC</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/e2gAAOSwYaVnZ1Bv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>2024-12-21T23:34:57.000Z</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DpQAAOSwibRnZ1CG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr"/>
+      <c r="Q36" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Casper Ruud</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Tennis Collection</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Casper Ruud 2024 Topps Royalty The Grip Relic 5/5 Bookend Rare Tennis Card</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>1200.00 USD</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366667075611</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:46 UTC</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ZJ8AAeSwvd5qpxGE/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13T21:27:02.000Z</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr"/>
+      <c r="O37" s="2" t="inlineStr"/>
+      <c r="P37" s="2" t="inlineStr"/>
+      <c r="Q37" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff - 2024 Topps Royalty Tennis Auto Jumbo Relic Book Card Platinum 1/1</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>20000.00 USD</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147491453138</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:46 UTC</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/MN8AAeSwdSZqd11I/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-08T16:46:42.000Z</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vR4AAeSwhrBqd11I/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr"/>
+      <c r="P38" s="2" t="inlineStr"/>
+      <c r="Q38" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Unknown player</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva 2024 Topps Royalty Tennis BASE CARD GOLD 01/10 #39 RC Russia /10</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>1499.99 USD</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/188727023268</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:46 UTC</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/F2sAAeSwfwRqbfNE/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01T13:23:37.000Z</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Zf4AAeSwqmpqbfNI/s-l1600.jpg | https://i.ebayimg.com/images/g/McsAAeSwwzRqbfNS/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="inlineStr"/>
+      <c r="Q39" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Nastasja Scunk</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Rookie Jumbo Relic Card - Nastasja Schunk - NJR-NS 1/5</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>179.00 USD</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237022311038</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:46 UTC</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/UDEAAeSwGNVqLiIE/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22T00:29:03.000Z</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="inlineStr"/>
+      <c r="P40" s="2" t="inlineStr"/>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Monica Seles</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Collection Tennis</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Collection MONICA SELES ROYAL DECREE ON CARD AUTO # 1/25</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>129.95 USD</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/127965695784</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:46 UTC</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jY8AAeSw6EJqT3tX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09T11:03:03.000Z</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/FmoAAeSwVplqT3ti/s-l1600.jpg | https://i.ebayimg.com/images/g/ZzUAAeSwgf5qT3uW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="inlineStr"/>
+      <c r="Q41" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Liv Hovde</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Liv Hovde Auto Autograph Jumbo Relic Book Cards RC 1/5</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>125.00 USD</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/188619166333</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:46 UTC</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3mcAAeSw6EJqTvoc/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09T01:32:44.000Z</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jrEAAeSwkSpqTvol/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr"/>
+      <c r="P42" s="2" t="inlineStr"/>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Belinda Bencic</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Royalty / Museum / Premium Set</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Belinda Bencic TRUE 1/1 Auto – Topps Royalty / Museum Style – Certified On-Card</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>9999.00 USD</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366167294565</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:46 UTC</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/y6IAAeSw9lhpf5pL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01T18:33:59.000Z</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/1FUAAeSwiG1pf5pH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr"/>
+      <c r="P43" s="2" t="inlineStr"/>
+      <c r="Q43" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Elisabetta Cocciaretto</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Pursuit of Greatness Signatures</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Platinum Elisabetta Cocciaretto 1/1 On Card Rookie Auto RC</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>250.00 USD</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/397076397929?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2FTx5g15zVJp%2Bp82z7SRBxqGT0tI3NZlSwJsFtWRFFj6Qs2rrErfHOEZWOzS6g8BbVuOutX2RrSG38P0iQnE%2FkUcAMFivPuCYrFdmVPwLM%2FUQ5%2BK%2BtigLJLEkWzF80yiblQIE4I4zLcVwW%2B1UltRCRdi%2FT0Fjhn12tTlQPOP6wnP4WfCaGykjcVkwmmXzTDlLg%3D</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:46 UTC</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ZnUAAeSwUntozkt2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>2025-09-20T20:54:44.000Z</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/o-MAAeSwbVhozkt3/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr"/>
+      <c r="P44" s="2" t="inlineStr"/>
+      <c r="Q44" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Unknown player</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS ROYALTY TENNIS FERNANDA CONTRERAS ROOKIE ON CARD AUTOGRAPH GREEN 5/5</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>49.99 USD</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/146819155965</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:46 UTC</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~JYAAeSwQ6hovlj-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>2025-09-08T04:20:01.000Z</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/49QAAeSwtQZovlj-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P45" s="2" t="inlineStr"/>
+      <c r="Q45" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Celine Naef</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Celine Naef Rookie (RC) Relic Auto Card 01/25 First on Print</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>125.00 USD</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/365702809369</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:46 UTC</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/q9IAAeSwHp9oYy~A/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>2025-07-01T00:50:03.000Z</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/mVEAAeSwbANoYy~A/s-l1600.jpg | https://i.ebayimg.com/images/g/3pwAAeSwDQpoYy~A/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="inlineStr"/>
+      <c r="Q46" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Madison Keys, Bjorn Fratangelo</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS ROYALTY MADISON KEYS/BJORN FRATANGELO DUAL ON CARD AUTO 1/25 FOTL</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>200.00 USD</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/365679604515</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:46 UTC</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XSEAAOSwkOdoUrGl/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>2025-06-18T12:35:54.000Z</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9k8AAOSwPJNoUrGp/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O47" s="2" t="inlineStr"/>
+      <c r="P47" s="2" t="inlineStr"/>
+      <c r="Q47" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Chris Evert</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis - Chris Evert Ambassador On Card Auto Green 1/5 HOF!</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>324.95 USD</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/177181200780?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8AuIfbNyo3V69EFy06H5LwSXQTk9KXMIlegtr7lbsBujdfxhtKQaWjsk9dOPpf9pYIew010H8RARY%2B3DCNdrqT87YKDICmNSUgJpGV3MTtvoXht%2BdpDBbi4AGwq9nsqPeKrlUqafZxYs3JbCTZdLEqGTGIIA3ufFIwSxyjXOiFybV4wNTmgABI%2FDLo4YXcMZQ%3D</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:46 UTC</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/FUIAAOSwVwpoSQ4N/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>2025-06-11T05:10:50.000Z</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ONsAAOSwU9hoSQ4U/s-l1600.jpg | https://i.ebayimg.com/images/g/6V0AAOSwyU5oSQ4X/s-l1600.jpg | https://i.ebayimg.com/images/g/b5kAAOSwT9FoSQ4c/s-l1600.jpg | https://i.ebayimg.com/images/g/jkAAAOSwAW1oSQ4m/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="inlineStr"/>
+      <c r="Q48" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Aryna Sabalenka</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis Ambassador Aryna Sabalenka - On Card Auto #AA-AS #1/5</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>800.00 USD</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/197403785524</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:46 UTC</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/934AAeSwrz1oQ9J6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>2025-06-07T05:50:02.000Z</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RZkAAeSwQV1oQ9J5/s-l1600.jpg | https://i.ebayimg.com/images/g/6j0AAeSwPNxoQ9J6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P49" s="2" t="inlineStr"/>
+      <c r="Q49" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Erika Andreeva, Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis Mirra &amp; Erika Andreeva Dual Auto Card 01/25</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>550.00 USD</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/256957827624</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:46 UTC</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/o5YAAOSwU9hoPNBq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>2025-06-01T22:09:02.000Z</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/iroAAOSwb-loPNB9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr"/>
+      <c r="P50" s="2" t="inlineStr"/>
+      <c r="Q50" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Lindsay Davenport</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Tennis</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis Lindsay Davenport 5/5 On Card Auto Influential Ink</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>165.00 USD</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/187249127817</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:46 UTC</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/oVQAAeSw6ZtoMNdJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>2025-05-23T20:16:12.000Z</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vMoAAeSwrCtoMNdJ/s-l1600.jpg | https://i.ebayimg.com/images/g/0JYAAeSwKbZoMNdJ/s-l1600.jpg | https://i.ebayimg.com/images/g/zEAAAeSwRm5oMNdJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P51" s="2" t="inlineStr"/>
+      <c r="Q51" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Unknown player</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Tennis</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis Jamie Murray On Card Auto Relic /10 Superior Signature</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>140.00 USD</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/187245949209</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:46 UTC</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/THcAAeSwJ2FoL30U/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>2025-05-22T19:40:02.000Z</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/1cEAAeSwoURoL30U/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O52" s="2" t="inlineStr"/>
+      <c r="P52" s="2" t="inlineStr"/>
+      <c r="Q52" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R52" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
@@ -1540,6 +4724,45 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId51"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-17 01:12 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R52"/>
+  <dimension ref="A1:R57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4709,6 +4709,410 @@
         </is>
       </c>
       <c r="R52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Clement Chidekh</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Clement Chidekh superfractor papa Auto Card 1/1</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>895.00 USD</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257747241544</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 01:11 UTC</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XMIAAeSwfuZqqwes/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16T21:19:32.000Z</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr"/>
+      <c r="O53" s="2" t="inlineStr"/>
+      <c r="P53" s="2" t="inlineStr"/>
+      <c r="Q53" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Matteo Arnaldi</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Matteo Arnaldi Green Refractor 001/125 Rookie Card 2025 Topps Chrome Tennis #55</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>1/125</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>001 of 125</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>1.43 USD</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/198646816171</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 01:11 UTC</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Lg0AAeSwNoNqi4m2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T00:33:11.000Z</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/viMAAeSw-dlqi4m2/s-l1600.jpg | https://i.ebayimg.com/images/g/eYQAAeSwWkZqi4m4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="inlineStr"/>
+      <c r="Q54" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Camila Osorio</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis Camila Osorio Purple #TCA-COO Auto Card 10/10</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>250.00 USD</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/267738883315</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 01:12 UTC</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/sicAAeSwYlpqZTgh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25T22:31:07.000Z</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/l1AAAeSwPGtqZTgi/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O55" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P55" s="2" t="inlineStr"/>
+      <c r="Q55" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Elina Avanesyan</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Autograph Rookie Card-Elina Avanesyan #CA-EAN +1/75 Youthquake</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>1/75</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>001 of 75</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>24.99 USD</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/188682528328?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2BLMWfl1HqImc9MgCC81YJ8LCLYbXmN2%2F2q8GHiMYE2SLrh7%2BkmQcmP1RWBM8x8IEmU3%2F9jPj6ZBbN7IXhj2cPK4dl%2FnBxN%2FanDJRTP9T4nxBEOPhX%2Br0ACHEvzVYs4ycZxSH6%2FOzM9SYFiW8or1xlHk95QI0sQ0ukNx2EXibXY%2FR432l2X5XzeHZ7iGnWXl%2FQ%3D</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 01:12 UTC</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/MJwAAeSwzIxqYTwU/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22T21:56:36.000Z</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QXYAAeSwYaxqYTwe/s-l1600.jpg | https://i.ebayimg.com/images/g/6~kAAeSwydZqYTwC/s-l1600.jpg | https://i.ebayimg.com/images/g/80wAAeSw6PpqYTwH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr"/>
+      <c r="P56" s="2" t="inlineStr"/>
+      <c r="Q56" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Tracy Austin</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Autograph Card Tracy Austin 50/50 Bookend</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>61.06 USD</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407064568256</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 01:12 UTC</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/kDIAAeSwINxqUa2d/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11T02:44:24.000Z</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/6cwAAeSwogFqUa2d/s-l1600.jpg | https://i.ebayimg.com/images/g/pU4AAeSwafFqUa2c/s-l1600.jpg | https://i.ebayimg.com/images/g/kMEAAeSw24RqUa2c/s-l1600.jpg | https://i.ebayimg.com/images/g/lrsAAeSwWEBqUa2d/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O57" s="2" t="inlineStr"/>
+      <c r="P57" s="2" t="inlineStr"/>
+      <c r="Q57" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R57" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -4763,6 +5167,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-17 05:34 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R57"/>
+  <dimension ref="A1:S57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -555,6 +555,11 @@
       <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Caution</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Sport</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scan results, 2026-09-17 11:24 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S57"/>
+  <dimension ref="A1:S62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5118,6 +5118,439 @@
         </is>
       </c>
       <c r="R57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Denis Shapovalov</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Sapphire</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS SAPPHIRE DENIS SHAPOVALOV ORANGE REFRACTOR 01/25</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>11.99 USD</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178200164707</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/UbsAAeSwePZqJR3D/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-07T07:30:46.000Z</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YGwAAeSwr3JqJR3C/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P58" s="2" t="inlineStr"/>
+      <c r="Q58" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R58" s="2" t="inlineStr"/>
+      <c r="S58" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Denis Shapovalov</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Tennis DENIS SHAPOVALOV Relic Patch Pink Refractor #15/15</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>last of 15 (15/15)</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>35.71 USD</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/135541582489?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2FOxjE3swvSnr6x%2BcUdBCa%2F2aFvF%2BGhwkvnKFh2U%2FSyiSXIKOOrR0DYP%2BIUCXkwjvqkZvWCuFruqdtzzO%2BwmkpNz8ZaAVz22eGZqEDdd%2BaWSLpn%2BUIWrLYKG65UutJi4CfqB6cXAFRX%2BWvy2U6Vc2i1hDQkEHe%2FIeh1k2lGZ1EyA9pmsNU0vK6toXIvCyvV98E%3D</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 11:24 UTC</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/WUAAAOSwILJnp8wI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>2025-02-08T21:28:01.000Z</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JEEAAOSwB45np8wI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P59" s="2" t="inlineStr"/>
+      <c r="Q59" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R59" s="2" t="inlineStr"/>
+      <c r="S59" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Denis Shapovalov</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty ---DENIS SHAPOVOLOV---SUPERIOR SIGNATURES----25/25</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>33.99 USD</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/277226055395?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8sii8dZ2NTWKWr3udTqAN0%2Bj%2BQgPtw35kQOZ6BTMOl6gpOCiE2M9U9HRB94mBNhMZabeOAbBLvl5dwkX8Nj4Em%2FK6l4VX%2FCb%2FjyYeslKxmUPCWTeE28PBHDsB5mdSqPL8e1CpVR4gOfjgg19wfisw33W1MMyJAmQO82ARxLGIaEV17nc8zXty%2F9dC%2B5G7qQco%3D</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 11:24 UTC</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8qoAAOSwlNloVqys/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>2025-06-21T13:00:09.000Z</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/A0IAAOSwvUdoQe1I/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O60" s="2" t="inlineStr"/>
+      <c r="P60" s="2" t="inlineStr"/>
+      <c r="Q60" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R60" s="2" t="inlineStr"/>
+      <c r="S60" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Denis Shapovalov</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty --DENIS SHAPOVALOV--REGALIA RELICS-10/10</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>49.99 USD</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/286633957331?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8oA8FEjurqn1Qc5IKB50nNeGGzg3%2B0Kb%2BwVk7kLfryhPaqTqAWqfoLGP7CrrCkRMXq0L4kK9xi8vwDEnXkgXupwrboTKixPEwwXShZFcrScTQLTaBlZ7vimckVsKMU8ecDWZ4VgsaUdn%2BpN6RCWS0Vek5BDS%2BFu5qCX0CKs30ELvbV%2FOXEWt5CsA7PBLkMNyI%3D</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 11:24 UTC</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QBUAAOSwJTBoRagX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>2025-06-08T15:12:12.000Z</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/D9UAAOSw3LloOzw8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O61" s="2" t="inlineStr"/>
+      <c r="P61" s="2" t="inlineStr"/>
+      <c r="Q61" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R61" s="2" t="inlineStr"/>
+      <c r="S61" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Denis Shapovalov</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Royalty UFC Benoit Saint Denis Blue Patch Logo /25 #SR-BS 1/25 🔥</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>24.99 USD</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/198140975712?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2BP1qpLPrPnGBOMNtL%2FDg2zr4aSgHJlBXlxW%2F7XSFeql6TqEVIT9YpxCnBWU3V8qHgbqSjZpkr%2BLaX9GHEwFNY8hOKJXk44drx3%2B4gf43bQ2%2BwBgeeCGNndY0Hxv25cnDtQEGuhPQU89KnhaOPPillFWBJU6N5pffqG1s9Bs9eJS%2BrIXGO%2BdmPerj5iAYC%2Bbto%3D</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 11:24 UTC</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/t7cAAeSwWZ5poS7I/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-27T05:46:46.000Z</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/rwkAAeSwKOBpoS7I/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O62" s="2" t="inlineStr"/>
+      <c r="P62" s="2" t="inlineStr"/>
+      <c r="Q62" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R62" s="2" t="inlineStr"/>
+      <c r="S62" s="2" t="inlineStr">
+        <is>
+          <t>Mixed Martial Arts (MMA)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -5177,6 +5610,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="rId61"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-17 11:29 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S62"/>
+  <dimension ref="A1:S74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5549,6 +5549,1062 @@
       <c r="S62" s="2" t="inlineStr">
         <is>
           <t>Mixed Martial Arts (MMA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Coco Gauff Gold Refractor Auto 01/50 Autograph BOOKEND</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>250.00 USD</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377443211029</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 11:28 UTC</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/l1kAAeSw2rZqi9VM/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24T05:24:56.000Z</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-x8AAeSwvr5qi9Ri/s-l1600.jpg | https://i.ebayimg.com/images/g/kggAAeSwrd5qi9R3/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P63" s="2" t="inlineStr"/>
+      <c r="Q63" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R63" s="2" t="inlineStr"/>
+      <c r="S63" s="2" t="inlineStr">
+        <is>
+          <t>Tennis, Tennis (网球)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Tennis #100 Coco Gauff Superfractor RC Rookie 1/1</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>99999.99 USD</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/158216025928</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 11:28 UTC</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RSkAAeSw0FZqiw8m/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23T15:23:29.000Z</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/MXgAAeSw2G9qiw8m/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O64" s="2" t="inlineStr"/>
+      <c r="P64" s="2" t="inlineStr"/>
+      <c r="Q64" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R64" s="2" t="inlineStr"/>
+      <c r="S64" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Coco Gauff Youthquake YQE-1 Black Refractor 1/2</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>001 of 2</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>1200.00 USD</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/267632338165?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde94QILwgsF6b5MhL%2B6dajJOGYehvdzGKBXN0uoQyk73TANbJhj2waxYZyWnqZxvuDh424AKGMBiAaJuHWaEycomDDunUTxjB4UBA%2FtxS74ePOm%2B3pGJD6%2BOSvbQFZYdgqZ5W1lm%2Fw27wOJqy%2FzxPVAUZ9KM6Nu%2FVLZ8U52TSnuTdj%2FbYu%2BIJj6BK3%2FDnxCZGLk%3D</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 11:28 UTC</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DXEAAeSwdX9p1VLx/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07T18:58:01.000Z</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N65" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vj4AAeSwMmVp1VLy/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P65" s="2" t="inlineStr"/>
+      <c r="Q65" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R65" s="2" t="inlineStr"/>
+      <c r="S65" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Youthquake Orange Refractor #YQE-1 Coco Gauff 01/25</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>59.99 USD</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147232002947</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 11:28 UTC</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/VNIAAeSwJdRpyvQd/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-30T22:22:52.000Z</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/hv0AAeSwXXlpyvQc/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O66" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P66" s="2" t="inlineStr"/>
+      <c r="Q66" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R66" s="2" t="inlineStr"/>
+      <c r="S66" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff Venus Williams 2025 Topps Chrome Tennis DUAL REFRACTOR 25/25 Auto /25</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>799.99 USD</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/188058829439</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 11:28 UTC</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/IWEAAeSwPo5pkHp4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-14T13:38:32.000Z</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RA8AAeSw2zhpkHp~/s-l1600.jpg | https://i.ebayimg.com/images/g/hywAAeSwGf9pkHqO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O67" s="2" t="inlineStr"/>
+      <c r="P67" s="2" t="inlineStr"/>
+      <c r="Q67" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R67" s="2" t="inlineStr"/>
+      <c r="S67" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Topps Chrome Graphite Tennis Signatures Coco Gauff White Refractor Auto 10/10</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>2600.00 USD</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/277175218300</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 11:28 UTC</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/BswAAeSweIdoQiho/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>2025-06-05T23:27:30.000Z</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/z0EAAeSwro9oQiUs/s-l1600.jpg | https://i.ebayimg.com/images/g/e8QAAeSwM8doQiUt/s-l1600.jpg | https://i.ebayimg.com/images/g/Pn4AAeSw9A1oQiUt/s-l1600.jpg | https://i.ebayimg.com/images/g/TMAAAeSwcD9oQiUt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P68" s="2" t="inlineStr"/>
+      <c r="Q68" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R68" s="2" t="inlineStr"/>
+      <c r="S68" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2021  Coco Gauff Topps Chrome Tennis Sapphire Orange  25/25 #100 </t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>1600.00 USD</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/356548731666</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 11:28 UTC</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/qAMAAeSwKzlnp-k7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>2025-02-08T23:34:41.000Z</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/zDgAAeSw~bJnp-k7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O69" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P69" s="2" t="inlineStr"/>
+      <c r="Q69" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R69" s="2" t="inlineStr"/>
+      <c r="S69" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff Signed 2021 Topps Chrome Purple Wave Rookie Auto /199 Psa MINT 9/9 RC</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>9/9</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>last of 9 (9/9)</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>1499.99 USD</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/266799599958?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8YR%2FnUfBNeNkdszwCfTj64SNTp9EoY4AM%2FzoA4kBMt1Hq9czt%2BwnKgJ%2FkszqYiCiZMWN1I2qTQhUcjRvhBCAyyuzuTUbUf9Q4mupjnR2wUkkUmWi8IgBZ5FZ2zaw1GZED%2BRnpboKxUeZzD3pTE3Z0dsnMYDczA%2FPXHBrP3kZcu72nP9fNPRLMZMxH2IX5TSb0%3D</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 11:28 UTC</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/x~IAAOSw06hmOpSj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>2024-05-06T22:40:45.000Z</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bjoAAOSwXTVmOVxg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P70" s="2" t="inlineStr"/>
+      <c r="Q70" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R70" s="2" t="inlineStr"/>
+      <c r="S70" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff Signed 2021 Topps Chrome #100 Refractor Rookie Card Auto Psa MINT 9/9</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>9/9</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>last of 9 (9/9)</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>1124.99 USD</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/266799597038?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde9sMGRiJGpr3ZAjlEoSi1hG8AUE3DuCjia1ISOrkWvXPdvkOyILCsYBVMJGv23%2B7DvtXSfbXI5Ku0oTmwLbABA0wKmzrezbusyaRdBWCITYJ9rydT%2FvGlIN1%2BLU%2BvC2OzwXQ8S70A5t0auwVvvR%2BDIVS4fADkkizCbasyH%2FMqclgRPDECzVYVZE5moDbU35I7w%3D</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 11:28 UTC</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/qx8AAOSwg75mOpTJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>2024-05-06T22:37:52.000Z</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ONYAAOSwCz5mOVu5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O71" s="2" t="inlineStr">
+        <is>
+          <t>mint</t>
+        </is>
+      </c>
+      <c r="P71" s="2" t="inlineStr"/>
+      <c r="Q71" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R71" s="2" t="inlineStr"/>
+      <c r="S71" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff Signed 2021 Topps Chrome #100 Refractor Rookie Card Auto Psa MINT 9/9</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>9/9</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>last of 9 (9/9)</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>1124.99 USD</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/266799595640?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2BeBrdIt0aIvy3Sc8%2Bxgr40dYAc10duX51R1XvbGUvyW%2Fml9iRMvYxOblHqE8%2BJ8UTaLaXWncbKVl6q80i4zCSHsy5ePNK4UTZZeeC6u7ygfk6o6H5baVsE8kQRA15vrnD5k9CBG5gp%2BPAZZK0hrc%2F5Ee9xrW4tfGQJyyo17DnpLSTw9SJLC1hzUN%2F%2BmWy4Hq4%3D</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 11:28 UTC</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Xq4AAOSwIzJmOpTx/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>2024-05-06T22:37:05.000Z</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/oVYAAOSwG1dmOVt-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O72" s="2" t="inlineStr">
+        <is>
+          <t>mint</t>
+        </is>
+      </c>
+      <c r="P72" s="2" t="inlineStr"/>
+      <c r="Q72" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R72" s="2" t="inlineStr"/>
+      <c r="S72" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - [Base] - Blue</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Blue 1/25 Coco Gauff #50 9et</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>114.68 USD</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237030956019</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 11:29 UTC</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gzMAAeSwnsNqjrN9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26T09:32:52.000Z</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9FgAAeSw5RdqjrN9/s-l1600.jpg | https://i.ebayimg.com/images/g/exQAAeSw7F9qjrN9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O73" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P73" s="2" t="inlineStr"/>
+      <c r="Q73" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R73" s="2" t="inlineStr"/>
+      <c r="S73" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty-Prodigious Pair Coco Gauff,Jessica Pegula #PSP-PG Gold 10/10</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>160.00 USD</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237022302018</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 11:29 UTC</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/EMwAAeSwiRFqN0B4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22T00:26:40.000Z</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="inlineStr"/>
+      <c r="O74" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P74" s="2" t="inlineStr"/>
+      <c r="Q74" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R74" s="2" t="inlineStr"/>
+      <c r="S74" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
         </is>
       </c>
     </row>
@@ -5615,6 +6671,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId73"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-17 11:58 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S74"/>
+  <dimension ref="A1:S75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6603,6 +6603,91 @@
       </c>
       <c r="R74" s="2" t="inlineStr"/>
       <c r="S74" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Denis Shapovalov</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis Denis Shapovalov 1st Pineapple Refractor 77/77 ≈1/1</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>77/77</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>last of 77 (77/77)</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/188938764146</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 11:58 UTC</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DtEAAeSwn35qqro2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T03:57:07.000Z</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N75" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/FBMAAeSw69Rqqro6/s-l1600.jpg | https://i.ebayimg.com/images/g/fA0AAeSwE4dqqro9/s-l1600.jpg | https://i.ebayimg.com/images/g/0LcAAeSwkOJqqrpE/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O75" s="2" t="inlineStr"/>
+      <c r="P75" s="2" t="inlineStr"/>
+      <c r="Q75" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R75" s="2" t="inlineStr"/>
+      <c r="S75" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -6683,6 +6768,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId74"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-17 13:10 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S75"/>
+  <dimension ref="A1:S76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6688,6 +6688,91 @@
       </c>
       <c r="R75" s="2" t="inlineStr"/>
       <c r="S75" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Joao Fonseca, João Fonseca</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>NetPro / 2026 NETPRO Premium Rainbow</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Joao Fonseca 2026 Netpro Premium Rainbow Auto RC 150/150 4A-JF SEALED 🎾</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>150/150</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>last of 150 (150/150)</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>845.00 USD</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298654435050?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde9uwKcpWabAdrqtHAKmd%2BSn0xOHN8DYpVq3v8TY%2FiHcGdXih3K23EZPG45oPRcVQbu4GaM60MXBGzOEtf7BBVFsV0UIvLELip9xmZkS%2FLue8VtEx%2B9z3GENMtGWm8g40Bq7zYpCUYVGP1GRT91gt2N4gJq0wSeDkQHW%2BGcAbxLC%2B5%2BHMTaJ4j2A3CalJnX29oM%3D</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:10 UTC</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/p~QAAeSwezBqnz-I/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07T22:50:40.000Z</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ckcAAeSwehhqnz-I/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O76" s="2" t="inlineStr"/>
+      <c r="P76" s="2" t="inlineStr"/>
+      <c r="Q76" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R76" s="2" t="inlineStr"/>
+      <c r="S76" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -6769,6 +6854,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId75"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-17 14:13 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S76"/>
+  <dimension ref="A1:S83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6773,6 +6773,617 @@
       </c>
       <c r="R76" s="2" t="inlineStr"/>
       <c r="S76" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>NetPro / NetPro Premium Autograph</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>🌈2022 NetPro Premium Autograph Carlos Alcaraz Rainbow Auto/250 Rare 10/10 SPAU2</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>25000.00 USD</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/204611174369</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 14:12 UTC</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/D5UAAOSwfrllndK3/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>2024-01-09T23:18:58.000Z</t>
+        </is>
+      </c>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L77" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>Rare Edition (Rare) 10</t>
+        </is>
+      </c>
+      <c r="N77" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/s0MAAOSwKRplndIY/s-l1600.jpg | https://i.ebayimg.com/images/g/YPoAAOSw3hFlndIa/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O77" s="2" t="inlineStr"/>
+      <c r="P77" s="2" t="inlineStr"/>
+      <c r="Q77" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R77" s="2" t="inlineStr"/>
+      <c r="S77" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Carlos Alcaraz Aqua Refractor #1 /199</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>1/199</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>001 of 199</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>25.00 USD</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/206510108410</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 14:13 UTC</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Bz4AAeSwjhxqie7T/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22T18:48:54.000Z</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DIQAAeSwKVhqie7V/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O78" s="2" t="inlineStr">
+        <is>
+          <t>aqua</t>
+        </is>
+      </c>
+      <c r="P78" s="2" t="inlineStr"/>
+      <c r="Q78" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R78" s="2" t="inlineStr"/>
+      <c r="S78" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome - Youthquake Carlos Alcaraz #YQE-6 Gold Refractor 50/50</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>500.00 USD</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/318627785306</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 14:13 UTC</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/lMUAAeSwPGtqYuEs/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24T03:51:34.000Z</t>
+        </is>
+      </c>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L79" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N79" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/h0IAAeSw46tqYuEe/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O79" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P79" s="2" t="inlineStr"/>
+      <c r="Q79" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R79" s="2" t="inlineStr"/>
+      <c r="S79" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz Auto 10/10 9.5 POP 1 Youthquake Black – 2025 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>7087.29 USD</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168414452573</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 14:13 UTC</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/cpYAAeSwZYRqGlXp/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30T03:14:55.000Z</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="inlineStr"/>
+      <c r="O80" s="2" t="inlineStr"/>
+      <c r="P80" s="2" t="inlineStr"/>
+      <c r="Q80" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R80" s="2" t="inlineStr"/>
+      <c r="S80" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite Tennis</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Carlos Alcaraz Break Point Red Crystalline 1/1 BP-15</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>13999.00 USD</t>
+        </is>
+      </c>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366653109547</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 14:13 UTC</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RFIAAeSw9kBqneRD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06T22:23:00.000Z</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L81" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N81" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/J1IAAeSwMfVqneRL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O81" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P81" s="2" t="inlineStr"/>
+      <c r="Q81" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R81" s="2" t="inlineStr"/>
+      <c r="S81" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Carlos Alcaraz Full Extension White Refractor # 1/10 🔥🔥🔥</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>357.44 USD</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/206509227424</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 14:13 UTC</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/CCkAAeSwXSZqiL27/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T21:07:24.000Z</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N82" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SpIAAeSwW8NqiL3E/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O82" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P82" s="2" t="inlineStr"/>
+      <c r="Q82" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R82" s="2" t="inlineStr"/>
+      <c r="S82" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Now</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Now Tennis Carlos Alcaraz #8-AR Match-Used Ball Auto Red 1/5</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>20000.00 USD</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237069905130?amdata=enc%3AAQALAAAAsCHNgUiiE%2FjQhlDTaMiAde8Q7HXRlPe%2BChK9gnHUbxVkI7XK1iuHCg4%2Bd1%2Bja9Uwhms9FAe5YzbtuduIB1T9s%2BZC%2Fhksh1OJJlUvQl%2BZ2ToUadQXelRkyQyxR1WKujNC%2BwdOLBLH4EAs%2F2vbRAtNqvagKuqmArUQ4Z%2B4%2FW3987rotZJZsevbgb7MuygJzW2zvI1xgSLZcdqru949E493gYhxH2gOtqqrNu7oOesX%2BeTV</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 14:13 UTC</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/pgIAAeSwaENqqaTo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15T20:05:10.000Z</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L83" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M83" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N83" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/cuUAAeSwCxdqqaTo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O83" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P83" s="2" t="inlineStr"/>
+      <c r="Q83" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R83" s="2" t="inlineStr"/>
+      <c r="S83" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -6855,6 +7466,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId82"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-17 15:04 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S83"/>
+  <dimension ref="A1:S91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7384,6 +7384,706 @@
       </c>
       <c r="R83" s="2" t="inlineStr"/>
       <c r="S83" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Shelton</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2025 Topps Chrome ATP Tour Ben Shelton #36 Serial Numbered 01/50</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>295.00 USD</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/318880590549</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:03 UTC</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/B1QAAeSwDZhqqz4P/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T01:11:55.000Z</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N84" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YiMAAeSwollqqz36/s-l1600.jpg | https://i.ebayimg.com/images/g/HBYAAeSwYHhqqz36/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O84" s="2" t="inlineStr"/>
+      <c r="P84" s="2" t="inlineStr"/>
+      <c r="Q84" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R84" s="2" t="inlineStr"/>
+      <c r="S84" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Shelton</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis Ben Shelton RC Court Masters Graphite 1/1 ONE OF ONE</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>9999.00 USD</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407214284726</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:03 UTC</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/k2YAAeSwIWdqpvxh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13T19:42:17.000Z</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L85" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N85" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/5vEAAeSw-hBqpnzq/s-l1600.jpg | https://i.ebayimg.com/images/g/~qcAAeSwx6lqpnzr/s-l1600.jpg | https://i.ebayimg.com/images/g/0zAAAeSwwlhqpvxd/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O85" s="2" t="inlineStr"/>
+      <c r="P85" s="2" t="inlineStr"/>
+      <c r="Q85" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R85" s="2" t="inlineStr"/>
+      <c r="S85" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Shelton</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS CHROME TENNIS TIAFOE/SHELTON DUAL AUTO BLACK REFRACTOR #1/10 PSA 8</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>2999.99 USD</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/800643584364</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:03 UTC</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/CmEAAeSwXTlqo1jV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11T01:30:43.000Z</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L86" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA)</t>
+        </is>
+      </c>
+      <c r="N86" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/EZsAAeSwD19qo1jV/s-l1600.jpg | https://i.ebayimg.com/images/g/3aYAAeSw9ltqo1jV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O86" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P86" s="2" t="inlineStr"/>
+      <c r="Q86" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R86" s="2" t="inlineStr"/>
+      <c r="S86" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Shelton</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024 TOPPS CHROME TENNIS ACES AUTO RED REFRACTOR BEN SHELTON RC 1 /5 PSA 10 </t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>12500.00 USD</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117404967062?amdata=enc%3AAQALAAAAsCHNgUiiE%2FjQhlDTaMiAde99UqkxkGbTsX05VZrCxXwCbsxJg9FcrhxBnJQw6mH42EBqHqWupfQbVOMnW7zOxZurArq2nKzyifOrTXOtMpVPV5oWg1Pe79EsMOpbc17ivlyCWbOzUoRJ5NKZXzQIf%2FxETPVj6MqFdanAiw1OmIsgMClT9y9m2cAZtTScYct0Fn5qnKL2ARjF2qhyyr8aYf54gmG3tBbQ8d9%2BPMhJwFie</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:03 UTC</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gfcAAeSwflRqcTtv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09T23:28:32.000Z</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L87" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t>PSA 10</t>
+        </is>
+      </c>
+      <c r="N87" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HF4AAeSwuchqcTt2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O87" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P87" s="2" t="inlineStr"/>
+      <c r="Q87" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R87" s="2" t="inlineStr"/>
+      <c r="S87" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Shelton</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Relics Pink Refractor 15/15 Ben Shelton Rookie RC 0r9h</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>last of 15 (15/15)</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>225.05 USD</t>
+        </is>
+      </c>
+      <c r="G88" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257728758107</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:04 UTC</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/I8AAAeSww-FqnkLY/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07T04:49:31.000Z</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/oW8AAeSw0yNqnkLY/s-l1600.jpg | https://i.ebayimg.com/images/g/wiYAAeSw5bdqnkLY/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P88" s="2" t="inlineStr"/>
+      <c r="Q88" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R88" s="2" t="inlineStr"/>
+      <c r="S88" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Shelton</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Tennis Royalty Ben Shelton Rookie Relic Auto Gold 01/10 RRA-BS#HT</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>41.00 USD</t>
+        </is>
+      </c>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/198647084332</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:04 UTC</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3-AAAeSwE6lqq1Q5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T02:48:00.000Z</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/NfgAAeSwamhqq1Q5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O89" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P89" s="2" t="inlineStr"/>
+      <c r="Q89" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R89" s="2" t="inlineStr"/>
+      <c r="S89" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Shelton</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Tennis</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty BEN SHELTON Triumph Relic Signatures GREEN 5/5 ROOKIE Auto RC</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>2500.00 USD</t>
+        </is>
+      </c>
+      <c r="G90" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147563407578</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:04 UTC</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0IUAAeSwXfNqoiMU/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10T03:27:45.000Z</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/I7EAAeSwZs9qoiMV/s-l1600.jpg | https://i.ebayimg.com/images/g/sQIAAeSwyXhqoiMV/s-l1600.jpg | https://i.ebayimg.com/images/g/~gAAAeSwWEVqoiMU/s-l1600.jpg | https://i.ebayimg.com/images/g/zIkAAeSw14xqoiMX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P90" s="2" t="inlineStr"/>
+      <c r="Q90" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R90" s="2" t="inlineStr"/>
+      <c r="S90" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Shelton</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS ROYALTY TENNIS--FRITZ SHELTON TIAFOE PAUL-QUAD AUTO BOOKLET--1/1</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>15000.00 USD</t>
+        </is>
+      </c>
+      <c r="G91" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/277447598584?amdata=enc%3AAQALAAAAsCHNgUiiE%2FjQhlDTaMiAde%2FRlu6G1EySDKZCjuSVrpuOWkHdQEY3EYkaxntLxj60p7BaeY3OjARKLz2sXoCwXDAmcbJG%2BUMLsGUQzyQHG%2FDm%2FdzFCE65qzQgGSKKEd4VS7nv7%2Fyh3oxCCmLhasrczCPtktVYSE3hsZTHApg0tpWNtDooW4Ltiu3%2BnoQZn0LrWxQJhoyWoAzYOrCAd3PbEgDJKvHl%2FKwLjcubEMEh%2F5H1</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:04 UTC</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/e0IAAeSwZSxpXXFO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>2025-10-16T19:44:13.000Z</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L91" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/OFkAAOSwJUdoQed6/s-l1600.jpg | https://i.ebayimg.com/images/g/ydYAAOSwqQxoQedv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O91" s="2" t="inlineStr"/>
+      <c r="P91" s="2" t="inlineStr"/>
+      <c r="Q91" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R91" s="2" t="inlineStr"/>
+      <c r="S91" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -7473,6 +8173,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId90"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-18 02:09 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S91"/>
+  <dimension ref="A1:S103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8084,6 +8084,1058 @@
       </c>
       <c r="R91" s="2" t="inlineStr"/>
       <c r="S91" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Karolina Muchova</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - [Base] - Pink Geometric Refractor</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Pink Geometric Refractor 65/65 Karolina Muchova #39 1mw3</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>65/65</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>last of 65 (65/65)</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>15.19 USD</t>
+        </is>
+      </c>
+      <c r="G92" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336798860440</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 02:08 UTC</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Ei8AAeSwPOlqrIAg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T00:03:39.000Z</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L92" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/NyEAAeSwM0NqrIAg/s-l1600.jpg | https://i.ebayimg.com/images/g/ENAAAeSwVyhqrIAh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P92" s="2" t="inlineStr"/>
+      <c r="Q92" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R92" s="2" t="inlineStr"/>
+      <c r="S92" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Zverev</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Alexander Zverev Purple Geometric #’d 10 /10 Champ</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>219.99 USD</t>
+        </is>
+      </c>
+      <c r="G93" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/327362700127?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde9FRFXq%2FWG6bTVUb6zW2v%2F0o%2B9tfDXh%2FVafzr2aVDzBPU6Vu%2FPksvjnki15oyDHAtUApywAJox6231IIT0yL8Xk4KlexxqB1NUqFOY0DLo032LuRc%2BAAQCOmidbLPbjxyRk2sRqeevNHZ8qpGtRognx7EbU7RI%2BW9O%2Fd6lFnbhgcwh5mL3dUaWC448KiQ%2FW%2BC8%3D</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 02:08 UTC</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ANcAAeSwKJBqrGQK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T22:06:56.000Z</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L93" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M93" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N93" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/AeMAAeSw2DJqrGQK/s-l1600.jpg | https://i.ebayimg.com/images/g/1BwAAeSwx9pqrGQK/s-l1600.jpg | https://i.ebayimg.com/images/g/CZoAAeSwHYBqrGQJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O93" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P93" s="2" t="inlineStr"/>
+      <c r="Q93" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R93" s="2" t="inlineStr"/>
+      <c r="S93" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Andrea Pellegrino</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome - Andrea Pellegrino #32 Rookie Superfractor 1/1 (RC) PSA 9</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>1000.00 USD</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237074315189</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 02:08 UTC</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/L~MAAeSw-0FqrFD4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T20:44:52.000Z</t>
+        </is>
+      </c>
+      <c r="K94" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L94" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA)</t>
+        </is>
+      </c>
+      <c r="N94" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/P-oAAeSw0l5qrFD5/s-l1600.jpg | https://i.ebayimg.com/images/g/PlYAAeSw53JqrFD5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O94" s="2" t="inlineStr"/>
+      <c r="P94" s="2" t="inlineStr"/>
+      <c r="Q94" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R94" s="2" t="inlineStr"/>
+      <c r="S94" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Dominik Koepfer</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Dominik Koepfer 🇩🇪 RC | #01/77 Pineapple Refractor -- 2024 Topps Chrome 🎾 #94</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>1/77</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>001 of 77</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>7.95 USD</t>
+        </is>
+      </c>
+      <c r="G95" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178505705020?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2FUENRVsHATAW89pBoWf7UENfm9%2FtfXZQnUKWvX9MHIrOJ1bZWMvRkJxVeQc0eWkENVhNd%2BafH5z%2BL7kkyF2vU4FcLPiA3kPnojtBTvrUeoj%2BgRgeaObJGpybCxLBP2XKx5GibFPMu7UabaoqCB0xlTpNL1cYtT%2FKYnA%2FL8VxnzUEwkbxRlEe9vUguPMPcW1X4%3D</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 02:08 UTC</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gGEAAeSwFXdqrD~q/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T19:31:01.000Z</t>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L95" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M95" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N95" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ysQAAeSwBDhqrD~q/s-l1600.jpg | https://i.ebayimg.com/images/g/NUUAAeSw-TFqrD~q/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O95" s="2" t="inlineStr"/>
+      <c r="P95" s="2" t="inlineStr"/>
+      <c r="Q95" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R95" s="2" t="inlineStr"/>
+      <c r="S95" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Petra Kvitova</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Blue Refractor 250/250 Petra Kvitova #113 Rookie RC 1yj</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>250/250</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>last of 250 (250/250)</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>16.93 USD</t>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336798182101</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 02:08 UTC</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XrAAAeSwf8Fqq~Da/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T13:52:27.000Z</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N96" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/b8UAAeSwMXRqq~Db/s-l1600.jpg | https://i.ebayimg.com/images/g/5tcAAeSwBDhqq~Db/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O96" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P96" s="2" t="inlineStr"/>
+      <c r="Q96" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R96" s="2" t="inlineStr"/>
+      <c r="S96" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Karen Khachanov</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>2025 KAREN KHACHANOV 01/25 AUTO TOPPS CHROME GEOMETRIC AUTOGRAPHS</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>69.99 USD</t>
+        </is>
+      </c>
+      <c r="G97" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/158301159295</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 02:08 UTC</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/dv8AAeSw~H9qqMBr/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T08:27:01.000Z</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L97" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N97" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/MiEAAeSwZXtqqMBr/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O97" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P97" s="2" t="inlineStr"/>
+      <c r="Q97" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R97" s="2" t="inlineStr"/>
+      <c r="S97" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Andy Roddick</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Andy Roddick Gold Pineapple Refractor 1/77 Rare SP USA</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>1/77</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>001 of 77</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>49.99 USD</t>
+        </is>
+      </c>
+      <c r="G98" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147578992992?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde9sWzeJrcBfbBhS1feG0bd5ZC3NTiC0Hyc889IfHKy7HS88EkIsQGUvUSfsG4TE6gincF4PTlm0N7k9MUWQxAQiKozw7OUIdv5hyY1vfolbqr9AMHXQ73JTliPZArQqZ8utBYah15lkQr4a4mmSO5amdsXe2DFkR%2Fd1kRzFHhgEmPQ1tqMnp%2FrrKVNbkdHU6Ek%3D</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 02:09 UTC</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/qzMAAeSwJVJqq3Ta/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T05:06:13.000Z</t>
+        </is>
+      </c>
+      <c r="K98" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L98" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N98" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/WygAAeSwkFdqq3Ta/s-l1600.jpg | https://i.ebayimg.com/images/g/HGEAAeSw4lxqq3Ta/s-l1600.jpg | https://i.ebayimg.com/images/g/bVUAAeSwKexqq3TZ/s-l1600.jpg | https://i.ebayimg.com/images/g/Wj4AAeSwBKJqq3Ta/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O98" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P98" s="2" t="inlineStr"/>
+      <c r="Q98" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R98" s="2" t="inlineStr"/>
+      <c r="S98" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>Miomir Kecmanovic</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis Miomir Kecmanovic Gold Sapphire 01/50 1st on Print</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>2.99 USD</t>
+        </is>
+      </c>
+      <c r="G99" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147577440759</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 02:09 UTC</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KtgAAeSwkOJqqGz~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T02:48:01.000Z</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L99" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M99" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N99" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/S6AAAeSwFNNqqG0a/s-l1600.jpg | https://i.ebayimg.com/images/g/iJ0AAeSwTctqqG0n/s-l1600.jpg | https://i.ebayimg.com/images/g/fc8AAeSweQVqqG04/s-l1600.jpg | https://i.ebayimg.com/images/g/UboAAeSwKcBqqG0w/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O99" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P99" s="2" t="inlineStr"/>
+      <c r="Q99" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R99" s="2" t="inlineStr"/>
+      <c r="S99" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Omar Jasika</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS RED REFRACTOR OMAR JASIKA RC 1ST #1/5</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G100" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/318880235681</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 02:09 UTC</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/zDMAAeSwp-ZqqyFp/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T02:11:01.000Z</t>
+        </is>
+      </c>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L100" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M100" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N100" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/xUUAAeSwKYJqqyFv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O100" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P100" s="2" t="inlineStr"/>
+      <c r="Q100" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R100" s="2" t="inlineStr"/>
+      <c r="S100" s="2" t="inlineStr">
+        <is>
+          <t>Auto Racing, Baseball, Basketball, Soccer, Tennis, Volleyball, Wrestling</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr"/>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS PURPLE GEOMETRIC CAPTURED MARTA KOSTYUK #10/10</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>8.50 USD</t>
+        </is>
+      </c>
+      <c r="G101" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/318880211543</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 02:09 UTC</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8FIAAeSwnyhqqyDc/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T02:09:01.000Z</t>
+        </is>
+      </c>
+      <c r="K101" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L101" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N101" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8bgAAeSw25dqqyDi/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O101" s="2" t="inlineStr"/>
+      <c r="P101" s="2" t="inlineStr"/>
+      <c r="Q101" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R101" s="2" t="inlineStr"/>
+      <c r="S101" s="2" t="inlineStr">
+        <is>
+          <t>Auto Racing, Baseball, Basketball, Soccer, Tennis, Volleyball, Wrestling</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>VERONIKA KUDERMETOVA</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS CHROME SAPPHIRE TENNIS</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS CHROME SAPPHIRE TENNIS RED #6 VERONIKA KUDERMETOVA 5/5 PSA 9</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>50.00 USD</t>
+        </is>
+      </c>
+      <c r="G102" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307183077996</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 02:09 UTC</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2zMAAeSwfBJqqzss/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T00:57:08.000Z</t>
+        </is>
+      </c>
+      <c r="K102" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L102" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M102" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N102" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XaMAAeSwfmBqqzss/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O102" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P102" s="2" t="inlineStr"/>
+      <c r="Q102" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R102" s="2" t="inlineStr"/>
+      <c r="S102" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>ZOE KRUGER</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS CHROME TENNIS AUTOGRAPHS</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS CHROME TENNIS AUTOS BLACK REFRACTOR ZOE KRUGER 10/10 PSA 8 AUTO 10</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>75.00 USD</t>
+        </is>
+      </c>
+      <c r="G103" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117416198794</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 02:09 UTC</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/6zMAAeSwGb1qqzr~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T00:56:12.000Z</t>
+        </is>
+      </c>
+      <c r="K103" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L103" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 8</t>
+        </is>
+      </c>
+      <c r="N103" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/BNoAAeSwaw5qqzr~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O103" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P103" s="2" t="inlineStr"/>
+      <c r="Q103" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R103" s="2" t="inlineStr"/>
+      <c r="S103" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -8181,6 +9233,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G103" r:id="rId102"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-18 02:44 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S103"/>
+  <dimension ref="A1:S104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -9136,6 +9136,99 @@
       </c>
       <c r="R103" s="2" t="inlineStr"/>
       <c r="S103" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Roger Federer</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>2008 Ace G/S II US Open Mem Dual Mat Gold #15 1/5 Federer/Berankis PSA 8 Top Pop</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>600.00 USD</t>
+        </is>
+      </c>
+      <c r="G104" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168659428125</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 02:43 UTC</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ceAAAOSwm0liwM3K/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03T00:43:30.000Z</t>
+        </is>
+      </c>
+      <c r="K104" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L104" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M104" s="2" t="inlineStr">
+        <is>
+          <t>PSA 8</t>
+        </is>
+      </c>
+      <c r="N104" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Oy4AAOSwn29iwM3T/s-l1600.jpg | https://i.ebayimg.com/images/g/9JYAAOSw4ApiwM3e/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O104" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P104" s="2" t="inlineStr"/>
+      <c r="Q104" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R104" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic: check the numbering is stamped, not on a circle sticker</t>
+        </is>
+      </c>
+      <c r="S104" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -9245,6 +9338,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G101" r:id="rId100"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G102" r:id="rId101"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G104" r:id="rId103"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-18 03:41 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S104"/>
+  <dimension ref="A1:S115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -9229,6 +9229,977 @@
         </is>
       </c>
       <c r="S104" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Roger Federer</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic / 2005 Ace Authentic Signature Series</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>2005 Ace Authentic Signature Series - Court Kings Roger Federer #CK-1 /500</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>1/500</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>001 of 500</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>49.99 USD</t>
+        </is>
+      </c>
+      <c r="G105" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178156772910?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2FiDBrSVLk64sPTGci1A8L%2FT%2BjAwx%2FMLvJorBCOYmG14KmRGr%2B0XSJAg1Kbdbi6xoyatl%2FMaojk18G%2FMcxlfI6XrYQKKrdJlQ8S3C00ip7PxlVZLDelz4P0QzPjsq%2Bju%2BQsuhfb4jeCOCkGJDhicdZcL84tAl6NSgcGqddw0HjqgbiEJyaP5XT%2F5TjQP8uyRDk%3D</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 03:40 UTC</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nAAAAeSwEPFqEL0j/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-22T20:32:46.000Z</t>
+        </is>
+      </c>
+      <c r="K105" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L105" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M105" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N105" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jjUAAeSwa5xqEL0k/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O105" s="2" t="inlineStr"/>
+      <c r="P105" s="2" t="inlineStr"/>
+      <c r="Q105" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R105" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic autograph: on-card or sticker not stated; check by eye</t>
+        </is>
+      </c>
+      <c r="S105" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Roger Federer</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic / 2008 Ace Authentic</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>2008 Ace Authentic Novak Djokovic &amp; Roger Federer Press Plate 1/1</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>1999.99 USD</t>
+        </is>
+      </c>
+      <c r="G106" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/126120695424</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 03:40 UTC</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SGMAAOSw~jplG2M0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J106" s="2" t="inlineStr">
+        <is>
+          <t>2023-10-03T00:46:55.000Z</t>
+        </is>
+      </c>
+      <c r="K106" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L106" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M106" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N106" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/s2QAAOSwCBNlG2NG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O106" s="2" t="inlineStr"/>
+      <c r="P106" s="2" t="inlineStr"/>
+      <c r="Q106" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R106" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic: check the numbering is stamped, not on a circle sticker</t>
+        </is>
+      </c>
+      <c r="S106" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome #200 Coco Gauff Green Refractor # 1/99</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>1/99</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>001 of 99</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>18.80 USD</t>
+        </is>
+      </c>
+      <c r="G107" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/158167082429</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 03:40 UTC</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ejQAAeSwNtZqd0aC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:01:37.000Z</t>
+        </is>
+      </c>
+      <c r="K107" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L107" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M107" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N107" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XEQAAeSwlShqd0aC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O107" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P107" s="2" t="inlineStr"/>
+      <c r="Q107" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R107" s="2" t="inlineStr"/>
+      <c r="S107" s="2" t="inlineStr">
+        <is>
+          <t>TENNIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Coco Gauff Purple Geometric Refractor # /10 🔥🔥🔥 1/1 on eBay</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>285.00 USD</t>
+        </is>
+      </c>
+      <c r="G108" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336726755483</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 03:40 UTC</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ukkAAeSwwapqG0Wg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T02:52:47.000Z</t>
+        </is>
+      </c>
+      <c r="K108" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L108" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N108" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Ra0AAeSwZwhqG0Wg/s-l1600.jpg | https://i.ebayimg.com/images/g/W3UAAeSw~hNqG0Wh/s-l1600.jpg | https://i.ebayimg.com/images/g/VCgAAeSwhZtqG0Wi/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O108" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P108" s="2" t="inlineStr"/>
+      <c r="Q108" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R108" s="2" t="inlineStr"/>
+      <c r="S108" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025 Topps Chrome Tennis Coco Gauff Red Geometric Refractor Auto 1/5 </t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>699.95 USD</t>
+        </is>
+      </c>
+      <c r="G109" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168150284709</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 03:40 UTC</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/z0cAAeSwMdJpi648/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-10T22:22:41.000Z</t>
+        </is>
+      </c>
+      <c r="K109" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L109" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M109" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N109" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/raYAAeSwgeJpi648/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O109" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P109" s="2" t="inlineStr"/>
+      <c r="Q109" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R109" s="2" t="inlineStr"/>
+      <c r="S109" s="2" t="inlineStr">
+        <is>
+          <t>Baseball, Basketball, Football, Mixed Martial Arts (MMA), Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite Tennis</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Tennis Pink Refractor Coco Gauff #21 01/15</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>89.99 USD</t>
+        </is>
+      </c>
+      <c r="G110" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287580989073</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 03:41 UTC</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YxsAAeSw-OhqpH4-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11T22:17:35.000Z</t>
+        </is>
+      </c>
+      <c r="K110" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L110" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N110" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9IoAAeSw-M1qpH4-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O110" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P110" s="2" t="inlineStr"/>
+      <c r="Q110" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R110" s="2" t="inlineStr"/>
+      <c r="S110" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite Tennis</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff-2026 Topps Graphite Tour Relic Auto Gold SSP #01/25-Game Used🔥🔥</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>299.00 USD</t>
+        </is>
+      </c>
+      <c r="G111" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/158297227522</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 03:41 UTC</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Gx0AAeSwhthqnQDm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16T06:00:14.000Z</t>
+        </is>
+      </c>
+      <c r="K111" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L111" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M111" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N111" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/q-sAAeSwG9FqnQDm/s-l1600.jpg | https://i.ebayimg.com/images/g/ZsgAAeSwhFRqnQDm/s-l1600.jpg | https://i.ebayimg.com/images/g/q7gAAeSwmElqnQDm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O111" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P111" s="2" t="inlineStr"/>
+      <c r="Q111" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R111" s="2" t="inlineStr"/>
+      <c r="S111" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Coco Gauff Full Extension White Refractor /10 🔥 1/1 on eBay</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>315.00 USD</t>
+        </is>
+      </c>
+      <c r="G112" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336726755481</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 03:41 UTC</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/M9IAAeSwgglqJ1aX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T02:52:47.000Z</t>
+        </is>
+      </c>
+      <c r="K112" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L112" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M112" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N112" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-pwAAeSwtvZqJ1aY/s-l1600.jpg | https://i.ebayimg.com/images/g/78wAAeSw~JxqJ1aZ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O112" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P112" s="2" t="inlineStr"/>
+      <c r="Q112" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R112" s="2" t="inlineStr"/>
+      <c r="S112" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Tennis Coco Gauff Blue Rally Relic 50/50</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>125.00 USD</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178084450257</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 03:41 UTC</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/VKkAAeSwpzNp79xo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J113" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-27T22:01:18.000Z</t>
+        </is>
+      </c>
+      <c r="K113" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L113" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M113" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N113" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/l9cAAeSwWi9p79xo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O113" s="2" t="inlineStr"/>
+      <c r="P113" s="2" t="inlineStr"/>
+      <c r="Q113" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R113" s="2" t="inlineStr"/>
+      <c r="S113" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Coco Gauff Superior Relic Signatures 1/5 PSA 10 Auto 10 NH44</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>50000.00 USD</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407206150641</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 03:41 UTC</t>
+        </is>
+      </c>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/99oAAeSwtfhqolW1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10T07:00:03.000Z</t>
+        </is>
+      </c>
+      <c r="K114" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L114" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M114" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 10.0</t>
+        </is>
+      </c>
+      <c r="N114" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/oEwAAeSwDudqolW2/s-l1600.jpg | https://i.ebayimg.com/images/g/eLYAAeSwks5qolW0/s-l1600.jpg | https://i.ebayimg.com/images/g/eWsAAeSwFu5qolW0/s-l1600.jpg | https://i.ebayimg.com/images/g/hCcAAeSwGtFqolW0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O114" s="2" t="inlineStr"/>
+      <c r="P114" s="2" t="inlineStr"/>
+      <c r="Q114" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R114" s="2" t="inlineStr"/>
+      <c r="S114" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Now</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Now Tennis Carlos Alcaraz #5 Red Foil /5 PSA 9 1/5</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>399.99 USD</t>
+        </is>
+      </c>
+      <c r="G115" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/327362616691</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 03:41 UTC</t>
+        </is>
+      </c>
+      <c r="I115" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/a5cAAeSwWP1qrEyF/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J115" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T20:25:44.000Z</t>
+        </is>
+      </c>
+      <c r="K115" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L115" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M115" s="2" t="inlineStr">
+        <is>
+          <t>PSA 9</t>
+        </is>
+      </c>
+      <c r="N115" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7FgAAeSwSmdqrEx0/s-l1600.jpg | https://i.ebayimg.com/images/g/ttMAAeSwKfZqrExt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O115" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P115" s="2" t="inlineStr"/>
+      <c r="Q115" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R115" s="2" t="inlineStr"/>
+      <c r="S115" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -9339,6 +10310,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G102" r:id="rId101"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G103" r:id="rId102"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G115" r:id="rId114"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-18 10:40 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S183"/>
+  <dimension ref="A1:S185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -16184,6 +16184,176 @@
         </is>
       </c>
       <c r="S183" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>YUE YUAN</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS CHROME TENNIS SUPERFRACTOR 1/1 #7 YUE YUAN 1/1 PSA 10</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>999.99 USD</t>
+        </is>
+      </c>
+      <c r="G184" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298685251941</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:40 UTC</t>
+        </is>
+      </c>
+      <c r="I184" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0~oAAeSwSmdqrQmx/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J184" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T09:49:09.000Z</t>
+        </is>
+      </c>
+      <c r="K184" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L184" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M184" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 10</t>
+        </is>
+      </c>
+      <c r="N184" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ovkAAeSwnJNqrQmx/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O184" s="2" t="inlineStr"/>
+      <c r="P184" s="2" t="inlineStr"/>
+      <c r="Q184" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R184" s="2" t="inlineStr"/>
+      <c r="S184" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>UGO HUMBERT</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS CHROME TENNIS SUPERFRACTOR 1/1 #101 UGO HUMBERT 1/1 PSA 9</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="inlineStr">
+        <is>
+          <t>899.99 USD</t>
+        </is>
+      </c>
+      <c r="G185" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117418478439</t>
+        </is>
+      </c>
+      <c r="H185" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:40 UTC</t>
+        </is>
+      </c>
+      <c r="I185" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SusAAeSw96JqrQma/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J185" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T09:48:19.000Z</t>
+        </is>
+      </c>
+      <c r="K185" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L185" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M185" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N185" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/L6YAAeSwfuZqrQma/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O185" s="2" t="inlineStr"/>
+      <c r="P185" s="2" t="inlineStr"/>
+      <c r="Q185" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R185" s="2" t="inlineStr"/>
+      <c r="S185" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -16373,6 +16543,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G181" r:id="rId180"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G182" r:id="rId181"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G183" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G184" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G185" r:id="rId184"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-18 11:23 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S185"/>
+  <dimension ref="A1:S187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -16354,6 +16354,184 @@
       </c>
       <c r="R185" s="2" t="inlineStr"/>
       <c r="S185" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>Chris Eubanks</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - [Base] - Orange Refractor</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Orange Refractor 1/25 Chris Eubanks #143 v3r</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>14.63 USD</t>
+        </is>
+      </c>
+      <c r="G186" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237075299501</t>
+        </is>
+      </c>
+      <c r="H186" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 11:23 UTC</t>
+        </is>
+      </c>
+      <c r="I186" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3SIAAeSwRrRqrRfI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J186" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T10:49:09.000Z</t>
+        </is>
+      </c>
+      <c r="K186" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L186" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M186" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N186" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ikwAAeSwMyBqrRfI/s-l1600.jpg | https://i.ebayimg.com/images/g/hywAAeSwD91qrRfJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O186" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P186" s="2" t="inlineStr"/>
+      <c r="Q186" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R186" s="2" t="inlineStr"/>
+      <c r="S186" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>Robin Montgomery</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - Autographs I - Blue Geometric Refractor</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome I Blue Geometric Refractor 150/150 Robin Montgomery Auto 14sd</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>150/150</t>
+        </is>
+      </c>
+      <c r="E187" s="2" t="inlineStr">
+        <is>
+          <t>last of 150 (150/150)</t>
+        </is>
+      </c>
+      <c r="F187" s="2" t="inlineStr">
+        <is>
+          <t>11.18 USD</t>
+        </is>
+      </c>
+      <c r="G187" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336799526603</t>
+        </is>
+      </c>
+      <c r="H187" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 11:23 UTC</t>
+        </is>
+      </c>
+      <c r="I187" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XQ8AAeSwi8lqrRVc/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J187" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T10:40:25.000Z</t>
+        </is>
+      </c>
+      <c r="K187" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L187" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M187" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N187" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/K2wAAeSweKZqrRVc/s-l1600.jpg | https://i.ebayimg.com/images/g/co4AAeSwXFlqrRVc/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O187" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P187" s="2" t="inlineStr"/>
+      <c r="Q187" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R187" s="2" t="inlineStr"/>
+      <c r="S187" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -16545,6 +16723,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G183" r:id="rId182"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G184" r:id="rId183"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G185" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G186" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G187" r:id="rId186"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-18 12:40 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S187"/>
+  <dimension ref="A1:S195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -16532,6 +16532,706 @@
       </c>
       <c r="R187" s="2" t="inlineStr"/>
       <c r="S187" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Zverev</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Sapphire Green /125 Alexander Zverev #74 125/125 BOOKEND</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>125/125</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>last of 125 (125/125)</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="inlineStr">
+        <is>
+          <t>40.00 USD</t>
+        </is>
+      </c>
+      <c r="G188" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168677731005</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 12:39 UTC</t>
+        </is>
+      </c>
+      <c r="I188" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ppQAAeSwAkNqok6i/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J188" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10T06:31:54.000Z</t>
+        </is>
+      </c>
+      <c r="K188" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L188" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M188" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N188" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/sb8AAeSwZU5qok6i/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O188" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P188" s="2" t="inlineStr"/>
+      <c r="Q188" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R188" s="2" t="inlineStr"/>
+      <c r="S188" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Zverev</t>
+        </is>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis Alexander Zverev Pineapple Refractor /77 BOOKEND 77/77</t>
+        </is>
+      </c>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>77/77</t>
+        </is>
+      </c>
+      <c r="E189" s="2" t="inlineStr">
+        <is>
+          <t>last of 77 (77/77)</t>
+        </is>
+      </c>
+      <c r="F189" s="2" t="inlineStr">
+        <is>
+          <t>75.00 USD</t>
+        </is>
+      </c>
+      <c r="G189" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168677713300</t>
+        </is>
+      </c>
+      <c r="H189" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 12:39 UTC</t>
+        </is>
+      </c>
+      <c r="I189" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/xc0AAeSwoL9qok0f/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J189" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10T06:25:12.000Z</t>
+        </is>
+      </c>
+      <c r="K189" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L189" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M189" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N189" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/qKEAAeSw0EJqok0f/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O189" s="2" t="inlineStr"/>
+      <c r="P189" s="2" t="inlineStr"/>
+      <c r="Q189" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R189" s="2" t="inlineStr"/>
+      <c r="S189" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Zverev</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Zverev #74 Topps Chrome 2024 Tennis SUPERFRACTOR 1/1 Gold CGC 9.5</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>9500.00 USD</t>
+        </is>
+      </c>
+      <c r="G190" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366655452344?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2BMhjLtG8u%2BD0tpGy%2F1JvlQbYAt28s9Dk1Hgli1KmaqeRHgisRydwWUPEMkbeiAycM8xDLTrPg%2FnJmXcETTGPOwKfpC9MRG9kbKWimaZzXWkZhf1nHtQdcfM1caLgpqoVEzONSMW59ObDVtGRj1UWcTlCm1Mp7ihm5aZa4Fj%2FYfNkYJwlnrkyHgvC3ERXUVrV4%3D</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 12:40 UTC</t>
+        </is>
+      </c>
+      <c r="I190" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/IT8AAeSweeRqKvru/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J190" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08T03:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="K190" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L190" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M190" s="2" t="inlineStr">
+        <is>
+          <t>CGC 9.5</t>
+        </is>
+      </c>
+      <c r="N190" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JyUAAeSwK3ZqKvru/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O190" s="2" t="inlineStr"/>
+      <c r="P190" s="2" t="inlineStr"/>
+      <c r="Q190" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R190" s="2" t="inlineStr"/>
+      <c r="S190" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Zverev</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite - Match Masters Alexander Zverev #MM-15 Red Crystalline 1/1</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E191" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F191" s="2" t="inlineStr">
+        <is>
+          <t>2200.00 USD</t>
+        </is>
+      </c>
+      <c r="G191" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/158039607844</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 12:40 UTC</t>
+        </is>
+      </c>
+      <c r="I191" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Y-MAAeSwznxqQvkQ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J191" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30T01:28:56.000Z</t>
+        </is>
+      </c>
+      <c r="K191" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L191" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M191" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N191" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RN8AAeSwa4hqQvkH/s-l1600.jpg | https://i.ebayimg.com/images/g/bbYAAeSwxARqQvkT/s-l1600.jpg | https://i.ebayimg.com/images/g/KzAAAeSw211qQvkV/s-l1600.jpg | https://i.ebayimg.com/images/g/SswAAeSwEZtqQvmL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O191" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P191" s="2" t="inlineStr"/>
+      <c r="Q191" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R191" s="2" t="inlineStr"/>
+      <c r="S191" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>Paula Badosa</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome #64 Paula Badosa Pineapple Refractor 77/77</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>77/77</t>
+        </is>
+      </c>
+      <c r="E192" s="2" t="inlineStr">
+        <is>
+          <t>last of 77 (77/77)</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="inlineStr">
+        <is>
+          <t>25.00 USD</t>
+        </is>
+      </c>
+      <c r="G192" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257725911186?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2B4ow0dblNEclOok%2FhURNAqcIVoRi3E%2FB11UYDWEQz46lGjAvnceee5D3wPqCRp2UvulMXN31aJG0ACyvR%2BuGRF0z9jZH%2FE8yUGDgqxSDqvdj6Z5HR92D0G9IzPPBszszF%2Bar%2Bxpk1M5qViA839ZQii0La0l9ws8oWgo2XzM1nzU6j30meAbeMSyQmjNasPu%2BA%3D</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 12:40 UTC</t>
+        </is>
+      </c>
+      <c r="I192" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Z4QAAeSwM89qnIKK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J192" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05T20:56:48.000Z</t>
+        </is>
+      </c>
+      <c r="K192" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L192" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M192" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N192" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JvUAAeSwGDJqnIKK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O192" s="2" t="inlineStr"/>
+      <c r="P192" s="2" t="inlineStr"/>
+      <c r="Q192" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R192" s="2" t="inlineStr"/>
+      <c r="S192" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>Paula Badosa</t>
+        </is>
+      </c>
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C193" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME SAPPHIRE PAULA BADOSA #21 PURPLE REFRACTOR @ 1/10 @</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E193" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F193" s="2" t="inlineStr">
+        <is>
+          <t>79.99 USD</t>
+        </is>
+      </c>
+      <c r="G193" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168630845092</t>
+        </is>
+      </c>
+      <c r="H193" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 12:40 UTC</t>
+        </is>
+      </c>
+      <c r="I193" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bGgAAeSw0FZqiGLS/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J193" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T14:40:03.000Z</t>
+        </is>
+      </c>
+      <c r="K193" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L193" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M193" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N193" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gxUAAeSwEphqiGLS/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O193" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P193" s="2" t="inlineStr"/>
+      <c r="Q193" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R193" s="2" t="inlineStr"/>
+      <c r="S193" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>Paula Badosa</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME SAPPHIRE PAULA BADOSA #21 RED REFRACTOR @ 5/5 @</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E194" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F194" s="2" t="inlineStr">
+        <is>
+          <t>109.99 USD</t>
+        </is>
+      </c>
+      <c r="G194" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147235993196</t>
+        </is>
+      </c>
+      <c r="H194" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 12:40 UTC</t>
+        </is>
+      </c>
+      <c r="I194" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/UWAAAeSw0SNpzZuz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J194" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01T22:29:50.000Z</t>
+        </is>
+      </c>
+      <c r="K194" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L194" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M194" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N194" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/dfQAAeSwNOtpzZuz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O194" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P194" s="2" t="inlineStr"/>
+      <c r="Q194" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R194" s="2" t="inlineStr"/>
+      <c r="S194" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>Paula Badosa</t>
+        </is>
+      </c>
+      <c r="B195" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C195" s="2" t="inlineStr">
+        <is>
+          <t>2026 TOPPS GRAPHITE PAULA BADOSA ALL-COURT #AC-11 GOLD REFRACTOR @ 25/25 @</t>
+        </is>
+      </c>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E195" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F195" s="2" t="inlineStr">
+        <is>
+          <t>31.99 USD</t>
+        </is>
+      </c>
+      <c r="G195" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147301743849</t>
+        </is>
+      </c>
+      <c r="H195" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 12:40 UTC</t>
+        </is>
+      </c>
+      <c r="I195" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/zz0AAeSwzp1p~l54/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J195" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T22:08:08.000Z</t>
+        </is>
+      </c>
+      <c r="K195" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L195" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M195" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N195" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XfwAAeSwu-dp~l54/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O195" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P195" s="2" t="inlineStr"/>
+      <c r="Q195" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R195" s="2" t="inlineStr"/>
+      <c r="S195" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -16725,6 +17425,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G185" r:id="rId184"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G186" r:id="rId185"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G187" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G188" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G189" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G190" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G191" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G192" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G193" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G194" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G195" r:id="rId194"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-18 12:53 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S195"/>
+  <dimension ref="A1:S200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -17232,6 +17232,439 @@
       </c>
       <c r="R195" s="2" t="inlineStr"/>
       <c r="S195" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Nadal</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>NetPro / 2003 NetPro</t>
+        </is>
+      </c>
+      <c r="C196" s="2" t="inlineStr">
+        <is>
+          <t>2003 NETPRO E27 R NADAL ROOKIE GEM MT 10 AUTO 10 1/2 of 8500+ PSA GRADED ROOKIES</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="E196" s="2" t="inlineStr">
+        <is>
+          <t>001 of 2</t>
+        </is>
+      </c>
+      <c r="F196" s="2" t="inlineStr">
+        <is>
+          <t>100000.00 USD</t>
+        </is>
+      </c>
+      <c r="G196" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/188692048417</t>
+        </is>
+      </c>
+      <c r="H196" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 12:53 UTC</t>
+        </is>
+      </c>
+      <c r="I196" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/UpQAAeSwpwZqY76u/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J196" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24T19:55:31.000Z</t>
+        </is>
+      </c>
+      <c r="K196" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L196" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M196" s="2" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="N196" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Wy0AAeSwoi5qY76u/s-l1600.jpg | https://i.ebayimg.com/images/g/MDgAAeSwAY9qaQtN/s-l1600.jpg | https://i.ebayimg.com/images/g/t1gAAeSwWXRqaQtN/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O196" s="2" t="inlineStr"/>
+      <c r="P196" s="2" t="inlineStr"/>
+      <c r="Q196" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R196" s="2" t="inlineStr"/>
+      <c r="S196" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Nadal</t>
+        </is>
+      </c>
+      <c r="B197" s="2" t="inlineStr">
+        <is>
+          <t>NetPro</t>
+        </is>
+      </c>
+      <c r="C197" s="2" t="inlineStr">
+        <is>
+          <t>2012 NETPRO 20th Anniv. Rafael Nadal Int’l Ser. BB 1/1 77  PSA GEM MT 10 COA</t>
+        </is>
+      </c>
+      <c r="D197" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E197" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F197" s="2" t="inlineStr">
+        <is>
+          <t>15000.00 USD</t>
+        </is>
+      </c>
+      <c r="G197" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/188691975041</t>
+        </is>
+      </c>
+      <c r="H197" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 12:53 UTC</t>
+        </is>
+      </c>
+      <c r="I197" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/y34AAeSwgUdqY7r8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J197" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24T19:31:20.000Z</t>
+        </is>
+      </c>
+      <c r="K197" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L197" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M197" s="2" t="inlineStr">
+        <is>
+          <t>PSA 10</t>
+        </is>
+      </c>
+      <c r="N197" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uGAAAeSwe41qY7r8/s-l1600.jpg | https://i.ebayimg.com/images/g/748AAeSw0XBqY7r7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O197" s="2" t="inlineStr"/>
+      <c r="P197" s="2" t="inlineStr"/>
+      <c r="Q197" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R197" s="2" t="inlineStr"/>
+      <c r="S197" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Nadal</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Rafael Nadal Break Point Gold /25 25/25 BP-13 BOOKEND</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E198" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="inlineStr">
+        <is>
+          <t>207.27 USD</t>
+        </is>
+      </c>
+      <c r="G198" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298621827561?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2F81ZVuY5QaxInMQDc0y2OA9%2BhpxiKLHs1VqRXAym%2BisczYhh6X3EcH3%2B5s3NIrDlY1mY0M1U05hYZqsDV%2FnGAtWMbzTJ9u%2BhrVhtWL%2FgufnNbq6fluHzS1%2B4lrdut67hFlKe%2Frc7uFpxxKco230fEi7GAbOWpwEMylgVaK0sEwCInBNUL3dYruaGrTyjy%2FSnQ%3D</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 12:53 UTC</t>
+        </is>
+      </c>
+      <c r="I198" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/GokAAeSwqlBqkJJQ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J198" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27T19:41:42.000Z</t>
+        </is>
+      </c>
+      <c r="K198" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L198" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M198" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N198" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/GeQAAeSw1nRqkJJQ/s-l1600.jpg | https://i.ebayimg.com/images/g/IjcAAeSw9fJqkJJQ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O198" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P198" s="2" t="inlineStr"/>
+      <c r="Q198" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R198" s="2" t="inlineStr"/>
+      <c r="S198" s="2" t="inlineStr">
+        <is>
+          <t>Breaking</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Nadal</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic / 2008 Ace Authentic US Open</t>
+        </is>
+      </c>
+      <c r="C199" s="2" t="inlineStr">
+        <is>
+          <t>2013 ACE RAFAEL NADAL TOP 40 #T40-RN1 AUTHENTIC AUTOGRAPH AUTO 15/15 @ SEE SCAN</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="E199" s="2" t="inlineStr">
+        <is>
+          <t>last of 15 (15/15)</t>
+        </is>
+      </c>
+      <c r="F199" s="2" t="inlineStr">
+        <is>
+          <t>649.99 USD</t>
+        </is>
+      </c>
+      <c r="G199" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147540872970</t>
+        </is>
+      </c>
+      <c r="H199" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 12:53 UTC</t>
+        </is>
+      </c>
+      <c r="I199" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/dskAAeSwc8Fqlg1x/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J199" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31T23:34:28.000Z</t>
+        </is>
+      </c>
+      <c r="K199" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L199" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M199" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N199" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/pzUAAeSwNoNqlg1x/s-l1600.jpg | https://i.ebayimg.com/images/g/knkAAeSwuTdqlg1x/s-l1600.jpg | https://i.ebayimg.com/images/g/H4wAAeSwjspqlg1w/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O199" s="2" t="inlineStr"/>
+      <c r="P199" s="2" t="inlineStr"/>
+      <c r="Q199" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R199" s="2" t="inlineStr"/>
+      <c r="S199" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Nadal</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic / 2013 Ace Authentic Grand Slam</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t>2013 Ace Authentic Rafael Nadal &amp; Tommy Robredo RARE Dual Autos Autographs 3/3</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t>last of 3 (3/3)</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="inlineStr">
+        <is>
+          <t>2999.99 USD</t>
+        </is>
+      </c>
+      <c r="G200" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/125964427297</t>
+        </is>
+      </c>
+      <c r="H200" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 12:53 UTC</t>
+        </is>
+      </c>
+      <c r="I200" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uO8AAOSwg3BkfgJm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J200" s="2" t="inlineStr">
+        <is>
+          <t>2023-06-05T15:48:43.000Z</t>
+        </is>
+      </c>
+      <c r="K200" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L200" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M200" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N200" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ArIAAOSwecVkfgLJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O200" s="2" t="inlineStr"/>
+      <c r="P200" s="2" t="inlineStr"/>
+      <c r="Q200" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R200" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic autograph: on-card or sticker not stated; check by eye</t>
+        </is>
+      </c>
+      <c r="S200" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -17433,6 +17866,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G193" r:id="rId192"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G194" r:id="rId193"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G195" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G196" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G197" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G198" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G199" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G200" r:id="rId199"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-18 14:49 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S200"/>
+  <dimension ref="A1:S202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -17665,6 +17665,184 @@
         </is>
       </c>
       <c r="S200" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>Aleksandar Kovacevic</t>
+        </is>
+      </c>
+      <c r="B201" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C201" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Black Refractor 1/10 Aleksandar Kovacevic #138 Rookie RC 1w0z</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E201" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F201" s="2" t="inlineStr">
+        <is>
+          <t>115.24 USD</t>
+        </is>
+      </c>
+      <c r="G201" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237075598518</t>
+        </is>
+      </c>
+      <c r="H201" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 14:49 UTC</t>
+        </is>
+      </c>
+      <c r="I201" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ij4AAeSwVyhqrUC4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J201" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T13:45:28.000Z</t>
+        </is>
+      </c>
+      <c r="K201" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L201" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M201" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N201" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/lf8AAeSwdo1qrUC4/s-l1600.jpg | https://i.ebayimg.com/images/g/rpYAAeSw7k9qrUC4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O201" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P201" s="2" t="inlineStr"/>
+      <c r="Q201" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R201" s="2" t="inlineStr"/>
+      <c r="S201" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>Tatjana Maria</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Red Refractor 1/5 Tatjana Maria #3 Rookie RC 1w0z</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>87.64 USD</t>
+        </is>
+      </c>
+      <c r="G202" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237075592239</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 14:49 UTC</t>
+        </is>
+      </c>
+      <c r="I202" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HagAAeSwf8pqrT-6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J202" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T13:41:15.000Z</t>
+        </is>
+      </c>
+      <c r="K202" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L202" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M202" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N202" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ss0AAeSw9TBqrT-7/s-l1600.jpg | https://i.ebayimg.com/images/g/tYYAAeSwVCxqrT-7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O202" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P202" s="2" t="inlineStr"/>
+      <c r="Q202" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R202" s="2" t="inlineStr"/>
+      <c r="S202" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -17871,6 +18049,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G198" r:id="rId197"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G199" r:id="rId198"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G200" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G201" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G202" r:id="rId201"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-19 08:42 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S202"/>
+  <dimension ref="A1:S254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -17843,6 +17843,4570 @@
       </c>
       <c r="R202" s="2" t="inlineStr"/>
       <c r="S202" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>Pete Sampras</t>
+        </is>
+      </c>
+      <c r="B203" s="2" t="inlineStr">
+        <is>
+          <t>NetPro</t>
+        </is>
+      </c>
+      <c r="C203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NETPRO 23K Gold Prototype Pete Sampras Autograph Printing Plate 1/1 PSA 9 </t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E203" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F203" s="2" t="inlineStr">
+        <is>
+          <t>1399.30 USD</t>
+        </is>
+      </c>
+      <c r="G203" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/254849378591</t>
+        </is>
+      </c>
+      <c r="H203" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:40 UTC</t>
+        </is>
+      </c>
+      <c r="I203" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Lf4AAeSw87xqan6B/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J203" s="2" t="inlineStr">
+        <is>
+          <t>2021-01-29T17:31:57.000Z</t>
+        </is>
+      </c>
+      <c r="K203" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L203" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M203" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports (PSA)</t>
+        </is>
+      </c>
+      <c r="N203" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gCsAAeSwK8xqY8SQ/s-l1600.jpg | https://i.ebayimg.com/images/g/MgwAAeSwEMdqZ~Zk/s-l1600.jpg | https://i.ebayimg.com/images/g/GV0AAeSwAVhqdL1w/s-l1600.jpg | https://i.ebayimg.com/images/g/54IAAeSw24RqY8Oc/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O203" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P203" s="2" t="inlineStr"/>
+      <c r="Q203" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R203" s="2" t="inlineStr"/>
+      <c r="S203" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>Pete Sampras</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t>2021 Chrome Rose Gold Refractor 1/10 Pete Sampras SGC 9.5 Mint+ Auto HOF ob9</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E204" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="inlineStr">
+        <is>
+          <t>527.20 USD</t>
+        </is>
+      </c>
+      <c r="G204" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336775514776</t>
+        </is>
+      </c>
+      <c r="H204" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:40 UTC</t>
+        </is>
+      </c>
+      <c r="I204" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/b40AAeSwMf5qmNnL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J204" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03T02:20:58.000Z</t>
+        </is>
+      </c>
+      <c r="K204" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L204" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M204" s="2" t="inlineStr">
+        <is>
+          <t>Sportscard (SGC) 9.5 Mint+</t>
+        </is>
+      </c>
+      <c r="N204" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/AjMAAeSweY5qmNnL/s-l1600.jpg | https://i.ebayimg.com/images/g/BXoAAeSw7BNqmNnL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O204" s="2" t="inlineStr">
+        <is>
+          <t>rose</t>
+        </is>
+      </c>
+      <c r="P204" s="2" t="inlineStr"/>
+      <c r="Q204" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R204" s="2" t="inlineStr"/>
+      <c r="S204" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>Pete Sampras</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C205" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis #180 PETE SAMPRAS - Purple Geometric Refractor #15/15</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="E205" s="2" t="inlineStr">
+        <is>
+          <t>last of 15 (15/15)</t>
+        </is>
+      </c>
+      <c r="F205" s="2" t="inlineStr">
+        <is>
+          <t>85.00 USD</t>
+        </is>
+      </c>
+      <c r="G205" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/267277573487</t>
+        </is>
+      </c>
+      <c r="H205" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:40 UTC</t>
+        </is>
+      </c>
+      <c r="I205" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/a~oAAeSwBQpoQTDP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J205" s="2" t="inlineStr">
+        <is>
+          <t>2025-06-05T05:56:40.000Z</t>
+        </is>
+      </c>
+      <c r="K205" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L205" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M205" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N205" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ZkIAAeSw3CRoQTDP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O205" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P205" s="2" t="inlineStr"/>
+      <c r="Q205" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R205" s="2" t="inlineStr">
+        <is>
+          <t>title says 15/15 but eBay's details say 64/499; check by eye</t>
+        </is>
+      </c>
+      <c r="S205" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>Pete Sampras</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C206" s="2" t="inlineStr">
+        <is>
+          <t>2024 Graphite Legends of the Court Pink Refractor 1/15 Pete Sampras PSA 9 4vc</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E206" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="inlineStr">
+        <is>
+          <t>69.24 USD</t>
+        </is>
+      </c>
+      <c r="G206" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257693845289</t>
+        </is>
+      </c>
+      <c r="H206" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:40 UTC</t>
+        </is>
+      </c>
+      <c r="I206" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/EBwAAeSwF5Bqh7Vd/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J206" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T02:15:01.000Z</t>
+        </is>
+      </c>
+      <c r="K206" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L206" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M206" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports (PSA) 9 MINT</t>
+        </is>
+      </c>
+      <c r="N206" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JawAAeSwXSZqh7Vc/s-l1600.jpg | https://i.ebayimg.com/images/g/KsIAAeSwi55qh7Ve/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O206" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P206" s="2" t="inlineStr"/>
+      <c r="Q206" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R206" s="2" t="inlineStr"/>
+      <c r="S206" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>Andre Agassi</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t>NetPro</t>
+        </is>
+      </c>
+      <c r="C207" s="2" t="inlineStr">
+        <is>
+          <t>2011 NetPro 20th Anniversary Elite Star Andre Agassi Timeless Treasure #d 1/1</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E207" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F207" s="2" t="inlineStr">
+        <is>
+          <t>17802.50 USD</t>
+        </is>
+      </c>
+      <c r="G207" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/397643821634</t>
+        </is>
+      </c>
+      <c r="H207" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:40 UTC</t>
+        </is>
+      </c>
+      <c r="I207" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KXEAAeSwbtJpnYOK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J207" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-24T10:59:14.000Z</t>
+        </is>
+      </c>
+      <c r="K207" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L207" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M207" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N207" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2mAAAeSwVXNpnYOR/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O207" s="2" t="inlineStr"/>
+      <c r="P207" s="2" t="inlineStr"/>
+      <c r="Q207" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R207" s="2" t="inlineStr"/>
+      <c r="S207" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>Andre Agassi</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>NetPro / 1991 NetPro Prototype</t>
+        </is>
+      </c>
+      <c r="C208" s="2" t="inlineStr">
+        <is>
+          <t>2012 NetPro 20th Anniversary Buyback 1991 Andre Agassi Prototype Rookie 1/20</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>1/20</t>
+        </is>
+      </c>
+      <c r="E208" s="2" t="inlineStr">
+        <is>
+          <t>001 of 20</t>
+        </is>
+      </c>
+      <c r="F208" s="2" t="inlineStr">
+        <is>
+          <t>900.00 USD</t>
+        </is>
+      </c>
+      <c r="G208" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/135094720072?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde9HGVJSFduJvsq0KcU0J6VpyVsw%2BC5R%2BkOvBhARHZbjsEJrYYQaGInLOSMFB5HSJeby398LnPF1iiCa%2FGWYtPdWkK5Y5lbIP6eEIKVlRlQPZ2Xlpihc98v%2FkKrZnDfo9fh1WZE4TOgveN3%2BiptCic5lshUXktIfLcUoDaKZ6b3KCAQnxB0qZupTyxaOA9HqwVo%3D</t>
+        </is>
+      </c>
+      <c r="H208" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:40 UTC</t>
+        </is>
+      </c>
+      <c r="I208" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9s4AAOSwTyJmY5Rg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J208" s="2" t="inlineStr">
+        <is>
+          <t>2024-06-08T00:08:01.000Z</t>
+        </is>
+      </c>
+      <c r="K208" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L208" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M208" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N208" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~Z8AAOSwPKVmY5Rf/s-l1600.jpg | https://i.ebayimg.com/images/g/KHMAAOSwr2NmY5Rg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O208" s="2" t="inlineStr"/>
+      <c r="P208" s="2" t="inlineStr"/>
+      <c r="Q208" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R208" s="2" t="inlineStr"/>
+      <c r="S208" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>Andre Agassi</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C209" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Andre Agassi Orange Geometric 1st Print 01/25 PSA 10</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E209" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F209" s="2" t="inlineStr">
+        <is>
+          <t>121.00 USD</t>
+        </is>
+      </c>
+      <c r="G209" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147566942712?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8W0U3Gww6trZO%2F4x0KXjU4S8v4lC1foh5NFTQJA%2FnsSCYlO%2BSmqpGTcvHfkkhxzmta4HlX0h%2FoxP2JoC%2F01yqKkx2eld4QYtJGJdMstJiWLQXSS0YPMexmGJ1DVPlTbo1njagOwGn%2BLyATufuaWQiel5pVCoCjcMxGC4m33BM8G4LurK3rMOWjIPScrwdIa%2Bo%3D</t>
+        </is>
+      </c>
+      <c r="H209" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:40 UTC</t>
+        </is>
+      </c>
+      <c r="I209" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/qAAAAeSwm3xqpHdU/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J209" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11T21:49:14.000Z</t>
+        </is>
+      </c>
+      <c r="K209" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L209" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M209" s="2" t="inlineStr">
+        <is>
+          <t>PSA 10</t>
+        </is>
+      </c>
+      <c r="N209" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/sh0AAeSwdo1qpHdU/s-l1600.jpg | https://i.ebayimg.com/images/g/ysMAAeSwK7pqpHdU/s-l1600.jpg | https://i.ebayimg.com/images/g/y6AAAeSw92pqpHdU/s-l1600.jpg | https://i.ebayimg.com/images/g/Ht4AAeSwdt5qpHdV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O209" s="2" t="inlineStr"/>
+      <c r="P209" s="2" t="inlineStr"/>
+      <c r="Q209" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R209" s="2" t="inlineStr"/>
+      <c r="S209" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>Andre Agassi</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite Tennis</t>
+        </is>
+      </c>
+      <c r="C210" s="2" t="inlineStr">
+        <is>
+          <t>2026 TOPPS GRAPHITE TENNIS GRAND SLAM AUTO ANDRE AGASSI RED CRYSTALLINE-#1/1!</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E210" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F210" s="2" t="inlineStr">
+        <is>
+          <t>1360.00 USD</t>
+        </is>
+      </c>
+      <c r="G210" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/398356646296</t>
+        </is>
+      </c>
+      <c r="H210" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:40 UTC</t>
+        </is>
+      </c>
+      <c r="I210" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/zBcAAeSwNEpqGOO~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J210" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04T00:39:30.000Z</t>
+        </is>
+      </c>
+      <c r="K210" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L210" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M210" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N210" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/H9IAAeSwgmRqGONt/s-l1600.jpg | https://i.ebayimg.com/images/g/DlsAAeSw8ANqGOSC/s-l1600.jpg | https://i.ebayimg.com/images/g/2FMAAeSwiFZqGOQx/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O210" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P210" s="2" t="inlineStr"/>
+      <c r="Q210" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R210" s="2" t="inlineStr"/>
+      <c r="S210" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>Andre Agassi</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite Tennis</t>
+        </is>
+      </c>
+      <c r="C211" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS GRAPHITE TENNIS ANDRE AGASSI WHITE REFRACTOR SSP #137 #01/10!</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E211" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F211" s="2" t="inlineStr">
+        <is>
+          <t>199.99 USD</t>
+        </is>
+      </c>
+      <c r="G211" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/256757781027?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2Fe5BpmhtbV2oZAa2699GcpVudhAem5PEvo%2FKgd--EScASO%2FaQFxznDi12VUHBx3W0SQqnLG5SK1kLhK1SdC%2FbY7UMsZ54KeJZUxZbVp9TjhunUvKWbq3DobiELeyf%2BNfJdZa35gDT0nlLlgjuk5Jqaeb4qI5OEh60RbufX55CorOv6P%2BCqLM1sAf%2BI2pD%2BsQU%3D</t>
+        </is>
+      </c>
+      <c r="H211" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:40 UTC</t>
+        </is>
+      </c>
+      <c r="I211" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gIwAAOSwJDpnZjvp/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J211" s="2" t="inlineStr">
+        <is>
+          <t>2024-12-21T03:55:00.000Z</t>
+        </is>
+      </c>
+      <c r="K211" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L211" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M211" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N211" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/o9gAAOSwWY5nZjvo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O211" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P211" s="2" t="inlineStr"/>
+      <c r="Q211" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R211" s="2" t="inlineStr"/>
+      <c r="S211" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>Andre Agassi</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Influential Ink - Green</t>
+        </is>
+      </c>
+      <c r="C212" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Influential Ink Green 5/5 Andre Agassi #I-AA Auto 9et</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E212" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F212" s="2" t="inlineStr">
+        <is>
+          <t>1350.00 USD</t>
+        </is>
+      </c>
+      <c r="G212" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237042638805</t>
+        </is>
+      </c>
+      <c r="H212" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:40 UTC</t>
+        </is>
+      </c>
+      <c r="I212" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/I4IAAeSwpfhqltMs/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J212" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01T13:27:10.000Z</t>
+        </is>
+      </c>
+      <c r="K212" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L212" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M212" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N212" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TCkAAeSwj8NqltMs/s-l1600.jpg | https://i.ebayimg.com/images/g/j-sAAeSw2G9qltMt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O212" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P212" s="2" t="inlineStr"/>
+      <c r="Q212" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R212" s="2" t="inlineStr"/>
+      <c r="S212" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>Andre Agassi</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty</t>
+        </is>
+      </c>
+      <c r="C213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024 Topps Royalty Andre Agassi Influential Ink Auto Platinum 1/1 One of One </t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E213" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F213" s="2" t="inlineStr">
+        <is>
+          <t>3999.99 USD</t>
+        </is>
+      </c>
+      <c r="G213" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/187606197450</t>
+        </is>
+      </c>
+      <c r="H213" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:40 UTC</t>
+        </is>
+      </c>
+      <c r="I213" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uMsAAeSwCr1o2cCp/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J213" s="2" t="inlineStr">
+        <is>
+          <t>2025-09-28T23:12:26.000Z</t>
+        </is>
+      </c>
+      <c r="K213" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L213" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M213" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N213" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/sLAAAeSwebRo2cCo/s-l1600.jpg | https://i.ebayimg.com/images/g/uo0AAeSwgSZo2cCo/s-l1600.jpg | https://i.ebayimg.com/images/g/KDkAAeSwfFdo2cCo/s-l1600.jpg | https://i.ebayimg.com/images/g/rMIAAeSwV8Jo2cCo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O213" s="2" t="inlineStr"/>
+      <c r="P213" s="2" t="inlineStr"/>
+      <c r="Q213" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R213" s="2" t="inlineStr"/>
+      <c r="S213" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>Andre Agassi</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic</t>
+        </is>
+      </c>
+      <c r="C214" s="2" t="inlineStr">
+        <is>
+          <t>andre agassi ace authentic 2006 gold 4x jersey and one  black press 1/1</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E214" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F214" s="2" t="inlineStr">
+        <is>
+          <t>142.99 USD</t>
+        </is>
+      </c>
+      <c r="G214" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/115296423737</t>
+        </is>
+      </c>
+      <c r="H214" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:40 UTC</t>
+        </is>
+      </c>
+      <c r="I214" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0dEAAOSwe2Nh9rKP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J214" s="2" t="inlineStr">
+        <is>
+          <t>2022-03-15T16:54:30.000Z</t>
+        </is>
+      </c>
+      <c r="K214" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L214" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M214" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N214" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/VCAAAOSwTgBh9rKW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O214" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P214" s="2" t="inlineStr"/>
+      <c r="Q214" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R214" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic: check the numbering is stamped, not on a circle sticker</t>
+        </is>
+      </c>
+      <c r="S214" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>Martina Hingis</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C215" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome II Red Refractor 5/5 Martina Hingis #TCA-MHS Auto HOF 5h0</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E215" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F215" s="2" t="inlineStr">
+        <is>
+          <t>340.27 USD</t>
+        </is>
+      </c>
+      <c r="G215" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237060852025</t>
+        </is>
+      </c>
+      <c r="H215" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:40 UTC</t>
+        </is>
+      </c>
+      <c r="I215" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8VYAAeSwcvZqonFw/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J215" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10T08:43:54.000Z</t>
+        </is>
+      </c>
+      <c r="K215" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L215" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M215" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N215" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~KcAAeSwPlhqonFw/s-l1600.jpg | https://i.ebayimg.com/images/g/GrAAAeSwGDRqonFw/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O215" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P215" s="2" t="inlineStr"/>
+      <c r="Q215" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R215" s="2" t="inlineStr"/>
+      <c r="S215" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>Martina Hingis</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C216" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome MARTINA HINGIS Aces Auto-Superfractor #1/1 PSA 10 [ONE OF ONE]</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E216" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F216" s="2" t="inlineStr">
+        <is>
+          <t>4500.00 USD</t>
+        </is>
+      </c>
+      <c r="G216" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366668908955</t>
+        </is>
+      </c>
+      <c r="H216" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:40 UTC</t>
+        </is>
+      </c>
+      <c r="I216" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RiIAAeSwQBhqa7MR/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J216" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14T17:57:31.000Z</t>
+        </is>
+      </c>
+      <c r="K216" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L216" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M216" s="2" t="inlineStr">
+        <is>
+          <t>PSA 10</t>
+        </is>
+      </c>
+      <c r="N216" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/M7EAAeSwfZRqa7MR/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O216" s="2" t="inlineStr"/>
+      <c r="P216" s="2" t="inlineStr"/>
+      <c r="Q216" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R216" s="2" t="inlineStr"/>
+      <c r="S216" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>Martina Hingis</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C217" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Tennis Martina Hingis Conchita Martinez 1/5 C3 Grading 9.5</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E217" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F217" s="2" t="inlineStr">
+        <is>
+          <t>70.00 USD</t>
+        </is>
+      </c>
+      <c r="G217" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/167336494998</t>
+        </is>
+      </c>
+      <c r="H217" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:40 UTC</t>
+        </is>
+      </c>
+      <c r="I217" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/MtcAAOSwJNRndaYR/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J217" s="2" t="inlineStr">
+        <is>
+          <t>2025-02-24T03:06:10.000Z</t>
+        </is>
+      </c>
+      <c r="K217" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L217" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M217" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N217" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-qsAAOSwd1FndaYR/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O217" s="2" t="inlineStr"/>
+      <c r="P217" s="2" t="inlineStr"/>
+      <c r="Q217" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R217" s="2" t="inlineStr"/>
+      <c r="S217" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>Martina Hingis</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024 Topps Chrome Sapphire Tennis #152 Martina Hingis Purple 10/10 🇸🇰 </t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E218" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F218" s="2" t="inlineStr">
+        <is>
+          <t>135.00 USD</t>
+        </is>
+      </c>
+      <c r="G218" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/186925357470</t>
+        </is>
+      </c>
+      <c r="H218" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:40 UTC</t>
+        </is>
+      </c>
+      <c r="I218" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XDEAAOSw5ztnn7wv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J218" s="2" t="inlineStr">
+        <is>
+          <t>2025-02-02T18:42:22.000Z</t>
+        </is>
+      </c>
+      <c r="K218" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L218" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M218" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N218" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KCQAAOSwYjdnn7wv/s-l1600.jpg | https://i.ebayimg.com/images/g/1J8AAOSwlq9nn7wv/s-l1600.jpg | https://i.ebayimg.com/images/g/KrcAAOSwUW1nn7wv/s-l1600.jpg | https://i.ebayimg.com/images/g/o3MAAOSwjX5nn7ww/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O218" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P218" s="2" t="inlineStr"/>
+      <c r="Q218" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R218" s="2" t="inlineStr"/>
+      <c r="S218" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>Martina Hingis</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps</t>
+        </is>
+      </c>
+      <c r="C219" s="2" t="inlineStr">
+        <is>
+          <t>MARTINA HINGIS 2024 Topps Royalty Tennis Platinum 1/1 1of1 #47 SWISS HOF</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E219" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F219" s="2" t="inlineStr">
+        <is>
+          <t>499.99 USD</t>
+        </is>
+      </c>
+      <c r="G219" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/146746688282</t>
+        </is>
+      </c>
+      <c r="H219" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:40 UTC</t>
+        </is>
+      </c>
+      <c r="I219" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/R7IAAeSwkSlojeC0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J219" s="2" t="inlineStr">
+        <is>
+          <t>2025-08-02T09:59:56.000Z</t>
+        </is>
+      </c>
+      <c r="K219" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L219" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M219" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N219" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/C3MAAeSwEZ9ojeC0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O219" s="2" t="inlineStr"/>
+      <c r="P219" s="2" t="inlineStr"/>
+      <c r="Q219" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R219" s="2" t="inlineStr"/>
+      <c r="S219" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek</t>
+        </is>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C220" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Pink Geometric Refractor Iga Swiatek #10 RC 65/65 Tennis</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>65/65</t>
+        </is>
+      </c>
+      <c r="E220" s="2" t="inlineStr">
+        <is>
+          <t>last of 65 (65/65)</t>
+        </is>
+      </c>
+      <c r="F220" s="2" t="inlineStr">
+        <is>
+          <t>54.99 USD</t>
+        </is>
+      </c>
+      <c r="G220" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168671483634</t>
+        </is>
+      </c>
+      <c r="H220" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I220" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/WoQAAeSwwGJqnvU7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J220" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07T17:33:47.000Z</t>
+        </is>
+      </c>
+      <c r="K220" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L220" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M220" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N220" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ycAAAeSwQxlqnvVC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O220" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P220" s="2" t="inlineStr"/>
+      <c r="Q220" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R220" s="2" t="inlineStr"/>
+      <c r="S220" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek</t>
+        </is>
+      </c>
+      <c r="B221" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C221" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Dual Autographs Aryna Sabalenka/Iga Swiatek #CDA-SS 01/25</t>
+        </is>
+      </c>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E221" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F221" s="2" t="inlineStr">
+        <is>
+          <t>995.00 USD</t>
+        </is>
+      </c>
+      <c r="G221" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/397679640077</t>
+        </is>
+      </c>
+      <c r="H221" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I221" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/hCAAAeSwnNBpqfDu/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J221" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-05T21:19:52.000Z</t>
+        </is>
+      </c>
+      <c r="K221" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L221" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M221" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N221" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/GnEAAeSwJllpqfDu/s-l1600.jpg | https://i.ebayimg.com/images/g/IUUAAeSwFAlpqfDu/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O221" s="2" t="inlineStr"/>
+      <c r="P221" s="2" t="inlineStr"/>
+      <c r="Q221" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R221" s="2" t="inlineStr"/>
+      <c r="S221" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Sapphire</t>
+        </is>
+      </c>
+      <c r="C222" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Sapphire Tennis Iga Swiatek Auto AIV-IGA Orange 1/25 Refractor</t>
+        </is>
+      </c>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E222" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F222" s="2" t="inlineStr">
+        <is>
+          <t>1499.00 USD</t>
+        </is>
+      </c>
+      <c r="G222" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/198023479827?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2BHCqHzLIqGs4iASSHigDhtq1n%2FAW0taXCa%2FKEcuJnLDK8jOQKxnYODhdnLbLVydewZ3BkZMow98ZN%2FCZqH0NIo1JOR4tq7hJFQ%2BY3GaD2PIePU5uVe7Vt2f5qG%2BZuOS8UBfMYXfmdkBWg8xy4y0iopDh1FAI067cTNRReoA1SJTlRVY%2BVIgpk4QdTsLRYFIDw%3D</t>
+        </is>
+      </c>
+      <c r="H222" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I222" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gs8AAeSw-1VpZWeO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J222" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-12T21:30:10.000Z</t>
+        </is>
+      </c>
+      <c r="K222" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L222" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M222" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N222" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/g0oAAeSwuVhqhGPy/s-l1600.jpg | https://i.ebayimg.com/images/g/EhAAAeSwiyppZWeO/s-l1600.jpg | https://i.ebayimg.com/images/g/i6EAAeSw0yNqhGPy/s-l1600.jpg | https://i.ebayimg.com/images/g/XgQAAeSwNXNqhGPy/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O222" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P222" s="2" t="inlineStr"/>
+      <c r="Q222" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R222" s="2" t="inlineStr"/>
+      <c r="S222" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek</t>
+        </is>
+      </c>
+      <c r="B223" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C223" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek / Aryna Sabalenka 2024 Topps Chrome Red Refractor Center Court 1/5</t>
+        </is>
+      </c>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E223" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F223" s="2" t="inlineStr">
+        <is>
+          <t>324.99 USD</t>
+        </is>
+      </c>
+      <c r="G223" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/286958955814</t>
+        </is>
+      </c>
+      <c r="H223" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I223" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/MOoAAeSwai1pILh5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J223" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-21T19:09:23.000Z</t>
+        </is>
+      </c>
+      <c r="K223" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L223" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M223" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N223" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/LicAAeSwHo5pILh4/s-l1600.jpg | https://i.ebayimg.com/images/g/7LsAAeSwiuZpILh4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O223" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P223" s="2" t="inlineStr"/>
+      <c r="Q223" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R223" s="2" t="inlineStr"/>
+      <c r="S223" s="2" t="inlineStr">
+        <is>
+          <t>TENNIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek</t>
+        </is>
+      </c>
+      <c r="B224" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS ROYALTY TENNIS SUPERIOR RELIC SIGNAT...</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS ROYALTY TENNIS SUPERIOR RELIC SIGNATURES BLUE IGA SWIATEK 25/25 PSA 8</t>
+        </is>
+      </c>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E224" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F224" s="2" t="inlineStr">
+        <is>
+          <t>3025.25 USD</t>
+        </is>
+      </c>
+      <c r="G224" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117371804478</t>
+        </is>
+      </c>
+      <c r="H224" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I224" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/t4oAAeSw7DBqiGyj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J224" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21T15:15:59.000Z</t>
+        </is>
+      </c>
+      <c r="K224" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L224" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M224" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 8</t>
+        </is>
+      </c>
+      <c r="N224" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2IMAAeSwu3ZqiGyj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O224" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P224" s="2" t="inlineStr"/>
+      <c r="Q224" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R224" s="2" t="inlineStr"/>
+      <c r="S224" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Tennis</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr">
+        <is>
+          <t>Aryna Sabalenka Iga Swiatek 2024 Topps Royalty PRODIGIOUS PAIRINGS Platinum 1/1</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E225" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F225" s="2" t="inlineStr">
+        <is>
+          <t>3499.99 USD</t>
+        </is>
+      </c>
+      <c r="G225" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/188726944839</t>
+        </is>
+      </c>
+      <c r="H225" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I225" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/mm4AAeSwan9qbe3T/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J225" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01T13:03:33.000Z</t>
+        </is>
+      </c>
+      <c r="K225" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L225" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M225" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N225" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uF8AAeSw6JVqbe3X/s-l1600.jpg | https://i.ebayimg.com/images/g/KGIAAeSwnN9qbe3k/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O225" s="2" t="inlineStr"/>
+      <c r="P225" s="2" t="inlineStr"/>
+      <c r="Q225" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R225" s="2" t="inlineStr"/>
+      <c r="S225" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS---MIRRA ANDREEVA---YOUTHQUAKE----GOLD GEOMETRIC---01/50</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E226" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F226" s="2" t="inlineStr">
+        <is>
+          <t>49.99 USD</t>
+        </is>
+      </c>
+      <c r="G226" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/278353484392?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8csM5NZJoHuHqKKR8Xsx4KonrPXEzUrMj%2BzeGk8XaqMx%2Fc0Cn848ehtfJmY41JTnYQOuM3n%2BPxWR0ipL6jyWn%2BNj95fq19lhGcywQM5oPByzdTZNYUNEaaq2U9CkBm7HQuzPnCOKZ9QtotScoRhd2ZcT%2FnYTwiVhvJLxbY2TX%2BEezrybdbBpJQOlH8k82p%2F5A%3D</t>
+        </is>
+      </c>
+      <c r="H226" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I226" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YCgAAeSw0EJqnycR/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J226" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07T21:07:46.000Z</t>
+        </is>
+      </c>
+      <c r="K226" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L226" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M226" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N226" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/avcAAeSwivNqnycb/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O226" s="2" t="inlineStr"/>
+      <c r="P226" s="2" t="inlineStr"/>
+      <c r="Q226" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R226" s="2" t="inlineStr"/>
+      <c r="S226" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B227" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C227" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Sapphire Green 125/125 Erika Andreeva #24 Rookie RC 1u4</t>
+        </is>
+      </c>
+      <c r="D227" s="2" t="inlineStr">
+        <is>
+          <t>125/125</t>
+        </is>
+      </c>
+      <c r="E227" s="2" t="inlineStr">
+        <is>
+          <t>last of 125 (125/125)</t>
+        </is>
+      </c>
+      <c r="F227" s="2" t="inlineStr">
+        <is>
+          <t>8.59 USD</t>
+        </is>
+      </c>
+      <c r="G227" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257722103278</t>
+        </is>
+      </c>
+      <c r="H227" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I227" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/VKQAAeSwXyxqmkJX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J227" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04T03:59:21.000Z</t>
+        </is>
+      </c>
+      <c r="K227" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L227" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M227" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N227" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/kAEAAeSw4C1qmkJX/s-l1600.jpg | https://i.ebayimg.com/images/g/ts8AAeSwhAZqmkJX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O227" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P227" s="2" t="inlineStr"/>
+      <c r="Q227" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R227" s="2" t="inlineStr"/>
+      <c r="S227" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B228" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C228" s="2" t="inlineStr">
+        <is>
+          <t>Erika Andreeva 2024 Topps Chrome Tennis Black Refractor 01/10 #24 RC Rookie</t>
+        </is>
+      </c>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E228" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F228" s="2" t="inlineStr">
+        <is>
+          <t>59.99 USD</t>
+        </is>
+      </c>
+      <c r="G228" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287534721376</t>
+        </is>
+      </c>
+      <c r="H228" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I228" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/J0sAAeSw0Hxqhepj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J228" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-19T17:40:46.000Z</t>
+        </is>
+      </c>
+      <c r="K228" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L228" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M228" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N228" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/EboAAeSwJFFqhepj/s-l1600.jpg | https://i.ebayimg.com/images/g/jsQAAeSwZPBqhepj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O228" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P228" s="2" t="inlineStr"/>
+      <c r="Q228" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R228" s="2" t="inlineStr"/>
+      <c r="S228" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B229" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva / Erika 2024 Topps Chrome Dual Auto (RC) Refractor 25/25 Bookend!</t>
+        </is>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E229" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F229" s="2" t="inlineStr">
+        <is>
+          <t>949.99 USD</t>
+        </is>
+      </c>
+      <c r="G229" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/800136075863?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2BGimm7Sf8a2NuUz7xp59nhreSITHcQAkXKPP%2BiDKG1x5WimOwX4LDQmya4paCCVPwS%2FWVBIAHazodIuNJVdQ9pQDq1tXGIacvOVn8hehnQqzS4gmEtpkFOD%2B2lrPHEIOXy7KSgwwDnBS2JjZHd%2BkYd5hc4TZXj5cPdd51F98axWgLmh20DFPHaTcJ16UpzNbU%3D</t>
+        </is>
+      </c>
+      <c r="H229" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I229" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Q0MAAeSwDUZqJQCc/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J229" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-07T05:35:23.000Z</t>
+        </is>
+      </c>
+      <c r="K229" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L229" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M229" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N229" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Tk8AAeSwj1xqJQCc/s-l1600.jpg | https://i.ebayimg.com/images/g/aGkAAeSw-JNqJQCc/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O229" s="2" t="inlineStr">
+        <is>
+          <t>silver</t>
+        </is>
+      </c>
+      <c r="P229" s="2" t="inlineStr"/>
+      <c r="Q229" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R229" s="2" t="inlineStr"/>
+      <c r="S229" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Mirra Andreeva BLACK GEOMETRIC #2/2 SSP</t>
+        </is>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="E230" s="2" t="inlineStr">
+        <is>
+          <t>last of 2 (2/2)</t>
+        </is>
+      </c>
+      <c r="F230" s="2" t="inlineStr">
+        <is>
+          <t>2999.99 USD</t>
+        </is>
+      </c>
+      <c r="G230" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/406691198895</t>
+        </is>
+      </c>
+      <c r="H230" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I230" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QVEAAeSwtchpjM1p/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J230" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11T18:43:13.000Z</t>
+        </is>
+      </c>
+      <c r="K230" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L230" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M230" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N230" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RcIAAeSwi5dpjM1d/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O230" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P230" s="2" t="inlineStr"/>
+      <c r="Q230" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R230" s="2" t="inlineStr"/>
+      <c r="S230" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B231" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C231" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis Rookie /5 Mirra Andreeva eBay 1/1</t>
+        </is>
+      </c>
+      <c r="D231" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E231" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F231" s="2" t="inlineStr">
+        <is>
+          <t>6000.00 USD</t>
+        </is>
+      </c>
+      <c r="G231" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/405742187819</t>
+        </is>
+      </c>
+      <c r="H231" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I231" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gS8AAOSwBBNn9ayz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J231" s="2" t="inlineStr">
+        <is>
+          <t>2025-04-08T23:12:15.000Z</t>
+        </is>
+      </c>
+      <c r="K231" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L231" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M231" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N231" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DAMAAOSwU3Zn9ay4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O231" s="2" t="inlineStr"/>
+      <c r="P231" s="2" t="inlineStr"/>
+      <c r="Q231" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R231" s="2" t="inlineStr"/>
+      <c r="S231" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B232" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis Erika Andreeva Red Sapphire Rookie 1/5 RC SSP #24</t>
+        </is>
+      </c>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E232" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F232" s="2" t="inlineStr">
+        <is>
+          <t>169.99 USD</t>
+        </is>
+      </c>
+      <c r="G232" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/286446987237</t>
+        </is>
+      </c>
+      <c r="H232" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I232" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/yx8AAeSw7Fpn6CHz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J232" s="2" t="inlineStr">
+        <is>
+          <t>2025-03-29T16:39:08.000Z</t>
+        </is>
+      </c>
+      <c r="K232" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L232" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M232" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N232" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/y0wAAeSwoa5n6CHz/s-l1600.jpg | https://i.ebayimg.com/images/g/~bIAAeSwm5Jn6CHz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O232" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P232" s="2" t="inlineStr"/>
+      <c r="Q232" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R232" s="2" t="inlineStr"/>
+      <c r="S232" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B233" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Sapphire</t>
+        </is>
+      </c>
+      <c r="C233" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Sapphire #81 Mirra Andreeva Orange Refractor 25/25 Bookend!</t>
+        </is>
+      </c>
+      <c r="D233" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E233" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F233" s="2" t="inlineStr">
+        <is>
+          <t>750.00 USD</t>
+        </is>
+      </c>
+      <c r="G233" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/800333607311</t>
+        </is>
+      </c>
+      <c r="H233" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I233" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/PJQAAOSwG71nBsze/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J233" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13T12:17:29.000Z</t>
+        </is>
+      </c>
+      <c r="K233" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L233" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M233" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N233" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0QsAAOSwVOJnBsrq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O233" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P233" s="2" t="inlineStr"/>
+      <c r="Q233" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R233" s="2" t="inlineStr"/>
+      <c r="S233" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B234" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C234" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Pink Refractor 1/15 Erika Andreeva #131 Rookie RC 0y61</t>
+        </is>
+      </c>
+      <c r="D234" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E234" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F234" s="2" t="inlineStr">
+        <is>
+          <t>20.38 USD</t>
+        </is>
+      </c>
+      <c r="G234" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336757581983</t>
+        </is>
+      </c>
+      <c r="H234" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I234" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/OGkAAeSwTclqi0FH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J234" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23T18:46:39.000Z</t>
+        </is>
+      </c>
+      <c r="K234" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L234" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M234" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N234" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-2IAAeSw3B1qi0FH/s-l1600.jpg | https://i.ebayimg.com/images/g/DIwAAeSwgwRqi0FH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O234" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P234" s="2" t="inlineStr"/>
+      <c r="Q234" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R234" s="2" t="inlineStr"/>
+      <c r="S234" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B235" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Graphite</t>
+        </is>
+      </c>
+      <c r="C235" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva 2024 Topps Graphite Signature Serves Blue 50/50 Rookie Auto RC</t>
+        </is>
+      </c>
+      <c r="D235" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E235" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F235" s="2" t="inlineStr">
+        <is>
+          <t>324.99 USD</t>
+        </is>
+      </c>
+      <c r="G235" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287399078950</t>
+        </is>
+      </c>
+      <c r="H235" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I235" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KL0AAeSw~4xqMYr7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J235" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16T17:43:34.000Z</t>
+        </is>
+      </c>
+      <c r="K235" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L235" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M235" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N235" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/p3MAAeSwFU1qMYr7/s-l1600.jpg | https://i.ebayimg.com/images/g/brgAAeSwZKtqMYr7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O235" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P235" s="2" t="inlineStr"/>
+      <c r="Q235" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R235" s="2" t="inlineStr"/>
+      <c r="S235" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B236" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 TOPPS GRAPHITE TENNIS</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="inlineStr">
+        <is>
+          <t>2026 TOPPS GRAPHITE TENNIS----MIRRA ANDREEVA---SIGNATURE SERIES--10/10</t>
+        </is>
+      </c>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E236" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F236" s="2" t="inlineStr">
+        <is>
+          <t>249.99 USD</t>
+        </is>
+      </c>
+      <c r="G236" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287327793721?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2B5smWSdVCbrFOILqjF5zjb8Q2aNbuk3KtpGNuwQZ%2FNbVoWDU5M9dL217ShUiq79%2BlSyrQag3FAupG%2BOsSpIP9AKbcYIrT3Ihqdwo%2BDV1wn3HBlMmPpv8k0%2B2kJsJ7DrcH3juww3Ansptg6QzlltStBtlMl6RfYXweyVGvmlAPODV%2FqS26o1IKQ1VCc2OVLP2s%3D</t>
+        </is>
+      </c>
+      <c r="H236" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I236" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3UkAAeSwNylqA0TS/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J236" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-12T15:21:56.000Z</t>
+        </is>
+      </c>
+      <c r="K236" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L236" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M236" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N236" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/To4AAeSwf8FqA0Tf/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O236" s="2" t="inlineStr"/>
+      <c r="P236" s="2" t="inlineStr"/>
+      <c r="Q236" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R236" s="2" t="inlineStr"/>
+      <c r="S236" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B237" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps</t>
+        </is>
+      </c>
+      <c r="C237" s="2" t="inlineStr">
+        <is>
+          <t>RARE~~2024 Topps Graphite Tennis Notable Rivalries MIRRA/ERIKA ANDREEVA 10/10</t>
+        </is>
+      </c>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E237" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F237" s="2" t="inlineStr">
+        <is>
+          <t>92.99 USD</t>
+        </is>
+      </c>
+      <c r="G237" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/267298443703?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8w5qVYws52%2FOBN54PDfWmKl0rV4aMES0KILrcMwqJnE1fxq%2BgWB9X%2Fcx27vHDorSTmLHX6IwOvgGHNrRNdmBBKfOQv1a9dNZ%2FDTga3aHES6Hxcr7uVr%2BGPYFpSlPu88w6bU0w4FEfBZiCP6fOaZSVU%2BmuIICHzBwq4hnigUIuyolTgQtzqc6d1lJbF2qsTDs4%3D</t>
+        </is>
+      </c>
+      <c r="H237" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I237" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/zzwAAeSweJZoVvNF/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J237" s="2" t="inlineStr">
+        <is>
+          <t>2025-06-21T18:01:19.000Z</t>
+        </is>
+      </c>
+      <c r="K237" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L237" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M237" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N237" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/slEAAeSwJSloVvNE/s-l1600.jpg | https://i.ebayimg.com/images/g/OsgAAeSwfGxoVvNE/s-l1600.jpg | https://i.ebayimg.com/images/g/mWMAAeSwfAVoVvNF/s-l1600.jpg | https://i.ebayimg.com/images/g/xREAAeSwC89oVvNF/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O237" s="2" t="inlineStr"/>
+      <c r="P237" s="2" t="inlineStr"/>
+      <c r="Q237" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R237" s="2" t="inlineStr"/>
+      <c r="S237" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B238" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - [Base] - Blue</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Blue 1/25 Erika Andreeva #64 Rookie RC 01mu</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F238" s="2" t="inlineStr">
+        <is>
+          <t>17.50 USD</t>
+        </is>
+      </c>
+      <c r="G238" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336784798075</t>
+        </is>
+      </c>
+      <c r="H238" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I238" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Bf8AAeSwvtNqn~xu/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J238" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08T12:01:57.000Z</t>
+        </is>
+      </c>
+      <c r="K238" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L238" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M238" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N238" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~4EAAeSwHAVqn~xu/s-l1600.jpg | https://i.ebayimg.com/images/g/KKQAAeSw5y9qn~xu/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O238" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P238" s="2" t="inlineStr"/>
+      <c r="Q238" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R238" s="2" t="inlineStr"/>
+      <c r="S238" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B239" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Royalty Collection</t>
+        </is>
+      </c>
+      <c r="C239" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva 2024 Topps Royalty Collection #MA Racket Knob Patch Auto RC 1/1</t>
+        </is>
+      </c>
+      <c r="D239" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E239" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F239" s="2" t="inlineStr">
+        <is>
+          <t>129999.99 USD</t>
+        </is>
+      </c>
+      <c r="G239" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/157524068051</t>
+        </is>
+      </c>
+      <c r="H239" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I239" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/kBkAAeSwC9ppMxkQ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J239" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05T18:26:43.000Z</t>
+        </is>
+      </c>
+      <c r="K239" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L239" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M239" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N239" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QHYAAeSwy2xpMxkQ/s-l1600.jpg | https://i.ebayimg.com/images/g/uE8AAeSwcLppMxkQ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O239" s="2" t="inlineStr"/>
+      <c r="P239" s="2" t="inlineStr"/>
+      <c r="Q239" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R239" s="2" t="inlineStr"/>
+      <c r="S239" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B240" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="inlineStr">
+        <is>
+          <t>Topps Royalty Tennis Erika &amp; Mirra Andreeva /Brenda &amp; Linda Fruhvirtova Auto 1/5</t>
+        </is>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E240" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F240" s="2" t="inlineStr">
+        <is>
+          <t>499.00 USD</t>
+        </is>
+      </c>
+      <c r="G240" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/226797223828</t>
+        </is>
+      </c>
+      <c r="H240" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I240" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/L-wAAeSwo7JoQP5x/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J240" s="2" t="inlineStr">
+        <is>
+          <t>2025-06-05T02:28:08.000Z</t>
+        </is>
+      </c>
+      <c r="K240" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L240" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M240" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N240" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/aBwAAeSwCVVoQP5y/s-l1600.jpg | https://i.ebayimg.com/images/g/DdUAAeSwI8poQP54/s-l1600.jpg | https://i.ebayimg.com/images/g/tYIAAeSwvVtoQP56/s-l1600.jpg | https://i.ebayimg.com/images/g/kuAAAeSwvyNoQP5~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O240" s="2" t="inlineStr"/>
+      <c r="P240" s="2" t="inlineStr"/>
+      <c r="Q240" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R240" s="2" t="inlineStr"/>
+      <c r="S240" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B241" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis Andreeva Fruhvirtova Quad Auto Platinum 1/1</t>
+        </is>
+      </c>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E241" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F241" s="2" t="inlineStr">
+        <is>
+          <t>1999.99 USD</t>
+        </is>
+      </c>
+      <c r="G241" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/286593107104</t>
+        </is>
+      </c>
+      <c r="H241" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I241" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/5jIAAeSw1ENoMWa2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J241" s="2" t="inlineStr">
+        <is>
+          <t>2025-05-24T06:33:40.000Z</t>
+        </is>
+      </c>
+      <c r="K241" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L241" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M241" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N241" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TSUAAeSw8idoMWa6/s-l1600.jpg | https://i.ebayimg.com/images/g/JPQAAeSw1KhoMWa4/s-l1600.jpg | https://i.ebayimg.com/images/g/mz8AAeSwDnNoMWa2/s-l1600.jpg | https://i.ebayimg.com/images/g/ZEcAAeSwSXVoMWa2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O241" s="2" t="inlineStr"/>
+      <c r="P241" s="2" t="inlineStr"/>
+      <c r="Q241" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R241" s="2" t="inlineStr"/>
+      <c r="S241" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>Qinwen Zheng</t>
+        </is>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Qinwen Zheng Geometric auto eBay 1/1 🔥🔥🔥 tennis</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E242" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F242" s="2" t="inlineStr">
+        <is>
+          <t>225.00 USD</t>
+        </is>
+      </c>
+      <c r="G242" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336791576225</t>
+        </is>
+      </c>
+      <c r="H242" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I242" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Pa8AAeSwKexqpN1q/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J242" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13T02:29:52.000Z</t>
+        </is>
+      </c>
+      <c r="K242" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L242" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M242" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N242" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gcUAAeSwmvhqpN10/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O242" s="2" t="inlineStr"/>
+      <c r="P242" s="2" t="inlineStr"/>
+      <c r="Q242" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R242" s="2" t="inlineStr"/>
+      <c r="S242" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>Qinwen Zheng</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Qinwen Zheng From All Angles True Gold Refractor #01/50</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E243" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t>21.47 USD</t>
+        </is>
+      </c>
+      <c r="G243" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/820124917498</t>
+        </is>
+      </c>
+      <c r="H243" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I243" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/xusAAeSw7v5qoGMm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J243" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14T07:50:49.000Z</t>
+        </is>
+      </c>
+      <c r="K243" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L243" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M243" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N243" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/pcEAAeSwBsNqoGMn/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O243" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P243" s="2" t="inlineStr"/>
+      <c r="Q243" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R243" s="2" t="inlineStr"/>
+      <c r="S243" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>Qinwen Zheng</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2025 Chrome Sapphire Green Saisai Zheng #248 75/75 WTA Tour Tennis Card</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>75/75</t>
+        </is>
+      </c>
+      <c r="E244" s="2" t="inlineStr">
+        <is>
+          <t>last of 75 (75/75)</t>
+        </is>
+      </c>
+      <c r="F244" s="2" t="inlineStr">
+        <is>
+          <t>24.99 USD</t>
+        </is>
+      </c>
+      <c r="G244" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/227369776480?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde9TPFGtmNQ9KZAgGJP4LZZaT0ud7P09T9Z06x9dkNcBS5uDwPmmnIy8d2GAaB6FH12joQlae0MaegsE%2BFEg%2B5UWSFeDKdFucyvBP80USfUNKBGK%2BZq3IBuZZOFeUFvg9lNqcRW9uqLt5U%2FxVnZtLxrg1Th7X0luQzRQ0gpKRCic%2FiXAUcSnurtvYLsQVhnBV1g%3D</t>
+        </is>
+      </c>
+      <c r="H244" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I244" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Ot4AAeSw6mBqHzFF/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J244" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02T19:44:52.000Z</t>
+        </is>
+      </c>
+      <c r="K244" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L244" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M244" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N244" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/tMcAAeSwY41qHzFQ/s-l1600.jpg | https://i.ebayimg.com/images/g/Xl0AAeSwgmRqHzGO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O244" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P244" s="2" t="inlineStr"/>
+      <c r="Q244" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R244" s="2" t="inlineStr"/>
+      <c r="S244" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>Qinwen Zheng</t>
+        </is>
+      </c>
+      <c r="B245" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Qinwen Zheng /50 Gold Youthquake Refractor #YQE-3 01/50</t>
+        </is>
+      </c>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E245" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F245" s="2" t="inlineStr">
+        <is>
+          <t>64.85 USD</t>
+        </is>
+      </c>
+      <c r="G245" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/127701188353</t>
+        </is>
+      </c>
+      <c r="H245" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I245" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/StEAAeSwkI1pnMFK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J245" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23T21:07:51.000Z</t>
+        </is>
+      </c>
+      <c r="K245" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L245" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M245" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N245" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/F4MAAeSwKpxpnMFs/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O245" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P245" s="2" t="inlineStr"/>
+      <c r="Q245" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R245" s="2" t="inlineStr"/>
+      <c r="S245" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>Qinwen Zheng</t>
+        </is>
+      </c>
+      <c r="B246" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite - Ace Relics Qinwen Zheng #AR-QZG Gold Refractor 01/25</t>
+        </is>
+      </c>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E246" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F246" s="2" t="inlineStr">
+        <is>
+          <t>10.00 USD</t>
+        </is>
+      </c>
+      <c r="G246" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287594460424</t>
+        </is>
+      </c>
+      <c r="H246" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I246" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KaMAAeSwnLRqrXJZ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J246" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T17:20:42.000Z</t>
+        </is>
+      </c>
+      <c r="K246" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L246" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M246" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N246" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/K3gAAeSwYjtqrXJ1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O246" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P246" s="2" t="inlineStr"/>
+      <c r="Q246" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R246" s="2" t="inlineStr"/>
+      <c r="S246" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>Steffi Graf</t>
+        </is>
+      </c>
+      <c r="B247" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Steffi Graf Ace-1 Red Refractor 5/5</t>
+        </is>
+      </c>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E247" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F247" s="2" t="inlineStr">
+        <is>
+          <t>475.00 USD</t>
+        </is>
+      </c>
+      <c r="G247" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/206135560131</t>
+        </is>
+      </c>
+      <c r="H247" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:41 UTC</t>
+        </is>
+      </c>
+      <c r="I247" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/pJYAAeSw0e5ptIDo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J247" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-13T21:27:25.000Z</t>
+        </is>
+      </c>
+      <c r="K247" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L247" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M247" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N247" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/wKUAAeSwj4FptIDo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O247" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P247" s="2" t="inlineStr"/>
+      <c r="Q247" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R247" s="2" t="inlineStr"/>
+      <c r="S247" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>Steffi Graf</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Winning Streaks White Refractor 1/10 Steffi Graf #WS-SG v9t</t>
+        </is>
+      </c>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E248" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F248" s="2" t="inlineStr">
+        <is>
+          <t>75.58 USD</t>
+        </is>
+      </c>
+      <c r="G248" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237026062518</t>
+        </is>
+      </c>
+      <c r="H248" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:42 UTC</t>
+        </is>
+      </c>
+      <c r="I248" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/1LYAAeSwYQVqi4iC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J248" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23T23:52:43.000Z</t>
+        </is>
+      </c>
+      <c r="K248" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L248" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M248" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N248" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/1-4AAeSwdK5qi4iC/s-l1600.jpg | https://i.ebayimg.com/images/g/3ycAAeSwDFZqi4iC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O248" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P248" s="2" t="inlineStr"/>
+      <c r="Q248" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R248" s="2" t="inlineStr"/>
+      <c r="S248" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>Steffi Graf</t>
+        </is>
+      </c>
+      <c r="B249" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Steffi Graf topps graphite 2024 all metal 25/25 </t>
+        </is>
+      </c>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E249" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F249" s="2" t="inlineStr">
+        <is>
+          <t>42.90 USD</t>
+        </is>
+      </c>
+      <c r="G249" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/158066535507</t>
+        </is>
+      </c>
+      <c r="H249" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:42 UTC</t>
+        </is>
+      </c>
+      <c r="I249" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JoUAAeSwCOdqTkrb/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J249" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08T13:08:27.000Z</t>
+        </is>
+      </c>
+      <c r="K249" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L249" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M249" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N249" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YrkAAeSwbJRqTkrb/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O249" s="2" t="inlineStr"/>
+      <c r="P249" s="2" t="inlineStr"/>
+      <c r="Q249" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R249" s="2" t="inlineStr"/>
+      <c r="S249" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>Steffi Graf</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Monica Seles Steffi Graf 25/25 Notable Rivalries #NR-SG</t>
+        </is>
+      </c>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E250" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F250" s="2" t="inlineStr">
+        <is>
+          <t>39.99 USD</t>
+        </is>
+      </c>
+      <c r="G250" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/197675901415?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2FjaD3porRTHtKqWRQyPpFwlwl2fpNoQd2bU1jip62wOwaxJ73knAatbaYpfFFvj%2FdI3JQ%2BDzxRKBskw3Ly8W7Ul5Dkth%2BjEFexEiLok14pUulzlKHQiRnBQSrshdNRRTfP0gZPw2jfqPvF8XPUaCijvn1c7EdFYIcCTCV8li0HuZqDxIInLtGE8Uji8p%2BbbFg%3D</t>
+        </is>
+      </c>
+      <c r="H250" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:42 UTC</t>
+        </is>
+      </c>
+      <c r="I250" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JW8AAeSw2J9ou-S7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J250" s="2" t="inlineStr">
+        <is>
+          <t>2025-09-06T07:38:43.000Z</t>
+        </is>
+      </c>
+      <c r="K250" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L250" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M250" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N250" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/S6YAAeSwlRJou-S7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O250" s="2" t="inlineStr"/>
+      <c r="P250" s="2" t="inlineStr"/>
+      <c r="Q250" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R250" s="2" t="inlineStr"/>
+      <c r="S250" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>Maria Sharapova</t>
+        </is>
+      </c>
+      <c r="B251" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C251" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis MARIA SHARAPOVA #153 Rose Gold Refractor SP #1/20</t>
+        </is>
+      </c>
+      <c r="D251" s="2" t="inlineStr">
+        <is>
+          <t>1/20</t>
+        </is>
+      </c>
+      <c r="E251" s="2" t="inlineStr">
+        <is>
+          <t>001 of 20</t>
+        </is>
+      </c>
+      <c r="F251" s="2" t="inlineStr">
+        <is>
+          <t>129.95 USD</t>
+        </is>
+      </c>
+      <c r="G251" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287540422035</t>
+        </is>
+      </c>
+      <c r="H251" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:42 UTC</t>
+        </is>
+      </c>
+      <c r="I251" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vHkAAeSwL3VqihsC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J251" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22T21:57:24.000Z</t>
+        </is>
+      </c>
+      <c r="K251" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L251" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M251" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N251" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/kFsAAeSwVppqihnm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O251" s="2" t="inlineStr">
+        <is>
+          <t>rose</t>
+        </is>
+      </c>
+      <c r="P251" s="2" t="inlineStr"/>
+      <c r="Q251" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R251" s="2" t="inlineStr"/>
+      <c r="S251" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>Maria Sharapova</t>
+        </is>
+      </c>
+      <c r="B252" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="inlineStr">
+        <is>
+          <t>Maria Sharapova 2024 Topps Graphite Tennis #62 White Refractor #'d 10/10 SSP</t>
+        </is>
+      </c>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E252" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F252" s="2" t="inlineStr">
+        <is>
+          <t>99.99 USD</t>
+        </is>
+      </c>
+      <c r="G252" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287547390824?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2B8JBtij2dz74e3lECdQgfKucZ9Vodr9vBxjL0ZR%2Fby1fa8hLPRJhYWxcOTc%2FaRKFaoqicAWkxXpu28pr3rcGaZq7OTMxAJDAo6S2l%2FYXk1o2hic1S%2Bg08FZ9cKM09A3JA9nLblfQNNwA3T8xmTthB54cXe8NI9u6nG0rA2jmOd3Xk92K%2FR0UTX3GR7Nqq0sos%3D</t>
+        </is>
+      </c>
+      <c r="H252" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:42 UTC</t>
+        </is>
+      </c>
+      <c r="I252" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-9AAAeSw0KVqjyBS/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J252" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26T17:22:56.000Z</t>
+        </is>
+      </c>
+      <c r="K252" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L252" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M252" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N252" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ZBcAAeSwyIRqjyBT/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O252" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P252" s="2" t="inlineStr"/>
+      <c r="Q252" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R252" s="2" t="inlineStr"/>
+      <c r="S252" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>Maria Sharapova</t>
+        </is>
+      </c>
+      <c r="B253" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Legends Court Green Refractor Maria Sharapova #LOC-MA 01/75</t>
+        </is>
+      </c>
+      <c r="D253" s="2" t="inlineStr">
+        <is>
+          <t>1/75</t>
+        </is>
+      </c>
+      <c r="E253" s="2" t="inlineStr">
+        <is>
+          <t>001 of 75</t>
+        </is>
+      </c>
+      <c r="F253" s="2" t="inlineStr">
+        <is>
+          <t>49.99 USD</t>
+        </is>
+      </c>
+      <c r="G253" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147514111339?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8qdrs1pBU3NnzyD956zTq0YH28%2FioLTQRfKzdWftOvC2rz0IWoBzYp5LDeZMtYDVP97i70uQJSCXlRVlTOE%2FE4yqJdyd4V1ywUSyIrC4kO%2FGLfEAZBuvgiXh9%2BDTkBe4GuFHHX%2FUwhVDTWEQ94uGJbdacTJtmnt3L3WWtIH8Y32HttKopCQWYQw1CTNRaxRzg%3D</t>
+        </is>
+      </c>
+      <c r="H253" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:42 UTC</t>
+        </is>
+      </c>
+      <c r="I253" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/N~QAAeSwDFZqhRwN/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J253" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-19T03:00:08.000Z</t>
+        </is>
+      </c>
+      <c r="K253" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L253" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M253" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N253" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/EMgAAeSw5RdqhRwM/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O253" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P253" s="2" t="inlineStr"/>
+      <c r="Q253" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R253" s="2" t="inlineStr"/>
+      <c r="S253" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>Maria Sharapova</t>
+        </is>
+      </c>
+      <c r="B254" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic / 2011 Ace Authentic</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="inlineStr">
+        <is>
+          <t>Maria Sharapova 2011 Ace Authentic #84 Tennis, Printing Mistake Error Rare 1/1?</t>
+        </is>
+      </c>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E254" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F254" s="2" t="inlineStr">
+        <is>
+          <t>500.00 USD</t>
+        </is>
+      </c>
+      <c r="G254" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/286208359345?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2BPDX5UJfvdJSe60h3iMEIpOENkyS%2FdevqW9JgKqp19y0j3NuiyCLo%2F9TN8XeyQYzkSBiRv5ngZg2OHEIGl5D0tZEbN5Pfyo99LvcU9AfuWTlnjkQ5tJcwG0PUZwEHcvz4aZ77n%2BVOrLsRMX7MfucYegwIdKvyyS%2FhcerBLnLWXmoD06tVtaCQhU5hdxE3O%2Fco%3D</t>
+        </is>
+      </c>
+      <c r="H254" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:42 UTC</t>
+        </is>
+      </c>
+      <c r="I254" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TDUAAOSwPRZnWFFW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J254" s="2" t="inlineStr">
+        <is>
+          <t>2024-12-10T14:51:20.000Z</t>
+        </is>
+      </c>
+      <c r="K254" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L254" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M254" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N254" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8goAAOSwr8lnWFF7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O254" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P254" s="2" t="inlineStr"/>
+      <c r="Q254" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R254" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic: check the numbering is stamped, not on a circle sticker</t>
+        </is>
+      </c>
+      <c r="S254" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -18051,6 +22615,58 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G200" r:id="rId199"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G201" r:id="rId200"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G202" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G203" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G204" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G205" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G206" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G207" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G208" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G209" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G210" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G211" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G212" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G213" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G214" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G215" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G216" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G217" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G218" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G219" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G220" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G221" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G222" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G223" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G224" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G225" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G226" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G227" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G228" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G229" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G230" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G231" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G232" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G233" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G234" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G235" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G236" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G237" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G238" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G239" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G240" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G241" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G242" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G243" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G244" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G245" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G246" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G247" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G248" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G249" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G250" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G251" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G252" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G253" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G254" r:id="rId253"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-19 08:48 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S254"/>
+  <dimension ref="A1:S266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -22407,6 +22407,1066 @@
         </is>
       </c>
       <c r="S254" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>Mitchell Krueger</t>
+        </is>
+      </c>
+      <c r="B255" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome I Black Refractor 1/10 Mitchell Krueger #TCA-MKR Auto 1w0z</t>
+        </is>
+      </c>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E255" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F255" s="2" t="inlineStr">
+        <is>
+          <t>37.00 USD</t>
+        </is>
+      </c>
+      <c r="G255" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336801311274</t>
+        </is>
+      </c>
+      <c r="H255" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I255" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/tbQAAeSw32Nqrjil/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J255" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:24:17.000Z</t>
+        </is>
+      </c>
+      <c r="K255" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L255" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M255" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N255" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/lXgAAeSw3c5qrjil/s-l1600.jpg | https://i.ebayimg.com/images/g/vncAAeSwl9hqrjil/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O255" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P255" s="2" t="inlineStr"/>
+      <c r="Q255" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R255" s="2" t="inlineStr"/>
+      <c r="S255" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>Michael Stich</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Green Refractor 75/75 Michael Stich #64 HOF 10no</t>
+        </is>
+      </c>
+      <c r="D256" s="2" t="inlineStr">
+        <is>
+          <t>75/75</t>
+        </is>
+      </c>
+      <c r="E256" s="2" t="inlineStr">
+        <is>
+          <t>last of 75 (75/75)</t>
+        </is>
+      </c>
+      <c r="F256" s="2" t="inlineStr">
+        <is>
+          <t>7.73 USD</t>
+        </is>
+      </c>
+      <c r="G256" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257751880700</t>
+        </is>
+      </c>
+      <c r="H256" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I256" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YGIAAeSwDG9qrhkk/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J256" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T05:08:51.000Z</t>
+        </is>
+      </c>
+      <c r="K256" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L256" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M256" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N256" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/LD8AAeSwyXtqrhkk/s-l1600.jpg | https://i.ebayimg.com/images/g/dAcAAeSwvd5qrhkk/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O256" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P256" s="2" t="inlineStr"/>
+      <c r="Q256" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R256" s="2" t="inlineStr"/>
+      <c r="S256" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>Juan Pablo Ficovich</t>
+        </is>
+      </c>
+      <c r="B257" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Sapphire Juan Pablo Ficovich RC Orange 1/25 ≈1/1</t>
+        </is>
+      </c>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E257" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F257" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G257" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/188947582839</t>
+        </is>
+      </c>
+      <c r="H257" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I257" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/02sAAeSwCZ5qrVGD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J257" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T04:25:13.000Z</t>
+        </is>
+      </c>
+      <c r="K257" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L257" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M257" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N257" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/NpkAAeSwR25qrVGN/s-l1600.jpg | https://i.ebayimg.com/images/g/d6IAAeSw1XpqrVGR/s-l1600.jpg | https://i.ebayimg.com/images/g/prMAAeSwfuZqrVGU/s-l1600.jpg | https://i.ebayimg.com/images/g/KzoAAeSwXUJqrVGa/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O257" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P257" s="2" t="inlineStr"/>
+      <c r="Q257" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R257" s="2" t="inlineStr"/>
+      <c r="S257" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>Valentin Vacherot</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Valentin Vacherot RC Purple Geometric 1/10 ≈1/1</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E258" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F258" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G258" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/188947581303</t>
+        </is>
+      </c>
+      <c r="H258" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I258" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/lnEAAeSwK45qrVE6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J258" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T04:20:38.000Z</t>
+        </is>
+      </c>
+      <c r="K258" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L258" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M258" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N258" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nPsAAeSwoXNqrVFB/s-l1600.jpg | https://i.ebayimg.com/images/g/OcAAAeSw52lqrVFE/s-l1600.jpg | https://i.ebayimg.com/images/g/XW8AAeSwnkFqrVFK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O258" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P258" s="2" t="inlineStr"/>
+      <c r="Q258" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R258" s="2" t="inlineStr"/>
+      <c r="S258" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="inlineStr"/>
+      <c r="B259" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C259" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis J.J. Wolf 1st Gold Refractor 50/50 ≈1/1</t>
+        </is>
+      </c>
+      <c r="D259" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E259" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F259" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G259" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/188947580783</t>
+        </is>
+      </c>
+      <c r="H259" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I259" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0DMAAeSwfGNqrVEM/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J259" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T04:16:53.000Z</t>
+        </is>
+      </c>
+      <c r="K259" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L259" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M259" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N259" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-xUAAeSwE4dqrVER/s-l1600.jpg | https://i.ebayimg.com/images/g/CN4AAeSwBDhqrVEW/s-l1600.jpg | https://i.ebayimg.com/images/g/pKkAAeSw2MBqrVEc/s-l1600.jpg | https://i.ebayimg.com/images/g/-S8AAeSwCxdqrVEh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O259" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P259" s="2" t="inlineStr"/>
+      <c r="Q259" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R259" s="2" t="inlineStr"/>
+      <c r="S259" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>Albert Ramos-Vinolas</t>
+        </is>
+      </c>
+      <c r="B260" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="inlineStr">
+        <is>
+          <t>Albert Ramos-Viñolas 🇪🇸 #01/10 Purple Geometric Ref -- 2025 Topps Chrome #161</t>
+        </is>
+      </c>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E260" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F260" s="2" t="inlineStr">
+        <is>
+          <t>14.95 USD</t>
+        </is>
+      </c>
+      <c r="G260" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178509172329?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8dosYhk8lMK6KuZySgt%2BUUMd7uOf1HmwhkibaCQAlcPpsmMpdVGw4C9fiYJq%2FYLtdNslssSj2BzmqKED%2FgufV0DNpHK6dectWj3KBa00t1TfaZCF9BeyLu9G3aHj7WNvNhxVps9OxVdVlfrpyM3TopxWy60WMHkKG5R3Yn4wfhn0KEPFQg2xsgzExJ%2FrJpVB0%3D</t>
+        </is>
+      </c>
+      <c r="H260" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I260" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bqMAAeSw7U5qrgZg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J260" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T03:49:59.000Z</t>
+        </is>
+      </c>
+      <c r="K260" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L260" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M260" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N260" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/yU4AAeSwE01qrgZf/s-l1600.jpg | https://i.ebayimg.com/images/g/99UAAeSwXf5qrgZg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O260" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P260" s="2" t="inlineStr"/>
+      <c r="Q260" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R260" s="2" t="inlineStr"/>
+      <c r="S260" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="inlineStr">
+        <is>
+          <t>Charlie Pasarell</t>
+        </is>
+      </c>
+      <c r="B261" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C261" s="2" t="inlineStr">
+        <is>
+          <t>2021 Chrome Gold Wave Refractor 1/50 Charlie Pasarell Charles Rookie RC HOF 1u6</t>
+        </is>
+      </c>
+      <c r="D261" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E261" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F261" s="2" t="inlineStr">
+        <is>
+          <t>11.00 USD</t>
+        </is>
+      </c>
+      <c r="G261" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336800804918</t>
+        </is>
+      </c>
+      <c r="H261" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I261" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/354AAeSw96Jqrfu4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J261" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T03:03:19.000Z</t>
+        </is>
+      </c>
+      <c r="K261" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L261" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M261" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N261" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XxAAAeSwVbhqrfu4/s-l1600.jpg | https://i.ebayimg.com/images/g/VvkAAeSwXwlqrfu3/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O261" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P261" s="2" t="inlineStr"/>
+      <c r="Q261" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R261" s="2" t="inlineStr"/>
+      <c r="S261" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>Daniil Medvedev</t>
+        </is>
+      </c>
+      <c r="B262" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="inlineStr">
+        <is>
+          <t>Topps Graphite Tennis Daniil Medvedev Auto Relic 50/50</t>
+        </is>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E262" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F262" s="2" t="inlineStr">
+        <is>
+          <t>34.46 USD</t>
+        </is>
+      </c>
+      <c r="G262" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178507314095</t>
+        </is>
+      </c>
+      <c r="H262" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I262" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/c2kAAeSwKkJqrRW5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J262" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T16:55:01.000Z</t>
+        </is>
+      </c>
+      <c r="K262" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L262" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M262" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N262" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JV4AAeSwt3xqrRW7/s-l1600.jpg | https://i.ebayimg.com/images/g/crQAAeSw97tqrRW7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O262" s="2" t="inlineStr"/>
+      <c r="P262" s="2" t="inlineStr"/>
+      <c r="Q262" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R262" s="2" t="inlineStr"/>
+      <c r="S262" s="2" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>Madison Keys</t>
+        </is>
+      </c>
+      <c r="B263" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite Tennis</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Tennis #168 White Refractor Madison Keys 10/10 BOOKEND</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E263" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F263" s="2" t="inlineStr">
+        <is>
+          <t>49.99 USD</t>
+        </is>
+      </c>
+      <c r="G263" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/327363752552?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8Vk%2FU3y8tIYWd4jLKZR4QO9TFsKvuuMTskJ%2BqoOHC5iDMb6Ef%2F8mgrg8j%2BS6ifzAzE5hT1IKxkG6idDCSOGEsgweYuehh4C4EJIcrWbVcQ7cgri35Z02vmZT%2BBIKIO0CST0ExpbBjXHcRQMLh1gVvhTSjjeOWX7K3uGSaDmkubrWdh6Wf6oR749bRxdjaH6Fk%3D</t>
+        </is>
+      </c>
+      <c r="H263" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I263" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jj8AAeSwZBRqrVf6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J263" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T15:27:29.000Z</t>
+        </is>
+      </c>
+      <c r="K263" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L263" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M263" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N263" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7PcAAeSweQVqrVf6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O263" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P263" s="2" t="inlineStr"/>
+      <c r="Q263" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R263" s="2" t="inlineStr"/>
+      <c r="S263" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>Ekaterina Alexandrova</t>
+        </is>
+      </c>
+      <c r="B264" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - [Base] - Blue</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Blue 1/25 Ekaterina Alexandrova #71 Rookie RC 1e41</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E264" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F264" s="2" t="inlineStr">
+        <is>
+          <t>23.25 USD</t>
+        </is>
+      </c>
+      <c r="G264" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237076081764</t>
+        </is>
+      </c>
+      <c r="H264" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I264" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/GN0AAeSwd3NqrZPT/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J264" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T19:40:03.000Z</t>
+        </is>
+      </c>
+      <c r="K264" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L264" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M264" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N264" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JsUAAeSwm3xqrZPT/s-l1600.jpg | https://i.ebayimg.com/images/g/n~0AAeSwvoBqrZPT/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O264" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P264" s="2" t="inlineStr"/>
+      <c r="Q264" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R264" s="2" t="inlineStr"/>
+      <c r="S264" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="inlineStr">
+        <is>
+          <t>Katarina Srebotnik</t>
+        </is>
+      </c>
+      <c r="B265" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic</t>
+        </is>
+      </c>
+      <c r="C265" s="2" t="inlineStr">
+        <is>
+          <t>2013-14 ACE AUTHENTIC GRAND SLAM HEROES AUTO KATARINA SREBOTNIK 1/15 PSA 9 AUTO</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E265" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F265" s="2" t="inlineStr">
+        <is>
+          <t>15.00 USD</t>
+        </is>
+      </c>
+      <c r="G265" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117417992887</t>
+        </is>
+      </c>
+      <c r="H265" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:48 UTC</t>
+        </is>
+      </c>
+      <c r="I265" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/zoAAAeSwfGNqrJnc/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J265" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T01:49:00.000Z</t>
+        </is>
+      </c>
+      <c r="K265" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L265" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M265" s="2" t="inlineStr">
+        <is>
+          <t>PSA 9</t>
+        </is>
+      </c>
+      <c r="N265" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nhIAAeSwBa1qrJnd/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O265" s="2" t="inlineStr"/>
+      <c r="P265" s="2" t="inlineStr"/>
+      <c r="Q265" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R265" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic autograph: on-card or sticker not stated; check by eye</t>
+        </is>
+      </c>
+      <c r="S265" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Waske</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic / 2007 Ace Authentic Straight Sets</t>
+        </is>
+      </c>
+      <c r="C266" s="2" t="inlineStr">
+        <is>
+          <t>2007 Ace Authentic #40 Alexander Waske Straight Sets Press Plates Magenta 1/1</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E266" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F266" s="2" t="inlineStr">
+        <is>
+          <t>5.06 USD</t>
+        </is>
+      </c>
+      <c r="G266" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336800173554?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2B38O0U3%2FX12ZHQvBtkF0YUurVx1rK53BSIF8U1Hgq01LPd6%2Fkejhhrse4Ry8%2BwfhFCnYGtEQAfzvNQ4OVMYa44u72cIlEideY9X47gpWAKMq6fPdGrsWKr%2FVx7ApAcEjQ%2Fuy8f7Pb611%2FkAs1yF5uHBIrZusvmrOGlZpwgkRzuP6aTy8C6%2F4fIQ58g5xI8h68%3D</t>
+        </is>
+      </c>
+      <c r="H266" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:48 UTC</t>
+        </is>
+      </c>
+      <c r="I266" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/N6EAAOSwDeBh-KRO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J266" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T19:09:58.000Z</t>
+        </is>
+      </c>
+      <c r="K266" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L266" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M266" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N266" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/dHIAAOSw20tdimQc/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O266" s="2" t="inlineStr">
+        <is>
+          <t>magenta</t>
+        </is>
+      </c>
+      <c r="P266" s="2" t="inlineStr"/>
+      <c r="Q266" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R266" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic: check the numbering is stamped, not on a circle sticker</t>
+        </is>
+      </c>
+      <c r="S266" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -22667,6 +23727,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G252" r:id="rId251"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G253" r:id="rId252"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G254" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G255" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G256" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G257" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G258" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G259" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G260" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G261" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G262" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G263" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G264" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G265" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G266" r:id="rId265"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-19 11:55 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S266"/>
+  <dimension ref="A1:S267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -23467,6 +23467,91 @@
         </is>
       </c>
       <c r="S266" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz, Cristiano Ronaldo, Lionel Messi, Michael Jordan, Ronaldo</t>
+        </is>
+      </c>
+      <c r="B267" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C267" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2026 Graphite Tennis Carlos Alcaraz 1/1 Nike Swoosh Event-Worn Patch Red</t>
+        </is>
+      </c>
+      <c r="D267" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E267" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F267" s="2" t="inlineStr">
+        <is>
+          <t>17999.00 USD</t>
+        </is>
+      </c>
+      <c r="G267" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/198652446183</t>
+        </is>
+      </c>
+      <c r="H267" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 11:55 UTC</t>
+        </is>
+      </c>
+      <c r="I267" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/krQAAeSwaENqrknG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J267" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T08:47:22.000Z</t>
+        </is>
+      </c>
+      <c r="K267" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L267" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M267" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N267" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/72oAAeSwfmBqrknG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O267" s="2" t="inlineStr"/>
+      <c r="P267" s="2" t="inlineStr"/>
+      <c r="Q267" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R267" s="2" t="inlineStr"/>
+      <c r="S267" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -23739,6 +23824,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G264" r:id="rId263"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G265" r:id="rId264"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G266" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G267" r:id="rId266"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-20 12:48 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S267"/>
+  <dimension ref="A1:S281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -23552,6 +23552,1248 @@
       </c>
       <c r="R267" s="2" t="inlineStr"/>
       <c r="S267" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>Emma Navarro</t>
+        </is>
+      </c>
+      <c r="B268" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - [Base] - Aqua Refractor</t>
+        </is>
+      </c>
+      <c r="C268" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Aqua Refractor 199/199 Emma Navarro #10 17uv</t>
+        </is>
+      </c>
+      <c r="D268" s="2" t="inlineStr">
+        <is>
+          <t>199/199</t>
+        </is>
+      </c>
+      <c r="E268" s="2" t="inlineStr">
+        <is>
+          <t>last of 199 (199/199)</t>
+        </is>
+      </c>
+      <c r="F268" s="2" t="inlineStr">
+        <is>
+          <t>5.42 USD</t>
+        </is>
+      </c>
+      <c r="G268" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336803723251</t>
+        </is>
+      </c>
+      <c r="H268" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="I268" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TA0AAeSwZBRqr9I9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J268" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T12:25:53.000Z</t>
+        </is>
+      </c>
+      <c r="K268" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L268" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M268" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N268" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/wOUAAeSwVbhqr9I9/s-l1600.jpg | https://i.ebayimg.com/images/g/yPwAAeSwamhqr9I9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O268" s="2" t="inlineStr">
+        <is>
+          <t>aqua</t>
+        </is>
+      </c>
+      <c r="P268" s="2" t="inlineStr"/>
+      <c r="Q268" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R268" s="2" t="inlineStr"/>
+      <c r="S268" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="inlineStr">
+        <is>
+          <t>Maya Joint</t>
+        </is>
+      </c>
+      <c r="B269" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C269" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Sapphire Tennis Maya Joint Padparadscha Pink Refractor 1/1💎</t>
+        </is>
+      </c>
+      <c r="D269" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E269" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F269" s="2" t="inlineStr">
+        <is>
+          <t>1999.99 USD</t>
+        </is>
+      </c>
+      <c r="G269" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/318893587517</t>
+        </is>
+      </c>
+      <c r="H269" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="I269" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vDMAAeSwnLRqr3aT/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J269" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T06:04:09.000Z</t>
+        </is>
+      </c>
+      <c r="K269" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L269" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M269" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N269" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vpYAAeSwgQNqr3at/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O269" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P269" s="2" t="inlineStr"/>
+      <c r="Q269" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R269" s="2" t="inlineStr"/>
+      <c r="S269" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Zverev</t>
+        </is>
+      </c>
+      <c r="B270" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Alexander Zverev Sapphire Selections Superfractor 1/1 SSS-24</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E270" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F270" s="2" t="inlineStr">
+        <is>
+          <t>265.00 USD</t>
+        </is>
+      </c>
+      <c r="G270" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257753156669</t>
+        </is>
+      </c>
+      <c r="H270" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="I270" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/d~oAAeSweGhqrUNJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J270" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T02:33:01.000Z</t>
+        </is>
+      </c>
+      <c r="K270" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L270" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M270" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N270" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/w6AAAeSw-0FqrUNJ/s-l1600.jpg | https://i.ebayimg.com/images/g/P7cAAeSwANVqrUNI/s-l1600.jpg | https://i.ebayimg.com/images/g/jogAAeSwDK9qrUNJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O270" s="2" t="inlineStr"/>
+      <c r="P270" s="2" t="inlineStr"/>
+      <c r="Q270" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R270" s="2" t="inlineStr"/>
+      <c r="S270" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="inlineStr">
+        <is>
+          <t>Altug Celikbilek</t>
+        </is>
+      </c>
+      <c r="B271" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C271" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Sapphire #213 Altug Celikbilek Padparadscha 1/1 One of One</t>
+        </is>
+      </c>
+      <c r="D271" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E271" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F271" s="2" t="inlineStr">
+        <is>
+          <t>3.33 USD</t>
+        </is>
+      </c>
+      <c r="G271" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257753148621</t>
+        </is>
+      </c>
+      <c r="H271" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="I271" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/j-gAAeSw4ptqrUJH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J271" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T02:25:01.000Z</t>
+        </is>
+      </c>
+      <c r="K271" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L271" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M271" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N271" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/qUgAAeSwYntqrUJH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O271" s="2" t="inlineStr"/>
+      <c r="P271" s="2" t="inlineStr"/>
+      <c r="Q271" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R271" s="2" t="inlineStr"/>
+      <c r="S271" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
+          <t>Luciano Darderi</t>
+        </is>
+      </c>
+      <c r="B272" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Sapphire Luciano Darderi RC Orange Refractor 25/25 SSP</t>
+        </is>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E272" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F272" s="2" t="inlineStr">
+        <is>
+          <t>34.99 USD</t>
+        </is>
+      </c>
+      <c r="G272" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366679802010</t>
+        </is>
+      </c>
+      <c r="H272" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="I272" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vBYAAeSwfEZqr0CY/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J272" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T02:13:28.000Z</t>
+        </is>
+      </c>
+      <c r="K272" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L272" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M272" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N272" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jEkAAeSwpr5qr0CZ/s-l1600.jpg | https://i.ebayimg.com/images/g/LDUAAeSw2lNqr0CZ/s-l1600.jpg | https://i.ebayimg.com/images/g/mkwAAeSwJs5qr0CZ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O272" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P272" s="2" t="inlineStr"/>
+      <c r="Q272" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R272" s="2" t="inlineStr"/>
+      <c r="S272" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="inlineStr">
+        <is>
+          <t>Yanquiel Fernandez</t>
+        </is>
+      </c>
+      <c r="B273" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C273" s="2" t="inlineStr">
+        <is>
+          <t>2026 TOPPS CHROME TEAL REFRACTOR YANQUIEL FERNANDEZ RC AUTO #299/299</t>
+        </is>
+      </c>
+      <c r="D273" s="2" t="inlineStr">
+        <is>
+          <t>299/299</t>
+        </is>
+      </c>
+      <c r="E273" s="2" t="inlineStr">
+        <is>
+          <t>last of 299 (299/299)</t>
+        </is>
+      </c>
+      <c r="F273" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G273" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/318890911526</t>
+        </is>
+      </c>
+      <c r="H273" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="I273" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/P5QAAeSwkOJqro8r/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J273" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T02:13:01.000Z</t>
+        </is>
+      </c>
+      <c r="K273" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L273" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M273" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N273" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jsQAAeSwf9tqro8w/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O273" s="2" t="inlineStr">
+        <is>
+          <t>teal</t>
+        </is>
+      </c>
+      <c r="P273" s="2" t="inlineStr"/>
+      <c r="Q273" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R273" s="2" t="inlineStr"/>
+      <c r="S273" s="2" t="inlineStr">
+        <is>
+          <t>Auto Racing, Baseball, Basketball, Soccer, Tennis, Volleyball, Wrestling</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>HOLGER RUNE</t>
+        </is>
+      </c>
+      <c r="B274" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 TOPPS CHROME TENNIS CHROME AUTOGRAPHS</t>
+        </is>
+      </c>
+      <c r="C274" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS CHROME AUTO ORANGE GEOMETRIC HOLGER RUNE 25/25 PSA 9</t>
+        </is>
+      </c>
+      <c r="D274" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E274" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F274" s="2" t="inlineStr">
+        <is>
+          <t>1.25 USD</t>
+        </is>
+      </c>
+      <c r="G274" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117419302960</t>
+        </is>
+      </c>
+      <c r="H274" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="I274" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/maUAAeSwXf5qrZwB/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J274" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T01:11:00.000Z</t>
+        </is>
+      </c>
+      <c r="K274" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L274" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M274" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N274" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gMEAAeSwNsRqrZwB/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O274" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P274" s="2" t="inlineStr"/>
+      <c r="Q274" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R274" s="2" t="inlineStr"/>
+      <c r="S274" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="inlineStr">
+        <is>
+          <t>Bianca Andreescu</t>
+        </is>
+      </c>
+      <c r="B275" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C275" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome - Bianca Andreescu #185 FROZENFRACTOR -1/0 SSP</t>
+        </is>
+      </c>
+      <c r="D275" s="2" t="inlineStr">
+        <is>
+          <t>1/0</t>
+        </is>
+      </c>
+      <c r="E275" s="2" t="inlineStr">
+        <is>
+          <t>001 of 0</t>
+        </is>
+      </c>
+      <c r="F275" s="2" t="inlineStr">
+        <is>
+          <t>54.99 USD</t>
+        </is>
+      </c>
+      <c r="G275" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178510870113?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2Fp0Yhz7NIbwhjbNruA%2BymJ3%2BqmpKvdJKww8XcpU%2BYAlneMBwL6qFWQjso4xp0cFZWIW5n%2Bl01JLAiJxNDk1sONf2i%2ByPPopqLH3dsQiCaeJXqNaYpjrNtXzKQN66QV1FT39b7eupoa7BvMALZK77BzpCUs0sj3RhPXPepB%2BbDj5xA7Ka90%2BSC97giQ94BBD4s%3D</t>
+        </is>
+      </c>
+      <c r="H275" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="I275" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/6wUAAeSwYntqrcEO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J275" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T19:05:41.000Z</t>
+        </is>
+      </c>
+      <c r="K275" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L275" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M275" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N275" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/aT4AAeSwcFNqrcEO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O275" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P275" s="2" t="inlineStr"/>
+      <c r="Q275" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R275" s="2" t="inlineStr"/>
+      <c r="S275" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>Veronika Kudermetova</t>
+        </is>
+      </c>
+      <c r="B276" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite Tennis</t>
+        </is>
+      </c>
+      <c r="C276" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Tennis Veronika Kudermetova #147 Refractor 10/10 Bookend SP</t>
+        </is>
+      </c>
+      <c r="D276" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E276" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F276" s="2" t="inlineStr">
+        <is>
+          <t>0.76 USD</t>
+        </is>
+      </c>
+      <c r="G276" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168701452757</t>
+        </is>
+      </c>
+      <c r="H276" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="I276" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Yz4AAeSw32Nqrznl/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J276" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T01:42:19.000Z</t>
+        </is>
+      </c>
+      <c r="K276" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L276" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M276" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N276" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/NyUAAeSwZBRqrzns/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O276" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P276" s="2" t="inlineStr"/>
+      <c r="Q276" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R276" s="2" t="inlineStr"/>
+      <c r="S276" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
+        <is>
+          <t>John McEnroe</t>
+        </is>
+      </c>
+      <c r="B277" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025-2026 Topps</t>
+        </is>
+      </c>
+      <c r="C277" s="2" t="inlineStr">
+        <is>
+          <t>John McEnroe 2026 Topps Graphite Tennis #100 Pink 15/15 Bookend</t>
+        </is>
+      </c>
+      <c r="D277" s="2" t="inlineStr">
+        <is>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="E277" s="2" t="inlineStr">
+        <is>
+          <t>last of 15 (15/15)</t>
+        </is>
+      </c>
+      <c r="F277" s="2" t="inlineStr">
+        <is>
+          <t>10.00 USD</t>
+        </is>
+      </c>
+      <c r="G277" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168701421392</t>
+        </is>
+      </c>
+      <c r="H277" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="I277" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/W6IAAeSwnyhqrzXX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J277" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T01:25:10.000Z</t>
+        </is>
+      </c>
+      <c r="K277" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L277" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M277" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N277" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/IrgAAeSwjTNqrzXg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O277" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P277" s="2" t="inlineStr"/>
+      <c r="Q277" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R277" s="2" t="inlineStr"/>
+      <c r="S277" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>Ben Shelton</t>
+        </is>
+      </c>
+      <c r="B278" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C278" s="2" t="inlineStr">
+        <is>
+          <t>2026 TOPPS GRAPHITE TENNIS RALLY RELIC #RR-BS BEN SHELTON GOLD REFRACTOR #1/25</t>
+        </is>
+      </c>
+      <c r="D278" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E278" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F278" s="2" t="inlineStr">
+        <is>
+          <t>95.00 USD</t>
+        </is>
+      </c>
+      <c r="G278" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/398412036224</t>
+        </is>
+      </c>
+      <c r="H278" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="I278" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gpwAAeSwM-Nqrx2~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J278" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T23:45:41.000Z</t>
+        </is>
+      </c>
+      <c r="K278" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L278" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M278" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N278" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nsIAAeSwNyZqrx4C/s-l1600.jpg | https://i.ebayimg.com/images/g/0a0AAeSwyCpqrumz/s-l1600.jpg | https://i.ebayimg.com/images/g/nHwAAeSwn35qrx5E/s-l1600.jpg | https://i.ebayimg.com/images/g/hzUAAeSwN55qrueh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O278" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P278" s="2" t="inlineStr"/>
+      <c r="Q278" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R278" s="2" t="inlineStr"/>
+      <c r="S278" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="inlineStr">
+        <is>
+          <t>Francisco Cerundolo</t>
+        </is>
+      </c>
+      <c r="B279" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Star Relics - Blue</t>
+        </is>
+      </c>
+      <c r="C279" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Star Relics Blue 25/25 Francisco Cerundolo Rookie RC 9et</t>
+        </is>
+      </c>
+      <c r="D279" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E279" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F279" s="2" t="inlineStr">
+        <is>
+          <t>29.58 USD</t>
+        </is>
+      </c>
+      <c r="G279" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237078640458</t>
+        </is>
+      </c>
+      <c r="H279" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="I279" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/eu8AAeSwfEZqrvy8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J279" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T21:19:57.000Z</t>
+        </is>
+      </c>
+      <c r="K279" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L279" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M279" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N279" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HogAAeSw6pdqrvy8/s-l1600.jpg | https://i.ebayimg.com/images/g/hb0AAeSwMH9qrvy8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O279" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P279" s="2" t="inlineStr"/>
+      <c r="Q279" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R279" s="2" t="inlineStr"/>
+      <c r="S279" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="inlineStr">
+        <is>
+          <t>Lisa Raymond</t>
+        </is>
+      </c>
+      <c r="B280" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic</t>
+        </is>
+      </c>
+      <c r="C280" s="2" t="inlineStr">
+        <is>
+          <t>Lisa Raymond 2013 Ace Authentic Grand Slam Tennis Auto 25/25 Heroes [9hk</t>
+        </is>
+      </c>
+      <c r="D280" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E280" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F280" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G280" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377509427955</t>
+        </is>
+      </c>
+      <c r="H280" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="I280" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/NSMAAeSwVyhqrzTB/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J280" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T01:18:58.000Z</t>
+        </is>
+      </c>
+      <c r="K280" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L280" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M280" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N280" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RzkAAeSw2aZqrzTD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O280" s="2" t="inlineStr"/>
+      <c r="P280" s="2" t="inlineStr"/>
+      <c r="Q280" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R280" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic autograph: on-card or sticker not stated; check by eye</t>
+        </is>
+      </c>
+      <c r="S280" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="2" t="inlineStr">
+        <is>
+          <t>Tracy Austin</t>
+        </is>
+      </c>
+      <c r="B281" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic / 2008 Ace Authentic Grand Slam II</t>
+        </is>
+      </c>
+      <c r="C281" s="2" t="inlineStr">
+        <is>
+          <t>2008 Ace Grand Slam II Stars/Legends Jersey Gold 1/24 #JC19 Tracy Austin PSA 4</t>
+        </is>
+      </c>
+      <c r="D281" s="2" t="inlineStr">
+        <is>
+          <t>1/24</t>
+        </is>
+      </c>
+      <c r="E281" s="2" t="inlineStr">
+        <is>
+          <t>001 of 24</t>
+        </is>
+      </c>
+      <c r="F281" s="2" t="inlineStr">
+        <is>
+          <t>50.00 USD</t>
+        </is>
+      </c>
+      <c r="G281" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168701028720</t>
+        </is>
+      </c>
+      <c r="H281" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="I281" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/1F4AAOSwq2hm7HWW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J281" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T20:54:20.000Z</t>
+        </is>
+      </c>
+      <c r="K281" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L281" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M281" s="2" t="inlineStr">
+        <is>
+          <t>PSA 4</t>
+        </is>
+      </c>
+      <c r="N281" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~xIAAOSwyWFm7HWh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O281" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P281" s="2" t="inlineStr"/>
+      <c r="Q281" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R281" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic: check the numbering is stamped, not on a circle sticker</t>
+        </is>
+      </c>
+      <c r="S281" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -23825,6 +25067,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G265" r:id="rId264"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G266" r:id="rId265"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G267" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G268" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G269" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G270" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G271" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G272" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G273" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G274" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G275" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G276" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G277" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G278" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G279" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G280" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G281" r:id="rId280"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-21 00:48 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S281"/>
+  <dimension ref="A1:S282"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -24794,6 +24794,95 @@
         </is>
       </c>
       <c r="S281" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
+          <t>Noskova</t>
+        </is>
+      </c>
+      <c r="B282" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C282" s="2" t="inlineStr">
+        <is>
+          <t>Linda Noskova 2025 Topps Chrome Tennis RC Auto Superfractor 1/1</t>
+        </is>
+      </c>
+      <c r="D282" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E282" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F282" s="2" t="inlineStr">
+        <is>
+          <t>19999.99 USD</t>
+        </is>
+      </c>
+      <c r="G282" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377464009580</t>
+        </is>
+      </c>
+      <c r="H282" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21 00:48 UTC</t>
+        </is>
+      </c>
+      <c r="I282" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/FVAAAeSwTtFql5Ag/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J282" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02T03:09:03.000Z</t>
+        </is>
+      </c>
+      <c r="K282" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L282" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M282" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N282" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TNQAAeSwSGdql5BU/s-l1600.jpg | https://i.ebayimg.com/images/g/ZD0AAeSwskFql5CD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O282" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P282" s="2" t="inlineStr"/>
+      <c r="Q282" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R282" s="2" t="inlineStr"/>
+      <c r="S282" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -25081,6 +25170,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G279" r:id="rId278"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G280" r:id="rId279"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G281" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G282" r:id="rId281"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-21 10:05 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S282"/>
+  <dimension ref="A1:S292"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -24883,6 +24883,888 @@
       </c>
       <c r="R282" s="2" t="inlineStr"/>
       <c r="S282" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="2" t="inlineStr">
+        <is>
+          <t>Belinda Bencic</t>
+        </is>
+      </c>
+      <c r="B283" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C283" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Belinda Bennie BLACK  GEOMETRIC 2/2</t>
+        </is>
+      </c>
+      <c r="D283" s="2" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="E283" s="2" t="inlineStr">
+        <is>
+          <t>last of 2 (2/2)</t>
+        </is>
+      </c>
+      <c r="F283" s="2" t="inlineStr">
+        <is>
+          <t>299.99 USD</t>
+        </is>
+      </c>
+      <c r="G283" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/128090408654</t>
+        </is>
+      </c>
+      <c r="H283" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21 10:05 UTC</t>
+        </is>
+      </c>
+      <c r="I283" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/yigAAeSwzmBqsJ5u/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J283" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21T03:04:15.000Z</t>
+        </is>
+      </c>
+      <c r="K283" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L283" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M283" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N283" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2AEAAeSwahRqsJ5u/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O283" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P283" s="2" t="inlineStr"/>
+      <c r="Q283" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R283" s="2" t="inlineStr"/>
+      <c r="S283" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Zverev</t>
+        </is>
+      </c>
+      <c r="B284" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS CHROME TENNIS CAPTURED</t>
+        </is>
+      </c>
+      <c r="C284" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS CHROME TENNIS CAPTURED SUPERFRACTOR 1/1 ALEXANDER ZVEREV 1/1 PSA 10</t>
+        </is>
+      </c>
+      <c r="D284" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E284" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F284" s="2" t="inlineStr">
+        <is>
+          <t>9999.00 USD</t>
+        </is>
+      </c>
+      <c r="G284" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117418654093</t>
+        </is>
+      </c>
+      <c r="H284" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21 10:05 UTC</t>
+        </is>
+      </c>
+      <c r="I284" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RJcAAeSwIIxqrSGs/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J284" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21T01:43:00.000Z</t>
+        </is>
+      </c>
+      <c r="K284" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L284" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M284" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 10</t>
+        </is>
+      </c>
+      <c r="N284" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/FawAAeSwXS5qrSGs/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O284" s="2" t="inlineStr"/>
+      <c r="P284" s="2" t="inlineStr"/>
+      <c r="Q284" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R284" s="2" t="inlineStr"/>
+      <c r="S284" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="inlineStr">
+        <is>
+          <t>Stefan Edberg</t>
+        </is>
+      </c>
+      <c r="B285" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C285" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Stefan Edberg Aces Auto #AA-SE Orange Refractor 25/25</t>
+        </is>
+      </c>
+      <c r="D285" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E285" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F285" s="2" t="inlineStr">
+        <is>
+          <t>109.99 USD</t>
+        </is>
+      </c>
+      <c r="G285" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/820151763242?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8GlInYZquhB9w5W8iJ5bM5TkEIKg0gna5oUoEjGUgV04r0PlA5z97LxIVgQuWo%2BdjBCNfL2BHWgKvbbvGFEZMApjr6D%2BoYstT1X8iU57GaX4Y69kVq8tUeEb973KFN6lm6jfiWUyUciX%2F1LAykxWxWjNed0tN7lMQmg8HFNIpkuSUORfXOhbOR9izZAOGRsbs%3D</t>
+        </is>
+      </c>
+      <c r="H285" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21 10:05 UTC</t>
+        </is>
+      </c>
+      <c r="I285" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/fW4AAeSwPKNqsHg6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J285" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21T00:22:24.000Z</t>
+        </is>
+      </c>
+      <c r="K285" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L285" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M285" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N285" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/mscAAeSw4kFqsHg6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O285" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P285" s="2" t="inlineStr"/>
+      <c r="Q285" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R285" s="2" t="inlineStr"/>
+      <c r="S285" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>Lukas Neumayer</t>
+        </is>
+      </c>
+      <c r="B286" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C286" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis #269 Lukas Neumayer RC Black Refractor #d 10/10</t>
+        </is>
+      </c>
+      <c r="D286" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E286" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F286" s="2" t="inlineStr">
+        <is>
+          <t>14.99 USD</t>
+        </is>
+      </c>
+      <c r="G286" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/398415016762</t>
+        </is>
+      </c>
+      <c r="H286" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21 10:05 UTC</t>
+        </is>
+      </c>
+      <c r="I286" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/dX4AAeSwOydqsHEd/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J286" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T23:50:27.000Z</t>
+        </is>
+      </c>
+      <c r="K286" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L286" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M286" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N286" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Ty4AAeSwwelqsHEd/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O286" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P286" s="2" t="inlineStr"/>
+      <c r="Q286" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R286" s="2" t="inlineStr"/>
+      <c r="S286" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="2" t="inlineStr">
+        <is>
+          <t>Maya Joint</t>
+        </is>
+      </c>
+      <c r="B287" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C287" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Sapphire Tennis Maya Joint Padparadscha Pink Refractor 1/1💎</t>
+        </is>
+      </c>
+      <c r="D287" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E287" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F287" s="2" t="inlineStr">
+        <is>
+          <t>4.25 USD</t>
+        </is>
+      </c>
+      <c r="G287" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/318896212965</t>
+        </is>
+      </c>
+      <c r="H287" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21 10:05 UTC</t>
+        </is>
+      </c>
+      <c r="I287" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vDMAAeSwnLRqr3aT/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J287" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T19:43:00.000Z</t>
+        </is>
+      </c>
+      <c r="K287" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L287" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M287" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N287" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vpYAAeSwgQNqr3at/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O287" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P287" s="2" t="inlineStr"/>
+      <c r="Q287" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R287" s="2" t="inlineStr"/>
+      <c r="S287" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>Martina Navratilova</t>
+        </is>
+      </c>
+      <c r="B288" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C288" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Martina Navratilova Autographs II Orange Auto 01/25</t>
+        </is>
+      </c>
+      <c r="D288" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E288" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F288" s="2" t="inlineStr">
+        <is>
+          <t>55.00 USD</t>
+        </is>
+      </c>
+      <c r="G288" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168703001948</t>
+        </is>
+      </c>
+      <c r="H288" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21 10:05 UTC</t>
+        </is>
+      </c>
+      <c r="I288" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/boEAAeSwfmBqsCYl/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J288" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T18:30:49.000Z</t>
+        </is>
+      </c>
+      <c r="K288" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L288" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M288" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N288" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/VYIAAeSwaw5qsCYf/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O288" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P288" s="2" t="inlineStr"/>
+      <c r="Q288" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R288" s="2" t="inlineStr"/>
+      <c r="S288" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="2" t="inlineStr">
+        <is>
+          <t>Donna Vekic</t>
+        </is>
+      </c>
+      <c r="B289" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Sapphire Edition - [Base] - Purple</t>
+        </is>
+      </c>
+      <c r="C289" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Sapphire Purple 1/10 Donna Vekic #31 1d0h</t>
+        </is>
+      </c>
+      <c r="D289" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E289" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F289" s="2" t="inlineStr">
+        <is>
+          <t>24.98 USD</t>
+        </is>
+      </c>
+      <c r="G289" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237080095279</t>
+        </is>
+      </c>
+      <c r="H289" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21 10:05 UTC</t>
+        </is>
+      </c>
+      <c r="I289" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~IsAAeSw4kFqr-bk/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J289" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T13:58:55.000Z</t>
+        </is>
+      </c>
+      <c r="K289" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L289" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M289" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N289" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7sAAAeSwSmdqr-bk/s-l1600.jpg | https://i.ebayimg.com/images/g/pc0AAeSwmuxqr-bk/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O289" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P289" s="2" t="inlineStr"/>
+      <c r="Q289" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R289" s="2" t="inlineStr"/>
+      <c r="S289" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="2" t="inlineStr">
+        <is>
+          <t>Pete Sampras</t>
+        </is>
+      </c>
+      <c r="B290" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C290" s="2" t="inlineStr">
+        <is>
+          <t>2024 Graphite Legends of the Court Pink Refractor 1/15 Pete Sampras PSA 9 4vc</t>
+        </is>
+      </c>
+      <c r="D290" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E290" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F290" s="2" t="inlineStr">
+        <is>
+          <t>69.24 USD</t>
+        </is>
+      </c>
+      <c r="G290" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237081045425</t>
+        </is>
+      </c>
+      <c r="H290" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21 10:05 UTC</t>
+        </is>
+      </c>
+      <c r="I290" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/MBUAAeSwE01qsLmP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J290" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21T04:57:53.000Z</t>
+        </is>
+      </c>
+      <c r="K290" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L290" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M290" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports (PSA) 9 MINT</t>
+        </is>
+      </c>
+      <c r="N290" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/fOEAAeSwsntqsLmP/s-l1600.jpg | https://i.ebayimg.com/images/g/p8AAAeSwSbhqsLmQ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O290" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P290" s="2" t="inlineStr"/>
+      <c r="Q290" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R290" s="2" t="inlineStr"/>
+      <c r="S290" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="2" t="inlineStr">
+        <is>
+          <t>Terence Atmane</t>
+        </is>
+      </c>
+      <c r="B291" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite Tennis</t>
+        </is>
+      </c>
+      <c r="C291" s="2" t="inlineStr">
+        <is>
+          <t>TERENCE ATMANE 2026 TOPPS GRAPHITE SIGNATURES PINK AUTO 15/15 #GRS-TAE Q5446</t>
+        </is>
+      </c>
+      <c r="D291" s="2" t="inlineStr">
+        <is>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="E291" s="2" t="inlineStr">
+        <is>
+          <t>last of 15 (15/15)</t>
+        </is>
+      </c>
+      <c r="F291" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G291" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/278392748356</t>
+        </is>
+      </c>
+      <c r="H291" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21 10:05 UTC</t>
+        </is>
+      </c>
+      <c r="I291" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Dk8AAeSwfEZqr-a3/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J291" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21T00:37:00.000Z</t>
+        </is>
+      </c>
+      <c r="K291" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L291" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M291" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N291" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8mMAAeSwD91qr-a3/s-l1600.jpg | https://i.ebayimg.com/images/g/GvkAAeSwyCpqr-a3/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O291" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P291" s="2" t="inlineStr"/>
+      <c r="Q291" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R291" s="2" t="inlineStr"/>
+      <c r="S291" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="2" t="inlineStr">
+        <is>
+          <t>Francisco Cerundolo</t>
+        </is>
+      </c>
+      <c r="B292" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Star Relics</t>
+        </is>
+      </c>
+      <c r="C292" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Star Relics 75/75 Francisco Cerundolo #SRR-FC Rookie RC 9et</t>
+        </is>
+      </c>
+      <c r="D292" s="2" t="inlineStr">
+        <is>
+          <t>75/75</t>
+        </is>
+      </c>
+      <c r="E292" s="2" t="inlineStr">
+        <is>
+          <t>last of 75 (75/75)</t>
+        </is>
+      </c>
+      <c r="F292" s="2" t="inlineStr">
+        <is>
+          <t>29.58 USD</t>
+        </is>
+      </c>
+      <c r="G292" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257755612612</t>
+        </is>
+      </c>
+      <c r="H292" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21 10:05 UTC</t>
+        </is>
+      </c>
+      <c r="I292" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-FgAAeSwZXtqsIuH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J292" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21T01:41:28.000Z</t>
+        </is>
+      </c>
+      <c r="K292" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L292" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M292" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N292" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/FOYAAeSwuXtqsIuH/s-l1600.jpg | https://i.ebayimg.com/images/g/6~0AAeSwvoBqsIuH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O292" s="2" t="inlineStr"/>
+      <c r="P292" s="2" t="inlineStr"/>
+      <c r="Q292" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R292" s="2" t="inlineStr"/>
+      <c r="S292" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -25171,6 +26053,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G280" r:id="rId279"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G281" r:id="rId280"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G282" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G283" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G284" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G285" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G286" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G287" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G288" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G289" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G290" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G291" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G292" r:id="rId291"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-21 15:58 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S292"/>
+  <dimension ref="A1:S293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -25765,6 +25765,95 @@
       </c>
       <c r="R292" s="2" t="inlineStr"/>
       <c r="S292" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="2" t="inlineStr">
+        <is>
+          <t>Jack Draper</t>
+        </is>
+      </c>
+      <c r="B293" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Superior Signatures - Green</t>
+        </is>
+      </c>
+      <c r="C293" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Green 1/5 Jack Draper PSA Authentic Rookie Auto RC 0r9h</t>
+        </is>
+      </c>
+      <c r="D293" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E293" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F293" s="2" t="inlineStr">
+        <is>
+          <t>692.20 USD</t>
+        </is>
+      </c>
+      <c r="G293" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336805454552</t>
+        </is>
+      </c>
+      <c r="H293" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:58 UTC</t>
+        </is>
+      </c>
+      <c r="I293" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/kMcAAeSwPD5qsT~8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J293" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21T14:31:19.000Z</t>
+        </is>
+      </c>
+      <c r="K293" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L293" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M293" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports (PSA) Authentic</t>
+        </is>
+      </c>
+      <c r="N293" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/WIMAAeSwAetqsT~8/s-l1600.jpg | https://i.ebayimg.com/images/g/9UYAAeSwKfZqsT~8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O293" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P293" s="2" t="inlineStr"/>
+      <c r="Q293" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R293" s="2" t="inlineStr"/>
+      <c r="S293" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -26063,6 +26152,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G290" r:id="rId289"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G291" r:id="rId290"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G292" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G293" r:id="rId292"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-22 14:07 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S293"/>
+  <dimension ref="A1:S315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -25854,6 +25854,1936 @@
       </c>
       <c r="R293" s="2" t="inlineStr"/>
       <c r="S293" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Nadal</t>
+        </is>
+      </c>
+      <c r="B294" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C294" s="2" t="inlineStr">
+        <is>
+          <t>RAFAEL NADAL-----GOLD-----ACES 50/50-----BOOKEND-----2025 TOPPS CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="D294" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E294" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F294" s="2" t="inlineStr">
+        <is>
+          <t>2500.00 USD</t>
+        </is>
+      </c>
+      <c r="G294" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/278398688073</t>
+        </is>
+      </c>
+      <c r="H294" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:06 UTC</t>
+        </is>
+      </c>
+      <c r="I294" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/q~gAAeSwlvdqsn-N/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J294" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T13:17:11.000Z</t>
+        </is>
+      </c>
+      <c r="K294" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L294" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M294" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N294" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KiYAAeSwwQlqsn-Z/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O294" s="2" t="inlineStr"/>
+      <c r="P294" s="2" t="inlineStr"/>
+      <c r="Q294" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R294" s="2" t="inlineStr"/>
+      <c r="S294" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="2" t="inlineStr">
+        <is>
+          <t>Kostyuk</t>
+        </is>
+      </c>
+      <c r="B295" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 topps chrome</t>
+        </is>
+      </c>
+      <c r="C295" s="2" t="inlineStr">
+        <is>
+          <t>MARTA KOSTYUK 2025 Topps Chrome Tennis Purple Geometric 10/10 Auto CG48</t>
+        </is>
+      </c>
+      <c r="D295" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E295" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F295" s="2" t="inlineStr">
+        <is>
+          <t>200.00 USD</t>
+        </is>
+      </c>
+      <c r="G295" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407235900399</t>
+        </is>
+      </c>
+      <c r="H295" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:06 UTC</t>
+        </is>
+      </c>
+      <c r="I295" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/kDQAAeSwUHVqsh-A/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J295" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T06:24:27.000Z</t>
+        </is>
+      </c>
+      <c r="K295" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L295" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M295" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N295" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/hG8AAeSwOH5qsh-A/s-l1600.jpg | https://i.ebayimg.com/images/g/qDUAAeSwodJqsh-A/s-l1600.jpg | https://i.ebayimg.com/images/g/rCcAAeSwoNVqsh-A/s-l1600.jpg | https://i.ebayimg.com/images/g/jxUAAeSwz-pqsh-A/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O295" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P295" s="2" t="inlineStr"/>
+      <c r="Q295" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R295" s="2" t="inlineStr"/>
+      <c r="S295" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="2" t="inlineStr">
+        <is>
+          <t>Nick Kyrgios</t>
+        </is>
+      </c>
+      <c r="B296" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C296" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis Nick Kyrgios Green Refractor 01/99 # 187</t>
+        </is>
+      </c>
+      <c r="D296" s="2" t="inlineStr">
+        <is>
+          <t>1/99</t>
+        </is>
+      </c>
+      <c r="E296" s="2" t="inlineStr">
+        <is>
+          <t>001 of 99</t>
+        </is>
+      </c>
+      <c r="F296" s="2" t="inlineStr">
+        <is>
+          <t>9.99 USD</t>
+        </is>
+      </c>
+      <c r="G296" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366674866557</t>
+        </is>
+      </c>
+      <c r="H296" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:06 UTC</t>
+        </is>
+      </c>
+      <c r="I296" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/57gAAeSwANVqrAlC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J296" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T03:50:01.000Z</t>
+        </is>
+      </c>
+      <c r="K296" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L296" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M296" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N296" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vlsAAeSwLcNqrAlG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O296" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P296" s="2" t="inlineStr"/>
+      <c r="Q296" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R296" s="2" t="inlineStr"/>
+      <c r="S296" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="2" t="inlineStr">
+        <is>
+          <t>Louisa Chirico</t>
+        </is>
+      </c>
+      <c r="B297" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - [Base] - Blue Refractor</t>
+        </is>
+      </c>
+      <c r="C297" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Blue Refractor 150/150 Louisa Chirico #204 Rookie RC 17uv</t>
+        </is>
+      </c>
+      <c r="D297" s="2" t="inlineStr">
+        <is>
+          <t>150/150</t>
+        </is>
+      </c>
+      <c r="E297" s="2" t="inlineStr">
+        <is>
+          <t>last of 150 (150/150)</t>
+        </is>
+      </c>
+      <c r="F297" s="2" t="inlineStr">
+        <is>
+          <t>3.12 USD</t>
+        </is>
+      </c>
+      <c r="G297" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336806425630</t>
+        </is>
+      </c>
+      <c r="H297" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I297" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/yCEAAeSwFXJqsfLs/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J297" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T03:14:54.000Z</t>
+        </is>
+      </c>
+      <c r="K297" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L297" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M297" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N297" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Cm0AAeSwnLRqsfLt/s-l1600.jpg | https://i.ebayimg.com/images/g/8woAAeSwP-hqsfLt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O297" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P297" s="2" t="inlineStr"/>
+      <c r="Q297" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R297" s="2" t="inlineStr"/>
+      <c r="S297" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="2" t="inlineStr">
+        <is>
+          <t>Christopher O'Connell</t>
+        </is>
+      </c>
+      <c r="B298" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - [Base] - Pink Geometric Refractor</t>
+        </is>
+      </c>
+      <c r="C298" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Pink Geometric Refractor 65/65 Christopher O'Connell #96 17uv</t>
+        </is>
+      </c>
+      <c r="D298" s="2" t="inlineStr">
+        <is>
+          <t>65/65</t>
+        </is>
+      </c>
+      <c r="E298" s="2" t="inlineStr">
+        <is>
+          <t>last of 65 (65/65)</t>
+        </is>
+      </c>
+      <c r="F298" s="2" t="inlineStr">
+        <is>
+          <t>6.57 USD</t>
+        </is>
+      </c>
+      <c r="G298" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336806423242</t>
+        </is>
+      </c>
+      <c r="H298" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I298" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2w0AAeSwZsZqsfKL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J298" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T03:13:15.000Z</t>
+        </is>
+      </c>
+      <c r="K298" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L298" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M298" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N298" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/1AkAAeSwSkFqsfKL/s-l1600.jpg | https://i.ebayimg.com/images/g/MO0AAeSwtMVqsfKL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O298" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P298" s="2" t="inlineStr"/>
+      <c r="Q298" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R298" s="2" t="inlineStr"/>
+      <c r="S298" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="2" t="inlineStr">
+        <is>
+          <t>Heather Watson</t>
+        </is>
+      </c>
+      <c r="B299" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - Autographs I - Purple Geometric Refractor</t>
+        </is>
+      </c>
+      <c r="C299" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome I Purple Geometric Refractor 10/10 Heather Watson Auto 1hn7</t>
+        </is>
+      </c>
+      <c r="D299" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E299" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F299" s="2" t="inlineStr">
+        <is>
+          <t>16.35 USD</t>
+        </is>
+      </c>
+      <c r="G299" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336806423086</t>
+        </is>
+      </c>
+      <c r="H299" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I299" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/CJ0AAeSwGClqsfKI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J299" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T03:13:12.000Z</t>
+        </is>
+      </c>
+      <c r="K299" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L299" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M299" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N299" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/yqoAAeSwuQZqsfKI/s-l1600.jpg | https://i.ebayimg.com/images/g/-w0AAeSw04pqsfKI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O299" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P299" s="2" t="inlineStr"/>
+      <c r="Q299" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R299" s="2" t="inlineStr"/>
+      <c r="S299" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="2" t="inlineStr">
+        <is>
+          <t>Ugo Humbert</t>
+        </is>
+      </c>
+      <c r="B300" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C300" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis Ugo Humbert 1st Gold Sapphire 50/50 # 101</t>
+        </is>
+      </c>
+      <c r="D300" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E300" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F300" s="2" t="inlineStr">
+        <is>
+          <t>29.99 USD</t>
+        </is>
+      </c>
+      <c r="G300" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366670277968</t>
+        </is>
+      </c>
+      <c r="H300" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I300" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-NwAAeSwBuBqqRdP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J300" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T02:25:01.000Z</t>
+        </is>
+      </c>
+      <c r="K300" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L300" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M300" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N300" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/u2oAAeSwSaNqqRdR/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O300" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P300" s="2" t="inlineStr"/>
+      <c r="Q300" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R300" s="2" t="inlineStr"/>
+      <c r="S300" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="2" t="inlineStr">
+        <is>
+          <t>Yannick Hanfmann</t>
+        </is>
+      </c>
+      <c r="B301" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C301" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis Yannick Hanfmann 1st Blue Refractor 001/250 # 63</t>
+        </is>
+      </c>
+      <c r="D301" s="2" t="inlineStr">
+        <is>
+          <t>1/250</t>
+        </is>
+      </c>
+      <c r="E301" s="2" t="inlineStr">
+        <is>
+          <t>001 of 250</t>
+        </is>
+      </c>
+      <c r="F301" s="2" t="inlineStr">
+        <is>
+          <t>9.99 USD</t>
+        </is>
+      </c>
+      <c r="G301" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366669885963</t>
+        </is>
+      </c>
+      <c r="H301" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I301" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bBoAAeSwLcNqqNxo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J301" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T02:05:01.000Z</t>
+        </is>
+      </c>
+      <c r="K301" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L301" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M301" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N301" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/I5IAAeSwwelqqNxq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O301" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P301" s="2" t="inlineStr"/>
+      <c r="Q301" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R301" s="2" t="inlineStr"/>
+      <c r="S301" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="2" t="inlineStr">
+        <is>
+          <t>Margaret Smith Court/Chris Evert</t>
+        </is>
+      </c>
+      <c r="B302" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Chrome Battle of the Baseline</t>
+        </is>
+      </c>
+      <c r="C302" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Battle Margaret Smith Court Chris Evert Superfractor 1/1</t>
+        </is>
+      </c>
+      <c r="D302" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E302" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F302" s="2" t="inlineStr">
+        <is>
+          <t>849.99 USD</t>
+        </is>
+      </c>
+      <c r="G302" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/158319065090</t>
+        </is>
+      </c>
+      <c r="H302" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I302" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/1CgAAeSw7U5qseC6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J302" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T02:00:07.000Z</t>
+        </is>
+      </c>
+      <c r="K302" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L302" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M302" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N302" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/J~0AAeSwnyhqseC6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O302" s="2" t="inlineStr"/>
+      <c r="P302" s="2" t="inlineStr"/>
+      <c r="Q302" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R302" s="2" t="inlineStr"/>
+      <c r="S302" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="2" t="inlineStr">
+        <is>
+          <t>Hubert Hurkacz</t>
+        </is>
+      </c>
+      <c r="B303" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS CHROME SAPPHIRE TENNIS</t>
+        </is>
+      </c>
+      <c r="C303" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS CHROME SAPPHIRE TENNIS GOLD #125 HUBERT HURKACZ 1/50 PSA 9</t>
+        </is>
+      </c>
+      <c r="D303" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E303" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F303" s="2" t="inlineStr">
+        <is>
+          <t>129.00 USD</t>
+        </is>
+      </c>
+      <c r="G303" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298679346254</t>
+        </is>
+      </c>
+      <c r="H303" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I303" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/qgAAAeSw2uxqqmlV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J303" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T01:52:00.000Z</t>
+        </is>
+      </c>
+      <c r="K303" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L303" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M303" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N303" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/MZAAAeSwFVVqqmlU/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O303" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P303" s="2" t="inlineStr"/>
+      <c r="Q303" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R303" s="2" t="inlineStr"/>
+      <c r="S303" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="2" t="inlineStr">
+        <is>
+          <t>Martin Landaluce</t>
+        </is>
+      </c>
+      <c r="B304" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C304" s="2" t="inlineStr">
+        <is>
+          <t>Martin Landaluce 2024 Topps Chrome Gold Refractor RC Autograph Auto #'d 1/50</t>
+        </is>
+      </c>
+      <c r="D304" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E304" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F304" s="2" t="inlineStr">
+        <is>
+          <t>99.99 USD</t>
+        </is>
+      </c>
+      <c r="G304" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/206573097516</t>
+        </is>
+      </c>
+      <c r="H304" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I304" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/cBMAAeSwf9tqsdHt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J304" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T01:00:01.000Z</t>
+        </is>
+      </c>
+      <c r="K304" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L304" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M304" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N304" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/oCMAAeSwR7VqsdHu/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O304" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P304" s="2" t="inlineStr"/>
+      <c r="Q304" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R304" s="2" t="inlineStr"/>
+      <c r="S304" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="2" t="inlineStr">
+        <is>
+          <t>Alexandra Eala</t>
+        </is>
+      </c>
+      <c r="B305" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C305" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Alexandra Eala Autograph Red Refractor #1/5</t>
+        </is>
+      </c>
+      <c r="D305" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E305" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F305" s="2" t="inlineStr">
+        <is>
+          <t>511.00 USD</t>
+        </is>
+      </c>
+      <c r="G305" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/128090815134</t>
+        </is>
+      </c>
+      <c r="H305" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I305" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jJgAAeSwXYxqsOSG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J305" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T00:00:00.000Z</t>
+        </is>
+      </c>
+      <c r="K305" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L305" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M305" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N305" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/fX0AAeSwKYJqsOSG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O305" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P305" s="2" t="inlineStr"/>
+      <c r="Q305" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R305" s="2" t="inlineStr"/>
+      <c r="S305" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="2" t="inlineStr">
+        <is>
+          <t>Sofia Kenin</t>
+        </is>
+      </c>
+      <c r="B306" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C306" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Court Masters Pink Refractor 1/15 Sofia Kenin Rookie RC 0v2</t>
+        </is>
+      </c>
+      <c r="D306" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E306" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F306" s="2" t="inlineStr">
+        <is>
+          <t>23.83 USD</t>
+        </is>
+      </c>
+      <c r="G306" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257757587527</t>
+        </is>
+      </c>
+      <c r="H306" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I306" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/WbcAAeSwVXhqsdNh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J306" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T01:00:11.000Z</t>
+        </is>
+      </c>
+      <c r="K306" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L306" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M306" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N306" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/CRkAAeSwMaJqsdNh/s-l1600.jpg | https://i.ebayimg.com/images/g/X3UAAeSwUERqsdNh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O306" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P306" s="2" t="inlineStr"/>
+      <c r="Q306" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R306" s="2" t="inlineStr"/>
+      <c r="S306" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Nadal</t>
+        </is>
+      </c>
+      <c r="B307" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C307" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Rafael Nadal Match Masters Red Refractor #1/1 PSA 10</t>
+        </is>
+      </c>
+      <c r="D307" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E307" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F307" s="2" t="inlineStr">
+        <is>
+          <t>255.00 USD</t>
+        </is>
+      </c>
+      <c r="G307" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377513027705</t>
+        </is>
+      </c>
+      <c r="H307" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I307" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ypQAAeSwqrhqsUTT/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J307" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T00:30:00.000Z</t>
+        </is>
+      </c>
+      <c r="K307" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L307" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M307" s="2" t="inlineStr">
+        <is>
+          <t>PSA 10</t>
+        </is>
+      </c>
+      <c r="N307" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/y-AAAeSwKZ9qsUTT/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O307" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P307" s="2" t="inlineStr"/>
+      <c r="Q307" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R307" s="2" t="inlineStr"/>
+      <c r="S307" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="2" t="inlineStr">
+        <is>
+          <t>Caty Mcnally</t>
+        </is>
+      </c>
+      <c r="B308" s="2" t="inlineStr">
+        <is>
+          <t>TOPPS / GRAPHITE</t>
+        </is>
+      </c>
+      <c r="C308" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS GRAPHITE CATY MCNALLY RED CRYSTALLINE 1/1 INSCRIPTION AUTO "MY 1ST"</t>
+        </is>
+      </c>
+      <c r="D308" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E308" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F308" s="2" t="inlineStr">
+        <is>
+          <t>999.99 USD</t>
+        </is>
+      </c>
+      <c r="G308" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/188961840269</t>
+        </is>
+      </c>
+      <c r="H308" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I308" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/s5gAAeSwdIRqscJY/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J308" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21T23:47:33.000Z</t>
+        </is>
+      </c>
+      <c r="K308" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L308" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M308" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N308" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/na8AAeSw2DJqscJZ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O308" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P308" s="2" t="inlineStr"/>
+      <c r="Q308" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R308" s="2" t="inlineStr"/>
+      <c r="S308" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="2" t="inlineStr"/>
+      <c r="B309" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C309" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite - Match Point Marks Karen Khachanov Pink Refractor 1/15 (AU)</t>
+        </is>
+      </c>
+      <c r="D309" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E309" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F309" s="2" t="inlineStr">
+        <is>
+          <t>75.00 USD</t>
+        </is>
+      </c>
+      <c r="G309" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237082612083</t>
+        </is>
+      </c>
+      <c r="H309" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I309" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/xE0AAeSwfUpqsbAS/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J309" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21T22:32:19.000Z</t>
+        </is>
+      </c>
+      <c r="K309" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L309" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M309" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N309" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jvYAAeSwDTZqsbAS/s-l1600.jpg | https://i.ebayimg.com/images/g/1UAAAeSwSkFqsbAS/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O309" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P309" s="2" t="inlineStr"/>
+      <c r="Q309" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R309" s="2" t="inlineStr"/>
+      <c r="S309" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="2" t="inlineStr">
+        <is>
+          <t>Shintaro Mochizuki</t>
+        </is>
+      </c>
+      <c r="B310" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Imperial Ink - Gold</t>
+        </is>
+      </c>
+      <c r="C310" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Imperial Ink Gold 1/10 Shintaro Mochizuki Rookie Auto RC 1e41</t>
+        </is>
+      </c>
+      <c r="D310" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E310" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F310" s="2" t="inlineStr">
+        <is>
+          <t>115.24 USD</t>
+        </is>
+      </c>
+      <c r="G310" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336807063322</t>
+        </is>
+      </c>
+      <c r="H310" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I310" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/eqUAAeSwheFqsmC1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J310" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T11:03:15.000Z</t>
+        </is>
+      </c>
+      <c r="K310" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L310" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M310" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N310" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/eh4AAeSw7F1qsmC1/s-l1600.jpg | https://i.ebayimg.com/images/g/obYAAeSw1D5qsmC0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O310" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P310" s="2" t="inlineStr"/>
+      <c r="Q310" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R310" s="2" t="inlineStr"/>
+      <c r="S310" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="2" t="inlineStr">
+        <is>
+          <t>Sloane Stephens</t>
+        </is>
+      </c>
+      <c r="B311" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Royalty Collection Tennis</t>
+        </is>
+      </c>
+      <c r="C311" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2024 Royalty Collection Tennis Sloane Stephens Auto 1/1</t>
+        </is>
+      </c>
+      <c r="D311" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E311" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F311" s="2" t="inlineStr">
+        <is>
+          <t>447.14 USD</t>
+        </is>
+      </c>
+      <c r="G311" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147590973504</t>
+        </is>
+      </c>
+      <c r="H311" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I311" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/UpEAAeSwuxFqsly7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J311" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T10:50:19.000Z</t>
+        </is>
+      </c>
+      <c r="K311" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L311" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M311" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N311" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SfMAAeSwKelqslzA/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O311" s="2" t="inlineStr"/>
+      <c r="P311" s="2" t="inlineStr"/>
+      <c r="Q311" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R311" s="2" t="inlineStr"/>
+      <c r="S311" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="2" t="inlineStr">
+        <is>
+          <t>Emma Raducanu</t>
+        </is>
+      </c>
+      <c r="B312" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - [Base] - Green</t>
+        </is>
+      </c>
+      <c r="C312" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Green 5/5 Emma Raducanu #26 0q3g</t>
+        </is>
+      </c>
+      <c r="D312" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E312" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F312" s="2" t="inlineStr">
+        <is>
+          <t>262.99 USD</t>
+        </is>
+      </c>
+      <c r="G312" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336806759569</t>
+        </is>
+      </c>
+      <c r="H312" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I312" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/1HQAAeSwzslqsizQ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J312" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T07:21:51.000Z</t>
+        </is>
+      </c>
+      <c r="K312" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L312" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M312" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N312" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/p5EAAeSwfANqsizQ/s-l1600.jpg | https://i.ebayimg.com/images/g/2ekAAeSwLMRqsizQ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O312" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P312" s="2" t="inlineStr"/>
+      <c r="Q312" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R312" s="2" t="inlineStr"/>
+      <c r="S312" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="2" t="inlineStr">
+        <is>
+          <t>Andre Agassi</t>
+        </is>
+      </c>
+      <c r="B313" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Tennis</t>
+        </is>
+      </c>
+      <c r="C313" s="2" t="inlineStr">
+        <is>
+          <t>Andre Agassi 🇺🇸 #1/1 Platinum Ambassador Autographs--2024 Topps Royalty PSA 10</t>
+        </is>
+      </c>
+      <c r="D313" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E313" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F313" s="2" t="inlineStr">
+        <is>
+          <t>9999.95 USD</t>
+        </is>
+      </c>
+      <c r="G313" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178517749661?amdata=enc%3AAQALAAAAsCHNgUiiE%2FjQhlDTaMiAde81W79qS77k%2F4OvNjFs6Is85Gt8v0VOfhQWEUmOQ6Jzj8W0lLFel4nLbSnNrWvHUcpegN9NxGivhf2xHemnCD2MFP2ZgyByevvcX41clXi0QxbN7vJi24MQ%2F4mOEAaH%2B%2FP7ucBxAy9%2FhFPHIrLJljlaLLWFCLm4iUbFXEo525sYaZYM4Wv1lqvfOZ9bKql3Wsv7iaFEnFfIuVAqQquPZt8N</t>
+        </is>
+      </c>
+      <c r="H313" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I313" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/iy0AAeSwjQtqsfUB/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J313" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T03:53:23.000Z</t>
+        </is>
+      </c>
+      <c r="K313" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L313" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M313" s="2" t="inlineStr">
+        <is>
+          <t>PSA 10</t>
+        </is>
+      </c>
+      <c r="N313" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/b00AAeSwPD5qsfVH/s-l1600.jpg | https://i.ebayimg.com/images/g/MrcAAeSwqrhqsfUA/s-l1600.jpg | https://i.ebayimg.com/images/g/2M0AAeSwSbhqsfUB/s-l1600.jpg | https://i.ebayimg.com/images/g/JlUAAeSwuXtqsfUB/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O313" s="2" t="inlineStr"/>
+      <c r="P313" s="2" t="inlineStr"/>
+      <c r="Q313" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R313" s="2" t="inlineStr"/>
+      <c r="S313" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="2" t="inlineStr">
+        <is>
+          <t>Otto Virtanen</t>
+        </is>
+      </c>
+      <c r="B314" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Royalty Collection</t>
+        </is>
+      </c>
+      <c r="C314" s="2" t="inlineStr">
+        <is>
+          <t>Otto Virtanen 2024 Topps Royalty #TRS-OV Green Triumph Patch Auto 1/5</t>
+        </is>
+      </c>
+      <c r="D314" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E314" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F314" s="2" t="inlineStr">
+        <is>
+          <t>99.99 USD</t>
+        </is>
+      </c>
+      <c r="G314" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/158315213383</t>
+        </is>
+      </c>
+      <c r="H314" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I314" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/A8cAAeSwtMVqsIQl/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J314" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21T18:20:21.000Z</t>
+        </is>
+      </c>
+      <c r="K314" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L314" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M314" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N314" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/zm0AAeSwZBRqsIQl/s-l1600.jpg | https://i.ebayimg.com/images/g/zoYAAeSweGhqsIQl/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O314" s="2" t="inlineStr"/>
+      <c r="P314" s="2" t="inlineStr"/>
+      <c r="Q314" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R314" s="2" t="inlineStr"/>
+      <c r="S314" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="2" t="inlineStr">
+        <is>
+          <t>Jamie Murray</t>
+        </is>
+      </c>
+      <c r="B315" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps</t>
+        </is>
+      </c>
+      <c r="C315" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty -----JAMIE MURRAY-----SUPERIOR RELIC SIGNATURES--5/5 BOOKEND</t>
+        </is>
+      </c>
+      <c r="D315" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E315" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F315" s="2" t="inlineStr">
+        <is>
+          <t>77.99 USD</t>
+        </is>
+      </c>
+      <c r="G315" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/278396002958?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8uXd28409YwYuHqR1TAvMhL52SxMYB70WGlNuaUdRmbRJfV4bRoZgu6L4B4XV4HIuB1c5cPhnCdaHDflF3JSITtnEPQpEdeXjv3OL4hzNJ%2Fe57Z7xvFzhEk4tuQYjR2PIGgi2p94sOD4HdaOIk4mbvUcvl7UbmfZ7A9kEXUUYpRuqGRKuH%2F8VC3zXyJVeoAlA%3D</t>
+        </is>
+      </c>
+      <c r="H315" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:07 UTC</t>
+        </is>
+      </c>
+      <c r="I315" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/R0oAAeSwnJNqsVQN/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J315" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21T16:00:17.000Z</t>
+        </is>
+      </c>
+      <c r="K315" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L315" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M315" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N315" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gdcAAeSw21dqsVQA/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O315" s="2" t="inlineStr"/>
+      <c r="P315" s="2" t="inlineStr"/>
+      <c r="Q315" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R315" s="2" t="inlineStr"/>
+      <c r="S315" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -26153,6 +28083,28 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G291" r:id="rId290"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G292" r:id="rId291"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G293" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G294" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G295" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G296" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G297" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G298" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G299" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G300" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G301" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G302" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G303" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G304" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G305" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G306" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G307" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G308" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G309" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G310" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G311" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G312" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G313" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G314" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G315" r:id="rId314"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-23 08:47 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S315"/>
+  <dimension ref="A1:S336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -27784,6 +27784,1839 @@
       </c>
       <c r="R315" s="2" t="inlineStr"/>
       <c r="S315" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="2" t="inlineStr">
+        <is>
+          <t>Taylor Fritz</t>
+        </is>
+      </c>
+      <c r="B316" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 TOPPS CHROME TENNIS CAPTURED</t>
+        </is>
+      </c>
+      <c r="C316" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS CAPTURED RED REFRACTOR #CTD-22 TAYLOR FRITZ 5/5 PSA 9</t>
+        </is>
+      </c>
+      <c r="D316" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E316" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F316" s="2" t="inlineStr">
+        <is>
+          <t>159.99 USD</t>
+        </is>
+      </c>
+      <c r="G316" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117426587519</t>
+        </is>
+      </c>
+      <c r="H316" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I316" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/LuwAAeSwuAVqs1to/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J316" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23T04:52:56.000Z</t>
+        </is>
+      </c>
+      <c r="K316" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L316" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M316" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N316" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HpUAAeSwXG1qs1to/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O316" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P316" s="2" t="inlineStr"/>
+      <c r="Q316" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R316" s="2" t="inlineStr"/>
+      <c r="S316" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="2" t="inlineStr">
+        <is>
+          <t>Mayar Sherif</t>
+        </is>
+      </c>
+      <c r="B317" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Chrome</t>
+        </is>
+      </c>
+      <c r="C317" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome MAYAR SHERIF 2/2 Black Geometric Refractor #121</t>
+        </is>
+      </c>
+      <c r="D317" s="2" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="E317" s="2" t="inlineStr">
+        <is>
+          <t>last of 2 (2/2)</t>
+        </is>
+      </c>
+      <c r="F317" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G317" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307191765968</t>
+        </is>
+      </c>
+      <c r="H317" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I317" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/b00AAeSwICxqsevf/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J317" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23T03:54:00.000Z</t>
+        </is>
+      </c>
+      <c r="K317" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L317" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M317" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N317" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/63wAAeSwYllqsevf/s-l1600.jpg | https://i.ebayimg.com/images/g/BpYAAeSwo-lqsevf/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O317" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P317" s="2" t="inlineStr"/>
+      <c r="Q317" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R317" s="2" t="inlineStr"/>
+      <c r="S317" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="2" t="inlineStr">
+        <is>
+          <t>Harry Wendelken</t>
+        </is>
+      </c>
+      <c r="B318" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Chrome</t>
+        </is>
+      </c>
+      <c r="C318" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome HARRY WENDELKEN 50/50 Bookend RC Auto Gold Refractor #TCA-HWN</t>
+        </is>
+      </c>
+      <c r="D318" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E318" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F318" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G318" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307191765693</t>
+        </is>
+      </c>
+      <c r="H318" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I318" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/qkcAAeSweP9qsevc/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J318" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23T03:39:00.000Z</t>
+        </is>
+      </c>
+      <c r="K318" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L318" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M318" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N318" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YKoAAeSwax1qsevc/s-l1600.jpg | https://i.ebayimg.com/images/g/rt0AAeSw4~Bqsevc/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O318" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P318" s="2" t="inlineStr"/>
+      <c r="Q318" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R318" s="2" t="inlineStr"/>
+      <c r="S318" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="2" t="inlineStr">
+        <is>
+          <t>Venus Williams</t>
+        </is>
+      </c>
+      <c r="B319" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Chrome</t>
+        </is>
+      </c>
+      <c r="C319" s="2" t="inlineStr">
+        <is>
+          <t>Venus Williams 2024 Topps Chrome #200 Purple Refractor 499/499</t>
+        </is>
+      </c>
+      <c r="D319" s="2" t="inlineStr">
+        <is>
+          <t>499/499</t>
+        </is>
+      </c>
+      <c r="E319" s="2" t="inlineStr">
+        <is>
+          <t>last of 499 (499/499)</t>
+        </is>
+      </c>
+      <c r="F319" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G319" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/158325423670</t>
+        </is>
+      </c>
+      <c r="H319" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I319" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0zkAAeSw7k9qsvgH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J319" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:36:00.000Z</t>
+        </is>
+      </c>
+      <c r="K319" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L319" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M319" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N319" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Se4AAeSwvchqsvgH/s-l1600.jpg | https://i.ebayimg.com/images/g/Mi0AAeSw8lpqsvgI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O319" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P319" s="2" t="inlineStr"/>
+      <c r="Q319" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R319" s="2" t="inlineStr"/>
+      <c r="S319" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="2" t="inlineStr">
+        <is>
+          <t>Jelena Ostapenko</t>
+        </is>
+      </c>
+      <c r="B320" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C320" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Jelena Ostapenko Captured Green Geometric REF 1/75 TT07</t>
+        </is>
+      </c>
+      <c r="D320" s="2" t="inlineStr">
+        <is>
+          <t>1/75</t>
+        </is>
+      </c>
+      <c r="E320" s="2" t="inlineStr">
+        <is>
+          <t>001 of 75</t>
+        </is>
+      </c>
+      <c r="F320" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G320" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407237941160</t>
+        </is>
+      </c>
+      <c r="H320" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I320" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/a8gAAeSwaOxqsznt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J320" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:30:02.000Z</t>
+        </is>
+      </c>
+      <c r="K320" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L320" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M320" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N320" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/aWwAAeSweaVqsznx/s-l1600.jpg | https://i.ebayimg.com/images/g/RR4AAeSwc7dqsznq/s-l1600.jpg | https://i.ebayimg.com/images/g/SZ4AAeSwTH9qsznq/s-l1600.jpg | https://i.ebayimg.com/images/g/5FkAAeSwqBVqsznp/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O320" s="2" t="inlineStr"/>
+      <c r="P320" s="2" t="inlineStr"/>
+      <c r="Q320" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R320" s="2" t="inlineStr"/>
+      <c r="S320" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="2" t="inlineStr">
+        <is>
+          <t>Katie Volynets</t>
+        </is>
+      </c>
+      <c r="B321" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C321" s="2" t="inlineStr">
+        <is>
+          <t>Topps Chrome Tennis Katie Volynets #217  1/50 Gold</t>
+        </is>
+      </c>
+      <c r="D321" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E321" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F321" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G321" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117426344281</t>
+        </is>
+      </c>
+      <c r="H321" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I321" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/H44AAeSwKzpqsx4U/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J321" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23T00:32:43.000Z</t>
+        </is>
+      </c>
+      <c r="K321" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L321" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M321" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N321" s="2" t="inlineStr"/>
+      <c r="O321" s="2" t="inlineStr"/>
+      <c r="P321" s="2" t="inlineStr"/>
+      <c r="Q321" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R321" s="2" t="inlineStr"/>
+      <c r="S321" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="2" t="inlineStr">
+        <is>
+          <t>Flavio Cobolli</t>
+        </is>
+      </c>
+      <c r="B322" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C322" s="2" t="inlineStr">
+        <is>
+          <t>Flavio Cobolli 2025 Topps Chrome Tennis Youthquake Superfractor RC #YQE17 1/1</t>
+        </is>
+      </c>
+      <c r="D322" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E322" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F322" s="2" t="inlineStr">
+        <is>
+          <t>2999.99 USD</t>
+        </is>
+      </c>
+      <c r="G322" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366685949977</t>
+        </is>
+      </c>
+      <c r="H322" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I322" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/v~MAAeSwwD1qsxTB/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J322" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T23:46:25.000Z</t>
+        </is>
+      </c>
+      <c r="K322" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L322" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M322" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N322" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TTMAAeSwaqpqsxTB/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O322" s="2" t="inlineStr"/>
+      <c r="P322" s="2" t="inlineStr"/>
+      <c r="Q322" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R322" s="2" t="inlineStr"/>
+      <c r="S322" s="2" t="inlineStr">
+        <is>
+          <t>Baseball</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="2" t="inlineStr">
+        <is>
+          <t>Maximilian Marterer</t>
+        </is>
+      </c>
+      <c r="B323" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C323" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2025 Topps Chrome Maximilian Marterer Tennis #160 Serial Numbered 05/05</t>
+        </is>
+      </c>
+      <c r="D323" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E323" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F323" s="2" t="inlineStr">
+        <is>
+          <t>1.99 USD</t>
+        </is>
+      </c>
+      <c r="G323" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/398421962313</t>
+        </is>
+      </c>
+      <c r="H323" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I323" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/qS0AAeSw2i9qstND/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J323" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T22:21:37.000Z</t>
+        </is>
+      </c>
+      <c r="K323" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L323" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M323" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N323" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/49IAAeSwZv9qstND/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O323" s="2" t="inlineStr"/>
+      <c r="P323" s="2" t="inlineStr"/>
+      <c r="Q323" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R323" s="2" t="inlineStr"/>
+      <c r="S323" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="2" t="inlineStr">
+        <is>
+          <t>Grigor Dimitrov</t>
+        </is>
+      </c>
+      <c r="B324" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C324" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Grigor Dimitrov Superfractor 1/1 Auto #CA-GDV</t>
+        </is>
+      </c>
+      <c r="D324" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E324" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F324" s="2" t="inlineStr">
+        <is>
+          <t>1499.99 USD</t>
+        </is>
+      </c>
+      <c r="G324" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287602242602</t>
+        </is>
+      </c>
+      <c r="H324" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I324" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/OvEAAeSwHJ5qss95/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J324" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T18:57:30.000Z</t>
+        </is>
+      </c>
+      <c r="K324" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L324" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M324" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N324" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/aqUAAeSwfAZqss95/s-l1600.jpg | https://i.ebayimg.com/images/g/7t4AAeSw185qss96/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O324" s="2" t="inlineStr"/>
+      <c r="P324" s="2" t="inlineStr"/>
+      <c r="Q324" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R324" s="2" t="inlineStr"/>
+      <c r="S324" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="2" t="inlineStr">
+        <is>
+          <t>Gabriel Diallo</t>
+        </is>
+      </c>
+      <c r="B325" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C325" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS Gabriel Diallo  # 1/2 BLACK GEOMETRIC REFRACTOR</t>
+        </is>
+      </c>
+      <c r="D325" s="2" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="E325" s="2" t="inlineStr">
+        <is>
+          <t>001 of 2</t>
+        </is>
+      </c>
+      <c r="F325" s="2" t="inlineStr">
+        <is>
+          <t>100.00 USD</t>
+        </is>
+      </c>
+      <c r="G325" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117425750252?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2B87ek6GHzFF6A4Hv6OrQUVan%2F9lUGvdaIm06hfofuNA%2F3ZzibG697XxI6FmQ2Hyt2NKyRfLp1OH0ykY1o11AIj%2BnQGIlWoP98qhiOKbqk9R13x0F65kJW%2BlD4Kh3HVTEqObJ4TtTU0kPehG4OCtP2KUGq7s3aEOuJP52hTANVnSzIqSEW6WmUbmDGBsJQWaww%3D</t>
+        </is>
+      </c>
+      <c r="H325" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I325" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/wJoAAeSwrzppyS7-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J325" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T15:52:15.000Z</t>
+        </is>
+      </c>
+      <c r="K325" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L325" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M325" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N325" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/K-gAAeSw0z9pyS7-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O325" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P325" s="2" t="inlineStr"/>
+      <c r="Q325" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R325" s="2" t="inlineStr"/>
+      <c r="S325" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="2" t="inlineStr">
+        <is>
+          <t>Holger Rune</t>
+        </is>
+      </c>
+      <c r="B326" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C326" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Holger Rune Youthquake Red Refractor Auto 5/5 #YS-HG</t>
+        </is>
+      </c>
+      <c r="D326" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E326" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F326" s="2" t="inlineStr">
+        <is>
+          <t>399.99 USD</t>
+        </is>
+      </c>
+      <c r="G326" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287601934844</t>
+        </is>
+      </c>
+      <c r="H326" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I326" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TVcAAeSwBSZqsp5u/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J326" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T15:28:36.000Z</t>
+        </is>
+      </c>
+      <c r="K326" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L326" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M326" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N326" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/P90AAeSwrONqsp5u/s-l1600.jpg | https://i.ebayimg.com/images/g/lZ4AAeSw4R1qsp5u/s-l1600.jpg | https://i.ebayimg.com/images/g/THYAAeSwshlqsp5u/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O326" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P326" s="2" t="inlineStr"/>
+      <c r="Q326" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R326" s="2" t="inlineStr"/>
+      <c r="S326" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="2" t="inlineStr">
+        <is>
+          <t>Julia Riera</t>
+        </is>
+      </c>
+      <c r="B327" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C327" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Julia Riera RC Black Geometric 1/2</t>
+        </is>
+      </c>
+      <c r="D327" s="2" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="E327" s="2" t="inlineStr">
+        <is>
+          <t>001 of 2</t>
+        </is>
+      </c>
+      <c r="F327" s="2" t="inlineStr">
+        <is>
+          <t>150.00 USD</t>
+        </is>
+      </c>
+      <c r="G327" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117425693127?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2FoZSS%2BuwO074kmoMFEIKe9mdySc4sLQShFPwewSCIxVG960nL%2F66D1Vnr%2BjhJp%2FXiA7obPmvDpjYc6z6VcW%2FzziQUMsAqzGyd7Mw2xpKmnKfeRkAwx9Bmgh4fao9s1O%2BTjeqQ9bpIzAXRxlIGCWo7uc5IL8%2F7J3ZUhFqygFjNdCyRYe7KwJDhukvV7iZ6y%2FTk%3D</t>
+        </is>
+      </c>
+      <c r="H327" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I327" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SokAAeSwnPZplzsi/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J327" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T15:19:31.000Z</t>
+        </is>
+      </c>
+      <c r="K327" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L327" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M327" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N327" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XYsAAeSwLYRplzsi/s-l1600.jpg | https://i.ebayimg.com/images/g/TNAAAeSwvSNplzsh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O327" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P327" s="2" t="inlineStr"/>
+      <c r="Q327" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R327" s="2" t="inlineStr"/>
+      <c r="S327" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="2" t="inlineStr">
+        <is>
+          <t>Benoit Paire</t>
+        </is>
+      </c>
+      <c r="B328" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Chrome</t>
+        </is>
+      </c>
+      <c r="C328" s="2" t="inlineStr">
+        <is>
+          <t>Benoit Paire 2025 Topps Chrome Tennis #TCA-BPE Auto Black Refractor 01/10</t>
+        </is>
+      </c>
+      <c r="D328" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E328" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F328" s="2" t="inlineStr">
+        <is>
+          <t>15.00 USD</t>
+        </is>
+      </c>
+      <c r="G328" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117425686116</t>
+        </is>
+      </c>
+      <c r="H328" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I328" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/CIcAAeSwZQNqmZnL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J328" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T15:12:53.000Z</t>
+        </is>
+      </c>
+      <c r="K328" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L328" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M328" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N328" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ddwAAeSwcztqmZnL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O328" s="2" t="inlineStr">
+        <is>
+          <t>rose</t>
+        </is>
+      </c>
+      <c r="P328" s="2" t="inlineStr"/>
+      <c r="Q328" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R328" s="2" t="inlineStr"/>
+      <c r="S328" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="2" t="inlineStr">
+        <is>
+          <t>Marta Kostyuk</t>
+        </is>
+      </c>
+      <c r="B329" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C329" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis Marta Kostyuk Blue Refractor Auto 250/250</t>
+        </is>
+      </c>
+      <c r="D329" s="2" t="inlineStr">
+        <is>
+          <t>250/250</t>
+        </is>
+      </c>
+      <c r="E329" s="2" t="inlineStr">
+        <is>
+          <t>last of 250 (250/250)</t>
+        </is>
+      </c>
+      <c r="F329" s="2" t="inlineStr">
+        <is>
+          <t>50.00 USD</t>
+        </is>
+      </c>
+      <c r="G329" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117425686247</t>
+        </is>
+      </c>
+      <c r="H329" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I329" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/obMAAeSwzbZqmZ1n/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J329" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T15:12:53.000Z</t>
+        </is>
+      </c>
+      <c r="K329" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L329" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M329" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N329" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/T0cAAeSwJFFqmZ1n/s-l1600.jpg | https://i.ebayimg.com/images/g/CbEAAeSww-FqmZ1n/s-l1600.jpg | https://i.ebayimg.com/images/g/glIAAeSwuQVqmZ1n/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O329" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P329" s="2" t="inlineStr"/>
+      <c r="Q329" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R329" s="2" t="inlineStr"/>
+      <c r="S329" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="2" t="inlineStr">
+        <is>
+          <t>Giovanni Mpetshi Perricard</t>
+        </is>
+      </c>
+      <c r="B330" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Graphite</t>
+        </is>
+      </c>
+      <c r="C330" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite GIOVANNI MPETSHI PERRICARD 1/10 White Refractor #47</t>
+        </is>
+      </c>
+      <c r="D330" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E330" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F330" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G330" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307191765652</t>
+        </is>
+      </c>
+      <c r="H330" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I330" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/a9sAAeSwgQNqsevk/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J330" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23T03:35:00.000Z</t>
+        </is>
+      </c>
+      <c r="K330" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L330" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M330" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N330" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/k1wAAeSwq8Rqsevl/s-l1600.jpg | https://i.ebayimg.com/images/g/GjwAAeSwjBpqsevl/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O330" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P330" s="2" t="inlineStr"/>
+      <c r="Q330" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R330" s="2" t="inlineStr"/>
+      <c r="S330" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="2" t="inlineStr">
+        <is>
+          <t>Coleman Wong</t>
+        </is>
+      </c>
+      <c r="B331" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C331" s="2" t="inlineStr">
+        <is>
+          <t>Coleman Wong 🇭🇰 RC | #15/15 Pink Rally Relics -- 2024 Topps Graphite 🎾 Rookie</t>
+        </is>
+      </c>
+      <c r="D331" s="2" t="inlineStr">
+        <is>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="E331" s="2" t="inlineStr">
+        <is>
+          <t>last of 15 (15/15)</t>
+        </is>
+      </c>
+      <c r="F331" s="2" t="inlineStr">
+        <is>
+          <t>29.95 USD</t>
+        </is>
+      </c>
+      <c r="G331" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178519555584?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2F4vCiagn%2Fm4ZyJzzOROSYwVd7jZMDl7IMcGfKu4ZG0MXs0yL0rMK6mpVr%2FVtKcgJu7TyyD%2BbA3MW40SPmahKMYALSJ3lAacOK5ebbkUwnjEp7DsMm9M1KEtoR%2BUFlNsL5c9exM6AgXKwRrtqQsJylCEkpC%2FPNd37QTd4Sx79phI5gLgZFJ%2Bh5o5pJrWboHDWY%3D</t>
+        </is>
+      </c>
+      <c r="H331" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I331" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/hu4AAeSw1ylqss7~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J331" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T18:55:31.000Z</t>
+        </is>
+      </c>
+      <c r="K331" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L331" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M331" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N331" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/LnEAAeSwcxxqss7~/s-l1600.jpg | https://i.ebayimg.com/images/g/jxYAAeSwuGtqss7~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O331" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P331" s="2" t="inlineStr"/>
+      <c r="Q331" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R331" s="2" t="inlineStr"/>
+      <c r="S331" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="2" t="inlineStr">
+        <is>
+          <t>Guilio Zeppieri</t>
+        </is>
+      </c>
+      <c r="B332" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C332" s="2" t="inlineStr">
+        <is>
+          <t>🎾 2024 Topps Graphite Tennis Red Crystalline Guilio Zeppieri 1/1</t>
+        </is>
+      </c>
+      <c r="D332" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E332" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F332" s="2" t="inlineStr">
+        <is>
+          <t>200.00 USD</t>
+        </is>
+      </c>
+      <c r="G332" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117425761630</t>
+        </is>
+      </c>
+      <c r="H332" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I332" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7QQAAeSwjWtqohSn/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J332" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T16:05:59.000Z</t>
+        </is>
+      </c>
+      <c r="K332" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L332" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M332" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N332" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-QgAAeSwB7RqohSn/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O332" s="2" t="inlineStr"/>
+      <c r="P332" s="2" t="inlineStr"/>
+      <c r="Q332" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R332" s="2" t="inlineStr"/>
+      <c r="S332" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="2" t="inlineStr">
+        <is>
+          <t>Xiyu Wang</t>
+        </is>
+      </c>
+      <c r="B333" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C333" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Xiyu Wang White Refractor #10/10</t>
+        </is>
+      </c>
+      <c r="D333" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E333" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F333" s="2" t="inlineStr">
+        <is>
+          <t>11.00 USD</t>
+        </is>
+      </c>
+      <c r="G333" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117425713034?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2BjdhQqayMR1rWxvJilwek8HcByXZxekvmKB8QF8nrtYWqsGJoCa%2FsSTjkv7x0vcKgcq2fkqTzsWnROQ9yesIonaL%2FvrbqkwFMbG57kJ02eaoEZCCFWeyphKKoHnAjtozqJC3UGHiDVeU%2FlqmSXjLR%2BGCZujpOhpfNdVHpYw5Rbx%2B%2B6RBitW4sO%2BfJpPuY9kjA%3D</t>
+        </is>
+      </c>
+      <c r="H333" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I333" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Q6gAAeSwXbdp1bHJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J333" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T15:30:33.000Z</t>
+        </is>
+      </c>
+      <c r="K333" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L333" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M333" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N333" s="2" t="inlineStr"/>
+      <c r="O333" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P333" s="2" t="inlineStr"/>
+      <c r="Q333" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R333" s="2" t="inlineStr"/>
+      <c r="S333" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="2" t="inlineStr">
+        <is>
+          <t>Cameron Norrie</t>
+        </is>
+      </c>
+      <c r="B334" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS GRAPHITE CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="C334" s="2" t="inlineStr">
+        <is>
+          <t>Cameron Norrie 2024 Topps Graphite Tennis RED CRYSTALLINE 1/1 Match Masters</t>
+        </is>
+      </c>
+      <c r="D334" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E334" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F334" s="2" t="inlineStr">
+        <is>
+          <t>499.99 USD</t>
+        </is>
+      </c>
+      <c r="G334" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117425686201?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2BPyQ0Ru4zXbHnbvD777BmkZVZSxaBU3LMXPyCPfE4H1dzzG%2FEdRycVA%2BS%2FW3DgDuJ3hi2ayuktexZAxpSR5GFHCzU0CfW85QEaBfNxTYyfpiJKZol0DVCrEOYPpTPmBxe%2Bg8GSV7X5j1ZKQNSC2CW9KNibYretroud7Azv1ioUrbHXyoSymptNWVkwO7lx%2BVc%3D</t>
+        </is>
+      </c>
+      <c r="H334" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I334" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/K4UAAOSwzr1noj~V/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J334" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T15:12:53.000Z</t>
+        </is>
+      </c>
+      <c r="K334" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L334" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M334" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N334" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Z9sAAOSwwd1noj~W/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O334" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P334" s="2" t="inlineStr"/>
+      <c r="Q334" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R334" s="2" t="inlineStr"/>
+      <c r="S334" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="2" t="inlineStr">
+        <is>
+          <t>Samsonova Kudermetova</t>
+        </is>
+      </c>
+      <c r="B335" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty</t>
+        </is>
+      </c>
+      <c r="C335" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis Samsonova Kudermetova Dual AUTO 1/25 CGC 9 First Print</t>
+        </is>
+      </c>
+      <c r="D335" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E335" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F335" s="2" t="inlineStr">
+        <is>
+          <t>159.99 USD</t>
+        </is>
+      </c>
+      <c r="G335" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/137767908880?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2B1dWYQvQWv4Dq8SZJ07eFsAnf1KtYz237EM6RgzUiEu01dK2hBagtj4NOymNv6Z1VkcgvYC0BPhOXZ1ATG2WoYcCEl3Y%2BoeCQFPZnWkiHSmH5sbWr1KOLG%2FwJvKH4et5AvKnZUtYSWlPsvprBgIZdV5cM1vNhRMVlfrVJ9eLP6xpAcswhi%2FkK1EtNUZOFRPGE%3D</t>
+        </is>
+      </c>
+      <c r="H335" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I335" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uigAAeSwlvdqsvTH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J335" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T21:40:01.000Z</t>
+        </is>
+      </c>
+      <c r="K335" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L335" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M335" s="2" t="inlineStr">
+        <is>
+          <t>CGC 9</t>
+        </is>
+      </c>
+      <c r="N335" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DRIAAeSw5WFqsvTQ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O335" s="2" t="inlineStr"/>
+      <c r="P335" s="2" t="inlineStr"/>
+      <c r="Q335" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R335" s="2" t="inlineStr"/>
+      <c r="S335" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="2" t="inlineStr">
+        <is>
+          <t>Mariano Zabaleta</t>
+        </is>
+      </c>
+      <c r="B336" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic / 2006 Ace Authentics Heroes &amp; Legends</t>
+        </is>
+      </c>
+      <c r="C336" s="2" t="inlineStr">
+        <is>
+          <t>2006 Ace Authentics Heroes &amp; Legends Holofoil 100/100 Mariano Zabaleta #98 3bs</t>
+        </is>
+      </c>
+      <c r="D336" s="2" t="inlineStr">
+        <is>
+          <t>100/100</t>
+        </is>
+      </c>
+      <c r="E336" s="2" t="inlineStr">
+        <is>
+          <t>last of 100 (100/100)</t>
+        </is>
+      </c>
+      <c r="F336" s="2" t="inlineStr">
+        <is>
+          <t>7.73 USD</t>
+        </is>
+      </c>
+      <c r="G336" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237085592938</t>
+        </is>
+      </c>
+      <c r="H336" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:47 UTC</t>
+        </is>
+      </c>
+      <c r="I336" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/V7QAAeSwfsNqs4wV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J336" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23T08:18:32.000Z</t>
+        </is>
+      </c>
+      <c r="K336" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L336" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M336" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N336" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/LjQAAeSwVkNqs4wV/s-l1600.jpg | https://i.ebayimg.com/images/g/MmAAAeSwh4Fqs4wV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O336" s="2" t="inlineStr"/>
+      <c r="P336" s="2" t="inlineStr"/>
+      <c r="Q336" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R336" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic: check the numbering is stamped, not on a circle sticker</t>
+        </is>
+      </c>
+      <c r="S336" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -28105,6 +29938,27 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G313" r:id="rId312"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G314" r:id="rId313"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G315" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G316" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G317" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G318" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G319" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G320" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G321" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G322" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G323" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G324" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G325" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G326" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G327" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G328" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G329" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G330" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G331" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G332" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G333" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G334" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G335" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G336" r:id="rId335"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-23 14:19 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S336"/>
+  <dimension ref="A1:S338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -29617,6 +29617,180 @@
         </is>
       </c>
       <c r="S336" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Nadal</t>
+        </is>
+      </c>
+      <c r="B337" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C337" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Rafael Nadal Match Masters Red Crystalline  #1/1 PSA 10</t>
+        </is>
+      </c>
+      <c r="D337" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E337" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F337" s="2" t="inlineStr">
+        <is>
+          <t>500.00 USD</t>
+        </is>
+      </c>
+      <c r="G337" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/128093417356</t>
+        </is>
+      </c>
+      <c r="H337" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 14:19 UTC</t>
+        </is>
+      </c>
+      <c r="I337" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ypQAAeSwqrhqsUTT/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J337" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23T01:00:00.000Z</t>
+        </is>
+      </c>
+      <c r="K337" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L337" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M337" s="2" t="inlineStr">
+        <is>
+          <t>PSA 10</t>
+        </is>
+      </c>
+      <c r="N337" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/y-AAAeSwKZ9qsUTT/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O337" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P337" s="2" t="inlineStr"/>
+      <c r="Q337" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R337" s="2" t="inlineStr"/>
+      <c r="S337" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="2" t="inlineStr">
+        <is>
+          <t>Benoit Paire</t>
+        </is>
+      </c>
+      <c r="B338" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Royalty Collection</t>
+        </is>
+      </c>
+      <c r="C338" s="2" t="inlineStr">
+        <is>
+          <t>Benoit Paire 2024 Topps Royalty #PGS-BPE Platinum Pursuit of Greatness Auto 1/1</t>
+        </is>
+      </c>
+      <c r="D338" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E338" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F338" s="2" t="inlineStr">
+        <is>
+          <t>249.99 USD</t>
+        </is>
+      </c>
+      <c r="G338" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/158314500699</t>
+        </is>
+      </c>
+      <c r="H338" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 14:19 UTC</t>
+        </is>
+      </c>
+      <c r="I338" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9A0AAeSwEu1qsEHH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J338" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21T18:22:04.000Z</t>
+        </is>
+      </c>
+      <c r="K338" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L338" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M338" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N338" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-IIAAeSwPOlqsEHH/s-l1600.jpg | https://i.ebayimg.com/images/g/PmYAAeSwWP1qsEHH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O338" s="2" t="inlineStr"/>
+      <c r="P338" s="2" t="inlineStr"/>
+      <c r="Q338" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R338" s="2" t="inlineStr"/>
+      <c r="S338" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -29959,6 +30133,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G334" r:id="rId333"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G335" r:id="rId334"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G336" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G337" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G338" r:id="rId337"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-24 03:30 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S338"/>
+  <dimension ref="A1:S355"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -29791,6 +29791,1507 @@
       </c>
       <c r="R338" s="2" t="inlineStr"/>
       <c r="S338" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="2" t="inlineStr">
+        <is>
+          <t>Juan Pablo Ficovich</t>
+        </is>
+      </c>
+      <c r="B339" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C339" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Juan Pablo Ficovich Refractor Frozenfractor Rookie #-1/0</t>
+        </is>
+      </c>
+      <c r="D339" s="2" t="inlineStr">
+        <is>
+          <t>1/0</t>
+        </is>
+      </c>
+      <c r="E339" s="2" t="inlineStr">
+        <is>
+          <t>001 of 0</t>
+        </is>
+      </c>
+      <c r="F339" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G339" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377517551459</t>
+        </is>
+      </c>
+      <c r="H339" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:30 UTC</t>
+        </is>
+      </c>
+      <c r="I339" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8IwAAeSw7Alqs86t/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J339" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T01:54:20.000Z</t>
+        </is>
+      </c>
+      <c r="K339" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L339" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M339" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N339" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/91sAAeSw1jNqs86t/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O339" s="2" t="inlineStr"/>
+      <c r="P339" s="2" t="inlineStr"/>
+      <c r="Q339" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R339" s="2" t="inlineStr"/>
+      <c r="S339" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="2" t="inlineStr">
+        <is>
+          <t>Alejandro Tabilo</t>
+        </is>
+      </c>
+      <c r="B340" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C340" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Alejandro Tabilo Refractor Frozenfractor #-1/0</t>
+        </is>
+      </c>
+      <c r="D340" s="2" t="inlineStr">
+        <is>
+          <t>1/0</t>
+        </is>
+      </c>
+      <c r="E340" s="2" t="inlineStr">
+        <is>
+          <t>001 of 0</t>
+        </is>
+      </c>
+      <c r="F340" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G340" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377517551309</t>
+        </is>
+      </c>
+      <c r="H340" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:30 UTC</t>
+        </is>
+      </c>
+      <c r="I340" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-9sAAeSwwMBqs86t/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J340" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T01:53:28.000Z</t>
+        </is>
+      </c>
+      <c r="K340" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L340" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M340" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N340" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~YgAAeSwtExqs86t/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O340" s="2" t="inlineStr"/>
+      <c r="P340" s="2" t="inlineStr"/>
+      <c r="Q340" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R340" s="2" t="inlineStr"/>
+      <c r="S340" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="2" t="inlineStr">
+        <is>
+          <t>Maria Sakkari</t>
+        </is>
+      </c>
+      <c r="B341" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C341" s="2" t="inlineStr">
+        <is>
+          <t>MARIA SAKKARI 2025 TOPPS CHROME TENNIS PINK GEOMETRIC 1ST 65/65 #285 Q3694</t>
+        </is>
+      </c>
+      <c r="D341" s="2" t="inlineStr">
+        <is>
+          <t>65/65</t>
+        </is>
+      </c>
+      <c r="E341" s="2" t="inlineStr">
+        <is>
+          <t>last of 65 (65/65)</t>
+        </is>
+      </c>
+      <c r="F341" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G341" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/278403124451</t>
+        </is>
+      </c>
+      <c r="H341" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:30 UTC</t>
+        </is>
+      </c>
+      <c r="I341" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/IJcAAeSwbmxqtE0~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J341" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T01:43:00.000Z</t>
+        </is>
+      </c>
+      <c r="K341" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L341" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M341" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N341" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/LrUAAeSw8lBqtE0~/s-l1600.jpg | https://i.ebayimg.com/images/g/LdUAAeSw0SFqtE0-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O341" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P341" s="2" t="inlineStr"/>
+      <c r="Q341" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R341" s="2" t="inlineStr"/>
+      <c r="S341" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="2" t="inlineStr">
+        <is>
+          <t>Martina Trevisan</t>
+        </is>
+      </c>
+      <c r="B342" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C342" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Martina Trevisan 99/99 #151</t>
+        </is>
+      </c>
+      <c r="D342" s="2" t="inlineStr">
+        <is>
+          <t>99/99</t>
+        </is>
+      </c>
+      <c r="E342" s="2" t="inlineStr">
+        <is>
+          <t>last of 99 (99/99)</t>
+        </is>
+      </c>
+      <c r="F342" s="2" t="inlineStr">
+        <is>
+          <t>4.00 USD</t>
+        </is>
+      </c>
+      <c r="G342" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377518231756</t>
+        </is>
+      </c>
+      <c r="H342" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:30 UTC</t>
+        </is>
+      </c>
+      <c r="I342" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/mpgAAeSw6dRqtDWs/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J342" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T01:00:01.000Z</t>
+        </is>
+      </c>
+      <c r="K342" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L342" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M342" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N342" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/k58AAeSwj5pqtDWu/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O342" s="2" t="inlineStr"/>
+      <c r="P342" s="2" t="inlineStr"/>
+      <c r="Q342" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R342" s="2" t="inlineStr"/>
+      <c r="S342" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="2" t="inlineStr">
+        <is>
+          <t>Yulia Putintseva</t>
+        </is>
+      </c>
+      <c r="B343" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Chrome</t>
+        </is>
+      </c>
+      <c r="C343" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Yulia Putintseva #45 Pink Geometric Refractor 65/65</t>
+        </is>
+      </c>
+      <c r="D343" s="2" t="inlineStr">
+        <is>
+          <t>65/65</t>
+        </is>
+      </c>
+      <c r="E343" s="2" t="inlineStr">
+        <is>
+          <t>last of 65 (65/65)</t>
+        </is>
+      </c>
+      <c r="F343" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G343" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/188965907412</t>
+        </is>
+      </c>
+      <c r="H343" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:30 UTC</t>
+        </is>
+      </c>
+      <c r="I343" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vwgAAeSwoOtqsp4g/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J343" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T00:09:00.000Z</t>
+        </is>
+      </c>
+      <c r="K343" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L343" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M343" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N343" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/5dEAAeSwpDFqsp4g/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O343" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P343" s="2" t="inlineStr"/>
+      <c r="Q343" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R343" s="2" t="inlineStr"/>
+      <c r="S343" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="2" t="inlineStr">
+        <is>
+          <t>Yoshihito Nishioka</t>
+        </is>
+      </c>
+      <c r="B344" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C344" s="2" t="inlineStr">
+        <is>
+          <t>YOSHIHITO NISHIOKA 2024 TOPPS CHROME TENNIS PINK REFRACTOR 1ST 01/65 #12 Q3694</t>
+        </is>
+      </c>
+      <c r="D344" s="2" t="inlineStr">
+        <is>
+          <t>1/65</t>
+        </is>
+      </c>
+      <c r="E344" s="2" t="inlineStr">
+        <is>
+          <t>001 of 65</t>
+        </is>
+      </c>
+      <c r="F344" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G344" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/278402939243</t>
+        </is>
+      </c>
+      <c r="H344" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:30 UTC</t>
+        </is>
+      </c>
+      <c r="I344" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Z8kAAeSw-YBqtDif/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J344" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T00:00:00.000Z</t>
+        </is>
+      </c>
+      <c r="K344" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L344" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M344" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N344" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YfAAAeSw5B9qtDif/s-l1600.jpg | https://i.ebayimg.com/images/g/a~oAAeSwRHlqtDie/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O344" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P344" s="2" t="inlineStr"/>
+      <c r="Q344" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R344" s="2" t="inlineStr"/>
+      <c r="S344" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="2" t="inlineStr">
+        <is>
+          <t>Venus Williams</t>
+        </is>
+      </c>
+      <c r="B345" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C345" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Sapphire Green 125/125 Venus Williams #200 0e61</t>
+        </is>
+      </c>
+      <c r="D345" s="2" t="inlineStr">
+        <is>
+          <t>125/125</t>
+        </is>
+      </c>
+      <c r="E345" s="2" t="inlineStr">
+        <is>
+          <t>last of 125 (125/125)</t>
+        </is>
+      </c>
+      <c r="F345" s="2" t="inlineStr">
+        <is>
+          <t>6.58 USD</t>
+        </is>
+      </c>
+      <c r="G345" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257761689033</t>
+        </is>
+      </c>
+      <c r="H345" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:30 UTC</t>
+        </is>
+      </c>
+      <c r="I345" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HB0AAeSwyBBqtGCo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J345" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23T23:27:37.000Z</t>
+        </is>
+      </c>
+      <c r="K345" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L345" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M345" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N345" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HBwAAeSwyBBqtGCo/s-l1600.jpg | https://i.ebayimg.com/images/g/uPAAAeSwbz5qtGCo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O345" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P345" s="2" t="inlineStr"/>
+      <c r="Q345" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R345" s="2" t="inlineStr"/>
+      <c r="S345" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="2" t="inlineStr">
+        <is>
+          <t>Jimmy Connors</t>
+        </is>
+      </c>
+      <c r="B346" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C346" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Tennis #175 Jimmy Connors — Red Crystalline Refractor — 1/1</t>
+        </is>
+      </c>
+      <c r="D346" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E346" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F346" s="2" t="inlineStr">
+        <is>
+          <t>349.99 USD</t>
+        </is>
+      </c>
+      <c r="G346" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366688320828</t>
+        </is>
+      </c>
+      <c r="H346" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:30 UTC</t>
+        </is>
+      </c>
+      <c r="I346" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-ioAAeSwaahqtJZn/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J346" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T03:20:12.000Z</t>
+        </is>
+      </c>
+      <c r="K346" s="2" t="inlineStr">
+        <is>
+          <t>Auction + Buy It Now</t>
+        </is>
+      </c>
+      <c r="L346" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M346" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N346" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7b8AAeSw8lBqtJZX/s-l1600.jpg | https://i.ebayimg.com/images/g/~KcAAeSw2m9qtJZR/s-l1600.jpg | https://i.ebayimg.com/images/g/7XkAAeSwGA9qtJZY/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O346" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P346" s="2" t="inlineStr"/>
+      <c r="Q346" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R346" s="2" t="inlineStr"/>
+      <c r="S346" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="2" t="inlineStr">
+        <is>
+          <t>Victoria Jimenez Kasintseva</t>
+        </is>
+      </c>
+      <c r="B347" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C347" s="2" t="inlineStr">
+        <is>
+          <t>2024 Graphite Pink Refractor 15/15 Victoria Jimenez Kasintseva Rookie RC 5h0</t>
+        </is>
+      </c>
+      <c r="D347" s="2" t="inlineStr">
+        <is>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="E347" s="2" t="inlineStr">
+        <is>
+          <t>last of 15 (15/15)</t>
+        </is>
+      </c>
+      <c r="F347" s="2" t="inlineStr">
+        <is>
+          <t>15.48 USD</t>
+        </is>
+      </c>
+      <c r="G347" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257761976363</t>
+        </is>
+      </c>
+      <c r="H347" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:30 UTC</t>
+        </is>
+      </c>
+      <c r="I347" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Q78AAeSwvbtqtI1s/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J347" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T02:38:36.000Z</t>
+        </is>
+      </c>
+      <c r="K347" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L347" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M347" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N347" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/sKIAAeSwrcFqtI1s/s-l1600.jpg | https://i.ebayimg.com/images/g/wKAAAeSwbyVqtI1s/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O347" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P347" s="2" t="inlineStr"/>
+      <c r="Q347" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R347" s="2" t="inlineStr"/>
+      <c r="S347" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="2" t="inlineStr">
+        <is>
+          <t>Kayla Day</t>
+        </is>
+      </c>
+      <c r="B348" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C348" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Green Refractor 1/75 Kayla Day #105 Rookie RC 1g0c</t>
+        </is>
+      </c>
+      <c r="D348" s="2" t="inlineStr">
+        <is>
+          <t>1/75</t>
+        </is>
+      </c>
+      <c r="E348" s="2" t="inlineStr">
+        <is>
+          <t>001 of 75</t>
+        </is>
+      </c>
+      <c r="F348" s="2" t="inlineStr">
+        <is>
+          <t>7.73 USD</t>
+        </is>
+      </c>
+      <c r="G348" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237087143291</t>
+        </is>
+      </c>
+      <c r="H348" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:30 UTC</t>
+        </is>
+      </c>
+      <c r="I348" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/4pkAAeSwjtRqtHW7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J348" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T00:57:33.000Z</t>
+        </is>
+      </c>
+      <c r="K348" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L348" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M348" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N348" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/y5sAAeSwiSVqtHW7/s-l1600.jpg | https://i.ebayimg.com/images/g/ZKsAAeSwvbtqtHW7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O348" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P348" s="2" t="inlineStr"/>
+      <c r="Q348" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R348" s="2" t="inlineStr"/>
+      <c r="S348" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="2" t="inlineStr">
+        <is>
+          <t>Erika Andreeva</t>
+        </is>
+      </c>
+      <c r="B349" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C349" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Pink Refractor 1/15 Erika Andreeva #131 Rookie RC 0y61</t>
+        </is>
+      </c>
+      <c r="D349" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E349" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F349" s="2" t="inlineStr">
+        <is>
+          <t>20.38 USD</t>
+        </is>
+      </c>
+      <c r="G349" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237087060640</t>
+        </is>
+      </c>
+      <c r="H349" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:30 UTC</t>
+        </is>
+      </c>
+      <c r="I349" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/auMAAeSwHfFqtGk2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J349" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T00:04:05.000Z</t>
+        </is>
+      </c>
+      <c r="K349" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L349" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M349" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N349" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XagAAeSwxnxqtGk1/s-l1600.jpg | https://i.ebayimg.com/images/g/AbgAAeSwvbtqtGk2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O349" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P349" s="2" t="inlineStr"/>
+      <c r="Q349" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R349" s="2" t="inlineStr"/>
+      <c r="S349" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="2" t="inlineStr">
+        <is>
+          <t>Magda Linette</t>
+        </is>
+      </c>
+      <c r="B350" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C350" s="2" t="inlineStr">
+        <is>
+          <t>Magda Linette 2024 Topps Graphite Aqua Refractor 199/199 #74 BOOKEND</t>
+        </is>
+      </c>
+      <c r="D350" s="2" t="inlineStr">
+        <is>
+          <t>199/199</t>
+        </is>
+      </c>
+      <c r="E350" s="2" t="inlineStr">
+        <is>
+          <t>last of 199 (199/199)</t>
+        </is>
+      </c>
+      <c r="F350" s="2" t="inlineStr">
+        <is>
+          <t>6.95 USD</t>
+        </is>
+      </c>
+      <c r="G350" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168715526457</t>
+        </is>
+      </c>
+      <c r="H350" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:30 UTC</t>
+        </is>
+      </c>
+      <c r="I350" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/cXcAAeSw7AlqtE4f/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J350" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23T22:08:28.000Z</t>
+        </is>
+      </c>
+      <c r="K350" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L350" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M350" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N350" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/dS0AAeSwQIlqtE4f/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O350" s="2" t="inlineStr">
+        <is>
+          <t>aqua</t>
+        </is>
+      </c>
+      <c r="P350" s="2" t="inlineStr"/>
+      <c r="Q350" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R350" s="2" t="inlineStr"/>
+      <c r="S350" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="2" t="inlineStr">
+        <is>
+          <t>Beatriz Haddad Maia</t>
+        </is>
+      </c>
+      <c r="B351" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C351" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Green Refractor 75/75 Beatriz Haddad Maia #123 Rookie RC p6a</t>
+        </is>
+      </c>
+      <c r="D351" s="2" t="inlineStr">
+        <is>
+          <t>75/75</t>
+        </is>
+      </c>
+      <c r="E351" s="2" t="inlineStr">
+        <is>
+          <t>last of 75 (75/75)</t>
+        </is>
+      </c>
+      <c r="F351" s="2" t="inlineStr">
+        <is>
+          <t>12.33 USD</t>
+        </is>
+      </c>
+      <c r="G351" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257761002452</t>
+        </is>
+      </c>
+      <c r="H351" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:30 UTC</t>
+        </is>
+      </c>
+      <c r="I351" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jI8AAeSw9JNqs~bd/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J351" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23T15:56:14.000Z</t>
+        </is>
+      </c>
+      <c r="K351" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L351" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M351" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N351" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/4bYAAeSwZ-Rqs~bd/s-l1600.jpg | https://i.ebayimg.com/images/g/5REAAeSwuyVqs~be/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O351" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P351" s="2" t="inlineStr"/>
+      <c r="Q351" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R351" s="2" t="inlineStr"/>
+      <c r="S351" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="2" t="inlineStr">
+        <is>
+          <t>Garbine Muguruza</t>
+        </is>
+      </c>
+      <c r="B352" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C352" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Collection Garbine Muguruza Imperial Ink Platinum Auto #1/1</t>
+        </is>
+      </c>
+      <c r="D352" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E352" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F352" s="2" t="inlineStr">
+        <is>
+          <t>1.25 USD</t>
+        </is>
+      </c>
+      <c r="G352" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377518100450</t>
+        </is>
+      </c>
+      <c r="H352" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:30 UTC</t>
+        </is>
+      </c>
+      <c r="I352" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bwsAAeSwmFhqtCCt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J352" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T01:38:50.000Z</t>
+        </is>
+      </c>
+      <c r="K352" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L352" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M352" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N352" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/b-EAAeSw~XRqtCCt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O352" s="2" t="inlineStr"/>
+      <c r="P352" s="2" t="inlineStr"/>
+      <c r="Q352" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R352" s="2" t="inlineStr"/>
+      <c r="S352" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="2" t="inlineStr">
+        <is>
+          <t>Sloane Stephens</t>
+        </is>
+      </c>
+      <c r="B353" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Relic Jewels - Blue</t>
+        </is>
+      </c>
+      <c r="C353" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Relic Jewels Blue 25/25 Sloane Stephens #RCJ-SS 1e41</t>
+        </is>
+      </c>
+      <c r="D353" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E353" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F353" s="2" t="inlineStr">
+        <is>
+          <t>32.45 USD</t>
+        </is>
+      </c>
+      <c r="G353" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237087089081</t>
+        </is>
+      </c>
+      <c r="H353" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:30 UTC</t>
+        </is>
+      </c>
+      <c r="I353" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ahEAAeSwGA9qtG4z/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J353" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T00:25:25.000Z</t>
+        </is>
+      </c>
+      <c r="K353" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L353" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M353" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N353" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XT0AAeSwiMJqtG4z/s-l1600.jpg | https://i.ebayimg.com/images/g/ZasAAeSwMOxqtG4z/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O353" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P353" s="2" t="inlineStr"/>
+      <c r="Q353" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R353" s="2" t="inlineStr"/>
+      <c r="S353" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="2" t="inlineStr">
+        <is>
+          <t>Caroline Garcia</t>
+        </is>
+      </c>
+      <c r="B354" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - [Base] - Purple</t>
+        </is>
+      </c>
+      <c r="C354" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Purple 35/35 Caroline Garcia #95 Rookie RC 1e41</t>
+        </is>
+      </c>
+      <c r="D354" s="2" t="inlineStr">
+        <is>
+          <t>35/35</t>
+        </is>
+      </c>
+      <c r="E354" s="2" t="inlineStr">
+        <is>
+          <t>last of 35 (35/35)</t>
+        </is>
+      </c>
+      <c r="F354" s="2" t="inlineStr">
+        <is>
+          <t>20.38 USD</t>
+        </is>
+      </c>
+      <c r="G354" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336809246199</t>
+        </is>
+      </c>
+      <c r="H354" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:30 UTC</t>
+        </is>
+      </c>
+      <c r="I354" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/tyUAAeSwi6RqtA9t/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J354" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23T17:40:57.000Z</t>
+        </is>
+      </c>
+      <c r="K354" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L354" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M354" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N354" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/qMsAAeSwlQNqtA9t/s-l1600.jpg | https://i.ebayimg.com/images/g/s~sAAeSwqBJqtA9t/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O354" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P354" s="2" t="inlineStr"/>
+      <c r="Q354" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R354" s="2" t="inlineStr"/>
+      <c r="S354" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="2" t="inlineStr">
+        <is>
+          <t>Zack Fleishman</t>
+        </is>
+      </c>
+      <c r="B355" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic / 2008 Ace Authentic Grand Slam II</t>
+        </is>
+      </c>
+      <c r="C355" s="2" t="inlineStr">
+        <is>
+          <t>2008 Ace Authentic Grand Slam II Gold 24/24 Zack Fleishman #BT35 Auto 0h1</t>
+        </is>
+      </c>
+      <c r="D355" s="2" t="inlineStr">
+        <is>
+          <t>24/24</t>
+        </is>
+      </c>
+      <c r="E355" s="2" t="inlineStr">
+        <is>
+          <t>last of 24 (24/24)</t>
+        </is>
+      </c>
+      <c r="F355" s="2" t="inlineStr">
+        <is>
+          <t>18.07 USD</t>
+        </is>
+      </c>
+      <c r="G355" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257761895794</t>
+        </is>
+      </c>
+      <c r="H355" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:30 UTC</t>
+        </is>
+      </c>
+      <c r="I355" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/MWsAAeSwFEdqtIAW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J355" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T01:41:42.000Z</t>
+        </is>
+      </c>
+      <c r="K355" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L355" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M355" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N355" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KV4AAeSw6dRqtIAW/s-l1600.jpg | https://i.ebayimg.com/images/g/IqcAAeSwnl5qtIAW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O355" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P355" s="2" t="inlineStr"/>
+      <c r="Q355" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R355" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic autograph: on-card or sticker not stated; check by eye</t>
+        </is>
+      </c>
+      <c r="S355" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -30135,6 +31636,23 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G336" r:id="rId335"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G337" r:id="rId336"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G338" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G339" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G340" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G341" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G342" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G343" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G344" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G345" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G346" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G347" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G348" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G349" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G350" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G351" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G352" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G353" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G354" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G355" r:id="rId354"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-24 03:59 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S355"/>
+  <dimension ref="A1:S356"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -31292,6 +31292,91 @@
         </is>
       </c>
       <c r="S355" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="2" t="inlineStr">
+        <is>
+          <t>Sabalenka</t>
+        </is>
+      </c>
+      <c r="B356" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS CHROME TENNIS ACES</t>
+        </is>
+      </c>
+      <c r="C356" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS CHROME TENNIS ACES SUPERFRACTOR 1/1 #CASAS ARYNA SABALENKA 1/1 PSA 9</t>
+        </is>
+      </c>
+      <c r="D356" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E356" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F356" s="2" t="inlineStr">
+        <is>
+          <t>59000.00 USD</t>
+        </is>
+      </c>
+      <c r="G356" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298671302620</t>
+        </is>
+      </c>
+      <c r="H356" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 03:59 UTC</t>
+        </is>
+      </c>
+      <c r="I356" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/OrYAAeSwH3Zo0Pn1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J356" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13T17:58:53.000Z</t>
+        </is>
+      </c>
+      <c r="K356" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L356" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M356" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N356" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/PXIAAeSwnJto0Pn1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O356" s="2" t="inlineStr"/>
+      <c r="P356" s="2" t="inlineStr"/>
+      <c r="Q356" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R356" s="2" t="inlineStr"/>
+      <c r="S356" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -31653,6 +31738,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G353" r:id="rId352"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G354" r:id="rId353"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G355" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G356" r:id="rId355"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-24 14:18 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S356"/>
+  <dimension ref="A1:S362"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -31377,6 +31377,540 @@
       </c>
       <c r="R356" s="2" t="inlineStr"/>
       <c r="S356" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="2" t="inlineStr">
+        <is>
+          <t>Xiyu Wang</t>
+        </is>
+      </c>
+      <c r="B357" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C357" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Gold Refractor 1/50 Xiyu Wang #126 Rookie RC 3hd</t>
+        </is>
+      </c>
+      <c r="D357" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E357" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F357" s="2" t="inlineStr">
+        <is>
+          <t>17.73 USD</t>
+        </is>
+      </c>
+      <c r="G357" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257762724195</t>
+        </is>
+      </c>
+      <c r="H357" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:18 UTC</t>
+        </is>
+      </c>
+      <c r="I357" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/28QAAeSwMnxqtRUU/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J357" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T12:16:09.000Z</t>
+        </is>
+      </c>
+      <c r="K357" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L357" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M357" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N357" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YjsAAeSwIftqtRUU/s-l1600.jpg | https://i.ebayimg.com/images/g/XocAAeSw0ApqtRUU/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O357" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P357" s="2" t="inlineStr"/>
+      <c r="Q357" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R357" s="2" t="inlineStr"/>
+      <c r="S357" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="2" t="inlineStr">
+        <is>
+          <t>Yoshihito Nishioka</t>
+        </is>
+      </c>
+      <c r="B358" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - [Base] - Black Geometric Refractor</t>
+        </is>
+      </c>
+      <c r="C358" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Black Geometric Refractor 2/2 Yoshihito Nishioka #88 1e41</t>
+        </is>
+      </c>
+      <c r="D358" s="2" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="E358" s="2" t="inlineStr">
+        <is>
+          <t>last of 2 (2/2)</t>
+        </is>
+      </c>
+      <c r="F358" s="2" t="inlineStr">
+        <is>
+          <t>57.74 USD</t>
+        </is>
+      </c>
+      <c r="G358" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257762701229</t>
+        </is>
+      </c>
+      <c r="H358" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:18 UTC</t>
+        </is>
+      </c>
+      <c r="I358" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/t4UAAeSwcAFqtREd/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J358" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T12:00:17.000Z</t>
+        </is>
+      </c>
+      <c r="K358" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L358" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M358" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N358" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/t4cAAeSwcAFqtREd/s-l1600.jpg | https://i.ebayimg.com/images/g/INwAAeSwDtpqtREd/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O358" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P358" s="2" t="inlineStr"/>
+      <c r="Q358" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R358" s="2" t="inlineStr"/>
+      <c r="S358" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="2" t="inlineStr">
+        <is>
+          <t>Jack Draper</t>
+        </is>
+      </c>
+      <c r="B359" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C359" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome I Orange Refractor 25/25 Jack Draper Rookie Auto RC 0r9h</t>
+        </is>
+      </c>
+      <c r="D359" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E359" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F359" s="2" t="inlineStr">
+        <is>
+          <t>229.45 USD</t>
+        </is>
+      </c>
+      <c r="G359" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336810020810</t>
+        </is>
+      </c>
+      <c r="H359" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:18 UTC</t>
+        </is>
+      </c>
+      <c r="I359" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nS4AAeSwr5dqtJ8K/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J359" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T03:53:47.000Z</t>
+        </is>
+      </c>
+      <c r="K359" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L359" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M359" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N359" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nSsAAeSwr5dqtJ8K/s-l1600.jpg | https://i.ebayimg.com/images/g/p6gAAeSwRddqtJ8K/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O359" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P359" s="2" t="inlineStr"/>
+      <c r="Q359" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R359" s="2" t="inlineStr"/>
+      <c r="S359" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="2" t="inlineStr">
+        <is>
+          <t>Steffi Graf</t>
+        </is>
+      </c>
+      <c r="B360" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C360" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Winning Streaks White Refractor 1/10 Steffi Graf #WS-SG v9t</t>
+        </is>
+      </c>
+      <c r="D360" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E360" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F360" s="2" t="inlineStr">
+        <is>
+          <t>75.58 USD</t>
+        </is>
+      </c>
+      <c r="G360" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237087538009</t>
+        </is>
+      </c>
+      <c r="H360" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:18 UTC</t>
+        </is>
+      </c>
+      <c r="I360" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/t5YAAeSw8lBqtLTm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J360" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T05:27:02.000Z</t>
+        </is>
+      </c>
+      <c r="K360" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L360" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M360" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N360" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/t5gAAeSw8lBqtLTm/s-l1600.jpg | https://i.ebayimg.com/images/g/s7EAAeSw3q9qtLTm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O360" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P360" s="2" t="inlineStr"/>
+      <c r="Q360" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R360" s="2" t="inlineStr"/>
+      <c r="S360" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="2" t="inlineStr">
+        <is>
+          <t>Whitney Osuigwe</t>
+        </is>
+      </c>
+      <c r="B361" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Superior Signatures - Gold</t>
+        </is>
+      </c>
+      <c r="C361" s="2" t="inlineStr">
+        <is>
+          <t>2024 Royalty Superior Signatures Gold 10/10 Whitney Osuigwe Rookie Auto RC 1e41</t>
+        </is>
+      </c>
+      <c r="D361" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E361" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F361" s="2" t="inlineStr">
+        <is>
+          <t>29.58 USD</t>
+        </is>
+      </c>
+      <c r="G361" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257762653592</t>
+        </is>
+      </c>
+      <c r="H361" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:18 UTC</t>
+        </is>
+      </c>
+      <c r="I361" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/PN0AAeSwZ7pqtQcp/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J361" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T11:17:56.000Z</t>
+        </is>
+      </c>
+      <c r="K361" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L361" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M361" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N361" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Sz4AAeSwrABqtQcp/s-l1600.jpg | https://i.ebayimg.com/images/g/TMwAAeSw9tNqtQcp/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O361" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P361" s="2" t="inlineStr"/>
+      <c r="Q361" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R361" s="2" t="inlineStr"/>
+      <c r="S361" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="2" t="inlineStr">
+        <is>
+          <t>Pablo Carreno Busta</t>
+        </is>
+      </c>
+      <c r="B362" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Superior Signatures - Gold</t>
+        </is>
+      </c>
+      <c r="C362" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Gold 1/10 Pablo Carreno Busta #SS-PCB Rookie Auto RC 1e41</t>
+        </is>
+      </c>
+      <c r="D362" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E362" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F362" s="2" t="inlineStr">
+        <is>
+          <t>56.89 USD</t>
+        </is>
+      </c>
+      <c r="G362" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257762468218</t>
+        </is>
+      </c>
+      <c r="H362" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:18 UTC</t>
+        </is>
+      </c>
+      <c r="I362" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/lKAAAeSwqchqtOm9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J362" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T09:12:26.000Z</t>
+        </is>
+      </c>
+      <c r="K362" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L362" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M362" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N362" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/kFAAAeSw0PxqtOm9/s-l1600.jpg | https://i.ebayimg.com/images/g/hqAAAeSwi8tqtOm9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O362" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P362" s="2" t="inlineStr"/>
+      <c r="Q362" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R362" s="2" t="inlineStr"/>
+      <c r="S362" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -31739,6 +32273,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G354" r:id="rId353"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G355" r:id="rId354"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G356" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G357" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G358" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G359" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G360" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G361" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G362" r:id="rId361"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-25 14:42 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S362"/>
+  <dimension ref="A1:S380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -31911,6 +31911,1608 @@
       </c>
       <c r="R362" s="2" t="inlineStr"/>
       <c r="S362" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="2" t="inlineStr">
+        <is>
+          <t>Joao Fonseca</t>
+        </is>
+      </c>
+      <c r="B363" s="2" t="inlineStr">
+        <is>
+          <t>NetPro / 2026 NetPro Tennis</t>
+        </is>
+      </c>
+      <c r="C363" s="2" t="inlineStr">
+        <is>
+          <t>Aryna Sabalenka NetPro Premium Rainbow Red 01/10 Autograph #A-AS Auto SSP</t>
+        </is>
+      </c>
+      <c r="D363" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E363" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F363" s="2" t="inlineStr">
+        <is>
+          <t>2999.99 USD</t>
+        </is>
+      </c>
+      <c r="G363" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/188982822691</t>
+        </is>
+      </c>
+      <c r="H363" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:41 UTC</t>
+        </is>
+      </c>
+      <c r="I363" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/xYoAAeSwYw1qtnQg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J363" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T13:16:46.000Z</t>
+        </is>
+      </c>
+      <c r="K363" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L363" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M363" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N363" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DqIAAeSw6dRqtnQk/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O363" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P363" s="2" t="inlineStr"/>
+      <c r="Q363" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R363" s="2" t="inlineStr"/>
+      <c r="S363" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="2" t="inlineStr">
+        <is>
+          <t>Grigor Dimitrov</t>
+        </is>
+      </c>
+      <c r="B364" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C364" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Grigor Dimitrov Red 1/5 bookend #289</t>
+        </is>
+      </c>
+      <c r="D364" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E364" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F364" s="2" t="inlineStr">
+        <is>
+          <t>59.99 USD</t>
+        </is>
+      </c>
+      <c r="G364" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/820170935210</t>
+        </is>
+      </c>
+      <c r="H364" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:41 UTC</t>
+        </is>
+      </c>
+      <c r="I364" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/z0QAAeSwiYhqtoP3/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J364" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T14:37:25.000Z</t>
+        </is>
+      </c>
+      <c r="K364" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L364" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M364" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N364" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/l8IAAeSw6sNqtoPk/s-l1600.jpg | https://i.ebayimg.com/images/g/qwUAAeSw4VZqtoPk/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O364" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P364" s="2" t="inlineStr"/>
+      <c r="Q364" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R364" s="2" t="inlineStr"/>
+      <c r="S364" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="2" t="inlineStr">
+        <is>
+          <t>Wu Yibing</t>
+        </is>
+      </c>
+      <c r="B365" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C365" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis 11 Wu Yibing 1st Lime Green Refractor 299/299</t>
+        </is>
+      </c>
+      <c r="D365" s="2" t="inlineStr">
+        <is>
+          <t>299/299</t>
+        </is>
+      </c>
+      <c r="E365" s="2" t="inlineStr">
+        <is>
+          <t>last of 299 (299/299)</t>
+        </is>
+      </c>
+      <c r="F365" s="2" t="inlineStr">
+        <is>
+          <t>3.99 USD</t>
+        </is>
+      </c>
+      <c r="G365" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307198764626?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2FIY%2BncekcAzKhXKg4BFE8LaeFZKWfxAtJJATpfW5fwQwjvJHKaao5%2FP4Nh0%2FITXgg%2FGQr02OIiSs%2BQCp%2B6AAaUpjSacWEJDhEZn77U1uDWvTq2Okk5Y9G21cOdXgz9Of%2BWhj40xRuYgJJyu4wBOf%2FhLbhdZkXCGSyvfh2ILNfP5WzQFEOoBoozn9vHgZ4Weqo%3D</t>
+        </is>
+      </c>
+      <c r="H365" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:41 UTC</t>
+        </is>
+      </c>
+      <c r="I365" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/FfQAAeSwYxRqtn37/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J365" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T13:58:34.000Z</t>
+        </is>
+      </c>
+      <c r="K365" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L365" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M365" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N365" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/hFsAAeSwi8tqtn37/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O365" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P365" s="2" t="inlineStr"/>
+      <c r="Q365" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R365" s="2" t="inlineStr"/>
+      <c r="S365" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="2" t="inlineStr">
+        <is>
+          <t>Stan Smith</t>
+        </is>
+      </c>
+      <c r="B366" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C366" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Green Refractor 1/75 Stan Smith #62 HOF 1m01</t>
+        </is>
+      </c>
+      <c r="D366" s="2" t="inlineStr">
+        <is>
+          <t>1/75</t>
+        </is>
+      </c>
+      <c r="E366" s="2" t="inlineStr">
+        <is>
+          <t>001 of 75</t>
+        </is>
+      </c>
+      <c r="F366" s="2" t="inlineStr">
+        <is>
+          <t>23.82 USD</t>
+        </is>
+      </c>
+      <c r="G366" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336812460740</t>
+        </is>
+      </c>
+      <c r="H366" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:41 UTC</t>
+        </is>
+      </c>
+      <c r="I366" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/pZAAAeSwGABqtnrY/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J366" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T13:43:51.000Z</t>
+        </is>
+      </c>
+      <c r="K366" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L366" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M366" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N366" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/pJ8AAeSw4KJqtnrY/s-l1600.jpg | https://i.ebayimg.com/images/g/PUEAAeSwI1NqtnrY/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O366" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P366" s="2" t="inlineStr"/>
+      <c r="Q366" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R366" s="2" t="inlineStr"/>
+      <c r="S366" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="2" t="inlineStr">
+        <is>
+          <t>Pedro Cachin</t>
+        </is>
+      </c>
+      <c r="B367" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C367" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Gold Refractor 1/50 Pedro Cachin #112 Rookie RC 6q5</t>
+        </is>
+      </c>
+      <c r="D367" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E367" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F367" s="2" t="inlineStr">
+        <is>
+          <t>17.78 USD</t>
+        </is>
+      </c>
+      <c r="G367" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257764949894</t>
+        </is>
+      </c>
+      <c r="H367" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:41 UTC</t>
+        </is>
+      </c>
+      <c r="I367" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/D-YAAeSwGTlqtm4z/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J367" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T12:49:51.000Z</t>
+        </is>
+      </c>
+      <c r="K367" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L367" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M367" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N367" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/A9kAAeSwGAhqtm4z/s-l1600.jpg | https://i.ebayimg.com/images/g/KcUAAeSwJLxqtm4z/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O367" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P367" s="2" t="inlineStr"/>
+      <c r="Q367" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R367" s="2" t="inlineStr"/>
+      <c r="S367" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="2" t="inlineStr">
+        <is>
+          <t>Alycia Parks</t>
+        </is>
+      </c>
+      <c r="B368" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - Autographs I - Orange Refractor</t>
+        </is>
+      </c>
+      <c r="C368" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome I Orange Refractor 1/25 Alycia Parks Rookie Auto RC 7ba</t>
+        </is>
+      </c>
+      <c r="D368" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E368" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F368" s="2" t="inlineStr">
+        <is>
+          <t>58.89 USD</t>
+        </is>
+      </c>
+      <c r="G368" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257764932059</t>
+        </is>
+      </c>
+      <c r="H368" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:41 UTC</t>
+        </is>
+      </c>
+      <c r="I368" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HO8AAeSwXutqtmrX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J368" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T12:35:36.000Z</t>
+        </is>
+      </c>
+      <c r="K368" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L368" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M368" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N368" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QO8AAeSwkepqtmrX/s-l1600.jpg | https://i.ebayimg.com/images/g/kngAAeSwdd1qtmrX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O368" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P368" s="2" t="inlineStr"/>
+      <c r="Q368" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R368" s="2" t="inlineStr"/>
+      <c r="S368" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="2" t="inlineStr">
+        <is>
+          <t>Bob Bryan</t>
+        </is>
+      </c>
+      <c r="B369" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C369" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Purple Wave Refractor 1/199 Bob Bryan #9 7tw</t>
+        </is>
+      </c>
+      <c r="D369" s="2" t="inlineStr">
+        <is>
+          <t>1/199</t>
+        </is>
+      </c>
+      <c r="E369" s="2" t="inlineStr">
+        <is>
+          <t>001 of 199</t>
+        </is>
+      </c>
+      <c r="F369" s="2" t="inlineStr">
+        <is>
+          <t>3.91 USD</t>
+        </is>
+      </c>
+      <c r="G369" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336812368844</t>
+        </is>
+      </c>
+      <c r="H369" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:41 UTC</t>
+        </is>
+      </c>
+      <c r="I369" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0QAAAeSwrwFqtmmU/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J369" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T12:30:11.000Z</t>
+        </is>
+      </c>
+      <c r="K369" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L369" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M369" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N369" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/1E4AAeSwmIRqtmmU/s-l1600.jpg | https://i.ebayimg.com/images/g/rzkAAeSwWw1qtmmU/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O369" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P369" s="2" t="inlineStr"/>
+      <c r="Q369" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R369" s="2" t="inlineStr"/>
+      <c r="S369" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="2" t="inlineStr">
+        <is>
+          <t>Novak Djokovic</t>
+        </is>
+      </c>
+      <c r="B370" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Graphite</t>
+        </is>
+      </c>
+      <c r="C370" s="2" t="inlineStr">
+        <is>
+          <t>Novak Djokovic 2024 Topps Graphite White Refractor Auto 1/10</t>
+        </is>
+      </c>
+      <c r="D370" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E370" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F370" s="2" t="inlineStr">
+        <is>
+          <t>1125.00 USD</t>
+        </is>
+      </c>
+      <c r="G370" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/158335130434</t>
+        </is>
+      </c>
+      <c r="H370" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:41 UTC</t>
+        </is>
+      </c>
+      <c r="I370" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2FYAAeSwJitqtbsx/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J370" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T01:04:00.000Z</t>
+        </is>
+      </c>
+      <c r="K370" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L370" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M370" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N370" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/xEgAAeSwLmFqtbsx/s-l1600.jpg | https://i.ebayimg.com/images/g/7hIAAeSwKqZqtbsx/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O370" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P370" s="2" t="inlineStr"/>
+      <c r="Q370" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R370" s="2" t="inlineStr"/>
+      <c r="S370" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek</t>
+        </is>
+      </c>
+      <c r="B371" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Graphite</t>
+        </is>
+      </c>
+      <c r="C371" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek 2024 Topps Graphite #GS-ISK Red Crystalline Refractor Auto 1/1</t>
+        </is>
+      </c>
+      <c r="D371" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E371" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F371" s="2" t="inlineStr">
+        <is>
+          <t>3550.00 USD</t>
+        </is>
+      </c>
+      <c r="G371" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/158335130445</t>
+        </is>
+      </c>
+      <c r="H371" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:41 UTC</t>
+        </is>
+      </c>
+      <c r="I371" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/y2QAAeSwuiRqtbs0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J371" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T01:02:00.000Z</t>
+        </is>
+      </c>
+      <c r="K371" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L371" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M371" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N371" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/F7gAAeSwVqpqtbs0/s-l1600.jpg | https://i.ebayimg.com/images/g/vYwAAeSwdOhqtbs1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O371" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P371" s="2" t="inlineStr"/>
+      <c r="Q371" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R371" s="2" t="inlineStr"/>
+      <c r="S371" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="2" t="inlineStr">
+        <is>
+          <t>Victoria Jimenez Kasintseva</t>
+        </is>
+      </c>
+      <c r="B372" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C372" s="2" t="inlineStr">
+        <is>
+          <t>2024 Graphite Advantage 75/75 Victoria Jimenez Kasintseva Rookie Auto RC 0nr3</t>
+        </is>
+      </c>
+      <c r="D372" s="2" t="inlineStr">
+        <is>
+          <t>75/75</t>
+        </is>
+      </c>
+      <c r="E372" s="2" t="inlineStr">
+        <is>
+          <t>last of 75 (75/75)</t>
+        </is>
+      </c>
+      <c r="F372" s="2" t="inlineStr">
+        <is>
+          <t>11.98 USD</t>
+        </is>
+      </c>
+      <c r="G372" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336810989471</t>
+        </is>
+      </c>
+      <c r="H372" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:41 UTC</t>
+        </is>
+      </c>
+      <c r="I372" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TSEAAeSwtA5qtVSK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J372" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T16:48:09.000Z</t>
+        </is>
+      </c>
+      <c r="K372" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L372" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M372" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N372" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/wEwAAeSw~mRqtVSK/s-l1600.jpg | https://i.ebayimg.com/images/g/0iUAAeSwQLZqtVSK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O372" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P372" s="2" t="inlineStr"/>
+      <c r="Q372" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R372" s="2" t="inlineStr"/>
+      <c r="S372" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="2" t="inlineStr">
+        <is>
+          <t>Ryan Harrison</t>
+        </is>
+      </c>
+      <c r="B373" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Regalia Relics - Green</t>
+        </is>
+      </c>
+      <c r="C373" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Regalia Relics Green 5/5 Ryan Harrison #RER-RH Rookie RC 9et</t>
+        </is>
+      </c>
+      <c r="D373" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E373" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F373" s="2" t="inlineStr">
+        <is>
+          <t>58.33 USD</t>
+        </is>
+      </c>
+      <c r="G373" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237090153567</t>
+        </is>
+      </c>
+      <c r="H373" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:41 UTC</t>
+        </is>
+      </c>
+      <c r="I373" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ij0AAeSwGTlqtnVt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J373" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T13:20:43.000Z</t>
+        </is>
+      </c>
+      <c r="K373" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L373" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M373" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N373" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/sK0AAeSwA3FqtnVt/s-l1600.jpg | https://i.ebayimg.com/images/g/mbYAAeSwJOVqtnVt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O373" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P373" s="2" t="inlineStr"/>
+      <c r="Q373" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R373" s="2" t="inlineStr"/>
+      <c r="S373" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="2" t="inlineStr">
+        <is>
+          <t>Daniel Rincon</t>
+        </is>
+      </c>
+      <c r="B374" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Rookie Relic Autographs - Gold</t>
+        </is>
+      </c>
+      <c r="C374" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Rookie Relic Gold 10/10 Daniel Rincon #RRA-DR Auto RC 3hd</t>
+        </is>
+      </c>
+      <c r="D374" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E374" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F374" s="2" t="inlineStr">
+        <is>
+          <t>35.03 USD</t>
+        </is>
+      </c>
+      <c r="G374" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257764864164</t>
+        </is>
+      </c>
+      <c r="H374" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:41 UTC</t>
+        </is>
+      </c>
+      <c r="I374" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/w~AAAeSwEstqtlwZ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J374" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:32:42.000Z</t>
+        </is>
+      </c>
+      <c r="K374" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L374" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M374" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N374" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9O4AAeSwLGtqtlwZ/s-l1600.jpg | https://i.ebayimg.com/images/g/LBEAAeSw9uZqtlwZ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O374" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P374" s="2" t="inlineStr"/>
+      <c r="Q374" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R374" s="2" t="inlineStr"/>
+      <c r="S374" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="2" t="inlineStr">
+        <is>
+          <t>Toby Kodat</t>
+        </is>
+      </c>
+      <c r="B375" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Rookie Jumbo Relics - Green</t>
+        </is>
+      </c>
+      <c r="C375" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Rookie Jumbo Relics Green 1/5 Toby Kodat #RJR-TK RC 1fl4</t>
+        </is>
+      </c>
+      <c r="D375" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E375" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F375" s="2" t="inlineStr">
+        <is>
+          <t>35.03 USD</t>
+        </is>
+      </c>
+      <c r="G375" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336812253487</t>
+        </is>
+      </c>
+      <c r="H375" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:41 UTC</t>
+        </is>
+      </c>
+      <c r="I375" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/R-kAAeSwGTlqtlIj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J375" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T10:50:10.000Z</t>
+        </is>
+      </c>
+      <c r="K375" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L375" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M375" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N375" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/N7MAAeSwq2VqtlIj/s-l1600.jpg | https://i.ebayimg.com/images/g/OpIAAeSwGAhqtlIj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O375" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P375" s="2" t="inlineStr"/>
+      <c r="Q375" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R375" s="2" t="inlineStr"/>
+      <c r="S375" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="2" t="inlineStr">
+        <is>
+          <t>Lorenzo Musetti</t>
+        </is>
+      </c>
+      <c r="B376" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Triumph Relic Signatures - Blue</t>
+        </is>
+      </c>
+      <c r="C376" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Blue 1/25 Lorenzo Musetti #TRS-LM Rookie Auto RC ne4</t>
+        </is>
+      </c>
+      <c r="D376" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E376" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F376" s="2" t="inlineStr">
+        <is>
+          <t>228.34 USD</t>
+        </is>
+      </c>
+      <c r="G376" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336812222146</t>
+        </is>
+      </c>
+      <c r="H376" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:41 UTC</t>
+        </is>
+      </c>
+      <c r="I376" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KRwAAeSwaHNqtkoo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J376" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T10:16:07.000Z</t>
+        </is>
+      </c>
+      <c r="K376" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L376" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M376" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N376" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/b4IAAeSw6OVqtkoo/s-l1600.jpg | https://i.ebayimg.com/images/g/6T0AAeSwFClqtkoo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O376" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P376" s="2" t="inlineStr"/>
+      <c r="Q376" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R376" s="2" t="inlineStr"/>
+      <c r="S376" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="2" t="inlineStr">
+        <is>
+          <t>Kilian Feldbausch</t>
+        </is>
+      </c>
+      <c r="B377" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Rookie Jumbo Relics - Gold</t>
+        </is>
+      </c>
+      <c r="C377" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Rookie Jumbo Relics Gold 1/10 Kilian Feldbausch #RJR-KF r5f</t>
+        </is>
+      </c>
+      <c r="D377" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E377" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F377" s="2" t="inlineStr">
+        <is>
+          <t>18.08 USD</t>
+        </is>
+      </c>
+      <c r="G377" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257764642976</t>
+        </is>
+      </c>
+      <c r="H377" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:41 UTC</t>
+        </is>
+      </c>
+      <c r="I377" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7e4AAeSwS1lqtit3/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J377" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T08:05:09.000Z</t>
+        </is>
+      </c>
+      <c r="K377" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L377" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M377" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N377" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/72QAAeSwnm9qtit3/s-l1600.jpg | https://i.ebayimg.com/images/g/BmwAAeSw8D1qtit3/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O377" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P377" s="2" t="inlineStr"/>
+      <c r="Q377" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R377" s="2" t="inlineStr"/>
+      <c r="S377" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="2" t="inlineStr">
+        <is>
+          <t>Taro Daniel</t>
+        </is>
+      </c>
+      <c r="B378" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Imperial Ink - Blue</t>
+        </is>
+      </c>
+      <c r="C378" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Imperial Ink Blue 1/25 Taro Daniel #II-TDL Rookie Auto RC 9et</t>
+        </is>
+      </c>
+      <c r="D378" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E378" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F378" s="2" t="inlineStr">
+        <is>
+          <t>41.08 USD</t>
+        </is>
+      </c>
+      <c r="G378" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237089480057</t>
+        </is>
+      </c>
+      <c r="H378" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:41 UTC</t>
+        </is>
+      </c>
+      <c r="I378" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/seIAAeSwG9lqtf3L/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J378" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T04:50:13.000Z</t>
+        </is>
+      </c>
+      <c r="K378" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L378" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M378" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N378" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~MkAAeSwIZxqtf3L/s-l1600.jpg | https://i.ebayimg.com/images/g/GikAAeSwXS1qtf3L/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O378" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P378" s="2" t="inlineStr"/>
+      <c r="Q378" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R378" s="2" t="inlineStr"/>
+      <c r="S378" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff, Emma Raducanu</t>
+        </is>
+      </c>
+      <c r="B379" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Collection Tennis</t>
+        </is>
+      </c>
+      <c r="C379" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2024 Royalty Tennis Coco Gauff Emma Raducanu Relic PSP-CR 25/25 BOOKEND🔥</t>
+        </is>
+      </c>
+      <c r="D379" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E379" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F379" s="2" t="inlineStr">
+        <is>
+          <t>79.99 USD</t>
+        </is>
+      </c>
+      <c r="G379" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336810841615</t>
+        </is>
+      </c>
+      <c r="H379" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:41 UTC</t>
+        </is>
+      </c>
+      <c r="I379" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/OHgAAeSw7AlqtTop/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J379" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T15:02:51.000Z</t>
+        </is>
+      </c>
+      <c r="K379" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L379" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M379" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N379" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TrYAAeSwmEBqtTn5/s-l1600.jpg | https://i.ebayimg.com/images/g/StEAAeSwiKpqtTn8/s-l1600.jpg | https://i.ebayimg.com/images/g/MWQAAeSwaSpqtTn6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O379" s="2" t="inlineStr"/>
+      <c r="P379" s="2" t="inlineStr"/>
+      <c r="Q379" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R379" s="2" t="inlineStr"/>
+      <c r="S379" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="2" t="inlineStr">
+        <is>
+          <t>Nicola Pietrangeli</t>
+        </is>
+      </c>
+      <c r="B380" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic, Inc / 2012 Ace Authentic Grand Slam 3 - [Base] - Printing Plate Cyan</t>
+        </is>
+      </c>
+      <c r="C380" s="2" t="inlineStr">
+        <is>
+          <t>2012 Ace Authentic Grand Slam 3 Printing Plate Cyan 1/1 Nicola Pietrangeli 0n8h</t>
+        </is>
+      </c>
+      <c r="D380" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E380" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F380" s="2" t="inlineStr">
+        <is>
+          <t>23.83 USD</t>
+        </is>
+      </c>
+      <c r="G380" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336811648493</t>
+        </is>
+      </c>
+      <c r="H380" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:41 UTC</t>
+        </is>
+      </c>
+      <c r="I380" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9TYAAeSwI1Nqtc1M/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J380" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T01:24:25.000Z</t>
+        </is>
+      </c>
+      <c r="K380" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L380" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M380" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N380" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2NUAAeSwylhqtc1M/s-l1600.jpg | https://i.ebayimg.com/images/g/c4MAAeSwKCNqtc1M/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O380" s="2" t="inlineStr">
+        <is>
+          <t>cyan</t>
+        </is>
+      </c>
+      <c r="P380" s="2" t="inlineStr"/>
+      <c r="Q380" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R380" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic, Inc: check the numbering is stamped, not on a circle sticker</t>
+        </is>
+      </c>
+      <c r="S380" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -32279,6 +33881,24 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G360" r:id="rId359"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G361" r:id="rId360"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G362" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G363" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G364" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G365" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G366" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G367" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G368" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G369" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G370" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G371" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G372" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G373" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G374" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G375" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G376" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G377" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G378" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G379" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G380" r:id="rId379"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-26 13:49 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S380"/>
+  <dimension ref="A1:S394"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -33513,6 +33513,1244 @@
         </is>
       </c>
       <c r="S380" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="2" t="inlineStr">
+        <is>
+          <t>Martina Navratilova</t>
+        </is>
+      </c>
+      <c r="B381" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C381" s="2" t="inlineStr">
+        <is>
+          <t>2021 Chrome Rose Gold Refractor 1/10 Martina Navratilova BGS 9.5 GEM MINT ob9</t>
+        </is>
+      </c>
+      <c r="D381" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E381" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F381" s="2" t="inlineStr">
+        <is>
+          <t>100.30 USD</t>
+        </is>
+      </c>
+      <c r="G381" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257766567843</t>
+        </is>
+      </c>
+      <c r="H381" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:48 UTC</t>
+        </is>
+      </c>
+      <c r="I381" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/oHkAAeSwhodqt33R/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J381" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T08:08:49.000Z</t>
+        </is>
+      </c>
+      <c r="K381" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L381" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M381" s="2" t="inlineStr">
+        <is>
+          <t>Beckett (BGS) 9.5 GEM MINT</t>
+        </is>
+      </c>
+      <c r="N381" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/LU0AAeSwlYNqt33R/s-l1600.jpg | https://i.ebayimg.com/images/g/BvgAAeSwDtpqt33R/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O381" s="2" t="inlineStr">
+        <is>
+          <t>rose</t>
+        </is>
+      </c>
+      <c r="P381" s="2" t="inlineStr"/>
+      <c r="Q381" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R381" s="2" t="inlineStr"/>
+      <c r="S381" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="2" t="inlineStr">
+        <is>
+          <t>Daria Kasatkina</t>
+        </is>
+      </c>
+      <c r="B382" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C382" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Black Refractor 10/10 Daria Kasatkina #146 Rookie RC 0t30</t>
+        </is>
+      </c>
+      <c r="D382" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E382" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F382" s="2" t="inlineStr">
+        <is>
+          <t>52.29 USD</t>
+        </is>
+      </c>
+      <c r="G382" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336813566693</t>
+        </is>
+      </c>
+      <c r="H382" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:48 UTC</t>
+        </is>
+      </c>
+      <c r="I382" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/6VoAAeSwrcFqt2W8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J382" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T06:26:05.000Z</t>
+        </is>
+      </c>
+      <c r="K382" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L382" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M382" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N382" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/IA8AAeSw0Pxqt2W8/s-l1600.jpg | https://i.ebayimg.com/images/g/EkMAAeSwiQdqt2W8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O382" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P382" s="2" t="inlineStr"/>
+      <c r="Q382" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R382" s="2" t="inlineStr"/>
+      <c r="S382" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="2" t="inlineStr">
+        <is>
+          <t>Alexandra Alex Eala</t>
+        </is>
+      </c>
+      <c r="B383" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C383" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Alexandra Alex Eala Pink Geometric 65/65 OC58</t>
+        </is>
+      </c>
+      <c r="D383" s="2" t="inlineStr">
+        <is>
+          <t>65/65</t>
+        </is>
+      </c>
+      <c r="E383" s="2" t="inlineStr">
+        <is>
+          <t>last of 65 (65/65)</t>
+        </is>
+      </c>
+      <c r="F383" s="2" t="inlineStr">
+        <is>
+          <t>4.25 USD</t>
+        </is>
+      </c>
+      <c r="G383" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407246290947</t>
+        </is>
+      </c>
+      <c r="H383" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:48 UTC</t>
+        </is>
+      </c>
+      <c r="I383" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/xXsAAeSwouBqt0E9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J383" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T03:50:21.000Z</t>
+        </is>
+      </c>
+      <c r="K383" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L383" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M383" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N383" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/85QAAeSw~7tqt0E9/s-l1600.jpg | https://i.ebayimg.com/images/g/ffYAAeSwffpqt0E9/s-l1600.jpg | https://i.ebayimg.com/images/g/jFIAAeSwbKtqt0E9/s-l1600.jpg | https://i.ebayimg.com/images/g/xJMAAeSweTFqt0E8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O383" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P383" s="2" t="inlineStr"/>
+      <c r="Q383" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R383" s="2" t="inlineStr"/>
+      <c r="S383" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="2" t="inlineStr">
+        <is>
+          <t>Luca Van Assche</t>
+        </is>
+      </c>
+      <c r="B384" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C384" s="2" t="inlineStr">
+        <is>
+          <t>2024 Graphite Match Masters Aqua Refractor 199/199 Luca Van Assche Rookie RC 7k8</t>
+        </is>
+      </c>
+      <c r="D384" s="2" t="inlineStr">
+        <is>
+          <t>199/199</t>
+        </is>
+      </c>
+      <c r="E384" s="2" t="inlineStr">
+        <is>
+          <t>last of 199 (199/199)</t>
+        </is>
+      </c>
+      <c r="F384" s="2" t="inlineStr">
+        <is>
+          <t>4.28 USD</t>
+        </is>
+      </c>
+      <c r="G384" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336813910375</t>
+        </is>
+      </c>
+      <c r="H384" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:48 UTC</t>
+        </is>
+      </c>
+      <c r="I384" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/BnYAAeSwOktqt7mC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J384" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T12:23:30.000Z</t>
+        </is>
+      </c>
+      <c r="K384" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L384" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M384" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N384" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/y9AAAeSwQLZqt7mD/s-l1600.jpg | https://i.ebayimg.com/images/g/C9YAAeSwcS9qt7mD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O384" s="2" t="inlineStr">
+        <is>
+          <t>aqua</t>
+        </is>
+      </c>
+      <c r="P384" s="2" t="inlineStr"/>
+      <c r="Q384" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R384" s="2" t="inlineStr"/>
+      <c r="S384" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="2" t="inlineStr">
+        <is>
+          <t>Joao Fonseca</t>
+        </is>
+      </c>
+      <c r="B385" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite Tennis</t>
+        </is>
+      </c>
+      <c r="C385" s="2" t="inlineStr">
+        <is>
+          <t>2026 TOPPS GRAPHITE TENNIS BREAK POINT JOAO FONSECA ROOKIE BLUE REFRACTOR-#01/50</t>
+        </is>
+      </c>
+      <c r="D385" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E385" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F385" s="2" t="inlineStr">
+        <is>
+          <t>74.00 USD</t>
+        </is>
+      </c>
+      <c r="G385" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/398432325612</t>
+        </is>
+      </c>
+      <c r="H385" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:48 UTC</t>
+        </is>
+      </c>
+      <c r="I385" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/dfgAAeSwiQdqtwhB/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J385" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T23:52:44.000Z</t>
+        </is>
+      </c>
+      <c r="K385" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L385" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M385" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N385" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7R0AAeSw0O5qtwc3/s-l1600.jpg | https://i.ebayimg.com/images/g/do8AAeSwFmBqtwj3/s-l1600.jpg | https://i.ebayimg.com/images/g/elsAAeSwlCJqtwij/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O385" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P385" s="2" t="inlineStr"/>
+      <c r="Q385" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R385" s="2" t="inlineStr"/>
+      <c r="S385" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="2" t="inlineStr">
+        <is>
+          <t>Sebastian Ofner</t>
+        </is>
+      </c>
+      <c r="B386" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C386" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Gold Refractor 25/25 Sebastian Ofner #18 Rookie RC nd3</t>
+        </is>
+      </c>
+      <c r="D386" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E386" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F386" s="2" t="inlineStr">
+        <is>
+          <t>14.34 USD</t>
+        </is>
+      </c>
+      <c r="G386" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257765432931</t>
+        </is>
+      </c>
+      <c r="H386" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:48 UTC</t>
+        </is>
+      </c>
+      <c r="I386" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SfUAAeSwl~pqtrdQ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J386" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T18:01:53.000Z</t>
+        </is>
+      </c>
+      <c r="K386" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L386" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M386" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N386" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/IK8AAeSwj5pqtrdQ/s-l1600.jpg | https://i.ebayimg.com/images/g/vbgAAeSw9uZqtrdQ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O386" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P386" s="2" t="inlineStr"/>
+      <c r="Q386" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R386" s="2" t="inlineStr"/>
+      <c r="S386" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B387" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS GRAPHITE TENNIS SIGNATURE SERVES</t>
+        </is>
+      </c>
+      <c r="C387" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS GRAPHITE TENNIS SIGNATURE SERVES MIRRA ANDREEVA RC 1/50 BLUE AUTO</t>
+        </is>
+      </c>
+      <c r="D387" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E387" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F387" s="2" t="inlineStr">
+        <is>
+          <t>225.00 USD</t>
+        </is>
+      </c>
+      <c r="G387" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366691884243?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2FtonuTnlUXHjma7OEMSokfoIvdBBt5GMBpbJCQ9lXn8KBZ1weIjYHlgldsT06yKjjau1Z6MkHcvjnxZNS5kPt1esS2%2B4RvQzy0BhFzI%2F0Cf3uTGsLrEldrogMeOFIDYMyULFZpZhv71BVDSmLxrEnJMUMBsMZFIGCAwXpQXYhfCfs857ZaVxRwoyc7xBxuOe8%3D</t>
+        </is>
+      </c>
+      <c r="H387" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:48 UTC</t>
+        </is>
+      </c>
+      <c r="I387" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/VCEAAeSwOZtqtqR1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J387" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T16:42:44.000Z</t>
+        </is>
+      </c>
+      <c r="K387" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L387" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M387" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N387" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/LV8AAeSwHmxqtqR1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O387" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P387" s="2" t="inlineStr"/>
+      <c r="Q387" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R387" s="2" t="inlineStr"/>
+      <c r="S387" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="2" t="inlineStr">
+        <is>
+          <t>Rinky Hijikata</t>
+        </is>
+      </c>
+      <c r="B388" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Rookie Autographs - Blue</t>
+        </is>
+      </c>
+      <c r="C388" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Rookie Blue 1/25 Rinky Hijikata #RA-RH Auto RC 9et</t>
+        </is>
+      </c>
+      <c r="D388" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E388" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F388" s="2" t="inlineStr">
+        <is>
+          <t>46.83 USD</t>
+        </is>
+      </c>
+      <c r="G388" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257766860060</t>
+        </is>
+      </c>
+      <c r="H388" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:48 UTC</t>
+        </is>
+      </c>
+      <c r="I388" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JNEAAeSwtN5qt7BQ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J388" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:45:18.000Z</t>
+        </is>
+      </c>
+      <c r="K388" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L388" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M388" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N388" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/kMkAAeSwY5Bqt7BQ/s-l1600.jpg | https://i.ebayimg.com/images/g/NlMAAeSwA0Jqt7BQ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O388" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P388" s="2" t="inlineStr"/>
+      <c r="Q388" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R388" s="2" t="inlineStr"/>
+      <c r="S388" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="2" t="inlineStr">
+        <is>
+          <t>Taro Daniel</t>
+        </is>
+      </c>
+      <c r="B389" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Pursuit of Greatness Signatures - Gold</t>
+        </is>
+      </c>
+      <c r="C389" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Gold 10/10 Taro Daniel #PGS-TDL Rookie Auto RC 1e41</t>
+        </is>
+      </c>
+      <c r="D389" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E389" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F389" s="2" t="inlineStr">
+        <is>
+          <t>28.99 USD</t>
+        </is>
+      </c>
+      <c r="G389" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237091139998</t>
+        </is>
+      </c>
+      <c r="H389" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:48 UTC</t>
+        </is>
+      </c>
+      <c r="I389" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KG4AAeSwStVqtzQv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J389" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T02:54:40.000Z</t>
+        </is>
+      </c>
+      <c r="K389" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L389" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M389" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N389" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/cBIAAeSwPyFqtzQv/s-l1600.jpg | https://i.ebayimg.com/images/g/YzIAAeSwbhdqtzQv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O389" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P389" s="2" t="inlineStr"/>
+      <c r="Q389" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R389" s="2" t="inlineStr"/>
+      <c r="S389" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="2" t="inlineStr">
+        <is>
+          <t>Alex de Minaur</t>
+        </is>
+      </c>
+      <c r="B390" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Royalty Collection</t>
+        </is>
+      </c>
+      <c r="C390" s="2" t="inlineStr">
+        <is>
+          <t>Alex de Minaur 2024 Topps Royalty Tennis Regalia Relic Signatures 1/75 TF1</t>
+        </is>
+      </c>
+      <c r="D390" s="2" t="inlineStr">
+        <is>
+          <t>1/75</t>
+        </is>
+      </c>
+      <c r="E390" s="2" t="inlineStr">
+        <is>
+          <t>001 of 75</t>
+        </is>
+      </c>
+      <c r="F390" s="2" t="inlineStr">
+        <is>
+          <t>1.25 USD</t>
+        </is>
+      </c>
+      <c r="G390" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/267795781474</t>
+        </is>
+      </c>
+      <c r="H390" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:48 UTC</t>
+        </is>
+      </c>
+      <c r="I390" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/P7YAAeSwtUBqttww/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J390" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T02:37:00.000Z</t>
+        </is>
+      </c>
+      <c r="K390" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L390" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M390" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N390" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/K-IAAeSwGGtqttww/s-l1600.jpg | https://i.ebayimg.com/images/g/8WcAAeSwSL1qttww/s-l1600.jpg | https://i.ebayimg.com/images/g/BeEAAeSwVvlqttww/s-l1600.jpg | https://i.ebayimg.com/images/g/GzkAAeSwoZtqttww/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O390" s="2" t="inlineStr"/>
+      <c r="P390" s="2" t="inlineStr"/>
+      <c r="Q390" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R390" s="2" t="inlineStr"/>
+      <c r="S390" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="2" t="inlineStr">
+        <is>
+          <t>Shintaro Mochizuki</t>
+        </is>
+      </c>
+      <c r="B391" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Imperial Ink - Green</t>
+        </is>
+      </c>
+      <c r="C391" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Imperial Ink Green 1/5 Shintaro Mochizuki Rookie Auto RC 1e41</t>
+        </is>
+      </c>
+      <c r="D391" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E391" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F391" s="2" t="inlineStr">
+        <is>
+          <t>66.95 USD</t>
+        </is>
+      </c>
+      <c r="G391" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257765836760</t>
+        </is>
+      </c>
+      <c r="H391" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:49 UTC</t>
+        </is>
+      </c>
+      <c r="I391" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JL8AAeSwQLZqtvpN/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J391" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T22:47:38.000Z</t>
+        </is>
+      </c>
+      <c r="K391" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L391" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M391" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N391" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/38cAAeSwssFqtvpN/s-l1600.jpg | https://i.ebayimg.com/images/g/p6MAAeSwdOhqtvpN/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O391" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P391" s="2" t="inlineStr"/>
+      <c r="Q391" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R391" s="2" t="inlineStr"/>
+      <c r="S391" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="2" t="inlineStr">
+        <is>
+          <t>Zizou Bergs</t>
+        </is>
+      </c>
+      <c r="B392" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Tennis</t>
+        </is>
+      </c>
+      <c r="C392" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis Zizou Bergs #RER-ZB Regalia Relic Patch Platinum 1/1</t>
+        </is>
+      </c>
+      <c r="D392" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E392" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F392" s="2" t="inlineStr">
+        <is>
+          <t>1100.00 USD</t>
+        </is>
+      </c>
+      <c r="G392" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/188983921914</t>
+        </is>
+      </c>
+      <c r="H392" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:49 UTC</t>
+        </is>
+      </c>
+      <c r="I392" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/OlEAAeSwzpZqtrYC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J392" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T18:01:05.000Z</t>
+        </is>
+      </c>
+      <c r="K392" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L392" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M392" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N392" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/eKMAAeSwr5dqtrYC/s-l1600.jpg | https://i.ebayimg.com/images/g/WYIAAeSw1E5qtrYC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O392" s="2" t="inlineStr"/>
+      <c r="P392" s="2" t="inlineStr"/>
+      <c r="Q392" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R392" s="2" t="inlineStr"/>
+      <c r="S392" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="2" t="inlineStr">
+        <is>
+          <t>Aryna Sabalenka</t>
+        </is>
+      </c>
+      <c r="B393" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Tennis</t>
+        </is>
+      </c>
+      <c r="C393" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Aryna Sabalenka Superior Relic Auto Green #1/5 Nike Swoosh</t>
+        </is>
+      </c>
+      <c r="D393" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E393" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F393" s="2" t="inlineStr">
+        <is>
+          <t>4000.00 USD</t>
+        </is>
+      </c>
+      <c r="G393" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/188983916493</t>
+        </is>
+      </c>
+      <c r="H393" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:49 UTC</t>
+        </is>
+      </c>
+      <c r="I393" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HMMAAeSwGRBqtrRV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J393" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T17:56:14.000Z</t>
+        </is>
+      </c>
+      <c r="K393" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L393" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M393" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N393" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/NpoAAeSwtN5qtrRU/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O393" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P393" s="2" t="inlineStr"/>
+      <c r="Q393" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R393" s="2" t="inlineStr"/>
+      <c r="S393" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="2" t="inlineStr">
+        <is>
+          <t>Joao Fonseca</t>
+        </is>
+      </c>
+      <c r="B394" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Now</t>
+        </is>
+      </c>
+      <c r="C394" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Now Joao Fonseca French Open Djokivic RED AUTOGRAPH (#'d 5/5) Rookie</t>
+        </is>
+      </c>
+      <c r="D394" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E394" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F394" s="2" t="inlineStr">
+        <is>
+          <t>1025.00 USD</t>
+        </is>
+      </c>
+      <c r="G394" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298707273016</t>
+        </is>
+      </c>
+      <c r="H394" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:49 UTC</t>
+        </is>
+      </c>
+      <c r="I394" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/zXoAAeSwuhlqtvcw/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J394" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T00:01:01.000Z</t>
+        </is>
+      </c>
+      <c r="K394" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L394" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M394" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA)</t>
+        </is>
+      </c>
+      <c r="N394" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/OYoAAeSw1kVqtvc8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O394" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P394" s="2" t="inlineStr"/>
+      <c r="Q394" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R394" s="2" t="inlineStr"/>
+      <c r="S394" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -33899,6 +35137,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G378" r:id="rId377"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G379" r:id="rId378"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G380" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G381" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G382" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G383" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G384" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G385" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G386" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G387" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G388" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G389" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G390" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G391" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G392" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G393" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G394" r:id="rId393"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-27 14:48 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S394"/>
+  <dimension ref="A1:S418"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -34751,6 +34751,2122 @@
       </c>
       <c r="R394" s="2" t="inlineStr"/>
       <c r="S394" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="2" t="inlineStr">
+        <is>
+          <t>Ugo Humbert</t>
+        </is>
+      </c>
+      <c r="B395" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C395" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Purple Geometric Refractor 1/15 Ugo Humbert Rookie RC 1e41</t>
+        </is>
+      </c>
+      <c r="D395" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E395" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F395" s="2" t="inlineStr">
+        <is>
+          <t>23.25 USD</t>
+        </is>
+      </c>
+      <c r="G395" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237093351030</t>
+        </is>
+      </c>
+      <c r="H395" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I395" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/zKcAAeSwJsNquQgc/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J395" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T12:11:08.000Z</t>
+        </is>
+      </c>
+      <c r="K395" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L395" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M395" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N395" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/xScAAeSw4KJquQgb/s-l1600.jpg | https://i.ebayimg.com/images/g/aGoAAeSwlYNquQgb/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O395" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P395" s="2" t="inlineStr"/>
+      <c r="Q395" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R395" s="2" t="inlineStr"/>
+      <c r="S395" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="2" t="inlineStr">
+        <is>
+          <t>Julia Grabher</t>
+        </is>
+      </c>
+      <c r="B396" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C396" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome FrozenFractor -1/5 Julia Grabher #97 Rookie RC 0t30</t>
+        </is>
+      </c>
+      <c r="D396" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E396" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F396" s="2" t="inlineStr">
+        <is>
+          <t>75.29 USD</t>
+        </is>
+      </c>
+      <c r="G396" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336815278333</t>
+        </is>
+      </c>
+      <c r="H396" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I396" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ir0AAeSwjQRquPLf/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J396" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T10:40:32.000Z</t>
+        </is>
+      </c>
+      <c r="K396" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L396" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M396" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N396" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/6oMAAeSwa3NquPLf/s-l1600.jpg | https://i.ebayimg.com/images/g/okEAAeSwSGxquPLf/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O396" s="2" t="inlineStr"/>
+      <c r="P396" s="2" t="inlineStr"/>
+      <c r="Q396" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R396" s="2" t="inlineStr"/>
+      <c r="S396" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="2" t="inlineStr">
+        <is>
+          <t>Brenda Fruhvirtova</t>
+        </is>
+      </c>
+      <c r="B397" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C397" s="2" t="inlineStr">
+        <is>
+          <t>2024 Chrome Pink Geometric Refractor 65/65 Brenda Fruhvirtova #156 Rookie RC 9et</t>
+        </is>
+      </c>
+      <c r="D397" s="2" t="inlineStr">
+        <is>
+          <t>65/65</t>
+        </is>
+      </c>
+      <c r="E397" s="2" t="inlineStr">
+        <is>
+          <t>last of 65 (65/65)</t>
+        </is>
+      </c>
+      <c r="F397" s="2" t="inlineStr">
+        <is>
+          <t>10.03 USD</t>
+        </is>
+      </c>
+      <c r="G397" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257768383785</t>
+        </is>
+      </c>
+      <c r="H397" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I397" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~LEAAeSwnulquMWr/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J397" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T07:27:36.000Z</t>
+        </is>
+      </c>
+      <c r="K397" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L397" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M397" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N397" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/y40AAeSweVVquMWr/s-l1600.jpg | https://i.ebayimg.com/images/g/xUMAAeSw7xdquMWr/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O397" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P397" s="2" t="inlineStr"/>
+      <c r="Q397" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R397" s="2" t="inlineStr"/>
+      <c r="S397" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="2" t="inlineStr">
+        <is>
+          <t>Yue Yuan</t>
+        </is>
+      </c>
+      <c r="B398" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C398" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome FrozenFractor -1/5 Yue Yuan #7 Rookie RC ux8</t>
+        </is>
+      </c>
+      <c r="D398" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E398" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F398" s="2" t="inlineStr">
+        <is>
+          <t>92.83 USD</t>
+        </is>
+      </c>
+      <c r="G398" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336815050592</t>
+        </is>
+      </c>
+      <c r="H398" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I398" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/f7EAAeSwM99quL8J/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J398" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T06:59:22.000Z</t>
+        </is>
+      </c>
+      <c r="K398" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L398" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M398" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N398" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vs8AAeSwYu9quL8J/s-l1600.jpg | https://i.ebayimg.com/images/g/rMIAAeSwh-dquL8J/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O398" s="2" t="inlineStr"/>
+      <c r="P398" s="2" t="inlineStr"/>
+      <c r="Q398" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R398" s="2" t="inlineStr"/>
+      <c r="S398" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="2" t="inlineStr">
+        <is>
+          <t>Pete Sampras</t>
+        </is>
+      </c>
+      <c r="B399" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS CHROME TENNIS IMAGE VARIATION AUTOGR...</t>
+        </is>
+      </c>
+      <c r="C399" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS CHROME TENNIS IMAGE VARIATION AUTOS #AIVPSS PETE SAMPRAS 1/1 PSA 8</t>
+        </is>
+      </c>
+      <c r="D399" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E399" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F399" s="2" t="inlineStr">
+        <is>
+          <t>45000.00 USD</t>
+        </is>
+      </c>
+      <c r="G399" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298710325094</t>
+        </is>
+      </c>
+      <c r="H399" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I399" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/tMAAAeSwcTJquJE5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J399" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T03:43:51.000Z</t>
+        </is>
+      </c>
+      <c r="K399" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L399" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M399" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 8</t>
+        </is>
+      </c>
+      <c r="N399" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SLYAAeSw4KJquJE5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O399" s="2" t="inlineStr"/>
+      <c r="P399" s="2" t="inlineStr"/>
+      <c r="Q399" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R399" s="2" t="inlineStr"/>
+      <c r="S399" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="2" t="inlineStr">
+        <is>
+          <t>Jack Draper</t>
+        </is>
+      </c>
+      <c r="B400" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Sapphire Edition - [Base] - Red</t>
+        </is>
+      </c>
+      <c r="C400" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Sapphire Red 1/5 Jack Draper #28 0r9h</t>
+        </is>
+      </c>
+      <c r="D400" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E400" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F400" s="2" t="inlineStr">
+        <is>
+          <t>175.55 USD</t>
+        </is>
+      </c>
+      <c r="G400" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237092797323</t>
+        </is>
+      </c>
+      <c r="H400" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I400" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/u1UAAeSwNiZquIxI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J400" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T03:22:50.000Z</t>
+        </is>
+      </c>
+      <c r="K400" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L400" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M400" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N400" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/IjAAAeSwg0dquIxI/s-l1600.jpg | https://i.ebayimg.com/images/g/suIAAeSw7AlquIxI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O400" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P400" s="2" t="inlineStr"/>
+      <c r="Q400" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R400" s="2" t="inlineStr"/>
+      <c r="S400" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="2" t="inlineStr">
+        <is>
+          <t>Paula Badosa</t>
+        </is>
+      </c>
+      <c r="B401" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C401" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Orange Refractor Captured #15 Paula Badosa 1/25</t>
+        </is>
+      </c>
+      <c r="D401" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E401" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F401" s="2" t="inlineStr">
+        <is>
+          <t>25.00 USD</t>
+        </is>
+      </c>
+      <c r="G401" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/278412675735</t>
+        </is>
+      </c>
+      <c r="H401" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I401" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DsEAAeSwdFlquHju/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J401" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T02:01:25.000Z</t>
+        </is>
+      </c>
+      <c r="K401" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L401" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M401" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N401" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/z2MAAeSwMnxquHju/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O401" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P401" s="2" t="inlineStr"/>
+      <c r="Q401" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R401" s="2" t="inlineStr"/>
+      <c r="S401" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek</t>
+        </is>
+      </c>
+      <c r="B402" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C402" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek 2025 Topps Chrome Sapphire Tennis Purple Sapphire 01/10 PSA 10 [2hk</t>
+        </is>
+      </c>
+      <c r="D402" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E402" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F402" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G402" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377525584734</t>
+        </is>
+      </c>
+      <c r="H402" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I402" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~6kAAeSw75lquHP6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J402" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T01:39:07.000Z</t>
+        </is>
+      </c>
+      <c r="K402" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L402" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M402" s="2" t="inlineStr">
+        <is>
+          <t>PSA 10</t>
+        </is>
+      </c>
+      <c r="N402" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/5AMAAeSwbhdquHP8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O402" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P402" s="2" t="inlineStr"/>
+      <c r="Q402" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R402" s="2" t="inlineStr"/>
+      <c r="S402" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="2" t="inlineStr">
+        <is>
+          <t>Xiyu Wang</t>
+        </is>
+      </c>
+      <c r="B403" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite - Rally Relics - Pink Refractor</t>
+        </is>
+      </c>
+      <c r="C403" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Rally Relics Pink Refractor 15/15 Xiyu Wang #RR-XW 17uv</t>
+        </is>
+      </c>
+      <c r="D403" s="2" t="inlineStr">
+        <is>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="E403" s="2" t="inlineStr">
+        <is>
+          <t>last of 15 (15/15)</t>
+        </is>
+      </c>
+      <c r="F403" s="2" t="inlineStr">
+        <is>
+          <t>18.07 USD</t>
+        </is>
+      </c>
+      <c r="G403" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336815443288</t>
+        </is>
+      </c>
+      <c r="H403" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I403" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/xEoAAeSwY5BquRpG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J403" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T13:28:37.000Z</t>
+        </is>
+      </c>
+      <c r="K403" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L403" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M403" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N403" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/PCoAAeSwcTJquRpG/s-l1600.jpg | https://i.ebayimg.com/images/g/dlQAAeSwHn1quRpG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O403" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P403" s="2" t="inlineStr"/>
+      <c r="Q403" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R403" s="2" t="inlineStr"/>
+      <c r="S403" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="2" t="inlineStr">
+        <is>
+          <t>Elena Rybakina</t>
+        </is>
+      </c>
+      <c r="B404" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C404" s="2" t="inlineStr">
+        <is>
+          <t>1/1 2024 Topps Graphite T. Elena Rybakina Match Masters Red Crystalline CGC 10</t>
+        </is>
+      </c>
+      <c r="D404" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E404" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F404" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G404" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366694544851</t>
+        </is>
+      </c>
+      <c r="H404" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I404" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jwAAAeSwPKBquIZd/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J404" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T02:57:33.000Z</t>
+        </is>
+      </c>
+      <c r="K404" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L404" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M404" s="2" t="inlineStr">
+        <is>
+          <t>CGC 10</t>
+        </is>
+      </c>
+      <c r="N404" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/OzUAAeSwpPxquIZd/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O404" s="2" t="inlineStr"/>
+      <c r="P404" s="2" t="inlineStr"/>
+      <c r="Q404" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R404" s="2" t="inlineStr"/>
+      <c r="S404" s="2" t="inlineStr">
+        <is>
+          <t>Tennis (网球)</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="2" t="inlineStr">
+        <is>
+          <t>Benoit Paire</t>
+        </is>
+      </c>
+      <c r="B405" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C405" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Ace Relics Pink Refractor 1/15 Benoit Paire Rookie RC z6o</t>
+        </is>
+      </c>
+      <c r="D405" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E405" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F405" s="2" t="inlineStr">
+        <is>
+          <t>9.74 USD</t>
+        </is>
+      </c>
+      <c r="G405" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336814426301</t>
+        </is>
+      </c>
+      <c r="H405" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I405" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2b0AAeSwDLBquC4h/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J405" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T20:41:07.000Z</t>
+        </is>
+      </c>
+      <c r="K405" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L405" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M405" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N405" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/IOoAAeSwmxxquC4h/s-l1600.jpg | https://i.ebayimg.com/images/g/JIEAAeSwkepquC4h/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O405" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P405" s="2" t="inlineStr"/>
+      <c r="Q405" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R405" s="2" t="inlineStr"/>
+      <c r="S405" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="2" t="inlineStr">
+        <is>
+          <t>Taylor Fritz</t>
+        </is>
+      </c>
+      <c r="B406" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C406" s="2" t="inlineStr">
+        <is>
+          <t>2024 Graphite Court Masters Green Refractor 75/75 Taylor Fritz Rookie RC 3p5</t>
+        </is>
+      </c>
+      <c r="D406" s="2" t="inlineStr">
+        <is>
+          <t>75/75</t>
+        </is>
+      </c>
+      <c r="E406" s="2" t="inlineStr">
+        <is>
+          <t>last of 75 (75/75)</t>
+        </is>
+      </c>
+      <c r="F406" s="2" t="inlineStr">
+        <is>
+          <t>23.83 USD</t>
+        </is>
+      </c>
+      <c r="G406" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257767567076</t>
+        </is>
+      </c>
+      <c r="H406" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I406" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/d98AAeSw75lquC03/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J406" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T20:37:03.000Z</t>
+        </is>
+      </c>
+      <c r="K406" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L406" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M406" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N406" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/By0AAeSwtN5quC03/s-l1600.jpg | https://i.ebayimg.com/images/g/mZwAAeSw6z9quC03/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O406" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P406" s="2" t="inlineStr"/>
+      <c r="Q406" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R406" s="2" t="inlineStr"/>
+      <c r="S406" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="2" t="inlineStr">
+        <is>
+          <t>Eva Guerrero Alvarez</t>
+        </is>
+      </c>
+      <c r="B407" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C407" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Green Refractor 1/75 Eva Guerrero Alvarez #126 Rookie RC 0z5</t>
+        </is>
+      </c>
+      <c r="D407" s="2" t="inlineStr">
+        <is>
+          <t>1/75</t>
+        </is>
+      </c>
+      <c r="E407" s="2" t="inlineStr">
+        <is>
+          <t>001 of 75</t>
+        </is>
+      </c>
+      <c r="F407" s="2" t="inlineStr">
+        <is>
+          <t>6.28 USD</t>
+        </is>
+      </c>
+      <c r="G407" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336814026049</t>
+        </is>
+      </c>
+      <c r="H407" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I407" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/tFkAAeSwIZxqt9S9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J407" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T14:19:40.000Z</t>
+        </is>
+      </c>
+      <c r="K407" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L407" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M407" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N407" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-g4AAeSwrWJqt9S9/s-l1600.jpg | https://i.ebayimg.com/images/g/skUAAeSw6z9qt9S9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O407" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P407" s="2" t="inlineStr"/>
+      <c r="Q407" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R407" s="2" t="inlineStr"/>
+      <c r="S407" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="2" t="inlineStr">
+        <is>
+          <t>Patrick Kypson</t>
+        </is>
+      </c>
+      <c r="B408" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Superior Relic Signatures - Gold</t>
+        </is>
+      </c>
+      <c r="C408" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Gold 10/10 Patrick Kypson #SRS-PK Rookie Auto RC 9et</t>
+        </is>
+      </c>
+      <c r="D408" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E408" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F408" s="2" t="inlineStr">
+        <is>
+          <t>64.08 USD</t>
+        </is>
+      </c>
+      <c r="G408" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257768820932</t>
+        </is>
+      </c>
+      <c r="H408" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I408" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TYEAAeSwj5pquQ-~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J408" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T12:43:45.000Z</t>
+        </is>
+      </c>
+      <c r="K408" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L408" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M408" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N408" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uLsAAeSwFEdquQ-~/s-l1600.jpg | https://i.ebayimg.com/images/g/E~QAAeSw~7tquQ-~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O408" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P408" s="2" t="inlineStr"/>
+      <c r="Q408" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R408" s="2" t="inlineStr"/>
+      <c r="S408" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="2" t="inlineStr">
+        <is>
+          <t>Casper Ruud</t>
+        </is>
+      </c>
+      <c r="B409" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS ROYALTY TENNIS REGALIA RELIC SIGNATURES</t>
+        </is>
+      </c>
+      <c r="C409" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS ROYALTY TENNIS REGALIA RELIC SIG BLUE CASPER RUUD 25/25 PSA 8 AUTO</t>
+        </is>
+      </c>
+      <c r="D409" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E409" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F409" s="2" t="inlineStr">
+        <is>
+          <t>2.25 USD</t>
+        </is>
+      </c>
+      <c r="G409" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117431493175</t>
+        </is>
+      </c>
+      <c r="H409" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I409" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/amwAAeSw40FqtuqN/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J409" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T01:53:00.000Z</t>
+        </is>
+      </c>
+      <c r="K409" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L409" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M409" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 8</t>
+        </is>
+      </c>
+      <c r="N409" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YOYAAeSwbyVqtuqN/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O409" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P409" s="2" t="inlineStr"/>
+      <c r="Q409" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R409" s="2" t="inlineStr"/>
+      <c r="S409" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek</t>
+        </is>
+      </c>
+      <c r="B410" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C410" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek 2024 Topps Royalty Superior Relic Signatures Green 5/5 PSA 10 [2hk</t>
+        </is>
+      </c>
+      <c r="D410" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E410" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F410" s="2" t="inlineStr">
+        <is>
+          <t>338.00 USD</t>
+        </is>
+      </c>
+      <c r="G410" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377525582109</t>
+        </is>
+      </c>
+      <c r="H410" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I410" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uS4AAeSw0PxquHMG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J410" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T01:35:04.000Z</t>
+        </is>
+      </c>
+      <c r="K410" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L410" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M410" s="2" t="inlineStr">
+        <is>
+          <t>PSA 10</t>
+        </is>
+      </c>
+      <c r="N410" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/FC0AAeSwVBZquHMI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O410" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P410" s="2" t="inlineStr"/>
+      <c r="Q410" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R410" s="2" t="inlineStr"/>
+      <c r="S410" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="2" t="inlineStr">
+        <is>
+          <t>Alejandro Davidovich Fokina</t>
+        </is>
+      </c>
+      <c r="B411" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - [Base] - Green</t>
+        </is>
+      </c>
+      <c r="C411" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Green 5/5 Alejandro Davidovich Fokina #63 9et</t>
+        </is>
+      </c>
+      <c r="D411" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E411" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F411" s="2" t="inlineStr">
+        <is>
+          <t>87.08 USD</t>
+        </is>
+      </c>
+      <c r="G411" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237092501601</t>
+        </is>
+      </c>
+      <c r="H411" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I411" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/h08AAeSwabxquEKZ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J411" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T22:08:25.000Z</t>
+        </is>
+      </c>
+      <c r="K411" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L411" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M411" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N411" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/EBMAAeSw3XxquEKZ/s-l1600.jpg | https://i.ebayimg.com/images/g/T1YAAeSweTFquEKZ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O411" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P411" s="2" t="inlineStr"/>
+      <c r="Q411" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R411" s="2" t="inlineStr"/>
+      <c r="S411" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="2" t="inlineStr">
+        <is>
+          <t>Zizou Bergs</t>
+        </is>
+      </c>
+      <c r="B412" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Regalia Relics - Blue</t>
+        </is>
+      </c>
+      <c r="C412" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Regalia Relics Blue 25/25 Zizou Bergs #RER-ZB Rookie RC 13ql</t>
+        </is>
+      </c>
+      <c r="D412" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E412" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F412" s="2" t="inlineStr">
+        <is>
+          <t>38.49 USD</t>
+        </is>
+      </c>
+      <c r="G412" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336814194529</t>
+        </is>
+      </c>
+      <c r="H412" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I412" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ZxcAAeSwyBBqt~ku/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J412" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T16:55:11.000Z</t>
+        </is>
+      </c>
+      <c r="K412" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L412" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M412" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N412" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/VwQAAeSwffpqt~ku/s-l1600.jpg | https://i.ebayimg.com/images/g/V~0AAeSwhcFqt~ku/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O412" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P412" s="2" t="inlineStr"/>
+      <c r="Q412" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R412" s="2" t="inlineStr"/>
+      <c r="S412" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="2" t="inlineStr">
+        <is>
+          <t>Veronika Kudermetova</t>
+        </is>
+      </c>
+      <c r="B413" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Star Relics - Blue</t>
+        </is>
+      </c>
+      <c r="C413" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Star Relics Blue 1/25 Veronika Kudermetova Rookie RC 6ns</t>
+        </is>
+      </c>
+      <c r="D413" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E413" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F413" s="2" t="inlineStr">
+        <is>
+          <t>29.58 USD</t>
+        </is>
+      </c>
+      <c r="G413" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257767169889</t>
+        </is>
+      </c>
+      <c r="H413" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I413" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/th8AAeSw~VFqt-p3/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J413" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T15:52:24.000Z</t>
+        </is>
+      </c>
+      <c r="K413" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L413" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M413" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N413" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/zOIAAeSw1xZqt-p3/s-l1600.jpg | https://i.ebayimg.com/images/g/ID8AAeSwqNZqt-p3/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O413" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P413" s="2" t="inlineStr"/>
+      <c r="Q413" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R413" s="2" t="inlineStr"/>
+      <c r="S413" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="2" t="inlineStr">
+        <is>
+          <t>Casper Ruud</t>
+        </is>
+      </c>
+      <c r="B414" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Regalia Relic Signatures</t>
+        </is>
+      </c>
+      <c r="C414" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Regalia Relic Signatures 1/75 Casper Ruud Rookie Auto RC 1fl4</t>
+        </is>
+      </c>
+      <c r="D414" s="2" t="inlineStr">
+        <is>
+          <t>1/75</t>
+        </is>
+      </c>
+      <c r="E414" s="2" t="inlineStr">
+        <is>
+          <t>001 of 75</t>
+        </is>
+      </c>
+      <c r="F414" s="2" t="inlineStr">
+        <is>
+          <t>86.73 USD</t>
+        </is>
+      </c>
+      <c r="G414" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257767161909</t>
+        </is>
+      </c>
+      <c r="H414" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I414" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nSkAAeSwVJRqt-ek/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J414" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T15:40:16.000Z</t>
+        </is>
+      </c>
+      <c r="K414" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L414" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M414" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N414" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0qAAAeSwouBqt-ek/s-l1600.jpg | https://i.ebayimg.com/images/g/0TEAAeSweTFqt-ek/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O414" s="2" t="inlineStr"/>
+      <c r="P414" s="2" t="inlineStr"/>
+      <c r="Q414" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R414" s="2" t="inlineStr"/>
+      <c r="S414" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="2" t="inlineStr">
+        <is>
+          <t>Liudmila Samsonova</t>
+        </is>
+      </c>
+      <c r="B415" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Prodigious Pairings - Gold</t>
+        </is>
+      </c>
+      <c r="C415" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Gold 10/10 Liudmila Samsonova Anna Kalinskaya Rookie RC 9et</t>
+        </is>
+      </c>
+      <c r="D415" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E415" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F415" s="2" t="inlineStr">
+        <is>
+          <t>69.83 USD</t>
+        </is>
+      </c>
+      <c r="G415" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336814042494</t>
+        </is>
+      </c>
+      <c r="H415" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I415" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/l3UAAeSwTD9qt9hn/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J415" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T14:35:18.000Z</t>
+        </is>
+      </c>
+      <c r="K415" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L415" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M415" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N415" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vvQAAeSwGGtqt9ho/s-l1600.jpg | https://i.ebayimg.com/images/g/nlsAAeSwpAVqt9hn/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O415" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P415" s="2" t="inlineStr"/>
+      <c r="Q415" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R415" s="2" t="inlineStr"/>
+      <c r="S415" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="2" t="inlineStr">
+        <is>
+          <t>Chris Eubanks</t>
+        </is>
+      </c>
+      <c r="B416" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Superior Signatures - Blue</t>
+        </is>
+      </c>
+      <c r="C416" s="2" t="inlineStr">
+        <is>
+          <t>2024 Royalty Superior Signatures Blue 25/25 Chris Eubanks Rookie Auto RC 9et</t>
+        </is>
+      </c>
+      <c r="D416" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E416" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F416" s="2" t="inlineStr">
+        <is>
+          <t>52.58 USD</t>
+        </is>
+      </c>
+      <c r="G416" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237092002465</t>
+        </is>
+      </c>
+      <c r="H416" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I416" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Xc4AAeSwlYNqt9bf/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J416" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T14:28:47.000Z</t>
+        </is>
+      </c>
+      <c r="K416" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L416" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M416" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N416" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YscAAeSwRHlqt9bf/s-l1600.jpg | https://i.ebayimg.com/images/g/W4cAAeSwKRxqt9bf/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O416" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P416" s="2" t="inlineStr"/>
+      <c r="Q416" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R416" s="2" t="inlineStr"/>
+      <c r="S416" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="2" t="inlineStr">
+        <is>
+          <t>Emiliana Arango</t>
+        </is>
+      </c>
+      <c r="B417" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Regalia Relic Signatures - Gold</t>
+        </is>
+      </c>
+      <c r="C417" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Gold 1/10 Emiliana Arango #RRS-EAO Rookie Auto RC 9et</t>
+        </is>
+      </c>
+      <c r="D417" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E417" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F417" s="2" t="inlineStr">
+        <is>
+          <t>87.08 USD</t>
+        </is>
+      </c>
+      <c r="G417" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237092000377</t>
+        </is>
+      </c>
+      <c r="H417" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I417" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DlsAAeSwIftqt9Z5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J417" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T14:27:04.000Z</t>
+        </is>
+      </c>
+      <c r="K417" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L417" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M417" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N417" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/qWYAAeSwbyVqt9Z5/s-l1600.jpg | https://i.ebayimg.com/images/g/lHkAAeSwh-dqt9Z5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O417" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P417" s="2" t="inlineStr"/>
+      <c r="Q417" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R417" s="2" t="inlineStr"/>
+      <c r="S417" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="2" t="inlineStr">
+        <is>
+          <t>Ethan Quinn</t>
+        </is>
+      </c>
+      <c r="B418" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Rookie Relic Autographs - Blue</t>
+        </is>
+      </c>
+      <c r="C418" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Rookie Relic Blue 1/25 Ethan Quinn #RRA-EQ Auto RC 9et</t>
+        </is>
+      </c>
+      <c r="D418" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E418" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F418" s="2" t="inlineStr">
+        <is>
+          <t>69.83 USD</t>
+        </is>
+      </c>
+      <c r="G418" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237091962886</t>
+        </is>
+      </c>
+      <c r="H418" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:47 UTC</t>
+        </is>
+      </c>
+      <c r="I418" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/L5EAAeSwxSZqt9Ax/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J418" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T14:00:13.000Z</t>
+        </is>
+      </c>
+      <c r="K418" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L418" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M418" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N418" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/OiMAAeSwi8tqt9Ax/s-l1600.jpg | https://i.ebayimg.com/images/g/ke8AAeSwSHNqt9Ax/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O418" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P418" s="2" t="inlineStr"/>
+      <c r="Q418" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R418" s="2" t="inlineStr"/>
+      <c r="S418" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -35151,6 +37267,30 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G392" r:id="rId391"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G393" r:id="rId392"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G394" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G395" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G396" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G397" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G398" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G399" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G400" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G401" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G402" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G403" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G404" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G405" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G406" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G407" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G408" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G409" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G410" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G411" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G412" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G413" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G414" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G415" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G416" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G417" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G418" r:id="rId417"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-28 02:26 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S418"/>
+  <dimension ref="A1:S427"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -36867,6 +36867,795 @@
       </c>
       <c r="R418" s="2" t="inlineStr"/>
       <c r="S418" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="2" t="inlineStr">
+        <is>
+          <t>Alexandra Eala</t>
+        </is>
+      </c>
+      <c r="B419" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C419" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Sapphire Edition #171 Alexandra Eala PADPARADSCHA 1/1</t>
+        </is>
+      </c>
+      <c r="D419" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E419" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F419" s="2" t="inlineStr">
+        <is>
+          <t>47000.00 USD</t>
+        </is>
+      </c>
+      <c r="G419" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298712839443</t>
+        </is>
+      </c>
+      <c r="H419" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 02:25 UTC</t>
+        </is>
+      </c>
+      <c r="I419" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SNIAAeSw6OVquc16/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J419" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T02:15:40.000Z</t>
+        </is>
+      </c>
+      <c r="K419" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L419" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M419" s="2" t="inlineStr">
+        <is>
+          <t>Beckett Grading Services (BGS) 8.5</t>
+        </is>
+      </c>
+      <c r="N419" s="2" t="inlineStr"/>
+      <c r="O419" s="2" t="inlineStr"/>
+      <c r="P419" s="2" t="inlineStr"/>
+      <c r="Q419" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R419" s="2" t="inlineStr"/>
+      <c r="S419" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="2" t="inlineStr">
+        <is>
+          <t>Alexandra Eala</t>
+        </is>
+      </c>
+      <c r="B420" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 TOPPS CHROME TENNIS CHROME AUTOGRAPHS</t>
+        </is>
+      </c>
+      <c r="C420" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS CHROME AUTO RED GEOMETRIC ALEXANDRA EALA 5/5 PSA 9</t>
+        </is>
+      </c>
+      <c r="D420" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E420" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F420" s="2" t="inlineStr">
+        <is>
+          <t>1.25 USD</t>
+        </is>
+      </c>
+      <c r="G420" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307196584302</t>
+        </is>
+      </c>
+      <c r="H420" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 02:25 UTC</t>
+        </is>
+      </c>
+      <c r="I420" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/hfAAAeSwbz5qtTOt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J420" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T01:28:00.000Z</t>
+        </is>
+      </c>
+      <c r="K420" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L420" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M420" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N420" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vuwAAeSw6z1qtTOt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O420" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P420" s="2" t="inlineStr"/>
+      <c r="Q420" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R420" s="2" t="inlineStr"/>
+      <c r="S420" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="2" t="inlineStr">
+        <is>
+          <t>Emilio Nava</t>
+        </is>
+      </c>
+      <c r="B421" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C421" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Emilio Nava #227 Black Refractor 1/10 B1</t>
+        </is>
+      </c>
+      <c r="D421" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E421" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F421" s="2" t="inlineStr">
+        <is>
+          <t>1.99 USD</t>
+        </is>
+      </c>
+      <c r="G421" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178526361879</t>
+        </is>
+      </c>
+      <c r="H421" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 02:25 UTC</t>
+        </is>
+      </c>
+      <c r="I421" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KkQAAeSwBXRp5pts/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J421" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T00:16:00.000Z</t>
+        </is>
+      </c>
+      <c r="K421" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L421" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M421" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N421" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/PcQAAeSw0lVp5ptv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O421" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P421" s="2" t="inlineStr"/>
+      <c r="Q421" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R421" s="2" t="inlineStr"/>
+      <c r="S421" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="2" t="inlineStr">
+        <is>
+          <t>Mirjam Bjorklund</t>
+        </is>
+      </c>
+      <c r="B422" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C422" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome I Black Refractor 10/10 Mirjam Bjorklund Rookie Auto RC 0r9h</t>
+        </is>
+      </c>
+      <c r="D422" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E422" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F422" s="2" t="inlineStr">
+        <is>
+          <t>41.07 USD</t>
+        </is>
+      </c>
+      <c r="G422" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336815973717</t>
+        </is>
+      </c>
+      <c r="H422" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 02:25 UTC</t>
+        </is>
+      </c>
+      <c r="I422" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ocYAAeSw-zpquYT1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J422" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T21:03:45.000Z</t>
+        </is>
+      </c>
+      <c r="K422" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L422" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M422" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N422" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uXYAAeSwaTFquYT1/s-l1600.jpg | https://i.ebayimg.com/images/g/x2MAAeSwVUdquYT1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O422" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P422" s="2" t="inlineStr"/>
+      <c r="Q422" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R422" s="2" t="inlineStr"/>
+      <c r="S422" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="2" t="inlineStr">
+        <is>
+          <t>Steffi Graf</t>
+        </is>
+      </c>
+      <c r="B423" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C423" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite - Steffi Graf #104 Blue Refractor 50/50</t>
+        </is>
+      </c>
+      <c r="D423" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E423" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F423" s="2" t="inlineStr">
+        <is>
+          <t>1.50 USD</t>
+        </is>
+      </c>
+      <c r="G423" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287613040104</t>
+        </is>
+      </c>
+      <c r="H423" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 02:26 UTC</t>
+        </is>
+      </c>
+      <c r="I423" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/dCAAAeSwGRBqubLA/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J423" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T00:21:04.000Z</t>
+        </is>
+      </c>
+      <c r="K423" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L423" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M423" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N423" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/P~MAAeSw3CxqubLO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O423" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P423" s="2" t="inlineStr"/>
+      <c r="Q423" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R423" s="2" t="inlineStr"/>
+      <c r="S423" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="2" t="inlineStr">
+        <is>
+          <t>Daniel Rincon</t>
+        </is>
+      </c>
+      <c r="B424" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C424" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Relics Green Refractor 75/75 Daniel Rincon Rookie RC 03xg</t>
+        </is>
+      </c>
+      <c r="D424" s="2" t="inlineStr">
+        <is>
+          <t>75/75</t>
+        </is>
+      </c>
+      <c r="E424" s="2" t="inlineStr">
+        <is>
+          <t>last of 75 (75/75)</t>
+        </is>
+      </c>
+      <c r="F424" s="2" t="inlineStr">
+        <is>
+          <t>3.12 USD</t>
+        </is>
+      </c>
+      <c r="G424" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237094026187</t>
+        </is>
+      </c>
+      <c r="H424" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 02:26 UTC</t>
+        </is>
+      </c>
+      <c r="I424" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DjUAAeSwnNlquZSP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J424" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T22:10:22.000Z</t>
+        </is>
+      </c>
+      <c r="K424" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L424" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M424" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N424" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/W6YAAeSw3XxquZSP/s-l1600.jpg | https://i.ebayimg.com/images/g/N4sAAeSwbZtquZSP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O424" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P424" s="2" t="inlineStr"/>
+      <c r="Q424" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R424" s="2" t="inlineStr"/>
+      <c r="S424" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="2" t="inlineStr">
+        <is>
+          <t>Donna Vekic</t>
+        </is>
+      </c>
+      <c r="B425" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C425" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Gold Refractor 1/25 Donna Vekic #166 Rookie RC ld5</t>
+        </is>
+      </c>
+      <c r="D425" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E425" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F425" s="2" t="inlineStr">
+        <is>
+          <t>12.32 USD</t>
+        </is>
+      </c>
+      <c r="G425" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257769499247</t>
+        </is>
+      </c>
+      <c r="H425" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 02:26 UTC</t>
+        </is>
+      </c>
+      <c r="I425" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/n1wAAeSwQLZquXBj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J425" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T19:35:59.000Z</t>
+        </is>
+      </c>
+      <c r="K425" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L425" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M425" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N425" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9MUAAeSwXS1quXBj/s-l1600.jpg | https://i.ebayimg.com/images/g/Y-YAAeSwT59quXBj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O425" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P425" s="2" t="inlineStr"/>
+      <c r="Q425" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R425" s="2" t="inlineStr"/>
+      <c r="S425" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="2" t="inlineStr">
+        <is>
+          <t>Ulises Blanch</t>
+        </is>
+      </c>
+      <c r="B426" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Collection Tennis</t>
+        </is>
+      </c>
+      <c r="C426" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Collection Tennis Ulises Blanch TRS-UB Auto Relic 01/10</t>
+        </is>
+      </c>
+      <c r="D426" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E426" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F426" s="2" t="inlineStr">
+        <is>
+          <t>50.00 USD</t>
+        </is>
+      </c>
+      <c r="G426" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168731513984</t>
+        </is>
+      </c>
+      <c r="H426" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 02:26 UTC</t>
+        </is>
+      </c>
+      <c r="I426" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SWQAAeSwU6ZqucgX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J426" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T01:54:46.000Z</t>
+        </is>
+      </c>
+      <c r="K426" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L426" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M426" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N426" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TWAAAeSwVCdqucgn/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O426" s="2" t="inlineStr"/>
+      <c r="P426" s="2" t="inlineStr"/>
+      <c r="Q426" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R426" s="2" t="inlineStr"/>
+      <c r="S426" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="2" t="inlineStr">
+        <is>
+          <t>Jan-Lennard Struff</t>
+        </is>
+      </c>
+      <c r="B427" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - [Base] - Green</t>
+        </is>
+      </c>
+      <c r="C427" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Green 1/5 Jan-Lennard Struff #62 0r9h</t>
+        </is>
+      </c>
+      <c r="D427" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E427" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F427" s="2" t="inlineStr">
+        <is>
+          <t>41.08 USD</t>
+        </is>
+      </c>
+      <c r="G427" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237093783618</t>
+        </is>
+      </c>
+      <c r="H427" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 02:26 UTC</t>
+        </is>
+      </c>
+      <c r="I427" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nXAAAeSwj5ZquV0~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J427" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27T18:14:20.000Z</t>
+        </is>
+      </c>
+      <c r="K427" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L427" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M427" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N427" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JygAAeSw3MtquV0-/s-l1600.jpg | https://i.ebayimg.com/images/g/SGIAAeSwiMJquV0~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O427" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P427" s="2" t="inlineStr"/>
+      <c r="Q427" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R427" s="2" t="inlineStr"/>
+      <c r="S427" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -37291,6 +38080,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G416" r:id="rId415"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G417" r:id="rId416"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G418" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G419" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G420" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G421" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G422" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G423" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G424" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G425" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G426" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G427" r:id="rId426"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-28 05:44 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S427"/>
+  <dimension ref="A1:S430"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37656,6 +37656,269 @@
       </c>
       <c r="R427" s="2" t="inlineStr"/>
       <c r="S427" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="2" t="inlineStr">
+        <is>
+          <t>Christina Mchale</t>
+        </is>
+      </c>
+      <c r="B428" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C428" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Mini-Diamond Refractor 1/125 Christina McHale Rookie RC nd3</t>
+        </is>
+      </c>
+      <c r="D428" s="2" t="inlineStr">
+        <is>
+          <t>1/125</t>
+        </is>
+      </c>
+      <c r="E428" s="2" t="inlineStr">
+        <is>
+          <t>001 of 125</t>
+        </is>
+      </c>
+      <c r="F428" s="2" t="inlineStr">
+        <is>
+          <t>5.43 USD</t>
+        </is>
+      </c>
+      <c r="G428" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257770343364</t>
+        </is>
+      </c>
+      <c r="H428" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 05:44 UTC</t>
+        </is>
+      </c>
+      <c r="I428" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2ucAAeSwpAVqufIO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J428" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T04:49:17.000Z</t>
+        </is>
+      </c>
+      <c r="K428" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L428" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M428" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N428" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/yhAAAeSwzetqufIN/s-l1600.jpg | https://i.ebayimg.com/images/g/E2QAAeSwuWBqufIO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O428" s="2" t="inlineStr"/>
+      <c r="P428" s="2" t="inlineStr"/>
+      <c r="Q428" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R428" s="2" t="inlineStr"/>
+      <c r="S428" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="2" t="inlineStr">
+        <is>
+          <t>Dusan Lajovic</t>
+        </is>
+      </c>
+      <c r="B429" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C429" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Dusan Lajovic Red Geometric Refractor #99 5/5 BY88</t>
+        </is>
+      </c>
+      <c r="D429" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E429" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F429" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G429" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407250904055</t>
+        </is>
+      </c>
+      <c r="H429" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 05:44 UTC</t>
+        </is>
+      </c>
+      <c r="I429" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vWsAAeSwq7tqudTF/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J429" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T02:44:17.000Z</t>
+        </is>
+      </c>
+      <c r="K429" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L429" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M429" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N429" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/wK4AAeSwCjBqudTF/s-l1600.jpg | https://i.ebayimg.com/images/g/s3kAAeSws~pqudTE/s-l1600.jpg | https://i.ebayimg.com/images/g/0RMAAeSwsEpqudTE/s-l1600.jpg | https://i.ebayimg.com/images/g/yfkAAeSwGTlqudTE/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O429" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P429" s="2" t="inlineStr"/>
+      <c r="Q429" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R429" s="2" t="inlineStr"/>
+      <c r="S429" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="2" t="inlineStr">
+        <is>
+          <t>Patrick Kypson</t>
+        </is>
+      </c>
+      <c r="B430" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C430" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Patrick Kypson Auto Purple Refraction 10/10 #CA-PKN BY88</t>
+        </is>
+      </c>
+      <c r="D430" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E430" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F430" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G430" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407250901003</t>
+        </is>
+      </c>
+      <c r="H430" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 05:44 UTC</t>
+        </is>
+      </c>
+      <c r="I430" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bXcAAeSwdOhqudSH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J430" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T02:43:18.000Z</t>
+        </is>
+      </c>
+      <c r="K430" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L430" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M430" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N430" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/kBkAAeSwzd1qudSH/s-l1600.jpg | https://i.ebayimg.com/images/g/idUAAeSw3CxqudSG/s-l1600.jpg | https://i.ebayimg.com/images/g/TZUAAeSwEcNqudSG/s-l1600.jpg | https://i.ebayimg.com/images/g/o0oAAeSw2YBqudSG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O430" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P430" s="2" t="inlineStr"/>
+      <c r="Q430" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R430" s="2" t="inlineStr"/>
+      <c r="S430" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -38089,6 +38352,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G425" r:id="rId424"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G426" r:id="rId425"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G427" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G428" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G429" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G430" r:id="rId429"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-28 17:46 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S430"/>
+  <dimension ref="A1:S441"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37919,6 +37919,977 @@
       </c>
       <c r="R430" s="2" t="inlineStr"/>
       <c r="S430" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="2" t="inlineStr">
+        <is>
+          <t>Liudmila Samsonova</t>
+        </is>
+      </c>
+      <c r="B431" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C431" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis 128 Liudmila Samsonova 1st Lime Green Refractor 001/299</t>
+        </is>
+      </c>
+      <c r="D431" s="2" t="inlineStr">
+        <is>
+          <t>1/299</t>
+        </is>
+      </c>
+      <c r="E431" s="2" t="inlineStr">
+        <is>
+          <t>001 of 299</t>
+        </is>
+      </c>
+      <c r="F431" s="2" t="inlineStr">
+        <is>
+          <t>4.99 USD</t>
+        </is>
+      </c>
+      <c r="G431" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307203630876?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8iQwzP8jCfH1k6e--pvIBFBYpxIYySXAikU1l7Yv1o5zrym9b4jYqIVVVyruDHENPoT7XMiUTLExBpJ3wOYWFhaQ0%2B6B%2FKrl%2Bg6jlPId9uApf%2FCE5W69K8AZ%2B01SVGg1cUPtYOE2NMeUGIWrykkOoHUrvD6aVbmc4SXsDZ7Zg4d1PzJ3Et34Osl6Mm5DSIOXw%3D</t>
+        </is>
+      </c>
+      <c r="H431" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:45 UTC</t>
+        </is>
+      </c>
+      <c r="I431" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HUUAAeSwpvhqunG2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J431" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T13:55:40.000Z</t>
+        </is>
+      </c>
+      <c r="K431" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L431" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M431" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N431" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SR8AAeSw-UZqunG2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O431" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P431" s="2" t="inlineStr"/>
+      <c r="Q431" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R431" s="2" t="inlineStr"/>
+      <c r="S431" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="2" t="inlineStr">
+        <is>
+          <t>Emiliana Arango</t>
+        </is>
+      </c>
+      <c r="B432" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS CHROME TENNIS AUTOGRAPHS</t>
+        </is>
+      </c>
+      <c r="C432" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS CHROME TENNIS AUTOS RED REFRACTOR #TCAEAO EMILIANA ARANGO 5/5 PSA 9</t>
+        </is>
+      </c>
+      <c r="D432" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E432" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F432" s="2" t="inlineStr">
+        <is>
+          <t>245.00 USD</t>
+        </is>
+      </c>
+      <c r="G432" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307203571733</t>
+        </is>
+      </c>
+      <c r="H432" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:46 UTC</t>
+        </is>
+      </c>
+      <c r="I432" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ALYAAeSwp~tqumWv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J432" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T13:02:33.000Z</t>
+        </is>
+      </c>
+      <c r="K432" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L432" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M432" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N432" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/rCAAAeSwekZqumWu/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O432" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P432" s="2" t="inlineStr"/>
+      <c r="Q432" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R432" s="2" t="inlineStr"/>
+      <c r="S432" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="2" t="inlineStr">
+        <is>
+          <t>Christopher O'Connell</t>
+        </is>
+      </c>
+      <c r="B433" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - [Base] - Gold Refractor</t>
+        </is>
+      </c>
+      <c r="C433" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Gold Refractor 1/50 Christopher O'Connell #96 6q5</t>
+        </is>
+      </c>
+      <c r="D433" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E433" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F433" s="2" t="inlineStr">
+        <is>
+          <t>10.02 USD</t>
+        </is>
+      </c>
+      <c r="G433" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257771059832</t>
+        </is>
+      </c>
+      <c r="H433" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:46 UTC</t>
+        </is>
+      </c>
+      <c r="I433" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/VCQAAeSw7sxqumKy/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J433" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T12:49:53.000Z</t>
+        </is>
+      </c>
+      <c r="K433" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L433" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M433" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N433" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/VRMAAeSwdFdqumKx/s-l1600.jpg | https://i.ebayimg.com/images/g/WxgAAeSwZztqumKy/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O433" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P433" s="2" t="inlineStr"/>
+      <c r="Q433" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R433" s="2" t="inlineStr"/>
+      <c r="S433" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Bublik</t>
+        </is>
+      </c>
+      <c r="B434" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C434" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Bublik 🇰🇿 #001/150 Blue Refractor -- 2025 Topps Chrome 🎾 #49</t>
+        </is>
+      </c>
+      <c r="D434" s="2" t="inlineStr">
+        <is>
+          <t>1/150</t>
+        </is>
+      </c>
+      <c r="E434" s="2" t="inlineStr">
+        <is>
+          <t>001 of 150</t>
+        </is>
+      </c>
+      <c r="F434" s="2" t="inlineStr">
+        <is>
+          <t>4.95 USD</t>
+        </is>
+      </c>
+      <c r="G434" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178536125618?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8chJUP3u6FO%2Bs%2FDvvkWAhVpgmrwBxIP%2B6ZKg3qhONGfVXgQl%2F97Pe9Df9fU18qcjtmnz6rIxV1iughy3827NUKOUYrNWNj5FjudIHbNe3j3PqfQi%2BZNbTEhN0uUAKi%2FuuPdFyeDJUuT9w6CqaPP3A1aRiK9xSl4yBkRBOqxxxPvNtatTDRr%2FeCp3p5hQ6dv3o%3D</t>
+        </is>
+      </c>
+      <c r="H434" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:46 UTC</t>
+        </is>
+      </c>
+      <c r="I434" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/WtMAAeSww8Fqul-x/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J434" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T12:38:24.000Z</t>
+        </is>
+      </c>
+      <c r="K434" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L434" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M434" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N434" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/UccAAeSwNG5qul-x/s-l1600.jpg | https://i.ebayimg.com/images/g/J10AAeSw2-Zqul-x/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O434" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P434" s="2" t="inlineStr"/>
+      <c r="Q434" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R434" s="2" t="inlineStr"/>
+      <c r="S434" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="2" t="inlineStr">
+        <is>
+          <t>Mikael Ymer</t>
+        </is>
+      </c>
+      <c r="B435" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C435" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis Mikael Ymer GOLD REFRACTOR 50/50 BOOKEND #129</t>
+        </is>
+      </c>
+      <c r="D435" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E435" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F435" s="2" t="inlineStr">
+        <is>
+          <t>44.99 USD</t>
+        </is>
+      </c>
+      <c r="G435" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/820182114412</t>
+        </is>
+      </c>
+      <c r="H435" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:46 UTC</t>
+        </is>
+      </c>
+      <c r="I435" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JqwAAeSw~Dtqulwl/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J435" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T12:27:24.000Z</t>
+        </is>
+      </c>
+      <c r="K435" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L435" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M435" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N435" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HsEAAeSwusxqulwm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O435" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P435" s="2" t="inlineStr"/>
+      <c r="Q435" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R435" s="2" t="inlineStr"/>
+      <c r="S435" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="2" t="inlineStr">
+        <is>
+          <t>Leandro Riedi</t>
+        </is>
+      </c>
+      <c r="B436" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C436" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Orange Refractor 1/25 Leandro Riedi #199 pe8</t>
+        </is>
+      </c>
+      <c r="D436" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E436" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F436" s="2" t="inlineStr">
+        <is>
+          <t>18.08 USD</t>
+        </is>
+      </c>
+      <c r="G436" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237094927203</t>
+        </is>
+      </c>
+      <c r="H436" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:46 UTC</t>
+        </is>
+      </c>
+      <c r="I436" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/qMUAAeSwsGZqukMO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J436" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T10:34:43.000Z</t>
+        </is>
+      </c>
+      <c r="K436" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L436" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M436" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N436" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/lfgAAeSwl~pqukMO/s-l1600.jpg | https://i.ebayimg.com/images/g/hk0AAeSwVJRqukMO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O436" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P436" s="2" t="inlineStr"/>
+      <c r="Q436" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R436" s="2" t="inlineStr"/>
+      <c r="S436" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="2" t="inlineStr">
+        <is>
+          <t>Emma Raducanu</t>
+        </is>
+      </c>
+      <c r="B437" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C437" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2026 Graphite Emma Raducanu #68 Serial Numbered 01/25 WTA Tennis</t>
+        </is>
+      </c>
+      <c r="D437" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E437" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F437" s="2" t="inlineStr">
+        <is>
+          <t>50.00 USD</t>
+        </is>
+      </c>
+      <c r="G437" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/318930101746</t>
+        </is>
+      </c>
+      <c r="H437" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:46 UTC</t>
+        </is>
+      </c>
+      <c r="I437" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TNQAAeSwcTxqup5N/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J437" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T17:06:59.000Z</t>
+        </is>
+      </c>
+      <c r="K437" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L437" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M437" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N437" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/g8EAAeSwFr5qup5J/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O437" s="2" t="inlineStr"/>
+      <c r="P437" s="2" t="inlineStr"/>
+      <c r="Q437" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R437" s="2" t="inlineStr"/>
+      <c r="S437" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="2" t="inlineStr">
+        <is>
+          <t>Ivan Lendl</t>
+        </is>
+      </c>
+      <c r="B438" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps</t>
+        </is>
+      </c>
+      <c r="C438" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Tennis Ivan Lendl Grand Slam Signatures Blue Auto 50/50</t>
+        </is>
+      </c>
+      <c r="D438" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E438" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F438" s="2" t="inlineStr">
+        <is>
+          <t>99.99 USD</t>
+        </is>
+      </c>
+      <c r="G438" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/206588316197</t>
+        </is>
+      </c>
+      <c r="H438" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:46 UTC</t>
+        </is>
+      </c>
+      <c r="I438" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/1WYAAeSwEb1qte6D/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J438" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T16:44:44.000Z</t>
+        </is>
+      </c>
+      <c r="K438" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L438" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M438" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N438" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/4UUAAeSw2EJqte5R/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O438" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P438" s="2" t="inlineStr"/>
+      <c r="Q438" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R438" s="2" t="inlineStr"/>
+      <c r="S438" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="2" t="inlineStr">
+        <is>
+          <t>Maria Sakkari</t>
+        </is>
+      </c>
+      <c r="B439" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite - [Base] - Red Crystalline Refractor</t>
+        </is>
+      </c>
+      <c r="C439" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Red Crystalline Refractor 1/1 Maria Sakkari #123 0i4v</t>
+        </is>
+      </c>
+      <c r="D439" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E439" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F439" s="2" t="inlineStr">
+        <is>
+          <t>271.25 USD</t>
+        </is>
+      </c>
+      <c r="G439" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336816821512</t>
+        </is>
+      </c>
+      <c r="H439" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:46 UTC</t>
+        </is>
+      </c>
+      <c r="I439" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/kl8AAeSwVJRqujJi/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J439" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T09:23:30.000Z</t>
+        </is>
+      </c>
+      <c r="K439" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L439" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M439" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N439" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/mokAAeSwSb1qujJi/s-l1600.jpg | https://i.ebayimg.com/images/g/WFoAAeSw7epqujJi/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O439" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P439" s="2" t="inlineStr"/>
+      <c r="Q439" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R439" s="2" t="inlineStr"/>
+      <c r="S439" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="2" t="inlineStr">
+        <is>
+          <t>Ulises Blanch</t>
+        </is>
+      </c>
+      <c r="B440" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C440" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Green Refractor 1/75 Ulises Blanch Rookie Auto RC 07r3</t>
+        </is>
+      </c>
+      <c r="D440" s="2" t="inlineStr">
+        <is>
+          <t>1/75</t>
+        </is>
+      </c>
+      <c r="E440" s="2" t="inlineStr">
+        <is>
+          <t>001 of 75</t>
+        </is>
+      </c>
+      <c r="F440" s="2" t="inlineStr">
+        <is>
+          <t>7.73 USD</t>
+        </is>
+      </c>
+      <c r="G440" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237094769708</t>
+        </is>
+      </c>
+      <c r="H440" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:46 UTC</t>
+        </is>
+      </c>
+      <c r="I440" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/v44AAeSwpPxquimJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J440" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T08:46:03.000Z</t>
+        </is>
+      </c>
+      <c r="K440" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L440" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M440" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N440" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DOIAAeSwQutquimJ/s-l1600.jpg | https://i.ebayimg.com/images/g/A9kAAeSw8sxquimJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O440" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P440" s="2" t="inlineStr"/>
+      <c r="Q440" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R440" s="2" t="inlineStr"/>
+      <c r="S440" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="2" t="inlineStr">
+        <is>
+          <t>Elisabetta Cocciaretto</t>
+        </is>
+      </c>
+      <c r="B441" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C441" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis The Grip Relic Elisabetta Cocciaretto Platinum 1/1</t>
+        </is>
+      </c>
+      <c r="D441" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E441" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F441" s="2" t="inlineStr">
+        <is>
+          <t>500.00 USD</t>
+        </is>
+      </c>
+      <c r="G441" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/189005543981</t>
+        </is>
+      </c>
+      <c r="H441" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:46 UTC</t>
+        </is>
+      </c>
+      <c r="I441" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/INYAAeSwzFpquosO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J441" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T15:43:39.000Z</t>
+        </is>
+      </c>
+      <c r="K441" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L441" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M441" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N441" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/H8oAAeSww9VquosU/s-l1600.jpg | https://i.ebayimg.com/images/g/~mIAAeSwm3FquosZ/s-l1600.jpg | https://i.ebayimg.com/images/g/Jm0AAeSwBN5quose/s-l1600.jpg | https://i.ebayimg.com/images/g/~0kAAeSwl3Nquosj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O441" s="2" t="inlineStr"/>
+      <c r="P441" s="2" t="inlineStr"/>
+      <c r="Q441" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R441" s="2" t="inlineStr"/>
+      <c r="S441" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -38355,6 +39326,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G428" r:id="rId427"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G429" r:id="rId428"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G430" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G431" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G432" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G433" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G434" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G435" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G436" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G437" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G438" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G439" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G440" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G441" r:id="rId440"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-29 16:04 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S441"/>
+  <dimension ref="A1:S449"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38890,6 +38890,718 @@
       </c>
       <c r="R441" s="2" t="inlineStr"/>
       <c r="S441" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="2" t="inlineStr">
+        <is>
+          <t>Mackie McDonald</t>
+        </is>
+      </c>
+      <c r="B442" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Sapphire Edition - [Base] - Orange</t>
+        </is>
+      </c>
+      <c r="C442" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Sapphire Orange 25/25 Mackie McDonald Mackenzie #145 1g10</t>
+        </is>
+      </c>
+      <c r="D442" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E442" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F442" s="2" t="inlineStr">
+        <is>
+          <t>4.85 USD</t>
+        </is>
+      </c>
+      <c r="G442" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237096298596</t>
+        </is>
+      </c>
+      <c r="H442" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:03 UTC</t>
+        </is>
+      </c>
+      <c r="I442" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Xu8AAeSwmrNqu0Tm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J442" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29T04:56:02.000Z</t>
+        </is>
+      </c>
+      <c r="K442" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L442" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M442" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N442" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XxMAAeSwrX9qu0Tm/s-l1600.jpg | https://i.ebayimg.com/images/g/-SsAAeSwUMdqu0Tm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O442" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P442" s="2" t="inlineStr"/>
+      <c r="Q442" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R442" s="2" t="inlineStr"/>
+      <c r="S442" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="2" t="inlineStr">
+        <is>
+          <t>Petra Kvitova</t>
+        </is>
+      </c>
+      <c r="B443" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C443" s="2" t="inlineStr">
+        <is>
+          <t>2025 PETRA KVITOVA 25/25 AUTO TOPPS CHROME REFRACTOR AUTOGRAPHS (read)</t>
+        </is>
+      </c>
+      <c r="D443" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E443" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F443" s="2" t="inlineStr">
+        <is>
+          <t>36.99 USD</t>
+        </is>
+      </c>
+      <c r="G443" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/158359568444?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde9PFDl9m6aG%2FI0A9%2BTrTVHpOoSv9rV0FS37uEHzOa5R9sOKwV1cp1kurE1rMF1lPNi03KGYYJNDayDxlkCegipnbFGjsaWnMhpdZDQUeOgccM%2FJr5MGkf%2FRPgCNuwDDhzVLGD9t3a0Wlj6N5SrZjNwAfK8bt7UEOQIPszNkTdCIdYyYezxAZLXWBSQOt5lYBDI%3D</t>
+        </is>
+      </c>
+      <c r="H443" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:03 UTC</t>
+        </is>
+      </c>
+      <c r="I443" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/E6QAAeSwbz5quNH9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J443" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29T02:30:43.000Z</t>
+        </is>
+      </c>
+      <c r="K443" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L443" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M443" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N443" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ZlQAAeSwpAVquNH9/s-l1600.jpg | https://i.ebayimg.com/images/g/fhkAAeSwffpquNH-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O443" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P443" s="2" t="inlineStr"/>
+      <c r="Q443" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R443" s="2" t="inlineStr"/>
+      <c r="S443" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="2" t="inlineStr">
+        <is>
+          <t>Elisabetta Cocciaretto</t>
+        </is>
+      </c>
+      <c r="B444" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C444" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Sapphire Green 1/125 Elisabetta Cocciaretto Rookie RC 0nr3</t>
+        </is>
+      </c>
+      <c r="D444" s="2" t="inlineStr">
+        <is>
+          <t>1/125</t>
+        </is>
+      </c>
+      <c r="E444" s="2" t="inlineStr">
+        <is>
+          <t>001 of 125</t>
+        </is>
+      </c>
+      <c r="F444" s="2" t="inlineStr">
+        <is>
+          <t>7.50 USD</t>
+        </is>
+      </c>
+      <c r="G444" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237096031202</t>
+        </is>
+      </c>
+      <c r="H444" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:03 UTC</t>
+        </is>
+      </c>
+      <c r="I444" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ivUAAeSwtJFquxHQ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J444" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29T01:17:04.000Z</t>
+        </is>
+      </c>
+      <c r="K444" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L444" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M444" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N444" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jgYAAeSwZ2ZquxHQ/s-l1600.jpg | https://i.ebayimg.com/images/g/jbMAAeSw271quxHQ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O444" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P444" s="2" t="inlineStr"/>
+      <c r="Q444" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R444" s="2" t="inlineStr"/>
+      <c r="S444" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="2" t="inlineStr">
+        <is>
+          <t>Linda Noskova</t>
+        </is>
+      </c>
+      <c r="B445" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C445" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026 Topps Graphite Linda Noskova Match Point Marks Gold Refractor Auto 1/25 </t>
+        </is>
+      </c>
+      <c r="D445" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E445" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F445" s="2" t="inlineStr">
+        <is>
+          <t>18.00 USD</t>
+        </is>
+      </c>
+      <c r="G445" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168737553304</t>
+        </is>
+      </c>
+      <c r="H445" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:03 UTC</t>
+        </is>
+      </c>
+      <c r="I445" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/pLIAAeSwNghqu0sD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J445" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29T05:22:44.000Z</t>
+        </is>
+      </c>
+      <c r="K445" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L445" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M445" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N445" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/pPQAAeSwASdqu0sL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O445" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P445" s="2" t="inlineStr"/>
+      <c r="Q445" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R445" s="2" t="inlineStr"/>
+      <c r="S445" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="2" t="inlineStr">
+        <is>
+          <t>Ekaterina Alexandrova</t>
+        </is>
+      </c>
+      <c r="B446" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C446" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Aqua Refractor 1/199 Ekaterina Alexandrova #67 Rookie RC pe8</t>
+        </is>
+      </c>
+      <c r="D446" s="2" t="inlineStr">
+        <is>
+          <t>1/199</t>
+        </is>
+      </c>
+      <c r="E446" s="2" t="inlineStr">
+        <is>
+          <t>001 of 199</t>
+        </is>
+      </c>
+      <c r="F446" s="2" t="inlineStr">
+        <is>
+          <t>14.63 USD</t>
+        </is>
+      </c>
+      <c r="G446" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257772225006</t>
+        </is>
+      </c>
+      <c r="H446" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:03 UTC</t>
+        </is>
+      </c>
+      <c r="I446" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/hUEAAeSwXUBquxx~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J446" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29T02:02:39.000Z</t>
+        </is>
+      </c>
+      <c r="K446" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L446" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M446" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N446" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gscAAeSw3GJquxx-/s-l1600.jpg | https://i.ebayimg.com/images/g/mG8AAeSwpG5quxx-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O446" s="2" t="inlineStr">
+        <is>
+          <t>aqua</t>
+        </is>
+      </c>
+      <c r="P446" s="2" t="inlineStr"/>
+      <c r="Q446" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R446" s="2" t="inlineStr"/>
+      <c r="S446" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="2" t="inlineStr">
+        <is>
+          <t>Marcos Giron</t>
+        </is>
+      </c>
+      <c r="B447" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C447" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Red Crystalline Refractor 1/1 Marcos Giron Rookie RC 1e41</t>
+        </is>
+      </c>
+      <c r="D447" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E447" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F447" s="2" t="inlineStr">
+        <is>
+          <t>254.75 USD</t>
+        </is>
+      </c>
+      <c r="G447" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257771873560</t>
+        </is>
+      </c>
+      <c r="H447" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:03 UTC</t>
+        </is>
+      </c>
+      <c r="I447" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/IIAAAeSwuxRquuGp/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J447" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T21:51:35.000Z</t>
+        </is>
+      </c>
+      <c r="K447" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L447" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M447" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N447" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/G7cAAeSwmwpquuGp/s-l1600.jpg | https://i.ebayimg.com/images/g/Gd0AAeSw-UZquuGp/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O447" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P447" s="2" t="inlineStr"/>
+      <c r="Q447" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R447" s="2" t="inlineStr"/>
+      <c r="S447" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="2" t="inlineStr">
+        <is>
+          <t>Brandon Holt</t>
+        </is>
+      </c>
+      <c r="B448" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Regalia Relics - Gold</t>
+        </is>
+      </c>
+      <c r="C448" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Regalia Relics Gold 1/10 Brandon Holt #RER-BH 9et</t>
+        </is>
+      </c>
+      <c r="D448" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E448" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F448" s="2" t="inlineStr">
+        <is>
+          <t>41.08 USD</t>
+        </is>
+      </c>
+      <c r="G448" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237095594928</t>
+        </is>
+      </c>
+      <c r="H448" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:03 UTC</t>
+        </is>
+      </c>
+      <c r="I448" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Vg8AAeSwZ2ZqurZP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J448" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T18:46:40.000Z</t>
+        </is>
+      </c>
+      <c r="K448" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L448" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M448" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N448" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/73QAAeSw7bpqurZP/s-l1600.jpg | https://i.ebayimg.com/images/g/VecAAeSw9HBqurZP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O448" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P448" s="2" t="inlineStr"/>
+      <c r="Q448" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R448" s="2" t="inlineStr"/>
+      <c r="S448" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="2" t="inlineStr">
+        <is>
+          <t>Mitchell Krueger</t>
+        </is>
+      </c>
+      <c r="B449" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Regalia Relics - Blue</t>
+        </is>
+      </c>
+      <c r="C449" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Regalia Relics Blue 1/25 Mitchell Krueger #RER-MR 9et</t>
+        </is>
+      </c>
+      <c r="D449" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E449" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F449" s="2" t="inlineStr">
+        <is>
+          <t>18.08 USD</t>
+        </is>
+      </c>
+      <c r="G449" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336817463568</t>
+        </is>
+      </c>
+      <c r="H449" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:03 UTC</t>
+        </is>
+      </c>
+      <c r="I449" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TfcAAeSwZ2hqurXD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J449" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T18:44:13.000Z</t>
+        </is>
+      </c>
+      <c r="K449" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L449" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M449" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N449" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SbgAAeSwfndqurXD/s-l1600.jpg | https://i.ebayimg.com/images/g/RbkAAeSwkkdqurXD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O449" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P449" s="2" t="inlineStr"/>
+      <c r="Q449" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R449" s="2" t="inlineStr"/>
+      <c r="S449" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -39337,6 +40049,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G439" r:id="rId438"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G440" r:id="rId439"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G441" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G442" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G443" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G444" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G445" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G446" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G447" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G448" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G449" r:id="rId448"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-30 16:02 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S449"/>
+  <dimension ref="A1:S463"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -39602,6 +39602,1236 @@
       </c>
       <c r="R449" s="2" t="inlineStr"/>
       <c r="S449" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="2" t="inlineStr"/>
+      <c r="B450" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Royalty</t>
+        </is>
+      </c>
+      <c r="C450" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Jessica Pegula Madison Keys Black 10/10 Auto Dual</t>
+        </is>
+      </c>
+      <c r="D450" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E450" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F450" s="2" t="inlineStr">
+        <is>
+          <t>499.99 USD</t>
+        </is>
+      </c>
+      <c r="G450" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336820947328</t>
+        </is>
+      </c>
+      <c r="H450" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:01 UTC</t>
+        </is>
+      </c>
+      <c r="I450" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Sq4AAeSwWMNqvSxG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J450" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T15:36:37.000Z</t>
+        </is>
+      </c>
+      <c r="K450" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L450" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M450" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N450" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/V-0AAeSwsv9qvSxG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O450" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P450" s="2" t="inlineStr"/>
+      <c r="Q450" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R450" s="2" t="inlineStr"/>
+      <c r="S450" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="2" t="inlineStr">
+        <is>
+          <t>Alexandra Eala</t>
+        </is>
+      </c>
+      <c r="B451" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C451" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Alexandra Eala #101 Gold Geometric Refractor 01/50</t>
+        </is>
+      </c>
+      <c r="D451" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E451" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F451" s="2" t="inlineStr">
+        <is>
+          <t>225.00 USD</t>
+        </is>
+      </c>
+      <c r="G451" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168745910814</t>
+        </is>
+      </c>
+      <c r="H451" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:01 UTC</t>
+        </is>
+      </c>
+      <c r="I451" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0RkAAeSw24tqvSkP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J451" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T15:22:41.000Z</t>
+        </is>
+      </c>
+      <c r="K451" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L451" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M451" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N451" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/1D8AAeSwNG5qvSkP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O451" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P451" s="2" t="inlineStr"/>
+      <c r="Q451" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R451" s="2" t="inlineStr"/>
+      <c r="S451" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="2" t="inlineStr">
+        <is>
+          <t>Aryna Sabalenka</t>
+        </is>
+      </c>
+      <c r="B452" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="C452" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS CHROME TENNIS PINK GEOMETRIC REFRACTOR #21 ARYNA SABALENKA 1/65 PSA 9</t>
+        </is>
+      </c>
+      <c r="D452" s="2" t="inlineStr">
+        <is>
+          <t>1/65</t>
+        </is>
+      </c>
+      <c r="E452" s="2" t="inlineStr">
+        <is>
+          <t>001 of 65</t>
+        </is>
+      </c>
+      <c r="F452" s="2" t="inlineStr">
+        <is>
+          <t>69.69 USD</t>
+        </is>
+      </c>
+      <c r="G452" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117439909234</t>
+        </is>
+      </c>
+      <c r="H452" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:01 UTC</t>
+        </is>
+      </c>
+      <c r="I452" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/eYQAAeSwoH1qvSKi/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J452" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T14:53:21.000Z</t>
+        </is>
+      </c>
+      <c r="K452" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L452" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M452" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N452" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SVQAAeSwFJ9qvSKi/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O452" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P452" s="2" t="inlineStr"/>
+      <c r="Q452" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R452" s="2" t="inlineStr"/>
+      <c r="S452" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="2" t="inlineStr">
+        <is>
+          <t>Zoe Kruger</t>
+        </is>
+      </c>
+      <c r="B453" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS CHROME TENNIS AUTOGRAPHS</t>
+        </is>
+      </c>
+      <c r="C453" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS CHROME TENNIS AUTOS BLACK REFRACTOR ZOE KRUGER 10/10 PSA 8 AUTO 10</t>
+        </is>
+      </c>
+      <c r="D453" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E453" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F453" s="2" t="inlineStr">
+        <is>
+          <t>75.00 USD</t>
+        </is>
+      </c>
+      <c r="G453" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307206830137</t>
+        </is>
+      </c>
+      <c r="H453" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:01 UTC</t>
+        </is>
+      </c>
+      <c r="I453" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/m1YAAeSwkhlqvRrJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J453" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T14:19:51.000Z</t>
+        </is>
+      </c>
+      <c r="K453" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L453" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M453" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 8</t>
+        </is>
+      </c>
+      <c r="N453" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uTQAAeSwQ6VqvRrJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O453" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P453" s="2" t="inlineStr"/>
+      <c r="Q453" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R453" s="2" t="inlineStr"/>
+      <c r="S453" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="2" t="inlineStr">
+        <is>
+          <t>Joao Fonseca, Beatriz Haddad Maia</t>
+        </is>
+      </c>
+      <c r="B454" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C454" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis JOAO FONSECA/BEATRIZ HADDAD MAIA Dual Auto 1/25</t>
+        </is>
+      </c>
+      <c r="D454" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E454" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F454" s="2" t="inlineStr">
+        <is>
+          <t>7500.00 USD</t>
+        </is>
+      </c>
+      <c r="G454" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147609436157?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde9bo1YDFiEKrLXCF%2BZ23o8THHzcsjTC1jrh1PWVnNj1UCpUIdY%2FP3EhSgEKSr4BOz98GnMuf9kkBeU98IXDPOwg9gYIc0p1REDsDR%2BGx8pixM5WAqfftXvK5Jb8PUTFOalDr8tt4m1w2uulNxJiZR%2B457UJ0HBbSyXvWW4W2ZUA0Q8Xh5f7%2B5rcpFCG7XFDR90%3D</t>
+        </is>
+      </c>
+      <c r="H454" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:01 UTC</t>
+        </is>
+      </c>
+      <c r="I454" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/zSYAAeSwEFNqvLK9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J454" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T06:57:58.000Z</t>
+        </is>
+      </c>
+      <c r="K454" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L454" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M454" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N454" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/j-AAAeSwj~lqvLK9/s-l1600.jpg | https://i.ebayimg.com/images/g/cWQAAeSwqYhqvLK8/s-l1600.jpg | https://i.ebayimg.com/images/g/sBQAAeSwr9JqvLK8/s-l1600.jpg | https://i.ebayimg.com/images/g/gAwAAeSwZPtqvLK9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O454" s="2" t="inlineStr"/>
+      <c r="P454" s="2" t="inlineStr"/>
+      <c r="Q454" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R454" s="2" t="inlineStr"/>
+      <c r="S454" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="2" t="inlineStr">
+        <is>
+          <t>Jonas Bjorkman</t>
+        </is>
+      </c>
+      <c r="B455" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C455" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Rose Gold Refractor 10/10 Jonas Bjorkman Jonas Björkman #6 nd3</t>
+        </is>
+      </c>
+      <c r="D455" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E455" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F455" s="2" t="inlineStr">
+        <is>
+          <t>52.29 USD</t>
+        </is>
+      </c>
+      <c r="G455" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237098080252</t>
+        </is>
+      </c>
+      <c r="H455" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:02 UTC</t>
+        </is>
+      </c>
+      <c r="I455" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/rHQAAeSwc4VqvIce/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J455" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T03:49:49.000Z</t>
+        </is>
+      </c>
+      <c r="K455" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L455" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M455" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N455" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/oLQAAeSw4PpqvIce/s-l1600.jpg | https://i.ebayimg.com/images/g/0rkAAeSwnBlqvIce/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O455" s="2" t="inlineStr">
+        <is>
+          <t>rose</t>
+        </is>
+      </c>
+      <c r="P455" s="2" t="inlineStr"/>
+      <c r="Q455" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R455" s="2" t="inlineStr"/>
+      <c r="S455" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="2" t="inlineStr">
+        <is>
+          <t>Giovanni Mpetshi Perricard</t>
+        </is>
+      </c>
+      <c r="B456" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C456" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Giovanni Mpetshi Perricard Gold Youthquake 1/50 🔥</t>
+        </is>
+      </c>
+      <c r="D456" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E456" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F456" s="2" t="inlineStr">
+        <is>
+          <t>119.99 USD</t>
+        </is>
+      </c>
+      <c r="G456" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377532844646</t>
+        </is>
+      </c>
+      <c r="H456" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:02 UTC</t>
+        </is>
+      </c>
+      <c r="I456" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SlgAAeSwEWlqvIDH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J456" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T03:25:13.000Z</t>
+        </is>
+      </c>
+      <c r="K456" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L456" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M456" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N456" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/mxcAAeSwoH1qvIC8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O456" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P456" s="2" t="inlineStr"/>
+      <c r="Q456" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R456" s="2" t="inlineStr"/>
+      <c r="S456" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="2" t="inlineStr">
+        <is>
+          <t>Brenda Fruhvirtova</t>
+        </is>
+      </c>
+      <c r="B457" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C457" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2026 Topps Graphite Tennis Brenda Fruhvirtova Relic GR-BF 25/25</t>
+        </is>
+      </c>
+      <c r="D457" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E457" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F457" s="2" t="inlineStr">
+        <is>
+          <t>4.49 USD</t>
+        </is>
+      </c>
+      <c r="G457" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168742658283</t>
+        </is>
+      </c>
+      <c r="H457" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:02 UTC</t>
+        </is>
+      </c>
+      <c r="I457" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-NgAAeSwUMdqvE6Y/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J457" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29T23:50:29.000Z</t>
+        </is>
+      </c>
+      <c r="K457" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L457" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M457" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N457" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ZPgAAeSwxclqvE6J/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O457" s="2" t="inlineStr"/>
+      <c r="P457" s="2" t="inlineStr"/>
+      <c r="Q457" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R457" s="2" t="inlineStr"/>
+      <c r="S457" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="2" t="inlineStr">
+        <is>
+          <t>Novak Djokovic</t>
+        </is>
+      </c>
+      <c r="B458" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C458" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Tennis Novak Djokovic BP-6 Red Crystalline 1/1 - PSA 8 GOAT</t>
+        </is>
+      </c>
+      <c r="D458" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E458" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F458" s="2" t="inlineStr">
+        <is>
+          <t>20000.00 USD</t>
+        </is>
+      </c>
+      <c r="G458" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237097760593</t>
+        </is>
+      </c>
+      <c r="H458" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:02 UTC</t>
+        </is>
+      </c>
+      <c r="I458" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/iwkAAeSwFY1qvEPp/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J458" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29T23:06:34.000Z</t>
+        </is>
+      </c>
+      <c r="K458" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L458" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M458" s="2" t="inlineStr">
+        <is>
+          <t>PSA 8</t>
+        </is>
+      </c>
+      <c r="N458" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/4W4AAeSwIG5qvEPp/s-l1600.jpg | https://i.ebayimg.com/images/g/rTQAAeSwXvtqvEPq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O458" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P458" s="2" t="inlineStr"/>
+      <c r="Q458" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R458" s="2" t="inlineStr"/>
+      <c r="S458" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="2" t="inlineStr">
+        <is>
+          <t>Louisa Chirico</t>
+        </is>
+      </c>
+      <c r="B459" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C459" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Tour Relic Green Refractor 75/75 Louisa Chirico Auto 04ap</t>
+        </is>
+      </c>
+      <c r="D459" s="2" t="inlineStr">
+        <is>
+          <t>75/75</t>
+        </is>
+      </c>
+      <c r="E459" s="2" t="inlineStr">
+        <is>
+          <t>last of 75 (75/75)</t>
+        </is>
+      </c>
+      <c r="F459" s="2" t="inlineStr">
+        <is>
+          <t>6.46 USD</t>
+        </is>
+      </c>
+      <c r="G459" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336819480910</t>
+        </is>
+      </c>
+      <c r="H459" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:02 UTC</t>
+        </is>
+      </c>
+      <c r="I459" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/zx4AAeSwO2lqvChu/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J459" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29T21:05:51.000Z</t>
+        </is>
+      </c>
+      <c r="K459" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L459" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M459" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N459" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/AzUAAeSwoDtqvChu/s-l1600.jpg | https://i.ebayimg.com/images/g/zQ8AAeSwk7BqvChu/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O459" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P459" s="2" t="inlineStr"/>
+      <c r="Q459" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R459" s="2" t="inlineStr"/>
+      <c r="S459" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="2" t="inlineStr">
+        <is>
+          <t>Emilio Nava</t>
+        </is>
+      </c>
+      <c r="B460" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Regalia Relics - Gold</t>
+        </is>
+      </c>
+      <c r="C460" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Regalia Relics Gold 10/10 Emilio Nava #RER-EN Rookie RC 5ov</t>
+        </is>
+      </c>
+      <c r="D460" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E460" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F460" s="2" t="inlineStr">
+        <is>
+          <t>23.82 USD</t>
+        </is>
+      </c>
+      <c r="G460" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336820028696</t>
+        </is>
+      </c>
+      <c r="H460" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:02 UTC</t>
+        </is>
+      </c>
+      <c r="I460" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/y6EAAeSwhlNqvIYE/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J460" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T03:45:06.000Z</t>
+        </is>
+      </c>
+      <c r="K460" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L460" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M460" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N460" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uKsAAeSwkkdqvIYE/s-l1600.jpg | https://i.ebayimg.com/images/g/wFEAAeSw9nRqvIYE/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O460" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P460" s="2" t="inlineStr"/>
+      <c r="Q460" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R460" s="2" t="inlineStr"/>
+      <c r="S460" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="2" t="inlineStr">
+        <is>
+          <t>Elena Rybakina</t>
+        </is>
+      </c>
+      <c r="B461" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C461" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Elena Rybakina Superior Signatures Platinum Auto #1/1</t>
+        </is>
+      </c>
+      <c r="D461" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E461" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F461" s="2" t="inlineStr">
+        <is>
+          <t>2425.00 USD</t>
+        </is>
+      </c>
+      <c r="G461" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/128105292627</t>
+        </is>
+      </c>
+      <c r="H461" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:02 UTC</t>
+        </is>
+      </c>
+      <c r="I461" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/g3EAAeSwu~Vqu-1g/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J461" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T00:30:00.000Z</t>
+        </is>
+      </c>
+      <c r="K461" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L461" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M461" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N461" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/u-cAAeSwE3Zqu-1g/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O461" s="2" t="inlineStr"/>
+      <c r="P461" s="2" t="inlineStr"/>
+      <c r="Q461" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R461" s="2" t="inlineStr"/>
+      <c r="S461" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B462" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Now</t>
+        </is>
+      </c>
+      <c r="C462" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Now Tennis Carlos Alcaraz #8-AR Match-Used Ball Auto Red 5/5</t>
+        </is>
+      </c>
+      <c r="D462" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E462" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F462" s="2" t="inlineStr">
+        <is>
+          <t>20000.00 USD</t>
+        </is>
+      </c>
+      <c r="G462" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/318936213260</t>
+        </is>
+      </c>
+      <c r="H462" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:02 UTC</t>
+        </is>
+      </c>
+      <c r="I462" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/qj0AAeSwjjpqvISc/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J462" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T03:43:02.000Z</t>
+        </is>
+      </c>
+      <c r="K462" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L462" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M462" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N462" s="2" t="inlineStr"/>
+      <c r="O462" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P462" s="2" t="inlineStr"/>
+      <c r="Q462" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R462" s="2" t="inlineStr"/>
+      <c r="S462" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="2" t="inlineStr">
+        <is>
+          <t>Stan Smith</t>
+        </is>
+      </c>
+      <c r="B463" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic / 2013 Ace Authentic Grand Slam</t>
+        </is>
+      </c>
+      <c r="C463" s="2" t="inlineStr">
+        <is>
+          <t>2013 Ace Authentic Auto Blue 5/5 #SS1 Stan Smith PSA 9 (Top Pop, Pop 1)</t>
+        </is>
+      </c>
+      <c r="D463" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E463" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F463" s="2" t="inlineStr">
+        <is>
+          <t>125.00 USD</t>
+        </is>
+      </c>
+      <c r="G463" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168742729275</t>
+        </is>
+      </c>
+      <c r="H463" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:02 UTC</t>
+        </is>
+      </c>
+      <c r="I463" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/rqgAAOSw~dlld1nT/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J463" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T00:36:40.000Z</t>
+        </is>
+      </c>
+      <c r="K463" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L463" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M463" s="2" t="inlineStr">
+        <is>
+          <t>PSA 9</t>
+        </is>
+      </c>
+      <c r="N463" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9IAAAOSwx4Jld1nc/s-l1600.jpg | https://i.ebayimg.com/images/g/~ZEAAOSwxKZld1nl/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O463" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P463" s="2" t="inlineStr"/>
+      <c r="Q463" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R463" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic autograph: on-card or sticker not stated; check by eye</t>
+        </is>
+      </c>
+      <c r="S463" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -40057,6 +41287,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G447" r:id="rId446"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G448" r:id="rId447"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G449" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G450" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G451" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G452" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G453" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G454" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G455" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G456" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G457" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G458" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G459" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G460" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G461" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G462" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G463" r:id="rId462"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-09-30 23:42 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S463"/>
+  <dimension ref="A1:S493"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -40832,6 +40832,2640 @@
         </is>
       </c>
       <c r="S463" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="2" t="inlineStr">
+        <is>
+          <t>Marta Kostyuk</t>
+        </is>
+      </c>
+      <c r="B464" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C464" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis MARTA KOSTYUK Destiny Superfractor 1/1</t>
+        </is>
+      </c>
+      <c r="D464" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E464" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F464" s="2" t="inlineStr">
+        <is>
+          <t>1495.00 USD</t>
+        </is>
+      </c>
+      <c r="G464" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/128108051285</t>
+        </is>
+      </c>
+      <c r="H464" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:41 UTC</t>
+        </is>
+      </c>
+      <c r="I464" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/rkwAAeSw~yNqvZvK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J464" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T23:32:20.000Z</t>
+        </is>
+      </c>
+      <c r="K464" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L464" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M464" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N464" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nikAAeSwFrlqvZvK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O464" s="2" t="inlineStr"/>
+      <c r="P464" s="2" t="inlineStr"/>
+      <c r="Q464" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R464" s="2" t="inlineStr"/>
+      <c r="S464" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek</t>
+        </is>
+      </c>
+      <c r="B465" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C465" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Iga Swiatek Auto 1/99 eBay 1/1!!</t>
+        </is>
+      </c>
+      <c r="D465" s="2" t="inlineStr">
+        <is>
+          <t>1/99</t>
+        </is>
+      </c>
+      <c r="E465" s="2" t="inlineStr">
+        <is>
+          <t>001 of 99</t>
+        </is>
+      </c>
+      <c r="F465" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G465" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/398448655744</t>
+        </is>
+      </c>
+      <c r="H465" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:41 UTC</t>
+        </is>
+      </c>
+      <c r="I465" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/sXsAAeSwzF9qvZls/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J465" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T23:21:53.000Z</t>
+        </is>
+      </c>
+      <c r="K465" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L465" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M465" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N465" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9TsAAeSwXvtqvZls/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O465" s="2" t="inlineStr"/>
+      <c r="P465" s="2" t="inlineStr"/>
+      <c r="Q465" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R465" s="2" t="inlineStr"/>
+      <c r="S465" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="2" t="inlineStr">
+        <is>
+          <t>Taylor Fritz</t>
+        </is>
+      </c>
+      <c r="B466" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C466" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Taylor Fritz Frozen Fractor -1/0</t>
+        </is>
+      </c>
+      <c r="D466" s="2" t="inlineStr">
+        <is>
+          <t>1/0</t>
+        </is>
+      </c>
+      <c r="E466" s="2" t="inlineStr">
+        <is>
+          <t>001 of 0</t>
+        </is>
+      </c>
+      <c r="F466" s="2" t="inlineStr">
+        <is>
+          <t>250.00 USD</t>
+        </is>
+      </c>
+      <c r="G466" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407258150548?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2F%2BmXHMDbVuXn5CgpAjAjSA4Z2cw7j6Ypoy6hVwWnuMfgXSMaG1rhDh%2BAbnLtwarRwXBFxd13N4RZyZDJB1AESOUPCXZYwn5iTaAuFE0Q2hF50wWKWduOAy1J8EYTXYcu7ynKMddeVqWC1zFVbXZGeP7BLK3%2BpuXPKO8L7Cj%2FnQku4eblaiZFpXduDHWNm6WyM%3D</t>
+        </is>
+      </c>
+      <c r="H466" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:41 UTC</t>
+        </is>
+      </c>
+      <c r="I466" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/IuQAAeSwo29qvZC~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J466" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T22:46:04.000Z</t>
+        </is>
+      </c>
+      <c r="K466" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L466" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M466" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA)</t>
+        </is>
+      </c>
+      <c r="N466" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ZOAAAeSwN89qvZC~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O466" s="2" t="inlineStr"/>
+      <c r="P466" s="2" t="inlineStr"/>
+      <c r="Q466" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R466" s="2" t="inlineStr"/>
+      <c r="S466" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B467" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C467" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Carlos Alcaraz Orange Auto 1/25 First On Print AO-CAZ</t>
+        </is>
+      </c>
+      <c r="D467" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E467" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F467" s="2" t="inlineStr">
+        <is>
+          <t>3499.00 USD</t>
+        </is>
+      </c>
+      <c r="G467" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/398448534586?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2BaJKCfJJuMF%2BLNNiPc2GTOTmf0fTXinToc0PthsCgU3axnTcNd7QARmyl7Ax2bcNhRcV3WjPt1g7z4RijRLig8awxlJXkrEcXpb0JNRThDwwm4uocTo9Se8byHAJ53o%2Fr7hnflhh0vu61EysZYRyaXQJcUyqTpzMZT0xa5OOcJDNvSSQn%2FyDpy8Lrg1ivrh24%3D</t>
+        </is>
+      </c>
+      <c r="H467" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:41 UTC</t>
+        </is>
+      </c>
+      <c r="I467" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8~gAAeSw~yNqvYxj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J467" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T22:28:11.000Z</t>
+        </is>
+      </c>
+      <c r="K467" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L467" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M467" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N467" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HKQAAeSwSk9qvYxj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O467" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P467" s="2" t="inlineStr"/>
+      <c r="Q467" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R467" s="2" t="inlineStr"/>
+      <c r="S467" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="2" t="inlineStr">
+        <is>
+          <t>Lulu Sun</t>
+        </is>
+      </c>
+      <c r="B468" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C468" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Lulu Sun Rookie Auto RC Black 10/10 On Card!</t>
+        </is>
+      </c>
+      <c r="D468" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E468" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F468" s="2" t="inlineStr">
+        <is>
+          <t>499.99 USD</t>
+        </is>
+      </c>
+      <c r="G468" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168747156159</t>
+        </is>
+      </c>
+      <c r="H468" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:41 UTC</t>
+        </is>
+      </c>
+      <c r="I468" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/CjsAAeSwJxpqvYzL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J468" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T22:27:51.000Z</t>
+        </is>
+      </c>
+      <c r="K468" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L468" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M468" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N468" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0SgAAeSwdvtqvYzL/s-l1600.jpg | https://i.ebayimg.com/images/g/aC0AAeSwCcBqvYzK/s-l1600.jpg | https://i.ebayimg.com/images/g/k1sAAeSwWMNqvYzK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O468" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P468" s="2" t="inlineStr"/>
+      <c r="Q468" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R468" s="2" t="inlineStr"/>
+      <c r="S468" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="2" t="inlineStr">
+        <is>
+          <t>Casper Ruud</t>
+        </is>
+      </c>
+      <c r="B469" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C469" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Casper Ruud Aces Black Auto 1/10</t>
+        </is>
+      </c>
+      <c r="D469" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E469" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F469" s="2" t="inlineStr">
+        <is>
+          <t>250.00 USD</t>
+        </is>
+      </c>
+      <c r="G469" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/398448520844</t>
+        </is>
+      </c>
+      <c r="H469" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:41 UTC</t>
+        </is>
+      </c>
+      <c r="I469" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SeQAAeSwjjpqvYpo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J469" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T22:18:24.000Z</t>
+        </is>
+      </c>
+      <c r="K469" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L469" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M469" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N469" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9V8AAeSwGgNqvYpo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O469" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P469" s="2" t="inlineStr"/>
+      <c r="Q469" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R469" s="2" t="inlineStr"/>
+      <c r="S469" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B470" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C470" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Carlos Alcaraz Destiny Orange Geometric #1/25 First on Print</t>
+        </is>
+      </c>
+      <c r="D470" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E470" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F470" s="2" t="inlineStr">
+        <is>
+          <t>124.99 USD</t>
+        </is>
+      </c>
+      <c r="G470" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287618992566</t>
+        </is>
+      </c>
+      <c r="H470" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:41 UTC</t>
+        </is>
+      </c>
+      <c r="I470" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QVMAAeSwdLZqvYpQ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J470" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T22:15:45.000Z</t>
+        </is>
+      </c>
+      <c r="K470" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L470" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M470" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N470" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/4vcAAeSwkkdqvYpQ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O470" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P470" s="2" t="inlineStr"/>
+      <c r="Q470" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R470" s="2" t="inlineStr"/>
+      <c r="S470" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="2" t="inlineStr">
+        <is>
+          <t>Veronika Kudermetova</t>
+        </is>
+      </c>
+      <c r="B471" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C471" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Veronika Kudermetova SUPERFRACTOR 1/1</t>
+        </is>
+      </c>
+      <c r="D471" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E471" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F471" s="2" t="inlineStr">
+        <is>
+          <t>1499.99 USD</t>
+        </is>
+      </c>
+      <c r="G471" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/189020856809</t>
+        </is>
+      </c>
+      <c r="H471" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:41 UTC</t>
+        </is>
+      </c>
+      <c r="I471" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DLkAAeSwqWZqvYUC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J471" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T21:56:38.000Z</t>
+        </is>
+      </c>
+      <c r="K471" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L471" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M471" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N471" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ujcAAeSwbHBqvYUK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O471" s="2" t="inlineStr"/>
+      <c r="P471" s="2" t="inlineStr"/>
+      <c r="Q471" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R471" s="2" t="inlineStr"/>
+      <c r="S471" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="2" t="inlineStr">
+        <is>
+          <t>Hugo Gaston</t>
+        </is>
+      </c>
+      <c r="B472" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C472" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis HUGO GASTON On Card AUTO PINK REFRACTOR 1/250 1ST ONE</t>
+        </is>
+      </c>
+      <c r="D472" s="2" t="inlineStr">
+        <is>
+          <t>1/250</t>
+        </is>
+      </c>
+      <c r="E472" s="2" t="inlineStr">
+        <is>
+          <t>001 of 250</t>
+        </is>
+      </c>
+      <c r="F472" s="2" t="inlineStr">
+        <is>
+          <t>14.99 USD</t>
+        </is>
+      </c>
+      <c r="G472" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/206593525714</t>
+        </is>
+      </c>
+      <c r="H472" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I472" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gCwAAeSw8NZqvYNI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J472" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T21:49:52.000Z</t>
+        </is>
+      </c>
+      <c r="K472" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L472" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M472" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N472" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/o9UAAeSwtJFqvYNK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O472" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P472" s="2" t="inlineStr"/>
+      <c r="Q472" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R472" s="2" t="inlineStr"/>
+      <c r="S472" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="2" t="inlineStr">
+        <is>
+          <t>Genie Bouchard</t>
+        </is>
+      </c>
+      <c r="B473" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Royalty</t>
+        </is>
+      </c>
+      <c r="C473" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Genie Bouchard 1/50 Gold Auto Bookend</t>
+        </is>
+      </c>
+      <c r="D473" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E473" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F473" s="2" t="inlineStr">
+        <is>
+          <t>89.99 USD</t>
+        </is>
+      </c>
+      <c r="G473" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336821350452</t>
+        </is>
+      </c>
+      <c r="H473" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I473" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TiUAAeSwNG5qvX5Q/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J473" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T21:26:17.000Z</t>
+        </is>
+      </c>
+      <c r="K473" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L473" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M473" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N473" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/tEkAAeSwG7pqvX5Q/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O473" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P473" s="2" t="inlineStr"/>
+      <c r="Q473" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R473" s="2" t="inlineStr"/>
+      <c r="S473" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="2" t="inlineStr">
+        <is>
+          <t>Ivan Lendl</t>
+        </is>
+      </c>
+      <c r="B474" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C474" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Ivan Lendl World Number 1 Superfractor 1/1 On Card Auto</t>
+        </is>
+      </c>
+      <c r="D474" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E474" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F474" s="2" t="inlineStr">
+        <is>
+          <t>45000.00 USD</t>
+        </is>
+      </c>
+      <c r="G474" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/206593486588</t>
+        </is>
+      </c>
+      <c r="H474" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I474" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TwIAAeSwtJFqvXxR/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J474" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T21:20:07.000Z</t>
+        </is>
+      </c>
+      <c r="K474" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L474" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M474" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N474" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RogAAeSwKRpqvXxC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O474" s="2" t="inlineStr"/>
+      <c r="P474" s="2" t="inlineStr"/>
+      <c r="Q474" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R474" s="2" t="inlineStr"/>
+      <c r="S474" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="2" t="inlineStr">
+        <is>
+          <t>Karolina Pliskova</t>
+        </is>
+      </c>
+      <c r="B475" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C475" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Karolina Pliskova AO-KPA Geometric Blue Auto 150/150</t>
+        </is>
+      </c>
+      <c r="D475" s="2" t="inlineStr">
+        <is>
+          <t>150/150</t>
+        </is>
+      </c>
+      <c r="E475" s="2" t="inlineStr">
+        <is>
+          <t>last of 150 (150/150)</t>
+        </is>
+      </c>
+      <c r="F475" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G475" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/198678703892</t>
+        </is>
+      </c>
+      <c r="H475" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I475" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KPQAAeSwms9qvXcT/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J475" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T21:16:10.000Z</t>
+        </is>
+      </c>
+      <c r="K475" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L475" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M475" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N475" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/018AAeSw6fBqvXca/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O475" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P475" s="2" t="inlineStr"/>
+      <c r="Q475" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R475" s="2" t="inlineStr"/>
+      <c r="S475" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="2" t="inlineStr">
+        <is>
+          <t>Naomi Osaka</t>
+        </is>
+      </c>
+      <c r="B476" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Royalty</t>
+        </is>
+      </c>
+      <c r="C476" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Naomi Osaka Green Auto 1/99</t>
+        </is>
+      </c>
+      <c r="D476" s="2" t="inlineStr">
+        <is>
+          <t>1/99</t>
+        </is>
+      </c>
+      <c r="E476" s="2" t="inlineStr">
+        <is>
+          <t>001 of 99</t>
+        </is>
+      </c>
+      <c r="F476" s="2" t="inlineStr">
+        <is>
+          <t>159.00 USD</t>
+        </is>
+      </c>
+      <c r="G476" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/227546576188?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8uI9UDpzN2FpR2PrFcIr%2B2GFBknzPuN8XM2%2F8foRVuKjMcgP4S3Wa0zT%2Fk%2FkV8UyyyDTN99m3JOoy%2FF%2B5X176mBH3gWS3slq4faS3t0ZxfrgHbe4jdQuVboGdFu6qfv%2B28eGYfWMRgjYQO5Qv8i%2FRgAw%2F7OHHYtJST4vxXmmISRPZi8KmVs7O8azshCVtY3oY%3D</t>
+        </is>
+      </c>
+      <c r="H476" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I476" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jDAAAeSwPGFqvXoG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J476" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T21:08:20.000Z</t>
+        </is>
+      </c>
+      <c r="K476" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L476" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M476" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N476" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/MBUAAeSwSihqvXoN/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O476" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P476" s="2" t="inlineStr"/>
+      <c r="Q476" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R476" s="2" t="inlineStr"/>
+      <c r="S476" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="2" t="inlineStr">
+        <is>
+          <t>Naomi Osaka</t>
+        </is>
+      </c>
+      <c r="B477" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Royalty</t>
+        </is>
+      </c>
+      <c r="C477" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Naomi Osaka Green Auto 1/99</t>
+        </is>
+      </c>
+      <c r="D477" s="2" t="inlineStr">
+        <is>
+          <t>1/99</t>
+        </is>
+      </c>
+      <c r="E477" s="2" t="inlineStr">
+        <is>
+          <t>001 of 99</t>
+        </is>
+      </c>
+      <c r="F477" s="2" t="inlineStr">
+        <is>
+          <t>199.99 USD</t>
+        </is>
+      </c>
+      <c r="G477" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336821314371</t>
+        </is>
+      </c>
+      <c r="H477" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I477" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/00AAAeSwNG5qvXYo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J477" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T20:51:29.000Z</t>
+        </is>
+      </c>
+      <c r="K477" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L477" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M477" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N477" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/B0YAAeSw6HJqvXYo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O477" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P477" s="2" t="inlineStr"/>
+      <c r="Q477" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R477" s="2" t="inlineStr"/>
+      <c r="S477" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="2" t="inlineStr">
+        <is>
+          <t>Sara Sorribes Tormo</t>
+        </is>
+      </c>
+      <c r="B478" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Sapphire Edition - [Base] - Padparadscha</t>
+        </is>
+      </c>
+      <c r="C478" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Sapphire Padparadscha 1/1 Sara Sorribes Tormo PSA 9 MINT 1e41</t>
+        </is>
+      </c>
+      <c r="D478" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E478" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F478" s="2" t="inlineStr">
+        <is>
+          <t>201.95 USD</t>
+        </is>
+      </c>
+      <c r="G478" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237099438261</t>
+        </is>
+      </c>
+      <c r="H478" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I478" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7BYAAeSwuP5qvXRJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J478" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T20:41:41.000Z</t>
+        </is>
+      </c>
+      <c r="K478" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L478" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M478" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports (PSA) 9 MINT</t>
+        </is>
+      </c>
+      <c r="N478" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/iJ4AAeSw78VqvXRJ/s-l1600.jpg | https://i.ebayimg.com/images/g/FgYAAeSwHeFqvXRJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O478" s="2" t="inlineStr"/>
+      <c r="P478" s="2" t="inlineStr"/>
+      <c r="Q478" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R478" s="2" t="inlineStr"/>
+      <c r="S478" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="2" t="inlineStr">
+        <is>
+          <t>Eva Lys</t>
+        </is>
+      </c>
+      <c r="B479" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C479" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Red Geometric Autograph Eva Lys AT-ELS 🔥5/5 BOOKEND🔥</t>
+        </is>
+      </c>
+      <c r="D479" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E479" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F479" s="2" t="inlineStr">
+        <is>
+          <t>400.00 USD</t>
+        </is>
+      </c>
+      <c r="G479" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287618809609</t>
+        </is>
+      </c>
+      <c r="H479" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I479" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-2QAAeSwMYpqvWhq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J479" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T19:59:56.000Z</t>
+        </is>
+      </c>
+      <c r="K479" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L479" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M479" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N479" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SREAAeSwXUBqvWht/s-l1600.jpg | https://i.ebayimg.com/images/g/J50AAeSwc4VqvWhu/s-l1600.jpg | https://i.ebayimg.com/images/g/VKEAAeSweydqvWhu/s-l1600.jpg | https://i.ebayimg.com/images/g/CeIAAeSwzh1qvWhs/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O479" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P479" s="2" t="inlineStr"/>
+      <c r="Q479" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R479" s="2" t="inlineStr"/>
+      <c r="S479" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="2" t="inlineStr">
+        <is>
+          <t>Diana Shnaider</t>
+        </is>
+      </c>
+      <c r="B480" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C480" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Diana Shnaider #AO-DSR Orange Refractor Auto 25/25 ON-CARD</t>
+        </is>
+      </c>
+      <c r="D480" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E480" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F480" s="2" t="inlineStr">
+        <is>
+          <t>79.99 USD</t>
+        </is>
+      </c>
+      <c r="G480" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257775412898</t>
+        </is>
+      </c>
+      <c r="H480" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I480" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2x8AAeSw-ZRqvWE-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J480" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T19:51:28.000Z</t>
+        </is>
+      </c>
+      <c r="K480" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L480" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M480" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA)</t>
+        </is>
+      </c>
+      <c r="N480" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vBwAAeSwusxqvWE9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O480" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P480" s="2" t="inlineStr"/>
+      <c r="Q480" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R480" s="2" t="inlineStr"/>
+      <c r="S480" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="2" t="inlineStr">
+        <is>
+          <t>Tracy Austin</t>
+        </is>
+      </c>
+      <c r="B481" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Royalty</t>
+        </is>
+      </c>
+      <c r="C481" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Tracy Austin Red Auto 5/5</t>
+        </is>
+      </c>
+      <c r="D481" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E481" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F481" s="2" t="inlineStr">
+        <is>
+          <t>499.99 USD</t>
+        </is>
+      </c>
+      <c r="G481" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336821233118</t>
+        </is>
+      </c>
+      <c r="H481" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I481" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YwYAAeSwqWZqvWgb/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J481" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T19:51:27.000Z</t>
+        </is>
+      </c>
+      <c r="K481" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L481" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M481" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N481" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/AEcAAeSwXnZqvWga/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O481" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P481" s="2" t="inlineStr"/>
+      <c r="Q481" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R481" s="2" t="inlineStr"/>
+      <c r="S481" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="2" t="inlineStr">
+        <is>
+          <t>Jessica Pegula, madison keys</t>
+        </is>
+      </c>
+      <c r="B482" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C482" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Jessica Pegula Madison Keys Dual Auto # 1/25</t>
+        </is>
+      </c>
+      <c r="D482" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E482" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F482" s="2" t="inlineStr">
+        <is>
+          <t>249.99 USD</t>
+        </is>
+      </c>
+      <c r="G482" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178542865377</t>
+        </is>
+      </c>
+      <c r="H482" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I482" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KYwAAeSwt~tqvWb-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J482" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T19:48:23.000Z</t>
+        </is>
+      </c>
+      <c r="K482" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L482" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M482" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N482" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/AUUAAeSw0-xqvWb-/s-l1600.jpg | https://i.ebayimg.com/images/g/RcQAAeSwtChqvWcA/s-l1600.jpg | https://i.ebayimg.com/images/g/agwAAeSwYa5qvWcA/s-l1600.jpg | https://i.ebayimg.com/images/g/Q4cAAeSweHNqvWcC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O482" s="2" t="inlineStr"/>
+      <c r="P482" s="2" t="inlineStr"/>
+      <c r="Q482" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R482" s="2" t="inlineStr"/>
+      <c r="S482" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="2" t="inlineStr">
+        <is>
+          <t>Hubert Hurkacz</t>
+        </is>
+      </c>
+      <c r="B483" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C483" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Hubert Hurkacz AUTO Red Refractor 5/5 BOOKEND</t>
+        </is>
+      </c>
+      <c r="D483" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E483" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F483" s="2" t="inlineStr">
+        <is>
+          <t>325.00 USD</t>
+        </is>
+      </c>
+      <c r="G483" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237099372713</t>
+        </is>
+      </c>
+      <c r="H483" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I483" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JSIAAeSwWAZqvWS8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J483" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T19:36:39.000Z</t>
+        </is>
+      </c>
+      <c r="K483" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L483" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M483" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N483" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/LlEAAeSwG7pqvWS8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O483" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P483" s="2" t="inlineStr"/>
+      <c r="Q483" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R483" s="2" t="inlineStr"/>
+      <c r="S483" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="2" t="inlineStr">
+        <is>
+          <t>Eva Lys Frozenfractor</t>
+        </is>
+      </c>
+      <c r="B484" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C484" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Eva Lys FROZENFRACTOR -1/0 SSP Bookend Case Hit</t>
+        </is>
+      </c>
+      <c r="D484" s="2" t="inlineStr">
+        <is>
+          <t>1/0</t>
+        </is>
+      </c>
+      <c r="E484" s="2" t="inlineStr">
+        <is>
+          <t>001 of 0</t>
+        </is>
+      </c>
+      <c r="F484" s="2" t="inlineStr">
+        <is>
+          <t>500.00 USD</t>
+        </is>
+      </c>
+      <c r="G484" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237099365348</t>
+        </is>
+      </c>
+      <c r="H484" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I484" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8kUAAeSwGgNqvWPV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J484" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T19:34:41.000Z</t>
+        </is>
+      </c>
+      <c r="K484" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L484" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M484" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N484" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9PQAAeSwhtVqvWPV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O484" s="2" t="inlineStr"/>
+      <c r="P484" s="2" t="inlineStr"/>
+      <c r="Q484" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R484" s="2" t="inlineStr"/>
+      <c r="S484" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B485" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C485" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Carlos Alcaraz #50 Black Refractor 10/10</t>
+        </is>
+      </c>
+      <c r="D485" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E485" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F485" s="2" t="inlineStr">
+        <is>
+          <t>3999.99 USD</t>
+        </is>
+      </c>
+      <c r="G485" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/158371151113</t>
+        </is>
+      </c>
+      <c r="H485" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I485" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/q78AAeSwj~lqvWEk/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J485" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T19:27:07.000Z</t>
+        </is>
+      </c>
+      <c r="K485" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L485" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M485" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N485" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/tIgAAeSwBU9qvWE3/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O485" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P485" s="2" t="inlineStr"/>
+      <c r="Q485" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R485" s="2" t="inlineStr"/>
+      <c r="S485" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="2" t="inlineStr">
+        <is>
+          <t>Eva Lys Solus</t>
+        </is>
+      </c>
+      <c r="B486" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C486" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Eva Lys Solus Case Hit 1/1 Suprefractor</t>
+        </is>
+      </c>
+      <c r="D486" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E486" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F486" s="2" t="inlineStr">
+        <is>
+          <t>5750.00 USD</t>
+        </is>
+      </c>
+      <c r="G486" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/227546460067</t>
+        </is>
+      </c>
+      <c r="H486" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I486" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/E3sAAeSwbItqvWCL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J486" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T19:24:05.000Z</t>
+        </is>
+      </c>
+      <c r="K486" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L486" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M486" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N486" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/l-8AAeSwFr5qvWCL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O486" s="2" t="inlineStr"/>
+      <c r="P486" s="2" t="inlineStr"/>
+      <c r="Q486" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R486" s="2" t="inlineStr"/>
+      <c r="S486" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B487" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C487" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Mirra Andreeva Destiny Black Geometric 10/10</t>
+        </is>
+      </c>
+      <c r="D487" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E487" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F487" s="2" t="inlineStr">
+        <is>
+          <t>500.00 USD</t>
+        </is>
+      </c>
+      <c r="G487" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/227546460072</t>
+        </is>
+      </c>
+      <c r="H487" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I487" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/xUIAAeSw8~lqvWCi/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J487" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T19:24:05.000Z</t>
+        </is>
+      </c>
+      <c r="K487" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L487" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M487" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N487" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/AcMAAeSwn2NqvWCh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O487" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P487" s="2" t="inlineStr"/>
+      <c r="Q487" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R487" s="2" t="inlineStr"/>
+      <c r="S487" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="2" t="inlineStr">
+        <is>
+          <t>Ben Shelton</t>
+        </is>
+      </c>
+      <c r="B488" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C488" s="2" t="inlineStr">
+        <is>
+          <t>Ben Shelton Geometric Red Auto 5 /5 Topps Chrome Tennis 2026</t>
+        </is>
+      </c>
+      <c r="D488" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E488" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F488" s="2" t="inlineStr">
+        <is>
+          <t>3402.60 USD</t>
+        </is>
+      </c>
+      <c r="G488" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298721316911</t>
+        </is>
+      </c>
+      <c r="H488" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I488" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/z6MAAeSwZe5qvUzn/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J488" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T17:57:26.000Z</t>
+        </is>
+      </c>
+      <c r="K488" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L488" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M488" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N488" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/UFEAAeSwRWxqvUzn/s-l1600.jpg | https://i.ebayimg.com/images/g/v5wAAeSwWMNqvUzn/s-l1600.jpg | https://i.ebayimg.com/images/g/osAAAeSw8NZqvUzn/s-l1600.jpg | https://i.ebayimg.com/images/g/ctoAAeSwG~dqvUzo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O488" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P488" s="2" t="inlineStr"/>
+      <c r="Q488" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R488" s="2" t="inlineStr"/>
+      <c r="S488" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="2" t="inlineStr">
+        <is>
+          <t>Maria Sharapova</t>
+        </is>
+      </c>
+      <c r="B489" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C489" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Maria Sharapova Auto 1/99 Green Bookend</t>
+        </is>
+      </c>
+      <c r="D489" s="2" t="inlineStr">
+        <is>
+          <t>1/99</t>
+        </is>
+      </c>
+      <c r="E489" s="2" t="inlineStr">
+        <is>
+          <t>001 of 99</t>
+        </is>
+      </c>
+      <c r="F489" s="2" t="inlineStr">
+        <is>
+          <t>299.99 USD</t>
+        </is>
+      </c>
+      <c r="G489" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/318939037480</t>
+        </is>
+      </c>
+      <c r="H489" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I489" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/r4kAAeSwt-dqvUVn/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J489" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T17:23:38.000Z</t>
+        </is>
+      </c>
+      <c r="K489" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L489" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M489" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N489" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/NgYAAeSw3aVqvUVn/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O489" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P489" s="2" t="inlineStr"/>
+      <c r="Q489" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R489" s="2" t="inlineStr"/>
+      <c r="S489" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="2" t="inlineStr">
+        <is>
+          <t>Martina Hingis</t>
+        </is>
+      </c>
+      <c r="B490" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C490" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Martina Hingis Red 1/5 Refractor SSP 181</t>
+        </is>
+      </c>
+      <c r="D490" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E490" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F490" s="2" t="inlineStr">
+        <is>
+          <t>249.99 USD</t>
+        </is>
+      </c>
+      <c r="G490" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/318939030038</t>
+        </is>
+      </c>
+      <c r="H490" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I490" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/L8sAAeSwo29qvUR9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J490" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T17:19:32.000Z</t>
+        </is>
+      </c>
+      <c r="K490" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L490" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M490" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N490" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/udoAAeSwevlqvUR9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O490" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P490" s="2" t="inlineStr"/>
+      <c r="Q490" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R490" s="2" t="inlineStr"/>
+      <c r="S490" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="2" t="inlineStr">
+        <is>
+          <t>John McEnroe</t>
+        </is>
+      </c>
+      <c r="B491" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C491" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis John McEnroe Black 10/10 Auto</t>
+        </is>
+      </c>
+      <c r="D491" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E491" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F491" s="2" t="inlineStr">
+        <is>
+          <t>499.99 USD</t>
+        </is>
+      </c>
+      <c r="G491" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/318938985996</t>
+        </is>
+      </c>
+      <c r="H491" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I491" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/H74AAeSwNG5qvUKF/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J491" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T17:11:11.000Z</t>
+        </is>
+      </c>
+      <c r="K491" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L491" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M491" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N491" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/PLEAAeSwV71qvUKF/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O491" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P491" s="2" t="inlineStr"/>
+      <c r="Q491" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R491" s="2" t="inlineStr"/>
+      <c r="S491" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="2" t="inlineStr">
+        <is>
+          <t>Stefanos Tsitsipas</t>
+        </is>
+      </c>
+      <c r="B492" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C492" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Stefanos Tsitsipas Yellow #29 275/275</t>
+        </is>
+      </c>
+      <c r="D492" s="2" t="inlineStr">
+        <is>
+          <t>275/275</t>
+        </is>
+      </c>
+      <c r="E492" s="2" t="inlineStr">
+        <is>
+          <t>last of 275 (275/275)</t>
+        </is>
+      </c>
+      <c r="F492" s="2" t="inlineStr">
+        <is>
+          <t>10.00 USD</t>
+        </is>
+      </c>
+      <c r="G492" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/820190313050</t>
+        </is>
+      </c>
+      <c r="H492" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I492" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/IbAAAeSwdaZqvT4M/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J492" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T16:52:47.000Z</t>
+        </is>
+      </c>
+      <c r="K492" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L492" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M492" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N492" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/6N4AAeSwLuRqvT35/s-l1600.jpg | https://i.ebayimg.com/images/g/320AAeSw6fBqvT39/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O492" s="2" t="inlineStr">
+        <is>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="P492" s="2" t="inlineStr"/>
+      <c r="Q492" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R492" s="2" t="inlineStr"/>
+      <c r="S492" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="2" t="inlineStr">
+        <is>
+          <t>Taylor Fritz</t>
+        </is>
+      </c>
+      <c r="B493" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps</t>
+        </is>
+      </c>
+      <c r="C493" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Taylor Fritz RC Triumph Relic Gold Auto 1/10 PSA 9 POP 2 💎</t>
+        </is>
+      </c>
+      <c r="D493" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E493" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F493" s="2" t="inlineStr">
+        <is>
+          <t>699.00 USD</t>
+        </is>
+      </c>
+      <c r="G493" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/198678402346?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2FZ%2Fd%2BS4Ws4IgpBR77jblxEXDIxQ7%2FywqlUd8Pn2pYhnoH60Ycw0ux20AS%2BaRloY4OEftYP4M3KqQJCqMMfGHqegKvlB20MwwqfPUotdXe%2Fo2MIuSchmIj8nJyoEDF0Xy0P6OddBYuhJrHEKsqWPpHryRkuSFq%2Fms1KPdPmawhEnk687%2BMP%2FRhlV08BH3Tkxfk%3D</t>
+        </is>
+      </c>
+      <c r="H493" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:42 UTC</t>
+        </is>
+      </c>
+      <c r="I493" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jHgAAeSwH99qvUin/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J493" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T17:37:38.000Z</t>
+        </is>
+      </c>
+      <c r="K493" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L493" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M493" s="2" t="inlineStr">
+        <is>
+          <t>PSA 9</t>
+        </is>
+      </c>
+      <c r="N493" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gycAAeSwHk9qvUin/s-l1600.jpg | https://i.ebayimg.com/images/g/IVgAAeSwA8xqvUin/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O493" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P493" s="2" t="inlineStr"/>
+      <c r="Q493" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R493" s="2" t="inlineStr"/>
+      <c r="S493" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -41301,6 +43935,36 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G461" r:id="rId460"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G462" r:id="rId461"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G463" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G464" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G465" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G466" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G467" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G468" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G469" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G470" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G471" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G472" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G473" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G474" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G475" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G476" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G477" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G478" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G479" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G480" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G481" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G482" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G483" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G484" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G485" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G486" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G487" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G488" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G489" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G490" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G491" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G492" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G493" r:id="rId492"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-01 16:38 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S493"/>
+  <dimension ref="A1:S522"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -43466,6 +43466,2547 @@
       </c>
       <c r="R493" s="2" t="inlineStr"/>
       <c r="S493" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="2" t="inlineStr">
+        <is>
+          <t>Diana Shnaider</t>
+        </is>
+      </c>
+      <c r="B494" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C494" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Diana Schnaider Frozen Fractor -1/0 FrozenFractor</t>
+        </is>
+      </c>
+      <c r="D494" s="2" t="inlineStr">
+        <is>
+          <t>1/0</t>
+        </is>
+      </c>
+      <c r="E494" s="2" t="inlineStr">
+        <is>
+          <t>001 of 0</t>
+        </is>
+      </c>
+      <c r="F494" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G494" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298724141773</t>
+        </is>
+      </c>
+      <c r="H494" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I494" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/EC4AAeSwTLBqvlxP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J494" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T16:07:00.000Z</t>
+        </is>
+      </c>
+      <c r="K494" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L494" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M494" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA)</t>
+        </is>
+      </c>
+      <c r="N494" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YRgAAeSwFJ9qvlxN/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O494" s="2" t="inlineStr"/>
+      <c r="P494" s="2" t="inlineStr"/>
+      <c r="Q494" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R494" s="2" t="inlineStr"/>
+      <c r="S494" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="2" t="inlineStr">
+        <is>
+          <t>Maria Sharapova</t>
+        </is>
+      </c>
+      <c r="B495" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C495" s="2" t="inlineStr">
+        <is>
+          <t>Maria Sharapova 2026 Topps Chrome ON-CARD Auto #25/25 World Number 1 Autograph</t>
+        </is>
+      </c>
+      <c r="D495" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E495" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F495" s="2" t="inlineStr">
+        <is>
+          <t>544.00 USD</t>
+        </is>
+      </c>
+      <c r="G495" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/327383137016</t>
+        </is>
+      </c>
+      <c r="H495" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I495" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HxEAAeSwWAZqvnpO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J495" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T15:23:00.000Z</t>
+        </is>
+      </c>
+      <c r="K495" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L495" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M495" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N495" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~ogAAeSwihBqvnpb/s-l1600.jpg | https://i.ebayimg.com/images/g/wscAAeSw6xhqvnpq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O495" s="2" t="inlineStr"/>
+      <c r="P495" s="2" t="inlineStr"/>
+      <c r="Q495" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R495" s="2" t="inlineStr"/>
+      <c r="S495" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="2" t="inlineStr">
+        <is>
+          <t>Marcos Giron</t>
+        </is>
+      </c>
+      <c r="B496" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C496" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis MARCOS GIRON #104 Red Geometric Refractor 1/5 First!</t>
+        </is>
+      </c>
+      <c r="D496" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E496" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F496" s="2" t="inlineStr">
+        <is>
+          <t>49.99 USD</t>
+        </is>
+      </c>
+      <c r="G496" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298724190182</t>
+        </is>
+      </c>
+      <c r="H496" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I496" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8J8AAeSwsQBqvnf2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J496" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T15:12:39.000Z</t>
+        </is>
+      </c>
+      <c r="K496" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L496" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M496" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N496" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/X98AAeSwgRpqvnf2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O496" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P496" s="2" t="inlineStr"/>
+      <c r="Q496" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R496" s="2" t="inlineStr"/>
+      <c r="S496" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" s="2" t="inlineStr">
+        <is>
+          <t>Valentin Vacherot</t>
+        </is>
+      </c>
+      <c r="B497" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C497" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis VALENTIN VACHEROT GOLD Geometric Refractor 1/50 1/1</t>
+        </is>
+      </c>
+      <c r="D497" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E497" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F497" s="2" t="inlineStr">
+        <is>
+          <t>39.99 USD</t>
+        </is>
+      </c>
+      <c r="G497" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298724135204</t>
+        </is>
+      </c>
+      <c r="H497" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I497" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/GyAAAeSwjjZqvnKZ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J497" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T14:50:44.000Z</t>
+        </is>
+      </c>
+      <c r="K497" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L497" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M497" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N497" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/AYwAAeSwi0lqvnKZ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O497" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P497" s="2" t="inlineStr"/>
+      <c r="Q497" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R497" s="2" t="inlineStr"/>
+      <c r="S497" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="2" t="inlineStr">
+        <is>
+          <t>Jim Courier</t>
+        </is>
+      </c>
+      <c r="B498" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C498" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis JIM COURIER #144 Purple Geometric Refractor 1/75 1/1</t>
+        </is>
+      </c>
+      <c r="D498" s="2" t="inlineStr">
+        <is>
+          <t>1/75</t>
+        </is>
+      </c>
+      <c r="E498" s="2" t="inlineStr">
+        <is>
+          <t>001 of 75</t>
+        </is>
+      </c>
+      <c r="F498" s="2" t="inlineStr">
+        <is>
+          <t>19.99 USD</t>
+        </is>
+      </c>
+      <c r="G498" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307208874926</t>
+        </is>
+      </c>
+      <c r="H498" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I498" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/s3YAAeSwiVpqvm5~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J498" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T14:32:01.000Z</t>
+        </is>
+      </c>
+      <c r="K498" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L498" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M498" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N498" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/CXkAAeSwok1qvm5-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O498" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P498" s="2" t="inlineStr"/>
+      <c r="Q498" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R498" s="2" t="inlineStr"/>
+      <c r="S498" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="2" t="inlineStr">
+        <is>
+          <t>Tallon Griekspoor</t>
+        </is>
+      </c>
+      <c r="B499" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C499" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Topps Chrome Tennis 2026 Tallon Griekspoor Superfractor #106 1/1 </t>
+        </is>
+      </c>
+      <c r="D499" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E499" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F499" s="2" t="inlineStr">
+        <is>
+          <t>500.00 USD</t>
+        </is>
+      </c>
+      <c r="G499" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/206595133421</t>
+        </is>
+      </c>
+      <c r="H499" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I499" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/LoMAAeSwASdqvmk5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J499" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T14:08:21.000Z</t>
+        </is>
+      </c>
+      <c r="K499" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L499" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M499" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N499" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/o58AAeSwq-Jqvmj6/s-l1600.jpg | https://i.ebayimg.com/images/g/4PUAAeSw4mRqvmj6/s-l1600.jpg | https://i.ebayimg.com/images/g/rB0AAeSwXUBqvmj6/s-l1600.jpg | https://i.ebayimg.com/images/g/PIkAAeSwxCtqvmj7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O499" s="2" t="inlineStr"/>
+      <c r="P499" s="2" t="inlineStr"/>
+      <c r="Q499" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R499" s="2" t="inlineStr"/>
+      <c r="S499" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="2" t="inlineStr">
+        <is>
+          <t>Taylah Preston</t>
+        </is>
+      </c>
+      <c r="B500" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - [Base] - Aqua Refractor</t>
+        </is>
+      </c>
+      <c r="C500" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Aqua Refractor 199/199 Taylah Preston #187 1l2l</t>
+        </is>
+      </c>
+      <c r="D500" s="2" t="inlineStr">
+        <is>
+          <t>199/199</t>
+        </is>
+      </c>
+      <c r="E500" s="2" t="inlineStr">
+        <is>
+          <t>last of 199 (199/199)</t>
+        </is>
+      </c>
+      <c r="F500" s="2" t="inlineStr">
+        <is>
+          <t>3.13 USD</t>
+        </is>
+      </c>
+      <c r="G500" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257776454635</t>
+        </is>
+      </c>
+      <c r="H500" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I500" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/i2IAAeSw-wtqvlvq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J500" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T13:09:55.000Z</t>
+        </is>
+      </c>
+      <c r="K500" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L500" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M500" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N500" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/AqUAAeSwesVqvlvq/s-l1600.jpg | https://i.ebayimg.com/images/g/lzQAAeSwrz1qvlvq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O500" s="2" t="inlineStr">
+        <is>
+          <t>aqua</t>
+        </is>
+      </c>
+      <c r="P500" s="2" t="inlineStr"/>
+      <c r="Q500" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R500" s="2" t="inlineStr"/>
+      <c r="S500" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" s="2" t="inlineStr">
+        <is>
+          <t>Matteo Gigante</t>
+        </is>
+      </c>
+      <c r="B501" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C501" s="2" t="inlineStr">
+        <is>
+          <t>Matteo Gigante 2026 Topps Chrome Tennis PURPLE REFRACTOR Card #115 1/75</t>
+        </is>
+      </c>
+      <c r="D501" s="2" t="inlineStr">
+        <is>
+          <t>1/75</t>
+        </is>
+      </c>
+      <c r="E501" s="2" t="inlineStr">
+        <is>
+          <t>001 of 75</t>
+        </is>
+      </c>
+      <c r="F501" s="2" t="inlineStr">
+        <is>
+          <t>19.99 USD</t>
+        </is>
+      </c>
+      <c r="G501" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237100270805?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2Bm%2Bp4nNp6tqjfrcr2YRRGXQWA1s6DDQto1ch9NYykp2xZli1Xw5VwxBUOKwBTYfKiNyjedp0d0Vysv%2BFuuLUbglwRbzkBWOTD0TD0djF4VrLKpPlCYd769DNm4iYzbFHb8EkE4FmiumYPs3EPUW5z1wlcwa4xoUQrhaJ3tJFBxtHCdtb5KtsrB2PxmQx6cN%2FY%3D</t>
+        </is>
+      </c>
+      <c r="H501" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I501" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ZSAAAeSwzF9qvkCp/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J501" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T11:13:44.000Z</t>
+        </is>
+      </c>
+      <c r="K501" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L501" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M501" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N501" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-S4AAeSwcWhqvkCq/s-l1600.jpg | https://i.ebayimg.com/images/g/iygAAeSwSihqvkCr/s-l1600.jpg | https://i.ebayimg.com/images/g/bawAAeSwm~FqvkCq/s-l1600.jpg | https://i.ebayimg.com/images/g/n1sAAeSwt~tqvkCr/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O501" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P501" s="2" t="inlineStr"/>
+      <c r="Q501" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R501" s="2" t="inlineStr"/>
+      <c r="S501" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" s="2" t="inlineStr">
+        <is>
+          <t>Michael Mmoh</t>
+        </is>
+      </c>
+      <c r="B502" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C502" s="2" t="inlineStr">
+        <is>
+          <t>Michael Mmoh 2025 Topps Chrome Sapphire Tennis Padparadscha Refractor Auto 1/1</t>
+        </is>
+      </c>
+      <c r="D502" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E502" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F502" s="2" t="inlineStr">
+        <is>
+          <t>699.99 USD</t>
+        </is>
+      </c>
+      <c r="G502" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336822101655</t>
+        </is>
+      </c>
+      <c r="H502" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I502" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SigAAeSwS8Jqvjia/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J502" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T10:51:18.000Z</t>
+        </is>
+      </c>
+      <c r="K502" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L502" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M502" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N502" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KHsAAeSwtChqvjia/s-l1600.jpg | https://i.ebayimg.com/images/g/SRQAAeSwnBlqvjia/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O502" s="2" t="inlineStr"/>
+      <c r="P502" s="2" t="inlineStr"/>
+      <c r="Q502" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R502" s="2" t="inlineStr"/>
+      <c r="S502" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="2" t="inlineStr">
+        <is>
+          <t>Dusan Lajovic</t>
+        </is>
+      </c>
+      <c r="B503" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 TOPPS CHROME SAPPHIRE EDITION TENNIS</t>
+        </is>
+      </c>
+      <c r="C503" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME SAPPHIRE EDITION TENNIS #99 DUSAN LAJOVIC 1/1 PSA 9</t>
+        </is>
+      </c>
+      <c r="D503" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E503" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F503" s="2" t="inlineStr">
+        <is>
+          <t>799.00 USD</t>
+        </is>
+      </c>
+      <c r="G503" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298723558595</t>
+        </is>
+      </c>
+      <c r="H503" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I503" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ANUAAeSwjnBqvjpF/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J503" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T10:46:31.000Z</t>
+        </is>
+      </c>
+      <c r="K503" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L503" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M503" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N503" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/6SYAAeSw1uFqvjpF/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O503" s="2" t="inlineStr"/>
+      <c r="P503" s="2" t="inlineStr"/>
+      <c r="Q503" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R503" s="2" t="inlineStr"/>
+      <c r="S503" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Nadal</t>
+        </is>
+      </c>
+      <c r="B504" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C504" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Rafael Nadal Geometric Purple Refractor 75/75 Bookend</t>
+        </is>
+      </c>
+      <c r="D504" s="2" t="inlineStr">
+        <is>
+          <t>75/75</t>
+        </is>
+      </c>
+      <c r="E504" s="2" t="inlineStr">
+        <is>
+          <t>last of 75 (75/75)</t>
+        </is>
+      </c>
+      <c r="F504" s="2" t="inlineStr">
+        <is>
+          <t>450.00 USD</t>
+        </is>
+      </c>
+      <c r="G504" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/158373750268</t>
+        </is>
+      </c>
+      <c r="H504" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I504" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ng8AAeSwzJpqviYu/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J504" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T09:26:33.000Z</t>
+        </is>
+      </c>
+      <c r="K504" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L504" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M504" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N504" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/A~cAAeSwjvhqviYU/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O504" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P504" s="2" t="inlineStr"/>
+      <c r="Q504" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R504" s="2" t="inlineStr"/>
+      <c r="S504" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="2" t="inlineStr">
+        <is>
+          <t>Clara Tauson</t>
+        </is>
+      </c>
+      <c r="B505" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C505" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2026 Chrome Tennis Clara Tauson Frozen Fractor -1/0</t>
+        </is>
+      </c>
+      <c r="D505" s="2" t="inlineStr">
+        <is>
+          <t>1/0</t>
+        </is>
+      </c>
+      <c r="E505" s="2" t="inlineStr">
+        <is>
+          <t>001 of 0</t>
+        </is>
+      </c>
+      <c r="F505" s="2" t="inlineStr">
+        <is>
+          <t>1000.00 USD</t>
+        </is>
+      </c>
+      <c r="G505" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/206594338547?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2F5XxX1Clz6vkiJWdoL79V9BwY3ZT%2FGvmCmx489RvYvuu%2BrN8uJHdNP3IDMe%2BvjPsHY1cdMhxmh5CQBP963%2B4U93JEIUC8MjSXfMbrJHShfHN5dpqrhI7LA2ZpvmRGcSD%2FW6p%2FinLMb8bB1sjKmukYI%2BmvAhmQ%2F2JV2tv0s%2F95b%2BX9Drh5UKHHCJpwXBIbLCG8%3D</t>
+        </is>
+      </c>
+      <c r="H505" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I505" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/NmEAAeSwUMdqvfu4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J505" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T06:21:51.000Z</t>
+        </is>
+      </c>
+      <c r="K505" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L505" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M505" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N505" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/FOIAAeSwutRqvfur/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O505" s="2" t="inlineStr"/>
+      <c r="P505" s="2" t="inlineStr"/>
+      <c r="Q505" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R505" s="2" t="inlineStr"/>
+      <c r="S505" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="2" t="inlineStr">
+        <is>
+          <t>Naomi Osaka</t>
+        </is>
+      </c>
+      <c r="B506" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C506" s="2" t="inlineStr">
+        <is>
+          <t>Naomi Osaka 2026 Topps Chrome Tennis SP Orange Geometric World Number 1 /25</t>
+        </is>
+      </c>
+      <c r="D506" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E506" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F506" s="2" t="inlineStr">
+        <is>
+          <t>119.99 USD</t>
+        </is>
+      </c>
+      <c r="G506" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/206594287521</t>
+        </is>
+      </c>
+      <c r="H506" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I506" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QiAAAeSwFBxqvfJz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J506" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T05:41:45.000Z</t>
+        </is>
+      </c>
+      <c r="K506" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L506" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M506" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N506" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/EwsAAeSwGTNqvfJz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O506" s="2" t="inlineStr"/>
+      <c r="P506" s="2" t="inlineStr"/>
+      <c r="Q506" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R506" s="2" t="inlineStr"/>
+      <c r="S506" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="2" t="inlineStr">
+        <is>
+          <t>Danielle Collins</t>
+        </is>
+      </c>
+      <c r="B507" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C507" s="2" t="inlineStr">
+        <is>
+          <t>Danielle Collins Auto Aces 1/1 Superfractor 2026 Topps Chrome Tennis AA-DC</t>
+        </is>
+      </c>
+      <c r="D507" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E507" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F507" s="2" t="inlineStr">
+        <is>
+          <t>2000.00 USD</t>
+        </is>
+      </c>
+      <c r="G507" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336821814768</t>
+        </is>
+      </c>
+      <c r="H507" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I507" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/u~wAAeSwFJ9qvfCa/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J507" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T05:38:55.000Z</t>
+        </is>
+      </c>
+      <c r="K507" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L507" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M507" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N507" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/BR4AAeSwfndqvfCa/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O507" s="2" t="inlineStr"/>
+      <c r="P507" s="2" t="inlineStr"/>
+      <c r="Q507" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R507" s="2" t="inlineStr"/>
+      <c r="S507" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="2" t="inlineStr">
+        <is>
+          <t>Eva Lys</t>
+        </is>
+      </c>
+      <c r="B508" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C508" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Eva Lys Orange Geometric Refractor #1/25</t>
+        </is>
+      </c>
+      <c r="D508" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E508" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F508" s="2" t="inlineStr">
+        <is>
+          <t>7.50 USD</t>
+        </is>
+      </c>
+      <c r="G508" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366703122460</t>
+        </is>
+      </c>
+      <c r="H508" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I508" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/VEMAAeSw79ZqveOI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J508" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T04:37:42.000Z</t>
+        </is>
+      </c>
+      <c r="K508" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L508" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M508" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N508" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HdsAAeSwAOdqveOI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O508" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P508" s="2" t="inlineStr"/>
+      <c r="Q508" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R508" s="2" t="inlineStr"/>
+      <c r="S508" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="2" t="inlineStr">
+        <is>
+          <t>Joao Fonseca</t>
+        </is>
+      </c>
+      <c r="B509" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Chrome Tennis Destiny Gold Geometric</t>
+        </is>
+      </c>
+      <c r="C509" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Joao Fonseca Destiny Gold Geometric RC 1/50 Refractor</t>
+        </is>
+      </c>
+      <c r="D509" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E509" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F509" s="2" t="inlineStr">
+        <is>
+          <t>449.95 USD</t>
+        </is>
+      </c>
+      <c r="G509" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/327382425551</t>
+        </is>
+      </c>
+      <c r="H509" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I509" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/iLQAAeSwOTVqvd2s/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J509" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T04:13:55.000Z</t>
+        </is>
+      </c>
+      <c r="K509" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L509" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M509" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N509" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0VAAAeSw7tFqvd2s/s-l1600.jpg | https://i.ebayimg.com/images/g/2ogAAeSwamhqvd2s/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O509" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P509" s="2" t="inlineStr"/>
+      <c r="Q509" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R509" s="2" t="inlineStr"/>
+      <c r="S509" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="2" t="inlineStr">
+        <is>
+          <t>Linda Noskova</t>
+        </is>
+      </c>
+      <c r="B510" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C510" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome LINDA NOSKOVA Black 10/10 Refractor Auto #AT-LNA SSP</t>
+        </is>
+      </c>
+      <c r="D510" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E510" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F510" s="2" t="inlineStr">
+        <is>
+          <t>849.95 USD</t>
+        </is>
+      </c>
+      <c r="G510" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/327382409920</t>
+        </is>
+      </c>
+      <c r="H510" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I510" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/rdsAAeSwo29qvdmM/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J510" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T03:56:57.000Z</t>
+        </is>
+      </c>
+      <c r="K510" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L510" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M510" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N510" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/tQcAAeSwO9VqvdmM/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O510" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P510" s="2" t="inlineStr"/>
+      <c r="Q510" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R510" s="2" t="inlineStr"/>
+      <c r="S510" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="2" t="inlineStr">
+        <is>
+          <t>Denis Shapovalov</t>
+        </is>
+      </c>
+      <c r="B511" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C511" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Denis Shapovalov Frozenfractor -1/0</t>
+        </is>
+      </c>
+      <c r="D511" s="2" t="inlineStr">
+        <is>
+          <t>1/0</t>
+        </is>
+      </c>
+      <c r="E511" s="2" t="inlineStr">
+        <is>
+          <t>001 of 0</t>
+        </is>
+      </c>
+      <c r="F511" s="2" t="inlineStr">
+        <is>
+          <t>499.99 USD</t>
+        </is>
+      </c>
+      <c r="G511" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/327382355170</t>
+        </is>
+      </c>
+      <c r="H511" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I511" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TMcAAeSwt-dqvc4~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J511" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T03:08:47.000Z</t>
+        </is>
+      </c>
+      <c r="K511" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L511" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M511" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N511" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JqUAAeSwASdqvc4~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O511" s="2" t="inlineStr"/>
+      <c r="P511" s="2" t="inlineStr"/>
+      <c r="Q511" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R511" s="2" t="inlineStr"/>
+      <c r="S511" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="2" t="inlineStr">
+        <is>
+          <t>Paula Badosa</t>
+        </is>
+      </c>
+      <c r="B512" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C512" s="2" t="inlineStr">
+        <is>
+          <t>1/1!!! Topps chrome 2026 Paula Badosa SuperFractor 1/1!!</t>
+        </is>
+      </c>
+      <c r="D512" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E512" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F512" s="2" t="inlineStr">
+        <is>
+          <t>10000.00 USD</t>
+        </is>
+      </c>
+      <c r="G512" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/800741127380</t>
+        </is>
+      </c>
+      <c r="H512" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I512" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HYEAAeSwkJlqvcml/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J512" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:51:25.000Z</t>
+        </is>
+      </c>
+      <c r="K512" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L512" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M512" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N512" s="2" t="inlineStr"/>
+      <c r="O512" s="2" t="inlineStr"/>
+      <c r="P512" s="2" t="inlineStr"/>
+      <c r="Q512" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R512" s="2" t="inlineStr"/>
+      <c r="S512" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="2" t="inlineStr">
+        <is>
+          <t>Ugo Humbert</t>
+        </is>
+      </c>
+      <c r="B513" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C513" s="2" t="inlineStr">
+        <is>
+          <t>2026 TOPPS CHROME TENNIS UGO HUMBERT BLACK ACES ON CARD AUTO CARD 10/10 SSSP</t>
+        </is>
+      </c>
+      <c r="D513" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E513" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F513" s="2" t="inlineStr">
+        <is>
+          <t>999.99 USD</t>
+        </is>
+      </c>
+      <c r="G513" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/227546894357?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde9qRMrHuOcLd92t3ai7w8Q4GWoZJMtgDXxLTzQc9LMu6zgVXGg%2F7lAkDYUv0UtjN%2F3COoD8Ni1zIrUtEVYOhANTQJh7mqizGq%2FumvJwH3%2FEv0LRhOU%2BlV29Flf%2BbrBdjyBopCy3Qe1ldCmKERLhRAuSZHThro--9qHlKpT%2BEdfUT4Z2ah1RLDUIdeaSPqrxcmo%3D</t>
+        </is>
+      </c>
+      <c r="H513" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I513" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3OwAAeSwASdqvck~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J513" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:45:31.000Z</t>
+        </is>
+      </c>
+      <c r="K513" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L513" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M513" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N513" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3KYAAeSwxclqvclB/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O513" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P513" s="2" t="inlineStr"/>
+      <c r="Q513" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R513" s="2" t="inlineStr"/>
+      <c r="S513" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="2" t="inlineStr">
+        <is>
+          <t>Novak Djokovic</t>
+        </is>
+      </c>
+      <c r="B514" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C514" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Novak Djokovic Green Geometric Auto 99/99</t>
+        </is>
+      </c>
+      <c r="D514" s="2" t="inlineStr">
+        <is>
+          <t>99/99</t>
+        </is>
+      </c>
+      <c r="E514" s="2" t="inlineStr">
+        <is>
+          <t>last of 99 (99/99)</t>
+        </is>
+      </c>
+      <c r="F514" s="2" t="inlineStr">
+        <is>
+          <t>1299.00 USD</t>
+        </is>
+      </c>
+      <c r="G514" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407258439203</t>
+        </is>
+      </c>
+      <c r="H514" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I514" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QH8AAeSwK7lqvchr/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J514" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:43:32.000Z</t>
+        </is>
+      </c>
+      <c r="K514" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L514" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M514" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA)</t>
+        </is>
+      </c>
+      <c r="N514" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7mUAAeSwoWtqvchs/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O514" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P514" s="2" t="inlineStr"/>
+      <c r="Q514" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R514" s="2" t="inlineStr"/>
+      <c r="S514" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="2" t="inlineStr">
+        <is>
+          <t>Benoit Paire</t>
+        </is>
+      </c>
+      <c r="B515" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C515" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Benoit Paire #178 BLACK Wave Refractor Bookend 10/10</t>
+        </is>
+      </c>
+      <c r="D515" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E515" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F515" s="2" t="inlineStr">
+        <is>
+          <t>24.00 USD</t>
+        </is>
+      </c>
+      <c r="G515" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298722561152?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde92VXMfCHR%2BdSI4ueDagAPOIf48R1H62E3bJNF1IiL05BSBNDyn7GLYbMPx7AsAStzZWicMVpOXPT6HfX7ouYYgUcJ5%2FUwevaoUHDfg109MRBWRHMj03A8y2FPupcjFlmvF80Tua%2FoVfPWZkSFdclUybDoMnduVi3DL4fagpkrd3hKO9mp3MFhp7WvC5%2BRwCN0%3D</t>
+        </is>
+      </c>
+      <c r="H515" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I515" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/luYAAeSwo29qvcSN/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J515" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:27:37.000Z</t>
+        </is>
+      </c>
+      <c r="K515" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L515" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M515" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N515" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/FQ8AAeSwihBqvcSN/s-l1600.jpg | https://i.ebayimg.com/images/g/7asAAeSwN89qvcSM/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O515" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P515" s="2" t="inlineStr"/>
+      <c r="Q515" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R515" s="2" t="inlineStr"/>
+      <c r="S515" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="2" t="inlineStr">
+        <is>
+          <t>Ben Shelton</t>
+        </is>
+      </c>
+      <c r="B516" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite Tennis</t>
+        </is>
+      </c>
+      <c r="C516" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Tennis #16 Red Crystalline Refractor Ben Shelton 1/1</t>
+        </is>
+      </c>
+      <c r="D516" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E516" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F516" s="2" t="inlineStr">
+        <is>
+          <t>6500.00 USD</t>
+        </is>
+      </c>
+      <c r="G516" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/327383157663?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8duoRltVuuC8dOCWFj76KhitY4dTOfkIHMFlVKr9h8JdI10YRWQTsCs8ExOQ4XQGweGNgnj2cqKR2N5iDvBWSQN%2BdV9kzhfQEyhrnfqtYjrFEnINMOw%2BRA%2BjNjOQifmL5DbXM%2B0wO9r9faVL4FBQT9tx4oyZls5SL7c3aPxvr30hoWi%2Fw7yBCamODyb%2BOjAOQ%3D</t>
+        </is>
+      </c>
+      <c r="H516" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I516" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/LUYAAeSwy6Rqvn00/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J516" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T15:36:34.000Z</t>
+        </is>
+      </c>
+      <c r="K516" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L516" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M516" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N516" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-rYAAeSwtjZqvn00/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O516" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P516" s="2" t="inlineStr"/>
+      <c r="Q516" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R516" s="2" t="inlineStr"/>
+      <c r="S516" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="2" t="inlineStr">
+        <is>
+          <t>Liv Hovde</t>
+        </is>
+      </c>
+      <c r="B517" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C517" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Liv Hovde Signature Relics Pink #01/15!</t>
+        </is>
+      </c>
+      <c r="D517" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E517" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F517" s="2" t="inlineStr">
+        <is>
+          <t>49.99 USD</t>
+        </is>
+      </c>
+      <c r="G517" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178544295161</t>
+        </is>
+      </c>
+      <c r="H517" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I517" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/LEMAAeSw3JBqvgc4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J517" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T07:12:37.000Z</t>
+        </is>
+      </c>
+      <c r="K517" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L517" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M517" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N517" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/R1YAAeSwmwpqvgdA/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O517" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P517" s="2" t="inlineStr"/>
+      <c r="Q517" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R517" s="2" t="inlineStr"/>
+      <c r="S517" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="2" t="inlineStr">
+        <is>
+          <t>Ben Shelton</t>
+        </is>
+      </c>
+      <c r="B518" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Graphite</t>
+        </is>
+      </c>
+      <c r="C518" s="2" t="inlineStr">
+        <is>
+          <t>Ben Shelton 2024 Topps Graphite Gold Refractor 25/25 #125 RC</t>
+        </is>
+      </c>
+      <c r="D518" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E518" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F518" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G518" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237097814808</t>
+        </is>
+      </c>
+      <c r="H518" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I518" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/K34AAeSwkJlqvFIz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J518" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T01:46:00.000Z</t>
+        </is>
+      </c>
+      <c r="K518" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L518" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M518" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N518" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TN4AAeSw60pqvFIz/s-l1600.jpg | https://i.ebayimg.com/images/g/LBcAAeSw8tlqvFIz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O518" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P518" s="2" t="inlineStr"/>
+      <c r="Q518" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R518" s="2" t="inlineStr"/>
+      <c r="S518" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" s="2" t="inlineStr">
+        <is>
+          <t>Steffi Graf</t>
+        </is>
+      </c>
+      <c r="B519" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Graphite</t>
+        </is>
+      </c>
+      <c r="C519" s="2" t="inlineStr">
+        <is>
+          <t>Steffi Graf 2024 Topps Graphite Pink Refractor 1/15 Winning Streaks #WS-SG</t>
+        </is>
+      </c>
+      <c r="D519" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E519" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F519" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G519" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237097814642</t>
+        </is>
+      </c>
+      <c r="H519" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I519" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/LsIAAeSwbHBqvFIv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J519" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T00:57:00.000Z</t>
+        </is>
+      </c>
+      <c r="K519" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L519" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M519" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N519" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/MkQAAeSwm~FqvFIv/s-l1600.jpg | https://i.ebayimg.com/images/g/MD4AAeSwPjJqvFIv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O519" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P519" s="2" t="inlineStr"/>
+      <c r="Q519" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R519" s="2" t="inlineStr"/>
+      <c r="S519" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek</t>
+        </is>
+      </c>
+      <c r="B520" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS ROYALTY TENNIS AMBASSADOR AUTOGRAPHS</t>
+        </is>
+      </c>
+      <c r="C520" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS ROYALTY TENNIS AMBASSADOR AUTOS BLUE #AAIS IGA SWIATEK 1/25 PSA 9</t>
+        </is>
+      </c>
+      <c r="D520" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E520" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F520" s="2" t="inlineStr">
+        <is>
+          <t>5000.00 USD</t>
+        </is>
+      </c>
+      <c r="G520" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307208652717</t>
+        </is>
+      </c>
+      <c r="H520" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I520" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/dSIAAeSwWwhqvkyC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J520" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T12:04:17.000Z</t>
+        </is>
+      </c>
+      <c r="K520" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L520" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M520" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N520" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ejcAAeSwbAVqvkyC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O520" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P520" s="2" t="inlineStr"/>
+      <c r="Q520" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R520" s="2" t="inlineStr"/>
+      <c r="S520" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" s="2" t="inlineStr">
+        <is>
+          <t>Lindsay Davenport</t>
+        </is>
+      </c>
+      <c r="B521" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Royalty Collection</t>
+        </is>
+      </c>
+      <c r="C521" s="2" t="inlineStr">
+        <is>
+          <t>Lindsay Davenport 2024 Royalty Purple 35/35 #87</t>
+        </is>
+      </c>
+      <c r="D521" s="2" t="inlineStr">
+        <is>
+          <t>35/35</t>
+        </is>
+      </c>
+      <c r="E521" s="2" t="inlineStr">
+        <is>
+          <t>last of 35 (35/35)</t>
+        </is>
+      </c>
+      <c r="F521" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G521" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237097814645</t>
+        </is>
+      </c>
+      <c r="H521" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I521" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/LuAAAeSwkixqvFIl/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J521" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T01:06:00.000Z</t>
+        </is>
+      </c>
+      <c r="K521" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L521" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M521" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N521" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/wPEAAeSwH99qvFIl/s-l1600.jpg | https://i.ebayimg.com/images/g/MHwAAeSwfKVqvFIl/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O521" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P521" s="2" t="inlineStr"/>
+      <c r="Q521" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R521" s="2" t="inlineStr"/>
+      <c r="S521" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="2" t="inlineStr">
+        <is>
+          <t>Roger Federer</t>
+        </is>
+      </c>
+      <c r="B522" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic</t>
+        </is>
+      </c>
+      <c r="C522" s="2" t="inlineStr">
+        <is>
+          <t>2008 Ace G/S II US Open Mem Dual Mat Gold #15 1/5 Federer/Berankis PSA 8 Top Pop</t>
+        </is>
+      </c>
+      <c r="D522" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E522" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F522" s="2" t="inlineStr">
+        <is>
+          <t>600.00 USD</t>
+        </is>
+      </c>
+      <c r="G522" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168747448895</t>
+        </is>
+      </c>
+      <c r="H522" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:37 UTC</t>
+        </is>
+      </c>
+      <c r="I522" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ceAAAOSwm0liwM3K/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J522" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T00:28:42.000Z</t>
+        </is>
+      </c>
+      <c r="K522" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L522" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M522" s="2" t="inlineStr">
+        <is>
+          <t>PSA 8</t>
+        </is>
+      </c>
+      <c r="N522" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Oy4AAOSwn29iwM3T/s-l1600.jpg | https://i.ebayimg.com/images/g/9JYAAOSw4ApiwM3e/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O522" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P522" s="2" t="inlineStr"/>
+      <c r="Q522" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R522" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic: check the numbering is stamped, not on a circle sticker</t>
+        </is>
+      </c>
+      <c r="S522" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -43965,6 +46506,35 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G491" r:id="rId490"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G492" r:id="rId491"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G493" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G494" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G495" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G496" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G497" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G498" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G499" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G500" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G501" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G502" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G503" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G504" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G505" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G506" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G507" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G508" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G509" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G510" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G511" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G512" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G513" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G514" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G515" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G516" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G517" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G518" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G519" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G520" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G521" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G522" r:id="rId521"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-02 14:15 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S522"/>
+  <dimension ref="A1:S541"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -46007,6 +46007,1665 @@
         </is>
       </c>
       <c r="S522" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B523" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite Tennis</t>
+        </is>
+      </c>
+      <c r="C523" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff-2026 Topps Graphite Tour Relic Auto Gold SSP #01/25-Game Used🔥🔥</t>
+        </is>
+      </c>
+      <c r="D523" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E523" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F523" s="2" t="inlineStr">
+        <is>
+          <t>299.00 USD</t>
+        </is>
+      </c>
+      <c r="G523" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168748202753</t>
+        </is>
+      </c>
+      <c r="H523" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:13 UTC</t>
+        </is>
+      </c>
+      <c r="I523" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Gx0AAeSwhthqnQDm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J523" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T06:00:39.000Z</t>
+        </is>
+      </c>
+      <c r="K523" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L523" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M523" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N523" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/q-sAAeSwG9FqnQDm/s-l1600.jpg | https://i.ebayimg.com/images/g/ZsgAAeSwhFRqnQDm/s-l1600.jpg | https://i.ebayimg.com/images/g/q7gAAeSwmElqnQDm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O523" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P523" s="2" t="inlineStr"/>
+      <c r="Q523" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R523" s="2" t="inlineStr"/>
+      <c r="S523" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B524" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Tennis</t>
+        </is>
+      </c>
+      <c r="C524" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis Swiatek Sabalenka Gauff Triple On Card Auto 1/1</t>
+        </is>
+      </c>
+      <c r="D524" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E524" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F524" s="2" t="inlineStr">
+        <is>
+          <t>50000.00 USD</t>
+        </is>
+      </c>
+      <c r="G524" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/146615439732</t>
+        </is>
+      </c>
+      <c r="H524" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:13 UTC</t>
+        </is>
+      </c>
+      <c r="I524" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/BooAAOSwNZ5oOaRD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J524" s="2" t="inlineStr">
+        <is>
+          <t>2025-05-30T12:28:34.000Z</t>
+        </is>
+      </c>
+      <c r="K524" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L524" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M524" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N524" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/baEAAOSwoJ5oOaRD/s-l1600.jpg | https://i.ebayimg.com/images/g/L48AAOSwBx1oOaRD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O524" s="2" t="inlineStr"/>
+      <c r="P524" s="2" t="inlineStr"/>
+      <c r="Q524" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R524" s="2" t="inlineStr"/>
+      <c r="S524" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B525" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Tennis</t>
+        </is>
+      </c>
+      <c r="C525" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis Coco Gauff 5/5 Relic Jewles Patch Match Worn</t>
+        </is>
+      </c>
+      <c r="D525" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E525" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F525" s="2" t="inlineStr">
+        <is>
+          <t>600.00 USD</t>
+        </is>
+      </c>
+      <c r="G525" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/146585101826?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde9HCUgSK7lIhRp3lCTHePxuS1N7k3duiMzNbxB1uBYaGYD8IvH9Up%2F7H0%2BiK5teaxc01IaXO1h0bFllN7MRJcAQWIur6Wesr%2BvmpxkPS6o%2FEet0PBtZtjLEgP7QMutnUXFh5ocW1Emhe55Jk7X4wj1HK0mbe0qQ8kgt0qZX7dFjI9C7pcctIuj%2Br2pmfUePKys%3D</t>
+        </is>
+      </c>
+      <c r="H525" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:13 UTC</t>
+        </is>
+      </c>
+      <c r="I525" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/BxEAAOSwAkRoJoqk/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J525" s="2" t="inlineStr">
+        <is>
+          <t>2025-05-16T00:45:52.000Z</t>
+        </is>
+      </c>
+      <c r="K525" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L525" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M525" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N525" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/dVAAAOSwCkZoJoqg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O525" s="2" t="inlineStr"/>
+      <c r="P525" s="2" t="inlineStr"/>
+      <c r="Q525" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R525" s="2" t="inlineStr"/>
+      <c r="S525" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B526" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis Tennis</t>
+        </is>
+      </c>
+      <c r="C526" s="2" t="inlineStr">
+        <is>
+          <t>CARLOS ALCARAZ 2026 TOPPS CHROME DESTINY BLACK GEOMETRIC 10/10 #DTY-ALC Q7656</t>
+        </is>
+      </c>
+      <c r="D526" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E526" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F526" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G526" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/278427015374</t>
+        </is>
+      </c>
+      <c r="H526" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:13 UTC</t>
+        </is>
+      </c>
+      <c r="I526" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/EaIAAeSwpM9qvuUb/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J526" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T01:51:00.000Z</t>
+        </is>
+      </c>
+      <c r="K526" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L526" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M526" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N526" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/c30AAeSwU8xqvuUc/s-l1600.jpg | https://i.ebayimg.com/images/g/UskAAeSwxclqvuUb/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O526" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P526" s="2" t="inlineStr"/>
+      <c r="Q526" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R526" s="2" t="inlineStr"/>
+      <c r="S526" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B527" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C527" s="2" t="inlineStr">
+        <is>
+          <t>CARLOS ALCARAZ 2026 TOPPS CHROME TENNIS ORANGE GEOMETRIC 25/25 #50 Q7656</t>
+        </is>
+      </c>
+      <c r="D527" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E527" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F527" s="2" t="inlineStr">
+        <is>
+          <t>4.25 USD</t>
+        </is>
+      </c>
+      <c r="G527" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/278426851487</t>
+        </is>
+      </c>
+      <c r="H527" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:13 UTC</t>
+        </is>
+      </c>
+      <c r="I527" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QCYAAeSwAUNqvtHq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J527" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T00:15:00.000Z</t>
+        </is>
+      </c>
+      <c r="K527" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L527" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M527" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N527" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Oy0AAeSwFY5qvtHq/s-l1600.jpg | https://i.ebayimg.com/images/g/SBkAAeSwxn9qvtHq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O527" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P527" s="2" t="inlineStr"/>
+      <c r="Q527" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R527" s="2" t="inlineStr"/>
+      <c r="S527" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B528" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C528" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz 2026 Topps Chrome Tennis World Number 1 Red Geometric 1/5 #WNO-CA</t>
+        </is>
+      </c>
+      <c r="D528" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E528" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F528" s="2" t="inlineStr">
+        <is>
+          <t>3499.99 USD</t>
+        </is>
+      </c>
+      <c r="G528" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/189021348458</t>
+        </is>
+      </c>
+      <c r="H528" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:13 UTC</t>
+        </is>
+      </c>
+      <c r="I528" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bSkAAeSwmP5qvahe/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J528" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T00:26:49.000Z</t>
+        </is>
+      </c>
+      <c r="K528" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L528" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M528" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N528" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XSkAAeSw8wtqvahe/s-l1600.jpg | https://i.ebayimg.com/images/g/Tw0AAeSwLbBqvahd/s-l1600.jpg | https://i.ebayimg.com/images/g/Yo4AAeSwVABqvahd/s-l1600.jpg | https://i.ebayimg.com/images/g/RtIAAeSw~yNqvahe/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O528" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P528" s="2" t="inlineStr"/>
+      <c r="Q528" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R528" s="2" t="inlineStr"/>
+      <c r="S528" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B529" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C529" s="2" t="inlineStr">
+        <is>
+          <t>Topps Chrome 2026 Tennis Carlos Alcaraz World No. 1 /150 Insert WNO-CA</t>
+        </is>
+      </c>
+      <c r="D529" s="2" t="inlineStr">
+        <is>
+          <t>1/150</t>
+        </is>
+      </c>
+      <c r="E529" s="2" t="inlineStr">
+        <is>
+          <t>001 of 150</t>
+        </is>
+      </c>
+      <c r="F529" s="2" t="inlineStr">
+        <is>
+          <t>200.00 USD</t>
+        </is>
+      </c>
+      <c r="G529" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/158372000192</t>
+        </is>
+      </c>
+      <c r="H529" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:13 UTC</t>
+        </is>
+      </c>
+      <c r="I529" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QVkAAeSwgZ1qvafq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J529" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T00:24:21.000Z</t>
+        </is>
+      </c>
+      <c r="K529" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L529" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M529" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N529" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HwwAAeSw-ftqvafY/s-l1600.jpg | https://i.ebayimg.com/images/g/t8IAAeSwtChqvafY/s-l1600.jpg | https://i.ebayimg.com/images/g/tacAAeSwutRqvafY/s-l1600.jpg | https://i.ebayimg.com/images/g/T8AAAeSwZPtqvafY/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O529" s="2" t="inlineStr"/>
+      <c r="P529" s="2" t="inlineStr"/>
+      <c r="Q529" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R529" s="2" t="inlineStr"/>
+      <c r="S529" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" s="2" t="inlineStr">
+        <is>
+          <t>Pete Sampras</t>
+        </is>
+      </c>
+      <c r="B530" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C530" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Pete Sampras World No. 1 Insert WNO-PS 01/10 FIRST CARD</t>
+        </is>
+      </c>
+      <c r="D530" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E530" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F530" s="2" t="inlineStr">
+        <is>
+          <t>500.00 USD</t>
+        </is>
+      </c>
+      <c r="G530" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/128109781429</t>
+        </is>
+      </c>
+      <c r="H530" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:13 UTC</t>
+        </is>
+      </c>
+      <c r="I530" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/chMAAeSw8~lqvs-s/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J530" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T21:22:57.000Z</t>
+        </is>
+      </c>
+      <c r="K530" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L530" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M530" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N530" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/lVQAAeSwSEpqvs6s/s-l1600.jpg | https://i.ebayimg.com/images/g/bcsAAeSw6HJqvs6s/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O530" s="2" t="inlineStr"/>
+      <c r="P530" s="2" t="inlineStr"/>
+      <c r="Q530" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R530" s="2" t="inlineStr"/>
+      <c r="S530" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" s="2" t="inlineStr">
+        <is>
+          <t>Andre Agassi</t>
+        </is>
+      </c>
+      <c r="B531" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Tennis</t>
+        </is>
+      </c>
+      <c r="C531" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis Andre Agassi 1/1 On Card Auto Royal Decree</t>
+        </is>
+      </c>
+      <c r="D531" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E531" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F531" s="2" t="inlineStr">
+        <is>
+          <t>20000.00 USD</t>
+        </is>
+      </c>
+      <c r="G531" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/146605040386?amdata=enc%3AAQALAAAAsCHNgUiiE%2FjQhlDTaMiAde%2BnIJHZn8d%2BQSQsuUuxm7P7wTUecSjc6TTGtdYnv%2Bj6RZMROhD%2BA1X84mnMDcD4%2BfWB4taxtMaNlJSShFVPXvwNcnFsonXTDPSp2jNdNL0oxU%2FSXln4AkVN4X8C6EFIK5E%2FZzN6W1l8Sb59xCUyDAnQ6ZEdaHayhGOUw9EdJV1wMamk4U2KRKyMLsUWf1LGRlJlsnGspZLqF6tl9Pj%2BvPCY</t>
+        </is>
+      </c>
+      <c r="H531" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:13 UTC</t>
+        </is>
+      </c>
+      <c r="I531" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/tUMAAOSwURBoMzWt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J531" s="2" t="inlineStr">
+        <is>
+          <t>2025-05-25T15:23:03.000Z</t>
+        </is>
+      </c>
+      <c r="K531" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L531" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M531" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N531" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/kmkAAOSwD~VoMzWt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O531" s="2" t="inlineStr"/>
+      <c r="P531" s="2" t="inlineStr"/>
+      <c r="Q531" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R531" s="2" t="inlineStr"/>
+      <c r="S531" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Nadal</t>
+        </is>
+      </c>
+      <c r="B532" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C532" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Rafael Nadal World Number 1 Auto 25/25</t>
+        </is>
+      </c>
+      <c r="D532" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E532" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F532" s="2" t="inlineStr">
+        <is>
+          <t>9999.00 USD</t>
+        </is>
+      </c>
+      <c r="G532" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/820194842647</t>
+        </is>
+      </c>
+      <c r="H532" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:14 UTC</t>
+        </is>
+      </c>
+      <c r="I532" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/WaoAAeSwNuFqvxF4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J532" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T02:11:52.000Z</t>
+        </is>
+      </c>
+      <c r="K532" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L532" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M532" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N532" s="2" t="inlineStr"/>
+      <c r="O532" s="2" t="inlineStr"/>
+      <c r="P532" s="2" t="inlineStr"/>
+      <c r="Q532" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R532" s="2" t="inlineStr"/>
+      <c r="S532" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Nadal</t>
+        </is>
+      </c>
+      <c r="B533" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C533" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2026 Chrome Tennis Rafael Nadal GOLD Refractor World No. 1 /50</t>
+        </is>
+      </c>
+      <c r="D533" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E533" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F533" s="2" t="inlineStr">
+        <is>
+          <t>1799.00 USD</t>
+        </is>
+      </c>
+      <c r="G533" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377535034098</t>
+        </is>
+      </c>
+      <c r="H533" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:14 UTC</t>
+        </is>
+      </c>
+      <c r="I533" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/FvsAAeSw3P1qvbZN/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J533" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T01:26:10.000Z</t>
+        </is>
+      </c>
+      <c r="K533" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L533" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M533" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N533" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/CfMAAeSwIVdqvbZS/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O533" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P533" s="2" t="inlineStr"/>
+      <c r="Q533" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R533" s="2" t="inlineStr"/>
+      <c r="S533" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" s="2" t="inlineStr">
+        <is>
+          <t>Martina Hingis</t>
+        </is>
+      </c>
+      <c r="B534" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C534" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis Martina Hingis #152 Rose Gold Refractor #’d 20/20</t>
+        </is>
+      </c>
+      <c r="D534" s="2" t="inlineStr">
+        <is>
+          <t>20/20</t>
+        </is>
+      </c>
+      <c r="E534" s="2" t="inlineStr">
+        <is>
+          <t>last of 20 (20/20)</t>
+        </is>
+      </c>
+      <c r="F534" s="2" t="inlineStr">
+        <is>
+          <t>5.50 USD</t>
+        </is>
+      </c>
+      <c r="G534" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/800730385256</t>
+        </is>
+      </c>
+      <c r="H534" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:14 UTC</t>
+        </is>
+      </c>
+      <c r="I534" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7IEAAeSw~yNqutsj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J534" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T21:25:49.000Z</t>
+        </is>
+      </c>
+      <c r="K534" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L534" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M534" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N534" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/5J0AAeSww8Fqutss/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O534" s="2" t="inlineStr">
+        <is>
+          <t>rose</t>
+        </is>
+      </c>
+      <c r="P534" s="2" t="inlineStr"/>
+      <c r="Q534" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R534" s="2" t="inlineStr"/>
+      <c r="S534" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek</t>
+        </is>
+      </c>
+      <c r="B535" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C535" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis #AO-ISK Iga Swiatek Auto Orange Geometric 01/25</t>
+        </is>
+      </c>
+      <c r="D535" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E535" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F535" s="2" t="inlineStr">
+        <is>
+          <t>599.95 USD</t>
+        </is>
+      </c>
+      <c r="G535" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336822718795</t>
+        </is>
+      </c>
+      <c r="H535" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:14 UTC</t>
+        </is>
+      </c>
+      <c r="I535" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/PGMAAeSwD7VqvSrB/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J535" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T20:43:52.000Z</t>
+        </is>
+      </c>
+      <c r="K535" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L535" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M535" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N535" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~loAAeSweVRqvSrD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O535" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P535" s="2" t="inlineStr"/>
+      <c r="Q535" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R535" s="2" t="inlineStr"/>
+      <c r="S535" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" s="2" t="inlineStr">
+        <is>
+          <t>Qinwen Zheng</t>
+        </is>
+      </c>
+      <c r="B536" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C536" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite - Ace Relics Qinwen Zheng #AR-QZG Gold Refractor 01/25</t>
+        </is>
+      </c>
+      <c r="D536" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E536" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F536" s="2" t="inlineStr">
+        <is>
+          <t>31.00 USD</t>
+        </is>
+      </c>
+      <c r="G536" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287608378402</t>
+        </is>
+      </c>
+      <c r="H536" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:14 UTC</t>
+        </is>
+      </c>
+      <c r="I536" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KaMAAeSwnLRqrXJZ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J536" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T17:41:46.000Z</t>
+        </is>
+      </c>
+      <c r="K536" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L536" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M536" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N536" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/K3gAAeSwYjtqrXJ1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O536" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P536" s="2" t="inlineStr"/>
+      <c r="Q536" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R536" s="2" t="inlineStr"/>
+      <c r="S536" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" s="2" t="inlineStr">
+        <is>
+          <t>Qinwen Zheng</t>
+        </is>
+      </c>
+      <c r="B537" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Tennis</t>
+        </is>
+      </c>
+      <c r="C537" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis Qinwen Zheng 1/1 Regalia Relic Auto Signatures</t>
+        </is>
+      </c>
+      <c r="D537" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E537" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F537" s="2" t="inlineStr">
+        <is>
+          <t>20000.00 USD</t>
+        </is>
+      </c>
+      <c r="G537" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147109451508</t>
+        </is>
+      </c>
+      <c r="H537" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:14 UTC</t>
+        </is>
+      </c>
+      <c r="I537" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ABEAAOSweWFoLiUJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J537" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-22T20:32:50.000Z</t>
+        </is>
+      </c>
+      <c r="K537" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L537" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M537" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N537" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/MHsAAOSwgOxoLiUJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O537" s="2" t="inlineStr"/>
+      <c r="P537" s="2" t="inlineStr"/>
+      <c r="Q537" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R537" s="2" t="inlineStr"/>
+      <c r="S537" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" s="2" t="inlineStr">
+        <is>
+          <t>Steffi Graf</t>
+        </is>
+      </c>
+      <c r="B538" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C538" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Steffi Graf #AO-SGC Geometric Red Auto 1/5 Autograph</t>
+        </is>
+      </c>
+      <c r="D538" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E538" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F538" s="2" t="inlineStr">
+        <is>
+          <t>799.99 USD</t>
+        </is>
+      </c>
+      <c r="G538" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257777115784</t>
+        </is>
+      </c>
+      <c r="H538" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:14 UTC</t>
+        </is>
+      </c>
+      <c r="I538" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2j0AAeSwgRpqvs9d/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J538" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T21:59:27.000Z</t>
+        </is>
+      </c>
+      <c r="K538" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L538" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M538" s="2" t="inlineStr">
+        <is>
+          <t>SGC</t>
+        </is>
+      </c>
+      <c r="N538" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/4bMAAeSww8Zqvs9d/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O538" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P538" s="2" t="inlineStr"/>
+      <c r="Q538" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R538" s="2" t="inlineStr"/>
+      <c r="S538" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" s="2" t="inlineStr">
+        <is>
+          <t>Maria Sharapova</t>
+        </is>
+      </c>
+      <c r="B539" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Sapphire Tennis</t>
+        </is>
+      </c>
+      <c r="C539" s="2" t="inlineStr">
+        <is>
+          <t>MARIA SHARAPOVA 2024 TOPPS CHROME SAPPHIRE TENNIS RED 1/5 #153 PSA 9 Q4263</t>
+        </is>
+      </c>
+      <c r="D539" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E539" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F539" s="2" t="inlineStr">
+        <is>
+          <t>157.50 USD</t>
+        </is>
+      </c>
+      <c r="G539" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/278420055966</t>
+        </is>
+      </c>
+      <c r="H539" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:15 UTC</t>
+        </is>
+      </c>
+      <c r="I539" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9dIAAeSwPolqu7XI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J539" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T01:30:00.000Z</t>
+        </is>
+      </c>
+      <c r="K539" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L539" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M539" s="2" t="inlineStr">
+        <is>
+          <t>PSA 9</t>
+        </is>
+      </c>
+      <c r="N539" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8lMAAeSwEVFqu7XI/s-l1600.jpg | https://i.ebayimg.com/images/g/-VMAAeSw8tlqu7XH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O539" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P539" s="2" t="inlineStr"/>
+      <c r="Q539" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R539" s="2" t="inlineStr"/>
+      <c r="S539" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" s="2" t="inlineStr">
+        <is>
+          <t>Ben Shelton</t>
+        </is>
+      </c>
+      <c r="B540" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C540" s="2" t="inlineStr">
+        <is>
+          <t>Ben Shelton Geometric Red Auto 5 /5 Topps Chrome Tennis 2026</t>
+        </is>
+      </c>
+      <c r="D540" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E540" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F540" s="2" t="inlineStr">
+        <is>
+          <t>2023.92 USD</t>
+        </is>
+      </c>
+      <c r="G540" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298723502704</t>
+        </is>
+      </c>
+      <c r="H540" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:15 UTC</t>
+        </is>
+      </c>
+      <c r="I540" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/z6MAAeSwZe5qvUzn/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J540" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T10:24:14.000Z</t>
+        </is>
+      </c>
+      <c r="K540" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L540" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M540" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N540" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/UFEAAeSwRWxqvUzn/s-l1600.jpg | https://i.ebayimg.com/images/g/v5wAAeSwWMNqvUzn/s-l1600.jpg | https://i.ebayimg.com/images/g/osAAAeSw8NZqvUzn/s-l1600.jpg | https://i.ebayimg.com/images/g/ctoAAeSwG~dqvUzo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O540" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P540" s="2" t="inlineStr"/>
+      <c r="Q540" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R540" s="2" t="inlineStr"/>
+      <c r="S540" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" s="2" t="inlineStr">
+        <is>
+          <t>Ben Shelton</t>
+        </is>
+      </c>
+      <c r="B541" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C541" s="2" t="inlineStr">
+        <is>
+          <t>25 Topps Chrome Tennis BEN SHELTON 🇺🇸 From All Angles Gold Ref 1/50 bookend!</t>
+        </is>
+      </c>
+      <c r="D541" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E541" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F541" s="2" t="inlineStr">
+        <is>
+          <t>59.99 USD</t>
+        </is>
+      </c>
+      <c r="G541" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/227540401982</t>
+        </is>
+      </c>
+      <c r="H541" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 14:15 UTC</t>
+        </is>
+      </c>
+      <c r="I541" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ttUAAeSw3Mtqt-Gf/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J541" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T15:16:05.000Z</t>
+        </is>
+      </c>
+      <c r="K541" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L541" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M541" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N541" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2GwAAeSw0WBqt-GV/s-l1600.jpg | https://i.ebayimg.com/images/g/I~YAAeSwJ4Zqt-Ga/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O541" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P541" s="2" t="inlineStr"/>
+      <c r="Q541" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R541" s="2" t="inlineStr"/>
+      <c r="S541" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -46535,6 +48194,25 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G520" r:id="rId519"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G521" r:id="rId520"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G522" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G523" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G524" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G525" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G526" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G527" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G528" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G529" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G530" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G531" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G532" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G533" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G534" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G535" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G536" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G537" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G538" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G539" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G540" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G541" r:id="rId540"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-02 15:56 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S541"/>
+  <dimension ref="A1:S559"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -47666,6 +47666,1568 @@
       </c>
       <c r="R541" s="2" t="inlineStr"/>
       <c r="S541" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" s="2" t="inlineStr">
+        <is>
+          <t>Linda Noskova</t>
+        </is>
+      </c>
+      <c r="B542" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C542" s="2" t="inlineStr">
+        <is>
+          <t>Linda Noskova 2026 Topps Chrome Tennis Destiny Geometric 25/25</t>
+        </is>
+      </c>
+      <c r="D542" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E542" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F542" s="2" t="inlineStr">
+        <is>
+          <t>9.99 USD</t>
+        </is>
+      </c>
+      <c r="G542" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147614964138</t>
+        </is>
+      </c>
+      <c r="H542" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:55 UTC</t>
+        </is>
+      </c>
+      <c r="I542" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9gMAAeSwTMVqv81X/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J542" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T15:27:46.000Z</t>
+        </is>
+      </c>
+      <c r="K542" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L542" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M542" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N542" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/C78AAeSwG8Zqv81Y/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O542" s="2" t="inlineStr"/>
+      <c r="P542" s="2" t="inlineStr"/>
+      <c r="Q542" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R542" s="2" t="inlineStr"/>
+      <c r="S542" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" s="2" t="inlineStr">
+        <is>
+          <t>Tristan Schoolkate</t>
+        </is>
+      </c>
+      <c r="B543" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C543" s="2" t="inlineStr">
+        <is>
+          <t>Tristan Schoolkate 2026 Topps Chrome Orange Geometric Refractor Rookie 25/25...</t>
+        </is>
+      </c>
+      <c r="D543" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E543" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F543" s="2" t="inlineStr">
+        <is>
+          <t>9.99 USD</t>
+        </is>
+      </c>
+      <c r="G543" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/137804735975</t>
+        </is>
+      </c>
+      <c r="H543" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:55 UTC</t>
+        </is>
+      </c>
+      <c r="I543" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9jkAAeSw0-xqv80A/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J543" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T15:26:19.000Z</t>
+        </is>
+      </c>
+      <c r="K543" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L543" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M543" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N543" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Me8AAeSwA8xqv80A/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O543" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P543" s="2" t="inlineStr"/>
+      <c r="Q543" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R543" s="2" t="inlineStr"/>
+      <c r="S543" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="2" t="inlineStr">
+        <is>
+          <t>Chris Eubanks</t>
+        </is>
+      </c>
+      <c r="B544" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C544" s="2" t="inlineStr">
+        <is>
+          <t>CHRIS EUBANKS 2026 Topps Chrome Tennis Autograph AUTO Superfractor 1/1 AT-CES</t>
+        </is>
+      </c>
+      <c r="D544" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E544" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F544" s="2" t="inlineStr">
+        <is>
+          <t>1299.99 USD</t>
+        </is>
+      </c>
+      <c r="G544" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/267801676913</t>
+        </is>
+      </c>
+      <c r="H544" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:55 UTC</t>
+        </is>
+      </c>
+      <c r="I544" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/F3oAAeSw6HJqv8wE/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J544" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T15:25:55.000Z</t>
+        </is>
+      </c>
+      <c r="K544" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L544" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M544" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N544" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8vcAAeSw-Cpqv8w2/s-l1600.jpg | https://i.ebayimg.com/images/g/N8gAAeSwt~tqv8w3/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O544" s="2" t="inlineStr"/>
+      <c r="P544" s="2" t="inlineStr"/>
+      <c r="Q544" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R544" s="2" t="inlineStr"/>
+      <c r="S544" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" s="2" t="inlineStr">
+        <is>
+          <t>Garbine Muguruza</t>
+        </is>
+      </c>
+      <c r="B545" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C545" s="2" t="inlineStr">
+        <is>
+          <t>Garbine Muguruza 01/10 Black Refractor 2026 Topps Chrome Tennis #163</t>
+        </is>
+      </c>
+      <c r="D545" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E545" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F545" s="2" t="inlineStr">
+        <is>
+          <t>19.99 USD</t>
+        </is>
+      </c>
+      <c r="G545" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287622263931</t>
+        </is>
+      </c>
+      <c r="H545" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:55 UTC</t>
+        </is>
+      </c>
+      <c r="I545" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ssgAAeSwG1Zqv8sC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J545" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T15:18:36.000Z</t>
+        </is>
+      </c>
+      <c r="K545" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L545" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M545" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N545" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/GYkAAeSwCbFqv8sC/s-l1600.jpg | https://i.ebayimg.com/images/g/cfIAAeSwrRRqv8sC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O545" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P545" s="2" t="inlineStr"/>
+      <c r="Q545" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R545" s="2" t="inlineStr"/>
+      <c r="S545" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="2" t="inlineStr">
+        <is>
+          <t>Donna Vekic</t>
+        </is>
+      </c>
+      <c r="B546" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C546" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Blue Refractor 250/250 Donna Vekic #48 Rookie RC 16xu</t>
+        </is>
+      </c>
+      <c r="D546" s="2" t="inlineStr">
+        <is>
+          <t>250/250</t>
+        </is>
+      </c>
+      <c r="E546" s="2" t="inlineStr">
+        <is>
+          <t>last of 250 (250/250)</t>
+        </is>
+      </c>
+      <c r="F546" s="2" t="inlineStr">
+        <is>
+          <t>4.28 USD</t>
+        </is>
+      </c>
+      <c r="G546" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336823904872</t>
+        </is>
+      </c>
+      <c r="H546" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:55 UTC</t>
+        </is>
+      </c>
+      <c r="I546" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/BH4AAeSwykJqv8sx/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J546" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T15:17:02.000Z</t>
+        </is>
+      </c>
+      <c r="K546" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L546" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M546" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N546" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/yLcAAeSwASdqv8sx/s-l1600.jpg | https://i.ebayimg.com/images/g/~dMAAeSw6XBqv8sx/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O546" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P546" s="2" t="inlineStr"/>
+      <c r="Q546" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R546" s="2" t="inlineStr"/>
+      <c r="S546" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" s="2" t="inlineStr">
+        <is>
+          <t>Taylah Preston</t>
+        </is>
+      </c>
+      <c r="B547" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C547" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Tennis Taylah Preston Superfractor Rookie 1/1 RC SSP #72</t>
+        </is>
+      </c>
+      <c r="D547" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E547" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F547" s="2" t="inlineStr">
+        <is>
+          <t>1999.99 USD</t>
+        </is>
+      </c>
+      <c r="G547" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287622214982</t>
+        </is>
+      </c>
+      <c r="H547" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:55 UTC</t>
+        </is>
+      </c>
+      <c r="I547" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SFEAAeSwPhtqv8GV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J547" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:37:47.000Z</t>
+        </is>
+      </c>
+      <c r="K547" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L547" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M547" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N547" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/sR4AAeSwSohqv8GV/s-l1600.jpg | https://i.ebayimg.com/images/g/C00AAeSwG1Zqv8GV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O547" s="2" t="inlineStr"/>
+      <c r="P547" s="2" t="inlineStr"/>
+      <c r="Q547" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R547" s="2" t="inlineStr"/>
+      <c r="S547" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="2" t="inlineStr">
+        <is>
+          <t>Tommy Paul</t>
+        </is>
+      </c>
+      <c r="B548" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C548" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis #AO-TPL Tommy Paul Refractor On Card Auto 25/25</t>
+        </is>
+      </c>
+      <c r="D548" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E548" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F548" s="2" t="inlineStr">
+        <is>
+          <t>350.00 USD</t>
+        </is>
+      </c>
+      <c r="G548" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237101925693</t>
+        </is>
+      </c>
+      <c r="H548" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:55 UTC</t>
+        </is>
+      </c>
+      <c r="I548" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/b5QAAeSwZPtqv5s1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J548" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T11:54:15.000Z</t>
+        </is>
+      </c>
+      <c r="K548" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L548" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M548" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N548" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/n5IAAeSwNYZqv5s8/s-l1600.jpg | https://i.ebayimg.com/images/g/iEwAAeSw-ndqv5tA/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O548" s="2" t="inlineStr"/>
+      <c r="P548" s="2" t="inlineStr"/>
+      <c r="Q548" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R548" s="2" t="inlineStr"/>
+      <c r="S548" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" s="2" t="inlineStr">
+        <is>
+          <t>Tristan Boyer</t>
+        </is>
+      </c>
+      <c r="B549" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C549" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2025 Chrome Tennis Tristan Boyer Autographs Rookie Auto Gold 50 /50 CA-TBR</t>
+        </is>
+      </c>
+      <c r="D549" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E549" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F549" s="2" t="inlineStr">
+        <is>
+          <t>50.00 USD</t>
+        </is>
+      </c>
+      <c r="G549" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/920000419878?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2F4%2B%2FFqWR7xD8urnq2chJuZ0OZ%2F70avygeOFDWPD75%2BEw11oXl3gJ8L6b0iM%2F6ZpME0G9tLo%2BJ5WdXRD5PScVfrv%2FA4BbwaQOXCmwOvElxg6Vee05l%2B3w6icbNcCdSx0r78jP6n1cdjHWA12Wtgd8YkD7da7XbJTd%2F3JxgA5chGkiA3%2F9yG8YMN3QjYo1hMTWo%3D</t>
+        </is>
+      </c>
+      <c r="H549" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:55 UTC</t>
+        </is>
+      </c>
+      <c r="I549" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RqYAAeSwkJlqv3am/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J549" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T09:18:26.000Z</t>
+        </is>
+      </c>
+      <c r="K549" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L549" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M549" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N549" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/BaIAAeSwV7hqv3ah/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O549" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P549" s="2" t="inlineStr"/>
+      <c r="Q549" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R549" s="2" t="inlineStr"/>
+      <c r="S549" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="2" t="inlineStr">
+        <is>
+          <t>Martina Navratilova</t>
+        </is>
+      </c>
+      <c r="B550" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C550" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Martina Navratilova Autograph Geometric RED 1/5</t>
+        </is>
+      </c>
+      <c r="D550" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E550" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F550" s="2" t="inlineStr">
+        <is>
+          <t>240.00 USD</t>
+        </is>
+      </c>
+      <c r="G550" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/318945390026</t>
+        </is>
+      </c>
+      <c r="H550" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:55 UTC</t>
+        </is>
+      </c>
+      <c r="I550" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/x2QAAeSwPnxqvzoi/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J550" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T05:00:38.000Z</t>
+        </is>
+      </c>
+      <c r="K550" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L550" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M550" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N550" s="2" t="inlineStr"/>
+      <c r="O550" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P550" s="2" t="inlineStr"/>
+      <c r="Q550" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R550" s="2" t="inlineStr"/>
+      <c r="S550" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" s="2" t="inlineStr">
+        <is>
+          <t>Jan Kodes</t>
+        </is>
+      </c>
+      <c r="B551" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C551" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Blue Refractor 1/99 Jan Kodes Jan Kodeš #36 HOF 0rs8</t>
+        </is>
+      </c>
+      <c r="D551" s="2" t="inlineStr">
+        <is>
+          <t>1/99</t>
+        </is>
+      </c>
+      <c r="E551" s="2" t="inlineStr">
+        <is>
+          <t>001 of 99</t>
+        </is>
+      </c>
+      <c r="F551" s="2" t="inlineStr">
+        <is>
+          <t>7.73 USD</t>
+        </is>
+      </c>
+      <c r="G551" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257777492943</t>
+        </is>
+      </c>
+      <c r="H551" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:56 UTC</t>
+        </is>
+      </c>
+      <c r="I551" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/UfEAAeSwBGFqvylK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J551" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T03:46:19.000Z</t>
+        </is>
+      </c>
+      <c r="K551" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L551" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M551" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N551" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/yVUAAeSwusFqvylK/s-l1600.jpg | https://i.ebayimg.com/images/g/nt0AAeSwn2NqvylK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O551" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P551" s="2" t="inlineStr"/>
+      <c r="Q551" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R551" s="2" t="inlineStr"/>
+      <c r="S551" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="2" t="inlineStr">
+        <is>
+          <t>Claire Liu</t>
+        </is>
+      </c>
+      <c r="B552" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C552" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Claire Liu 1/1 Superfractor 🔥</t>
+        </is>
+      </c>
+      <c r="D552" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E552" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F552" s="2" t="inlineStr">
+        <is>
+          <t>2000.00 USD</t>
+        </is>
+      </c>
+      <c r="G552" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/267801258459</t>
+        </is>
+      </c>
+      <c r="H552" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:56 UTC</t>
+        </is>
+      </c>
+      <c r="I552" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/hVQAAeSwJUJqvyCb/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J552" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T03:13:59.000Z</t>
+        </is>
+      </c>
+      <c r="K552" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L552" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M552" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA)</t>
+        </is>
+      </c>
+      <c r="N552" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JBUAAeSwCAxqvyCq/s-l1600.jpg | https://i.ebayimg.com/images/g/KQwAAeSwuw9qvyCi/s-l1600.jpg | https://i.ebayimg.com/images/g/2DoAAeSwEVFqvyCq/s-l1600.jpg | https://i.ebayimg.com/images/g/E4MAAeSw0zlqvyCn/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O552" s="2" t="inlineStr"/>
+      <c r="P552" s="2" t="inlineStr"/>
+      <c r="Q552" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R552" s="2" t="inlineStr"/>
+      <c r="S552" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" s="2" t="inlineStr">
+        <is>
+          <t>Talia Gibson</t>
+        </is>
+      </c>
+      <c r="B553" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C553" s="2" t="inlineStr">
+        <is>
+          <t>Topps Chrome Tennis 2026 Talia Gibson RC Auto AT-TGN FrozenFractor -1/0</t>
+        </is>
+      </c>
+      <c r="D553" s="2" t="inlineStr">
+        <is>
+          <t>1/0</t>
+        </is>
+      </c>
+      <c r="E553" s="2" t="inlineStr">
+        <is>
+          <t>001 of 0</t>
+        </is>
+      </c>
+      <c r="F553" s="2" t="inlineStr">
+        <is>
+          <t>1000.00 USD</t>
+        </is>
+      </c>
+      <c r="G553" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/198681656571</t>
+        </is>
+      </c>
+      <c r="H553" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:56 UTC</t>
+        </is>
+      </c>
+      <c r="I553" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KPsAAeSwADJqvx~R/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J553" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T03:07:16.000Z</t>
+        </is>
+      </c>
+      <c r="K553" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L553" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M553" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N553" s="2" t="inlineStr"/>
+      <c r="O553" s="2" t="inlineStr"/>
+      <c r="P553" s="2" t="inlineStr"/>
+      <c r="Q553" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R553" s="2" t="inlineStr"/>
+      <c r="S553" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="2" t="inlineStr">
+        <is>
+          <t>Garbine Muguruza</t>
+        </is>
+      </c>
+      <c r="B554" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite - Tour Relic Autographs - Red Crystalline Ref</t>
+        </is>
+      </c>
+      <c r="C554" s="2" t="inlineStr">
+        <is>
+          <t>2026 Graphite Red Crystalline Refractor 1/1 Garbine Muguruza Garbiñe Auto 1n9c</t>
+        </is>
+      </c>
+      <c r="D554" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E554" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F554" s="2" t="inlineStr">
+        <is>
+          <t>1021.10 USD</t>
+        </is>
+      </c>
+      <c r="G554" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237101002366</t>
+        </is>
+      </c>
+      <c r="H554" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:56 UTC</t>
+        </is>
+      </c>
+      <c r="I554" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/mWkAAeSwxHtqvtMN/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J554" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T21:38:21.000Z</t>
+        </is>
+      </c>
+      <c r="K554" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L554" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M554" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N554" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/pycAAeSwD3ZqvtMN/s-l1600.jpg | https://i.ebayimg.com/images/g/m4kAAeSwQG5qvtMM/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O554" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P554" s="2" t="inlineStr"/>
+      <c r="Q554" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R554" s="2" t="inlineStr"/>
+      <c r="S554" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" s="2" t="inlineStr">
+        <is>
+          <t>Hubert Hurkacz</t>
+        </is>
+      </c>
+      <c r="B555" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps</t>
+        </is>
+      </c>
+      <c r="C555" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Tennis Graphite Hubert Hurkacz #GR-HH Red Crystalline Relic 1/1</t>
+        </is>
+      </c>
+      <c r="D555" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E555" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F555" s="2" t="inlineStr">
+        <is>
+          <t>599.99 USD</t>
+        </is>
+      </c>
+      <c r="G555" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377536909143?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2B2a6i5jQLMaKCHrAr0VueGJPQoXtwAgRU%2B44EYA%2BtOltGqwxEQWt0mYdSXejxhfYuFXaJt6agNsFvW1YMq1xBqXv7cvg3oRKx59uGFSHnu2binJwYnYRRfHNkrilEEGwhS0EN%2BgASJY8SUk0RmunHMV6j1RgZWEk%2F9p9tI8hMLc%2B3iix6fawreOC6%2FnWzory0%3D</t>
+        </is>
+      </c>
+      <c r="H555" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:56 UTC</t>
+        </is>
+      </c>
+      <c r="I555" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TIkAAeSwjSVqvrXw/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J555" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T19:40:22.000Z</t>
+        </is>
+      </c>
+      <c r="K555" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L555" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M555" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N555" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/5JUAAeSwSohqvrXz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O555" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P555" s="2" t="inlineStr"/>
+      <c r="Q555" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R555" s="2" t="inlineStr"/>
+      <c r="S555" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" s="2" t="inlineStr">
+        <is>
+          <t>Ugo Humbert</t>
+        </is>
+      </c>
+      <c r="B556" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C556" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis Ugo Humbert Gold 1/10 #23 WE45</t>
+        </is>
+      </c>
+      <c r="D556" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E556" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F556" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G556" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407260552249</t>
+        </is>
+      </c>
+      <c r="H556" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:56 UTC</t>
+        </is>
+      </c>
+      <c r="I556" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DqYAAeSwo29qvw7~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J556" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T01:54:04.000Z</t>
+        </is>
+      </c>
+      <c r="K556" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L556" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M556" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N556" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Fd8AAeSwamhqvw8D/s-l1600.jpg | https://i.ebayimg.com/images/g/GOgAAeSwpEBqvw77/s-l1600.jpg | https://i.ebayimg.com/images/g/Qa0AAeSwGgNqvw77/s-l1600.jpg | https://i.ebayimg.com/images/g/UkYAAeSwV71qvw77/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O556" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P556" s="2" t="inlineStr"/>
+      <c r="Q556" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R556" s="2" t="inlineStr"/>
+      <c r="S556" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="2" t="inlineStr">
+        <is>
+          <t>Garbine Muguruza</t>
+        </is>
+      </c>
+      <c r="B557" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C557" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Garbine Muguruza Star Relics Patch EU 75/75 #SRR-GM WE45</t>
+        </is>
+      </c>
+      <c r="D557" s="2" t="inlineStr">
+        <is>
+          <t>75/75</t>
+        </is>
+      </c>
+      <c r="E557" s="2" t="inlineStr">
+        <is>
+          <t>last of 75 (75/75)</t>
+        </is>
+      </c>
+      <c r="F557" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G557" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407260546320</t>
+        </is>
+      </c>
+      <c r="H557" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:56 UTC</t>
+        </is>
+      </c>
+      <c r="I557" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/cskAAeSw2t1qvw3S/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J557" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T01:49:05.000Z</t>
+        </is>
+      </c>
+      <c r="K557" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L557" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M557" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N557" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YigAAeSwjnBqvw3W/s-l1600.jpg | https://i.ebayimg.com/images/g/NCQAAeSw8z5qvw3P/s-l1600.jpg | https://i.ebayimg.com/images/g/XmIAAeSwimhqvw3P/s-l1600.jpg | https://i.ebayimg.com/images/g/SMMAAeSwznhqvw3P/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O557" s="2" t="inlineStr"/>
+      <c r="P557" s="2" t="inlineStr"/>
+      <c r="Q557" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R557" s="2" t="inlineStr"/>
+      <c r="S557" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="2" t="inlineStr">
+        <is>
+          <t>Chris Eubanks</t>
+        </is>
+      </c>
+      <c r="B558" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C558" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Chris Eubanks Pursuit of Greatness Auto Blue 25/25 WE45</t>
+        </is>
+      </c>
+      <c r="D558" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E558" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F558" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G558" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407260537843</t>
+        </is>
+      </c>
+      <c r="H558" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:56 UTC</t>
+        </is>
+      </c>
+      <c r="I558" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/BSgAAeSw03dqvwvx/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J558" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T01:41:02.000Z</t>
+        </is>
+      </c>
+      <c r="K558" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L558" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M558" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N558" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/OgsAAeSwNYZqvwv1/s-l1600.jpg | https://i.ebayimg.com/images/g/OfYAAeSwNYZqvwvz/s-l1600.jpg | https://i.ebayimg.com/images/g/vgIAAeSw1MJqvwvu/s-l1600.jpg | https://i.ebayimg.com/images/g/LbAAAeSwoH1qvwvu/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O558" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P558" s="2" t="inlineStr"/>
+      <c r="Q558" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R558" s="2" t="inlineStr"/>
+      <c r="S558" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" s="2" t="inlineStr">
+        <is>
+          <t>Jessica Pegula</t>
+        </is>
+      </c>
+      <c r="B559" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Regalia Relic Signatures</t>
+        </is>
+      </c>
+      <c r="C559" s="2" t="inlineStr">
+        <is>
+          <t>2024 Royalty Regalia Relic Signatures 75/75 Jessica Pegula Rookie Auto RC 3s8</t>
+        </is>
+      </c>
+      <c r="D559" s="2" t="inlineStr">
+        <is>
+          <t>75/75</t>
+        </is>
+      </c>
+      <c r="E559" s="2" t="inlineStr">
+        <is>
+          <t>last of 75 (75/75)</t>
+        </is>
+      </c>
+      <c r="F559" s="2" t="inlineStr">
+        <is>
+          <t>98.58 USD</t>
+        </is>
+      </c>
+      <c r="G559" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237101027062</t>
+        </is>
+      </c>
+      <c r="H559" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:56 UTC</t>
+        </is>
+      </c>
+      <c r="I559" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/mNIAAeSwmfZqvto9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J559" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T22:08:57.000Z</t>
+        </is>
+      </c>
+      <c r="K559" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L559" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M559" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N559" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/6CsAAeSwsQBqvto9/s-l1600.jpg | https://i.ebayimg.com/images/g/P3sAAeSwdqFqvto-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O559" s="2" t="inlineStr"/>
+      <c r="P559" s="2" t="inlineStr"/>
+      <c r="Q559" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R559" s="2" t="inlineStr"/>
+      <c r="S559" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -48213,6 +49775,24 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G539" r:id="rId538"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G540" r:id="rId539"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G541" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G542" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G543" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G544" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G545" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G546" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G547" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G548" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G549" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G550" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G551" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G552" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G553" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G554" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G555" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G556" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G557" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G558" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G559" r:id="rId558"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-03 14:24 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S559"/>
+  <dimension ref="A1:S581"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -49228,6 +49228,1952 @@
       </c>
       <c r="R559" s="2" t="inlineStr"/>
       <c r="S559" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" s="2" t="inlineStr">
+        <is>
+          <t>Aryna Sabalenka</t>
+        </is>
+      </c>
+      <c r="B560" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C560" s="2" t="inlineStr">
+        <is>
+          <t>Aryna Sabalenka 2026 Topps Chrome Tennis WORLD NUMBER 1 /25 Auto #NOS-AS SSP</t>
+        </is>
+      </c>
+      <c r="D560" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E560" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F560" s="2" t="inlineStr">
+        <is>
+          <t>999.99 USD</t>
+        </is>
+      </c>
+      <c r="G560" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/189037750260</t>
+        </is>
+      </c>
+      <c r="H560" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I560" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/emgAAeSwVIxqwPyn/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J560" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T13:02:30.000Z</t>
+        </is>
+      </c>
+      <c r="K560" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L560" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M560" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N560" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RIEAAeSwkkdqwPyu/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O560" s="2" t="inlineStr"/>
+      <c r="P560" s="2" t="inlineStr"/>
+      <c r="Q560" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R560" s="2" t="inlineStr"/>
+      <c r="S560" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B561" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C561" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff 2025 Topps Chrome Tennis #200 True Black Refractor 1/10 RARE!</t>
+        </is>
+      </c>
+      <c r="D561" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E561" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F561" s="2" t="inlineStr">
+        <is>
+          <t>382.58 USD</t>
+        </is>
+      </c>
+      <c r="G561" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178550962234?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2FTP4UUyH5vUuQWFVD9vXlmeq2xqua2Kb0sOUSG%2Bp%2BYCC2mvEH1F3hh%2BXDyx9L6R31gpBUrIIjreG3o2XNkWnEKzhhYl3a5FApZbhocKiOhwt3DSVJvB7RC51jr5nTu1TpLMVK5uxo3%2FEUa52zEswK9WiwWWiuS3G9M9EF4KOtO5JCtCr07QjyIldE8hCaOhHw%3D</t>
+        </is>
+      </c>
+      <c r="H561" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I561" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/WxoAAeSwJHBqwPkA/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J561" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T12:51:48.000Z</t>
+        </is>
+      </c>
+      <c r="K561" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L561" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M561" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N561" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Fq4AAeSw1FNqwPkK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O561" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P561" s="2" t="inlineStr"/>
+      <c r="Q561" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R561" s="2" t="inlineStr"/>
+      <c r="S561" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" s="2" t="inlineStr">
+        <is>
+          <t>Naomi Osaka</t>
+        </is>
+      </c>
+      <c r="B562" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C562" s="2" t="inlineStr">
+        <is>
+          <t>Naomi Osaka 2026 Topps Chrome Tennis ORANGE REFRACTOR 01/25 #66 /25</t>
+        </is>
+      </c>
+      <c r="D562" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E562" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F562" s="2" t="inlineStr">
+        <is>
+          <t>79.99 USD</t>
+        </is>
+      </c>
+      <c r="G562" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/189037597925</t>
+        </is>
+      </c>
+      <c r="H562" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I562" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/CB4AAeSwmh9qwPSP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J562" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T12:27:12.000Z</t>
+        </is>
+      </c>
+      <c r="K562" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L562" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M562" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N562" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/VA0AAeSwASdqwPR7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O562" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P562" s="2" t="inlineStr"/>
+      <c r="Q562" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R562" s="2" t="inlineStr"/>
+      <c r="S562" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" s="2" t="inlineStr">
+        <is>
+          <t>Maria Sharapova</t>
+        </is>
+      </c>
+      <c r="B563" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C563" s="2" t="inlineStr">
+        <is>
+          <t>Maria Sharapova 2026 Topps Chrome Tennis World Number 1 ORANGE 25/25 #WNO-MS /25</t>
+        </is>
+      </c>
+      <c r="D563" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E563" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F563" s="2" t="inlineStr">
+        <is>
+          <t>149.99 USD</t>
+        </is>
+      </c>
+      <c r="G563" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/189037590751</t>
+        </is>
+      </c>
+      <c r="H563" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I563" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/6BMAAeSwZztqwPNO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J563" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T12:22:28.000Z</t>
+        </is>
+      </c>
+      <c r="K563" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L563" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M563" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N563" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/4gMAAeSwNnNqwPMs/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O563" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P563" s="2" t="inlineStr"/>
+      <c r="Q563" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R563" s="2" t="inlineStr"/>
+      <c r="S563" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" s="2" t="inlineStr">
+        <is>
+          <t>Valentin Vacherot</t>
+        </is>
+      </c>
+      <c r="B564" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C564" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis #AT-VVT Valentin Vacherot Blue Refractor 150/150</t>
+        </is>
+      </c>
+      <c r="D564" s="2" t="inlineStr">
+        <is>
+          <t>150/150</t>
+        </is>
+      </c>
+      <c r="E564" s="2" t="inlineStr">
+        <is>
+          <t>last of 150 (150/150)</t>
+        </is>
+      </c>
+      <c r="F564" s="2" t="inlineStr">
+        <is>
+          <t>15.00 USD</t>
+        </is>
+      </c>
+      <c r="G564" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/128112475331</t>
+        </is>
+      </c>
+      <c r="H564" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I564" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0fsAAeSwASdqwOqX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J564" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T11:45:45.000Z</t>
+        </is>
+      </c>
+      <c r="K564" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L564" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M564" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N564" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TmgAAeSwPjJqwOqW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O564" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P564" s="2" t="inlineStr"/>
+      <c r="Q564" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R564" s="2" t="inlineStr"/>
+      <c r="S564" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" s="2" t="inlineStr">
+        <is>
+          <t>Pedro Cachin</t>
+        </is>
+      </c>
+      <c r="B565" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C565" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Aqua Refractor 399/399 Pedro Cachin #112 Rookie RC sc8</t>
+        </is>
+      </c>
+      <c r="D565" s="2" t="inlineStr">
+        <is>
+          <t>399/399</t>
+        </is>
+      </c>
+      <c r="E565" s="2" t="inlineStr">
+        <is>
+          <t>last of 399 (399/399)</t>
+        </is>
+      </c>
+      <c r="F565" s="2" t="inlineStr">
+        <is>
+          <t>1.63 USD</t>
+        </is>
+      </c>
+      <c r="G565" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336825093628</t>
+        </is>
+      </c>
+      <c r="H565" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I565" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/BvUAAeSwm-xqwNEL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J565" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T09:54:20.000Z</t>
+        </is>
+      </c>
+      <c r="K565" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L565" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M565" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N565" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-GwAAeSwnpJqwNEL/s-l1600.jpg | https://i.ebayimg.com/images/g/PXEAAeSwOoxqwNEL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O565" s="2" t="inlineStr">
+        <is>
+          <t>aqua</t>
+        </is>
+      </c>
+      <c r="P565" s="2" t="inlineStr"/>
+      <c r="Q565" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R565" s="2" t="inlineStr"/>
+      <c r="S565" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" s="2" t="inlineStr">
+        <is>
+          <t>Zeynep Sonmez</t>
+        </is>
+      </c>
+      <c r="B566" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C566" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2026 Topps Chrome Tennis Zeynep Sonmez RC Autograph AT-ZSZ 5/5</t>
+        </is>
+      </c>
+      <c r="D566" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E566" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F566" s="2" t="inlineStr">
+        <is>
+          <t>450.19 USD</t>
+        </is>
+      </c>
+      <c r="G566" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407262978117?amdata=enc%3AAQALAAAAsCHNgUiiE%2FjQhlDTaMiAde9xarZA40uKuodqwinDbJr%2F9M%2FbC%2Bl8l7SLAAJcaTJvYn%2F4oAXLqiTt1AkTK%2F72%2BcHqsRYDjeWDSvJoaDak3CCLx4aHXu82IYSODzzJ9y82sFds8Q5exTaRkq0O7OIuke%2FQl%2BELBhNA%2FwT4odfRw7%2BGxoZSQdpgEAd%2B8Uoe%2Bu6gyB1n%2BCqye7qt8vow58DJoK4WBESZsaKuzbsvDT2t%2FplS</t>
+        </is>
+      </c>
+      <c r="H566" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I566" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/GkQAAeSwCbFqwLCb/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J566" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T07:53:42.000Z</t>
+        </is>
+      </c>
+      <c r="K566" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L566" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M566" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N566" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/1ycAAeSwh3ZqwLA0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O566" s="2" t="inlineStr"/>
+      <c r="P566" s="2" t="inlineStr"/>
+      <c r="Q566" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R566" s="2" t="inlineStr"/>
+      <c r="S566" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" s="2" t="inlineStr">
+        <is>
+          <t>Elina Svitolina</t>
+        </is>
+      </c>
+      <c r="B567" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 topps chrome</t>
+        </is>
+      </c>
+      <c r="C567" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2026 Chrome Tennis Elina Svitolina 5/5 Autographs II Auto #CA-ESA sp rare</t>
+        </is>
+      </c>
+      <c r="D567" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E567" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F567" s="2" t="inlineStr">
+        <is>
+          <t>500.00 USD</t>
+        </is>
+      </c>
+      <c r="G567" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168758151805?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde92sy0Y67ZANVKnCfj8A2dbIA2OXu9s%2FfHQ650z9IH2GBIycgmRlpjezIa4rGo1jfkWp3CuXLe0hcTFJLHVgQo0j2Rkwc%2BiXSj9n8BWn3%2F8C0jxflAvipaS%2BEYL4mbSU6kmzAFxAS%2BG0zBUM6WCc8FfEKRA40htVHYSRyCiXvjLEK%2B7VUyp3Hnph%2FqK9iHITiQ%3D</t>
+        </is>
+      </c>
+      <c r="H567" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I567" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ezkAAeSwcPhqwLIf/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J567" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T07:44:19.000Z</t>
+        </is>
+      </c>
+      <c r="K567" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L567" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M567" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N567" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3k4AAeSwWsdqwLIT/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O567" s="2" t="inlineStr"/>
+      <c r="P567" s="2" t="inlineStr"/>
+      <c r="Q567" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R567" s="2" t="inlineStr"/>
+      <c r="S567" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" s="2" t="inlineStr">
+        <is>
+          <t>John Newcombe</t>
+        </is>
+      </c>
+      <c r="B568" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C568" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Aqua Refractor 150/150 John Newcombe #49 HOF 7ba</t>
+        </is>
+      </c>
+      <c r="D568" s="2" t="inlineStr">
+        <is>
+          <t>150/150</t>
+        </is>
+      </c>
+      <c r="E568" s="2" t="inlineStr">
+        <is>
+          <t>last of 150 (150/150)</t>
+        </is>
+      </c>
+      <c r="F568" s="2" t="inlineStr">
+        <is>
+          <t>7.72 USD</t>
+        </is>
+      </c>
+      <c r="G568" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336824898264</t>
+        </is>
+      </c>
+      <c r="H568" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I568" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/j8MAAeSwG2VqwKaf/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J568" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T06:53:19.000Z</t>
+        </is>
+      </c>
+      <c r="K568" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L568" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M568" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N568" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3f4AAeSwp0JqwKaf/s-l1600.jpg | https://i.ebayimg.com/images/g/G40AAeSwAUNqwKaf/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O568" s="2" t="inlineStr">
+        <is>
+          <t>aqua</t>
+        </is>
+      </c>
+      <c r="P568" s="2" t="inlineStr"/>
+      <c r="Q568" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R568" s="2" t="inlineStr"/>
+      <c r="S568" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" s="2" t="inlineStr">
+        <is>
+          <t>Alexandra Eala</t>
+        </is>
+      </c>
+      <c r="B569" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Chrome</t>
+        </is>
+      </c>
+      <c r="C569" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Alexandra Eala #YQ-AE YouthQuake Orange Refractor 01/25</t>
+        </is>
+      </c>
+      <c r="D569" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E569" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F569" s="2" t="inlineStr">
+        <is>
+          <t>299.95 USD</t>
+        </is>
+      </c>
+      <c r="G569" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178550037820</t>
+        </is>
+      </c>
+      <c r="H569" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I569" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/kZwAAeSwGcxqwIX6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J569" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T04:37:16.000Z</t>
+        </is>
+      </c>
+      <c r="K569" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L569" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M569" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N569" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/6WwAAeSwOJdqwIX6/s-l1600.jpg | https://i.ebayimg.com/images/g/ypIAAeSwUPVqwIX6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O569" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P569" s="2" t="inlineStr"/>
+      <c r="Q569" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R569" s="2" t="inlineStr"/>
+      <c r="S569" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" s="2" t="inlineStr">
+        <is>
+          <t>Michael Chang</t>
+        </is>
+      </c>
+      <c r="B570" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C570" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis #129 Michael Chang Black 10/10 Bookend</t>
+        </is>
+      </c>
+      <c r="D570" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E570" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F570" s="2" t="inlineStr">
+        <is>
+          <t>175.43 USD</t>
+        </is>
+      </c>
+      <c r="G570" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168757667744</t>
+        </is>
+      </c>
+      <c r="H570" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I570" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YhsAAeSwlxpqwH47/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J570" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T04:08:04.000Z</t>
+        </is>
+      </c>
+      <c r="K570" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L570" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M570" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N570" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/FRIAAeSwinFqwH5E/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O570" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P570" s="2" t="inlineStr"/>
+      <c r="Q570" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R570" s="2" t="inlineStr"/>
+      <c r="S570" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" s="2" t="inlineStr">
+        <is>
+          <t>Viktorija Golubic</t>
+        </is>
+      </c>
+      <c r="B571" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C571" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Pink Geometric Refractor 65/65 Viktorija Golubic Rookie RC 3hd</t>
+        </is>
+      </c>
+      <c r="D571" s="2" t="inlineStr">
+        <is>
+          <t>65/65</t>
+        </is>
+      </c>
+      <c r="E571" s="2" t="inlineStr">
+        <is>
+          <t>last of 65 (65/65)</t>
+        </is>
+      </c>
+      <c r="F571" s="2" t="inlineStr">
+        <is>
+          <t>42.75 USD</t>
+        </is>
+      </c>
+      <c r="G571" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237103023929</t>
+        </is>
+      </c>
+      <c r="H571" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I571" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/n3IAAeSwqcpqwH8o/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J571" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T04:04:58.000Z</t>
+        </is>
+      </c>
+      <c r="K571" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L571" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M571" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports (PSA) 10 GEM MT</t>
+        </is>
+      </c>
+      <c r="N571" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jWsAAeSw9nRqwH8o/s-l1600.jpg | https://i.ebayimg.com/images/g/1TMAAeSwUJNqwH8p/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O571" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P571" s="2" t="inlineStr"/>
+      <c r="Q571" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R571" s="2" t="inlineStr"/>
+      <c r="S571" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" s="2" t="inlineStr">
+        <is>
+          <t>Emma Navarro</t>
+        </is>
+      </c>
+      <c r="B572" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C572" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis - Emma Navarro DESTINY BLACK GEO Auto Book End 10/10</t>
+        </is>
+      </c>
+      <c r="D572" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E572" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F572" s="2" t="inlineStr">
+        <is>
+          <t>400.00 USD</t>
+        </is>
+      </c>
+      <c r="G572" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/189035786837?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde9hxu%2FvtWibGAoY%2BOG45usifz8EEi%2BOTNVk%2Br4D6aPA883f2Pj%2FZFrYcHxjsnZCZtKF0Z7g5BulddyWJaiZcaLMHnPL9XaEda56bVBc7Wj6IE5CIzx3i1GQVDs3C7pybdWKD28jyoi8dp0wKOOvtRmoL0UpJPBFbh0V%2FxxjKGebGjuwluCIfvrGv1ug8gvAuCc%3D</t>
+        </is>
+      </c>
+      <c r="H572" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I572" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/iB0AAeSwPnxqwH0A/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J572" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T03:57:13.000Z</t>
+        </is>
+      </c>
+      <c r="K572" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L572" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M572" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N572" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-1cAAeSwK7lqwH0B/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O572" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P572" s="2" t="inlineStr"/>
+      <c r="Q572" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R572" s="2" t="inlineStr"/>
+      <c r="S572" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" s="2" t="inlineStr">
+        <is>
+          <t>Pete Sampras</t>
+        </is>
+      </c>
+      <c r="B573" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C573" s="2" t="inlineStr">
+        <is>
+          <t>2021 Chrome Rose Gold Refractor 1/10 Pete Sampras SGC 9.5 Mint+ Auto HOF ob9</t>
+        </is>
+      </c>
+      <c r="D573" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E573" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F573" s="2" t="inlineStr">
+        <is>
+          <t>527.20 USD</t>
+        </is>
+      </c>
+      <c r="G573" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257779111115</t>
+        </is>
+      </c>
+      <c r="H573" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I573" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TqkAAeSwmE1qwHub/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J573" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T03:49:48.000Z</t>
+        </is>
+      </c>
+      <c r="K573" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L573" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M573" s="2" t="inlineStr">
+        <is>
+          <t>Sportscard (SGC) 9.5 Mint+</t>
+        </is>
+      </c>
+      <c r="N573" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/PzgAAeSwGcxqwHub/s-l1600.jpg | https://i.ebayimg.com/images/g/V8MAAeSwkkdqwHub/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O573" s="2" t="inlineStr">
+        <is>
+          <t>rose</t>
+        </is>
+      </c>
+      <c r="P573" s="2" t="inlineStr"/>
+      <c r="Q573" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R573" s="2" t="inlineStr"/>
+      <c r="S573" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Bublik</t>
+        </is>
+      </c>
+      <c r="B574" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Chrome</t>
+        </is>
+      </c>
+      <c r="C574" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Bublik 2026 Topps Chrome Tennis Auto Green Geometric Refrac 1/99 TF1</t>
+        </is>
+      </c>
+      <c r="D574" s="2" t="inlineStr">
+        <is>
+          <t>1/99</t>
+        </is>
+      </c>
+      <c r="E574" s="2" t="inlineStr">
+        <is>
+          <t>001 of 99</t>
+        </is>
+      </c>
+      <c r="F574" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G574" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257779048039</t>
+        </is>
+      </c>
+      <c r="H574" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I574" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/lVEAAeSwLbBqwG2u/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J574" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T03:05:00.000Z</t>
+        </is>
+      </c>
+      <c r="K574" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L574" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M574" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N574" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bVwAAeSwp1NqwG2u/s-l1600.jpg | https://i.ebayimg.com/images/g/GEEAAeSw1N1qwG2u/s-l1600.jpg | https://i.ebayimg.com/images/g/n3sAAeSwNrpqwG2u/s-l1600.jpg | https://i.ebayimg.com/images/g/lTMAAeSwxCtqwG2u/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O574" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P574" s="2" t="inlineStr"/>
+      <c r="Q574" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R574" s="2" t="inlineStr"/>
+      <c r="S574" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" s="2" t="inlineStr">
+        <is>
+          <t>Ashlyn Krueger</t>
+        </is>
+      </c>
+      <c r="B575" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C575" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2024 Topps Graphite Ashlyn Krueger #195 Green Refractor RC 75/75 bookend</t>
+        </is>
+      </c>
+      <c r="D575" s="2" t="inlineStr">
+        <is>
+          <t>75/75</t>
+        </is>
+      </c>
+      <c r="E575" s="2" t="inlineStr">
+        <is>
+          <t>last of 75 (75/75)</t>
+        </is>
+      </c>
+      <c r="F575" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G575" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298729401579</t>
+        </is>
+      </c>
+      <c r="H575" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I575" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/fFAAAeSwSaZqwO4o/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J575" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T12:00:29.000Z</t>
+        </is>
+      </c>
+      <c r="K575" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L575" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M575" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N575" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/rkUAAeSwOJ1qwO4X/s-l1600.jpg | https://i.ebayimg.com/images/g/mq0AAeSwtjZqwO4c/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O575" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P575" s="2" t="inlineStr"/>
+      <c r="Q575" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R575" s="2" t="inlineStr"/>
+      <c r="S575" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" s="2" t="inlineStr">
+        <is>
+          <t>Danielle Collins</t>
+        </is>
+      </c>
+      <c r="B576" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C576" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Danielle Collins #40 Gold 1/25 WE45</t>
+        </is>
+      </c>
+      <c r="D576" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E576" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F576" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G576" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407262577514</t>
+        </is>
+      </c>
+      <c r="H576" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I576" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/69wAAeSwUMdqwF9T/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J576" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T01:50:01.000Z</t>
+        </is>
+      </c>
+      <c r="K576" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L576" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M576" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N576" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Zp0AAeSwk7BqwF9T/s-l1600.jpg | https://i.ebayimg.com/images/g/MFEAAeSwn2NqwF9L/s-l1600.jpg | https://i.ebayimg.com/images/g/NuEAAeSwdqFqwF9L/s-l1600.jpg | https://i.ebayimg.com/images/g/HxoAAeSwnpJqwF9L/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O576" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P576" s="2" t="inlineStr"/>
+      <c r="Q576" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R576" s="2" t="inlineStr"/>
+      <c r="S576" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" s="2" t="inlineStr">
+        <is>
+          <t>Paula Badosa</t>
+        </is>
+      </c>
+      <c r="B577" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C577" s="2" t="inlineStr">
+        <is>
+          <t>2026 TOPPS GRAPHITE PAULA BADOSA #BP-16 BREAK POINT WHITE REFRACTOR @ 1/10 @</t>
+        </is>
+      </c>
+      <c r="D577" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E577" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F577" s="2" t="inlineStr">
+        <is>
+          <t>49.99 USD</t>
+        </is>
+      </c>
+      <c r="G577" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168756302793</t>
+        </is>
+      </c>
+      <c r="H577" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I577" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/d5IAAeSwAUVqv-X1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J577" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T17:17:51.000Z</t>
+        </is>
+      </c>
+      <c r="K577" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L577" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M577" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N577" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/eyMAAeSw7CRqv-X1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O577" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P577" s="2" t="inlineStr"/>
+      <c r="Q577" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R577" s="2" t="inlineStr"/>
+      <c r="S577" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" s="2" t="inlineStr">
+        <is>
+          <t>Frances Tiafoe</t>
+        </is>
+      </c>
+      <c r="B578" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps</t>
+        </is>
+      </c>
+      <c r="C578" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Tennis Frances Tiafoe Red Crystalline Relic Auto 1/1 SSP</t>
+        </is>
+      </c>
+      <c r="D578" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E578" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F578" s="2" t="inlineStr">
+        <is>
+          <t>1749.99 USD</t>
+        </is>
+      </c>
+      <c r="G578" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287622379842</t>
+        </is>
+      </c>
+      <c r="H578" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I578" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/g8kAAeSwGTNqv-U0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J578" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T17:09:48.000Z</t>
+        </is>
+      </c>
+      <c r="K578" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L578" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M578" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N578" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HHEAAeSwmcFqv-U0/s-l1600.jpg | https://i.ebayimg.com/images/g/sY8AAeSw0jZqv-U0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O578" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P578" s="2" t="inlineStr"/>
+      <c r="Q578" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R578" s="2" t="inlineStr"/>
+      <c r="S578" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" s="2" t="inlineStr">
+        <is>
+          <t>Andy Roddick</t>
+        </is>
+      </c>
+      <c r="B579" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Collection Tennis</t>
+        </is>
+      </c>
+      <c r="C579" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2024 Royalty Collection Tennis Andy Roddick Ambassador Auto AA-AR 10/10</t>
+        </is>
+      </c>
+      <c r="D579" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E579" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F579" s="2" t="inlineStr">
+        <is>
+          <t>313.02 USD</t>
+        </is>
+      </c>
+      <c r="G579" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/820197924887</t>
+        </is>
+      </c>
+      <c r="H579" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I579" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/LCMAAeSw~yNqwGV0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J579" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T02:16:38.000Z</t>
+        </is>
+      </c>
+      <c r="K579" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L579" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M579" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N579" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JIwAAeSw24tqwGV0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O579" s="2" t="inlineStr"/>
+      <c r="P579" s="2" t="inlineStr"/>
+      <c r="Q579" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R579" s="2" t="inlineStr"/>
+      <c r="S579" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" s="2" t="inlineStr">
+        <is>
+          <t>Ken Rosewall</t>
+        </is>
+      </c>
+      <c r="B580" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic / 2008 Ace Authentic US Open</t>
+        </is>
+      </c>
+      <c r="C580" s="2" t="inlineStr">
+        <is>
+          <t>2008 Ace Authentic US Open Auto 79/79 Ken Rosewall #US29 Auto HOF 0n64</t>
+        </is>
+      </c>
+      <c r="D580" s="2" t="inlineStr">
+        <is>
+          <t>79/79</t>
+        </is>
+      </c>
+      <c r="E580" s="2" t="inlineStr">
+        <is>
+          <t>last of 79 (79/79)</t>
+        </is>
+      </c>
+      <c r="F580" s="2" t="inlineStr">
+        <is>
+          <t>174.95 USD</t>
+        </is>
+      </c>
+      <c r="G580" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237103396393</t>
+        </is>
+      </c>
+      <c r="H580" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I580" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-gMAAeSwn6dqwNEY/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J580" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T09:54:32.000Z</t>
+        </is>
+      </c>
+      <c r="K580" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L580" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M580" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N580" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/oPIAAeSw7bpqwNEZ/s-l1600.jpg | https://i.ebayimg.com/images/g/E08AAeSwbItqwNEb/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O580" s="2" t="inlineStr"/>
+      <c r="P580" s="2" t="inlineStr"/>
+      <c r="Q580" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R580" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic autograph: on-card or sticker not stated; check by eye</t>
+        </is>
+      </c>
+      <c r="S580" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" s="2" t="inlineStr">
+        <is>
+          <t>Mike Bryan, Lisa Raymond</t>
+        </is>
+      </c>
+      <c r="B581" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic</t>
+        </is>
+      </c>
+      <c r="C581" s="2" t="inlineStr">
+        <is>
+          <t>2013 Ace Perfect Partners Blue Auto 1/5 #PP-35 Raymond/Bryan PSA 8.5 (Top Pop)</t>
+        </is>
+      </c>
+      <c r="D581" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E581" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F581" s="2" t="inlineStr">
+        <is>
+          <t>75.00 USD</t>
+        </is>
+      </c>
+      <c r="G581" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168757038695</t>
+        </is>
+      </c>
+      <c r="H581" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:23 UTC</t>
+        </is>
+      </c>
+      <c r="I581" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/FZgAAOSwuURlU5g1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J581" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T23:11:38.000Z</t>
+        </is>
+      </c>
+      <c r="K581" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L581" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M581" s="2" t="inlineStr">
+        <is>
+          <t>PSA 8.5</t>
+        </is>
+      </c>
+      <c r="N581" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Z~wAAOSwL4RlU5g~/s-l1600.jpg | https://i.ebayimg.com/images/g/oHkAAOSwtY1lU5hJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O581" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P581" s="2" t="inlineStr"/>
+      <c r="Q581" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R581" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic autograph: on-card or sticker not stated; check by eye</t>
+        </is>
+      </c>
+      <c r="S581" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -49793,6 +51739,28 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G557" r:id="rId556"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G558" r:id="rId557"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G559" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G560" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G561" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G562" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G563" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G564" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G565" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G566" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G567" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G568" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G569" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G570" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G571" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G572" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G573" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G574" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G575" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G576" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G577" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G578" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G579" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G580" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G581" r:id="rId580"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-04 14:56 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S581"/>
+  <dimension ref="A1:S597"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -51174,6 +51174,1418 @@
         </is>
       </c>
       <c r="S581" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" s="2" t="inlineStr">
+        <is>
+          <t>Elina Avanesyan</t>
+        </is>
+      </c>
+      <c r="B582" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C582" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Elina Avanesyan Aqua Refractor /199 #119 001/199</t>
+        </is>
+      </c>
+      <c r="D582" s="2" t="inlineStr">
+        <is>
+          <t>1/199</t>
+        </is>
+      </c>
+      <c r="E582" s="2" t="inlineStr">
+        <is>
+          <t>001 of 199</t>
+        </is>
+      </c>
+      <c r="F582" s="2" t="inlineStr">
+        <is>
+          <t>14.99 USD</t>
+        </is>
+      </c>
+      <c r="G582" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/960011150832</t>
+        </is>
+      </c>
+      <c r="H582" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:55 UTC</t>
+        </is>
+      </c>
+      <c r="I582" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/AhEAAeSwtIlqwfLv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J582" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T06:34:20.000Z</t>
+        </is>
+      </c>
+      <c r="K582" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L582" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M582" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N582" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/1PgAAeSweCtqwfLv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O582" s="2" t="inlineStr">
+        <is>
+          <t>aqua</t>
+        </is>
+      </c>
+      <c r="P582" s="2" t="inlineStr"/>
+      <c r="Q582" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R582" s="2" t="inlineStr"/>
+      <c r="S582" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" s="2" t="inlineStr">
+        <is>
+          <t>Erika Andreeva</t>
+        </is>
+      </c>
+      <c r="B583" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C583" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Sapphire Green 125/125 Erika Andreeva #24 Rookie RC 1u4</t>
+        </is>
+      </c>
+      <c r="D583" s="2" t="inlineStr">
+        <is>
+          <t>125/125</t>
+        </is>
+      </c>
+      <c r="E583" s="2" t="inlineStr">
+        <is>
+          <t>last of 125 (125/125)</t>
+        </is>
+      </c>
+      <c r="F583" s="2" t="inlineStr">
+        <is>
+          <t>8.59 USD</t>
+        </is>
+      </c>
+      <c r="G583" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257780944112</t>
+        </is>
+      </c>
+      <c r="H583" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:55 UTC</t>
+        </is>
+      </c>
+      <c r="I583" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jIgAAeSwFBxqwd9H/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J583" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T05:07:12.000Z</t>
+        </is>
+      </c>
+      <c r="K583" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L583" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M583" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N583" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RqoAAeSwqAFqwd9I/s-l1600.jpg | https://i.ebayimg.com/images/g/i4EAAeSw3GJqwd9H/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O583" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P583" s="2" t="inlineStr"/>
+      <c r="Q583" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R583" s="2" t="inlineStr"/>
+      <c r="S583" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" s="2" t="inlineStr">
+        <is>
+          <t>Bernarda Pera</t>
+        </is>
+      </c>
+      <c r="B584" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C584" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome I Black Refractor 1/10 Bernarda Pera #TCA-BPA Auto 1w0z</t>
+        </is>
+      </c>
+      <c r="D584" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E584" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F584" s="2" t="inlineStr">
+        <is>
+          <t>29.58 USD</t>
+        </is>
+      </c>
+      <c r="G584" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336826299416</t>
+        </is>
+      </c>
+      <c r="H584" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:55 UTC</t>
+        </is>
+      </c>
+      <c r="I584" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uvwAAeSwTMVqwcrt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J584" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T03:40:31.000Z</t>
+        </is>
+      </c>
+      <c r="K584" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L584" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M584" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N584" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/h04AAeSw7Z5qwcrt/s-l1600.jpg | https://i.ebayimg.com/images/g/QC0AAeSwPGRqwcrt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O584" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P584" s="2" t="inlineStr"/>
+      <c r="Q584" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R584" s="2" t="inlineStr"/>
+      <c r="S584" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" s="2" t="inlineStr">
+        <is>
+          <t>Eva Lys</t>
+        </is>
+      </c>
+      <c r="B585" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C585" s="2" t="inlineStr">
+        <is>
+          <t>🎮MA 2026 TOPPS CHROME TENNIS AUTO ORANGE REFRACTOR 1/25 EVA LYS</t>
+        </is>
+      </c>
+      <c r="D585" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E585" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F585" s="2" t="inlineStr">
+        <is>
+          <t>5.50 USD</t>
+        </is>
+      </c>
+      <c r="G585" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/800754747781</t>
+        </is>
+      </c>
+      <c r="H585" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:55 UTC</t>
+        </is>
+      </c>
+      <c r="I585" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/rP8AAeSwHBNqv~Jn/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J585" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T03:16:00.000Z</t>
+        </is>
+      </c>
+      <c r="K585" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L585" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M585" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N585" s="2" t="inlineStr"/>
+      <c r="O585" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P585" s="2" t="inlineStr"/>
+      <c r="Q585" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R585" s="2" t="inlineStr"/>
+      <c r="S585" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" s="2" t="inlineStr">
+        <is>
+          <t>Jasmine Paolini</t>
+        </is>
+      </c>
+      <c r="B586" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C586" s="2" t="inlineStr">
+        <is>
+          <t>JASMINE PAOLINI Topps Chrome 2026 Tennis Aces Auto Red CASE HIT #5/5</t>
+        </is>
+      </c>
+      <c r="D586" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E586" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F586" s="2" t="inlineStr">
+        <is>
+          <t>949.99 USD</t>
+        </is>
+      </c>
+      <c r="G586" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/960010318634</t>
+        </is>
+      </c>
+      <c r="H586" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:55 UTC</t>
+        </is>
+      </c>
+      <c r="I586" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/s9gAAeSwimhqwbhO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J586" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T02:23:49.000Z</t>
+        </is>
+      </c>
+      <c r="K586" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L586" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M586" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N586" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/kucAAeSwXUBqwbhF/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O586" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P586" s="2" t="inlineStr"/>
+      <c r="Q586" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R586" s="2" t="inlineStr"/>
+      <c r="S586" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" s="2" t="inlineStr">
+        <is>
+          <t>Elina Svitolina</t>
+        </is>
+      </c>
+      <c r="B587" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C587" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Elina Svitolina Aces Auto Superfractor 1/1</t>
+        </is>
+      </c>
+      <c r="D587" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E587" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F587" s="2" t="inlineStr">
+        <is>
+          <t>2000.00 USD</t>
+        </is>
+      </c>
+      <c r="G587" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307212742310</t>
+        </is>
+      </c>
+      <c r="H587" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:55 UTC</t>
+        </is>
+      </c>
+      <c r="I587" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ZvMAAeSwgA5qwbe8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J587" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T02:22:07.000Z</t>
+        </is>
+      </c>
+      <c r="K587" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L587" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M587" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N587" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/VEEAAeSwyIdqwbfC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O587" s="2" t="inlineStr"/>
+      <c r="P587" s="2" t="inlineStr"/>
+      <c r="Q587" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R587" s="2" t="inlineStr"/>
+      <c r="S587" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="2" t="inlineStr">
+        <is>
+          <t>Donna Vekic</t>
+        </is>
+      </c>
+      <c r="B588" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C588" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Purple Geometric Refractor 15/15 Donna Vekic #48 Rookie RC ld5</t>
+        </is>
+      </c>
+      <c r="D588" s="2" t="inlineStr">
+        <is>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="E588" s="2" t="inlineStr">
+        <is>
+          <t>last of 15 (15/15)</t>
+        </is>
+      </c>
+      <c r="F588" s="2" t="inlineStr">
+        <is>
+          <t>58.32 USD</t>
+        </is>
+      </c>
+      <c r="G588" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237104737201</t>
+        </is>
+      </c>
+      <c r="H588" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:55 UTC</t>
+        </is>
+      </c>
+      <c r="I588" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TREAAeSwCbFqwbaK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J588" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T02:13:27.000Z</t>
+        </is>
+      </c>
+      <c r="K588" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L588" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M588" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N588" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0tIAAeSwFtBqwbaK/s-l1600.jpg | https://i.ebayimg.com/images/g/vpsAAeSwEWlqwbaK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O588" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P588" s="2" t="inlineStr"/>
+      <c r="Q588" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R588" s="2" t="inlineStr"/>
+      <c r="S588" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" s="2" t="inlineStr">
+        <is>
+          <t>Karen Khachanov</t>
+        </is>
+      </c>
+      <c r="B589" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C589" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis KAREN KHACHANOV #31 YELLOW REFRACTOR 1/275 1ST ONE</t>
+        </is>
+      </c>
+      <c r="D589" s="2" t="inlineStr">
+        <is>
+          <t>1/275</t>
+        </is>
+      </c>
+      <c r="E589" s="2" t="inlineStr">
+        <is>
+          <t>001 of 275</t>
+        </is>
+      </c>
+      <c r="F589" s="2" t="inlineStr">
+        <is>
+          <t>7.99 USD</t>
+        </is>
+      </c>
+      <c r="G589" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/206600752151</t>
+        </is>
+      </c>
+      <c r="H589" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:55 UTC</t>
+        </is>
+      </c>
+      <c r="I589" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/M4IAAeSw4dRqwbEs/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J589" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T01:55:18.000Z</t>
+        </is>
+      </c>
+      <c r="K589" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L589" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M589" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N589" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KAkAAeSwrRRqwbEu/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O589" s="2" t="inlineStr">
+        <is>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="P589" s="2" t="inlineStr"/>
+      <c r="Q589" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R589" s="2" t="inlineStr"/>
+      <c r="S589" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="2" t="inlineStr">
+        <is>
+          <t>Daniel Rincon</t>
+        </is>
+      </c>
+      <c r="B590" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C590" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Daniel Rincon Auto Green Refractor 99/99 #AT-DRN PI08</t>
+        </is>
+      </c>
+      <c r="D590" s="2" t="inlineStr">
+        <is>
+          <t>99/99</t>
+        </is>
+      </c>
+      <c r="E590" s="2" t="inlineStr">
+        <is>
+          <t>last of 99 (99/99)</t>
+        </is>
+      </c>
+      <c r="F590" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G590" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407264698178</t>
+        </is>
+      </c>
+      <c r="H590" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:55 UTC</t>
+        </is>
+      </c>
+      <c r="I590" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/h5wAAeSwRWxqwa1P/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J590" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T01:35:01.000Z</t>
+        </is>
+      </c>
+      <c r="K590" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L590" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M590" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N590" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/67wAAeSwCbFqwa1O/s-l1600.jpg | https://i.ebayimg.com/images/g/oy8AAeSwtupqwa1H/s-l1600.jpg | https://i.ebayimg.com/images/g/ipwAAeSwf-1qwa1H/s-l1600.jpg | https://i.ebayimg.com/images/g/QToAAeSwkJlqwa1H/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O590" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P590" s="2" t="inlineStr"/>
+      <c r="Q590" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R590" s="2" t="inlineStr"/>
+      <c r="S590" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" s="2" t="inlineStr">
+        <is>
+          <t>Danielle Collins</t>
+        </is>
+      </c>
+      <c r="B591" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C591" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis Danielle Collins 1st Gold Refractor 1/50 Lot*4 TT07</t>
+        </is>
+      </c>
+      <c r="D591" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E591" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F591" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G591" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407264697282</t>
+        </is>
+      </c>
+      <c r="H591" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:55 UTC</t>
+        </is>
+      </c>
+      <c r="I591" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TPkAAeSwfndqwa1Q/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J591" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T01:34:02.000Z</t>
+        </is>
+      </c>
+      <c r="K591" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L591" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M591" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N591" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TMgAAeSwgRpqwa1T/s-l1600.jpg | https://i.ebayimg.com/images/g/l90AAeSw78Vqwa1N/s-l1600.jpg | https://i.ebayimg.com/images/g/KiEAAeSwZztqwa1N/s-l1600.jpg | https://i.ebayimg.com/images/g/-HoAAeSwgA5qwa1N/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O591" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P591" s="2" t="inlineStr"/>
+      <c r="Q591" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R591" s="2" t="inlineStr"/>
+      <c r="S591" s="2" t="inlineStr"/>
+    </row>
+    <row r="592">
+      <c r="A592" s="2" t="inlineStr">
+        <is>
+          <t>Caroline Garcia</t>
+        </is>
+      </c>
+      <c r="B592" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C592" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Caroline Garcia Gold Refractor 1/50 #147 PI08</t>
+        </is>
+      </c>
+      <c r="D592" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E592" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F592" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G592" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407264696209</t>
+        </is>
+      </c>
+      <c r="H592" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:55 UTC</t>
+        </is>
+      </c>
+      <c r="I592" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JKoAAeSwtJFqwa0S/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J592" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T01:33:02.000Z</t>
+        </is>
+      </c>
+      <c r="K592" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M592" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N592" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/AvAAAeSwSaZqwa0V/s-l1600.jpg | https://i.ebayimg.com/images/g/56IAAeSwN1hqwa0P/s-l1600.jpg | https://i.ebayimg.com/images/g/AxEAAeSwn6dqwa0P/s-l1600.jpg | https://i.ebayimg.com/images/g/YYcAAeSwoDtqwa0P/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O592" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P592" s="2" t="inlineStr"/>
+      <c r="Q592" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R592" s="2" t="inlineStr"/>
+      <c r="S592" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" s="2" t="inlineStr">
+        <is>
+          <t>Peyton Stearns</t>
+        </is>
+      </c>
+      <c r="B593" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C593" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Peyton Stearns Auto Black Refractor 1/10 #AT-PSS PI08</t>
+        </is>
+      </c>
+      <c r="D593" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E593" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F593" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G593" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407264692752</t>
+        </is>
+      </c>
+      <c r="H593" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:55 UTC</t>
+        </is>
+      </c>
+      <c r="I593" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-6MAAeSwiWpqwaxv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J593" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T01:30:12.000Z</t>
+        </is>
+      </c>
+      <c r="K593" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L593" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M593" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N593" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/5R4AAeSw5XZqwaxz/s-l1600.jpg | https://i.ebayimg.com/images/g/3psAAeSwBGFqwaxs/s-l1600.jpg | https://i.ebayimg.com/images/g/8bkAAeSwpb1qwaxs/s-l1600.jpg | https://i.ebayimg.com/images/g/AsEAAeSw585qwaxs/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O593" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P593" s="2" t="inlineStr"/>
+      <c r="Q593" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R593" s="2" t="inlineStr"/>
+      <c r="S593" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" s="2" t="inlineStr">
+        <is>
+          <t>Vit Kopriva</t>
+        </is>
+      </c>
+      <c r="B594" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C594" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Pink Geometric Refractor 1/65 Vit Kopriva #72 Rookie RC 1cc7</t>
+        </is>
+      </c>
+      <c r="D594" s="2" t="inlineStr">
+        <is>
+          <t>1/65</t>
+        </is>
+      </c>
+      <c r="E594" s="2" t="inlineStr">
+        <is>
+          <t>001 of 65</t>
+        </is>
+      </c>
+      <c r="F594" s="2" t="inlineStr">
+        <is>
+          <t>11.75 USD</t>
+        </is>
+      </c>
+      <c r="G594" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257780649268</t>
+        </is>
+      </c>
+      <c r="H594" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:55 UTC</t>
+        </is>
+      </c>
+      <c r="I594" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-zMAAeSw9HBqwaq9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J594" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T01:14:16.000Z</t>
+        </is>
+      </c>
+      <c r="K594" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L594" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M594" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N594" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/59oAAeSw5oZqwaq~/s-l1600.jpg | https://i.ebayimg.com/images/g/M0UAAeSwgRpqwaq~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O594" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P594" s="2" t="inlineStr"/>
+      <c r="Q594" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R594" s="2" t="inlineStr"/>
+      <c r="S594" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" s="2" t="inlineStr">
+        <is>
+          <t>Abdullah Shelbayh</t>
+        </is>
+      </c>
+      <c r="B595" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C595" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Orange Refractor 25/25 Abdullah Shelbayh #172 Rookie RC 1cc7</t>
+        </is>
+      </c>
+      <c r="D595" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E595" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F595" s="2" t="inlineStr">
+        <is>
+          <t>9.74 USD</t>
+        </is>
+      </c>
+      <c r="G595" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336826128688</t>
+        </is>
+      </c>
+      <c r="H595" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:55 UTC</t>
+        </is>
+      </c>
+      <c r="I595" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/4doAAeSw60pqwaet/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J595" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T01:10:05.000Z</t>
+        </is>
+      </c>
+      <c r="K595" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L595" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M595" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N595" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/wk0AAeSwt~tqwaet/s-l1600.jpg | https://i.ebayimg.com/images/g/8bwAAeSweHNqwaet/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O595" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P595" s="2" t="inlineStr"/>
+      <c r="Q595" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R595" s="2" t="inlineStr"/>
+      <c r="S595" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" s="2" t="inlineStr">
+        <is>
+          <t>Nastasja Schunk</t>
+        </is>
+      </c>
+      <c r="B596" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C596" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Red Crystalline Refractor 1/1 Nastasja Schunk Rookie RC 1e41</t>
+        </is>
+      </c>
+      <c r="D596" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E596" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F596" s="2" t="inlineStr">
+        <is>
+          <t>166.75 USD</t>
+        </is>
+      </c>
+      <c r="G596" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257780905790</t>
+        </is>
+      </c>
+      <c r="H596" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:55 UTC</t>
+        </is>
+      </c>
+      <c r="I596" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/648AAeSwSohqwdge/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J596" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T04:36:47.000Z</t>
+        </is>
+      </c>
+      <c r="K596" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M596" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N596" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/r5UAAeSwoWtqwdge/s-l1600.jpg | https://i.ebayimg.com/images/g/9DUAAeSwmcFqwdge/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O596" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P596" s="2" t="inlineStr"/>
+      <c r="Q596" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R596" s="2" t="inlineStr"/>
+      <c r="S596" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" s="2" t="inlineStr">
+        <is>
+          <t>Daniil Medvedev</t>
+        </is>
+      </c>
+      <c r="B597" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS ROYALTY TENNIS SUPERIOR RELIC SIGNAT...</t>
+        </is>
+      </c>
+      <c r="C597" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS ROYALTY TENNIS SUPERIOR RELIC SIGNATURES DANIIL MEDVEDEV 1/5 PSA 8</t>
+        </is>
+      </c>
+      <c r="D597" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E597" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F597" s="2" t="inlineStr">
+        <is>
+          <t>598.79 USD</t>
+        </is>
+      </c>
+      <c r="G597" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117445108788</t>
+        </is>
+      </c>
+      <c r="H597" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:56 UTC</t>
+        </is>
+      </c>
+      <c r="I597" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8p4AAeSwm~FqwR5t/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J597" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T15:24:27.000Z</t>
+        </is>
+      </c>
+      <c r="K597" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L597" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M597" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 8</t>
+        </is>
+      </c>
+      <c r="N597" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/c5cAAeSwu9pqwR5t/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O597" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P597" s="2" t="inlineStr"/>
+      <c r="Q597" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R597" s="2" t="inlineStr"/>
+      <c r="S597" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -51761,6 +53173,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G579" r:id="rId578"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G580" r:id="rId579"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G581" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G582" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G583" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G584" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G585" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G586" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G587" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G588" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G589" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G590" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G591" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G592" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G593" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G594" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G595" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G596" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G597" r:id="rId596"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-05 12:44 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S597"/>
+  <dimension ref="A1:S602"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -52586,6 +52586,439 @@
       </c>
       <c r="R597" s="2" t="inlineStr"/>
       <c r="S597" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B598" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 TOPPS CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="C598" s="2" t="inlineStr">
+        <is>
+          <t>CARLOS ALCARAZ 2026 TOPPS CHROME TENNIS HOBBY 1/3 CASE 4 BOX PLAYER BREAK #3</t>
+        </is>
+      </c>
+      <c r="D598" s="2" t="inlineStr">
+        <is>
+          <t>1/3</t>
+        </is>
+      </c>
+      <c r="E598" s="2" t="inlineStr">
+        <is>
+          <t>001 of 3</t>
+        </is>
+      </c>
+      <c r="F598" s="2" t="inlineStr">
+        <is>
+          <t>5.99 USD</t>
+        </is>
+      </c>
+      <c r="G598" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/137811615072</t>
+        </is>
+      </c>
+      <c r="H598" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 12:43 UTC</t>
+        </is>
+      </c>
+      <c r="I598" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ULEAAeSwLbBqvs0y/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J598" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T23:30:00.000Z</t>
+        </is>
+      </c>
+      <c r="K598" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L598" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M598" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N598" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/w-cAAeSw~XZqvs1G/s-l1600.jpg | https://i.ebayimg.com/images/g/xsYAAeSwEBZqvs05/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O598" s="2" t="inlineStr"/>
+      <c r="P598" s="2" t="inlineStr"/>
+      <c r="Q598" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R598" s="2" t="inlineStr"/>
+      <c r="S598" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B599" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 TOPPS CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="C599" s="2" t="inlineStr">
+        <is>
+          <t>CARLOS ALCARAZ 2026 TOPPS CHROME TENNIS HOBBY 1/3 CASE 4 BOX PLAYER BREAK #2</t>
+        </is>
+      </c>
+      <c r="D599" s="2" t="inlineStr">
+        <is>
+          <t>1/3</t>
+        </is>
+      </c>
+      <c r="E599" s="2" t="inlineStr">
+        <is>
+          <t>001 of 3</t>
+        </is>
+      </c>
+      <c r="F599" s="2" t="inlineStr">
+        <is>
+          <t>6.50 USD</t>
+        </is>
+      </c>
+      <c r="G599" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147616453261</t>
+        </is>
+      </c>
+      <c r="H599" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 12:43 UTC</t>
+        </is>
+      </c>
+      <c r="I599" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ULEAAeSwLbBqvs0y/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J599" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T23:30:00.000Z</t>
+        </is>
+      </c>
+      <c r="K599" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L599" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M599" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N599" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/w-cAAeSw~XZqvs1G/s-l1600.jpg | https://i.ebayimg.com/images/g/xsYAAeSwEBZqvs05/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O599" s="2" t="inlineStr"/>
+      <c r="P599" s="2" t="inlineStr"/>
+      <c r="Q599" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R599" s="2" t="inlineStr"/>
+      <c r="S599" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B600" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C600" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2026 Topps Chrome Carlos Alcaraz #50 Black Raywave 10/10</t>
+        </is>
+      </c>
+      <c r="D600" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E600" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F600" s="2" t="inlineStr">
+        <is>
+          <t>2000.00 USD</t>
+        </is>
+      </c>
+      <c r="G600" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/960005394642</t>
+        </is>
+      </c>
+      <c r="H600" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 12:43 UTC</t>
+        </is>
+      </c>
+      <c r="I600" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Om4AAeSwttBqwEgG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J600" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T00:16:44.000Z</t>
+        </is>
+      </c>
+      <c r="K600" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L600" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M600" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N600" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bgQAAeSwAUVqwEf5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O600" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P600" s="2" t="inlineStr"/>
+      <c r="Q600" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R600" s="2" t="inlineStr"/>
+      <c r="S600" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B601" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 TOPPS CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="C601" s="2" t="inlineStr">
+        <is>
+          <t>CARLOS ALCARAZ 2026 TOPPS CHROME TENNIS HOBBY 1/3 CASE 4 BOX PLAYER BREAK #1</t>
+        </is>
+      </c>
+      <c r="D601" s="2" t="inlineStr">
+        <is>
+          <t>1/3</t>
+        </is>
+      </c>
+      <c r="E601" s="2" t="inlineStr">
+        <is>
+          <t>001 of 3</t>
+        </is>
+      </c>
+      <c r="F601" s="2" t="inlineStr">
+        <is>
+          <t>5.99 USD</t>
+        </is>
+      </c>
+      <c r="G601" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/860001997980</t>
+        </is>
+      </c>
+      <c r="H601" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 12:43 UTC</t>
+        </is>
+      </c>
+      <c r="I601" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ULEAAeSwLbBqvs0y/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J601" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T23:30:00.000Z</t>
+        </is>
+      </c>
+      <c r="K601" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L601" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M601" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N601" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/w-cAAeSw~XZqvs1G/s-l1600.jpg | https://i.ebayimg.com/images/g/xsYAAeSwEBZqvs05/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O601" s="2" t="inlineStr"/>
+      <c r="P601" s="2" t="inlineStr"/>
+      <c r="Q601" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R601" s="2" t="inlineStr"/>
+      <c r="S601" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B602" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Royalty</t>
+        </is>
+      </c>
+      <c r="C602" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Carlos Alcaraz 199/199 Teal Bookend 50</t>
+        </is>
+      </c>
+      <c r="D602" s="2" t="inlineStr">
+        <is>
+          <t>199/199</t>
+        </is>
+      </c>
+      <c r="E602" s="2" t="inlineStr">
+        <is>
+          <t>last of 199 (199/199)</t>
+        </is>
+      </c>
+      <c r="F602" s="2" t="inlineStr">
+        <is>
+          <t>137.99 USD</t>
+        </is>
+      </c>
+      <c r="G602" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336824055996</t>
+        </is>
+      </c>
+      <c r="H602" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 12:43 UTC</t>
+        </is>
+      </c>
+      <c r="I602" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/hqYAAeSwBU9qv-kR/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J602" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T17:26:09.000Z</t>
+        </is>
+      </c>
+      <c r="K602" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M602" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N602" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QicAAeSw3i9qv-kR/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O602" s="2" t="inlineStr">
+        <is>
+          <t>teal</t>
+        </is>
+      </c>
+      <c r="P602" s="2" t="inlineStr"/>
+      <c r="Q602" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R602" s="2" t="inlineStr"/>
+      <c r="S602" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -53189,6 +53622,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G595" r:id="rId594"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G596" r:id="rId595"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G597" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G598" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G599" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G600" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G601" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G602" r:id="rId601"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-05 18:44 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S602"/>
+  <dimension ref="A1:S627"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -53019,6 +53019,2215 @@
       </c>
       <c r="R602" s="2" t="inlineStr"/>
       <c r="S602" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" s="2" t="inlineStr">
+        <is>
+          <t>Terence Atmane</t>
+        </is>
+      </c>
+      <c r="B603" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Tennis Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C603" s="2" t="inlineStr">
+        <is>
+          <t>Terence Atmane 2025 Topps Chrome Tennis Sapphire Padparadscha Rookie RC 1/1 #175</t>
+        </is>
+      </c>
+      <c r="D603" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E603" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F603" s="2" t="inlineStr">
+        <is>
+          <t>799.99 USD</t>
+        </is>
+      </c>
+      <c r="G603" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287628757270</t>
+        </is>
+      </c>
+      <c r="H603" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I603" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/AdwAAeSwButqw-nC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J603" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T18:18:59.000Z</t>
+        </is>
+      </c>
+      <c r="K603" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L603" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M603" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N603" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/18AAAeSwzZpqw-nC/s-l1600.jpg | https://i.ebayimg.com/images/g/hg4AAeSwEWlqw-nB/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O603" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P603" s="2" t="inlineStr"/>
+      <c r="Q603" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R603" s="2" t="inlineStr"/>
+      <c r="S603" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="2" t="inlineStr">
+        <is>
+          <t>Aryna Sabalenka</t>
+        </is>
+      </c>
+      <c r="B604" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 topps chrome</t>
+        </is>
+      </c>
+      <c r="C604" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Aryna Sabalenka Auto Blue Geometric 001/150 SP #AO-ASA</t>
+        </is>
+      </c>
+      <c r="D604" s="2" t="inlineStr">
+        <is>
+          <t>1/150</t>
+        </is>
+      </c>
+      <c r="E604" s="2" t="inlineStr">
+        <is>
+          <t>001 of 150</t>
+        </is>
+      </c>
+      <c r="F604" s="2" t="inlineStr">
+        <is>
+          <t>391.24 USD</t>
+        </is>
+      </c>
+      <c r="G604" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/820206629946</t>
+        </is>
+      </c>
+      <c r="H604" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I604" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/E6kAAeSwr9Jqw88~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J604" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T16:25:21.000Z</t>
+        </is>
+      </c>
+      <c r="K604" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L604" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M604" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N604" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/FWUAAeSweydqw88~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O604" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P604" s="2" t="inlineStr"/>
+      <c r="Q604" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R604" s="2" t="inlineStr"/>
+      <c r="S604" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="2" t="inlineStr">
+        <is>
+          <t>Aryna Sabalenka</t>
+        </is>
+      </c>
+      <c r="B605" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C605" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024 Topps Chrome Tennis Aryna Sabalenka Superfractor 1/1 PSA 9 #21 Grail </t>
+        </is>
+      </c>
+      <c r="D605" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E605" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F605" s="2" t="inlineStr">
+        <is>
+          <t>49999.99 USD</t>
+        </is>
+      </c>
+      <c r="G605" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287628411382</t>
+        </is>
+      </c>
+      <c r="H605" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I605" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/43QAAeSwEWlqw7tk/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J605" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T15:01:01.000Z</t>
+        </is>
+      </c>
+      <c r="K605" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L605" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M605" s="2" t="inlineStr">
+        <is>
+          <t>PSA 9</t>
+        </is>
+      </c>
+      <c r="N605" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/s8kAAeSwZe5qw7tk/s-l1600.jpg | https://i.ebayimg.com/images/g/ng4AAeSwq-Jqw7tk/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O605" s="2" t="inlineStr"/>
+      <c r="P605" s="2" t="inlineStr"/>
+      <c r="Q605" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R605" s="2" t="inlineStr"/>
+      <c r="S605" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="2" t="inlineStr">
+        <is>
+          <t>Benoit Paire</t>
+        </is>
+      </c>
+      <c r="B606" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Chrome</t>
+        </is>
+      </c>
+      <c r="C606" s="2" t="inlineStr">
+        <is>
+          <t>Benoit Paire 2025 Topps Chrome Tennis #TCA-BPE Auto Black Refractor 01/10</t>
+        </is>
+      </c>
+      <c r="D606" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E606" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F606" s="2" t="inlineStr">
+        <is>
+          <t>15.00 USD</t>
+        </is>
+      </c>
+      <c r="G606" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117448759931?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2Fo%2Bmlm%2B5jOZv4dDg2pPmwZdy%2BQrZPBinuGBEHbVbN5UpkjwCSzHMOjHy5AkqGTDIlQJKa6y%2Bptww9brGztY27DELmKzfPbvh3VJ4uB0flfppWvMpAk8mgKbCiFiAg6me8fjluNMxTUEMZ5va8U%2BGizcfI5W1SBQ1Y12SRQFB7ngRx5N0QR52Cd98i35pLU7E4%3D</t>
+        </is>
+      </c>
+      <c r="H606" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I606" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/CIcAAeSwZQNqmZnL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J606" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T14:45:58.000Z</t>
+        </is>
+      </c>
+      <c r="K606" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M606" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N606" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ddwAAeSwcztqmZnL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O606" s="2" t="inlineStr">
+        <is>
+          <t>rose</t>
+        </is>
+      </c>
+      <c r="P606" s="2" t="inlineStr"/>
+      <c r="Q606" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R606" s="2" t="inlineStr"/>
+      <c r="S606" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" s="2" t="inlineStr">
+        <is>
+          <t>Gabriel Diallo</t>
+        </is>
+      </c>
+      <c r="B607" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C607" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS Gabriel Diallo  # 1/2 BLACK GEOMETRIC REFRACTOR</t>
+        </is>
+      </c>
+      <c r="D607" s="2" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="E607" s="2" t="inlineStr">
+        <is>
+          <t>001 of 2</t>
+        </is>
+      </c>
+      <c r="F607" s="2" t="inlineStr">
+        <is>
+          <t>100.00 USD</t>
+        </is>
+      </c>
+      <c r="G607" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117448752033?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8TTNAwXnxKHerKLP92FYnC1KtyamXVQ2Xrx%2BCgCo2JBtHfI%2B6UDWahjtBqjCdj2zGYkupHdSf5xswvtIGZHXY6c3zWiUbidafkUUBK9IJx8WYubwUkzpouXeBlfUhNDoZJ5PVTqy4chs74Bn07m6fjpzFMztZ9NYLcuqV%2BNOIxl%2FQLiS89i4MZ3oGPLoNc2cI%3D</t>
+        </is>
+      </c>
+      <c r="H607" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I607" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/wJoAAeSwrzppyS7-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J607" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T14:41:10.000Z</t>
+        </is>
+      </c>
+      <c r="K607" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L607" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M607" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N607" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/K-gAAeSw0z9pyS7-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O607" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P607" s="2" t="inlineStr"/>
+      <c r="Q607" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R607" s="2" t="inlineStr"/>
+      <c r="S607" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" s="2" t="inlineStr">
+        <is>
+          <t>Julia Riera</t>
+        </is>
+      </c>
+      <c r="B608" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C608" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Julia Riera RC Black Geometric 1/2</t>
+        </is>
+      </c>
+      <c r="D608" s="2" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="E608" s="2" t="inlineStr">
+        <is>
+          <t>001 of 2</t>
+        </is>
+      </c>
+      <c r="F608" s="2" t="inlineStr">
+        <is>
+          <t>150.00 USD</t>
+        </is>
+      </c>
+      <c r="G608" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117448720254?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde90uOZPqrruf2fEnS33FlqyRLNUYDwfDyVY4XIB2irdrmduT1y4W%2BrKFz6jSR6Dc8eglQEy6RZkP%2BhLuEFEfep85sGxxY%2F8FdtOUb7V5AQgKT%2Bk1%2BH2LtSrtbAwlxCXqAvEuL0amepnmlAlrUjTE%2F0yw9MhQ6%2B1OvQ2o%2B1vopbJ750Nl7yo2PAjlqtmLTgVT8Q%3D</t>
+        </is>
+      </c>
+      <c r="H608" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I608" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SokAAeSwnPZplzsi/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J608" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T14:17:10.000Z</t>
+        </is>
+      </c>
+      <c r="K608" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L608" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M608" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N608" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XYsAAeSwLYRplzsi/s-l1600.jpg | https://i.ebayimg.com/images/g/TNAAAeSwvSNplzsh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O608" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P608" s="2" t="inlineStr"/>
+      <c r="Q608" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R608" s="2" t="inlineStr"/>
+      <c r="S608" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="2" t="inlineStr">
+        <is>
+          <t>Marta Kostyuk</t>
+        </is>
+      </c>
+      <c r="B609" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C609" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis Marta Kostyuk Blue Refractor Auto 250/250</t>
+        </is>
+      </c>
+      <c r="D609" s="2" t="inlineStr">
+        <is>
+          <t>250/250</t>
+        </is>
+      </c>
+      <c r="E609" s="2" t="inlineStr">
+        <is>
+          <t>last of 250 (250/250)</t>
+        </is>
+      </c>
+      <c r="F609" s="2" t="inlineStr">
+        <is>
+          <t>50.00 USD</t>
+        </is>
+      </c>
+      <c r="G609" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117448717399?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2BsIc7ZPXh5LNeuPDikSp7HZHezEgr%2BIU67O6BvOQE0AKAHFPxg4ZfWjW4WxfoOWAxraq6FaTcza5JT%2FNKlXRYf8d4bb1rVQr3819nPcv89q8dFPW91C1YZegQFAy6rAumXanJW2iVmL%2BObb0TtrMifKNufVVR0eWec6bdaaw1QB0m3i6vg5TcJr2K8hHwi81s%3D</t>
+        </is>
+      </c>
+      <c r="H609" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I609" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/obMAAeSwzbZqmZ1n/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J609" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T14:12:39.000Z</t>
+        </is>
+      </c>
+      <c r="K609" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L609" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M609" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N609" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/T0cAAeSwJFFqmZ1n/s-l1600.jpg | https://i.ebayimg.com/images/g/CbEAAeSww-FqmZ1n/s-l1600.jpg | https://i.ebayimg.com/images/g/glIAAeSwuQVqmZ1n/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O609" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P609" s="2" t="inlineStr"/>
+      <c r="Q609" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R609" s="2" t="inlineStr"/>
+      <c r="S609" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" s="2" t="inlineStr">
+        <is>
+          <t>Gigi Fernandez</t>
+        </is>
+      </c>
+      <c r="B610" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C610" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Green Refractor 1/75 Gigi Fernandez Gigi Fernández #24 HOF ux8</t>
+        </is>
+      </c>
+      <c r="D610" s="2" t="inlineStr">
+        <is>
+          <t>1/75</t>
+        </is>
+      </c>
+      <c r="E610" s="2" t="inlineStr">
+        <is>
+          <t>001 of 75</t>
+        </is>
+      </c>
+      <c r="F610" s="2" t="inlineStr">
+        <is>
+          <t>9.73 USD</t>
+        </is>
+      </c>
+      <c r="G610" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336828591634</t>
+        </is>
+      </c>
+      <c r="H610" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I610" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uSsAAeSwVABqw18s/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J610" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T08:25:17.000Z</t>
+        </is>
+      </c>
+      <c r="K610" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L610" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M610" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N610" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/glkAAeSwuP5qw18s/s-l1600.jpg | https://i.ebayimg.com/images/g/d6IAAeSwADBqw18s/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O610" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P610" s="2" t="inlineStr"/>
+      <c r="Q610" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R610" s="2" t="inlineStr"/>
+      <c r="S610" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" s="2" t="inlineStr">
+        <is>
+          <t>Andy Murray</t>
+        </is>
+      </c>
+      <c r="B611" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Chrome</t>
+        </is>
+      </c>
+      <c r="C611" s="2" t="inlineStr">
+        <is>
+          <t>Andy Murray 2025 Topps Chrome Tennis Frozenfractor -1/0</t>
+        </is>
+      </c>
+      <c r="D611" s="2" t="inlineStr">
+        <is>
+          <t>1/0</t>
+        </is>
+      </c>
+      <c r="E611" s="2" t="inlineStr">
+        <is>
+          <t>001 of 0</t>
+        </is>
+      </c>
+      <c r="F611" s="2" t="inlineStr">
+        <is>
+          <t>249.99 USD</t>
+        </is>
+      </c>
+      <c r="G611" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/137813280855</t>
+        </is>
+      </c>
+      <c r="H611" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I611" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uR8AAeSwhlNqwxco/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J611" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T03:19:45.000Z</t>
+        </is>
+      </c>
+      <c r="K611" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L611" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M611" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N611" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/4GQAAeSwQ6Vqwxc1/s-l1600.jpg | https://i.ebayimg.com/images/g/hTIAAeSw--pqwxcy/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O611" s="2" t="inlineStr"/>
+      <c r="P611" s="2" t="inlineStr"/>
+      <c r="Q611" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R611" s="2" t="inlineStr"/>
+      <c r="S611" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="2" t="inlineStr">
+        <is>
+          <t>Andrey Rublev</t>
+        </is>
+      </c>
+      <c r="B612" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - [Base] - Red Geometric Refractor</t>
+        </is>
+      </c>
+      <c r="C612" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Red Geometric Refractor 1/5 Andrey Rublev #7 v9t</t>
+        </is>
+      </c>
+      <c r="D612" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E612" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F612" s="2" t="inlineStr">
+        <is>
+          <t>77.88 USD</t>
+        </is>
+      </c>
+      <c r="G612" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257782524513</t>
+        </is>
+      </c>
+      <c r="H612" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I612" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/15MAAeSw0zlqwxLl/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J612" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:59:51.000Z</t>
+        </is>
+      </c>
+      <c r="K612" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L612" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M612" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N612" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/lzEAAeSwEhdqwxLl/s-l1600.jpg | https://i.ebayimg.com/images/g/080AAeSw79ZqwxLl/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O612" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P612" s="2" t="inlineStr"/>
+      <c r="Q612" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R612" s="2" t="inlineStr"/>
+      <c r="S612" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" s="2" t="inlineStr">
+        <is>
+          <t>Frances Tiafoe</t>
+        </is>
+      </c>
+      <c r="B613" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Chrome</t>
+        </is>
+      </c>
+      <c r="C613" s="2" t="inlineStr">
+        <is>
+          <t>Frances Tiafoe 2026 Topps Chrome #93 Pink Refractor 1/250</t>
+        </is>
+      </c>
+      <c r="D613" s="2" t="inlineStr">
+        <is>
+          <t>1/250</t>
+        </is>
+      </c>
+      <c r="E613" s="2" t="inlineStr">
+        <is>
+          <t>001 of 250</t>
+        </is>
+      </c>
+      <c r="F613" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G613" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/960012974768</t>
+        </is>
+      </c>
+      <c r="H613" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I613" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-zQAAeSwCFxqwnta/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J613" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:58:00.000Z</t>
+        </is>
+      </c>
+      <c r="K613" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L613" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M613" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N613" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uVEAAeSwt-dqwnta/s-l1600.jpg | https://i.ebayimg.com/images/g/wa0AAeSwXvtqwnta/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O613" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P613" s="2" t="inlineStr"/>
+      <c r="Q613" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R613" s="2" t="inlineStr"/>
+      <c r="S613" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="2" t="inlineStr">
+        <is>
+          <t>Cameron Norrie</t>
+        </is>
+      </c>
+      <c r="B614" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS GRAPHITE CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="C614" s="2" t="inlineStr">
+        <is>
+          <t>Cameron Norrie 2024 Topps Graphite Tennis RED CRYSTALLINE 1/1 Match Masters</t>
+        </is>
+      </c>
+      <c r="D614" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E614" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F614" s="2" t="inlineStr">
+        <is>
+          <t>499.99 USD</t>
+        </is>
+      </c>
+      <c r="G614" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117448759914?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8JXSd4TEvAybvljj7IiEySnaZqQWxT8czG6Zf7Ai2yU%2FngxGpUrKgqzQVZj0QLRIzpeTWJdZxe9w3dD9uYP%2F7g4kFjZcbTPjbLysE2mV6lfyavtpRlFNH%2FuUarDLINzKPyfsptxNEqscLAcrwniv15CbErf7366VVhJNfCoba7qkuKh1N8UryQly4mXGYu6vs%3D</t>
+        </is>
+      </c>
+      <c r="H614" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I614" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/K4UAAOSwzr1noj~V/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J614" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T14:45:58.000Z</t>
+        </is>
+      </c>
+      <c r="K614" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L614" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M614" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N614" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Z9sAAOSwwd1noj~W/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O614" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P614" s="2" t="inlineStr"/>
+      <c r="Q614" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R614" s="2" t="inlineStr"/>
+      <c r="S614" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" s="2" t="inlineStr">
+        <is>
+          <t>Guilio Zeppieri</t>
+        </is>
+      </c>
+      <c r="B615" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C615" s="2" t="inlineStr">
+        <is>
+          <t>🎾 2024 Topps Graphite Tennis Red Crystalline Guilio Zeppieri 1/1</t>
+        </is>
+      </c>
+      <c r="D615" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E615" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F615" s="2" t="inlineStr">
+        <is>
+          <t>200.00 USD</t>
+        </is>
+      </c>
+      <c r="G615" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117448759826?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2B%2Fx4NVf1YK2b5h2XYfvtGdGg1O8UtHtm03192m3ElqqE1WwAQ%2BR7ADW6mkycPLINdTJG3MTm4OESbru%2Fk%2FgSBK23f5BeGuvPX8RF3QOE%2BBMWnQbmLJ1FMkW4tCayFsK6%2BAuZCZxTiwqpFl0Rir4nUskEJk9MIcW7RozfFn8UchGlYlA%2FpSzicIJWrlmnh86V0%3D</t>
+        </is>
+      </c>
+      <c r="H615" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I615" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7QQAAeSwjWtqohSn/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J615" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T14:45:57.000Z</t>
+        </is>
+      </c>
+      <c r="K615" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L615" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M615" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N615" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-QgAAeSwB7RqohSn/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O615" s="2" t="inlineStr"/>
+      <c r="P615" s="2" t="inlineStr"/>
+      <c r="Q615" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R615" s="2" t="inlineStr"/>
+      <c r="S615" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="2" t="inlineStr">
+        <is>
+          <t>Xiyu Wang</t>
+        </is>
+      </c>
+      <c r="B616" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C616" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Xiyu Wang White Refractor #10/10</t>
+        </is>
+      </c>
+      <c r="D616" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E616" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F616" s="2" t="inlineStr">
+        <is>
+          <t>11.00 USD</t>
+        </is>
+      </c>
+      <c r="G616" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117448722047?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2BDmQaauefasUP11Bkj82jqhZvT2b3xkiYTOEmcxZ2WPDqi4TxGO9tnr3QEQeg0qhI0eynWOs4jNoCMh2Fl1AYoY39pP7%2Fs6eWMFeS%2Bu7gdwWoBSCd3uOduHOPY%2BlPT%2BcRucsTdh%2Buf1V3SVtI%2BEypylOeUUCzT2h%2FV8WzunoT1F1N9%2BqLzLfduybSJKD4pBhg%3D</t>
+        </is>
+      </c>
+      <c r="H616" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I616" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Q6gAAeSwXbdp1bHJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J616" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T14:18:48.000Z</t>
+        </is>
+      </c>
+      <c r="K616" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L616" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M616" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N616" s="2" t="inlineStr"/>
+      <c r="O616" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P616" s="2" t="inlineStr"/>
+      <c r="Q616" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R616" s="2" t="inlineStr"/>
+      <c r="S616" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="2" t="inlineStr">
+        <is>
+          <t>Yulia Putintseva</t>
+        </is>
+      </c>
+      <c r="B617" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C617" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite #184 Yulia Putintseva Red Crystalline 1/1</t>
+        </is>
+      </c>
+      <c r="D617" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E617" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F617" s="2" t="inlineStr">
+        <is>
+          <t>399.99 USD</t>
+        </is>
+      </c>
+      <c r="G617" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/327388938846?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8QbzVeZDjpQOONmUFcZHisKv6QxEwRtuchfNhNU5Ld6cR9kRzX7ZGJH4%2FXWJCPo9nshegBKSUkDEFviAcW5lNXk8IHPiXovzhpxQqftFgFnXPO7zBMYmakBqLeHJ4zswaHnwHzbswJMj%2F5MtiZoaKr2YMgS%2BMbeNdBFwe87eKNtXNYHxtDbGSQEKb62dG%2FCs0%3D</t>
+        </is>
+      </c>
+      <c r="H617" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I617" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DEQAAeSwoYdqw0Gd/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J617" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T06:22:23.000Z</t>
+        </is>
+      </c>
+      <c r="K617" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L617" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M617" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N617" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/20sAAeSwfCZqw0Ge/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O617" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P617" s="2" t="inlineStr"/>
+      <c r="Q617" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R617" s="2" t="inlineStr"/>
+      <c r="S617" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="2" t="inlineStr">
+        <is>
+          <t>Elina Svitolina</t>
+        </is>
+      </c>
+      <c r="B618" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite Tennis</t>
+        </is>
+      </c>
+      <c r="C618" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Elina Svitolina Signature Serves Pink Auto 1/15 SIS-ES</t>
+        </is>
+      </c>
+      <c r="D618" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E618" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F618" s="2" t="inlineStr">
+        <is>
+          <t>12.28 USD</t>
+        </is>
+      </c>
+      <c r="G618" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168761921161</t>
+        </is>
+      </c>
+      <c r="H618" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I618" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/rcgAAeSwPjJqwvsT/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J618" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T01:19:31.000Z</t>
+        </is>
+      </c>
+      <c r="K618" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L618" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M618" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N618" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/tX8AAeSwYa5qwvsU/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O618" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P618" s="2" t="inlineStr"/>
+      <c r="Q618" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R618" s="2" t="inlineStr"/>
+      <c r="S618" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="2" t="inlineStr">
+        <is>
+          <t>Victoria Azarenka</t>
+        </is>
+      </c>
+      <c r="B619" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Relic Jewels - Green</t>
+        </is>
+      </c>
+      <c r="C619" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Relic Jewels Green 5/5 Victoria Azarenka #RCJ-VA 1e41</t>
+        </is>
+      </c>
+      <c r="D619" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E619" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F619" s="2" t="inlineStr">
+        <is>
+          <t>66.95 USD</t>
+        </is>
+      </c>
+      <c r="G619" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237108065371</t>
+        </is>
+      </c>
+      <c r="H619" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I619" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nHUAAeSwqrZqw-Y5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J619" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T18:01:29.000Z</t>
+        </is>
+      </c>
+      <c r="K619" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L619" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M619" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N619" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bYIAAeSweUNqw-Y6/s-l1600.jpg | https://i.ebayimg.com/images/g/W1MAAeSwyIdqw-Y5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O619" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P619" s="2" t="inlineStr"/>
+      <c r="Q619" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R619" s="2" t="inlineStr"/>
+      <c r="S619" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="2" t="inlineStr">
+        <is>
+          <t>Anna Kalinskaya</t>
+        </is>
+      </c>
+      <c r="B620" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Tennis</t>
+        </is>
+      </c>
+      <c r="C620" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis Anna Kalinskaya Pursuit Of Greatness Auto Platinum 1/1</t>
+        </is>
+      </c>
+      <c r="D620" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E620" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F620" s="2" t="inlineStr">
+        <is>
+          <t>3500.00 USD</t>
+        </is>
+      </c>
+      <c r="G620" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/189046774459</t>
+        </is>
+      </c>
+      <c r="H620" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I620" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/fGYAAeSwSohqw9Jo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J620" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T16:40:03.000Z</t>
+        </is>
+      </c>
+      <c r="K620" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L620" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M620" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N620" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/wPMAAeSw~hNqw9Hx/s-l1600.jpg | https://i.ebayimg.com/images/g/VxAAAeSw8qtqw9Hx/s-l1600.jpg | https://i.ebayimg.com/images/g/8moAAeSwVVRqw9Hv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O620" s="2" t="inlineStr"/>
+      <c r="P620" s="2" t="inlineStr"/>
+      <c r="Q620" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R620" s="2" t="inlineStr"/>
+      <c r="S620" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="2" t="inlineStr">
+        <is>
+          <t>Elena Rybakina</t>
+        </is>
+      </c>
+      <c r="B621" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS ROYALTY TENNIS REGALIA RELIC SIGNATURES</t>
+        </is>
+      </c>
+      <c r="C621" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS ROYALTY TENNIS REGALIA RELIC SIGNATURES ELENA RYBAKINA 1/10 PSA 9</t>
+        </is>
+      </c>
+      <c r="D621" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E621" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F621" s="2" t="inlineStr">
+        <is>
+          <t>2000.00 USD</t>
+        </is>
+      </c>
+      <c r="G621" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298734110602</t>
+        </is>
+      </c>
+      <c r="H621" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I621" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/OzUAAeSwOTVqw2OE/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J621" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T08:43:49.000Z</t>
+        </is>
+      </c>
+      <c r="K621" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L621" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M621" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N621" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/D2AAAeSweHNqw2OE/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O621" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P621" s="2" t="inlineStr"/>
+      <c r="Q621" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R621" s="2" t="inlineStr"/>
+      <c r="S621" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek</t>
+        </is>
+      </c>
+      <c r="B622" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS ROYALTY TENNIS AMBASSADOR AUTOGRAPHS</t>
+        </is>
+      </c>
+      <c r="C622" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS ROYALTY TENNIS AMBASSADOR AUTOS BLUE #AAIS IGA SWIATEK 1/25 PSA 9</t>
+        </is>
+      </c>
+      <c r="D622" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E622" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F622" s="2" t="inlineStr">
+        <is>
+          <t>2000.00 USD</t>
+        </is>
+      </c>
+      <c r="G622" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307214691874</t>
+        </is>
+      </c>
+      <c r="H622" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I622" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/5hgAAeSwAJ5qw13o/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J622" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T08:19:50.000Z</t>
+        </is>
+      </c>
+      <c r="K622" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L622" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M622" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N622" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/h04AAeSwniBqw13o/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O622" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P622" s="2" t="inlineStr"/>
+      <c r="Q622" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R622" s="2" t="inlineStr"/>
+      <c r="S622" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek</t>
+        </is>
+      </c>
+      <c r="B623" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS ROYALTY TENNIS SUPERIOR RELIC SIGNAT...</t>
+        </is>
+      </c>
+      <c r="C623" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS ROYALTY TENNIS SUPERIOR RELIC SIGNATURES BLUE IGA SWIATEK 25/25 PSA 8</t>
+        </is>
+      </c>
+      <c r="D623" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E623" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F623" s="2" t="inlineStr">
+        <is>
+          <t>1500.00 USD</t>
+        </is>
+      </c>
+      <c r="G623" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117448064747</t>
+        </is>
+      </c>
+      <c r="H623" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:43 UTC</t>
+        </is>
+      </c>
+      <c r="I623" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/D30AAeSwHVJqw13A/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J623" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T08:19:12.000Z</t>
+        </is>
+      </c>
+      <c r="K623" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L623" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M623" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 8</t>
+        </is>
+      </c>
+      <c r="N623" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3VAAAeSwzF9qw13A/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O623" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P623" s="2" t="inlineStr"/>
+      <c r="Q623" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R623" s="2" t="inlineStr"/>
+      <c r="S623" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="2" t="inlineStr">
+        <is>
+          <t>Taylor Fritz</t>
+        </is>
+      </c>
+      <c r="B624" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps</t>
+        </is>
+      </c>
+      <c r="C624" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis Taylor Fritz Regalia Relic Auto 5/5 #RRS-TFZ</t>
+        </is>
+      </c>
+      <c r="D624" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E624" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F624" s="2" t="inlineStr">
+        <is>
+          <t>6.50 USD</t>
+        </is>
+      </c>
+      <c r="G624" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/860008046624</t>
+        </is>
+      </c>
+      <c r="H624" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:44 UTC</t>
+        </is>
+      </c>
+      <c r="I624" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~hgAAeSwV9RqwopX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J624" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:54:00.000Z</t>
+        </is>
+      </c>
+      <c r="K624" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L624" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M624" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N624" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/lpYAAeSwc2FqwopY/s-l1600.jpg | https://i.ebayimg.com/images/g/AJgAAeSw2g1qwopY/s-l1600.jpg | https://i.ebayimg.com/images/g/lcQAAeSwfZZqwopZ/s-l1600.jpg | https://i.ebayimg.com/images/g/lX4AAeSw4GFqwopa/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O624" s="2" t="inlineStr"/>
+      <c r="P624" s="2" t="inlineStr"/>
+      <c r="Q624" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R624" s="2" t="inlineStr"/>
+      <c r="S624" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B625" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - [Base] - Blue</t>
+        </is>
+      </c>
+      <c r="C625" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Blue 1/25 Coco Gauff #50</t>
+        </is>
+      </c>
+      <c r="D625" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E625" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F625" s="2" t="inlineStr">
+        <is>
+          <t>9.99 USD</t>
+        </is>
+      </c>
+      <c r="G625" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237102586681</t>
+        </is>
+      </c>
+      <c r="H625" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:44 UTC</t>
+        </is>
+      </c>
+      <c r="I625" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9XMAAeSwlspqwAzJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J625" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:39:27.000Z</t>
+        </is>
+      </c>
+      <c r="K625" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L625" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M625" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N625" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QgcAAeSwUJNqwAzJ/s-l1600.jpg | https://i.ebayimg.com/images/g/1D4AAeSw16hqwAzJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O625" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P625" s="2" t="inlineStr"/>
+      <c r="Q625" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R625" s="2" t="inlineStr"/>
+      <c r="S625" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="2" t="inlineStr">
+        <is>
+          <t>Richarlison</t>
+        </is>
+      </c>
+      <c r="B626" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps</t>
+        </is>
+      </c>
+      <c r="C626" s="2" t="inlineStr">
+        <is>
+          <t>Richarlison - 2026 Topps Royalty EPL Black 10/10 Bookend Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="D626" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E626" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F626" s="2" t="inlineStr">
+        <is>
+          <t>30.00 USD</t>
+        </is>
+      </c>
+      <c r="G626" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/128114946573?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2FQ6BPKF0d7Ws0hMQlIq4N%2FRZKSHcRGs9n8fgN3CdfrDciVakMtBxXc3cs7gQ6vqsIhEJnIKUGoykdeOMenAeoyawjYzoYq0KF%2FFFCQrLg2DgTNMBJRpOQNnA16GqZAKpX3IbteYLQn5eEJk1fFFw81nYCLX1cjUPOpfbssRQSFVjgVOHY9khNAJwX2TV1EUJc%3D</t>
+        </is>
+      </c>
+      <c r="H626" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:44 UTC</t>
+        </is>
+      </c>
+      <c r="I626" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/i8gAAeSwG7pqwsdq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J626" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T21:41:31.000Z</t>
+        </is>
+      </c>
+      <c r="K626" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L626" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M626" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N626" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/rbQAAeSwFtBqwsdq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O626" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P626" s="2" t="inlineStr"/>
+      <c r="Q626" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R626" s="2" t="inlineStr">
+        <is>
+          <t>listing ticks 2 sports, which settles nothing; check by eye</t>
+        </is>
+      </c>
+      <c r="S626" s="2" t="inlineStr">
+        <is>
+          <t>Soccer, Futbol</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="2" t="inlineStr">
+        <is>
+          <t>Jim Courier</t>
+        </is>
+      </c>
+      <c r="B627" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic</t>
+        </is>
+      </c>
+      <c r="C627" s="2" t="inlineStr">
+        <is>
+          <t>2013 Ace Auth HOF Legends Blue 5/5 #JC1 Jim Courier PSA 10 (Top Pop, Pop 1)</t>
+        </is>
+      </c>
+      <c r="D627" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E627" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F627" s="2" t="inlineStr">
+        <is>
+          <t>275.00 USD</t>
+        </is>
+      </c>
+      <c r="G627" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168761975176</t>
+        </is>
+      </c>
+      <c r="H627" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:44 UTC</t>
+        </is>
+      </c>
+      <c r="I627" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/IcUAAOSwMRpj2aD2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J627" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T01:51:43.000Z</t>
+        </is>
+      </c>
+      <c r="K627" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L627" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M627" s="2" t="inlineStr">
+        <is>
+          <t>PSA 10</t>
+        </is>
+      </c>
+      <c r="N627" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/6EcAAOSw7R1j2aEA/s-l1600.jpg | https://i.ebayimg.com/images/g/ymIAAOSwictj2aEO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O627" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P627" s="2" t="inlineStr"/>
+      <c r="Q627" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R627" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic: check the numbering is stamped, not on a circle sticker</t>
+        </is>
+      </c>
+      <c r="S627" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -53627,6 +55836,31 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G600" r:id="rId599"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G601" r:id="rId600"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G602" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G603" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G604" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G605" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G606" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G607" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G608" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G609" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G610" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G611" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G612" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G613" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G614" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G615" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G616" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G617" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G618" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G619" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G620" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G621" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G622" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G623" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G624" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G625" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G626" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G627" r:id="rId626"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-06 03:55 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S627"/>
+  <dimension ref="A1:S630"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -55228,6 +55228,261 @@
         </is>
       </c>
       <c r="S627" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Nadal</t>
+        </is>
+      </c>
+      <c r="B628" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 TOPPS CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="C628" s="2" t="inlineStr">
+        <is>
+          <t>RAFAEL NADAL 2026 TOPPS CHROME TENNIS HOBBY 1/3 CASE 4 BOX PLAYER BREAK #3</t>
+        </is>
+      </c>
+      <c r="D628" s="2" t="inlineStr">
+        <is>
+          <t>1/3</t>
+        </is>
+      </c>
+      <c r="E628" s="2" t="inlineStr">
+        <is>
+          <t>001 of 3</t>
+        </is>
+      </c>
+      <c r="F628" s="2" t="inlineStr">
+        <is>
+          <t>5.99 USD</t>
+        </is>
+      </c>
+      <c r="G628" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/860007556264</t>
+        </is>
+      </c>
+      <c r="H628" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 03:55 UTC</t>
+        </is>
+      </c>
+      <c r="I628" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ULEAAeSwLbBqvs0y/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J628" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T00:18:00.000Z</t>
+        </is>
+      </c>
+      <c r="K628" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L628" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M628" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N628" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/w-cAAeSw~XZqvs1G/s-l1600.jpg | https://i.ebayimg.com/images/g/xsYAAeSwEBZqvs05/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O628" s="2" t="inlineStr"/>
+      <c r="P628" s="2" t="inlineStr"/>
+      <c r="Q628" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R628" s="2" t="inlineStr"/>
+      <c r="S628" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Nadal</t>
+        </is>
+      </c>
+      <c r="B629" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 TOPPS CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="C629" s="2" t="inlineStr">
+        <is>
+          <t>RAFAEL NADAL 2026 TOPPS CHROME TENNIS HOBBY 1/3 CASE 4 BOX PLAYER BREAK #2</t>
+        </is>
+      </c>
+      <c r="D629" s="2" t="inlineStr">
+        <is>
+          <t>1/3</t>
+        </is>
+      </c>
+      <c r="E629" s="2" t="inlineStr">
+        <is>
+          <t>001 of 3</t>
+        </is>
+      </c>
+      <c r="F629" s="2" t="inlineStr">
+        <is>
+          <t>5.99 USD</t>
+        </is>
+      </c>
+      <c r="G629" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/860003244909</t>
+        </is>
+      </c>
+      <c r="H629" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 03:55 UTC</t>
+        </is>
+      </c>
+      <c r="I629" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ULEAAeSwLbBqvs0y/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J629" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T00:18:00.000Z</t>
+        </is>
+      </c>
+      <c r="K629" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L629" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M629" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N629" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/w-cAAeSw~XZqvs1G/s-l1600.jpg | https://i.ebayimg.com/images/g/xsYAAeSwEBZqvs05/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O629" s="2" t="inlineStr"/>
+      <c r="P629" s="2" t="inlineStr"/>
+      <c r="Q629" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R629" s="2" t="inlineStr"/>
+      <c r="S629" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Nadal</t>
+        </is>
+      </c>
+      <c r="B630" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 TOPPS CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="C630" s="2" t="inlineStr">
+        <is>
+          <t>RAFAEL NADAL 2026 TOPPS CHROME TENNIS HOBBY 1/3 CASE 4 BOX PLAYER BREAK #1</t>
+        </is>
+      </c>
+      <c r="D630" s="2" t="inlineStr">
+        <is>
+          <t>1/3</t>
+        </is>
+      </c>
+      <c r="E630" s="2" t="inlineStr">
+        <is>
+          <t>001 of 3</t>
+        </is>
+      </c>
+      <c r="F630" s="2" t="inlineStr">
+        <is>
+          <t>5.99 USD</t>
+        </is>
+      </c>
+      <c r="G630" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/860001996761</t>
+        </is>
+      </c>
+      <c r="H630" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 03:55 UTC</t>
+        </is>
+      </c>
+      <c r="I630" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ULEAAeSwLbBqvs0y/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J630" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T00:18:00.000Z</t>
+        </is>
+      </c>
+      <c r="K630" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L630" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M630" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N630" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/w-cAAeSw~XZqvs1G/s-l1600.jpg | https://i.ebayimg.com/images/g/xsYAAeSwEBZqvs05/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O630" s="2" t="inlineStr"/>
+      <c r="P630" s="2" t="inlineStr"/>
+      <c r="Q630" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R630" s="2" t="inlineStr"/>
+      <c r="S630" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -55861,6 +56116,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G625" r:id="rId624"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G626" r:id="rId625"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G627" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G628" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G629" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G630" r:id="rId629"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-06 16:08 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S630"/>
+  <dimension ref="A1:S656"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -55483,6 +55483,2308 @@
       </c>
       <c r="R630" s="2" t="inlineStr"/>
       <c r="S630" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="2" t="inlineStr">
+        <is>
+          <t>Ivan Lendl</t>
+        </is>
+      </c>
+      <c r="B631" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C631" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Ivan Lendl Superfractor 1/1 - FIRST TOPPS CHROME CARD</t>
+        </is>
+      </c>
+      <c r="D631" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E631" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F631" s="2" t="inlineStr">
+        <is>
+          <t>5999.99 USD</t>
+        </is>
+      </c>
+      <c r="G631" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366715916608</t>
+        </is>
+      </c>
+      <c r="H631" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I631" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Mw0AAeSwmZdqxRUO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J631" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T15:39:51.000Z</t>
+        </is>
+      </c>
+      <c r="K631" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L631" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M631" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N631" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/suIAAeSwaYpqxRUP/s-l1600.jpg | https://i.ebayimg.com/images/g/MFkAAeSwI7ZqxRUP/s-l1600.jpg | https://i.ebayimg.com/images/g/~4sAAeSwD1JqxRUP/s-l1600.jpg | https://i.ebayimg.com/images/g/CgIAAeSwH99qxRUP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O631" s="2" t="inlineStr"/>
+      <c r="P631" s="2" t="inlineStr"/>
+      <c r="Q631" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R631" s="2" t="inlineStr"/>
+      <c r="S631" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="2" t="inlineStr">
+        <is>
+          <t>Peyton Stearns</t>
+        </is>
+      </c>
+      <c r="B632" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C632" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Peyton Stearns Youthquake 01/50 Gold Geometric #YQ-PS</t>
+        </is>
+      </c>
+      <c r="D632" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E632" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F632" s="2" t="inlineStr">
+        <is>
+          <t>12.99 USD</t>
+        </is>
+      </c>
+      <c r="G632" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287631277874</t>
+        </is>
+      </c>
+      <c r="H632" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I632" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/phEAAeSwJxpqxRXJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J632" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T15:38:41.000Z</t>
+        </is>
+      </c>
+      <c r="K632" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L632" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M632" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N632" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/K7IAAeSwPV5qxRXJ/s-l1600.jpg | https://i.ebayimg.com/images/g/naEAAeSwwSlqxRXI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O632" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P632" s="2" t="inlineStr"/>
+      <c r="Q632" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R632" s="2" t="inlineStr"/>
+      <c r="S632" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="2" t="inlineStr">
+        <is>
+          <t>Renata Jamrichova</t>
+        </is>
+      </c>
+      <c r="B633" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C633" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Renata Jamrichova TRUE RED 1ST on Print 1/5</t>
+        </is>
+      </c>
+      <c r="D633" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E633" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F633" s="2" t="inlineStr">
+        <is>
+          <t>400.00 USD</t>
+        </is>
+      </c>
+      <c r="G633" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/189051958495?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde9jEVqNQxh7HWGNiOMgCsWYQz%2FVsaoB3d%2BnANPxz6ikdqGnnBPZUYHPeZQHw1m3iZTjjYfWQP5uVzLYmoRClzXzoKE2KgGtsk5AGFklDeZEYj%2Fvo21WrYOjx6YbbNuLmUn3uTlVNtnDryGpV8hwowjMuzmV5Zb3I7eqkEW1fnwYnpGTzIp3mWg65cQRqv4VhGI%3D</t>
+        </is>
+      </c>
+      <c r="H633" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I633" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/VSsAAeSw87lqxREC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J633" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T15:17:49.000Z</t>
+        </is>
+      </c>
+      <c r="K633" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L633" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M633" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N633" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/wGAAAeSwTPNqxREH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O633" s="2" t="inlineStr"/>
+      <c r="P633" s="2" t="inlineStr"/>
+      <c r="Q633" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R633" s="2" t="inlineStr"/>
+      <c r="S633" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="2" t="inlineStr">
+        <is>
+          <t>Jakub Mensik</t>
+        </is>
+      </c>
+      <c r="B634" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C634" s="2" t="inlineStr">
+        <is>
+          <t>Topps Chrome Tennis 2026 Jakub Mensik Black Refractor 1/10</t>
+        </is>
+      </c>
+      <c r="D634" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E634" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F634" s="2" t="inlineStr">
+        <is>
+          <t>225.00 USD</t>
+        </is>
+      </c>
+      <c r="G634" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/278439667893</t>
+        </is>
+      </c>
+      <c r="H634" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I634" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jZYAAeSwp1NqxPzd/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J634" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T13:52:10.000Z</t>
+        </is>
+      </c>
+      <c r="K634" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L634" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M634" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N634" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/S8EAAeSwihBqxPze/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O634" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P634" s="2" t="inlineStr"/>
+      <c r="Q634" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R634" s="2" t="inlineStr"/>
+      <c r="S634" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="2" t="inlineStr">
+        <is>
+          <t>Victoria Azarenka</t>
+        </is>
+      </c>
+      <c r="B635" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C635" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Victoria Azarenka World No. 1 Auto NO-VA 1/5 Red</t>
+        </is>
+      </c>
+      <c r="D635" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E635" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F635" s="2" t="inlineStr">
+        <is>
+          <t>149.95 USD</t>
+        </is>
+      </c>
+      <c r="G635" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366715552155</t>
+        </is>
+      </c>
+      <c r="H635" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I635" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/m0QAAeSw7PpqxPNi/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J635" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T13:12:33.000Z</t>
+        </is>
+      </c>
+      <c r="K635" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L635" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M635" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N635" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/q8MAAeSwwqpqxPNx/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O635" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P635" s="2" t="inlineStr"/>
+      <c r="Q635" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R635" s="2" t="inlineStr"/>
+      <c r="S635" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="2" t="inlineStr">
+        <is>
+          <t>Louisa Chirico</t>
+        </is>
+      </c>
+      <c r="B636" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C636" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Louisa Chirico CA-LCO Auto Orange I Geo 1/25</t>
+        </is>
+      </c>
+      <c r="D636" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E636" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F636" s="2" t="inlineStr">
+        <is>
+          <t>0.40 USD</t>
+        </is>
+      </c>
+      <c r="G636" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366715529831</t>
+        </is>
+      </c>
+      <c r="H636" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I636" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/sLMAAeSwc~RqxPE-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J636" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T13:03:04.000Z</t>
+        </is>
+      </c>
+      <c r="K636" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L636" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M636" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N636" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gncAAeSwiGpqxPEx/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O636" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P636" s="2" t="inlineStr"/>
+      <c r="Q636" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R636" s="2" t="inlineStr"/>
+      <c r="S636" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="2" t="inlineStr">
+        <is>
+          <t>Mackie McDonald</t>
+        </is>
+      </c>
+      <c r="B637" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C637" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Sapphire II Purple 10/10 Mackie McDonald Mackenzie Auto 1d0h</t>
+        </is>
+      </c>
+      <c r="D637" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E637" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F637" s="2" t="inlineStr">
+        <is>
+          <t>57.18 USD</t>
+        </is>
+      </c>
+      <c r="G637" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336830947524</t>
+        </is>
+      </c>
+      <c r="H637" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I637" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0kcAAeSwtChqxNYN/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J637" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T11:04:46.000Z</t>
+        </is>
+      </c>
+      <c r="K637" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L637" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M637" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N637" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/GIUAAeSwqAFqxNYN/s-l1600.jpg | https://i.ebayimg.com/images/g/YU4AAeSwwcNqxNYN/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O637" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P637" s="2" t="inlineStr"/>
+      <c r="Q637" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R637" s="2" t="inlineStr"/>
+      <c r="S637" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="2" t="inlineStr">
+        <is>
+          <t>Daniil Medvedev</t>
+        </is>
+      </c>
+      <c r="B638" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C638" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Sapphire Orange 1/25 Daniil Medvedev #25 1d0h</t>
+        </is>
+      </c>
+      <c r="D638" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E638" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F638" s="2" t="inlineStr">
+        <is>
+          <t>110.08 USD</t>
+        </is>
+      </c>
+      <c r="G638" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336830902042</t>
+        </is>
+      </c>
+      <c r="H638" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I638" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~pkAAeSwwcNqxM9X/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J638" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T10:36:06.000Z</t>
+        </is>
+      </c>
+      <c r="K638" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L638" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M638" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N638" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uYgAAeSwm~FqxM9X/s-l1600.jpg | https://i.ebayimg.com/images/g/WMwAAeSwt~tqxM9X/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O638" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P638" s="2" t="inlineStr"/>
+      <c r="Q638" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R638" s="2" t="inlineStr"/>
+      <c r="S638" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="2" t="inlineStr">
+        <is>
+          <t>Ken Rosewall</t>
+        </is>
+      </c>
+      <c r="B639" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C639" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Blue RayWave Refractor 1/99 Ken Rosewall #23 HOF 7eo</t>
+        </is>
+      </c>
+      <c r="D639" s="2" t="inlineStr">
+        <is>
+          <t>1/99</t>
+        </is>
+      </c>
+      <c r="E639" s="2" t="inlineStr">
+        <is>
+          <t>001 of 99</t>
+        </is>
+      </c>
+      <c r="F639" s="2" t="inlineStr">
+        <is>
+          <t>12.33 USD</t>
+        </is>
+      </c>
+      <c r="G639" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257785366286</t>
+        </is>
+      </c>
+      <c r="H639" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I639" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/6nUAAeSw5AlqxMvH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J639" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T10:20:55.000Z</t>
+        </is>
+      </c>
+      <c r="K639" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L639" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M639" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N639" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7i0AAeSwZ2hqxMvH/s-l1600.jpg | https://i.ebayimg.com/images/g/Yh0AAeSw5XZqxMvH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O639" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P639" s="2" t="inlineStr"/>
+      <c r="Q639" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R639" s="2" t="inlineStr"/>
+      <c r="S639" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="2" t="inlineStr">
+        <is>
+          <t>Aljaz Bedene</t>
+        </is>
+      </c>
+      <c r="B640" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C640" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Gold Wave Refractor 1/50 Aljaz Bedene Aljaž #5 Rookie RC 14dq</t>
+        </is>
+      </c>
+      <c r="D640" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E640" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F640" s="2" t="inlineStr">
+        <is>
+          <t>12.32 USD</t>
+        </is>
+      </c>
+      <c r="G640" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336830834095</t>
+        </is>
+      </c>
+      <c r="H640" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I640" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/4ekAAeSw6HJqxMck/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J640" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T10:01:06.000Z</t>
+        </is>
+      </c>
+      <c r="K640" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L640" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M640" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N640" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/NKIAAeSwXvtqxMck/s-l1600.jpg | https://i.ebayimg.com/images/g/cNQAAeSwCAxqxMck/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O640" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P640" s="2" t="inlineStr"/>
+      <c r="Q640" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R640" s="2" t="inlineStr"/>
+      <c r="S640" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="2" t="inlineStr">
+        <is>
+          <t>Francisco Comesana</t>
+        </is>
+      </c>
+      <c r="B641" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C641" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Francisco Comesana RC 01/75 Purple Refractor #11</t>
+        </is>
+      </c>
+      <c r="D641" s="2" t="inlineStr">
+        <is>
+          <t>1/75</t>
+        </is>
+      </c>
+      <c r="E641" s="2" t="inlineStr">
+        <is>
+          <t>001 of 75</t>
+        </is>
+      </c>
+      <c r="F641" s="2" t="inlineStr">
+        <is>
+          <t>15.00 USD</t>
+        </is>
+      </c>
+      <c r="G641" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366715020277</t>
+        </is>
+      </c>
+      <c r="H641" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I641" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8hwAAeSw5oZqxMIi/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J641" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T09:42:01.000Z</t>
+        </is>
+      </c>
+      <c r="K641" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L641" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M641" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA)</t>
+        </is>
+      </c>
+      <c r="N641" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/lP4AAeSwZPtqxMIh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O641" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P641" s="2" t="inlineStr"/>
+      <c r="Q641" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R641" s="2" t="inlineStr"/>
+      <c r="S641" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="2" t="inlineStr">
+        <is>
+          <t>Eva Lys</t>
+        </is>
+      </c>
+      <c r="B642" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C642" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Eva Lys True Blue Refractor On-Card Auto 001/150</t>
+        </is>
+      </c>
+      <c r="D642" s="2" t="inlineStr">
+        <is>
+          <t>1/150</t>
+        </is>
+      </c>
+      <c r="E642" s="2" t="inlineStr">
+        <is>
+          <t>001 of 150</t>
+        </is>
+      </c>
+      <c r="F642" s="2" t="inlineStr">
+        <is>
+          <t>174.30 USD</t>
+        </is>
+      </c>
+      <c r="G642" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/227554552928?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde9VBUaqaA8JGiiXIWbYE4331IaT%2B75y8TOUe5tIkua5H%2F5yWmihYCZeBUmau3QOcSflFfrsPKbhRHJM5Q%2Fj0NqGPknZ1KUAm%2BOcKAMY5IMmlwpLoyyiXG2%2FjUZDw7iwcD9dWW1iNYUkAwACIzsNYm%2FLvwpQBCeTqwLgctxrCsYqUrFyCZGAfRBUSeTgh84e2io%3D</t>
+        </is>
+      </c>
+      <c r="H642" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I642" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/710AAeSwH1FqxJuy/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J642" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T06:59:38.000Z</t>
+        </is>
+      </c>
+      <c r="K642" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L642" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M642" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N642" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8uEAAeSwniBqxJuz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O642" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P642" s="2" t="inlineStr"/>
+      <c r="Q642" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R642" s="2" t="inlineStr"/>
+      <c r="S642" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="2" t="inlineStr">
+        <is>
+          <t>Harry Wendelken</t>
+        </is>
+      </c>
+      <c r="B643" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C643" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome I Rose Gold Refractor 1/20 Harry Wendelken #TCA-HWN Auto pe8</t>
+        </is>
+      </c>
+      <c r="D643" s="2" t="inlineStr">
+        <is>
+          <t>1/20</t>
+        </is>
+      </c>
+      <c r="E643" s="2" t="inlineStr">
+        <is>
+          <t>001 of 20</t>
+        </is>
+      </c>
+      <c r="F643" s="2" t="inlineStr">
+        <is>
+          <t>14.63 USD</t>
+        </is>
+      </c>
+      <c r="G643" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237109286925</t>
+        </is>
+      </c>
+      <c r="H643" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I643" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/oQ4AAeSwSk9qxJLh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J643" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T06:18:11.000Z</t>
+        </is>
+      </c>
+      <c r="K643" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L643" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M643" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N643" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~9YAAeSwOTVqxJLi/s-l1600.jpg | https://i.ebayimg.com/images/g/jooAAeSwEFNqxJLi/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O643" s="2" t="inlineStr">
+        <is>
+          <t>rose</t>
+        </is>
+      </c>
+      <c r="P643" s="2" t="inlineStr"/>
+      <c r="Q643" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R643" s="2" t="inlineStr"/>
+      <c r="S643" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="2" t="inlineStr">
+        <is>
+          <t>Jakub Mensik</t>
+        </is>
+      </c>
+      <c r="B644" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - [Base] - Black Geometric Refractor</t>
+        </is>
+      </c>
+      <c r="C644" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Black Geometric Refractor 2/2 Jakub Mensik #75 1e41</t>
+        </is>
+      </c>
+      <c r="D644" s="2" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="E644" s="2" t="inlineStr">
+        <is>
+          <t>last of 2 (2/2)</t>
+        </is>
+      </c>
+      <c r="F644" s="2" t="inlineStr">
+        <is>
+          <t>449.99 USD</t>
+        </is>
+      </c>
+      <c r="G644" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257784814574</t>
+        </is>
+      </c>
+      <c r="H644" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I644" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/UtkAAeSw5AlqxIeW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J644" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T05:29:59.000Z</t>
+        </is>
+      </c>
+      <c r="K644" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L644" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M644" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N644" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/LqUAAeSwGNdqxIeW/s-l1600.jpg | https://i.ebayimg.com/images/g/GUkAAeSwznhqxIeW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O644" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P644" s="2" t="inlineStr"/>
+      <c r="Q644" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R644" s="2" t="inlineStr"/>
+      <c r="S644" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="2" t="inlineStr">
+        <is>
+          <t>Taylor Fritz</t>
+        </is>
+      </c>
+      <c r="B645" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C645" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Captured Taylor Fritz Orange #01/25 #CTD-TF</t>
+        </is>
+      </c>
+      <c r="D645" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E645" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F645" s="2" t="inlineStr">
+        <is>
+          <t>24.99 USD</t>
+        </is>
+      </c>
+      <c r="G645" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/137817001488</t>
+        </is>
+      </c>
+      <c r="H645" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I645" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/lTwAAeSwclBqxHoG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J645" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T04:33:48.000Z</t>
+        </is>
+      </c>
+      <c r="K645" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L645" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M645" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N645" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QV4AAeSwpb1qxHoT/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O645" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P645" s="2" t="inlineStr"/>
+      <c r="Q645" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R645" s="2" t="inlineStr"/>
+      <c r="S645" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="2" t="inlineStr">
+        <is>
+          <t>Raphael Collignon</t>
+        </is>
+      </c>
+      <c r="B646" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C646" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Raphael Collignon Orange Geometric 25/25 Book End</t>
+        </is>
+      </c>
+      <c r="D646" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E646" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F646" s="2" t="inlineStr">
+        <is>
+          <t>17.99 USD</t>
+        </is>
+      </c>
+      <c r="G646" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/137816888153?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2FLpEiunfbjj65oAGiAW99SoLSw1g8Qp3%2BXHNBd3t%2F6qd0hM2dnhqTYJiPfpty8YVXKIskc2QRtDER6XqVoQRXKzm4V5L7RL23Z0p7KN6b6jR3pVDmx4ppE4ILtJ0dO1QnKBjDfegsFIt4iqMpc7QDk8XiXjPWSHy6cL35OC4HV5H4BNdXJQtfk2qMNe0sBSwY%3D</t>
+        </is>
+      </c>
+      <c r="H646" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I646" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/GSAAAeSwynBqxHAg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J646" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T03:53:53.000Z</t>
+        </is>
+      </c>
+      <c r="K646" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L646" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M646" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N646" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/aYsAAeSwUMVqxHAg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O646" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P646" s="2" t="inlineStr"/>
+      <c r="Q646" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R646" s="2" t="inlineStr"/>
+      <c r="S646" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="2" t="inlineStr">
+        <is>
+          <t>Matteo Gigante</t>
+        </is>
+      </c>
+      <c r="B647" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C647" s="2" t="inlineStr">
+        <is>
+          <t>Matteo Gigante 2026 Topps Chrome Tennis 25/25 Orange Geometric Auto AT-MGE</t>
+        </is>
+      </c>
+      <c r="D647" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E647" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F647" s="2" t="inlineStr">
+        <is>
+          <t>69.99 USD</t>
+        </is>
+      </c>
+      <c r="G647" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377547303446?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde9N0ItHEb76wAoU1943%2B6UR%2BuJTF2AnOVNoD9pDQsAxP1LLXmJtAgF3IWeM6u1VAyRn7G2FXjyCuC4kj5bHIXhRv62IFLEtKf3PWPZwX6eROD3BDrFTIAlUTWw3QeBsOrwtqH2sH8G6PCtavja8ZgGcHZDn%2FVAin5zizGqTsirWmJtUy8I4S7qtj4cktiiI8a0%3D</t>
+        </is>
+      </c>
+      <c r="H647" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I647" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nzEAAeSwSk9qxGaH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J647" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T03:18:47.000Z</t>
+        </is>
+      </c>
+      <c r="K647" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L647" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M647" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N647" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nzAAAeSwSk9qxGaH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O647" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P647" s="2" t="inlineStr"/>
+      <c r="Q647" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R647" s="2" t="inlineStr"/>
+      <c r="S647" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="2" t="inlineStr">
+        <is>
+          <t>Emma Navarro</t>
+        </is>
+      </c>
+      <c r="B648" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C648" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Destiny Emma Navarro orange refractor #25/25 LAST ONE!</t>
+        </is>
+      </c>
+      <c r="D648" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E648" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F648" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G648" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/206605777941</t>
+        </is>
+      </c>
+      <c r="H648" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I648" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/V~wAAeSwD1JqxF-x/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J648" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T02:41:04.000Z</t>
+        </is>
+      </c>
+      <c r="K648" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L648" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M648" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N648" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/poQAAeSwG~dqxF-x/s-l1600.jpg | https://i.ebayimg.com/images/g/YdAAAeSwtY1qxF-y/s-l1600.jpg | https://i.ebayimg.com/images/g/Ga0AAeSwPGFqxF-y/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O648" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P648" s="2" t="inlineStr"/>
+      <c r="Q648" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R648" s="2" t="inlineStr"/>
+      <c r="S648" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="2" t="inlineStr">
+        <is>
+          <t>Qinwen Zheng</t>
+        </is>
+      </c>
+      <c r="B649" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C649" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Qinwen Zheng true green refractor #99/99 LAST ONE MADE!</t>
+        </is>
+      </c>
+      <c r="D649" s="2" t="inlineStr">
+        <is>
+          <t>99/99</t>
+        </is>
+      </c>
+      <c r="E649" s="2" t="inlineStr">
+        <is>
+          <t>last of 99 (99/99)</t>
+        </is>
+      </c>
+      <c r="F649" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G649" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/206605773369</t>
+        </is>
+      </c>
+      <c r="H649" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I649" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DVQAAeSwf-1qxF6R/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J649" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T02:36:19.000Z</t>
+        </is>
+      </c>
+      <c r="K649" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L649" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M649" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N649" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/dVgAAeSwButqxF6R/s-l1600.jpg | https://i.ebayimg.com/images/g/qn4AAeSw4tZqxF6S/s-l1600.jpg | https://i.ebayimg.com/images/g/bI4AAeSwAUVqxF6S/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O649" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P649" s="2" t="inlineStr"/>
+      <c r="Q649" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R649" s="2" t="inlineStr"/>
+      <c r="S649" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="2" t="inlineStr">
+        <is>
+          <t>Ryan Harrison</t>
+        </is>
+      </c>
+      <c r="B650" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C650" s="2" t="inlineStr">
+        <is>
+          <t>2024 Graphite Tour Relic Pink Refractor 1/15 Ryan Harrison Rookie Auto RC ld5</t>
+        </is>
+      </c>
+      <c r="D650" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E650" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F650" s="2" t="inlineStr">
+        <is>
+          <t>18.07 USD</t>
+        </is>
+      </c>
+      <c r="G650" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237110162130</t>
+        </is>
+      </c>
+      <c r="H650" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I650" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/GjAAAeSwc~RqxPhe/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J650" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T13:30:59.000Z</t>
+        </is>
+      </c>
+      <c r="K650" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L650" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M650" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N650" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/w~kAAeSwzvFqxPhe/s-l1600.jpg | https://i.ebayimg.com/images/g/rjoAAeSw7Z5qxPhf/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O650" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P650" s="2" t="inlineStr"/>
+      <c r="Q650" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R650" s="2" t="inlineStr"/>
+      <c r="S650" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="2" t="inlineStr">
+        <is>
+          <t>Liv Hovde</t>
+        </is>
+      </c>
+      <c r="B651" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C651" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Blue Refractor 50/50 Liv Hovde #GSR-LHE Rookie Auto RC 1o52</t>
+        </is>
+      </c>
+      <c r="D651" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E651" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F651" s="2" t="inlineStr">
+        <is>
+          <t>21.24 USD</t>
+        </is>
+      </c>
+      <c r="G651" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336831120924</t>
+        </is>
+      </c>
+      <c r="H651" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I651" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ChsAAeSwTRhqxOzv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J651" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T12:42:24.000Z</t>
+        </is>
+      </c>
+      <c r="K651" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L651" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M651" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N651" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/W0kAAeSwoL5qxOzv/s-l1600.jpg | https://i.ebayimg.com/images/g/9dgAAeSw~kFqxOzv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O651" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P651" s="2" t="inlineStr"/>
+      <c r="Q651" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R651" s="2" t="inlineStr"/>
+      <c r="S651" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="2" t="inlineStr">
+        <is>
+          <t>Miomir Kecmanovic</t>
+        </is>
+      </c>
+      <c r="B652" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C652" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Green Refractor 1/75 Miomir Kecmanovic Rookie Auto RC 03j5</t>
+        </is>
+      </c>
+      <c r="D652" s="2" t="inlineStr">
+        <is>
+          <t>1/75</t>
+        </is>
+      </c>
+      <c r="E652" s="2" t="inlineStr">
+        <is>
+          <t>001 of 75</t>
+        </is>
+      </c>
+      <c r="F652" s="2" t="inlineStr">
+        <is>
+          <t>10.03 USD</t>
+        </is>
+      </c>
+      <c r="G652" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237109222180</t>
+        </is>
+      </c>
+      <c r="H652" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I652" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2qwAAeSwxn9qxIuX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J652" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T05:47:04.000Z</t>
+        </is>
+      </c>
+      <c r="K652" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L652" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M652" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N652" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/etAAAeSw7plqxIuX/s-l1600.jpg | https://i.ebayimg.com/images/g/UFgAAeSwAOdqxIuX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O652" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P652" s="2" t="inlineStr"/>
+      <c r="Q652" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R652" s="2" t="inlineStr"/>
+      <c r="S652" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" s="2" t="inlineStr">
+        <is>
+          <t>Ryan Harrison</t>
+        </is>
+      </c>
+      <c r="B653" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Superior Relic Signatures - Platinum</t>
+        </is>
+      </c>
+      <c r="C653" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Platinum 1/1 Ryan Harrison #SRS-RH Rookie Auto RC 0r9h</t>
+        </is>
+      </c>
+      <c r="D653" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E653" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F653" s="2" t="inlineStr">
+        <is>
+          <t>229.45 USD</t>
+        </is>
+      </c>
+      <c r="G653" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237110312918</t>
+        </is>
+      </c>
+      <c r="H653" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I653" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bQ8AAeSw-wtqxQkW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J653" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T14:42:31.000Z</t>
+        </is>
+      </c>
+      <c r="K653" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L653" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M653" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N653" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3x4AAeSw4PpqxQkW/s-l1600.jpg | https://i.ebayimg.com/images/g/bRIAAeSw-wtqxQkW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O653" s="2" t="inlineStr"/>
+      <c r="P653" s="2" t="inlineStr"/>
+      <c r="Q653" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R653" s="2" t="inlineStr"/>
+      <c r="S653" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="2" t="inlineStr">
+        <is>
+          <t>Garbine Muguruza</t>
+        </is>
+      </c>
+      <c r="B654" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Star Relics - Gold</t>
+        </is>
+      </c>
+      <c r="C654" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Star Relics Gold 10/10 Garbine Muguruza Rookie RC 1e41</t>
+        </is>
+      </c>
+      <c r="D654" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E654" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F654" s="2" t="inlineStr">
+        <is>
+          <t>46.25 USD</t>
+        </is>
+      </c>
+      <c r="G654" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257785032434</t>
+        </is>
+      </c>
+      <c r="H654" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I654" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/zTIAAeSw~kFqxKFs/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J654" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T07:20:13.000Z</t>
+        </is>
+      </c>
+      <c r="K654" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L654" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M654" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N654" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/5LIAAeSws4FqxKFs/s-l1600.jpg | https://i.ebayimg.com/images/g/4YsAAeSw~yNqxKFs/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O654" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P654" s="2" t="inlineStr"/>
+      <c r="Q654" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R654" s="2" t="inlineStr"/>
+      <c r="S654" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="2" t="inlineStr">
+        <is>
+          <t>Kim Clijsters</t>
+        </is>
+      </c>
+      <c r="B655" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - [Base] - Green</t>
+        </is>
+      </c>
+      <c r="C655" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Green 5/5 Kim Clijsters #68 Rookie RC 1e41</t>
+        </is>
+      </c>
+      <c r="D655" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E655" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F655" s="2" t="inlineStr">
+        <is>
+          <t>74.99 USD</t>
+        </is>
+      </c>
+      <c r="G655" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237109408264</t>
+        </is>
+      </c>
+      <c r="H655" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I655" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/orkAAeSwG1ZqxKFf/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J655" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T07:20:00.000Z</t>
+        </is>
+      </c>
+      <c r="K655" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L655" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M655" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N655" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/yysAAeSwG~dqxKFf/s-l1600.jpg | https://i.ebayimg.com/images/g/sIsAAeSwADJqxKFf/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O655" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P655" s="2" t="inlineStr"/>
+      <c r="Q655" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R655" s="2" t="inlineStr"/>
+      <c r="S655" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="2" t="inlineStr">
+        <is>
+          <t>John McEnroe</t>
+        </is>
+      </c>
+      <c r="B656" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Tennis</t>
+        </is>
+      </c>
+      <c r="C656" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> John McEnroe 2024 Topps Royalty Tennis INFLUENTIAL #25/25 Auto Last Print </t>
+        </is>
+      </c>
+      <c r="D656" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E656" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F656" s="2" t="inlineStr">
+        <is>
+          <t>349.99 USD</t>
+        </is>
+      </c>
+      <c r="G656" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/920011426810</t>
+        </is>
+      </c>
+      <c r="H656" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:07 UTC</t>
+        </is>
+      </c>
+      <c r="I656" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bo4AAeSwPolqxBE0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J656" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T21:07:33.000Z</t>
+        </is>
+      </c>
+      <c r="K656" s="2" t="inlineStr">
+        <is>
+          <t>Auction + Buy It Now</t>
+        </is>
+      </c>
+      <c r="L656" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M656" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N656" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XrMAAeSwa0hqxBE0/s-l1600.jpg | https://i.ebayimg.com/images/g/x0AAAeSwD1JqxBE0/s-l1600.jpg | https://i.ebayimg.com/images/g/h7oAAeSw8tlqxBE1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O656" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P656" s="2" t="inlineStr"/>
+      <c r="Q656" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R656" s="2" t="inlineStr"/>
+      <c r="S656" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -56119,6 +58421,32 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G628" r:id="rId627"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G629" r:id="rId628"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G630" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G631" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G632" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G633" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G634" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G635" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G636" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G637" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G638" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G639" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G640" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G641" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G642" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G643" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G644" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G645" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G646" r:id="rId645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G647" r:id="rId646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G648" r:id="rId647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G649" r:id="rId648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G650" r:id="rId649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G651" r:id="rId650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G652" r:id="rId651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G653" r:id="rId652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G654" r:id="rId653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G655" r:id="rId654"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G656" r:id="rId655"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-07 16:47 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S656"/>
+  <dimension ref="A1:S673"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -57785,6 +57785,1511 @@
       </c>
       <c r="R656" s="2" t="inlineStr"/>
       <c r="S656" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Nadal</t>
+        </is>
+      </c>
+      <c r="B657" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Chrome</t>
+        </is>
+      </c>
+      <c r="C657" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Rafael Nadal #AO-RNL Auto I Black Refractor 10/10 On Card</t>
+        </is>
+      </c>
+      <c r="D657" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E657" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F657" s="2" t="inlineStr">
+        <is>
+          <t>25000.00 USD</t>
+        </is>
+      </c>
+      <c r="G657" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/920017970729</t>
+        </is>
+      </c>
+      <c r="H657" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I657" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/xRcAAeSwlxpqxnXK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J657" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T16:38:35.000Z</t>
+        </is>
+      </c>
+      <c r="K657" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L657" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M657" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N657" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0XcAAeSw4dRqxnXK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O657" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P657" s="2" t="inlineStr"/>
+      <c r="Q657" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R657" s="2" t="inlineStr"/>
+      <c r="S657" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="2" t="inlineStr">
+        <is>
+          <t>Peyton Stearns</t>
+        </is>
+      </c>
+      <c r="B658" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C658" s="2" t="inlineStr">
+        <is>
+          <t>PEYTON STEARNS 2026 TOPPS CHROME TENNIS #96 FROZEN FRACTOR -1/0</t>
+        </is>
+      </c>
+      <c r="D658" s="2" t="inlineStr">
+        <is>
+          <t>1/0</t>
+        </is>
+      </c>
+      <c r="E658" s="2" t="inlineStr">
+        <is>
+          <t>001 of 0</t>
+        </is>
+      </c>
+      <c r="F658" s="2" t="inlineStr">
+        <is>
+          <t>299.99 USD</t>
+        </is>
+      </c>
+      <c r="G658" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/227556975778</t>
+        </is>
+      </c>
+      <c r="H658" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I658" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/5zQAAeSwNG5qxnAV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J658" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T16:15:30.000Z</t>
+        </is>
+      </c>
+      <c r="K658" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L658" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M658" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N658" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/enUAAeSwo29qxnAV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O658" s="2" t="inlineStr"/>
+      <c r="P658" s="2" t="inlineStr"/>
+      <c r="Q658" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R658" s="2" t="inlineStr"/>
+      <c r="S658" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="2" t="inlineStr">
+        <is>
+          <t>Patrick Kypson</t>
+        </is>
+      </c>
+      <c r="B659" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - Autographs I - Red Geometric Refractor</t>
+        </is>
+      </c>
+      <c r="C659" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome I Red Geometric Refractor 1/5 Patrick Kypson #CA-PKN Auto 1e41</t>
+        </is>
+      </c>
+      <c r="D659" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E659" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F659" s="2" t="inlineStr">
+        <is>
+          <t>34.74 USD</t>
+        </is>
+      </c>
+      <c r="G659" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336833645810</t>
+        </is>
+      </c>
+      <c r="H659" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I659" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7NEAAeSwAOdqxkTZ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J659" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T13:09:46.000Z</t>
+        </is>
+      </c>
+      <c r="K659" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L659" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M659" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N659" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QA4AAeSw6clqxkTZ/s-l1600.jpg | https://i.ebayimg.com/images/g/1o0AAeSwynBqxkTZ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O659" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P659" s="2" t="inlineStr"/>
+      <c r="Q659" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R659" s="2" t="inlineStr"/>
+      <c r="S659" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" s="2" t="inlineStr">
+        <is>
+          <t>Garbine Muguruza</t>
+        </is>
+      </c>
+      <c r="B660" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C660" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Red Refractor 1/5 Garbine Muguruza Garbiñe #39 Rookie RC 1w0z</t>
+        </is>
+      </c>
+      <c r="D660" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E660" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F660" s="2" t="inlineStr">
+        <is>
+          <t>121.10 USD</t>
+        </is>
+      </c>
+      <c r="G660" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257787483875</t>
+        </is>
+      </c>
+      <c r="H660" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I660" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/LlEAAeSwCCpqxjrp/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J660" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T12:27:20.000Z</t>
+        </is>
+      </c>
+      <c r="K660" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L660" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M660" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N660" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QYMAAeSwSk9qxjrq/s-l1600.jpg | https://i.ebayimg.com/images/g/zhEAAeSwPV5qxjrq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O660" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P660" s="2" t="inlineStr"/>
+      <c r="Q660" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R660" s="2" t="inlineStr"/>
+      <c r="S660" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="2" t="inlineStr">
+        <is>
+          <t>Andy Murray</t>
+        </is>
+      </c>
+      <c r="B661" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 TOPPS CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="C661" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS BLACK GEOMETRIC #180 ANDY MURRAY 2/2 PSA 8</t>
+        </is>
+      </c>
+      <c r="D661" s="2" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="E661" s="2" t="inlineStr">
+        <is>
+          <t>last of 2 (2/2)</t>
+        </is>
+      </c>
+      <c r="F661" s="2" t="inlineStr">
+        <is>
+          <t>225.00 USD</t>
+        </is>
+      </c>
+      <c r="G661" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307219191337</t>
+        </is>
+      </c>
+      <c r="H661" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I661" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/N~gAAeSwt-dqxjCa/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J661" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T11:43:22.000Z</t>
+        </is>
+      </c>
+      <c r="K661" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L661" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M661" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 8</t>
+        </is>
+      </c>
+      <c r="N661" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ylYAAeSwH99qxjCb/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O661" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P661" s="2" t="inlineStr"/>
+      <c r="Q661" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R661" s="2" t="inlineStr"/>
+      <c r="S661" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="2" t="inlineStr">
+        <is>
+          <t>Daniil Medvedev</t>
+        </is>
+      </c>
+      <c r="B662" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Sapphire</t>
+        </is>
+      </c>
+      <c r="C662" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Sapphire Daniil Medvedev Padparadscha 1/1 PSA 9</t>
+        </is>
+      </c>
+      <c r="D662" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E662" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F662" s="2" t="inlineStr">
+        <is>
+          <t>3000.00 USD</t>
+        </is>
+      </c>
+      <c r="G662" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237112257854?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2B3wWmCh4wbTXsflYmIbcsGpvJ8muXXA9FSNUmg8v7RokOLn2t6Rar8i%2BFSAmbVwYh%2BQqj%2BNDT%2Bj3h3cm3s70YnXwWaxfZg%2BHdFw%2BE%2FF5Kto5mpgFPtw45nIbtLi5P0pwDFtUqIl5rw1onjdWnRijp1lU%2BgcARvVyWzocWbfCPG7P%2BAK9OPB1O9Lzx6SC%2FRleI%3D</t>
+        </is>
+      </c>
+      <c r="H662" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I662" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/m8kAAeSwIFpqxgOs/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J662" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T08:31:42.000Z</t>
+        </is>
+      </c>
+      <c r="K662" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L662" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M662" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N662" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/v-QAAeSwG3JqxgO6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O662" s="2" t="inlineStr"/>
+      <c r="P662" s="2" t="inlineStr"/>
+      <c r="Q662" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R662" s="2" t="inlineStr"/>
+      <c r="S662" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="2" t="inlineStr">
+        <is>
+          <t>Anastasia Pavlyuchenkova</t>
+        </is>
+      </c>
+      <c r="B663" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - Autographs II - Black Refractor</t>
+        </is>
+      </c>
+      <c r="C663" s="2" t="inlineStr">
+        <is>
+          <t>2025 Chrome II Black Refractor 10/10 Anastasia Pavlyuchenkova Rookie Auto RC ob9</t>
+        </is>
+      </c>
+      <c r="D663" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E663" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F663" s="2" t="inlineStr">
+        <is>
+          <t>98.58 USD</t>
+        </is>
+      </c>
+      <c r="G663" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336833049556</t>
+        </is>
+      </c>
+      <c r="H663" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I663" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/NqkAAeSwO2lqxdZF/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J663" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T05:17:59.000Z</t>
+        </is>
+      </c>
+      <c r="K663" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L663" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M663" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N663" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HSkAAeSwjnBqxdZF/s-l1600.jpg | https://i.ebayimg.com/images/g/pKcAAeSw8DZqxdZF/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O663" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P663" s="2" t="inlineStr"/>
+      <c r="Q663" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R663" s="2" t="inlineStr"/>
+      <c r="S663" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" s="2" t="inlineStr">
+        <is>
+          <t>Harold Mayot</t>
+        </is>
+      </c>
+      <c r="B664" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C664" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Sapphire Aqua 199/199 Harold Mayot #75 Rookie RC 13kb</t>
+        </is>
+      </c>
+      <c r="D664" s="2" t="inlineStr">
+        <is>
+          <t>199/199</t>
+        </is>
+      </c>
+      <c r="E664" s="2" t="inlineStr">
+        <is>
+          <t>last of 199 (199/199)</t>
+        </is>
+      </c>
+      <c r="F664" s="2" t="inlineStr">
+        <is>
+          <t>5.43 USD</t>
+        </is>
+      </c>
+      <c r="G664" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257786843249</t>
+        </is>
+      </c>
+      <c r="H664" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I664" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/m1AAAeSwFBxqxb73/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J664" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T03:38:33.000Z</t>
+        </is>
+      </c>
+      <c r="K664" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L664" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M664" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N664" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/b00AAeSwOTVqxb73/s-l1600.jpg | https://i.ebayimg.com/images/g/O38AAeSwEVFqxb74/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O664" s="2" t="inlineStr">
+        <is>
+          <t>aqua</t>
+        </is>
+      </c>
+      <c r="P664" s="2" t="inlineStr"/>
+      <c r="Q664" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R664" s="2" t="inlineStr"/>
+      <c r="S664" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="2" t="inlineStr">
+        <is>
+          <t>Taylor Fritz</t>
+        </is>
+      </c>
+      <c r="B665" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C665" s="2" t="inlineStr">
+        <is>
+          <t>2024 Graphite Court Masters White Refractor 1/10 Taylor Fritz Rookie RC 1gs8</t>
+        </is>
+      </c>
+      <c r="D665" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E665" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F665" s="2" t="inlineStr">
+        <is>
+          <t>92.25 USD</t>
+        </is>
+      </c>
+      <c r="G665" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336833658909</t>
+        </is>
+      </c>
+      <c r="H665" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I665" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/OUoAAeSwNcxqxkdW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J665" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T13:20:23.000Z</t>
+        </is>
+      </c>
+      <c r="K665" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L665" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M665" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N665" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/kwQAAeSwnpJqxkdW/s-l1600.jpg | https://i.ebayimg.com/images/g/OUkAAeSwNcxqxkdW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O665" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P665" s="2" t="inlineStr"/>
+      <c r="Q665" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R665" s="2" t="inlineStr"/>
+      <c r="S665" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="2" t="inlineStr">
+        <is>
+          <t>Mitchell Krueger</t>
+        </is>
+      </c>
+      <c r="B666" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C666" s="2" t="inlineStr">
+        <is>
+          <t>2024 Graphite Signature Relics Gold Refractor 25/25 Mitchell Krueger Auto 1u6</t>
+        </is>
+      </c>
+      <c r="D666" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E666" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F666" s="2" t="inlineStr">
+        <is>
+          <t>6.00 USD</t>
+        </is>
+      </c>
+      <c r="G666" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237112171590</t>
+        </is>
+      </c>
+      <c r="H666" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I666" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-hkAAeSwKwRqxfUg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J666" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T07:28:45.000Z</t>
+        </is>
+      </c>
+      <c r="K666" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L666" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M666" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N666" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/5d0AAeSw~6pqxfUg/s-l1600.jpg | https://i.ebayimg.com/images/g/U1wAAeSwOHZqxfUg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O666" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P666" s="2" t="inlineStr"/>
+      <c r="Q666" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R666" s="2" t="inlineStr"/>
+      <c r="S666" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" s="2" t="inlineStr">
+        <is>
+          <t>Ben Shelton</t>
+        </is>
+      </c>
+      <c r="B667" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C667" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Relics Pink Refractor 15/15 Ben Shelton Rookie RC 0r9h</t>
+        </is>
+      </c>
+      <c r="D667" s="2" t="inlineStr">
+        <is>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="E667" s="2" t="inlineStr">
+        <is>
+          <t>last of 15 (15/15)</t>
+        </is>
+      </c>
+      <c r="F667" s="2" t="inlineStr">
+        <is>
+          <t>225.05 USD</t>
+        </is>
+      </c>
+      <c r="G667" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257786941351</t>
+        </is>
+      </c>
+      <c r="H667" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I667" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/51sAAeSw9KxqxdUJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J667" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T05:12:34.000Z</t>
+        </is>
+      </c>
+      <c r="K667" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L667" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M667" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N667" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/K3cAAeSw1~FqxdUJ/s-l1600.jpg | https://i.ebayimg.com/images/g/g64AAeSw~kFqxdUJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O667" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P667" s="2" t="inlineStr"/>
+      <c r="Q667" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R667" s="2" t="inlineStr"/>
+      <c r="S667" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" s="2" t="inlineStr">
+        <is>
+          <t>Ekaterina Alexandrova</t>
+        </is>
+      </c>
+      <c r="B668" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C668" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Ekaterina Alexandrova Red Crystalline Refractor #1/1 PSA 9</t>
+        </is>
+      </c>
+      <c r="D668" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E668" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F668" s="2" t="inlineStr">
+        <is>
+          <t>4.25 USD</t>
+        </is>
+      </c>
+      <c r="G668" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377548479030</t>
+        </is>
+      </c>
+      <c r="H668" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I668" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2t8AAeSwzWBqxOlU/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J668" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T01:47:22.000Z</t>
+        </is>
+      </c>
+      <c r="K668" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L668" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M668" s="2" t="inlineStr">
+        <is>
+          <t>PSA 9</t>
+        </is>
+      </c>
+      <c r="N668" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7YMAAeSwADBqxOlV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O668" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P668" s="2" t="inlineStr"/>
+      <c r="Q668" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R668" s="2" t="inlineStr"/>
+      <c r="S668" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" s="2" t="inlineStr">
+        <is>
+          <t>Jelena Ostapenko</t>
+        </is>
+      </c>
+      <c r="B669" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C669" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Jelena Ostapenko Red Crystalline Refractor 1/1</t>
+        </is>
+      </c>
+      <c r="D669" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E669" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F669" s="2" t="inlineStr">
+        <is>
+          <t>375.00 USD</t>
+        </is>
+      </c>
+      <c r="G669" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/128119581624</t>
+        </is>
+      </c>
+      <c r="H669" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I669" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Yo0AAeSwJfJqxW9h/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J669" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T22:03:30.000Z</t>
+        </is>
+      </c>
+      <c r="K669" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L669" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M669" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N669" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/D6gAAeSwxn9qxW-D/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O669" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P669" s="2" t="inlineStr"/>
+      <c r="Q669" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R669" s="2" t="inlineStr"/>
+      <c r="S669" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" s="2" t="inlineStr">
+        <is>
+          <t>Isabella Kruger</t>
+        </is>
+      </c>
+      <c r="B670" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Rookie Autographs - Gold</t>
+        </is>
+      </c>
+      <c r="C670" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Rookie Gold 10/10 Isabella Kruger #RA-IK Auto RC 9et</t>
+        </is>
+      </c>
+      <c r="D670" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E670" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F670" s="2" t="inlineStr">
+        <is>
+          <t>114.68 USD</t>
+        </is>
+      </c>
+      <c r="G670" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336833529282</t>
+        </is>
+      </c>
+      <c r="H670" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I670" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0o4AAeSwjnBqxjHv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J670" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T11:48:58.000Z</t>
+        </is>
+      </c>
+      <c r="K670" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L670" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M670" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N670" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vPAAAeSwKVdqxjHx/s-l1600.jpg | https://i.ebayimg.com/images/g/8lwAAeSw5etqxjHv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O670" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P670" s="2" t="inlineStr"/>
+      <c r="Q670" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R670" s="2" t="inlineStr"/>
+      <c r="S670" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="2" t="inlineStr">
+        <is>
+          <t>Bianca Andreescu</t>
+        </is>
+      </c>
+      <c r="B671" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Pursuit of Greatness Signatures - Gold</t>
+        </is>
+      </c>
+      <c r="C671" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Gold 10/10 Bianca Andreescu #PGS-BAU Rookie Auto RC 9et</t>
+        </is>
+      </c>
+      <c r="D671" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E671" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F671" s="2" t="inlineStr">
+        <is>
+          <t>114.68 USD</t>
+        </is>
+      </c>
+      <c r="G671" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237112541160</t>
+        </is>
+      </c>
+      <c r="H671" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I671" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/rqsAAeSwYa5qxjHl/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J671" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T11:48:53.000Z</t>
+        </is>
+      </c>
+      <c r="K671" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L671" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M671" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N671" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/fX8AAeSwG9dqxjHl/s-l1600.jpg | https://i.ebayimg.com/images/g/2z0AAeSwfCZqxjHm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O671" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P671" s="2" t="inlineStr"/>
+      <c r="Q671" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R671" s="2" t="inlineStr"/>
+      <c r="S671" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="2" t="inlineStr">
+        <is>
+          <t>Garbine Muguruza</t>
+        </is>
+      </c>
+      <c r="B672" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Star Relics - Gold</t>
+        </is>
+      </c>
+      <c r="C672" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Star Relics Gold 1/10 Garbine Muguruza #SRR-GM Rookie RC b6y</t>
+        </is>
+      </c>
+      <c r="D672" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E672" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F672" s="2" t="inlineStr">
+        <is>
+          <t>29.58 USD</t>
+        </is>
+      </c>
+      <c r="G672" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257786790718</t>
+        </is>
+      </c>
+      <c r="H672" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I672" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/OqQAAeSw8wtqxbIS/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J672" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T02:43:32.000Z</t>
+        </is>
+      </c>
+      <c r="K672" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L672" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M672" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N672" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KOsAAeSwmE1qxbIS/s-l1600.jpg | https://i.ebayimg.com/images/g/RUEAAeSwbItqxbIS/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O672" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P672" s="2" t="inlineStr"/>
+      <c r="Q672" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R672" s="2" t="inlineStr"/>
+      <c r="S672" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="2" t="inlineStr">
+        <is>
+          <t>Michael Mmoh</t>
+        </is>
+      </c>
+      <c r="B673" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Imperial Ink - Green</t>
+        </is>
+      </c>
+      <c r="C673" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Imperial Ink Green 1/5 Michael Mmoh Rookie Auto RC 1e41</t>
+        </is>
+      </c>
+      <c r="D673" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E673" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F673" s="2" t="inlineStr">
+        <is>
+          <t>33.60 USD</t>
+        </is>
+      </c>
+      <c r="G673" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237111062807</t>
+        </is>
+      </c>
+      <c r="H673" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I673" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/EVIAAeSwAJ5qxU6g/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J673" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T19:39:09.000Z</t>
+        </is>
+      </c>
+      <c r="K673" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L673" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M673" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N673" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/wOYAAeSwERVqxU6h/s-l1600.jpg | https://i.ebayimg.com/images/g/wN0AAeSwERVqxU6g/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O673" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P673" s="2" t="inlineStr"/>
+      <c r="Q673" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R673" s="2" t="inlineStr"/>
+      <c r="S673" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -58447,6 +59952,23 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G654" r:id="rId653"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G655" r:id="rId654"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G656" r:id="rId655"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G657" r:id="rId656"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G658" r:id="rId657"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G659" r:id="rId658"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G660" r:id="rId659"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G661" r:id="rId660"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G662" r:id="rId661"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G663" r:id="rId662"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G664" r:id="rId663"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G665" r:id="rId664"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G666" r:id="rId665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G667" r:id="rId666"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G668" r:id="rId667"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G669" r:id="rId668"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G670" r:id="rId669"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G671" r:id="rId670"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G672" r:id="rId671"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G673" r:id="rId672"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-08 16:47 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S673"/>
+  <dimension ref="A1:S688"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -59290,6 +59290,1329 @@
       </c>
       <c r="R673" s="2" t="inlineStr"/>
       <c r="S673" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B674" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C674" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Mirra Andreeva #5 Orange RayWave 01/25 First Numbered</t>
+        </is>
+      </c>
+      <c r="D674" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E674" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F674" s="2" t="inlineStr">
+        <is>
+          <t>129.99 USD</t>
+        </is>
+      </c>
+      <c r="G674" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287635650900</t>
+        </is>
+      </c>
+      <c r="H674" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I674" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-fsAAeSwBipqx8UD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J674" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T16:38:23.000Z</t>
+        </is>
+      </c>
+      <c r="K674" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L674" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M674" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N674" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/swsAAeSwWgFqx8UX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O674" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P674" s="2" t="inlineStr"/>
+      <c r="Q674" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R674" s="2" t="inlineStr"/>
+      <c r="S674" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="2" t="inlineStr">
+        <is>
+          <t>Leylah Fernandez</t>
+        </is>
+      </c>
+      <c r="B675" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C675" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Red Refractor YouthQuake Signatures Auto 5/5 Leylah Fernandez</t>
+        </is>
+      </c>
+      <c r="D675" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E675" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F675" s="2" t="inlineStr">
+        <is>
+          <t>299.99 USD</t>
+        </is>
+      </c>
+      <c r="G675" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/920021338735</t>
+        </is>
+      </c>
+      <c r="H675" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I675" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/tZ4AAeSw9~pqx8aD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J675" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T16:37:47.000Z</t>
+        </is>
+      </c>
+      <c r="K675" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L675" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M675" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N675" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/te4AAeSwKfxqx8aE/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O675" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P675" s="2" t="inlineStr"/>
+      <c r="Q675" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R675" s="2" t="inlineStr"/>
+      <c r="S675" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="2" t="inlineStr">
+        <is>
+          <t>Jessica</t>
+        </is>
+      </c>
+      <c r="B676" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C676" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis JESSICA BOUZAS MANEIRO Rookie Black On-Card Auto 01/10</t>
+        </is>
+      </c>
+      <c r="D676" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E676" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F676" s="2" t="inlineStr">
+        <is>
+          <t>99.99 USD</t>
+        </is>
+      </c>
+      <c r="G676" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/920021317037</t>
+        </is>
+      </c>
+      <c r="H676" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I676" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/pBcAAeSwUDFqx8Qc/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J676" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T16:29:23.000Z</t>
+        </is>
+      </c>
+      <c r="K676" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L676" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M676" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N676" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-jcAAeSwfBBqx8Qh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O676" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P676" s="2" t="inlineStr"/>
+      <c r="Q676" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R676" s="2" t="inlineStr"/>
+      <c r="S676" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="2" t="inlineStr">
+        <is>
+          <t>Stan Smith</t>
+        </is>
+      </c>
+      <c r="B677" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C677" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Rings of Honor Red Refractor 5/5 Stan Smith #ROH-10 HOF ob9</t>
+        </is>
+      </c>
+      <c r="D677" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E677" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F677" s="2" t="inlineStr">
+        <is>
+          <t>46.83 USD</t>
+        </is>
+      </c>
+      <c r="G677" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237114639557</t>
+        </is>
+      </c>
+      <c r="H677" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I677" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Vz8AAeSwt7tqx7He/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J677" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T15:08:10.000Z</t>
+        </is>
+      </c>
+      <c r="K677" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L677" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M677" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N677" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ipAAAeSwCFxqx7He/s-l1600.jpg | https://i.ebayimg.com/images/g/Z~4AAeSw-wtqx7He/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O677" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P677" s="2" t="inlineStr"/>
+      <c r="Q677" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R677" s="2" t="inlineStr"/>
+      <c r="S677" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="2" t="inlineStr">
+        <is>
+          <t>Luciano Darderi</t>
+        </is>
+      </c>
+      <c r="B678" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C678" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Luciano Darderi Yellow Refractor 1/275 Italy ATP</t>
+        </is>
+      </c>
+      <c r="D678" s="2" t="inlineStr">
+        <is>
+          <t>1/275</t>
+        </is>
+      </c>
+      <c r="E678" s="2" t="inlineStr">
+        <is>
+          <t>001 of 275</t>
+        </is>
+      </c>
+      <c r="F678" s="2" t="inlineStr">
+        <is>
+          <t>4.99 USD</t>
+        </is>
+      </c>
+      <c r="G678" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298743036461</t>
+        </is>
+      </c>
+      <c r="H678" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I678" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/fFsAAeSwG3Jqx62J/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J678" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T14:50:36.000Z</t>
+        </is>
+      </c>
+      <c r="K678" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L678" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M678" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N678" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/NFQAAeSwG2Nqx62L/s-l1600.jpg | https://i.ebayimg.com/images/g/aQYAAeSwRWxqx62P/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O678" s="2" t="inlineStr">
+        <is>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="P678" s="2" t="inlineStr"/>
+      <c r="Q678" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R678" s="2" t="inlineStr"/>
+      <c r="S678" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="2" t="inlineStr">
+        <is>
+          <t>Butch Buchholz</t>
+        </is>
+      </c>
+      <c r="B679" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C679" s="2" t="inlineStr">
+        <is>
+          <t>2021 Chrome Rings of Honor Red Refractor 5/5 Butch Buchholz Rookie RC HOF 18uq</t>
+        </is>
+      </c>
+      <c r="D679" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E679" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F679" s="2" t="inlineStr">
+        <is>
+          <t>52.58 USD</t>
+        </is>
+      </c>
+      <c r="G679" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257789094993</t>
+        </is>
+      </c>
+      <c r="H679" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I679" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/iC8AAeSwfKJqx6vX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J679" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T14:41:28.000Z</t>
+        </is>
+      </c>
+      <c r="K679" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L679" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M679" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N679" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/T00AAeSws4Fqx6vX/s-l1600.jpg | https://i.ebayimg.com/images/g/v40AAeSwI-dqx6vX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O679" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P679" s="2" t="inlineStr"/>
+      <c r="Q679" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R679" s="2" t="inlineStr"/>
+      <c r="S679" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz, Coco Gauff, Maria Sharapova, Novak Djokovic, Iva Jovic</t>
+        </is>
+      </c>
+      <c r="B680" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C680" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Guaranteed (Sapphire 1/1 Padparadscha Auto) Hot Pack</t>
+        </is>
+      </c>
+      <c r="D680" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E680" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F680" s="2" t="inlineStr">
+        <is>
+          <t>164.95 USD</t>
+        </is>
+      </c>
+      <c r="G680" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117454747902</t>
+        </is>
+      </c>
+      <c r="H680" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I680" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9iwAAeSwF7Vp7MsA/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J680" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T14:00:01.000Z</t>
+        </is>
+      </c>
+      <c r="K680" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L680" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M680" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N680" s="2" t="inlineStr"/>
+      <c r="O680" s="2" t="inlineStr"/>
+      <c r="P680" s="2" t="inlineStr"/>
+      <c r="Q680" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R680" s="2" t="inlineStr"/>
+      <c r="S680" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="2" t="inlineStr">
+        <is>
+          <t>Jan-Lennard Struff</t>
+        </is>
+      </c>
+      <c r="B681" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C681" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome 4/4 Jan-Lennard Struff #CA-JLS Rookie Auto RC 0lm</t>
+        </is>
+      </c>
+      <c r="D681" s="2" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="E681" s="2" t="inlineStr">
+        <is>
+          <t>last of 4 (4/4)</t>
+        </is>
+      </c>
+      <c r="F681" s="2" t="inlineStr">
+        <is>
+          <t>195.39 USD</t>
+        </is>
+      </c>
+      <c r="G681" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336835153567</t>
+        </is>
+      </c>
+      <c r="H681" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I681" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/39MAAeSwO9Vqx5Bu/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J681" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T12:44:32.000Z</t>
+        </is>
+      </c>
+      <c r="K681" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L681" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M681" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N681" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bk4AAeSwo29qx5Bu/s-l1600.jpg | https://i.ebayimg.com/images/g/WMEAAeSwc~Rqx5Bu/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O681" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P681" s="2" t="inlineStr"/>
+      <c r="Q681" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R681" s="2" t="inlineStr"/>
+      <c r="S681" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" s="2" t="inlineStr">
+        <is>
+          <t>Aryna Sabalenka</t>
+        </is>
+      </c>
+      <c r="B682" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C682" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Aryna Sabalenka 1/1 Solus SuperFractor SSP</t>
+        </is>
+      </c>
+      <c r="D682" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E682" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F682" s="2" t="inlineStr">
+        <is>
+          <t>20000.00 USD</t>
+        </is>
+      </c>
+      <c r="G682" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/800771877845</t>
+        </is>
+      </c>
+      <c r="H682" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I682" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Q~UAAeSwoWtqx4rB/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J682" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T12:26:42.000Z</t>
+        </is>
+      </c>
+      <c r="K682" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L682" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M682" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N682" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Q-sAAeSwoWtqx4rA/s-l1600.jpg | https://i.ebayimg.com/images/g/ZDsAAeSwXUBqx4rA/s-l1600.jpg | https://i.ebayimg.com/images/g/MfMAAeSwVI5qx4rA/s-l1600.jpg | https://i.ebayimg.com/images/g/mqIAAeSwOBxqx4rC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O682" s="2" t="inlineStr"/>
+      <c r="P682" s="2" t="inlineStr"/>
+      <c r="Q682" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R682" s="2" t="inlineStr"/>
+      <c r="S682" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="2" t="inlineStr">
+        <is>
+          <t>Ajla Tomljanovic</t>
+        </is>
+      </c>
+      <c r="B683" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Regalia Relic Signatures - Gold</t>
+        </is>
+      </c>
+      <c r="C683" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Gold 1/10 Ajla Tomljanovic PSA 9 MINT Rookie Auto RC 1i3m</t>
+        </is>
+      </c>
+      <c r="D683" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E683" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F683" s="2" t="inlineStr">
+        <is>
+          <t>174.95 USD</t>
+        </is>
+      </c>
+      <c r="G683" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237114605583</t>
+        </is>
+      </c>
+      <c r="H683" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I683" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/67AAAeSwsutqx6s6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J683" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T14:38:51.000Z</t>
+        </is>
+      </c>
+      <c r="K683" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L683" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M683" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports (PSA) 9 MINT</t>
+        </is>
+      </c>
+      <c r="N683" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/mpYAAeSwOJdqx6s7/s-l1600.jpg | https://i.ebayimg.com/images/g/KGUAAeSw--pqx6s7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O683" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P683" s="2" t="inlineStr"/>
+      <c r="Q683" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R683" s="2" t="inlineStr"/>
+      <c r="S683" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="2" t="inlineStr">
+        <is>
+          <t>Erika Andreeva</t>
+        </is>
+      </c>
+      <c r="B684" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - [Base] - Blue</t>
+        </is>
+      </c>
+      <c r="C684" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Blue 1/25 Erika Andreeva #64 Rookie RC 01mu</t>
+        </is>
+      </c>
+      <c r="D684" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E684" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F684" s="2" t="inlineStr">
+        <is>
+          <t>17.50 USD</t>
+        </is>
+      </c>
+      <c r="G684" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257788853290</t>
+        </is>
+      </c>
+      <c r="H684" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I684" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DYMAAeSwfKVqx3wP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J684" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T11:17:36.000Z</t>
+        </is>
+      </c>
+      <c r="K684" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L684" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M684" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N684" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/pY4AAeSw-wtqx3wP/s-l1600.jpg | https://i.ebayimg.com/images/g/1UAAAeSwG~dqx3wP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O684" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P684" s="2" t="inlineStr"/>
+      <c r="Q684" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R684" s="2" t="inlineStr"/>
+      <c r="S684" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="2" t="inlineStr">
+        <is>
+          <t>Pablo Carreno Busta</t>
+        </is>
+      </c>
+      <c r="B685" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Regalia Relic Signatures - Green</t>
+        </is>
+      </c>
+      <c r="C685" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Green 1/5 Pablo Carreno Busta #RRS-PCB Rookie Auto RC 1cc7</t>
+        </is>
+      </c>
+      <c r="D685" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E685" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F685" s="2" t="inlineStr">
+        <is>
+          <t>52.00 USD</t>
+        </is>
+      </c>
+      <c r="G685" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237113733630</t>
+        </is>
+      </c>
+      <c r="H685" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:46 UTC</t>
+        </is>
+      </c>
+      <c r="I685" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Y0oAAeSwbRNqxwub/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J685" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T03:17:49.000Z</t>
+        </is>
+      </c>
+      <c r="K685" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L685" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M685" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N685" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/K-gAAeSwa0hqxwub/s-l1600.jpg | https://i.ebayimg.com/images/g/hbcAAeSwwRFqxwub/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O685" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P685" s="2" t="inlineStr"/>
+      <c r="Q685" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R685" s="2" t="inlineStr"/>
+      <c r="S685" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="2" t="inlineStr">
+        <is>
+          <t>Erling Haaland</t>
+        </is>
+      </c>
+      <c r="B686" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps</t>
+        </is>
+      </c>
+      <c r="C686" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Royalty Erling Haaland On Card Auto Jumbo Relic Booklet 1/5 Man City</t>
+        </is>
+      </c>
+      <c r="D686" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E686" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F686" s="2" t="inlineStr">
+        <is>
+          <t>21043.77 USD</t>
+        </is>
+      </c>
+      <c r="G686" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/327393986764</t>
+        </is>
+      </c>
+      <c r="H686" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:47 UTC</t>
+        </is>
+      </c>
+      <c r="I686" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uOwAAeSwFtBqxuEh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J686" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T00:23:08.000Z</t>
+        </is>
+      </c>
+      <c r="K686" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L686" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M686" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N686" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YLcAAeSwIMdqxuEh/s-l1600.jpg | https://i.ebayimg.com/images/g/yjQAAeSwA8xqxuEi/s-l1600.jpg | https://i.ebayimg.com/images/g/ccAAAeSwmcFqxuEh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O686" s="2" t="inlineStr"/>
+      <c r="P686" s="2" t="inlineStr"/>
+      <c r="Q686" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R686" s="2" t="inlineStr">
+        <is>
+          <t>listing ticks 2 sports, which settles nothing; check by eye</t>
+        </is>
+      </c>
+      <c r="S686" s="2" t="inlineStr">
+        <is>
+          <t>Soccer, football</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" s="2" t="inlineStr">
+        <is>
+          <t>Harold Mayot</t>
+        </is>
+      </c>
+      <c r="B687" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Regalia Relics - Green</t>
+        </is>
+      </c>
+      <c r="C687" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Regalia Relics Green 1/5 Harold Mayot #RER-HM 14zh</t>
+        </is>
+      </c>
+      <c r="D687" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E687" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F687" s="2" t="inlineStr">
+        <is>
+          <t>52.57 USD</t>
+        </is>
+      </c>
+      <c r="G687" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257788091034</t>
+        </is>
+      </c>
+      <c r="H687" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:47 UTC</t>
+        </is>
+      </c>
+      <c r="I687" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/sosAAeSwSk9qxrR1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J687" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T21:05:58.000Z</t>
+        </is>
+      </c>
+      <c r="K687" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L687" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M687" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N687" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/pG0AAeSwgwVqxrR1/s-l1600.jpg | https://i.ebayimg.com/images/g/XQoAAeSwSohqxrR1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O687" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P687" s="2" t="inlineStr"/>
+      <c r="Q687" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R687" s="2" t="inlineStr"/>
+      <c r="S687" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="2" t="inlineStr">
+        <is>
+          <t>Alex de Minaur</t>
+        </is>
+      </c>
+      <c r="B688" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Pursuit of Greatness Signatures - Gold</t>
+        </is>
+      </c>
+      <c r="C688" s="2" t="inlineStr">
+        <is>
+          <t>2024 Royalty Pursuit of Greatness Signatures Gold 10/10 Alex de Minaur Auto 3s8</t>
+        </is>
+      </c>
+      <c r="D688" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E688" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F688" s="2" t="inlineStr">
+        <is>
+          <t>264.10 USD</t>
+        </is>
+      </c>
+      <c r="G688" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336833973622</t>
+        </is>
+      </c>
+      <c r="H688" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:47 UTC</t>
+        </is>
+      </c>
+      <c r="I688" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ex8AAeSwrdxqxoHz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J688" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T17:30:28.000Z</t>
+        </is>
+      </c>
+      <c r="K688" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L688" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M688" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N688" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vrkAAeSwPspqxoH0/s-l1600.jpg | https://i.ebayimg.com/images/g/lqkAAeSw0jZqxoH0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O688" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P688" s="2" t="inlineStr"/>
+      <c r="Q688" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R688" s="2" t="inlineStr"/>
+      <c r="S688" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -59969,6 +61292,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G671" r:id="rId670"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G672" r:id="rId671"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G673" r:id="rId672"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G674" r:id="rId673"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G675" r:id="rId674"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G676" r:id="rId675"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G677" r:id="rId676"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G678" r:id="rId677"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G679" r:id="rId678"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G680" r:id="rId679"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G681" r:id="rId680"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G682" r:id="rId681"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G683" r:id="rId682"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G684" r:id="rId683"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G685" r:id="rId684"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G686" r:id="rId685"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G687" r:id="rId686"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G688" r:id="rId687"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-09 16:27 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S688"/>
+  <dimension ref="A1:S709"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -60613,6 +60613,1859 @@
       </c>
       <c r="R688" s="2" t="inlineStr"/>
       <c r="S688" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="2" t="inlineStr">
+        <is>
+          <t>Pam Shriver</t>
+        </is>
+      </c>
+      <c r="B689" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C689" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Orange Refractor 25/25 Pam Shriver #CA-PS Auto HOF 7xr</t>
+        </is>
+      </c>
+      <c r="D689" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E689" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F689" s="2" t="inlineStr">
+        <is>
+          <t>142.55 USD</t>
+        </is>
+      </c>
+      <c r="G689" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336836844080</t>
+        </is>
+      </c>
+      <c r="H689" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I689" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/IIkAAeSwC5lqyQ9a/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J689" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T15:58:17.000Z</t>
+        </is>
+      </c>
+      <c r="K689" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L689" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M689" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N689" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JrIAAeSwrQBqyQ9a/s-l1600.jpg | https://i.ebayimg.com/images/g/KGQAAeSwg71qyQ9a/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O689" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P689" s="2" t="inlineStr"/>
+      <c r="Q689" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R689" s="2" t="inlineStr"/>
+      <c r="S689" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="2" t="inlineStr">
+        <is>
+          <t>Holger Rune</t>
+        </is>
+      </c>
+      <c r="B690" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C690" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Holger Rune Red Geometric Refractor 5/5 2026 Topps Chrome Tennis </t>
+        </is>
+      </c>
+      <c r="D690" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E690" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F690" s="2" t="inlineStr">
+        <is>
+          <t>275.00 USD</t>
+        </is>
+      </c>
+      <c r="G690" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168780854178</t>
+        </is>
+      </c>
+      <c r="H690" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I690" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Mq4AAeSwygRqyQfX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J690" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T15:27:52.000Z</t>
+        </is>
+      </c>
+      <c r="K690" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L690" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M690" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N690" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/y6EAAeSw2rlqyQfP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O690" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P690" s="2" t="inlineStr"/>
+      <c r="Q690" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R690" s="2" t="inlineStr"/>
+      <c r="S690" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="2" t="inlineStr">
+        <is>
+          <t>Titouan Droguet</t>
+        </is>
+      </c>
+      <c r="B691" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C691" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Sapphire Orange 1/25 Titouan Droguet #155 Rookie RC z6o</t>
+        </is>
+      </c>
+      <c r="D691" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E691" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F691" s="2" t="inlineStr">
+        <is>
+          <t>6.29 USD</t>
+        </is>
+      </c>
+      <c r="G691" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336836692399</t>
+        </is>
+      </c>
+      <c r="H691" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I691" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bOMAAeSwkBlqyPOe/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J691" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T13:59:59.000Z</t>
+        </is>
+      </c>
+      <c r="K691" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L691" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M691" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N691" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/dGAAAeSw1OxqyPOe/s-l1600.jpg | https://i.ebayimg.com/images/g/bI8AAeSw0~tqyPOe/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O691" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P691" s="2" t="inlineStr"/>
+      <c r="Q691" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R691" s="2" t="inlineStr"/>
+      <c r="S691" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="2" t="inlineStr">
+        <is>
+          <t>Alejandro Davidovich Fokina</t>
+        </is>
+      </c>
+      <c r="B692" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C692" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Sapphire Orange 25/25 Alejandro Davidovich Fokina #148 z7d</t>
+        </is>
+      </c>
+      <c r="D692" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E692" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F692" s="2" t="inlineStr">
+        <is>
+          <t>8.75 USD</t>
+        </is>
+      </c>
+      <c r="G692" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257790364112</t>
+        </is>
+      </c>
+      <c r="H692" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I692" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/BqIAAeSwHuNqyOBp/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J692" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T12:38:00.000Z</t>
+        </is>
+      </c>
+      <c r="K692" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L692" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M692" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N692" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/BwAAAeSwvx5qyOBp/s-l1600.jpg | https://i.ebayimg.com/images/g/B08AAeSwAmdqyOBo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O692" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P692" s="2" t="inlineStr"/>
+      <c r="Q692" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R692" s="2" t="inlineStr"/>
+      <c r="S692" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="2" t="inlineStr">
+        <is>
+          <t>Caty Mcnally</t>
+        </is>
+      </c>
+      <c r="B693" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C693" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Sapphire I Orange 1/25 Caty McNally #TCA-CMY Auto q3o</t>
+        </is>
+      </c>
+      <c r="D693" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E693" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F693" s="2" t="inlineStr">
+        <is>
+          <t>41.08 USD</t>
+        </is>
+      </c>
+      <c r="G693" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237115800813</t>
+        </is>
+      </c>
+      <c r="H693" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I693" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/e24AAeSwZeRqyMNt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J693" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T10:34:19.000Z</t>
+        </is>
+      </c>
+      <c r="K693" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L693" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M693" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N693" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/fNMAAeSwRkJqyMNt/s-l1600.jpg | https://i.ebayimg.com/images/g/ggsAAeSwwfJqyMNt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O693" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P693" s="2" t="inlineStr"/>
+      <c r="Q693" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R693" s="2" t="inlineStr"/>
+      <c r="S693" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" s="2" t="inlineStr">
+        <is>
+          <t>Nicolas Moreno De Alboran</t>
+        </is>
+      </c>
+      <c r="B694" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C694" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Sapphire I Purple 10/10 Nicolas Moreno de Alboran Auto q3o</t>
+        </is>
+      </c>
+      <c r="D694" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E694" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F694" s="2" t="inlineStr">
+        <is>
+          <t>52.58 USD</t>
+        </is>
+      </c>
+      <c r="G694" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237115788668</t>
+        </is>
+      </c>
+      <c r="H694" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I694" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/5QgAAeSwr6tqyMCH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J694" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T10:22:00.000Z</t>
+        </is>
+      </c>
+      <c r="K694" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L694" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M694" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N694" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3LwAAeSwFIFqyMCH/s-l1600.jpg | https://i.ebayimg.com/images/g/7C8AAeSwtqtqyMCH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O694" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P694" s="2" t="inlineStr"/>
+      <c r="Q694" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R694" s="2" t="inlineStr"/>
+      <c r="S694" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="2" t="inlineStr">
+        <is>
+          <t>Tracy Austin</t>
+        </is>
+      </c>
+      <c r="B695" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C695" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tracy Austin #180 Superfractor 1/1 WTA Tennis 🎾 💯🎾💯</t>
+        </is>
+      </c>
+      <c r="D695" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E695" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F695" s="2" t="inlineStr">
+        <is>
+          <t>829.02 USD</t>
+        </is>
+      </c>
+      <c r="G695" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/860025471706</t>
+        </is>
+      </c>
+      <c r="H695" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I695" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3NsAAeSw96hqyKVd/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J695" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T09:07:43.000Z</t>
+        </is>
+      </c>
+      <c r="K695" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L695" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M695" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N695" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ZFkAAeSwFEJqyKVd/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O695" s="2" t="inlineStr"/>
+      <c r="P695" s="2" t="inlineStr"/>
+      <c r="Q695" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R695" s="2" t="inlineStr"/>
+      <c r="S695" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" s="2" t="inlineStr">
+        <is>
+          <t>John McEnroe</t>
+        </is>
+      </c>
+      <c r="B696" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C696" s="2" t="inlineStr">
+        <is>
+          <t>John McEnroe 2026 Topps Chrome Tennis World Number 1 Superfractor 1/1</t>
+        </is>
+      </c>
+      <c r="D696" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E696" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F696" s="2" t="inlineStr">
+        <is>
+          <t>10000.00 USD</t>
+        </is>
+      </c>
+      <c r="G696" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407277733065</t>
+        </is>
+      </c>
+      <c r="H696" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I696" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gVsAAeSwXsFqyIzW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J696" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T06:48:08.000Z</t>
+        </is>
+      </c>
+      <c r="K696" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L696" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M696" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA)</t>
+        </is>
+      </c>
+      <c r="N696" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~qIAAeSwkdVqyIzX/s-l1600.jpg | https://i.ebayimg.com/images/g/FKgAAeSwhP1qyIzX/s-l1600.jpg | https://i.ebayimg.com/images/g/pscAAeSwBD9qyIzX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O696" s="2" t="inlineStr"/>
+      <c r="P696" s="2" t="inlineStr"/>
+      <c r="Q696" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R696" s="2" t="inlineStr"/>
+      <c r="S696" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="2" t="inlineStr">
+        <is>
+          <t>Chris Eubanks</t>
+        </is>
+      </c>
+      <c r="B697" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C697" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis Graphite Blue Chris Eubanks #28 50/50 Final Print</t>
+        </is>
+      </c>
+      <c r="D697" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E697" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F697" s="2" t="inlineStr">
+        <is>
+          <t>14.99 USD</t>
+        </is>
+      </c>
+      <c r="G697" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147627128123?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2F6lp%2B3RmE2NF2FbNalouxOxzr%2FnSUQsnKEL2E2KWgXvouR7kZdhrTog3gEKi%2FJtYmZi9lHaZD4ZZLYstJglo1%2BXr0gTyUc6OPfFy7Ra0em2byzbeYsCxaCflTDLU3%2FDFpALdSmOG83lsxlRdYP0MLN9LjY3m314WPMpraPWlvZkqBwtngHwghx%2Ftyz4oAh9as%3D</t>
+        </is>
+      </c>
+      <c r="H697" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I697" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/diEAAeSwjjZqyHy1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J697" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T05:34:21.000Z</t>
+        </is>
+      </c>
+      <c r="K697" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L697" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M697" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N697" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/I~IAAeSwjpdqyHy7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O697" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P697" s="2" t="inlineStr"/>
+      <c r="Q697" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R697" s="2" t="inlineStr"/>
+      <c r="S697" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="2" t="inlineStr">
+        <is>
+          <t>Marina Stakusic</t>
+        </is>
+      </c>
+      <c r="B698" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C698" s="2" t="inlineStr">
+        <is>
+          <t>Topps Chrome 2026 Tennis  Marina Stakusic Auto 01/25 Orange Geometric</t>
+        </is>
+      </c>
+      <c r="D698" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E698" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F698" s="2" t="inlineStr">
+        <is>
+          <t>40.00 USD</t>
+        </is>
+      </c>
+      <c r="G698" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/128123813649</t>
+        </is>
+      </c>
+      <c r="H698" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I698" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vXMAAeSw3~BqyGm5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J698" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T04:13:39.000Z</t>
+        </is>
+      </c>
+      <c r="K698" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L698" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M698" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N698" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/fJAAAeSw7wpqyGmt/s-l1600.jpg | https://i.ebayimg.com/images/g/b1cAAeSwsjNqyGmy/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O698" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P698" s="2" t="inlineStr"/>
+      <c r="Q698" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R698" s="2" t="inlineStr"/>
+      <c r="S698" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="2" t="inlineStr">
+        <is>
+          <t>Madison Keys</t>
+        </is>
+      </c>
+      <c r="B699" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C699" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Madison Keys Orange refractor Auto Autograph #1/25 1st!</t>
+        </is>
+      </c>
+      <c r="D699" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E699" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F699" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G699" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/206613092908</t>
+        </is>
+      </c>
+      <c r="H699" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I699" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/4m8AAeSwNXNqyGOD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J699" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:46:27.000Z</t>
+        </is>
+      </c>
+      <c r="K699" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L699" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M699" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N699" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/20QAAeSw7C1qyGOD/s-l1600.jpg | https://i.ebayimg.com/images/g/1mQAAeSwsDVqyGOE/s-l1600.jpg | https://i.ebayimg.com/images/g/1LgAAeSwEM5qyGOE/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O699" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P699" s="2" t="inlineStr"/>
+      <c r="Q699" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R699" s="2" t="inlineStr"/>
+      <c r="S699" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="2" t="inlineStr">
+        <is>
+          <t>Holger Rune</t>
+        </is>
+      </c>
+      <c r="B700" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C700" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Sapphire Gold 50/50 Holger Rune #161 Rookie RC ux8</t>
+        </is>
+      </c>
+      <c r="D700" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E700" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F700" s="2" t="inlineStr">
+        <is>
+          <t>52.58 USD</t>
+        </is>
+      </c>
+      <c r="G700" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336835975661</t>
+        </is>
+      </c>
+      <c r="H700" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I700" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QyYAAeSwtfFqyF0l/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J700" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:17:57.000Z</t>
+        </is>
+      </c>
+      <c r="K700" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L700" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M700" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N700" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/NWQAAeSwLo1qyF0l/s-l1600.jpg | https://i.ebayimg.com/images/g/P8gAAeSwovlqyF0l/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O700" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P700" s="2" t="inlineStr"/>
+      <c r="Q700" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R700" s="2" t="inlineStr"/>
+      <c r="S700" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="2" t="inlineStr">
+        <is>
+          <t>Benoit Paire Auto</t>
+        </is>
+      </c>
+      <c r="B701" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C701" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis SuperFractor 1/1 Benoit Paire Auto #TCABPE PSA 9 BG6</t>
+        </is>
+      </c>
+      <c r="D701" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E701" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F701" s="2" t="inlineStr">
+        <is>
+          <t>493.75 USD</t>
+        </is>
+      </c>
+      <c r="G701" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178566652860</t>
+        </is>
+      </c>
+      <c r="H701" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I701" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/tT0AAeSwZOZqxzwj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J701" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T03:05:00.000Z</t>
+        </is>
+      </c>
+      <c r="K701" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L701" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M701" s="2" t="inlineStr">
+        <is>
+          <t>PSA 9</t>
+        </is>
+      </c>
+      <c r="N701" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/A9sAAeSwbItqxzwj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O701" s="2" t="inlineStr"/>
+      <c r="P701" s="2" t="inlineStr"/>
+      <c r="Q701" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R701" s="2" t="inlineStr"/>
+      <c r="S701" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="2" t="inlineStr">
+        <is>
+          <t>Pete Sampras</t>
+        </is>
+      </c>
+      <c r="B702" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C702" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Pete Sampras FrozenFractor Refractor -1/0 #200</t>
+        </is>
+      </c>
+      <c r="D702" s="2" t="inlineStr">
+        <is>
+          <t>1/0</t>
+        </is>
+      </c>
+      <c r="E702" s="2" t="inlineStr">
+        <is>
+          <t>001 of 0</t>
+        </is>
+      </c>
+      <c r="F702" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G702" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178562335850</t>
+        </is>
+      </c>
+      <c r="H702" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I702" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bGUAAeSws4Fqxbp0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J702" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T02:49:01.000Z</t>
+        </is>
+      </c>
+      <c r="K702" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L702" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M702" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N702" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-isAAeSw3P1qxbp2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O702" s="2" t="inlineStr"/>
+      <c r="P702" s="2" t="inlineStr"/>
+      <c r="Q702" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R702" s="2" t="inlineStr"/>
+      <c r="S702" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="2" t="inlineStr">
+        <is>
+          <t>Alize Cornet</t>
+        </is>
+      </c>
+      <c r="B703" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C703" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Gold Refractor 25/25 Alize Cornet Alizé Cornet #3 z6o</t>
+        </is>
+      </c>
+      <c r="D703" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E703" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F703" s="2" t="inlineStr">
+        <is>
+          <t>6.58 USD</t>
+        </is>
+      </c>
+      <c r="G703" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336836750046</t>
+        </is>
+      </c>
+      <c r="H703" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I703" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/X1gAAeSwPpRqyPvP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J703" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:34:56.000Z</t>
+        </is>
+      </c>
+      <c r="K703" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L703" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M703" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N703" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/VqoAAeSwsNxqyPvP/s-l1600.jpg | https://i.ebayimg.com/images/g/WxgAAeSwlHlqyPvP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O703" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P703" s="2" t="inlineStr"/>
+      <c r="Q703" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R703" s="2" t="inlineStr"/>
+      <c r="S703" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="2" t="inlineStr">
+        <is>
+          <t>Martina Navratilova</t>
+        </is>
+      </c>
+      <c r="B704" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C704" s="2" t="inlineStr">
+        <is>
+          <t>2024 Graphite Legends of the Court Green Refractor 1/75 Martina Navratilova nd3</t>
+        </is>
+      </c>
+      <c r="D704" s="2" t="inlineStr">
+        <is>
+          <t>1/75</t>
+        </is>
+      </c>
+      <c r="E704" s="2" t="inlineStr">
+        <is>
+          <t>001 of 75</t>
+        </is>
+      </c>
+      <c r="F704" s="2" t="inlineStr">
+        <is>
+          <t>18.08 USD</t>
+        </is>
+      </c>
+      <c r="G704" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237115844254</t>
+        </is>
+      </c>
+      <c r="H704" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I704" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/cFcAAeSw7pxqyMwV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J704" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T11:11:18.000Z</t>
+        </is>
+      </c>
+      <c r="K704" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L704" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M704" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N704" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/1~UAAeSwogFqyMwV/s-l1600.jpg | https://i.ebayimg.com/images/g/-5AAAeSwejlqyMwV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O704" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P704" s="2" t="inlineStr"/>
+      <c r="Q704" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R704" s="2" t="inlineStr"/>
+      <c r="S704" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="2" t="inlineStr">
+        <is>
+          <t>Casper Ruud</t>
+        </is>
+      </c>
+      <c r="B705" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C705" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite White Refractor 10/10 Casper Ruud #168 Rookie RC 9et</t>
+        </is>
+      </c>
+      <c r="D705" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E705" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F705" s="2" t="inlineStr">
+        <is>
+          <t>114.68 USD</t>
+        </is>
+      </c>
+      <c r="G705" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237115357018</t>
+        </is>
+      </c>
+      <c r="H705" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I705" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TqMAAeSwnoFqyEq~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J705" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T01:59:27.000Z</t>
+        </is>
+      </c>
+      <c r="K705" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L705" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M705" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N705" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QMcAAeSw9G1qyEq~/s-l1600.jpg | https://i.ebayimg.com/images/g/NmwAAeSw5eZqyEq~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O705" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P705" s="2" t="inlineStr"/>
+      <c r="Q705" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R705" s="2" t="inlineStr"/>
+      <c r="S705" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="2" t="inlineStr">
+        <is>
+          <t>Jordan Thompson</t>
+        </is>
+      </c>
+      <c r="B706" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C706" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Relics White Refractor 10/10 Jordan Thompson Rookie RC 5ov</t>
+        </is>
+      </c>
+      <c r="D706" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E706" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F706" s="2" t="inlineStr">
+        <is>
+          <t>12.32 USD</t>
+        </is>
+      </c>
+      <c r="G706" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237115105770</t>
+        </is>
+      </c>
+      <c r="H706" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I706" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/migAAeSwjDtqyAV4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J706" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T21:03:53.000Z</t>
+        </is>
+      </c>
+      <c r="K706" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L706" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M706" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N706" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/mZwAAeSwmWxqyAV4/s-l1600.jpg | https://i.ebayimg.com/images/g/pEEAAeSwB9JqyAV4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O706" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P706" s="2" t="inlineStr"/>
+      <c r="Q706" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R706" s="2" t="inlineStr"/>
+      <c r="S706" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="2" t="inlineStr">
+        <is>
+          <t>Daniela Hantuchova</t>
+        </is>
+      </c>
+      <c r="B707" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - [Base] - Gold</t>
+        </is>
+      </c>
+      <c r="C707" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Gold 10/10 Daniela Hantuchova #86 1fl4</t>
+        </is>
+      </c>
+      <c r="D707" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E707" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F707" s="2" t="inlineStr">
+        <is>
+          <t>52.28 USD</t>
+        </is>
+      </c>
+      <c r="G707" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257790211729</t>
+        </is>
+      </c>
+      <c r="H707" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I707" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/6PcAAeSwljZqyMEA/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J707" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T10:24:02.000Z</t>
+        </is>
+      </c>
+      <c r="K707" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L707" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M707" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N707" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~5AAAeSwEplqyMEA/s-l1600.jpg | https://i.ebayimg.com/images/g/6z0AAeSw7G9qyMEA/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O707" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P707" s="2" t="inlineStr"/>
+      <c r="Q707" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R707" s="2" t="inlineStr"/>
+      <c r="S707" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="2" t="inlineStr">
+        <is>
+          <t>Hugo Gaston</t>
+        </is>
+      </c>
+      <c r="B708" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Star Relics - Green</t>
+        </is>
+      </c>
+      <c r="C708" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Star Relics Green 1/5 Hugo Gaston #SRR-HG Rookie RC 9et</t>
+        </is>
+      </c>
+      <c r="D708" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E708" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F708" s="2" t="inlineStr">
+        <is>
+          <t>75.58 USD</t>
+        </is>
+      </c>
+      <c r="G708" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336836112783</t>
+        </is>
+      </c>
+      <c r="H708" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I708" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/wNsAAeSwhP1qyIaR/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J708" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T06:14:42.000Z</t>
+        </is>
+      </c>
+      <c r="K708" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L708" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M708" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N708" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nwEAAeSwjpdqyIaR/s-l1600.jpg | https://i.ebayimg.com/images/g/qMIAAeSwfypqyIaR/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O708" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P708" s="2" t="inlineStr"/>
+      <c r="Q708" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R708" s="2" t="inlineStr"/>
+      <c r="S708" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" s="2" t="inlineStr">
+        <is>
+          <t>Hugo Gaston</t>
+        </is>
+      </c>
+      <c r="B709" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Regalia Relic Signatures - Green</t>
+        </is>
+      </c>
+      <c r="C709" s="2" t="inlineStr">
+        <is>
+          <t>2024 Royalty Regalia Relic Signatures Green 5/5 Hugo Gaston Rookie Auto RC 9et</t>
+        </is>
+      </c>
+      <c r="D709" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E709" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F709" s="2" t="inlineStr">
+        <is>
+          <t>87.08 USD</t>
+        </is>
+      </c>
+      <c r="G709" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257789880369</t>
+        </is>
+      </c>
+      <c r="H709" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:26 UTC</t>
+        </is>
+      </c>
+      <c r="I709" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Z18AAeSwrbhqyGnI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J709" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T04:11:54.000Z</t>
+        </is>
+      </c>
+      <c r="K709" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L709" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M709" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N709" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/dGEAAeSwGeBqyGnJ/s-l1600.jpg | https://i.ebayimg.com/images/g/ZDYAAeSwNhNqyGnJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O709" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P709" s="2" t="inlineStr"/>
+      <c r="Q709" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R709" s="2" t="inlineStr"/>
+      <c r="S709" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -61307,6 +63160,27 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G686" r:id="rId685"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G687" r:id="rId686"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G688" r:id="rId687"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G689" r:id="rId688"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G690" r:id="rId689"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G691" r:id="rId690"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G692" r:id="rId691"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G693" r:id="rId692"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G694" r:id="rId693"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G695" r:id="rId694"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G696" r:id="rId695"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G697" r:id="rId696"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G698" r:id="rId697"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G699" r:id="rId698"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G700" r:id="rId699"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G701" r:id="rId700"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G702" r:id="rId701"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G703" r:id="rId702"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G704" r:id="rId703"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G705" r:id="rId704"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G706" r:id="rId705"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G707" r:id="rId706"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G708" r:id="rId707"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G709" r:id="rId708"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-10 15:31 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S709"/>
+  <dimension ref="A1:S721"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -62466,6 +62466,1062 @@
       </c>
       <c r="R709" s="2" t="inlineStr"/>
       <c r="S709" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="2" t="inlineStr">
+        <is>
+          <t>Andrea Pellegrino</t>
+        </is>
+      </c>
+      <c r="B710" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Tennis Chrome</t>
+        </is>
+      </c>
+      <c r="C710" s="2" t="inlineStr">
+        <is>
+          <t>1/5 TOPPS CHROME TENNIS ADREA PELLEGRINO RED FIRST ON PRINT BOOKEND</t>
+        </is>
+      </c>
+      <c r="D710" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E710" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F710" s="2" t="inlineStr">
+        <is>
+          <t>9.99 USD</t>
+        </is>
+      </c>
+      <c r="G710" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/267809649888</t>
+        </is>
+      </c>
+      <c r="H710" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10 15:30 UTC</t>
+        </is>
+      </c>
+      <c r="I710" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/aa4AAeSwwhdqfGML/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J710" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T09:55:36.000Z</t>
+        </is>
+      </c>
+      <c r="K710" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L710" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M710" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N710" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-yYAAeSwgYVqfGL2/s-l1600.jpg | https://i.ebayimg.com/images/g/Ik0AAeSwZoJqfGL4/s-l1600.jpg | https://i.ebayimg.com/images/g/Lj0AAeSwvgtqfGL5/s-l1600.jpg | https://i.ebayimg.com/images/g/eY8AAeSw4VRqfGL5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O710" s="2" t="inlineStr"/>
+      <c r="P710" s="2" t="inlineStr"/>
+      <c r="Q710" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R710" s="2" t="inlineStr"/>
+      <c r="S710" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="2" t="inlineStr">
+        <is>
+          <t>Martina Hingis</t>
+        </is>
+      </c>
+      <c r="B711" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C711" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome II Red Refractor 5/5 Martina Hingis #TCA-MHS Auto HOF 5h0</t>
+        </is>
+      </c>
+      <c r="D711" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E711" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F711" s="2" t="inlineStr">
+        <is>
+          <t>340.27 USD</t>
+        </is>
+      </c>
+      <c r="G711" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336837905729</t>
+        </is>
+      </c>
+      <c r="H711" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10 15:30 UTC</t>
+        </is>
+      </c>
+      <c r="I711" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/B8cAAeSw1LJqye8~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J711" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T07:53:37.000Z</t>
+        </is>
+      </c>
+      <c r="K711" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L711" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M711" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N711" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/wgkAAeSwEPpqye8~/s-l1600.jpg | https://i.ebayimg.com/images/g/lv8AAeSw1o9qye8~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O711" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P711" s="2" t="inlineStr"/>
+      <c r="Q711" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R711" s="2" t="inlineStr"/>
+      <c r="S711" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="2" t="inlineStr">
+        <is>
+          <t>Fabian Marozsan</t>
+        </is>
+      </c>
+      <c r="B712" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C712" s="2" t="inlineStr">
+        <is>
+          <t>🎮ma 2026 Topps Chrome Tennis Red Refractor 5/5 Fabian Marozsan</t>
+        </is>
+      </c>
+      <c r="D712" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E712" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F712" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G712" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/800777485155</t>
+        </is>
+      </c>
+      <c r="H712" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10 15:30 UTC</t>
+        </is>
+      </c>
+      <c r="I712" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Jp4AAeSwDVJqx7XG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J712" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T05:33:00.000Z</t>
+        </is>
+      </c>
+      <c r="K712" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L712" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M712" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N712" s="2" t="inlineStr"/>
+      <c r="O712" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P712" s="2" t="inlineStr"/>
+      <c r="Q712" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R712" s="2" t="inlineStr"/>
+      <c r="S712" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="2" t="inlineStr">
+        <is>
+          <t>Patrick Kypson</t>
+        </is>
+      </c>
+      <c r="B713" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - [Base] - Orange Refractor</t>
+        </is>
+      </c>
+      <c r="C713" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Orange Refractor 25/25 Patrick Kypson #193 14ch</t>
+        </is>
+      </c>
+      <c r="D713" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E713" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F713" s="2" t="inlineStr">
+        <is>
+          <t>7.73 USD</t>
+        </is>
+      </c>
+      <c r="G713" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336837636767</t>
+        </is>
+      </c>
+      <c r="H713" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10 15:30 UTC</t>
+        </is>
+      </c>
+      <c r="I713" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/w4IAAeSwvJVqya~q/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J713" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T02:29:28.000Z</t>
+        </is>
+      </c>
+      <c r="K713" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L713" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M713" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N713" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/sD8AAeSwO9Fqya~q/s-l1600.jpg | https://i.ebayimg.com/images/g/ttEAAeSw59lqya~q/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O713" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P713" s="2" t="inlineStr"/>
+      <c r="Q713" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R713" s="2" t="inlineStr"/>
+      <c r="S713" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="2" t="inlineStr">
+        <is>
+          <t>Marta Kostyuk</t>
+        </is>
+      </c>
+      <c r="B714" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C714" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Destiny Marta Kostyuk #DTY-KOS Orange Geometric REF 25/25 AJ85</t>
+        </is>
+      </c>
+      <c r="D714" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E714" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F714" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G714" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407279648534</t>
+        </is>
+      </c>
+      <c r="H714" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10 15:30 UTC</t>
+        </is>
+      </c>
+      <c r="I714" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/E44AAeSwFG9qyaFP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J714" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T02:21:02.000Z</t>
+        </is>
+      </c>
+      <c r="K714" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L714" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M714" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N714" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/LlIAAeSwLWBqyaFT/s-l1600.jpg | https://i.ebayimg.com/images/g/-KYAAeSwsypqyaFM/s-l1600.jpg | https://i.ebayimg.com/images/g/9pUAAeSwtNdqyaFM/s-l1600.jpg | https://i.ebayimg.com/images/g/HT4AAeSwPd1qyaFM/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O714" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P714" s="2" t="inlineStr"/>
+      <c r="Q714" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R714" s="2" t="inlineStr"/>
+      <c r="S714" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="2" t="inlineStr">
+        <is>
+          <t>Nick Kyrgios</t>
+        </is>
+      </c>
+      <c r="B715" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps</t>
+        </is>
+      </c>
+      <c r="C715" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Nick Kyrgios Event Worn Relic Pink Refractor 1/15</t>
+        </is>
+      </c>
+      <c r="D715" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E715" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F715" s="2" t="inlineStr">
+        <is>
+          <t>30.00 USD</t>
+        </is>
+      </c>
+      <c r="G715" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377559709972?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8B%2FWe1UQ12HqQ%2Bq07EjQyYrQKJs%2FKxdxalZKGiUkM290SwKeGC%2BJrZR9K0CqXkrK6HWipir1Vj%2For2XlW5kiyrrI9RMgvYOpEoIH2UcLvCwuAf7LutHGvH2oK%2BA6x7Yuu1%2B8FLLHreOU9ja2pJzfK465HJ%2ByxtU%2FNjtYfQFwuFvMq5Vxu0gnVMHXiSughXw24%3D</t>
+        </is>
+      </c>
+      <c r="H715" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10 15:30 UTC</t>
+        </is>
+      </c>
+      <c r="I715" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~aAAAeSwyz5qylEL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J715" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T14:55:03.000Z</t>
+        </is>
+      </c>
+      <c r="K715" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L715" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M715" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N715" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Do0AAeSwfc9qylEL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O715" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P715" s="2" t="inlineStr"/>
+      <c r="Q715" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R715" s="2" t="inlineStr"/>
+      <c r="S715" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="2" t="inlineStr">
+        <is>
+          <t>Martina Navratilova</t>
+        </is>
+      </c>
+      <c r="B716" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C716" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Green Refractor 75/75 Martina Navratilova #80 HOF 04br</t>
+        </is>
+      </c>
+      <c r="D716" s="2" t="inlineStr">
+        <is>
+          <t>75/75</t>
+        </is>
+      </c>
+      <c r="E716" s="2" t="inlineStr">
+        <is>
+          <t>last of 75 (75/75)</t>
+        </is>
+      </c>
+      <c r="F716" s="2" t="inlineStr">
+        <is>
+          <t>18.93 USD</t>
+        </is>
+      </c>
+      <c r="G716" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257791447252</t>
+        </is>
+      </c>
+      <c r="H716" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10 15:30 UTC</t>
+        </is>
+      </c>
+      <c r="I716" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Jl4AAeSwVKFqybJg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J716" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T03:33:53.000Z</t>
+        </is>
+      </c>
+      <c r="K716" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L716" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M716" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N716" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TJ4AAeSw-v1qybJg/s-l1600.jpg | https://i.ebayimg.com/images/g/HtMAAeSwwQtqybJf/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O716" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P716" s="2" t="inlineStr"/>
+      <c r="Q716" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R716" s="2" t="inlineStr"/>
+      <c r="S716" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="2" t="inlineStr">
+        <is>
+          <t>Hugo Gaston</t>
+        </is>
+      </c>
+      <c r="B717" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C717" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Relics White Refractor 1/10 Hugo Gaston Rookie RC 1e41</t>
+        </is>
+      </c>
+      <c r="D717" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E717" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F717" s="2" t="inlineStr">
+        <is>
+          <t>11.74 USD</t>
+        </is>
+      </c>
+      <c r="G717" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257791011729</t>
+        </is>
+      </c>
+      <c r="H717" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10 15:30 UTC</t>
+        </is>
+      </c>
+      <c r="I717" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/6JIAAeSwyExqyVYp/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J717" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:00:25.000Z</t>
+        </is>
+      </c>
+      <c r="K717" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L717" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M717" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N717" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-YgAAeSwGMFqyVYp/s-l1600.jpg | https://i.ebayimg.com/images/g/PRkAAeSwWKBqyVYp/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O717" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P717" s="2" t="inlineStr"/>
+      <c r="Q717" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R717" s="2" t="inlineStr"/>
+      <c r="S717" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="2" t="inlineStr">
+        <is>
+          <t>Genie Bouchard</t>
+        </is>
+      </c>
+      <c r="B718" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Regalia Relic Signatures - Green</t>
+        </is>
+      </c>
+      <c r="C718" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Regalia Relic Signatures Green 1/5 Genie Bouchard Auto 1e41</t>
+        </is>
+      </c>
+      <c r="D718" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E718" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F718" s="2" t="inlineStr">
+        <is>
+          <t>174.99 USD</t>
+        </is>
+      </c>
+      <c r="G718" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257790984101</t>
+        </is>
+      </c>
+      <c r="H718" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10 15:31 UTC</t>
+        </is>
+      </c>
+      <c r="I718" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uIgAAeSwRSxqyVAv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J718" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T20:34:54.000Z</t>
+        </is>
+      </c>
+      <c r="K718" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L718" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M718" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N718" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/yAUAAeSw7ytqyVAv/s-l1600.jpg | https://i.ebayimg.com/images/g/sicAAeSwGq5qyVAv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O718" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P718" s="2" t="inlineStr"/>
+      <c r="Q718" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R718" s="2" t="inlineStr"/>
+      <c r="S718" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" s="2" t="inlineStr">
+        <is>
+          <t>Claire Liu</t>
+        </is>
+      </c>
+      <c r="B719" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Regalia Relic Signatures - Green</t>
+        </is>
+      </c>
+      <c r="C719" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Regalia Relic Signatures Green 1/5 Claire Liu Auto 1e41</t>
+        </is>
+      </c>
+      <c r="D719" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E719" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F719" s="2" t="inlineStr">
+        <is>
+          <t>57.74 USD</t>
+        </is>
+      </c>
+      <c r="G719" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336837025775</t>
+        </is>
+      </c>
+      <c r="H719" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10 15:31 UTC</t>
+        </is>
+      </c>
+      <c r="I719" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/1xEAAeSwH15qySvH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J719" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T17:59:35.000Z</t>
+        </is>
+      </c>
+      <c r="K719" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L719" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M719" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N719" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0W0AAeSwT0JqySvH/s-l1600.jpg | https://i.ebayimg.com/images/g/2JsAAeSwJbRqySvH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O719" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P719" s="2" t="inlineStr"/>
+      <c r="Q719" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R719" s="2" t="inlineStr"/>
+      <c r="S719" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="2" t="inlineStr">
+        <is>
+          <t>Elena Vesnina</t>
+        </is>
+      </c>
+      <c r="B720" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic / 2006 Ace Authentics Heroes &amp; Legends</t>
+        </is>
+      </c>
+      <c r="C720" s="2" t="inlineStr">
+        <is>
+          <t>2006 ACE ELENA VESNINA HEROES AND LEGENDS AUTO AUTOGRAPH #96 @ 1/475 @</t>
+        </is>
+      </c>
+      <c r="D720" s="2" t="inlineStr">
+        <is>
+          <t>1/475</t>
+        </is>
+      </c>
+      <c r="E720" s="2" t="inlineStr">
+        <is>
+          <t>001 of 475</t>
+        </is>
+      </c>
+      <c r="F720" s="2" t="inlineStr">
+        <is>
+          <t>14.99 USD</t>
+        </is>
+      </c>
+      <c r="G720" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147628353402</t>
+        </is>
+      </c>
+      <c r="H720" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10 15:31 UTC</t>
+        </is>
+      </c>
+      <c r="I720" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/qLQAAeSw06JqyXT5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J720" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T23:18:29.000Z</t>
+        </is>
+      </c>
+      <c r="K720" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L720" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M720" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N720" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/pA8AAeSwUJVqyXVX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O720" s="2" t="inlineStr"/>
+      <c r="P720" s="2" t="inlineStr"/>
+      <c r="Q720" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R720" s="2" t="inlineStr"/>
+      <c r="S720" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="2" t="inlineStr">
+        <is>
+          <t>Dominika Gibulkova</t>
+        </is>
+      </c>
+      <c r="B721" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic</t>
+        </is>
+      </c>
+      <c r="C721" s="2" t="inlineStr">
+        <is>
+          <t>Rare 2008 ACE Authentic #70 Dominika Gibulkova PSA 8 Rookie 1/1 Pop Highest GRD</t>
+        </is>
+      </c>
+      <c r="D721" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E721" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F721" s="2" t="inlineStr">
+        <is>
+          <t>2000.00 USD</t>
+        </is>
+      </c>
+      <c r="G721" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117457064021</t>
+        </is>
+      </c>
+      <c r="H721" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10 15:31 UTC</t>
+        </is>
+      </c>
+      <c r="I721" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/M1EAAeSwJF9qyTJP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J721" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T18:29:47.000Z</t>
+        </is>
+      </c>
+      <c r="K721" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L721" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M721" s="2" t="inlineStr">
+        <is>
+          <t>PSA 8</t>
+        </is>
+      </c>
+      <c r="N721" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/U3UAAeSwundqyTJP/s-l1600.jpg | https://i.ebayimg.com/images/g/CLUAAeSwXi1qyTJP/s-l1600.jpg | https://i.ebayimg.com/images/g/M1AAAeSwJF9qyTJP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O721" s="2" t="inlineStr"/>
+      <c r="P721" s="2" t="inlineStr"/>
+      <c r="Q721" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R721" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic: check the numbering is stamped, not on a circle sticker</t>
+        </is>
+      </c>
+      <c r="S721" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -63181,6 +64237,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G707" r:id="rId706"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G708" r:id="rId707"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G709" r:id="rId708"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G710" r:id="rId709"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G711" r:id="rId710"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G712" r:id="rId711"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G713" r:id="rId712"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G714" r:id="rId713"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G715" r:id="rId714"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G716" r:id="rId715"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G717" r:id="rId716"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G718" r:id="rId717"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G719" r:id="rId718"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G720" r:id="rId719"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G721" r:id="rId720"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-11 15:53 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S721"/>
+  <dimension ref="A1:S744"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -63522,6 +63522,2013 @@
         </is>
       </c>
       <c r="S721" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B722" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C722" s="2" t="inlineStr">
+        <is>
+          <t>1/1 Topps Chrome Tennis 2026 Coco Gauff Solus SO-CG Superfractor</t>
+        </is>
+      </c>
+      <c r="D722" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E722" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F722" s="2" t="inlineStr">
+        <is>
+          <t>16800.00 USD</t>
+        </is>
+      </c>
+      <c r="G722" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377561576729?amdata=enc%3AAQALAAAAsCHNgUiiE%2FjQhlDTaMiAde8jZ2Gt4ynRcKPjL%2BqbVeyVfkbaU%2Fqjo14o7l5lM7sCyVscm9XTtQl%2BF1zFi2ovmonveqBodkuMVP1JKVk7%2BJRQ6gn4daaPzES08Ng4t3nxrvmxmA4zaJCV3XBRjuFjiF01OD5zoJW4l%2BNxGfxK6wK9fqo7jE7iMCgRmqqw%2FiQPjPeydquJxPF017C%2FSNLHPsyr23MFIZDJYKRM%2BQsGuDw2</t>
+        </is>
+      </c>
+      <c r="H722" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I722" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-I4AAeSwlARqy0ac/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J722" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T08:21:08.000Z</t>
+        </is>
+      </c>
+      <c r="K722" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L722" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M722" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N722" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Z~4AAeSwhNRqy0a3/s-l1600.jpg | https://i.ebayimg.com/images/g/4soAAeSwxXlqy0aC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O722" s="2" t="inlineStr"/>
+      <c r="P722" s="2" t="inlineStr"/>
+      <c r="Q722" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R722" s="2" t="inlineStr"/>
+      <c r="S722" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="2" t="inlineStr">
+        <is>
+          <t>Arthur Fils</t>
+        </is>
+      </c>
+      <c r="B723" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C723" s="2" t="inlineStr">
+        <is>
+          <t>Arthur Fils - 2025 Topps Chrome Tennis Sapphire #32 5/5</t>
+        </is>
+      </c>
+      <c r="D723" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E723" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F723" s="2" t="inlineStr">
+        <is>
+          <t>5500.00 USD</t>
+        </is>
+      </c>
+      <c r="G723" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/327398835872</t>
+        </is>
+      </c>
+      <c r="H723" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I723" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2VYAAeSwHutqywNB/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J723" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T03:33:44.000Z</t>
+        </is>
+      </c>
+      <c r="K723" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L723" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M723" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N723" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/B-YAAeSwsm5qywNB/s-l1600.jpg | https://i.ebayimg.com/images/g/pkIAAeSwtcpqywNB/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O723" s="2" t="inlineStr"/>
+      <c r="P723" s="2" t="inlineStr"/>
+      <c r="Q723" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R723" s="2" t="inlineStr"/>
+      <c r="S723" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="2" t="inlineStr">
+        <is>
+          <t>Andy Murray</t>
+        </is>
+      </c>
+      <c r="B724" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C724" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Andy Murray World No.1 Black Geo 01/10 SSP</t>
+        </is>
+      </c>
+      <c r="D724" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E724" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F724" s="2" t="inlineStr">
+        <is>
+          <t>139.00 USD</t>
+        </is>
+      </c>
+      <c r="G724" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/198705687749?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde9%2BOZbI3YGSgmnPrGwfBG8bcRMLfs7SJYKve7llplvfifLbNNjJTNmcs0hwPVrMl7X96t26mJ0m9DApj8FPtPw678GmhjFc4pfiDpxpcdPThpiyGw1tqHooslmD8BV2FjIS4kPg2PH7Vt3Z4ndAsz%2Bfo3hE7cwAuA4n0Jr%2FX9YnnmeOhR9UKl5zPEC4ojK9Cs0%3D</t>
+        </is>
+      </c>
+      <c r="H724" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I724" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/qvcAAeSwEPpqyv0z/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J724" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T03:29:38.000Z</t>
+        </is>
+      </c>
+      <c r="K724" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L724" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M724" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N724" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/sPoAAeSwNgZqyv0z/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O724" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P724" s="2" t="inlineStr"/>
+      <c r="Q724" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R724" s="2" t="inlineStr"/>
+      <c r="S724" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="2" t="inlineStr">
+        <is>
+          <t>Jasmine Paolini</t>
+        </is>
+      </c>
+      <c r="B725" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C725" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Jasmine Paolini Frozenfractor -1/0 #40</t>
+        </is>
+      </c>
+      <c r="D725" s="2" t="inlineStr">
+        <is>
+          <t>1/0</t>
+        </is>
+      </c>
+      <c r="E725" s="2" t="inlineStr">
+        <is>
+          <t>001 of 0</t>
+        </is>
+      </c>
+      <c r="F725" s="2" t="inlineStr">
+        <is>
+          <t>500.00 USD</t>
+        </is>
+      </c>
+      <c r="G725" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287640734287</t>
+        </is>
+      </c>
+      <c r="H725" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I725" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/5s4AAeSwcKBqywDe/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J725" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T03:22:22.000Z</t>
+        </is>
+      </c>
+      <c r="K725" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L725" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M725" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N725" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/oUMAAeSwe~pqywDn/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O725" s="2" t="inlineStr"/>
+      <c r="P725" s="2" t="inlineStr"/>
+      <c r="Q725" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R725" s="2" t="inlineStr"/>
+      <c r="S725" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="2" t="inlineStr">
+        <is>
+          <t>Sebastian Baez</t>
+        </is>
+      </c>
+      <c r="B726" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C726" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Sebastian Baez FROZENFRACTOR -1/0 SSP One Of 5</t>
+        </is>
+      </c>
+      <c r="D726" s="2" t="inlineStr">
+        <is>
+          <t>1/0</t>
+        </is>
+      </c>
+      <c r="E726" s="2" t="inlineStr">
+        <is>
+          <t>001 of 0</t>
+        </is>
+      </c>
+      <c r="F726" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G726" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/920028583607</t>
+        </is>
+      </c>
+      <c r="H726" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I726" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/v0gAAeSwLb5qyvy9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J726" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T03:12:04.000Z</t>
+        </is>
+      </c>
+      <c r="K726" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L726" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M726" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N726" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uRAAAeSwozhqyvy-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O726" s="2" t="inlineStr"/>
+      <c r="P726" s="2" t="inlineStr"/>
+      <c r="Q726" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R726" s="2" t="inlineStr"/>
+      <c r="S726" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="2" t="inlineStr">
+        <is>
+          <t>Aryna Sabalenka</t>
+        </is>
+      </c>
+      <c r="B727" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 TOPPS CHROME TENNIS CHROME AUTOGRAPHS</t>
+        </is>
+      </c>
+      <c r="C727" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS CHROME AUTO RED GEOMETRIC ARYNA SABALENKA 1/5 PSA 10</t>
+        </is>
+      </c>
+      <c r="D727" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E727" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F727" s="2" t="inlineStr">
+        <is>
+          <t>3500.00 USD</t>
+        </is>
+      </c>
+      <c r="G727" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307223638380</t>
+        </is>
+      </c>
+      <c r="H727" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I727" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SY8AAeSwHa1qybOW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J727" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T01:54:00.000Z</t>
+        </is>
+      </c>
+      <c r="K727" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L727" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M727" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 10</t>
+        </is>
+      </c>
+      <c r="N727" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/GnsAAeSwu-NqybOW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O727" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P727" s="2" t="inlineStr"/>
+      <c r="Q727" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R727" s="2" t="inlineStr"/>
+      <c r="S727" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" s="2" t="inlineStr">
+        <is>
+          <t>Lulu Sun</t>
+        </is>
+      </c>
+      <c r="B728" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C728" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Lulu Sun RC Rookie Orange Geometric Refractor 1/25 DN43</t>
+        </is>
+      </c>
+      <c r="D728" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E728" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F728" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G728" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407281859602</t>
+        </is>
+      </c>
+      <c r="H728" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I728" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/tkIAAeSwRSxqyupo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J728" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T01:43:18.000Z</t>
+        </is>
+      </c>
+      <c r="K728" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L728" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M728" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N728" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/D8YAAeSwG3dqyupp/s-l1600.jpg | https://i.ebayimg.com/images/g/-esAAeSwGEtqyupo/s-l1600.jpg | https://i.ebayimg.com/images/g/1~oAAeSwVe5qyupo/s-l1600.jpg | https://i.ebayimg.com/images/g/rUQAAeSwGMFqyupo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O728" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P728" s="2" t="inlineStr"/>
+      <c r="Q728" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R728" s="2" t="inlineStr"/>
+      <c r="S728" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="2" t="inlineStr">
+        <is>
+          <t>Ben Shelton</t>
+        </is>
+      </c>
+      <c r="B729" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 TOPPS CHROME TENNIS YOUTHQUAKE AUTOGRAPHS</t>
+        </is>
+      </c>
+      <c r="C729" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS YOUTHQUAKE #YS-BS BEN SHELTON 1/10 PSA 8 DNA AUTO 10</t>
+        </is>
+      </c>
+      <c r="D729" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E729" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F729" s="2" t="inlineStr">
+        <is>
+          <t>37.00 USD</t>
+        </is>
+      </c>
+      <c r="G729" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/900001791674</t>
+        </is>
+      </c>
+      <c r="H729" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I729" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/e8EAAeSw2fxqyXp2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J729" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T01:00:00.000Z</t>
+        </is>
+      </c>
+      <c r="K729" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L729" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M729" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 8</t>
+        </is>
+      </c>
+      <c r="N729" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/izQAAeSwdzdqyXp1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O729" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P729" s="2" t="inlineStr"/>
+      <c r="Q729" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R729" s="2" t="inlineStr"/>
+      <c r="S729" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="2" t="inlineStr">
+        <is>
+          <t>Maria Sharapova</t>
+        </is>
+      </c>
+      <c r="B730" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C730" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis World Number 1 Maria Sharapova Red Geometric # 1 /5 🔥</t>
+        </is>
+      </c>
+      <c r="D730" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E730" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F730" s="2" t="inlineStr">
+        <is>
+          <t>1500.00 USD</t>
+        </is>
+      </c>
+      <c r="G730" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/820225893926</t>
+        </is>
+      </c>
+      <c r="H730" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I730" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~5YAAeSwBVpqytPP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J730" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T00:14:23.000Z</t>
+        </is>
+      </c>
+      <c r="K730" s="2" t="inlineStr">
+        <is>
+          <t>Auction + Buy It Now</t>
+        </is>
+      </c>
+      <c r="L730" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M730" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N730" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/5lMAAeSweAlqytPf/s-l1600.jpg | https://i.ebayimg.com/images/g/GJoAAeSwV19qytQN/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O730" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P730" s="2" t="inlineStr"/>
+      <c r="Q730" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R730" s="2" t="inlineStr"/>
+      <c r="S730" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="2" t="inlineStr">
+        <is>
+          <t>Jasmine Paolini</t>
+        </is>
+      </c>
+      <c r="B731" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C731" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Jasmine Paolini Orange Geometric 25/25 #40</t>
+        </is>
+      </c>
+      <c r="D731" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E731" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F731" s="2" t="inlineStr">
+        <is>
+          <t>11.99 USD</t>
+        </is>
+      </c>
+      <c r="G731" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336838266933</t>
+        </is>
+      </c>
+      <c r="H731" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I731" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3AcAAeSwB9ZqykzA/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J731" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T23:55:01.000Z</t>
+        </is>
+      </c>
+      <c r="K731" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L731" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M731" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N731" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DRoAAeSwmZNqykzB/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O731" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P731" s="2" t="inlineStr"/>
+      <c r="Q731" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R731" s="2" t="inlineStr"/>
+      <c r="S731" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="2" t="inlineStr">
+        <is>
+          <t>Jessica Pegula</t>
+        </is>
+      </c>
+      <c r="B732" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 TOPPS GRAPHITE TENNIS FULL EXTENSION</t>
+        </is>
+      </c>
+      <c r="C732" s="2" t="inlineStr">
+        <is>
+          <t>2026 TOPPS GRAPHITE TENNIS FULL EXTENSION #FE-6 JESSICA PEGULA 1/1 PSA 9</t>
+        </is>
+      </c>
+      <c r="D732" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E732" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F732" s="2" t="inlineStr">
+        <is>
+          <t>1999.00 USD</t>
+        </is>
+      </c>
+      <c r="G732" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/900006026528</t>
+        </is>
+      </c>
+      <c r="H732" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I732" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8lsAAeSwRSxqy6e8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J732" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T15:13:00.000Z</t>
+        </is>
+      </c>
+      <c r="K732" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L732" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M732" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N732" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0~cAAeSw4dJqy6e7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O732" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P732" s="2" t="inlineStr"/>
+      <c r="Q732" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R732" s="2" t="inlineStr"/>
+      <c r="S732" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="2" t="inlineStr">
+        <is>
+          <t>Claire Liu</t>
+        </is>
+      </c>
+      <c r="B733" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C733" s="2" t="inlineStr">
+        <is>
+          <t>Claire Liu 🇺🇸 #15/15 Pink Refractor -- 2026 Topps Graphite 🎾 #95</t>
+        </is>
+      </c>
+      <c r="D733" s="2" t="inlineStr">
+        <is>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="E733" s="2" t="inlineStr">
+        <is>
+          <t>last of 15 (15/15)</t>
+        </is>
+      </c>
+      <c r="F733" s="2" t="inlineStr">
+        <is>
+          <t>19.95 USD</t>
+        </is>
+      </c>
+      <c r="G733" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/880005598964?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2FV08g3PyGDx8nefW4tDeE%2BFb2uBG69kpPFFbbtuCK4zbQjdLR4seRtejtv2Er9x39VRhGBMzVUecBbG1oPIYnk0xylR6BtinpeweIrIjtd5Qaw%2F7oLUuCsirvp2gF9ylWowGwvgaLwY7y09iw7CGnKb77If3PjrtG4t1goIVhcsxGJeHjMFfvE5Yd%2B4jByCns%3D</t>
+        </is>
+      </c>
+      <c r="H733" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I733" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ZGUAAeSw2fxqytt4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J733" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T00:42:49.000Z</t>
+        </is>
+      </c>
+      <c r="K733" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L733" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M733" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N733" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ZQMAAeSw5YVqytt4/s-l1600.jpg | https://i.ebayimg.com/images/g/i-cAAeSwnahqytt5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O733" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P733" s="2" t="inlineStr"/>
+      <c r="Q733" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R733" s="2" t="inlineStr"/>
+      <c r="S733" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="2" t="inlineStr">
+        <is>
+          <t>Eva Lys</t>
+        </is>
+      </c>
+      <c r="B734" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps</t>
+        </is>
+      </c>
+      <c r="C734" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Tennis Eva Lys Gold Refractor #1/25</t>
+        </is>
+      </c>
+      <c r="D734" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E734" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F734" s="2" t="inlineStr">
+        <is>
+          <t>75.00 USD</t>
+        </is>
+      </c>
+      <c r="G734" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/820225904402</t>
+        </is>
+      </c>
+      <c r="H734" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I734" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QQMAAeSwmRFqytXB/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J734" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T00:19:09.000Z</t>
+        </is>
+      </c>
+      <c r="K734" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L734" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M734" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N734" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SXwAAeSw-~dqytXN/s-l1600.jpg | https://i.ebayimg.com/images/g/MH0AAeSw24ZqytXT/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O734" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P734" s="2" t="inlineStr"/>
+      <c r="Q734" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R734" s="2" t="inlineStr"/>
+      <c r="S734" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" s="2" t="inlineStr">
+        <is>
+          <t>Alexandra Eala</t>
+        </is>
+      </c>
+      <c r="B735" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C735" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Rc Alexandra Eala Tour Relic Auto Pink # 1/15 Color Match</t>
+        </is>
+      </c>
+      <c r="D735" s="2" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="E735" s="2" t="inlineStr">
+        <is>
+          <t>001 of 15</t>
+        </is>
+      </c>
+      <c r="F735" s="2" t="inlineStr">
+        <is>
+          <t>3000.00 USD</t>
+        </is>
+      </c>
+      <c r="G735" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/820225824434</t>
+        </is>
+      </c>
+      <c r="H735" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I735" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/uKIAAeSwb7lqysuu/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J735" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T23:37:42.000Z</t>
+        </is>
+      </c>
+      <c r="K735" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L735" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M735" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N735" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0LEAAeSw8wZqysu-/s-l1600.jpg | https://i.ebayimg.com/images/g/vpcAAeSwFONqysv6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O735" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P735" s="2" t="inlineStr"/>
+      <c r="Q735" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R735" s="2" t="inlineStr"/>
+      <c r="S735" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="2" t="inlineStr">
+        <is>
+          <t>Andre Agassi, Pete Sampras</t>
+        </is>
+      </c>
+      <c r="B736" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C736" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Notable Rivalries Andre Agassi/Pete Sampras 1/10 #X1059</t>
+        </is>
+      </c>
+      <c r="D736" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E736" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F736" s="2" t="inlineStr">
+        <is>
+          <t>39.99 USD</t>
+        </is>
+      </c>
+      <c r="G736" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/327397975249</t>
+        </is>
+      </c>
+      <c r="H736" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I736" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/6wEAAeSw-~dqylrK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J736" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T15:34:28.000Z</t>
+        </is>
+      </c>
+      <c r="K736" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L736" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M736" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N736" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/4BgAAeSwpIdqylrO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O736" s="2" t="inlineStr"/>
+      <c r="P736" s="2" t="inlineStr"/>
+      <c r="Q736" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R736" s="2" t="inlineStr"/>
+      <c r="S736" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="2" t="inlineStr">
+        <is>
+          <t>Jordan Thompson</t>
+        </is>
+      </c>
+      <c r="B737" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Star Relics - Green</t>
+        </is>
+      </c>
+      <c r="C737" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Star Relics Green 1/5 Jordan Thompson BGS 9.5 Rookie RC 3hd</t>
+        </is>
+      </c>
+      <c r="D737" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E737" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F737" s="2" t="inlineStr">
+        <is>
+          <t>46.24 USD</t>
+        </is>
+      </c>
+      <c r="G737" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257793494901</t>
+        </is>
+      </c>
+      <c r="H737" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I737" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-BEAAeSwdbRqy1Y0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J737" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T09:25:07.000Z</t>
+        </is>
+      </c>
+      <c r="K737" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L737" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M737" s="2" t="inlineStr">
+        <is>
+          <t>Beckett (BGS) 9.5 GEM MINT</t>
+        </is>
+      </c>
+      <c r="N737" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ABcAAeSweptqy1Y0/s-l1600.jpg | https://i.ebayimg.com/images/g/5PoAAeSwNgZqy1Y0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O737" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P737" s="2" t="inlineStr"/>
+      <c r="Q737" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R737" s="2" t="inlineStr"/>
+      <c r="S737" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="2" t="inlineStr">
+        <is>
+          <t>Michael Chang, Hubert Hurkacz, Jamie Murray, Michael Mmoh</t>
+        </is>
+      </c>
+      <c r="B738" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Collection Tennis</t>
+        </is>
+      </c>
+      <c r="C738" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis Auto Lot (x6) Michael Chang Hurkacz 01/75 Murray Mmoh</t>
+        </is>
+      </c>
+      <c r="D738" s="2" t="inlineStr">
+        <is>
+          <t>1/75</t>
+        </is>
+      </c>
+      <c r="E738" s="2" t="inlineStr">
+        <is>
+          <t>001 of 75</t>
+        </is>
+      </c>
+      <c r="F738" s="2" t="inlineStr">
+        <is>
+          <t>35.00 USD</t>
+        </is>
+      </c>
+      <c r="G738" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/860024064547</t>
+        </is>
+      </c>
+      <c r="H738" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I738" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/UfMAAeSwUKVqx~q9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J738" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T02:21:00.000Z</t>
+        </is>
+      </c>
+      <c r="K738" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L738" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M738" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N738" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HwAAAeSw-bxqx~q-/s-l1600.jpg | https://i.ebayimg.com/images/g/U3sAAeSwA7xqx~q-/s-l1600.jpg | https://i.ebayimg.com/images/g/TV4AAeSwkIlqx~q~/s-l1600.jpg | https://i.ebayimg.com/images/g/2lQAAeSwu-Zqx~rA/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O738" s="2" t="inlineStr"/>
+      <c r="P738" s="2" t="inlineStr"/>
+      <c r="Q738" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R738" s="2" t="inlineStr"/>
+      <c r="S738" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="2" t="inlineStr">
+        <is>
+          <t>Arthur Rinderknech</t>
+        </is>
+      </c>
+      <c r="B739" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Collection Tennis</t>
+        </is>
+      </c>
+      <c r="C739" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis Triumph Relic Auto /75 Lot (x3) Rinderknech 01/75</t>
+        </is>
+      </c>
+      <c r="D739" s="2" t="inlineStr">
+        <is>
+          <t>1/75</t>
+        </is>
+      </c>
+      <c r="E739" s="2" t="inlineStr">
+        <is>
+          <t>001 of 75</t>
+        </is>
+      </c>
+      <c r="F739" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G739" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/860024064451</t>
+        </is>
+      </c>
+      <c r="H739" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I739" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/IxQAAeSwUVFqx~qL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J739" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T02:16:00.000Z</t>
+        </is>
+      </c>
+      <c r="K739" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L739" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M739" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N739" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/xDAAAeSwnpRqx~qL/s-l1600.jpg | https://i.ebayimg.com/images/g/mEkAAeSwlUBqx~qM/s-l1600.jpg | https://i.ebayimg.com/images/g/HD0AAeSwmZxqx~qN/s-l1600.jpg | https://i.ebayimg.com/images/g/mEsAAeSwlUBqx~qN/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O739" s="2" t="inlineStr"/>
+      <c r="P739" s="2" t="inlineStr"/>
+      <c r="Q739" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R739" s="2" t="inlineStr"/>
+      <c r="S739" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="2" t="inlineStr">
+        <is>
+          <t>Kaichi Uchida</t>
+        </is>
+      </c>
+      <c r="B740" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Collection Tennis</t>
+        </is>
+      </c>
+      <c r="C740" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis Kaichi Uchida Imperial Ink Auto 1/5 + 50/75 Lot (x2)</t>
+        </is>
+      </c>
+      <c r="D740" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E740" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F740" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G740" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/860024064354</t>
+        </is>
+      </c>
+      <c r="H740" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I740" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/R1EAAeSw2jBqx~pO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J740" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T02:10:00.000Z</t>
+        </is>
+      </c>
+      <c r="K740" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L740" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M740" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N740" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TdEAAeSw9mxqx~pP/s-l1600.jpg | https://i.ebayimg.com/images/g/2ZUAAeSwu-Zqx~pQ/s-l1600.jpg | https://i.ebayimg.com/images/g/TdQAAeSw9mxqx~pR/s-l1600.jpg | https://i.ebayimg.com/images/g/T~MAAeSwCilqx~pT/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O740" s="2" t="inlineStr"/>
+      <c r="P740" s="2" t="inlineStr"/>
+      <c r="Q740" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R740" s="2" t="inlineStr"/>
+      <c r="S740" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="2" t="inlineStr">
+        <is>
+          <t>Daniel Rincon, Grigor Dimitrov, Kim Clijsters, Madison Keys</t>
+        </is>
+      </c>
+      <c r="B741" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty Collection Tennis</t>
+        </is>
+      </c>
+      <c r="C741" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis /99 Lot (x8) Clijsters Keys Dimitrov Rincon RC 01/99</t>
+        </is>
+      </c>
+      <c r="D741" s="2" t="inlineStr">
+        <is>
+          <t>1/99</t>
+        </is>
+      </c>
+      <c r="E741" s="2" t="inlineStr">
+        <is>
+          <t>001 of 99</t>
+        </is>
+      </c>
+      <c r="F741" s="2" t="inlineStr">
+        <is>
+          <t>10.55 USD</t>
+        </is>
+      </c>
+      <c r="G741" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/860024064223</t>
+        </is>
+      </c>
+      <c r="H741" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I741" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~GwAAeSw4YJqx~ng/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J741" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T02:02:00.000Z</t>
+        </is>
+      </c>
+      <c r="K741" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L741" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M741" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N741" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ShYAAeSwKsVqx~nh/s-l1600.jpg | https://i.ebayimg.com/images/g/vm4AAeSwsp1qx~ni/s-l1600.jpg | https://i.ebayimg.com/images/g/GAYAAeSwC5Rqx~ni/s-l1600.jpg | https://i.ebayimg.com/images/g/ICoAAeSwUHVqx~nj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O741" s="2" t="inlineStr"/>
+      <c r="P741" s="2" t="inlineStr"/>
+      <c r="Q741" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R741" s="2" t="inlineStr"/>
+      <c r="S741" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="2" t="inlineStr">
+        <is>
+          <t>Liudmila Samsonova</t>
+        </is>
+      </c>
+      <c r="B742" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Prodigious Pairings - Gold</t>
+        </is>
+      </c>
+      <c r="C742" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Dual Relic Gold 10/10 Samsonova Kalinskaya Rookie RC</t>
+        </is>
+      </c>
+      <c r="D742" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E742" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F742" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G742" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257789372778</t>
+        </is>
+      </c>
+      <c r="H742" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I742" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/WkwAAeSw6D9qx-bU/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J742" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T00:37:59.000Z</t>
+        </is>
+      </c>
+      <c r="K742" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L742" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M742" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N742" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/W-YAAeSwUmpqx-bU/s-l1600.jpg | https://i.ebayimg.com/images/g/Wo4AAeSwMdhqx-bU/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O742" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P742" s="2" t="inlineStr"/>
+      <c r="Q742" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R742" s="2" t="inlineStr"/>
+      <c r="S742" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="2" t="inlineStr">
+        <is>
+          <t>Novak Djokovic</t>
+        </is>
+      </c>
+      <c r="B743" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS ROYALTY TENNIS</t>
+        </is>
+      </c>
+      <c r="C743" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS ROYALTY TENNIS PLATINUM 1/1 #2 NOVAK DJOKOVIC 1/1 PSA 9</t>
+        </is>
+      </c>
+      <c r="D743" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E743" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F743" s="2" t="inlineStr">
+        <is>
+          <t>50000.00 USD</t>
+        </is>
+      </c>
+      <c r="G743" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307225101779</t>
+        </is>
+      </c>
+      <c r="H743" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I743" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ihoAAeSwmhhqysxD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J743" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T23:36:36.000Z</t>
+        </is>
+      </c>
+      <c r="K743" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L743" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M743" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N743" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bG8AAeSwi5ZqysxD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O743" s="2" t="inlineStr"/>
+      <c r="P743" s="2" t="inlineStr"/>
+      <c r="Q743" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R743" s="2" t="inlineStr"/>
+      <c r="S743" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="2" t="inlineStr">
+        <is>
+          <t>Karolina Muchova</t>
+        </is>
+      </c>
+      <c r="B744" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Triumph Relic Signatures - Blue</t>
+        </is>
+      </c>
+      <c r="C744" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Blue 25/25 Karolina Muchova #TRS-KM Rookie Auto RC sv0</t>
+        </is>
+      </c>
+      <c r="D744" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E744" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F744" s="2" t="inlineStr">
+        <is>
+          <t>158.50 USD</t>
+        </is>
+      </c>
+      <c r="G744" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237118108594</t>
+        </is>
+      </c>
+      <c r="H744" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:52 UTC</t>
+        </is>
+      </c>
+      <c r="I744" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/xvYAAeSwVUlqyrKI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J744" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T21:46:49.000Z</t>
+        </is>
+      </c>
+      <c r="K744" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L744" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M744" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N744" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/u3IAAeSwZ~lqyrKI/s-l1600.jpg | https://i.ebayimg.com/images/g/z~0AAeSwffVqyrKI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O744" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P744" s="2" t="inlineStr"/>
+      <c r="Q744" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R744" s="2" t="inlineStr"/>
+      <c r="S744" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -64249,6 +66256,29 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G719" r:id="rId718"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G720" r:id="rId719"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G721" r:id="rId720"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G722" r:id="rId721"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G723" r:id="rId722"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G724" r:id="rId723"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G725" r:id="rId724"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G726" r:id="rId725"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G727" r:id="rId726"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G728" r:id="rId727"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G729" r:id="rId728"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G730" r:id="rId729"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G731" r:id="rId730"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G732" r:id="rId731"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G733" r:id="rId732"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G734" r:id="rId733"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G735" r:id="rId734"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G736" r:id="rId735"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G737" r:id="rId736"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G738" r:id="rId737"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G739" r:id="rId738"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G740" r:id="rId739"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G741" r:id="rId740"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G742" r:id="rId741"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G743" r:id="rId742"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G744" r:id="rId743"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-12 03:11 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S744"/>
+  <dimension ref="A1:S765"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -65529,6 +65529,1847 @@
       </c>
       <c r="R744" s="2" t="inlineStr"/>
       <c r="S744" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B745" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C745" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Coco Gauff #1 Purple Raywave Refractor 75/75 AJ85</t>
+        </is>
+      </c>
+      <c r="D745" s="2" t="inlineStr">
+        <is>
+          <t>75/75</t>
+        </is>
+      </c>
+      <c r="E745" s="2" t="inlineStr">
+        <is>
+          <t>last of 75 (75/75)</t>
+        </is>
+      </c>
+      <c r="F745" s="2" t="inlineStr">
+        <is>
+          <t>1.25 USD</t>
+        </is>
+      </c>
+      <c r="G745" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407279596936</t>
+        </is>
+      </c>
+      <c r="H745" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:09 UTC</t>
+        </is>
+      </c>
+      <c r="I745" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8igAAeSwqeFqyZgt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J745" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T01:42:02.000Z</t>
+        </is>
+      </c>
+      <c r="K745" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L745" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M745" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N745" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/5DAAAeSwHZRqyZgw/s-l1600.jpg | https://i.ebayimg.com/images/g/wg8AAeSwyExqyZgq/s-l1600.jpg | https://i.ebayimg.com/images/g/-SMAAeSweUZqyZgq/s-l1600.jpg | https://i.ebayimg.com/images/g/1KoAAeSwtcpqyZgq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O745" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P745" s="2" t="inlineStr"/>
+      <c r="Q745" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R745" s="2" t="inlineStr"/>
+      <c r="S745" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B746" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C746" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Coco Gauff Autograph Black 10/10 On Card</t>
+        </is>
+      </c>
+      <c r="D746" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E746" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F746" s="2" t="inlineStr">
+        <is>
+          <t>2000.00 USD</t>
+        </is>
+      </c>
+      <c r="G746" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147628188100</t>
+        </is>
+      </c>
+      <c r="H746" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:09 UTC</t>
+        </is>
+      </c>
+      <c r="I746" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/xR4AAeSwtHBqyVOV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J746" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T20:51:40.000Z</t>
+        </is>
+      </c>
+      <c r="K746" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L746" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M746" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N746" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/AsQAAeSwiiZqyVOV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O746" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P746" s="2" t="inlineStr"/>
+      <c r="Q746" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R746" s="2" t="inlineStr"/>
+      <c r="S746" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff</t>
+        </is>
+      </c>
+      <c r="B747" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite Tennis</t>
+        </is>
+      </c>
+      <c r="C747" s="2" t="inlineStr">
+        <is>
+          <t>Coco Gauff-2026 Topps Graphite Tour Relic Auto Gold SSP #01/25-Game Used🔥🔥</t>
+        </is>
+      </c>
+      <c r="D747" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E747" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F747" s="2" t="inlineStr">
+        <is>
+          <t>299.00 USD</t>
+        </is>
+      </c>
+      <c r="G747" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/960051104681</t>
+        </is>
+      </c>
+      <c r="H747" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:09 UTC</t>
+        </is>
+      </c>
+      <c r="I747" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Gx0AAeSwhthqnQDm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J747" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T06:00:58.000Z</t>
+        </is>
+      </c>
+      <c r="K747" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L747" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M747" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N747" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/q-sAAeSwG9FqnQDm/s-l1600.jpg | https://i.ebayimg.com/images/g/ZsgAAeSwhFRqnQDm/s-l1600.jpg | https://i.ebayimg.com/images/g/q7gAAeSwmElqnQDm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O747" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P747" s="2" t="inlineStr"/>
+      <c r="Q747" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R747" s="2" t="inlineStr"/>
+      <c r="S747" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B748" s="2" t="inlineStr">
+        <is>
+          <t>NetPro / 2022 Netpro Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="C748" s="2" t="inlineStr">
+        <is>
+          <t>CARLOS ALCARAZ 2022 NETPRO GOLDEN SLAM SUPERFRACTOR RC #1/1 *SGC 10 GEM MINT*!</t>
+        </is>
+      </c>
+      <c r="D748" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E748" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F748" s="2" t="inlineStr">
+        <is>
+          <t>888000.00 USD</t>
+        </is>
+      </c>
+      <c r="G748" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377563128336</t>
+        </is>
+      </c>
+      <c r="H748" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:09 UTC</t>
+        </is>
+      </c>
+      <c r="I748" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/5j0AAeSwa3RqyNjz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J748" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T00:00:55.000Z</t>
+        </is>
+      </c>
+      <c r="K748" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L748" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M748" s="2" t="inlineStr">
+        <is>
+          <t>SGC 10</t>
+        </is>
+      </c>
+      <c r="N748" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/h74AAeSwYhNqyNg3/s-l1600.jpg | https://i.ebayimg.com/images/g/y6YAAeSwbaxqyNg5/s-l1600.jpg | https://i.ebayimg.com/images/g/1VIAAeSwBVpqyT8C/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O748" s="2" t="inlineStr"/>
+      <c r="P748" s="2" t="inlineStr"/>
+      <c r="Q748" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R748" s="2" t="inlineStr"/>
+      <c r="S748" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B749" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 TOPPS CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="C749" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS ORANGE GEOMETRIC #1 CARLOS ALCARAZ 1/25 PSA 10</t>
+        </is>
+      </c>
+      <c r="D749" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E749" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F749" s="2" t="inlineStr">
+        <is>
+          <t>500.00 USD</t>
+        </is>
+      </c>
+      <c r="G749" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298743407914</t>
+        </is>
+      </c>
+      <c r="H749" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:09 UTC</t>
+        </is>
+      </c>
+      <c r="I749" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/WPMAAeSwGxxqx-TS/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J749" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T01:51:00.000Z</t>
+        </is>
+      </c>
+      <c r="K749" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L749" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M749" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 10</t>
+        </is>
+      </c>
+      <c r="N749" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YogAAeSwxDNqx-TS/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O749" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P749" s="2" t="inlineStr"/>
+      <c r="Q749" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R749" s="2" t="inlineStr"/>
+      <c r="S749" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B750" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C750" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Carlos Alcaraz Destiny #DTY-ALC Red Geometric 1/5</t>
+        </is>
+      </c>
+      <c r="D750" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E750" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F750" s="2" t="inlineStr">
+        <is>
+          <t>1800.00 USD</t>
+        </is>
+      </c>
+      <c r="G750" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/860023915849</t>
+        </is>
+      </c>
+      <c r="H750" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:09 UTC</t>
+        </is>
+      </c>
+      <c r="I750" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XwYAAeSwCYJqx-UH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J750" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T18:53:48.000Z</t>
+        </is>
+      </c>
+      <c r="K750" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L750" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M750" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N750" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Y-IAAeSwqdFqx-UH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O750" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P750" s="2" t="inlineStr"/>
+      <c r="Q750" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R750" s="2" t="inlineStr"/>
+      <c r="S750" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="2" t="inlineStr">
+        <is>
+          <t>Pete Sampras</t>
+        </is>
+      </c>
+      <c r="B751" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C751" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Pete Sampras Red Geometric #200 #1/5</t>
+        </is>
+      </c>
+      <c r="D751" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E751" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F751" s="2" t="inlineStr">
+        <is>
+          <t>599.99 USD</t>
+        </is>
+      </c>
+      <c r="G751" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/128117057738</t>
+        </is>
+      </c>
+      <c r="H751" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:09 UTC</t>
+        </is>
+      </c>
+      <c r="I751" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JiQAAeSwznhqxCWy/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J751" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T22:34:18.000Z</t>
+        </is>
+      </c>
+      <c r="K751" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L751" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M751" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N751" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/hKEAAeSwQ6JqxCW8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O751" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P751" s="2" t="inlineStr"/>
+      <c r="Q751" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R751" s="2" t="inlineStr"/>
+      <c r="S751" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="2" t="inlineStr">
+        <is>
+          <t>Andre Agassi</t>
+        </is>
+      </c>
+      <c r="B752" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C752" s="2" t="inlineStr">
+        <is>
+          <t>Andre Agassi 2024 Topps Chrome Tennis Sapphire #168 Orange Refractor 25/25 SP</t>
+        </is>
+      </c>
+      <c r="D752" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E752" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F752" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G752" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/267809138384</t>
+        </is>
+      </c>
+      <c r="H752" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:10 UTC</t>
+        </is>
+      </c>
+      <c r="I752" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/lFoAAeSwkBlqyThG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J752" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T18:55:10.000Z</t>
+        </is>
+      </c>
+      <c r="K752" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L752" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M752" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N752" s="2" t="inlineStr"/>
+      <c r="O752" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P752" s="2" t="inlineStr"/>
+      <c r="Q752" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R752" s="2" t="inlineStr"/>
+      <c r="S752" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="2" t="inlineStr">
+        <is>
+          <t>Martina Hingis</t>
+        </is>
+      </c>
+      <c r="B753" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C753" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Martina Hingis World No. 1 /150 #WNO-MH Insert</t>
+        </is>
+      </c>
+      <c r="D753" s="2" t="inlineStr">
+        <is>
+          <t>1/150</t>
+        </is>
+      </c>
+      <c r="E753" s="2" t="inlineStr">
+        <is>
+          <t>001 of 150</t>
+        </is>
+      </c>
+      <c r="F753" s="2" t="inlineStr">
+        <is>
+          <t>9.99 USD</t>
+        </is>
+      </c>
+      <c r="G753" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407279232757</t>
+        </is>
+      </c>
+      <c r="H753" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:10 UTC</t>
+        </is>
+      </c>
+      <c r="I753" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/v7QAAeSwqRlqyWGz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J753" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:53:40.000Z</t>
+        </is>
+      </c>
+      <c r="K753" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L753" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M753" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N753" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/fYAAAeSwDNFqyWGz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O753" s="2" t="inlineStr"/>
+      <c r="P753" s="2" t="inlineStr"/>
+      <c r="Q753" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R753" s="2" t="inlineStr"/>
+      <c r="S753" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="2" t="inlineStr">
+        <is>
+          <t>Martina Hingis</t>
+        </is>
+      </c>
+      <c r="B754" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C754" s="2" t="inlineStr">
+        <is>
+          <t>1109 2026 TOPPS CHROME TENNIS MARTINA HINGIS SUPERFRACTOR 1/1</t>
+        </is>
+      </c>
+      <c r="D754" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E754" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F754" s="2" t="inlineStr">
+        <is>
+          <t>224.50 USD</t>
+        </is>
+      </c>
+      <c r="G754" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178559559393</t>
+        </is>
+      </c>
+      <c r="H754" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:10 UTC</t>
+        </is>
+      </c>
+      <c r="I754" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/mK4AAeSwGNdqxEbd/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J754" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T00:00:00.000Z</t>
+        </is>
+      </c>
+      <c r="K754" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L754" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M754" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA)</t>
+        </is>
+      </c>
+      <c r="N754" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2uIAAeSwU9tqxEbd/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O754" s="2" t="inlineStr"/>
+      <c r="P754" s="2" t="inlineStr"/>
+      <c r="Q754" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R754" s="2" t="inlineStr"/>
+      <c r="S754" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="2" t="inlineStr">
+        <is>
+          <t>Martina Hingis</t>
+        </is>
+      </c>
+      <c r="B755" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C755" s="2" t="inlineStr">
+        <is>
+          <t>Martina Hingis 2026 Topps Chrome Gold Refractor #181 50/50</t>
+        </is>
+      </c>
+      <c r="D755" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E755" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F755" s="2" t="inlineStr">
+        <is>
+          <t>99.99 USD</t>
+        </is>
+      </c>
+      <c r="G755" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366709000344</t>
+        </is>
+      </c>
+      <c r="H755" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:10 UTC</t>
+        </is>
+      </c>
+      <c r="I755" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7i4AAeSwesVqwWj0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J755" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T20:42:30.000Z</t>
+        </is>
+      </c>
+      <c r="K755" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L755" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M755" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N755" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RrAAAeSwCcBqwWj1/s-l1600.jpg | https://i.ebayimg.com/images/g/xoYAAeSwEWlqwWj1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O755" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P755" s="2" t="inlineStr"/>
+      <c r="Q755" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R755" s="2" t="inlineStr"/>
+      <c r="S755" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek</t>
+        </is>
+      </c>
+      <c r="B756" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C756" s="2" t="inlineStr">
+        <is>
+          <t>🔌iu 2026 Topps Chrome Tennis Captured Blue Refractor 1/150 Iga Swiatek</t>
+        </is>
+      </c>
+      <c r="D756" s="2" t="inlineStr">
+        <is>
+          <t>1/150</t>
+        </is>
+      </c>
+      <c r="E756" s="2" t="inlineStr">
+        <is>
+          <t>001 of 150</t>
+        </is>
+      </c>
+      <c r="F756" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G756" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/800770212969</t>
+        </is>
+      </c>
+      <c r="H756" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:10 UTC</t>
+        </is>
+      </c>
+      <c r="I756" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DQYAAeSwSX9qxUNW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J756" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T03:21:00.000Z</t>
+        </is>
+      </c>
+      <c r="K756" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L756" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M756" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N756" s="2" t="inlineStr"/>
+      <c r="O756" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P756" s="2" t="inlineStr"/>
+      <c r="Q756" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R756" s="2" t="inlineStr"/>
+      <c r="S756" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="2" t="inlineStr">
+        <is>
+          <t>Iga Swiatek</t>
+        </is>
+      </c>
+      <c r="B757" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C757" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Iga Swiatek Orange Geometric Refractor 1/25 #35 FOP</t>
+        </is>
+      </c>
+      <c r="D757" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E757" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F757" s="2" t="inlineStr">
+        <is>
+          <t>55.00 USD</t>
+        </is>
+      </c>
+      <c r="G757" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407268793803</t>
+        </is>
+      </c>
+      <c r="H757" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:10 UTC</t>
+        </is>
+      </c>
+      <c r="I757" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-uUAAeSwA9VqxB0u/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J757" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T21:57:26.000Z</t>
+        </is>
+      </c>
+      <c r="K757" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L757" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M757" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N757" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/sCUAAeSw1tRqxB00/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O757" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P757" s="2" t="inlineStr"/>
+      <c r="Q757" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R757" s="2" t="inlineStr"/>
+      <c r="S757" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Zverev</t>
+        </is>
+      </c>
+      <c r="B758" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C758" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Alexander Zverev Black Refractor #1/10</t>
+        </is>
+      </c>
+      <c r="D758" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E758" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F758" s="2" t="inlineStr">
+        <is>
+          <t>800.00 USD</t>
+        </is>
+      </c>
+      <c r="G758" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/189059034081</t>
+        </is>
+      </c>
+      <c r="H758" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:10 UTC</t>
+        </is>
+      </c>
+      <c r="I758" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bZYAAeSwNr5qxyDc/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J758" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T04:50:30.000Z</t>
+        </is>
+      </c>
+      <c r="K758" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L758" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M758" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N758" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RCIAAeSwjdRqxyDj/s-l1600.jpg | https://i.ebayimg.com/images/g/VxcAAeSw1~FqxyDo/s-l1600.jpg | https://i.ebayimg.com/images/g/xkkAAeSwJS9qxyDs/s-l1600.jpg | https://i.ebayimg.com/images/g/F8cAAeSwbHBqxyDw/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O758" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P758" s="2" t="inlineStr"/>
+      <c r="Q758" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R758" s="2" t="inlineStr"/>
+      <c r="S758" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B759" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C759" s="2" t="inlineStr">
+        <is>
+          <t>MIRRA ANDREEVA 2025 TOPPS CHROME TENNIS RED GEOMETRIC 5/5 #27 Q3861</t>
+        </is>
+      </c>
+      <c r="D759" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E759" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F759" s="2" t="inlineStr">
+        <is>
+          <t>14.50 USD</t>
+        </is>
+      </c>
+      <c r="G759" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/940001090701</t>
+        </is>
+      </c>
+      <c r="H759" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:10 UTC</t>
+        </is>
+      </c>
+      <c r="I759" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jp4AAeSwrQBqyQSJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J759" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T01:14:00.000Z</t>
+        </is>
+      </c>
+      <c r="K759" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L759" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M759" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N759" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/iOYAAeSwkBlqyQSJ/s-l1600.jpg | https://i.ebayimg.com/images/g/io4AAeSwLb5qyQSJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O759" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P759" s="2" t="inlineStr"/>
+      <c r="Q759" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R759" s="2" t="inlineStr"/>
+      <c r="S759" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B760" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C760" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Tennis Erika Andreeva Pineapple Refractor RC 77/77 Bookend</t>
+        </is>
+      </c>
+      <c r="D760" s="2" t="inlineStr">
+        <is>
+          <t>77/77</t>
+        </is>
+      </c>
+      <c r="E760" s="2" t="inlineStr">
+        <is>
+          <t>last of 77 (77/77)</t>
+        </is>
+      </c>
+      <c r="F760" s="2" t="inlineStr">
+        <is>
+          <t>10.00 USD</t>
+        </is>
+      </c>
+      <c r="G760" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237113226274</t>
+        </is>
+      </c>
+      <c r="H760" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:11 UTC</t>
+        </is>
+      </c>
+      <c r="I760" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JdEAAeSwqWZqxpSs/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J760" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T18:51:55.000Z</t>
+        </is>
+      </c>
+      <c r="K760" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L760" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M760" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N760" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JA4AAeSwq-JqxpS0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O760" s="2" t="inlineStr"/>
+      <c r="P760" s="2" t="inlineStr"/>
+      <c r="Q760" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R760" s="2" t="inlineStr"/>
+      <c r="S760" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="B761" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 26 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C761" s="2" t="inlineStr">
+        <is>
+          <t>26 Topps Chrome Tennis Mirra Andreeva Blue Geometric Auto Bookend  1/150!!!!</t>
+        </is>
+      </c>
+      <c r="D761" s="2" t="inlineStr">
+        <is>
+          <t>1/150</t>
+        </is>
+      </c>
+      <c r="E761" s="2" t="inlineStr">
+        <is>
+          <t>001 of 150</t>
+        </is>
+      </c>
+      <c r="F761" s="2" t="inlineStr">
+        <is>
+          <t>80.00 USD</t>
+        </is>
+      </c>
+      <c r="G761" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/206620007428</t>
+        </is>
+      </c>
+      <c r="H761" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:11 UTC</t>
+        </is>
+      </c>
+      <c r="I761" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YTMAAeSwO9VqwsHD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J761" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T21:20:40.000Z</t>
+        </is>
+      </c>
+      <c r="K761" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L761" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M761" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N761" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/shIAAeSw-ftqwsHB/s-l1600.jpg | https://i.ebayimg.com/images/g/6AsAAeSw9KxqwsHA/s-l1600.jpg | https://i.ebayimg.com/images/g/rUkAAeSw~C5qwsG-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O761" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P761" s="2" t="inlineStr"/>
+      <c r="Q761" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R761" s="2" t="inlineStr"/>
+      <c r="S761" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="2" t="inlineStr">
+        <is>
+          <t>Qinwen Zheng</t>
+        </is>
+      </c>
+      <c r="B762" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C762" s="2" t="inlineStr">
+        <is>
+          <t>Qinwen Zheng 2026 Topps Chrome Orange Geo Refractor Auto Autograph 25/25</t>
+        </is>
+      </c>
+      <c r="D762" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E762" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F762" s="2" t="inlineStr">
+        <is>
+          <t>599.00 USD</t>
+        </is>
+      </c>
+      <c r="G762" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168786106101</t>
+        </is>
+      </c>
+      <c r="H762" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:11 UTC</t>
+        </is>
+      </c>
+      <c r="I762" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/IDcAAeSwGVFqyE0j/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J762" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T21:24:55.000Z</t>
+        </is>
+      </c>
+      <c r="K762" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L762" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M762" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N762" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/aEAAAeSwB9JqyE0j/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O762" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P762" s="2" t="inlineStr"/>
+      <c r="Q762" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R762" s="2" t="inlineStr"/>
+      <c r="S762" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="2" t="inlineStr">
+        <is>
+          <t>Qinwen Zheng</t>
+        </is>
+      </c>
+      <c r="B763" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C763" s="2" t="inlineStr">
+        <is>
+          <t>QINWEN ZHENG 2025 TOPPS CHROME TENNIS #8 RED GEOMETRIC REFRACTOR 1/5 🔥</t>
+        </is>
+      </c>
+      <c r="D763" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E763" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F763" s="2" t="inlineStr">
+        <is>
+          <t>999.99 USD</t>
+        </is>
+      </c>
+      <c r="G763" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/206617398649?amdata=enc%3AAQALAAAAsCHNgUiiE%2FjQhlDTaMiAde8Z%2FykU9DerVW5vdEaQh8A8%2B%2B6suF6LLMJb7kNA02hh4Eiwo7Trq3hAVIv8kOYYomkvBa5Jg0fvcrVBN7g23j6nnXawQPmKBMWCkaBjcjZr3eDIGLR2OkB%2FYxtQGJkZgIHvXNSyl%2BQrFeXCO6UZHKQlIP45Y2cZpFIg7phVCFPVLe98od1bICve0KFmX2X0h0FV9mqHgSYQObiZPP5ipOqG</t>
+        </is>
+      </c>
+      <c r="H763" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:11 UTC</t>
+        </is>
+      </c>
+      <c r="I763" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TxcAAeSwF3dqyqQW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J763" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T20:47:31.000Z</t>
+        </is>
+      </c>
+      <c r="K763" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L763" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M763" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N763" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/AtwAAeSwWMVqyqQW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O763" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P763" s="2" t="inlineStr"/>
+      <c r="Q763" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R763" s="2" t="inlineStr"/>
+      <c r="S763" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" s="2" t="inlineStr">
+        <is>
+          <t>Qinwen Zheng</t>
+        </is>
+      </c>
+      <c r="B764" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Chrome Tennis Geometric Orange</t>
+        </is>
+      </c>
+      <c r="C764" s="2" t="inlineStr">
+        <is>
+          <t>2025  Topps Chrome Tennis Geometric Black Qinwen Zheng Auto 1/2 1/1 #CA-QZG</t>
+        </is>
+      </c>
+      <c r="D764" s="2" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="E764" s="2" t="inlineStr">
+        <is>
+          <t>001 of 2</t>
+        </is>
+      </c>
+      <c r="F764" s="2" t="inlineStr">
+        <is>
+          <t>3499.00 USD</t>
+        </is>
+      </c>
+      <c r="G764" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168769717765</t>
+        </is>
+      </c>
+      <c r="H764" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:11 UTC</t>
+        </is>
+      </c>
+      <c r="I764" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/cBkAAeSwU9tqxTZs/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J764" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T17:59:20.000Z</t>
+        </is>
+      </c>
+      <c r="K764" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L764" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M764" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N764" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nMcAAeSwUbVqxTZs/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O764" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P764" s="2" t="inlineStr"/>
+      <c r="Q764" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R764" s="2" t="inlineStr"/>
+      <c r="S764" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="2" t="inlineStr">
+        <is>
+          <t>Qinwen Zheng</t>
+        </is>
+      </c>
+      <c r="B765" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C765" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Qinwen Zheng Geometric auto eBay 1/1 🔥🔥🔥 tennis</t>
+        </is>
+      </c>
+      <c r="D765" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E765" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F765" s="2" t="inlineStr">
+        <is>
+          <t>325.00 USD</t>
+        </is>
+      </c>
+      <c r="G765" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336840477466</t>
+        </is>
+      </c>
+      <c r="H765" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 03:11 UTC</t>
+        </is>
+      </c>
+      <c r="I765" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Pa8AAeSwKexqpN1q/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J765" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T02:38:11.000Z</t>
+        </is>
+      </c>
+      <c r="K765" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L765" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M765" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N765" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gcUAAeSwmvhqpN10/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O765" s="2" t="inlineStr"/>
+      <c r="P765" s="2" t="inlineStr"/>
+      <c r="Q765" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R765" s="2" t="inlineStr"/>
+      <c r="S765" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -66279,6 +68120,27 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G742" r:id="rId741"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G743" r:id="rId742"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G744" r:id="rId743"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G745" r:id="rId744"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G746" r:id="rId745"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G747" r:id="rId746"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G748" r:id="rId747"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G749" r:id="rId748"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G750" r:id="rId749"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G751" r:id="rId750"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G752" r:id="rId751"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G753" r:id="rId752"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G754" r:id="rId753"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G755" r:id="rId754"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G756" r:id="rId755"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G757" r:id="rId756"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G758" r:id="rId757"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G759" r:id="rId758"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G760" r:id="rId759"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G761" r:id="rId760"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G762" r:id="rId761"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G763" r:id="rId762"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G764" r:id="rId763"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G765" r:id="rId764"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-12 05:12 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S765"/>
+  <dimension ref="A1:S766"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -67370,6 +67370,95 @@
       </c>
       <c r="R765" s="2" t="inlineStr"/>
       <c r="S765" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Nadal</t>
+        </is>
+      </c>
+      <c r="B766" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic</t>
+        </is>
+      </c>
+      <c r="C766" s="2" t="inlineStr">
+        <is>
+          <t>2008 Ace Auth. Rafael Nadal AUTO #S2 PSA 8 TOP POP 1/2 PSA Graded Tough Card!</t>
+        </is>
+      </c>
+      <c r="D766" s="2" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="E766" s="2" t="inlineStr">
+        <is>
+          <t>001 of 2</t>
+        </is>
+      </c>
+      <c r="F766" s="2" t="inlineStr">
+        <is>
+          <t>750.00 USD</t>
+        </is>
+      </c>
+      <c r="G766" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/188709642875</t>
+        </is>
+      </c>
+      <c r="H766" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 05:11 UTC</t>
+        </is>
+      </c>
+      <c r="I766" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/EOcAAeSw2OhqaUNV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J766" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29T00:06:20.000Z</t>
+        </is>
+      </c>
+      <c r="K766" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L766" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M766" s="2" t="inlineStr">
+        <is>
+          <t>PSA 8</t>
+        </is>
+      </c>
+      <c r="N766" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QnQAAeSwz-BqaUNV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O766" s="2" t="inlineStr"/>
+      <c r="P766" s="2" t="inlineStr"/>
+      <c r="Q766" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R766" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic autograph: on-card or sticker not stated; check by eye</t>
+        </is>
+      </c>
+      <c r="S766" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -68141,6 +68230,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G763" r:id="rId762"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G764" r:id="rId763"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G765" r:id="rId764"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G766" r:id="rId765"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-12 19:14 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S766"/>
+  <dimension ref="A1:S796"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -67459,6 +67459,2652 @@
         </is>
       </c>
       <c r="S766" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="2" t="inlineStr">
+        <is>
+          <t>Aryna Sabalenka</t>
+        </is>
+      </c>
+      <c r="B767" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C767" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Aryna Sabalenka Orange Geometric Captured #25/25 CTD-AS</t>
+        </is>
+      </c>
+      <c r="D767" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E767" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F767" s="2" t="inlineStr">
+        <is>
+          <t>129.99 USD</t>
+        </is>
+      </c>
+      <c r="G767" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/128131386792</t>
+        </is>
+      </c>
+      <c r="H767" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I767" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ndgAAeSwi21qzSlH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J767" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T18:40:03.000Z</t>
+        </is>
+      </c>
+      <c r="K767" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L767" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M767" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N767" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KsIAAeSwM05qzSlP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O767" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P767" s="2" t="inlineStr"/>
+      <c r="Q767" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R767" s="2" t="inlineStr"/>
+      <c r="S767" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="2" t="inlineStr">
+        <is>
+          <t>Qinwen Zheng</t>
+        </is>
+      </c>
+      <c r="B768" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C768" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Qinwen Zheng Black Geometric Destiny #01/10 DTY-ZHE</t>
+        </is>
+      </c>
+      <c r="D768" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E768" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F768" s="2" t="inlineStr">
+        <is>
+          <t>299.99 USD</t>
+        </is>
+      </c>
+      <c r="G768" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/128131383404</t>
+        </is>
+      </c>
+      <c r="H768" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I768" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ePsAAeSwZ6lqzSh9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J768" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T18:36:27.000Z</t>
+        </is>
+      </c>
+      <c r="K768" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L768" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M768" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N768" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/kpUAAeSwi21qzSiE/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O768" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P768" s="2" t="inlineStr"/>
+      <c r="Q768" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R768" s="2" t="inlineStr"/>
+      <c r="S768" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" s="2" t="inlineStr">
+        <is>
+          <t>Joao Fonseca</t>
+        </is>
+      </c>
+      <c r="B769" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Chrome Tennis Destiny Gold Geometric</t>
+        </is>
+      </c>
+      <c r="C769" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Joao Fonseca Destiny Gold Geometric RC 1/50 Refractor</t>
+        </is>
+      </c>
+      <c r="D769" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E769" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F769" s="2" t="inlineStr">
+        <is>
+          <t>49.99 USD</t>
+        </is>
+      </c>
+      <c r="G769" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/880011282298</t>
+        </is>
+      </c>
+      <c r="H769" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I769" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/K58AAeSwGEtqzRs9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J769" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T17:39:48.000Z</t>
+        </is>
+      </c>
+      <c r="K769" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L769" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M769" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N769" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XSgAAeSw24ZqzRs9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O769" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P769" s="2" t="inlineStr"/>
+      <c r="Q769" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R769" s="2" t="inlineStr"/>
+      <c r="S769" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="2" t="inlineStr">
+        <is>
+          <t>Erika Andreeva</t>
+        </is>
+      </c>
+      <c r="B770" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C770" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Erika Andreeva Orange Refractor 01/25  #24 Rookie RC</t>
+        </is>
+      </c>
+      <c r="D770" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E770" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F770" s="2" t="inlineStr">
+        <is>
+          <t>9.99 USD</t>
+        </is>
+      </c>
+      <c r="G770" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257795507719</t>
+        </is>
+      </c>
+      <c r="H770" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I770" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-NYAAeSwO9FqzRPz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J770" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T17:08:53.000Z</t>
+        </is>
+      </c>
+      <c r="K770" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L770" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M770" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N770" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HKoAAeSw0VlqzRPu/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O770" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P770" s="2" t="inlineStr"/>
+      <c r="Q770" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R770" s="2" t="inlineStr"/>
+      <c r="S770" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="2" t="inlineStr">
+        <is>
+          <t>Matteo Gigante</t>
+        </is>
+      </c>
+      <c r="B771" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C771" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2026 Topps Chrome Matteo Gigante #115 199/199 Tennis Card</t>
+        </is>
+      </c>
+      <c r="D771" s="2" t="inlineStr">
+        <is>
+          <t>199/199</t>
+        </is>
+      </c>
+      <c r="E771" s="2" t="inlineStr">
+        <is>
+          <t>last of 199 (199/199)</t>
+        </is>
+      </c>
+      <c r="F771" s="2" t="inlineStr">
+        <is>
+          <t>1.37 USD</t>
+        </is>
+      </c>
+      <c r="G771" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/920033051629</t>
+        </is>
+      </c>
+      <c r="H771" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I771" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/wUcAAeSww15qzQgo/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J771" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T16:18:59.000Z</t>
+        </is>
+      </c>
+      <c r="K771" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L771" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M771" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N771" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/eeYAAeSwonJqzQgU/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O771" s="2" t="inlineStr"/>
+      <c r="P771" s="2" t="inlineStr"/>
+      <c r="Q771" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R771" s="2" t="inlineStr"/>
+      <c r="S771" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="2" t="inlineStr">
+        <is>
+          <t>Chris Evert</t>
+        </is>
+      </c>
+      <c r="B772" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C772" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Chris Evert Black Geometric Bookend  10/10</t>
+        </is>
+      </c>
+      <c r="D772" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E772" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F772" s="2" t="inlineStr">
+        <is>
+          <t>90.00 USD</t>
+        </is>
+      </c>
+      <c r="G772" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/900008491827</t>
+        </is>
+      </c>
+      <c r="H772" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I772" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/GLsAAeSwcKBqzQXU/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J772" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T16:09:41.000Z</t>
+        </is>
+      </c>
+      <c r="K772" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L772" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M772" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N772" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/i4cAAeSwKT5qzQXR/s-l1600.jpg | https://i.ebayimg.com/images/g/cCUAAeSwUyJqzQXR/s-l1600.jpg | https://i.ebayimg.com/images/g/sOQAAeSwsy9qzQXS/s-l1600.jpg | https://i.ebayimg.com/images/g/NnAAAeSwa3RqzQXS/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O772" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="P772" s="2" t="inlineStr"/>
+      <c r="Q772" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R772" s="2" t="inlineStr"/>
+      <c r="S772" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="2" t="inlineStr">
+        <is>
+          <t>Erika Andreeva</t>
+        </is>
+      </c>
+      <c r="B773" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C773" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Erika Andreeva Base 1/5 Red Geometric Refractor CF18</t>
+        </is>
+      </c>
+      <c r="D773" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E773" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F773" s="2" t="inlineStr">
+        <is>
+          <t>50.00 USD</t>
+        </is>
+      </c>
+      <c r="G773" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/820231353094</t>
+        </is>
+      </c>
+      <c r="H773" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I773" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/zgAAAeSw-k5qzI5e/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J773" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T16:02:27.000Z</t>
+        </is>
+      </c>
+      <c r="K773" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L773" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M773" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N773" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gnYAAeSwUyJqzI5d/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O773" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P773" s="2" t="inlineStr"/>
+      <c r="Q773" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R773" s="2" t="inlineStr"/>
+      <c r="S773" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="2" t="inlineStr">
+        <is>
+          <t>Brandon Nakashima</t>
+        </is>
+      </c>
+      <c r="B774" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C774" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Brandon Nakashima Base 50/50 Gold Refractor #196 CF18</t>
+        </is>
+      </c>
+      <c r="D774" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E774" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F774" s="2" t="inlineStr">
+        <is>
+          <t>120.00 USD</t>
+        </is>
+      </c>
+      <c r="G774" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/820231353150</t>
+        </is>
+      </c>
+      <c r="H774" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I774" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/i7gAAeSwwE1qzLAk/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J774" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T16:01:54.000Z</t>
+        </is>
+      </c>
+      <c r="K774" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L774" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M774" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N774" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/N08AAeSwXgRqzLAk/s-l1600.jpg | https://i.ebayimg.com/images/g/8Z0AAeSwfwBqzLAl/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O774" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P774" s="2" t="inlineStr"/>
+      <c r="Q774" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R774" s="2" t="inlineStr"/>
+      <c r="S774" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="2" t="inlineStr">
+        <is>
+          <t>Brandon Nakashima</t>
+        </is>
+      </c>
+      <c r="B775" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C775" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Brandon Nakashima Base 50/50 Gold Refractor #196 CF18</t>
+        </is>
+      </c>
+      <c r="D775" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E775" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F775" s="2" t="inlineStr">
+        <is>
+          <t>50.00 USD</t>
+        </is>
+      </c>
+      <c r="G775" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/820231353160</t>
+        </is>
+      </c>
+      <c r="H775" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I775" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JjEAAeSwPQVqzK~n/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J775" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T16:01:54.000Z</t>
+        </is>
+      </c>
+      <c r="K775" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L775" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M775" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N775" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/wJ8AAeSwAzNqzK~n/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O775" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P775" s="2" t="inlineStr"/>
+      <c r="Q775" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R775" s="2" t="inlineStr"/>
+      <c r="S775" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="2" t="inlineStr">
+        <is>
+          <t>Monica Puig</t>
+        </is>
+      </c>
+      <c r="B776" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C776" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Pink Geometric Refractor 65/65 Monica Puig #157 Rookie RC 0q5k</t>
+        </is>
+      </c>
+      <c r="D776" s="2" t="inlineStr">
+        <is>
+          <t>65/65</t>
+        </is>
+      </c>
+      <c r="E776" s="2" t="inlineStr">
+        <is>
+          <t>last of 65 (65/65)</t>
+        </is>
+      </c>
+      <c r="F776" s="2" t="inlineStr">
+        <is>
+          <t>21.53 USD</t>
+        </is>
+      </c>
+      <c r="G776" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237120657997</t>
+        </is>
+      </c>
+      <c r="H776" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I776" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2OAAAeSwCjlqzQCV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J776" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T15:44:23.000Z</t>
+        </is>
+      </c>
+      <c r="K776" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L776" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M776" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N776" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/aEIAAeSw4y5qzQCV/s-l1600.jpg | https://i.ebayimg.com/images/g/HJUAAeSwB9ZqzQCV/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O776" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P776" s="2" t="inlineStr"/>
+      <c r="Q776" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R776" s="2" t="inlineStr"/>
+      <c r="S776" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="2" t="inlineStr">
+        <is>
+          <t>Zizou Bergs</t>
+        </is>
+      </c>
+      <c r="B777" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C777" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS CHROME TENNIS----ZIZOU BERGS---20/20---ROSE GOLD</t>
+        </is>
+      </c>
+      <c r="D777" s="2" t="inlineStr">
+        <is>
+          <t>20/20</t>
+        </is>
+      </c>
+      <c r="E777" s="2" t="inlineStr">
+        <is>
+          <t>last of 20 (20/20)</t>
+        </is>
+      </c>
+      <c r="F777" s="2" t="inlineStr">
+        <is>
+          <t>74.99 USD</t>
+        </is>
+      </c>
+      <c r="G777" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287643350676?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2Bw5lw3WM3DsO%2FjfQwY3wGBLWNGG7ErIRIIQzsaFCpzHbaEoOGcdiLGCvAtWVyOkNHXawKAdSvxp7luCYCF45Zdl5G8095GPi9ZgKvJ12XPmwpjMnpQDPctmfLpqJZ2sM0RFKzoU8w0c2M3gfb3kwmfM129B6J%2FCSeUSkXWYyUBSIFviuirngu3menekBhpex4%3D</t>
+        </is>
+      </c>
+      <c r="H777" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I777" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/UK4AAeSw42ZqzNEX/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J777" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T12:23:29.000Z</t>
+        </is>
+      </c>
+      <c r="K777" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L777" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M777" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N777" s="2" t="inlineStr"/>
+      <c r="O777" s="2" t="inlineStr"/>
+      <c r="P777" s="2" t="inlineStr"/>
+      <c r="Q777" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R777" s="2" t="inlineStr"/>
+      <c r="S777" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="2" t="inlineStr">
+        <is>
+          <t>Iva Jovic</t>
+        </is>
+      </c>
+      <c r="B778" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C778" s="2" t="inlineStr">
+        <is>
+          <t>Topps Chrome Tennis 2026 Iva Jovic Red Geometric Auto AT-IJC 5/5</t>
+        </is>
+      </c>
+      <c r="D778" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E778" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F778" s="2" t="inlineStr">
+        <is>
+          <t>1599.99 USD</t>
+        </is>
+      </c>
+      <c r="G778" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/920032200164</t>
+        </is>
+      </c>
+      <c r="H778" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I778" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/zgoAAeSwiFpqzAt6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J778" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T10:13:10.000Z</t>
+        </is>
+      </c>
+      <c r="K778" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L778" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M778" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N778" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RnsAAeSwu1dqzAjZ/s-l1600.jpg | https://i.ebayimg.com/images/g/qo8AAeSwu1pqzAjC/s-l1600.jpg | https://i.ebayimg.com/images/g/K5MAAeSwffVqzAjD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O778" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P778" s="2" t="inlineStr"/>
+      <c r="Q778" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R778" s="2" t="inlineStr"/>
+      <c r="S778" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="2" t="inlineStr">
+        <is>
+          <t>Thiago Agustin Tirante</t>
+        </is>
+      </c>
+      <c r="B779" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - [Base] - Black Geometric Refractor</t>
+        </is>
+      </c>
+      <c r="C779" s="2" t="inlineStr">
+        <is>
+          <t>2025 Chrome Black Geometric Refractor 2/2 Thiago Agustin Tirante Rookie RC 1w0z</t>
+        </is>
+      </c>
+      <c r="D779" s="2" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="E779" s="2" t="inlineStr">
+        <is>
+          <t>last of 2 (2/2)</t>
+        </is>
+      </c>
+      <c r="F779" s="2" t="inlineStr">
+        <is>
+          <t>207.95 USD</t>
+        </is>
+      </c>
+      <c r="G779" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257794986521</t>
+        </is>
+      </c>
+      <c r="H779" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I779" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TMcAAeSwHa1qzKML/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J779" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T09:04:58.000Z</t>
+        </is>
+      </c>
+      <c r="K779" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L779" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M779" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N779" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/yx4AAeSw-xtqzKML/s-l1600.jpg | https://i.ebayimg.com/images/g/-1sAAeSwyz5qzKML/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O779" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P779" s="2" t="inlineStr"/>
+      <c r="Q779" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R779" s="2" t="inlineStr"/>
+      <c r="S779" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="2" t="inlineStr">
+        <is>
+          <t>Kristy Pigeon</t>
+        </is>
+      </c>
+      <c r="B780" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2021 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C780" s="2" t="inlineStr">
+        <is>
+          <t>2021 Topps Chrome Red Refractor 1/5 Kristy Pigeon #CA-KP Rookie Auto RC HOF nd3</t>
+        </is>
+      </c>
+      <c r="D780" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E780" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F780" s="2" t="inlineStr">
+        <is>
+          <t>147.78 USD</t>
+        </is>
+      </c>
+      <c r="G780" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237120170482</t>
+        </is>
+      </c>
+      <c r="H780" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I780" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7JgAAeSwUR1qzJtH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J780" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T08:33:08.000Z</t>
+        </is>
+      </c>
+      <c r="K780" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L780" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M780" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N780" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Xd8AAeSw9D1qzJtH/s-l1600.jpg | https://i.ebayimg.com/images/g/zS0AAeSwHbxqzJtH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O780" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P780" s="2" t="inlineStr"/>
+      <c r="Q780" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R780" s="2" t="inlineStr"/>
+      <c r="S780" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="2" t="inlineStr">
+        <is>
+          <t>Borna Coric</t>
+        </is>
+      </c>
+      <c r="B781" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C781" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 2026 Topps Chrome Tennis Borna Coric Yellow Refractor 1/275 #128</t>
+        </is>
+      </c>
+      <c r="D781" s="2" t="inlineStr">
+        <is>
+          <t>1/275</t>
+        </is>
+      </c>
+      <c r="E781" s="2" t="inlineStr">
+        <is>
+          <t>001 of 275</t>
+        </is>
+      </c>
+      <c r="F781" s="2" t="inlineStr">
+        <is>
+          <t>1.99 USD</t>
+        </is>
+      </c>
+      <c r="G781" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/920031454098</t>
+        </is>
+      </c>
+      <c r="H781" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I781" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bAUAAeSwF3dqzGen/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J781" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T04:53:29.000Z</t>
+        </is>
+      </c>
+      <c r="K781" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L781" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M781" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N781" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Au0AAeSwb7lqzGen/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O781" s="2" t="inlineStr">
+        <is>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="P781" s="2" t="inlineStr"/>
+      <c r="Q781" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R781" s="2" t="inlineStr"/>
+      <c r="S781" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="2" t="inlineStr">
+        <is>
+          <t>Matteo Arnaldi</t>
+        </is>
+      </c>
+      <c r="B782" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C782" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 2026 Topps Chrome Tennis Matteo Arnaldi Pink Refractor Auto 1/250 #AT-MAI</t>
+        </is>
+      </c>
+      <c r="D782" s="2" t="inlineStr">
+        <is>
+          <t>1/250</t>
+        </is>
+      </c>
+      <c r="E782" s="2" t="inlineStr">
+        <is>
+          <t>001 of 250</t>
+        </is>
+      </c>
+      <c r="F782" s="2" t="inlineStr">
+        <is>
+          <t>5.99 USD</t>
+        </is>
+      </c>
+      <c r="G782" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/920031374045</t>
+        </is>
+      </c>
+      <c r="H782" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I782" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/hOsAAeSwo-RqzF50/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J782" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T04:14:25.000Z</t>
+        </is>
+      </c>
+      <c r="K782" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L782" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M782" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N782" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2poAAeSw5YVqzF50/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O782" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P782" s="2" t="inlineStr"/>
+      <c r="Q782" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R782" s="2" t="inlineStr"/>
+      <c r="S782" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="2" t="inlineStr">
+        <is>
+          <t>Hailey Baptiste</t>
+        </is>
+      </c>
+      <c r="B783" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C783" s="2" t="inlineStr">
+        <is>
+          <t>2026 TOPPS CHROME TENNIS #171 HAILEY BAPTISTE BLACK GEOMETRIC #10/10</t>
+        </is>
+      </c>
+      <c r="D783" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E783" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F783" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G783" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/900007108918</t>
+        </is>
+      </c>
+      <c r="H783" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I783" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/sWEAAeSwU9tqxuoK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J783" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T03:07:27.000Z</t>
+        </is>
+      </c>
+      <c r="K783" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L783" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M783" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N783" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/CjwAAeSw8qtqxuoP/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O783" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P783" s="2" t="inlineStr"/>
+      <c r="Q783" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R783" s="2" t="inlineStr"/>
+      <c r="S783" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="2" t="inlineStr">
+        <is>
+          <t>Garbine Muguruza</t>
+        </is>
+      </c>
+      <c r="B784" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - [Base] - Blue Refractor</t>
+        </is>
+      </c>
+      <c r="C784" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Blue Refractor 150/150 Garbine Muguruza Garbiñe #164 1p1u</t>
+        </is>
+      </c>
+      <c r="D784" s="2" t="inlineStr">
+        <is>
+          <t>150/150</t>
+        </is>
+      </c>
+      <c r="E784" s="2" t="inlineStr">
+        <is>
+          <t>last of 150 (150/150)</t>
+        </is>
+      </c>
+      <c r="F784" s="2" t="inlineStr">
+        <is>
+          <t>2.43 USD</t>
+        </is>
+      </c>
+      <c r="G784" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237119829845</t>
+        </is>
+      </c>
+      <c r="H784" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I784" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7u0AAeSwqRlqzEMt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J784" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T02:16:15.000Z</t>
+        </is>
+      </c>
+      <c r="K784" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L784" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M784" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N784" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/q38AAeSwbNpqzEMu/s-l1600.jpg | https://i.ebayimg.com/images/g/EcYAAeSwKT5qzEMt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O784" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P784" s="2" t="inlineStr"/>
+      <c r="Q784" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R784" s="2" t="inlineStr"/>
+      <c r="S784" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="2" t="inlineStr">
+        <is>
+          <t>Leandro Riedi</t>
+        </is>
+      </c>
+      <c r="B785" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C785" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Leandro Riedi Black Geometric 1/2 #154 FB11</t>
+        </is>
+      </c>
+      <c r="D785" s="2" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="E785" s="2" t="inlineStr">
+        <is>
+          <t>001 of 2</t>
+        </is>
+      </c>
+      <c r="F785" s="2" t="inlineStr">
+        <is>
+          <t>25.00 USD</t>
+        </is>
+      </c>
+      <c r="G785" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407283858134</t>
+        </is>
+      </c>
+      <c r="H785" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I785" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2wEAAeSwshRqzEDZ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J785" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T02:06:15.000Z</t>
+        </is>
+      </c>
+      <c r="K785" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L785" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M785" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N785" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HGcAAeSwsNpqzEDa/s-l1600.jpg | https://i.ebayimg.com/images/g/qHwAAeSw5YVqzEDY/s-l1600.jpg | https://i.ebayimg.com/images/g/yZ8AAeSwDtpqzEDY/s-l1600.jpg | https://i.ebayimg.com/images/g/~-4AAeSwi21qzEDY/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O785" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P785" s="2" t="inlineStr"/>
+      <c r="Q785" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R785" s="2" t="inlineStr"/>
+      <c r="S785" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="2" t="inlineStr">
+        <is>
+          <t>Flavio Cobolli</t>
+        </is>
+      </c>
+      <c r="B786" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topp Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C786" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Flavio Cobolli BLACK Refractor Parallel #8 10/10</t>
+        </is>
+      </c>
+      <c r="D786" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E786" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F786" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G786" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/840011881232</t>
+        </is>
+      </c>
+      <c r="H786" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I786" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2YUAAeSw8wZqzCz~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J786" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T02:06:00.000Z</t>
+        </is>
+      </c>
+      <c r="K786" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L786" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M786" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N786" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/mDEAAeSwOK1qzCz~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O786" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P786" s="2" t="inlineStr"/>
+      <c r="Q786" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R786" s="2" t="inlineStr"/>
+      <c r="S786" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="2" t="inlineStr">
+        <is>
+          <t>Anastasia Pavlyuchenkova</t>
+        </is>
+      </c>
+      <c r="B787" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C787" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Tennis Anastasia Pavlyuchenkova Red Crystalline Auto 1/1</t>
+        </is>
+      </c>
+      <c r="D787" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E787" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F787" s="2" t="inlineStr">
+        <is>
+          <t>100.00 USD</t>
+        </is>
+      </c>
+      <c r="G787" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/840014833396?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde9VhNhzP%2FSzliVasQTAX9ZACAGVRzzXeA%2BD8Ul5Y2gzje11U4p8pltwHyG1vDYGxY8uCeKoOIn6QIJy62UoMq0%2FP4OHvIOxHdcxa9xNQcRsCK4S0GqkZx984F2gMeWe15yatX08F5z3V6DaWhE8oA40v1z7edZAvSMTVnMyJsAyfkp3ijFj9GrfkAHZrL7jkrY%3D</t>
+        </is>
+      </c>
+      <c r="H787" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I787" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Xa0AAeSw0lhqzS14/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J787" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T19:03:13.000Z</t>
+        </is>
+      </c>
+      <c r="K787" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L787" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M787" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N787" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/fhEAAeSwjuZqzS1-/s-l1600.jpg | https://i.ebayimg.com/images/g/wgQAAeSwdOxqzS12/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O787" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P787" s="2" t="inlineStr"/>
+      <c r="Q787" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R787" s="2" t="inlineStr"/>
+      <c r="S787" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" s="2" t="inlineStr">
+        <is>
+          <t>Frances Tiafoe</t>
+        </is>
+      </c>
+      <c r="B788" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C788" s="2" t="inlineStr">
+        <is>
+          <t>Frances Tiafoe 1/50 BLUE Refractor! 2026 Topps Graphite Tennis Court Masters FOP</t>
+        </is>
+      </c>
+      <c r="D788" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E788" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F788" s="2" t="inlineStr">
+        <is>
+          <t>14.99 USD</t>
+        </is>
+      </c>
+      <c r="G788" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/860037195697?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde%2BzQu5ocKzzCMksXvnsbsw%2FS8MaGV1wAz4x2Vh3jIJ5l4UcFkVuLRSiFqWdV7SgsbFIMicIPd3R6KDEK9cpd%2FLGoULBgZrHCxf3riXhLlYZgXiG9fnQkmSiD8y9ZOjBsbOwh5Jo6S6Bgy7i8f8RM22L3NB8vYNcN7WRirZ7YDVPeG7oMmeb7mmDUAhRxmJDha0%3D</t>
+        </is>
+      </c>
+      <c r="H788" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I788" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YnAAAeSwbkRqzQwe/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J788" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T16:39:42.000Z</t>
+        </is>
+      </c>
+      <c r="K788" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L788" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M788" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N788" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0lIAAeSwaGRqzQwe/s-l1600.jpg | https://i.ebayimg.com/images/g/i4sAAeSwZ~lqzQwe/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O788" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P788" s="2" t="inlineStr"/>
+      <c r="Q788" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R788" s="2" t="inlineStr"/>
+      <c r="S788" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="2" t="inlineStr">
+        <is>
+          <t>Madison Keys</t>
+        </is>
+      </c>
+      <c r="B789" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C789" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Tennis Madison Keys Graphite Relic 1/10 White Refractor CF18</t>
+        </is>
+      </c>
+      <c r="D789" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E789" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F789" s="2" t="inlineStr">
+        <is>
+          <t>35.00 USD</t>
+        </is>
+      </c>
+      <c r="G789" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/820231353128</t>
+        </is>
+      </c>
+      <c r="H789" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I789" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/EHsAAeSweXtqzI1t/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J789" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T16:02:27.000Z</t>
+        </is>
+      </c>
+      <c r="K789" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L789" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M789" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N789" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/zjwAAeSwtYZqzI1t/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O789" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P789" s="2" t="inlineStr"/>
+      <c r="Q789" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R789" s="2" t="inlineStr"/>
+      <c r="S789" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" s="2" t="inlineStr">
+        <is>
+          <t>Ekaterina Alexandrova</t>
+        </is>
+      </c>
+      <c r="B790" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C790" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Blue Refractor 1/50 Ekaterina Alexandrova #67 Rookie RC 11ng</t>
+        </is>
+      </c>
+      <c r="D790" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E790" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F790" s="2" t="inlineStr">
+        <is>
+          <t>14.34 USD</t>
+        </is>
+      </c>
+      <c r="G790" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336840761895</t>
+        </is>
+      </c>
+      <c r="H790" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I790" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Yw8AAeSwZXVqzJCY/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J790" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T07:46:32.000Z</t>
+        </is>
+      </c>
+      <c r="K790" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L790" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M790" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N790" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/VBsAAeSwLTZqzJCY/s-l1600.jpg | https://i.ebayimg.com/images/g/idUAAeSwshRqzJCY/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O790" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P790" s="2" t="inlineStr"/>
+      <c r="Q790" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R790" s="2" t="inlineStr"/>
+      <c r="S790" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="2" t="inlineStr">
+        <is>
+          <t>Xiyu Wang</t>
+        </is>
+      </c>
+      <c r="B791" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite - Rally Relics - Pink Refractor</t>
+        </is>
+      </c>
+      <c r="C791" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Rally Relics Pink Refractor 15/15 Xiyu Wang #RR-XW</t>
+        </is>
+      </c>
+      <c r="D791" s="2" t="inlineStr">
+        <is>
+          <t>15/15</t>
+        </is>
+      </c>
+      <c r="E791" s="2" t="inlineStr">
+        <is>
+          <t>last of 15 (15/15)</t>
+        </is>
+      </c>
+      <c r="F791" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G791" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336837370210</t>
+        </is>
+      </c>
+      <c r="H791" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I791" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/5tQAAeSwygRqyWav/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J791" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T03:34:20.000Z</t>
+        </is>
+      </c>
+      <c r="K791" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L791" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M791" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N791" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ww0AAeSwL59qyWav/s-l1600.jpg | https://i.ebayimg.com/images/g/ww4AAeSwL59qyWav/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O791" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P791" s="2" t="inlineStr"/>
+      <c r="Q791" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R791" s="2" t="inlineStr"/>
+      <c r="S791" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="2" t="inlineStr">
+        <is>
+          <t>Elena Rybakina</t>
+        </is>
+      </c>
+      <c r="B792" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty</t>
+        </is>
+      </c>
+      <c r="C792" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis Elena Rybakina 1/1 Royal Decree Autograph Platinum PSA</t>
+        </is>
+      </c>
+      <c r="D792" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E792" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F792" s="2" t="inlineStr">
+        <is>
+          <t>16999.99 USD</t>
+        </is>
+      </c>
+      <c r="G792" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/128129745222</t>
+        </is>
+      </c>
+      <c r="H792" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I792" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~ssAAeSwEAZqzDz2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J792" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T01:56:12.000Z</t>
+        </is>
+      </c>
+      <c r="K792" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L792" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M792" s="2" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="N792" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/mY0AAeSwKfRqzDz2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O792" s="2" t="inlineStr"/>
+      <c r="P792" s="2" t="inlineStr"/>
+      <c r="Q792" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R792" s="2" t="inlineStr"/>
+      <c r="S792" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="2" t="inlineStr">
+        <is>
+          <t>Bernarda Pera</t>
+        </is>
+      </c>
+      <c r="B793" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - Star Relics - Green</t>
+        </is>
+      </c>
+      <c r="C793" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Star Relics Green 1/5 Bernarda Pera #SRR-BP 1e41</t>
+        </is>
+      </c>
+      <c r="D793" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E793" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F793" s="2" t="inlineStr">
+        <is>
+          <t>34.75 USD</t>
+        </is>
+      </c>
+      <c r="G793" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237119812938</t>
+        </is>
+      </c>
+      <c r="H793" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I793" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/JekAAeSwsNxqzDz7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J793" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T01:49:46.000Z</t>
+        </is>
+      </c>
+      <c r="K793" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L793" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M793" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N793" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/NBgAAeSwPd1qzDz7/s-l1600.jpg | https://i.ebayimg.com/images/g/J94AAeSw~1hqzDz7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O793" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P793" s="2" t="inlineStr"/>
+      <c r="Q793" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R793" s="2" t="inlineStr"/>
+      <c r="S793" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" s="2" t="inlineStr">
+        <is>
+          <t>Ben Shelton</t>
+        </is>
+      </c>
+      <c r="B794" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Now</t>
+        </is>
+      </c>
+      <c r="C794" s="2" t="inlineStr">
+        <is>
+          <t>2026 TOPPS NOW TENNIS ORANGE CARD 01/25 BEN SHELTON #21 1st GRAND SLAM FINAL BID</t>
+        </is>
+      </c>
+      <c r="D794" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E794" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F794" s="2" t="inlineStr">
+        <is>
+          <t>24.99 USD</t>
+        </is>
+      </c>
+      <c r="G794" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/206620385685</t>
+        </is>
+      </c>
+      <c r="H794" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I794" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/K4wAAeSwF-5qzDeA/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J794" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T01:29:08.000Z</t>
+        </is>
+      </c>
+      <c r="K794" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L794" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M794" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N794" s="2" t="inlineStr"/>
+      <c r="O794" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P794" s="2" t="inlineStr"/>
+      <c r="Q794" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R794" s="2" t="inlineStr"/>
+      <c r="S794" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="2" t="inlineStr">
+        <is>
+          <t>Elena Rybakina</t>
+        </is>
+      </c>
+      <c r="B795" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Now</t>
+        </is>
+      </c>
+      <c r="C795" s="2" t="inlineStr">
+        <is>
+          <t>Topps NOW 2026 Elena Rybakina #20 WTA Tour Tennis Card FOILFRACTOR 1/1</t>
+        </is>
+      </c>
+      <c r="D795" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E795" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F795" s="2" t="inlineStr">
+        <is>
+          <t>5000.00 USD</t>
+        </is>
+      </c>
+      <c r="G795" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366727481742</t>
+        </is>
+      </c>
+      <c r="H795" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I795" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KoQAAeSwKc9qy9tZ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J795" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T18:55:06.000Z</t>
+        </is>
+      </c>
+      <c r="K795" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L795" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M795" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N795" s="2" t="inlineStr"/>
+      <c r="O795" s="2" t="inlineStr"/>
+      <c r="P795" s="2" t="inlineStr"/>
+      <c r="Q795" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R795" s="2" t="inlineStr"/>
+      <c r="S795" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="2" t="inlineStr">
+        <is>
+          <t>Donald Young</t>
+        </is>
+      </c>
+      <c r="B796" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic / 2010 Ace Authentic</t>
+        </is>
+      </c>
+      <c r="C796" s="2" t="inlineStr">
+        <is>
+          <t>2010 Ace Authentic Gold 19/19 Donald Young #30 Auto 0f3</t>
+        </is>
+      </c>
+      <c r="D796" s="2" t="inlineStr">
+        <is>
+          <t>19/19</t>
+        </is>
+      </c>
+      <c r="E796" s="2" t="inlineStr">
+        <is>
+          <t>last of 19 (19/19)</t>
+        </is>
+      </c>
+      <c r="F796" s="2" t="inlineStr">
+        <is>
+          <t>7.71 USD</t>
+        </is>
+      </c>
+      <c r="G796" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336841424377</t>
+        </is>
+      </c>
+      <c r="H796" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 19:13 UTC</t>
+        </is>
+      </c>
+      <c r="I796" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/L7kAAeSwnd5qzR1t/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J796" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T17:47:26.000Z</t>
+        </is>
+      </c>
+      <c r="K796" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L796" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M796" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N796" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nRgAAeSwufhqzR1t/s-l1600.jpg | https://i.ebayimg.com/images/g/5toAAeSw1SdqzR1t/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O796" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P796" s="2" t="inlineStr"/>
+      <c r="Q796" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R796" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic autograph: on-card or sticker not stated; check by eye</t>
+        </is>
+      </c>
+      <c r="S796" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -68231,6 +70877,36 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G764" r:id="rId763"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G765" r:id="rId764"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G766" r:id="rId765"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G767" r:id="rId766"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G768" r:id="rId767"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G769" r:id="rId768"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G770" r:id="rId769"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G771" r:id="rId770"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G772" r:id="rId771"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G773" r:id="rId772"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G774" r:id="rId773"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G775" r:id="rId774"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G776" r:id="rId775"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G777" r:id="rId776"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G778" r:id="rId777"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G779" r:id="rId778"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G780" r:id="rId779"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G781" r:id="rId780"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G782" r:id="rId781"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G783" r:id="rId782"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G784" r:id="rId783"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G785" r:id="rId784"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G786" r:id="rId785"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G787" r:id="rId786"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G788" r:id="rId787"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G789" r:id="rId788"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G790" r:id="rId789"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G791" r:id="rId790"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G792" r:id="rId791"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G793" r:id="rId792"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G794" r:id="rId793"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G795" r:id="rId794"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G796" r:id="rId795"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-13 17:05 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S796"/>
+  <dimension ref="A1:S812"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -70105,6 +70105,1410 @@
         </is>
       </c>
       <c r="S796" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="2" t="inlineStr">
+        <is>
+          <t>Maya Joint</t>
+        </is>
+      </c>
+      <c r="B797" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C797" s="2" t="inlineStr">
+        <is>
+          <t>Maya Joint 2026 Topps Chrome Destiny True Orange Refractor 1/25 *First On Print*</t>
+        </is>
+      </c>
+      <c r="D797" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E797" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F797" s="2" t="inlineStr">
+        <is>
+          <t>80.00 USD</t>
+        </is>
+      </c>
+      <c r="G797" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/900011144299</t>
+        </is>
+      </c>
+      <c r="H797" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:03 UTC</t>
+        </is>
+      </c>
+      <c r="I797" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/floAAeSwH5Bqzloq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J797" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T16:26:35.000Z</t>
+        </is>
+      </c>
+      <c r="K797" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L797" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M797" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N797" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/lAQAAeSwGq5qzltm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O797" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P797" s="2" t="inlineStr"/>
+      <c r="Q797" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R797" s="2" t="inlineStr"/>
+      <c r="S797" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="2" t="inlineStr">
+        <is>
+          <t>Viktorija Golubic</t>
+        </is>
+      </c>
+      <c r="B798" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="C798" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Sapphire Red 1/5 Viktorija Golubic #4 Rookie RC 1w0z</t>
+        </is>
+      </c>
+      <c r="D798" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E798" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F798" s="2" t="inlineStr">
+        <is>
+          <t>29.87 USD</t>
+        </is>
+      </c>
+      <c r="G798" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257797098889</t>
+        </is>
+      </c>
+      <c r="H798" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:03 UTC</t>
+        </is>
+      </c>
+      <c r="I798" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/g-YAAeSwwHhqzltI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J798" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T16:23:33.000Z</t>
+        </is>
+      </c>
+      <c r="K798" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L798" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M798" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N798" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/boAAAeSwTlxqzltI/s-l1600.jpg | https://i.ebayimg.com/images/g/jQwAAeSwm0FqzltI/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O798" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P798" s="2" t="inlineStr"/>
+      <c r="Q798" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R798" s="2" t="inlineStr"/>
+      <c r="S798" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="2" t="inlineStr">
+        <is>
+          <t>Suzan Lamens</t>
+        </is>
+      </c>
+      <c r="B799" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C799" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Orange Geometric Suzan Lamens 25/25 RC Rookie #64</t>
+        </is>
+      </c>
+      <c r="D799" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E799" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F799" s="2" t="inlineStr">
+        <is>
+          <t>1.99 USD</t>
+        </is>
+      </c>
+      <c r="G799" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336842890283</t>
+        </is>
+      </c>
+      <c r="H799" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:03 UTC</t>
+        </is>
+      </c>
+      <c r="I799" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/O98AAeSwTEZqzllv/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J799" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T16:17:09.000Z</t>
+        </is>
+      </c>
+      <c r="K799" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L799" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M799" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N799" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/xJQAAeSwWfNqzllz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O799" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P799" s="2" t="inlineStr"/>
+      <c r="Q799" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R799" s="2" t="inlineStr"/>
+      <c r="S799" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="2" t="inlineStr">
+        <is>
+          <t>Alycia Parks</t>
+        </is>
+      </c>
+      <c r="B800" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C800" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Alycia Parks Chrome Black 1/10 ON CARD AUTO</t>
+        </is>
+      </c>
+      <c r="D800" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E800" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F800" s="2" t="inlineStr">
+        <is>
+          <t>3.25 USD</t>
+        </is>
+      </c>
+      <c r="G800" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/327403373645</t>
+        </is>
+      </c>
+      <c r="H800" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:03 UTC</t>
+        </is>
+      </c>
+      <c r="I800" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/dgQAAeSwopdqzk9s/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J800" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T15:35:24.000Z</t>
+        </is>
+      </c>
+      <c r="K800" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L800" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M800" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N800" s="2" t="inlineStr"/>
+      <c r="O800" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P800" s="2" t="inlineStr"/>
+      <c r="Q800" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R800" s="2" t="inlineStr"/>
+      <c r="S800" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="2" t="inlineStr">
+        <is>
+          <t>Ann Li</t>
+        </is>
+      </c>
+      <c r="B801" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - [Base] - Orange Geometric Refractor</t>
+        </is>
+      </c>
+      <c r="C801" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Orange Geometric Refractor 25/25 Ann Li #136 1th4</t>
+        </is>
+      </c>
+      <c r="D801" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E801" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F801" s="2" t="inlineStr">
+        <is>
+          <t>14.63 USD</t>
+        </is>
+      </c>
+      <c r="G801" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336842745220</t>
+        </is>
+      </c>
+      <c r="H801" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:03 UTC</t>
+        </is>
+      </c>
+      <c r="I801" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Gh8AAeSwsypqzji1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J801" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T13:56:04.000Z</t>
+        </is>
+      </c>
+      <c r="K801" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L801" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M801" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N801" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/5-oAAeSwsy9qzji1/s-l1600.jpg | https://i.ebayimg.com/images/g/MDEAAeSwcxhqzji1/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O801" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P801" s="2" t="inlineStr"/>
+      <c r="Q801" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R801" s="2" t="inlineStr"/>
+      <c r="S801" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="2" t="inlineStr">
+        <is>
+          <t>Chris Evert</t>
+        </is>
+      </c>
+      <c r="B802" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C802" s="2" t="inlineStr">
+        <is>
+          <t>CHRIS EVERT 💥 2026 Topps Chrome Tennis 1/1 World #1 on card Auto Superfractor</t>
+        </is>
+      </c>
+      <c r="D802" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E802" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F802" s="2" t="inlineStr">
+        <is>
+          <t>8500.00 USD</t>
+        </is>
+      </c>
+      <c r="G802" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168789346406</t>
+        </is>
+      </c>
+      <c r="H802" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:03 UTC</t>
+        </is>
+      </c>
+      <c r="I802" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vLQAAeSwAmdqzdtW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J802" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T07:20:29.000Z</t>
+        </is>
+      </c>
+      <c r="K802" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L802" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M802" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N802" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/gUsAAeSwcKBqzdtW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O802" s="2" t="inlineStr"/>
+      <c r="P802" s="2" t="inlineStr"/>
+      <c r="Q802" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R802" s="2" t="inlineStr"/>
+      <c r="S802" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="2" t="inlineStr">
+        <is>
+          <t>Daniil Medvedev</t>
+        </is>
+      </c>
+      <c r="B803" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C803" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Danil Medvedev True Orange Refractor 1/25 Captured SSP!</t>
+        </is>
+      </c>
+      <c r="D803" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E803" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F803" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G803" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/960060625747</t>
+        </is>
+      </c>
+      <c r="H803" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:03 UTC</t>
+        </is>
+      </c>
+      <c r="I803" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/n7YAAeSwa3Rqzcr9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J803" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T06:10:09.000Z</t>
+        </is>
+      </c>
+      <c r="K803" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L803" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M803" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N803" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/kjgAAeSwK8dqzcr9/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O803" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P803" s="2" t="inlineStr"/>
+      <c r="Q803" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R803" s="2" t="inlineStr"/>
+      <c r="S803" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="2" t="inlineStr">
+        <is>
+          <t>Radu Albot</t>
+        </is>
+      </c>
+      <c r="B804" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome - [Base] - Black Geometric Refractor</t>
+        </is>
+      </c>
+      <c r="C804" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Black Geometric Refractor 2/2 Radu Albot #166 Rookie RC 3h1</t>
+        </is>
+      </c>
+      <c r="D804" s="2" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="E804" s="2" t="inlineStr">
+        <is>
+          <t>last of 2 (2/2)</t>
+        </is>
+      </c>
+      <c r="F804" s="2" t="inlineStr">
+        <is>
+          <t>46.83 USD</t>
+        </is>
+      </c>
+      <c r="G804" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237121505034</t>
+        </is>
+      </c>
+      <c r="H804" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:03 UTC</t>
+        </is>
+      </c>
+      <c r="I804" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nt8AAeSwUrVqzb5y/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J804" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T05:14:28.000Z</t>
+        </is>
+      </c>
+      <c r="K804" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L804" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M804" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N804" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/in8AAeSwahNqzb5y/s-l1600.jpg | https://i.ebayimg.com/images/g/KD4AAeSwL1Nqzb5y/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O804" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P804" s="2" t="inlineStr"/>
+      <c r="Q804" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R804" s="2" t="inlineStr"/>
+      <c r="S804" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="2" t="inlineStr">
+        <is>
+          <t>Stefanos Tsitsipas</t>
+        </is>
+      </c>
+      <c r="B805" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C805" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2026 Chrome Tennis Stefanos Tsitsipas Captured Insert CTD-ST 1/50</t>
+        </is>
+      </c>
+      <c r="D805" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E805" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F805" s="2" t="inlineStr">
+        <is>
+          <t>100.00 USD</t>
+        </is>
+      </c>
+      <c r="G805" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366730393201</t>
+        </is>
+      </c>
+      <c r="H805" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:03 UTC</t>
+        </is>
+      </c>
+      <c r="I805" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/V0oAAeSw96FqzagD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J805" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T03:42:23.000Z</t>
+        </is>
+      </c>
+      <c r="K805" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L805" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M805" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N805" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Xq0AAeSweAlqzaf~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O805" s="2" t="inlineStr"/>
+      <c r="P805" s="2" t="inlineStr"/>
+      <c r="Q805" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R805" s="2" t="inlineStr"/>
+      <c r="S805" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="2" t="inlineStr">
+        <is>
+          <t>Maria Sharapova</t>
+        </is>
+      </c>
+      <c r="B806" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C806" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis MARIA SHARAPOVA Frozenfractor SSP -1/0 - Print Run Of 5</t>
+        </is>
+      </c>
+      <c r="D806" s="2" t="inlineStr">
+        <is>
+          <t>1/0</t>
+        </is>
+      </c>
+      <c r="E806" s="2" t="inlineStr">
+        <is>
+          <t>001 of 0</t>
+        </is>
+      </c>
+      <c r="F806" s="2" t="inlineStr">
+        <is>
+          <t>3188.49 USD</t>
+        </is>
+      </c>
+      <c r="G806" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377566183230?amdata=enc%3AAQALAAAAsCHNgUiiE%2FjQhlDTaMiAde8UE4Fuomao16pqjFKtugY6z%2FHu3eJt%2BT%2Firgv6RuYEpDjljqgMUxjv44GKfvVyqG1jHebO7B4Xhb3AAB6T8FP3HmDBw%2BaJiY%2BoV6%2BA5Ho6lfucHF9xtBHhz%2B%2BNsT3gnuLoSHDMLOfbk8EroXLJbACx%2B%2FZL%2BWILthkIdiRTFUPNM1zHTioiZnhHmgA0SCLXZvws7nTXs9A3WxB4RTtCAi3Y</t>
+        </is>
+      </c>
+      <c r="H806" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:03 UTC</t>
+        </is>
+      </c>
+      <c r="I806" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3FEAAeSwRypqzaFY/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J806" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T03:19:18.000Z</t>
+        </is>
+      </c>
+      <c r="K806" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L806" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M806" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N806" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ub4AAeSwL~xqzaFY/s-l1600.jpg | https://i.ebayimg.com/images/g/IIAAAeSwrTNqzaFY/s-l1600.jpg | https://i.ebayimg.com/images/g/N04AAeSw2epqzaFY/s-l1600.jpg | https://i.ebayimg.com/images/g/x0AAAeSwC5lqzaFZ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O806" s="2" t="inlineStr"/>
+      <c r="P806" s="2" t="inlineStr"/>
+      <c r="Q806" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R806" s="2" t="inlineStr"/>
+      <c r="S806" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="2" t="inlineStr">
+        <is>
+          <t>Daniil Medvedev</t>
+        </is>
+      </c>
+      <c r="B807" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome - Autograph - Red Geometric Refractor</t>
+        </is>
+      </c>
+      <c r="C807" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Red Geometric Refractor 5/5 Daniil Medvedev #AO-DMV Auto 1o0i</t>
+        </is>
+      </c>
+      <c r="D807" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E807" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F807" s="2" t="inlineStr">
+        <is>
+          <t>175.00 USD</t>
+        </is>
+      </c>
+      <c r="G807" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257796159623</t>
+        </is>
+      </c>
+      <c r="H807" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:04 UTC</t>
+        </is>
+      </c>
+      <c r="I807" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2K8AAeSwRypqzk88/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J807" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T02:25:58.000Z</t>
+        </is>
+      </c>
+      <c r="K807" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L807" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M807" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N807" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/h~4AAeSw0z9qzk88/s-l1600.jpg | https://i.ebayimg.com/images/g/IroAAeSwdzZqzk88/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O807" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P807" s="2" t="inlineStr"/>
+      <c r="Q807" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R807" s="2" t="inlineStr"/>
+      <c r="S807" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Bublik</t>
+        </is>
+      </c>
+      <c r="B808" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C808" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Alexander Bublik Red Geometric Auto #5/5 Bookend 🔥 🔥</t>
+        </is>
+      </c>
+      <c r="D808" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E808" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F808" s="2" t="inlineStr">
+        <is>
+          <t>300.00 USD</t>
+        </is>
+      </c>
+      <c r="G808" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/206623171739</t>
+        </is>
+      </c>
+      <c r="H808" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:04 UTC</t>
+        </is>
+      </c>
+      <c r="I808" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/n5UAAeSwTVlqzZYC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J808" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T02:25:47.000Z</t>
+        </is>
+      </c>
+      <c r="K808" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L808" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M808" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N808" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/d3oAAeSwF3dqzZYC/s-l1600.jpg | https://i.ebayimg.com/images/g/Tl8AAeSwKfRqzZYD/s-l1600.jpg | https://i.ebayimg.com/images/g/RngAAeSwNxRqzZYD/s-l1600.jpg | https://i.ebayimg.com/images/g/~98AAeSwozhqzZYE/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O808" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P808" s="2" t="inlineStr"/>
+      <c r="Q808" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R808" s="2" t="inlineStr"/>
+      <c r="S808" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="2" t="inlineStr">
+        <is>
+          <t>Max Purcell</t>
+        </is>
+      </c>
+      <c r="B809" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C809" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Max Purcell Black Refractor 01/10 First On Print</t>
+        </is>
+      </c>
+      <c r="D809" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E809" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F809" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G809" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/147632542705</t>
+        </is>
+      </c>
+      <c r="H809" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:04 UTC</t>
+        </is>
+      </c>
+      <c r="I809" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ItUAAeSwH1Fqxtg6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J809" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T02:18:01.000Z</t>
+        </is>
+      </c>
+      <c r="K809" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L809" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M809" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N809" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/BiwAAeSwS3ZqxthD/s-l1600.jpg | https://i.ebayimg.com/images/g/N9AAAeSwwqpqxthM/s-l1600.jpg | https://i.ebayimg.com/images/g/2NAAAeSwButqxthc/s-l1600.jpg | https://i.ebayimg.com/images/g/Y34AAeSwaH1qxthh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O809" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P809" s="2" t="inlineStr"/>
+      <c r="Q809" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R809" s="2" t="inlineStr"/>
+      <c r="S809" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B810" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C810" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Carlos Alcaraz Captured Orange Geometric Bookend 25/25</t>
+        </is>
+      </c>
+      <c r="D810" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E810" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F810" s="2" t="inlineStr">
+        <is>
+          <t>1.25 USD</t>
+        </is>
+      </c>
+      <c r="G810" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/920034387799</t>
+        </is>
+      </c>
+      <c r="H810" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:04 UTC</t>
+        </is>
+      </c>
+      <c r="I810" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3CkAAeSwrQBqzZJ7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J810" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T02:08:37.000Z</t>
+        </is>
+      </c>
+      <c r="K810" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L810" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M810" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N810" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Uq8AAeSwKT5qzZKC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O810" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P810" s="2" t="inlineStr"/>
+      <c r="Q810" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R810" s="2" t="inlineStr"/>
+      <c r="S810" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="2" t="inlineStr">
+        <is>
+          <t>Anna Blinkova</t>
+        </is>
+      </c>
+      <c r="B811" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C811" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Graphite Active Metal Gold 25/25 Anna Blinkova #ACM-85 Rookie RC z7d</t>
+        </is>
+      </c>
+      <c r="D811" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E811" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F811" s="2" t="inlineStr">
+        <is>
+          <t>23.13 USD</t>
+        </is>
+      </c>
+      <c r="G811" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257796153126</t>
+        </is>
+      </c>
+      <c r="H811" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:04 UTC</t>
+        </is>
+      </c>
+      <c r="I811" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/PYUAAeSwVT5qzZQh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J811" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T02:13:46.000Z</t>
+        </is>
+      </c>
+      <c r="K811" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L811" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M811" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N811" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3ngAAeSwnNFqzZQh/s-l1600.jpg | https://i.ebayimg.com/images/g/T2EAAeSw1LJqzZQh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O811" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P811" s="2" t="inlineStr"/>
+      <c r="Q811" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R811" s="2" t="inlineStr"/>
+      <c r="S811" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="2" t="inlineStr">
+        <is>
+          <t>Ashlyn Krueger</t>
+        </is>
+      </c>
+      <c r="B812" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty - [Base]</t>
+        </is>
+      </c>
+      <c r="C812" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty 99/99 Ashlyn Krueger #21 Rookie RC 9et</t>
+        </is>
+      </c>
+      <c r="D812" s="2" t="inlineStr">
+        <is>
+          <t>99/99</t>
+        </is>
+      </c>
+      <c r="E812" s="2" t="inlineStr">
+        <is>
+          <t>last of 99 (99/99)</t>
+        </is>
+      </c>
+      <c r="F812" s="2" t="inlineStr">
+        <is>
+          <t>23.83 USD</t>
+        </is>
+      </c>
+      <c r="G812" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336842074541</t>
+        </is>
+      </c>
+      <c r="H812" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 17:04 UTC</t>
+        </is>
+      </c>
+      <c r="I812" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/U8sAAeSwVl9qzaul/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J812" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T03:54:13.000Z</t>
+        </is>
+      </c>
+      <c r="K812" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L812" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M812" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N812" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/oLgAAeSw2epqzaum/s-l1600.jpg | https://i.ebayimg.com/images/g/XvEAAeSwx7Rqzaul/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O812" s="2" t="inlineStr"/>
+      <c r="P812" s="2" t="inlineStr"/>
+      <c r="Q812" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R812" s="2" t="inlineStr"/>
+      <c r="S812" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -70907,6 +72311,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G794" r:id="rId793"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G795" r:id="rId794"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G796" r:id="rId795"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G797" r:id="rId796"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G798" r:id="rId797"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G799" r:id="rId798"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G800" r:id="rId799"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G801" r:id="rId800"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G802" r:id="rId801"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G803" r:id="rId802"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G804" r:id="rId803"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G805" r:id="rId804"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G806" r:id="rId805"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G807" r:id="rId806"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G808" r:id="rId807"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G809" r:id="rId808"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G810" r:id="rId809"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G811" r:id="rId810"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G812" r:id="rId811"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-14 14:37 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S812"/>
+  <dimension ref="A1:S832"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -71509,6 +71509,1762 @@
       </c>
       <c r="R812" s="2" t="inlineStr"/>
       <c r="S812" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="2" t="inlineStr">
+        <is>
+          <t>Hailey Baptiste</t>
+        </is>
+      </c>
+      <c r="B813" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C813" s="2" t="inlineStr">
+        <is>
+          <t>Hailey Baptiste Topps Chrome Tennis AUTO Rainbow 10 Cards Superfractor 1/1</t>
+        </is>
+      </c>
+      <c r="D813" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E813" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F813" s="2" t="inlineStr">
+        <is>
+          <t>1999.00 USD</t>
+        </is>
+      </c>
+      <c r="G813" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366733407706</t>
+        </is>
+      </c>
+      <c r="H813" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:36 UTC</t>
+        </is>
+      </c>
+      <c r="I813" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0rgAAeSwFhRqz1eF/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J813" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T10:30:20.000Z</t>
+        </is>
+      </c>
+      <c r="K813" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L813" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M813" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N813" s="2" t="inlineStr"/>
+      <c r="O813" s="2" t="inlineStr"/>
+      <c r="P813" s="2" t="inlineStr"/>
+      <c r="Q813" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R813" s="2" t="inlineStr"/>
+      <c r="S813" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="2" t="inlineStr">
+        <is>
+          <t>Learner Tien</t>
+        </is>
+      </c>
+      <c r="B814" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C814" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Orange Geometric Refractor #112 Learner Tien #25/25 SP</t>
+        </is>
+      </c>
+      <c r="D814" s="2" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="E814" s="2" t="inlineStr">
+        <is>
+          <t>last of 25 (25/25)</t>
+        </is>
+      </c>
+      <c r="F814" s="2" t="inlineStr">
+        <is>
+          <t>29.99 USD</t>
+        </is>
+      </c>
+      <c r="G814" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377568975833</t>
+        </is>
+      </c>
+      <c r="H814" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:36 UTC</t>
+        </is>
+      </c>
+      <c r="I814" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/eUQAAeSwoX9qzwzK/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J814" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T05:03:12.000Z</t>
+        </is>
+      </c>
+      <c r="K814" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L814" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M814" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N814" s="2" t="inlineStr"/>
+      <c r="O814" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P814" s="2" t="inlineStr"/>
+      <c r="Q814" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R814" s="2" t="inlineStr"/>
+      <c r="S814" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="2" t="inlineStr">
+        <is>
+          <t>Hubert Hurkacz</t>
+        </is>
+      </c>
+      <c r="B815" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C815" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Hubert Hurkacz #164 Frozenfractor -1/0</t>
+        </is>
+      </c>
+      <c r="D815" s="2" t="inlineStr">
+        <is>
+          <t>1/0</t>
+        </is>
+      </c>
+      <c r="E815" s="2" t="inlineStr">
+        <is>
+          <t>001 of 0</t>
+        </is>
+      </c>
+      <c r="F815" s="2" t="inlineStr">
+        <is>
+          <t>299.99 USD</t>
+        </is>
+      </c>
+      <c r="G815" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/860042875139</t>
+        </is>
+      </c>
+      <c r="H815" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:36 UTC</t>
+        </is>
+      </c>
+      <c r="I815" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jVUAAeSwH5RqzwRG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J815" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T04:29:31.000Z</t>
+        </is>
+      </c>
+      <c r="K815" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L815" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M815" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N815" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TYgAAeSwXi1qzwRG/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O815" s="2" t="inlineStr"/>
+      <c r="P815" s="2" t="inlineStr"/>
+      <c r="Q815" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R815" s="2" t="inlineStr"/>
+      <c r="S815" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="2" t="inlineStr">
+        <is>
+          <t>Renata Jamrichova</t>
+        </is>
+      </c>
+      <c r="B816" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C816" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Superfractor On Card Auto Renata Jamrichova 1/1 RC</t>
+        </is>
+      </c>
+      <c r="D816" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E816" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F816" s="2" t="inlineStr">
+        <is>
+          <t>5000.00 USD</t>
+        </is>
+      </c>
+      <c r="G816" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117465671886</t>
+        </is>
+      </c>
+      <c r="H816" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:36 UTC</t>
+        </is>
+      </c>
+      <c r="I816" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/pOYAAeSwNxRqzwMN/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J816" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T04:21:14.000Z</t>
+        </is>
+      </c>
+      <c r="K816" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L816" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M816" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N816" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/U14AAeSwuV5qzwMN/s-l1600.jpg | https://i.ebayimg.com/images/g/k94AAeSwVKFqzwMM/s-l1600.jpg | https://i.ebayimg.com/images/g/ye0AAeSwVUlqzwMN/s-l1600.jpg | https://i.ebayimg.com/images/g/RvMAAeSwKT5qzwMO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O816" s="2" t="inlineStr"/>
+      <c r="P816" s="2" t="inlineStr"/>
+      <c r="Q816" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R816" s="2" t="inlineStr"/>
+      <c r="S816" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="2" t="inlineStr">
+        <is>
+          <t>Elina Svitolina</t>
+        </is>
+      </c>
+      <c r="B817" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Chrome</t>
+        </is>
+      </c>
+      <c r="C817" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Elina Svitolina True Black Refractor Auto 10/10 PSA 8</t>
+        </is>
+      </c>
+      <c r="D817" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E817" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F817" s="2" t="inlineStr">
+        <is>
+          <t>199.99 USD</t>
+        </is>
+      </c>
+      <c r="G817" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/840019803668</t>
+        </is>
+      </c>
+      <c r="H817" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:36 UTC</t>
+        </is>
+      </c>
+      <c r="I817" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~WUAAeSwqIBqzv4Y/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J817" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T04:00:45.000Z</t>
+        </is>
+      </c>
+      <c r="K817" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L817" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M817" s="2" t="inlineStr">
+        <is>
+          <t>PSA 8</t>
+        </is>
+      </c>
+      <c r="N817" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Z~gAAeSwCbtqzv4Y/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O817" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P817" s="2" t="inlineStr"/>
+      <c r="Q817" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R817" s="2" t="inlineStr"/>
+      <c r="S817" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" s="2" t="inlineStr">
+        <is>
+          <t>Elina Svitolina</t>
+        </is>
+      </c>
+      <c r="B818" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Chrome</t>
+        </is>
+      </c>
+      <c r="C818" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Elina Svitolina Gold Refractor Auto 50/50 PSA 8</t>
+        </is>
+      </c>
+      <c r="D818" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E818" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F818" s="2" t="inlineStr">
+        <is>
+          <t>79.99 USD</t>
+        </is>
+      </c>
+      <c r="G818" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/840019796036</t>
+        </is>
+      </c>
+      <c r="H818" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:36 UTC</t>
+        </is>
+      </c>
+      <c r="I818" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~n8AAeSwi2pqzvyq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J818" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T03:55:52.000Z</t>
+        </is>
+      </c>
+      <c r="K818" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L818" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M818" s="2" t="inlineStr">
+        <is>
+          <t>PSA 8</t>
+        </is>
+      </c>
+      <c r="N818" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/fp8AAeSwNLtqzvyq/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O818" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P818" s="2" t="inlineStr"/>
+      <c r="Q818" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R818" s="2" t="inlineStr"/>
+      <c r="S818" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="2" t="inlineStr">
+        <is>
+          <t>Jasmine Paolini</t>
+        </is>
+      </c>
+      <c r="B819" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C819" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Jasmine Paolini #AA-JA Aces Auto Black 10/10≈1/1</t>
+        </is>
+      </c>
+      <c r="D819" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E819" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F819" s="2" t="inlineStr">
+        <is>
+          <t>1.25 USD</t>
+        </is>
+      </c>
+      <c r="G819" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/366732698472</t>
+        </is>
+      </c>
+      <c r="H819" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:36 UTC</t>
+        </is>
+      </c>
+      <c r="I819" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/pScAAeSwNgZqzvDk/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J819" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T03:01:57.000Z</t>
+        </is>
+      </c>
+      <c r="K819" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L819" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M819" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N819" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/r38AAeSwxc5qzvDl/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O819" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P819" s="2" t="inlineStr"/>
+      <c r="Q819" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R819" s="2" t="inlineStr"/>
+      <c r="S819" s="2" t="inlineStr">
+        <is>
+          <t>Tennis (网球)</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="2" t="inlineStr">
+        <is>
+          <t>Camila Osorio</t>
+        </is>
+      </c>
+      <c r="B820" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C820" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Camila Osorio Black 10/10</t>
+        </is>
+      </c>
+      <c r="D820" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E820" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F820" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G820" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257796954222</t>
+        </is>
+      </c>
+      <c r="H820" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:36 UTC</t>
+        </is>
+      </c>
+      <c r="I820" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/cYIAAeSwrRRqwCia/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J820" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:40:00.000Z</t>
+        </is>
+      </c>
+      <c r="K820" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L820" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M820" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N820" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QdEAAeSwRWxqwCiZ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O820" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P820" s="2" t="inlineStr"/>
+      <c r="Q820" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R820" s="2" t="inlineStr"/>
+      <c r="S820" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="2" t="inlineStr">
+        <is>
+          <t>Martin Landaluce</t>
+        </is>
+      </c>
+      <c r="B821" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Chrome</t>
+        </is>
+      </c>
+      <c r="C821" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Martin Landaluce Auto Blue Refractor #150/150 J46</t>
+        </is>
+      </c>
+      <c r="D821" s="2" t="inlineStr">
+        <is>
+          <t>150/150</t>
+        </is>
+      </c>
+      <c r="E821" s="2" t="inlineStr">
+        <is>
+          <t>last of 150 (150/150)</t>
+        </is>
+      </c>
+      <c r="F821" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G821" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/800792646176</t>
+        </is>
+      </c>
+      <c r="H821" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:36 UTC</t>
+        </is>
+      </c>
+      <c r="I821" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YS0AAeSwq6Zqzsyr/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J821" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:35:00.000Z</t>
+        </is>
+      </c>
+      <c r="K821" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L821" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M821" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N821" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/O-EAAeSw1Oxqzsyr/s-l1600.jpg | https://i.ebayimg.com/images/g/~NUAAeSwrQBqzsyr/s-l1600.jpg | https://i.ebayimg.com/images/g/~gwAAeSwe2Bqzsyr/s-l1600.jpg | https://i.ebayimg.com/images/g/-nAAAeSwlMpqzsyr/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O821" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P821" s="2" t="inlineStr"/>
+      <c r="Q821" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R821" s="2" t="inlineStr"/>
+      <c r="S821" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="2" t="inlineStr">
+        <is>
+          <t>Marina Stakusic</t>
+        </is>
+      </c>
+      <c r="B822" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C822" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Marina Stakusic Gold Geometric Refractor 50/50 1/1 SP</t>
+        </is>
+      </c>
+      <c r="D822" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E822" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F822" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G822" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/960062709906</t>
+        </is>
+      </c>
+      <c r="H822" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:36 UTC</t>
+        </is>
+      </c>
+      <c r="I822" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/zDIAAeSwTlxqzmMz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J822" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:28:01.000Z</t>
+        </is>
+      </c>
+      <c r="K822" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L822" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M822" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N822" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/J3oAAeSwElRqzmMx/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O822" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P822" s="2" t="inlineStr"/>
+      <c r="Q822" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R822" s="2" t="inlineStr"/>
+      <c r="S822" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="2" t="inlineStr">
+        <is>
+          <t>Billie Jean King</t>
+        </is>
+      </c>
+      <c r="B823" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C823" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Billie Jean King 001/150 Blue Geo Auto</t>
+        </is>
+      </c>
+      <c r="D823" s="2" t="inlineStr">
+        <is>
+          <t>1/150</t>
+        </is>
+      </c>
+      <c r="E823" s="2" t="inlineStr">
+        <is>
+          <t>001 of 150</t>
+        </is>
+      </c>
+      <c r="F823" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G823" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/257796954218</t>
+        </is>
+      </c>
+      <c r="H823" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:36 UTC</t>
+        </is>
+      </c>
+      <c r="I823" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7rUAAeSwpEBqwCuL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J823" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:23:00.000Z</t>
+        </is>
+      </c>
+      <c r="K823" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L823" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M823" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N823" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nxsAAeSwG~dqwCuL/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O823" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P823" s="2" t="inlineStr"/>
+      <c r="Q823" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R823" s="2" t="inlineStr"/>
+      <c r="S823" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="2" t="inlineStr">
+        <is>
+          <t>Arthur Fils Destiny</t>
+        </is>
+      </c>
+      <c r="B824" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C824" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Arthur Fils Destiny Gold Refractor 50/50 1/1 SP</t>
+        </is>
+      </c>
+      <c r="D824" s="2" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="E824" s="2" t="inlineStr">
+        <is>
+          <t>last of 50 (50/50)</t>
+        </is>
+      </c>
+      <c r="F824" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G824" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/960062578877</t>
+        </is>
+      </c>
+      <c r="H824" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:36 UTC</t>
+        </is>
+      </c>
+      <c r="I824" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/dq0AAeSwo-Rqzlgj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J824" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:00:01.000Z</t>
+        </is>
+      </c>
+      <c r="K824" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L824" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M824" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N824" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/v-EAAeSw0lhqzlgj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O824" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P824" s="2" t="inlineStr"/>
+      <c r="Q824" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R824" s="2" t="inlineStr"/>
+      <c r="S824" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" s="2" t="inlineStr">
+        <is>
+          <t>Petra Marcinko</t>
+        </is>
+      </c>
+      <c r="B825" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Graphite</t>
+        </is>
+      </c>
+      <c r="C825" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Tennis Petra Marcinko Rookie Auto Green Refractor #75/75 J61</t>
+        </is>
+      </c>
+      <c r="D825" s="2" t="inlineStr">
+        <is>
+          <t>75/75</t>
+        </is>
+      </c>
+      <c r="E825" s="2" t="inlineStr">
+        <is>
+          <t>last of 75 (75/75)</t>
+        </is>
+      </c>
+      <c r="F825" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G825" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/800792646156</t>
+        </is>
+      </c>
+      <c r="H825" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:36 UTC</t>
+        </is>
+      </c>
+      <c r="I825" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/BmsAAeSwHwBqzsys/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J825" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:16:00.000Z</t>
+        </is>
+      </c>
+      <c r="K825" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L825" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M825" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N825" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/MYYAAeSwonJqzsys/s-l1600.jpg | https://i.ebayimg.com/images/g/k1MAAeSwyz5qzsys/s-l1600.jpg | https://i.ebayimg.com/images/g/AaYAAeSwXi1qzsys/s-l1600.jpg | https://i.ebayimg.com/images/g/7aYAAeSwL~xqzsys/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O825" s="2" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="P825" s="2" t="inlineStr"/>
+      <c r="Q825" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R825" s="2" t="inlineStr"/>
+      <c r="S825" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" s="2" t="inlineStr">
+        <is>
+          <t>Victoria Mboko</t>
+        </is>
+      </c>
+      <c r="B826" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Graphite</t>
+        </is>
+      </c>
+      <c r="C826" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Tennis #79 Victoria Mboko White Refractor #01/10 J53</t>
+        </is>
+      </c>
+      <c r="D826" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E826" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F826" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G826" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/800792646154</t>
+        </is>
+      </c>
+      <c r="H826" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:36 UTC</t>
+        </is>
+      </c>
+      <c r="I826" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Vq4AAeSwUR1qzsy2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J826" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:14:00.000Z</t>
+        </is>
+      </c>
+      <c r="K826" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L826" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M826" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N826" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/vV8AAeSwhLpqzsy2/s-l1600.jpg | https://i.ebayimg.com/images/g/Ou8AAeSwXKFqzsy2/s-l1600.jpg | https://i.ebayimg.com/images/g/HaYAAeSwwQtqzsy2/s-l1600.jpg | https://i.ebayimg.com/images/g/tlgAAeSwyKxqzsy2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O826" s="2" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="P826" s="2" t="inlineStr"/>
+      <c r="Q826" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R826" s="2" t="inlineStr"/>
+      <c r="S826" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="2" t="inlineStr">
+        <is>
+          <t>Aryna Sabalenka</t>
+        </is>
+      </c>
+      <c r="B827" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps</t>
+        </is>
+      </c>
+      <c r="C827" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite Aryna Sabalenka Rally Relic Pink Bookend 1/1 🔥 # 15/15 SSP</t>
+        </is>
+      </c>
+      <c r="D827" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E827" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F827" s="2" t="inlineStr">
+        <is>
+          <t>115.00 USD</t>
+        </is>
+      </c>
+      <c r="G827" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/336843515930</t>
+        </is>
+      </c>
+      <c r="H827" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:36 UTC</t>
+        </is>
+      </c>
+      <c r="I827" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3PAAAeSwNINqJ13N/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J827" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:02:52.000Z</t>
+        </is>
+      </c>
+      <c r="K827" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L827" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M827" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N827" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/yUAAAeSwFkhqJ13O/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O827" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P827" s="2" t="inlineStr"/>
+      <c r="Q827" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R827" s="2" t="inlineStr"/>
+      <c r="S827" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="2" t="inlineStr">
+        <is>
+          <t>Novak Djokovic</t>
+        </is>
+      </c>
+      <c r="B828" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C828" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2026 Graphite Novak Djokovic Break Point Red Refractor 1/1 PSA 8</t>
+        </is>
+      </c>
+      <c r="D828" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E828" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F828" s="2" t="inlineStr">
+        <is>
+          <t>38000.00 USD</t>
+        </is>
+      </c>
+      <c r="G828" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/237122728808</t>
+        </is>
+      </c>
+      <c r="H828" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:36 UTC</t>
+        </is>
+      </c>
+      <c r="I828" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/h7MAAeSwhFtqzqkm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J828" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T21:57:37.000Z</t>
+        </is>
+      </c>
+      <c r="K828" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L828" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M828" s="2" t="inlineStr">
+        <is>
+          <t>PSA 8</t>
+        </is>
+      </c>
+      <c r="N828" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/UkAAAeSwM05qzqj6/s-l1600.jpg | https://i.ebayimg.com/images/g/v4cAAeSwN9Nqzqj6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O828" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P828" s="2" t="inlineStr"/>
+      <c r="Q828" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R828" s="2" t="inlineStr"/>
+      <c r="S828" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="2" t="inlineStr">
+        <is>
+          <t>Yuliia Starodubtseva</t>
+        </is>
+      </c>
+      <c r="B829" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C829" s="2" t="inlineStr">
+        <is>
+          <t>Topps 2026 Graphite Yuliia Starodubtseva RC 1/1 #107 WTA Tennis Red Crystalline</t>
+        </is>
+      </c>
+      <c r="D829" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E829" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F829" s="2" t="inlineStr">
+        <is>
+          <t>400.00 USD</t>
+        </is>
+      </c>
+      <c r="G829" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287646047840</t>
+        </is>
+      </c>
+      <c r="H829" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:36 UTC</t>
+        </is>
+      </c>
+      <c r="I829" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/lWUAAeSwbNpqznNj/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J829" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T18:09:18.000Z</t>
+        </is>
+      </c>
+      <c r="K829" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L829" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M829" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N829" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/GtUAAeSwTVlqznNT/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O829" s="2" t="inlineStr"/>
+      <c r="P829" s="2" t="inlineStr"/>
+      <c r="Q829" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R829" s="2" t="inlineStr"/>
+      <c r="S829" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="2" t="inlineStr">
+        <is>
+          <t>Ben Shelton</t>
+        </is>
+      </c>
+      <c r="B830" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C830" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Now Ben Shelton #21 Black Foil 01/10 Tennis US Open</t>
+        </is>
+      </c>
+      <c r="D830" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E830" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F830" s="2" t="inlineStr">
+        <is>
+          <t>499.00 USD</t>
+        </is>
+      </c>
+      <c r="G830" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/860042531509</t>
+        </is>
+      </c>
+      <c r="H830" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:37 UTC</t>
+        </is>
+      </c>
+      <c r="I830" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3W4AAeSwCbtqzuFg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J830" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T02:13:26.000Z</t>
+        </is>
+      </c>
+      <c r="K830" s="2" t="inlineStr">
+        <is>
+          <t>Auction + Buy It Now</t>
+        </is>
+      </c>
+      <c r="L830" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M830" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N830" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/c4IAAeSweptqzuFg/s-l1600.jpg | https://i.ebayimg.com/images/g/b70AAeSwXgRqzuVZ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O830" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P830" s="2" t="inlineStr"/>
+      <c r="Q830" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R830" s="2" t="inlineStr"/>
+      <c r="S830" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="2" t="inlineStr">
+        <is>
+          <t>Tracy Austin</t>
+        </is>
+      </c>
+      <c r="B831" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic / 2008 Ace Authentic Grand Slam II</t>
+        </is>
+      </c>
+      <c r="C831" s="2" t="inlineStr">
+        <is>
+          <t>2008 Ace Grand Slam II Stars/Legends Jersey Gold 1/24 #JC19 Tracy Austin PSA 4</t>
+        </is>
+      </c>
+      <c r="D831" s="2" t="inlineStr">
+        <is>
+          <t>1/24</t>
+        </is>
+      </c>
+      <c r="E831" s="2" t="inlineStr">
+        <is>
+          <t>001 of 24</t>
+        </is>
+      </c>
+      <c r="F831" s="2" t="inlineStr">
+        <is>
+          <t>50.00 USD</t>
+        </is>
+      </c>
+      <c r="G831" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168790996510</t>
+        </is>
+      </c>
+      <c r="H831" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:37 UTC</t>
+        </is>
+      </c>
+      <c r="I831" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/1F4AAOSwq2hm7HWW/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J831" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T01:15:45.000Z</t>
+        </is>
+      </c>
+      <c r="K831" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L831" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M831" s="2" t="inlineStr">
+        <is>
+          <t>PSA 4</t>
+        </is>
+      </c>
+      <c r="N831" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~xIAAOSwyWFm7HWh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O831" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P831" s="2" t="inlineStr"/>
+      <c r="Q831" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R831" s="2" t="inlineStr">
+        <is>
+          <t>Ace Authentic: check the numbering is stamped, not on a circle sticker</t>
+        </is>
+      </c>
+      <c r="S831" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="2" t="inlineStr">
+        <is>
+          <t>Steffi Graf</t>
+        </is>
+      </c>
+      <c r="B832" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C832" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Aces Autographs Steffi Graf Superfractor Auto 1/1 PSA AUTH</t>
+        </is>
+      </c>
+      <c r="D832" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E832" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F832" s="2" t="inlineStr">
+        <is>
+          <t>15000.00 USD</t>
+        </is>
+      </c>
+      <c r="G832" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407288527461</t>
+        </is>
+      </c>
+      <c r="H832" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:37 UTC</t>
+        </is>
+      </c>
+      <c r="I832" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/StEAAeSwVl9qztCC/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J832" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T00:53:15.000Z</t>
+        </is>
+      </c>
+      <c r="K832" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L832" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M832" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) Authentic</t>
+        </is>
+      </c>
+      <c r="N832" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2yAAAeSwBx5qztCD/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O832" s="2" t="inlineStr"/>
+      <c r="P832" s="2" t="inlineStr"/>
+      <c r="Q832" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R832" s="2" t="inlineStr"/>
+      <c r="S832" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -72327,6 +74083,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G810" r:id="rId809"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G811" r:id="rId810"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G812" r:id="rId811"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G813" r:id="rId812"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G814" r:id="rId813"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G815" r:id="rId814"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G816" r:id="rId815"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G817" r:id="rId816"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G818" r:id="rId817"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G819" r:id="rId818"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G820" r:id="rId819"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G821" r:id="rId820"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G822" r:id="rId821"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G823" r:id="rId822"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G824" r:id="rId823"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G825" r:id="rId824"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G826" r:id="rId825"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G827" r:id="rId826"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G828" r:id="rId827"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G829" r:id="rId828"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G830" r:id="rId829"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G831" r:id="rId830"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G832" r:id="rId831"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-15 00:28 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S832"/>
+  <dimension ref="A1:S842"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -73265,6 +73265,892 @@
       </c>
       <c r="R832" s="2" t="inlineStr"/>
       <c r="S832" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B833" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C833" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz 2026 Topps Chrome World Number 1 ORANGE Geometric Refractor 1/25</t>
+        </is>
+      </c>
+      <c r="D833" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E833" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F833" s="2" t="inlineStr">
+        <is>
+          <t>419.99 USD</t>
+        </is>
+      </c>
+      <c r="G833" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307229704184</t>
+        </is>
+      </c>
+      <c r="H833" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:27 UTC</t>
+        </is>
+      </c>
+      <c r="I833" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/8nkAAeSwrQBqzo0O/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J833" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T20:00:49.000Z</t>
+        </is>
+      </c>
+      <c r="K833" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L833" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M833" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N833" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ZHYAAeSwId9qzo0O/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O833" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P833" s="2" t="inlineStr"/>
+      <c r="Q833" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R833" s="2" t="inlineStr"/>
+      <c r="S833" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Alcaraz</t>
+        </is>
+      </c>
+      <c r="B834" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C834" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Carlos Alcaraz Destiny #DTY-ALC Red Geometric 1/5</t>
+        </is>
+      </c>
+      <c r="D834" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E834" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F834" s="2" t="inlineStr">
+        <is>
+          <t>224.50 USD</t>
+        </is>
+      </c>
+      <c r="G834" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/860042344491</t>
+        </is>
+      </c>
+      <c r="H834" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:27 UTC</t>
+        </is>
+      </c>
+      <c r="I834" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XwYAAeSwCYJqx-UH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J834" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T00:59:49.000Z</t>
+        </is>
+      </c>
+      <c r="K834" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L834" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M834" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N834" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Y-IAAeSwqdFqx-UH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O834" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P834" s="2" t="inlineStr"/>
+      <c r="Q834" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R834" s="2" t="inlineStr"/>
+      <c r="S834" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Nadal</t>
+        </is>
+      </c>
+      <c r="B835" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 TOPPS CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="C835" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS BLACK GEOMETRIC #281 RAFAEL NADAL 2/2 PSA 7</t>
+        </is>
+      </c>
+      <c r="D835" s="2" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="E835" s="2" t="inlineStr">
+        <is>
+          <t>last of 2 (2/2)</t>
+        </is>
+      </c>
+      <c r="F835" s="2" t="inlineStr">
+        <is>
+          <t>25000.00 USD</t>
+        </is>
+      </c>
+      <c r="G835" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117466925833</t>
+        </is>
+      </c>
+      <c r="H835" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:27 UTC</t>
+        </is>
+      </c>
+      <c r="I835" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/qTwAAeSwn6Nq0A5v/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J835" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T23:20:15.000Z</t>
+        </is>
+      </c>
+      <c r="K835" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L835" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M835" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 7</t>
+        </is>
+      </c>
+      <c r="N835" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/rZ4AAeSw1HVq0A5v/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O835" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P835" s="2" t="inlineStr"/>
+      <c r="Q835" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R835" s="2" t="inlineStr"/>
+      <c r="S835" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="2" t="inlineStr">
+        <is>
+          <t>Alexandra Eala</t>
+        </is>
+      </c>
+      <c r="B836" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C836" s="2" t="inlineStr">
+        <is>
+          <t>Alexandra Eala 2026 Topps Chrome Tennis Gold Geo Refractor Auto 1/50 1st #AT-AEA</t>
+        </is>
+      </c>
+      <c r="D836" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E836" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F836" s="2" t="inlineStr">
+        <is>
+          <t>999.00 USD</t>
+        </is>
+      </c>
+      <c r="G836" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/800792597853</t>
+        </is>
+      </c>
+      <c r="H836" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:28 UTC</t>
+        </is>
+      </c>
+      <c r="I836" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/tT4AAeSw7ytqzsc3/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J836" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T00:05:58.000Z</t>
+        </is>
+      </c>
+      <c r="K836" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L836" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M836" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N836" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/FJwAAeSwUJVqzsc-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O836" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P836" s="2" t="inlineStr"/>
+      <c r="Q836" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R836" s="2" t="inlineStr"/>
+      <c r="S836" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="2" t="inlineStr">
+        <is>
+          <t>Alexandra Eala</t>
+        </is>
+      </c>
+      <c r="B837" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C837" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS CHROME  TENNIS-----ALEXANDRA EALA---ROOKIE---BLACK---AUTO---01/10</t>
+        </is>
+      </c>
+      <c r="D837" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E837" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F837" s="2" t="inlineStr">
+        <is>
+          <t>24999.99 USD</t>
+        </is>
+      </c>
+      <c r="G837" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287503405293?amdata=enc%3AAQALAAAAsCHNgUiiE%2FjQhlDTaMiAde%2B1bPxxww--OJ0cuEUg8sUtohRMZun8mx9vmtKol3LIPdgo1Ap%2BrfGMro%2B7JHD4K1rgxdSx0VlHdhBwLW4p0uesJX1ckQlxHW%2BPX3qBeVers%2BVXTvTdUjDeRaJ1EKQcrR5nEkqZNrsjTJ%2BIlP5LJSjuczy96z5ZH9JLQM594CXa31GkIVE8gMFdMxk3IwtU5ywcQrx0NjgkZpIZTExOfkdU</t>
+        </is>
+      </c>
+      <c r="H837" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:28 UTC</t>
+        </is>
+      </c>
+      <c r="I837" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/eBoAAeSwstBqciXh/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J837" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04T17:50:02.000Z</t>
+        </is>
+      </c>
+      <c r="K837" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L837" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M837" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA)</t>
+        </is>
+      </c>
+      <c r="N837" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/kcIAAeSwD-lqciXt/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O837" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P837" s="2" t="inlineStr"/>
+      <c r="Q837" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R837" s="2" t="inlineStr"/>
+      <c r="S837" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="2" t="inlineStr">
+        <is>
+          <t>Eala</t>
+        </is>
+      </c>
+      <c r="B838" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C838" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS-ALEXANDRA EALA--RED REFRACTOR--BOOKEND AUTO--5/5--PSA 9</t>
+        </is>
+      </c>
+      <c r="D838" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E838" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F838" s="2" t="inlineStr">
+        <is>
+          <t>14999.00 USD</t>
+        </is>
+      </c>
+      <c r="G838" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/287454268896?amdata=enc%3AAQALAAAAsCHNgUiiE%2FjQhlDTaMiAde8IrwkQy%2Beh6PlhTmYJ%2FDywbF9DY8Ke5jhlJL2nOLLLttTPHnmJJFg6oCnC5j8Xu6hwGzcxA2ZkB0KLkcmLT8g%2BYjA44%2B%2F%2Bo2z85ZYjJx3M%2BaDVsm1as66eYrILOJyrhHNAzN3v%2BFOJBEeLfFKYOvbs8x0D3gcz7kb%2FAt7YUVRDIXJ2CNUDIJE8QqpzMCsTpyShmO%2FfbVgDcN7pDy5abHTj</t>
+        </is>
+      </c>
+      <c r="H838" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:28 UTC</t>
+        </is>
+      </c>
+      <c r="I838" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/yGAAAeSwDB5qUjQu/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J838" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11T12:20:26.000Z</t>
+        </is>
+      </c>
+      <c r="K838" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L838" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M838" s="2" t="inlineStr">
+        <is>
+          <t>PSA 9</t>
+        </is>
+      </c>
+      <c r="N838" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/g1AAAeSwvqJqUjQ6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O838" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P838" s="2" t="inlineStr"/>
+      <c r="Q838" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R838" s="2" t="inlineStr"/>
+      <c r="S838" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="2" t="inlineStr">
+        <is>
+          <t>Alexandra Eala</t>
+        </is>
+      </c>
+      <c r="B839" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C839" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Sapphire Edition #171 Alexandra Eala Red 1/5 ≈1/1</t>
+        </is>
+      </c>
+      <c r="D839" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E839" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F839" s="2" t="inlineStr">
+        <is>
+          <t>2000.00 USD</t>
+        </is>
+      </c>
+      <c r="G839" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/188250044345</t>
+        </is>
+      </c>
+      <c r="H839" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:28 UTC</t>
+        </is>
+      </c>
+      <c r="I839" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/DK4AAeSw6o1p05y0/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J839" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06T11:45:53.000Z</t>
+        </is>
+      </c>
+      <c r="K839" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L839" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M839" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N839" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/IJUAAeSwQONp05y0/s-l1600.jpg | https://i.ebayimg.com/images/g/sCgAAeSwh-Bp05yz/s-l1600.jpg | https://i.ebayimg.com/images/g/vy0AAeSwtrFp05yz/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O839" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P839" s="2" t="inlineStr"/>
+      <c r="Q839" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R839" s="2" t="inlineStr"/>
+      <c r="S839" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="2" t="inlineStr">
+        <is>
+          <t>Alexandra Eala</t>
+        </is>
+      </c>
+      <c r="B840" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Graphite</t>
+        </is>
+      </c>
+      <c r="C840" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Graphite - Tour Relic Autographs  Alexandra Eala - Numbered 10/10</t>
+        </is>
+      </c>
+      <c r="D840" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E840" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F840" s="2" t="inlineStr">
+        <is>
+          <t>3900.00 USD</t>
+        </is>
+      </c>
+      <c r="G840" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/800463243501</t>
+        </is>
+      </c>
+      <c r="H840" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:28 UTC</t>
+        </is>
+      </c>
+      <c r="I840" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/YP4AAeSwEbBqcp5a/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J840" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05T02:22:33.000Z</t>
+        </is>
+      </c>
+      <c r="K840" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L840" s="2" t="inlineStr">
+        <is>
+          <t>Patch auto</t>
+        </is>
+      </c>
+      <c r="M840" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N840" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/QLwAAeSwlcJqcp5a/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O840" s="2" t="inlineStr"/>
+      <c r="P840" s="2" t="inlineStr"/>
+      <c r="Q840" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R840" s="2" t="inlineStr"/>
+      <c r="S840" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" s="2" t="inlineStr">
+        <is>
+          <t>Joao Fonseca</t>
+        </is>
+      </c>
+      <c r="B841" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C841" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis RC Joao Fonseca Youthquake Blue Refractor 150/150</t>
+        </is>
+      </c>
+      <c r="D841" s="2" t="inlineStr">
+        <is>
+          <t>150/150</t>
+        </is>
+      </c>
+      <c r="E841" s="2" t="inlineStr">
+        <is>
+          <t>last of 150 (150/150)</t>
+        </is>
+      </c>
+      <c r="F841" s="2" t="inlineStr">
+        <is>
+          <t>120.00 USD</t>
+        </is>
+      </c>
+      <c r="G841" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/840019297594?amdata=enc%3AAQALAAAAoCHNgUiiE%2FjQhlDTaMiAde8mpyuo6ci%2Bk1Rc5UXU2%2B2UttbvSIXeoOYh0P%2FMaWnlK8L%2FP8lXRTiY6rIy5a2yRKzg%2FCdhW9yZW90f09bNqCOgjODvqxyoK1TQvMeM4Pa1Itke0Yy4V9XUX1AEa04%2BaCdjPphe8pVlqOBaE814Ta2fPO%2B1fAlJOYBiWY3RXH1Aeo6gKqKcZsHJU1VSZv7ALqo%3D</t>
+        </is>
+      </c>
+      <c r="H841" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:28 UTC</t>
+        </is>
+      </c>
+      <c r="I841" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ReUAAeSw-v1qzsh5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J841" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T00:11:48.000Z</t>
+        </is>
+      </c>
+      <c r="K841" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L841" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M841" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N841" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/oQoAAeSw0aZqzsiD/s-l1600.jpg | https://i.ebayimg.com/images/g/FLEAAeSwdOxqzsiJ/s-l1600.jpg | https://i.ebayimg.com/images/g/c0cAAeSwDS9qzsiP/s-l1600.jpg | https://i.ebayimg.com/images/g/owAAAeSwopdqzsg7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O841" s="2" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="P841" s="2" t="inlineStr"/>
+      <c r="Q841" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R841" s="2" t="inlineStr"/>
+      <c r="S841" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="2" t="inlineStr">
+        <is>
+          <t>Joao Fonseca</t>
+        </is>
+      </c>
+      <c r="B842" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C842" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Joao Fonseca #AO-JFA RC Rookie Auto Red Refractor 5/5</t>
+        </is>
+      </c>
+      <c r="D842" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E842" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F842" s="2" t="inlineStr">
+        <is>
+          <t>30000.00 USD</t>
+        </is>
+      </c>
+      <c r="G842" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298735724497</t>
+        </is>
+      </c>
+      <c r="H842" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 00:28 UTC</t>
+        </is>
+      </c>
+      <c r="I842" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/nbYAAeSw6clqxBvO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J842" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T21:52:12.000Z</t>
+        </is>
+      </c>
+      <c r="K842" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L842" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M842" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N842" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/bEgAAeSwzWBqxBvN/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O842" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P842" s="2" t="inlineStr"/>
+      <c r="Q842" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R842" s="2" t="inlineStr"/>
+      <c r="S842" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -74103,6 +74989,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G830" r:id="rId829"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G831" r:id="rId830"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G832" r:id="rId831"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G833" r:id="rId832"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G834" r:id="rId833"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G835" r:id="rId834"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G836" r:id="rId835"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G837" r:id="rId836"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G838" r:id="rId837"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G839" r:id="rId838"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G840" r:id="rId839"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G841" r:id="rId840"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G842" r:id="rId841"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scan results, 2026-10-15 01:45 UTC
</commit_message>
<xml_diff>
--- a/results/tennis_cards_verified.xlsx
+++ b/results/tennis_cards_verified.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S842"/>
+  <dimension ref="A1:S869"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -74151,6 +74151,2357 @@
       </c>
       <c r="R842" s="2" t="inlineStr"/>
       <c r="S842" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" s="2" t="inlineStr">
+        <is>
+          <t>Andrey Rublev</t>
+        </is>
+      </c>
+      <c r="B843" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 TOPPS CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="C843" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS SUPERFRACTOR 1/1 #7 ANDREY RUBLEV 1/1 PSA 8</t>
+        </is>
+      </c>
+      <c r="D843" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E843" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F843" s="2" t="inlineStr">
+        <is>
+          <t>5555.55 USD</t>
+        </is>
+      </c>
+      <c r="G843" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/900014157563</t>
+        </is>
+      </c>
+      <c r="H843" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I843" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0IYAAeSwTnhq0C9B/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J843" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T01:40:17.000Z</t>
+        </is>
+      </c>
+      <c r="K843" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L843" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M843" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 8</t>
+        </is>
+      </c>
+      <c r="N843" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ywgAAeSwvRdq0C9B/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O843" s="2" t="inlineStr"/>
+      <c r="P843" s="2" t="inlineStr"/>
+      <c r="Q843" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R843" s="2" t="inlineStr"/>
+      <c r="S843" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" s="2" t="inlineStr">
+        <is>
+          <t>Mariano Navone</t>
+        </is>
+      </c>
+      <c r="B844" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 TOPPS CHROME TENNIS CHROME AUTOGRAPHS</t>
+        </is>
+      </c>
+      <c r="C844" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS CHROME AUTOS SUPERFRACTOR 1/1 MARIANO NAVONE 1/1 PSA 8</t>
+        </is>
+      </c>
+      <c r="D844" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E844" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F844" s="2" t="inlineStr">
+        <is>
+          <t>2222.22 USD</t>
+        </is>
+      </c>
+      <c r="G844" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117467029061</t>
+        </is>
+      </c>
+      <c r="H844" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I844" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/224AAeSw86tq0C8R/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J844" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T01:39:30.000Z</t>
+        </is>
+      </c>
+      <c r="K844" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L844" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M844" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 8</t>
+        </is>
+      </c>
+      <c r="N844" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/0kwAAeSwjeRq0C8R/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O844" s="2" t="inlineStr"/>
+      <c r="P844" s="2" t="inlineStr"/>
+      <c r="Q844" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R844" s="2" t="inlineStr"/>
+      <c r="S844" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" s="2" t="inlineStr">
+        <is>
+          <t>Madison Keys</t>
+        </is>
+      </c>
+      <c r="B845" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 TOPPS CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="C845" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS SUPERFRACTOR 1/1 #33 MADISON KEYS 1/1 PSA 6</t>
+        </is>
+      </c>
+      <c r="D845" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E845" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F845" s="2" t="inlineStr">
+        <is>
+          <t>2222.22 USD</t>
+        </is>
+      </c>
+      <c r="G845" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307231852426</t>
+        </is>
+      </c>
+      <c r="H845" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I845" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/398AAeSw9Hhq0C77/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J845" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T01:39:08.000Z</t>
+        </is>
+      </c>
+      <c r="K845" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L845" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M845" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 6</t>
+        </is>
+      </c>
+      <c r="N845" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/2ggAAeSwT6Bq0C77/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O845" s="2" t="inlineStr"/>
+      <c r="P845" s="2" t="inlineStr"/>
+      <c r="Q845" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R845" s="2" t="inlineStr"/>
+      <c r="S845" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="2" t="inlineStr">
+        <is>
+          <t>Marta Kostyuk</t>
+        </is>
+      </c>
+      <c r="B846" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C846" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis - SUPERFRACTOR 1/1 #46 Marta Kostyuk 1 of 1 SUPER</t>
+        </is>
+      </c>
+      <c r="D846" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E846" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F846" s="2" t="inlineStr">
+        <is>
+          <t>999.95 USD</t>
+        </is>
+      </c>
+      <c r="G846" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/117467023579</t>
+        </is>
+      </c>
+      <c r="H846" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I846" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/xC4AAeSw8thq0CzR/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J846" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T01:31:22.000Z</t>
+        </is>
+      </c>
+      <c r="K846" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L846" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M846" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N846" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/yWcAAeSwz8lq0CzS/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O846" s="2" t="inlineStr"/>
+      <c r="P846" s="2" t="inlineStr"/>
+      <c r="Q846" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R846" s="2" t="inlineStr"/>
+      <c r="S846" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" s="2" t="inlineStr">
+        <is>
+          <t>John McEnroe</t>
+        </is>
+      </c>
+      <c r="B847" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis Tennis</t>
+        </is>
+      </c>
+      <c r="C847" s="2" t="inlineStr">
+        <is>
+          <t>JOHN MCENROE 2026 TOPPS CHROME GOLD GEOMETRIC REFRACTOR AUTO 01/50 #AO-JME Q7656</t>
+        </is>
+      </c>
+      <c r="D847" s="2" t="inlineStr">
+        <is>
+          <t>1/50</t>
+        </is>
+      </c>
+      <c r="E847" s="2" t="inlineStr">
+        <is>
+          <t>001 of 50</t>
+        </is>
+      </c>
+      <c r="F847" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G847" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/940014620983</t>
+        </is>
+      </c>
+      <c r="H847" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I847" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/aLYAAeSwssFq0CN8/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J847" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T01:29:00.000Z</t>
+        </is>
+      </c>
+      <c r="K847" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L847" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M847" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N847" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/XtIAAeSwLBlq0CN8/s-l1600.jpg | https://i.ebayimg.com/images/g/bSEAAeSwVaNq0CN7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O847" s="2" t="inlineStr">
+        <is>
+          <t>gold</t>
+        </is>
+      </c>
+      <c r="P847" s="2" t="inlineStr"/>
+      <c r="Q847" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R847" s="2" t="inlineStr"/>
+      <c r="S847" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="2" t="inlineStr">
+        <is>
+          <t>Iva Jovic</t>
+        </is>
+      </c>
+      <c r="B848" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 TOPPS CHROME TENNIS CHROME AUTOGRAPHS</t>
+        </is>
+      </c>
+      <c r="C848" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS CHROME AUTOS #CA-IJC IVA JOVIC 2/2 PSA 7 AUTO 10</t>
+        </is>
+      </c>
+      <c r="D848" s="2" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="E848" s="2" t="inlineStr">
+        <is>
+          <t>last of 2 (2/2)</t>
+        </is>
+      </c>
+      <c r="F848" s="2" t="inlineStr">
+        <is>
+          <t>5555.55 USD</t>
+        </is>
+      </c>
+      <c r="G848" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/900014139094</t>
+        </is>
+      </c>
+      <c r="H848" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I848" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ulUAAeSwGRZq0CrJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J848" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T01:21:12.000Z</t>
+        </is>
+      </c>
+      <c r="K848" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L848" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M848" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 7</t>
+        </is>
+      </c>
+      <c r="N848" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/tNEAAeSwWaNq0CrJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O848" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P848" s="2" t="inlineStr"/>
+      <c r="Q848" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R848" s="2" t="inlineStr"/>
+      <c r="S848" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="2" t="inlineStr">
+        <is>
+          <t>Alex De Minaur/Lorenzo Musetti</t>
+        </is>
+      </c>
+      <c r="B849" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS CHROME TENNIS DUAL AUTOGRAPHS</t>
+        </is>
+      </c>
+      <c r="C849" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS CHROME TENNIS DUAL AUTOS ALEX DE MINAUR/LORENZO MUSETTI 1/1 PSA 8</t>
+        </is>
+      </c>
+      <c r="D849" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E849" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F849" s="2" t="inlineStr">
+        <is>
+          <t>5555.55 USD</t>
+        </is>
+      </c>
+      <c r="G849" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/900014138770</t>
+        </is>
+      </c>
+      <c r="H849" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I849" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/oeoAAeSw6IBq0Cqx/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J849" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T01:20:50.000Z</t>
+        </is>
+      </c>
+      <c r="K849" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L849" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M849" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 8</t>
+        </is>
+      </c>
+      <c r="N849" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/qqoAAeSw-7Fq0Cqx/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O849" s="2" t="inlineStr"/>
+      <c r="P849" s="2" t="inlineStr"/>
+      <c r="Q849" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R849" s="2" t="inlineStr"/>
+      <c r="S849" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="2" t="inlineStr">
+        <is>
+          <t>Andy Roddick</t>
+        </is>
+      </c>
+      <c r="B850" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="C850" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS CHROME TENNIS SUPERFRACTOR 1/1 #104 ANDY RODDICK 1/1 PSA 9</t>
+        </is>
+      </c>
+      <c r="D850" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E850" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F850" s="2" t="inlineStr">
+        <is>
+          <t>15000.00 USD</t>
+        </is>
+      </c>
+      <c r="G850" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307231836576</t>
+        </is>
+      </c>
+      <c r="H850" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I850" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/pUQAAeSwmZlq0CqJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J850" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T01:19:57.000Z</t>
+        </is>
+      </c>
+      <c r="K850" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L850" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M850" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N850" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/NzIAAeSwwaRq0CqJ/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O850" s="2" t="inlineStr"/>
+      <c r="P850" s="2" t="inlineStr"/>
+      <c r="Q850" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R850" s="2" t="inlineStr"/>
+      <c r="S850" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="2" t="inlineStr">
+        <is>
+          <t>Leylah Fernandez</t>
+        </is>
+      </c>
+      <c r="B851" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 TOPPS CHROME TENNIS ACES AUTOGRAPHS</t>
+        </is>
+      </c>
+      <c r="C851" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME TENNIS ACES AUTOS RED REFRACTOR LEYLAH FERNANDEZ 1/5 PSA 10</t>
+        </is>
+      </c>
+      <c r="D851" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E851" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F851" s="2" t="inlineStr">
+        <is>
+          <t>2222.22 USD</t>
+        </is>
+      </c>
+      <c r="G851" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/900014135438</t>
+        </is>
+      </c>
+      <c r="H851" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I851" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/l-YAAeSwTcdq0Cog/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J851" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T01:18:23.000Z</t>
+        </is>
+      </c>
+      <c r="K851" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L851" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M851" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 10</t>
+        </is>
+      </c>
+      <c r="N851" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/mT4AAeSwFwBq0Cog/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O851" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P851" s="2" t="inlineStr"/>
+      <c r="Q851" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R851" s="2" t="inlineStr"/>
+      <c r="S851" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="2" t="inlineStr">
+        <is>
+          <t>Dalibor Svrcina</t>
+        </is>
+      </c>
+      <c r="B852" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS CHROME TENNIS</t>
+        </is>
+      </c>
+      <c r="C852" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS CHROME TENNIS SUPERFRACTOR 1/1 #182 DALIBOR SVRCINA 1/1 PSA 10</t>
+        </is>
+      </c>
+      <c r="D852" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E852" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F852" s="2" t="inlineStr">
+        <is>
+          <t>1500.00 USD</t>
+        </is>
+      </c>
+      <c r="G852" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/900014134832</t>
+        </is>
+      </c>
+      <c r="H852" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I852" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/rsAAAeSwZV1q0Cnm/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J852" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T01:17:26.000Z</t>
+        </is>
+      </c>
+      <c r="K852" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L852" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M852" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 10</t>
+        </is>
+      </c>
+      <c r="N852" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/sLYAAeSwORxq0Cnl/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O852" s="2" t="inlineStr"/>
+      <c r="P852" s="2" t="inlineStr"/>
+      <c r="Q852" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R852" s="2" t="inlineStr"/>
+      <c r="S852" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" s="2" t="inlineStr">
+        <is>
+          <t>Andy Roddick</t>
+        </is>
+      </c>
+      <c r="B853" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 TOPPS CHROME SAPPHIRE EDITION TENNIS</t>
+        </is>
+      </c>
+      <c r="C853" s="2" t="inlineStr">
+        <is>
+          <t>2025 TOPPS CHROME SAPPHIRE EDITION TENNIS #219 ANDY RODDICK 1/1 PSA 7</t>
+        </is>
+      </c>
+      <c r="D853" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E853" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F853" s="2" t="inlineStr">
+        <is>
+          <t>10000.00 USD</t>
+        </is>
+      </c>
+      <c r="G853" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/307231832853</t>
+        </is>
+      </c>
+      <c r="H853" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I853" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ohUAAeSwO9Zq0Cm2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J853" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T01:16:40.000Z</t>
+        </is>
+      </c>
+      <c r="K853" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L853" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M853" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 7</t>
+        </is>
+      </c>
+      <c r="N853" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/mRoAAeSwC4Fq0Cm2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O853" s="2" t="inlineStr"/>
+      <c r="P853" s="2" t="inlineStr"/>
+      <c r="Q853" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R853" s="2" t="inlineStr"/>
+      <c r="S853" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" s="2" t="inlineStr">
+        <is>
+          <t>Louisa Chirico</t>
+        </is>
+      </c>
+      <c r="B854" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C854" s="2" t="inlineStr">
+        <is>
+          <t>Louisa Chirico 2026 Topps Chrome Black Refractor 10/10</t>
+        </is>
+      </c>
+      <c r="D854" s="2" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="E854" s="2" t="inlineStr">
+        <is>
+          <t>last of 10 (10/10)</t>
+        </is>
+      </c>
+      <c r="F854" s="2" t="inlineStr">
+        <is>
+          <t>1.75 USD</t>
+        </is>
+      </c>
+      <c r="G854" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/840021765150</t>
+        </is>
+      </c>
+      <c r="H854" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I854" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/T2oAAeSwK0Fqz8nA/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J854" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T01:02:00.000Z</t>
+        </is>
+      </c>
+      <c r="K854" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L854" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M854" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N854" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/6HUAAeSwgx5qz8nA/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O854" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P854" s="2" t="inlineStr"/>
+      <c r="Q854" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R854" s="2" t="inlineStr"/>
+      <c r="S854" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="2" t="inlineStr">
+        <is>
+          <t>Bjorn Fratangelo</t>
+        </is>
+      </c>
+      <c r="B855" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C855" s="2" t="inlineStr">
+        <is>
+          <t>Bjorn Fratangelo 2026 Topps Chrome Tennis Auto II Pink Refractor 250/250 [2hk</t>
+        </is>
+      </c>
+      <c r="D855" s="2" t="inlineStr">
+        <is>
+          <t>250/250</t>
+        </is>
+      </c>
+      <c r="E855" s="2" t="inlineStr">
+        <is>
+          <t>last of 250 (250/250)</t>
+        </is>
+      </c>
+      <c r="F855" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G855" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/377571441055</t>
+        </is>
+      </c>
+      <c r="H855" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I855" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/faoAAeSw86tq0CX-/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J855" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T01:00:46.000Z</t>
+        </is>
+      </c>
+      <c r="K855" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L855" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M855" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N855" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/fBoAAeSw8thq0CX~/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O855" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="P855" s="2" t="inlineStr"/>
+      <c r="Q855" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R855" s="2" t="inlineStr"/>
+      <c r="S855" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="2" t="inlineStr">
+        <is>
+          <t>Max Purcell</t>
+        </is>
+      </c>
+      <c r="B856" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C856" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Tennis Max Purcell Aces Auto Superfractor 1/1 BGS 9.5 Auto 10</t>
+        </is>
+      </c>
+      <c r="D856" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E856" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F856" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G856" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/900013811585</t>
+        </is>
+      </c>
+      <c r="H856" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I856" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/6DMAAeSwfrZqz-Kb/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J856" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T01:00:01.000Z</t>
+        </is>
+      </c>
+      <c r="K856" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L856" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M856" s="2" t="inlineStr">
+        <is>
+          <t>BGS 9.5</t>
+        </is>
+      </c>
+      <c r="N856" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/jPoAAeSwDOlqz-Kb/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O856" s="2" t="inlineStr"/>
+      <c r="P856" s="2" t="inlineStr"/>
+      <c r="Q856" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R856" s="2" t="inlineStr"/>
+      <c r="S856" s="2" t="inlineStr">
+        <is>
+          <t>Auto Racing</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="2" t="inlineStr">
+        <is>
+          <t>Destiny Flavio Cobolli</t>
+        </is>
+      </c>
+      <c r="B857" s="2" t="inlineStr">
+        <is>
+          <t>Topps</t>
+        </is>
+      </c>
+      <c r="C857" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Destiny Flavio Cobolli Red Geometric Refractor 5/5</t>
+        </is>
+      </c>
+      <c r="D857" s="2" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E857" s="2" t="inlineStr">
+        <is>
+          <t>last of 5 (5/5)</t>
+        </is>
+      </c>
+      <c r="F857" s="2" t="inlineStr">
+        <is>
+          <t>0.99 USD</t>
+        </is>
+      </c>
+      <c r="G857" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/960064732225</t>
+        </is>
+      </c>
+      <c r="H857" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I857" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/sHUAAeSwmn1qzvx3/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J857" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T00:40:01.000Z</t>
+        </is>
+      </c>
+      <c r="K857" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L857" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M857" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N857" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~ZwAAeSw6Zlqzvx4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O857" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P857" s="2" t="inlineStr"/>
+      <c r="Q857" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R857" s="2" t="inlineStr"/>
+      <c r="S857" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" s="2" t="inlineStr">
+        <is>
+          <t>Magda Linette</t>
+        </is>
+      </c>
+      <c r="B858" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C858" s="2" t="inlineStr">
+        <is>
+          <t>MAGDA LINETTE 2026 TOPPS CHROME TENNIS YELLOW REFRACTOR 1/275 #149 Q0154</t>
+        </is>
+      </c>
+      <c r="D858" s="2" t="inlineStr">
+        <is>
+          <t>1/275</t>
+        </is>
+      </c>
+      <c r="E858" s="2" t="inlineStr">
+        <is>
+          <t>001 of 275</t>
+        </is>
+      </c>
+      <c r="F858" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G858" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/940014207732</t>
+        </is>
+      </c>
+      <c r="H858" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I858" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9JQAAeSwmRBqz6s5/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J858" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T00:39:00.000Z</t>
+        </is>
+      </c>
+      <c r="K858" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L858" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M858" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N858" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/Xx8AAeSwJiJqz6s5/s-l1600.jpg | https://i.ebayimg.com/images/g/X2cAAeSwxl5qz6s4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O858" s="2" t="inlineStr">
+        <is>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="P858" s="2" t="inlineStr"/>
+      <c r="Q858" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R858" s="2" t="inlineStr"/>
+      <c r="S858" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" s="2" t="inlineStr">
+        <is>
+          <t>Daniel Rincon</t>
+        </is>
+      </c>
+      <c r="B859" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis Tennis</t>
+        </is>
+      </c>
+      <c r="C859" s="2" t="inlineStr">
+        <is>
+          <t>DANIEL RINCON 2026 TOPPS CHROME ORANGE GEOMETRIC REFRACTOR AUTO 01/25 Q7656</t>
+        </is>
+      </c>
+      <c r="D859" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E859" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F859" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G859" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/940014610655</t>
+        </is>
+      </c>
+      <c r="H859" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I859" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/SAEAAeSwfrZq0CAO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J859" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T00:35:25.000Z</t>
+        </is>
+      </c>
+      <c r="K859" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L859" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M859" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N859" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RnYAAeSwiVdq0CAP/s-l1600.jpg | https://i.ebayimg.com/images/g/ShUAAeSwBJdq0CAO/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O859" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P859" s="2" t="inlineStr"/>
+      <c r="Q859" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R859" s="2" t="inlineStr"/>
+      <c r="S859" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" s="2" t="inlineStr">
+        <is>
+          <t>Nicolas Mejia</t>
+        </is>
+      </c>
+      <c r="B860" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C860" s="2" t="inlineStr">
+        <is>
+          <t>NICOLAS MEJIA 2026 TOPPS CHROME ORANGE GEOMETRIC REFRACTOR 01/25 #187 Q7656</t>
+        </is>
+      </c>
+      <c r="D860" s="2" t="inlineStr">
+        <is>
+          <t>1/25</t>
+        </is>
+      </c>
+      <c r="E860" s="2" t="inlineStr">
+        <is>
+          <t>001 of 25</t>
+        </is>
+      </c>
+      <c r="F860" s="2" t="inlineStr">
+        <is>
+          <t>1.00 USD</t>
+        </is>
+      </c>
+      <c r="G860" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/940014610618</t>
+        </is>
+      </c>
+      <c r="H860" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I860" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TY0AAeSwmYdq0CAH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J860" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T00:35:20.000Z</t>
+        </is>
+      </c>
+      <c r="K860" s="2" t="inlineStr">
+        <is>
+          <t>Auction</t>
+        </is>
+      </c>
+      <c r="L860" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M860" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N860" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/RCkAAeSwh-Nq0CAI/s-l1600.jpg | https://i.ebayimg.com/images/g/RqwAAeSw6nZq0CAH/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O860" s="2" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="P860" s="2" t="inlineStr"/>
+      <c r="Q860" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R860" s="2" t="inlineStr"/>
+      <c r="S860" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" s="2" t="inlineStr">
+        <is>
+          <t>Elina Svitolina</t>
+        </is>
+      </c>
+      <c r="B861" s="2" t="inlineStr">
+        <is>
+          <t>Topps / Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C861" s="2" t="inlineStr">
+        <is>
+          <t>Topps Chrome 2026 Elina Svitolina #95 Superfractor 1/1 WTA Tennis Card</t>
+        </is>
+      </c>
+      <c r="D861" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E861" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F861" s="2" t="inlineStr">
+        <is>
+          <t>2700.00 USD</t>
+        </is>
+      </c>
+      <c r="G861" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/407291044860</t>
+        </is>
+      </c>
+      <c r="H861" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I861" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/HAkAAeSwtG1q0Bwg/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J861" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T00:21:07.000Z</t>
+        </is>
+      </c>
+      <c r="K861" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L861" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M861" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N861" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/KPUAAeSwQiFq0Bv7/s-l1600.jpg | https://i.ebayimg.com/images/g/JIoAAeSwdOtq0Bv7/s-l1600.jpg | https://i.ebayimg.com/images/g/ICgAAeSwutRq0Bv7/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O861" s="2" t="inlineStr"/>
+      <c r="P861" s="2" t="inlineStr"/>
+      <c r="Q861" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R861" s="2" t="inlineStr"/>
+      <c r="S861" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" s="2" t="inlineStr">
+        <is>
+          <t>Mirra Andreeva, Conchita Martinez</t>
+        </is>
+      </c>
+      <c r="B862" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C862" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Mirra Andreeva / Conchita Martinez Dual Auto 1/10 Black</t>
+        </is>
+      </c>
+      <c r="D862" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E862" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F862" s="2" t="inlineStr">
+        <is>
+          <t>4999.00 USD</t>
+        </is>
+      </c>
+      <c r="G862" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/227567814251</t>
+        </is>
+      </c>
+      <c r="H862" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I862" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/-MUAAeSwu-1q0Bc6/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J862" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T00:03:59.000Z</t>
+        </is>
+      </c>
+      <c r="K862" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L862" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M862" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N862" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/~vYAAeSwylZq0Bco/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O862" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P862" s="2" t="inlineStr"/>
+      <c r="Q862" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R862" s="2" t="inlineStr"/>
+      <c r="S862" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="2" t="inlineStr">
+        <is>
+          <t>Alex Michelsen</t>
+        </is>
+      </c>
+      <c r="B863" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C863" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Alex Michelsen Youthquake #YQ-AM Black Geometric 1/10</t>
+        </is>
+      </c>
+      <c r="D863" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E863" s="2" t="inlineStr">
+        <is>
+          <t>001 of 10</t>
+        </is>
+      </c>
+      <c r="F863" s="2" t="inlineStr">
+        <is>
+          <t>49.99 USD</t>
+        </is>
+      </c>
+      <c r="G863" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/860045172629</t>
+        </is>
+      </c>
+      <c r="H863" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I863" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/eJwAAeSwkWNqz~Db/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J863" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T21:16:53.000Z</t>
+        </is>
+      </c>
+      <c r="K863" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L863" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M863" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N863" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/ZUcAAeSwrX5qz~Db/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O863" s="2" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="P863" s="2" t="inlineStr"/>
+      <c r="Q863" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R863" s="2" t="inlineStr"/>
+      <c r="S863" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Moya</t>
+        </is>
+      </c>
+      <c r="B864" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C864" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Carlos Moya World No.1 #WNO-CM Red Geometric 1/5</t>
+        </is>
+      </c>
+      <c r="D864" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E864" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F864" s="2" t="inlineStr">
+        <is>
+          <t>149.99 USD</t>
+        </is>
+      </c>
+      <c r="G864" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/860045167705</t>
+        </is>
+      </c>
+      <c r="H864" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I864" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/aZUAAeSwC4Fqz-~2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J864" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T21:12:55.000Z</t>
+        </is>
+      </c>
+      <c r="K864" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L864" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M864" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N864" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/V3oAAeSwq5hqz-~2/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O864" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P864" s="2" t="inlineStr"/>
+      <c r="Q864" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R864" s="2" t="inlineStr"/>
+      <c r="S864" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="2" t="inlineStr">
+        <is>
+          <t>Aryna Sabalenka</t>
+        </is>
+      </c>
+      <c r="B865" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="C865" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Winners Alliance Captured Aryna Sabalenka CTD-18 #1/2 SSP</t>
+        </is>
+      </c>
+      <c r="D865" s="2" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="E865" s="2" t="inlineStr">
+        <is>
+          <t>001 of 2</t>
+        </is>
+      </c>
+      <c r="F865" s="2" t="inlineStr">
+        <is>
+          <t>599.99 USD</t>
+        </is>
+      </c>
+      <c r="G865" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/227567697696</t>
+        </is>
+      </c>
+      <c r="H865" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I865" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/dXUAAeSwJzhqz~BE/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J865" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T21:12:53.000Z</t>
+        </is>
+      </c>
+      <c r="K865" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L865" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M865" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N865" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/e3YAAeSwQvlqz~Aq/s-l1600.jpg | https://i.ebayimg.com/images/g/fBkAAeSwxtBqz~As/s-l1600.jpg | https://i.ebayimg.com/images/g/e~gAAeSwT6Bqz~Ay/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O865" s="2" t="inlineStr"/>
+      <c r="P865" s="2" t="inlineStr"/>
+      <c r="Q865" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R865" s="2" t="inlineStr"/>
+      <c r="S865" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" s="2" t="inlineStr">
+        <is>
+          <t>Otto Virtanen</t>
+        </is>
+      </c>
+      <c r="B866" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2026 Topps Chrome Tennis</t>
+        </is>
+      </c>
+      <c r="C866" s="2" t="inlineStr">
+        <is>
+          <t>2026 Topps Chrome Tennis Otto Virtanen Red Geometric Auto 1/5</t>
+        </is>
+      </c>
+      <c r="D866" s="2" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E866" s="2" t="inlineStr">
+        <is>
+          <t>001 of 5</t>
+        </is>
+      </c>
+      <c r="F866" s="2" t="inlineStr">
+        <is>
+          <t>99.99 USD</t>
+        </is>
+      </c>
+      <c r="G866" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/860045163593</t>
+        </is>
+      </c>
+      <c r="H866" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I866" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/TPMAAeSwMmBqz-9a/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J866" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T21:10:26.000Z</t>
+        </is>
+      </c>
+      <c r="K866" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L866" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M866" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N866" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/W88AAeSwPLtqz-9Z/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O866" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P866" s="2" t="inlineStr"/>
+      <c r="Q866" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R866" s="2" t="inlineStr"/>
+      <c r="S866" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="2" t="inlineStr">
+        <is>
+          <t>Andy Roddick</t>
+        </is>
+      </c>
+      <c r="B867" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS GRAPHITE TENNIS</t>
+        </is>
+      </c>
+      <c r="C867" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS GRAPHITE TENNIS RED CRYSTALLINE REFRACTOR 1/1 ANDY RODDICK 1/1 PSA 9</t>
+        </is>
+      </c>
+      <c r="D867" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E867" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F867" s="2" t="inlineStr">
+        <is>
+          <t>3333.33 USD</t>
+        </is>
+      </c>
+      <c r="G867" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/900014157327</t>
+        </is>
+      </c>
+      <c r="H867" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I867" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/zJgAAeSw8XRq0C8s/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J867" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T01:39:57.000Z</t>
+        </is>
+      </c>
+      <c r="K867" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L867" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="M867" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 9</t>
+        </is>
+      </c>
+      <c r="N867" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/3H8AAeSwqaxq0C8s/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O867" s="2" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="P867" s="2" t="inlineStr"/>
+      <c r="Q867" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="R867" s="2" t="inlineStr"/>
+      <c r="S867" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" s="2" t="inlineStr">
+        <is>
+          <t>Pablo Carreno Busta</t>
+        </is>
+      </c>
+      <c r="B868" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 TOPPS ROYALTY TENNIS SUPERIOR SIGNATURES</t>
+        </is>
+      </c>
+      <c r="C868" s="2" t="inlineStr">
+        <is>
+          <t>2024 TOPPS ROYALTY TENNIS SUPERIOR SIGNATURES PABLO CARRENO BUSTA 1/1 PSA 10</t>
+        </is>
+      </c>
+      <c r="D868" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E868" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F868" s="2" t="inlineStr">
+        <is>
+          <t>2222.22 USD</t>
+        </is>
+      </c>
+      <c r="G868" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/900014158348</t>
+        </is>
+      </c>
+      <c r="H868" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I868" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/x8cAAeSwtKFq0C94/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J868" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T01:41:14.000Z</t>
+        </is>
+      </c>
+      <c r="K868" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L868" s="2" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="M868" s="2" t="inlineStr">
+        <is>
+          <t>Professional Sports Authenticator (PSA) 10</t>
+        </is>
+      </c>
+      <c r="N868" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/1aYAAeSw~Qtq0C94/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O868" s="2" t="inlineStr"/>
+      <c r="P868" s="2" t="inlineStr"/>
+      <c r="Q868" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R868" s="2" t="inlineStr"/>
+      <c r="S868" s="2" t="inlineStr">
+        <is>
+          <t>Tennis</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="2" t="inlineStr">
+        <is>
+          <t>Garbine Muguruza Babolat</t>
+        </is>
+      </c>
+      <c r="B869" s="2" t="inlineStr">
+        <is>
+          <t>Topps / 2024 Topps Royalty</t>
+        </is>
+      </c>
+      <c r="C869" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Royalty Tennis The Grip Relic Platinum 1/1 Garbine Muguruza Babolat</t>
+        </is>
+      </c>
+      <c r="D869" s="2" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E869" s="2" t="inlineStr">
+        <is>
+          <t>True 1/1 (both bookends)</t>
+        </is>
+      </c>
+      <c r="F869" s="2" t="inlineStr">
+        <is>
+          <t>799.99 USD</t>
+        </is>
+      </c>
+      <c r="G869" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/168793241415</t>
+        </is>
+      </c>
+      <c r="H869" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 01:45 UTC</t>
+        </is>
+      </c>
+      <c r="I869" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/7SgAAeSwa2Vq0BX4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="J869" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T23:55:26.000Z</t>
+        </is>
+      </c>
+      <c r="K869" s="2" t="inlineStr">
+        <is>
+          <t>Buy It Now</t>
+        </is>
+      </c>
+      <c r="L869" s="2" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="M869" s="2" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N869" s="2" t="inlineStr">
+        <is>
+          <t>https://i.ebayimg.com/images/g/9PwAAeSwm1tq0BX4/s-l1600.jpg</t>
+        </is>
+      </c>
+      <c r="O869" s="2" t="inlineStr"/>
+      <c r="P869" s="2" t="inlineStr"/>
+      <c r="Q869" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R869" s="2" t="inlineStr"/>
+      <c r="S869" s="2" t="inlineStr">
         <is>
           <t>Tennis</t>
         </is>
@@ -74999,6 +77350,33 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G840" r:id="rId839"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G841" r:id="rId840"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G842" r:id="rId841"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G843" r:id="rId842"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G844" r:id="rId843"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G845" r:id="rId844"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G846" r:id="rId845"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G847" r:id="rId846"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G848" r:id="rId847"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G849" r:id="rId848"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G850" r:id="rId849"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G851" r:id="rId850"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G852" r:id="rId851"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G853" r:id="rId852"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G854" r:id="rId853"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G855" r:id="rId854"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G856" r:id="rId855"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G857" r:id="rId856"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G858" r:id="rId857"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G859" r:id="rId858"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G860" r:id="rId859"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G861" r:id="rId860"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G862" r:id="rId861"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G863" r:id="rId862"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G864" r:id="rId863"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G865" r:id="rId864"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G866" r:id="rId865"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G867" r:id="rId866"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G868" r:id="rId867"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G869" r:id="rId868"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>